<commit_message>
Added Line Details Validation and Line Amount in 'from PR to PO' test scenarios
Added Line Details Validation and Line Amount in 'from PR to PO' test scenarios
</commit_message>
<xml_diff>
--- a/testdata/ItemDetails.xlsx
+++ b/testdata/ItemDetails.xlsx
@@ -84,7 +84,7 @@
     <t>GENERAL U-100</t>
   </si>
   <si>
-    <t>GWL_ITEM_DISIMILAR_UOM</t>
+    <t>GWL_ITEM_DISSIMILAR_UOM</t>
   </si>
   <si>
     <t>FG WAREHOUSE 100</t>
@@ -1409,7 +1409,7 @@
         <v>19</v>
       </c>
       <c r="E3" s="3">
-        <v>20</v>
+        <v>6</v>
       </c>
       <c r="F3" s="4" t="s">
         <v>20</v>

</xml_diff>

<commit_message>
Merged Main & Resolved Conflicts
Merged Main And Resolved Conflicts
</commit_message>
<xml_diff>
--- a/testdata/ItemDetails.xlsx
+++ b/testdata/ItemDetails.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="19200" windowHeight="6920"/>
+    <workbookView windowWidth="23040" windowHeight="9120" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="PR Details" sheetId="1" r:id="rId1"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="25">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="77" uniqueCount="44">
   <si>
     <t>ITEM_NAME</t>
   </si>
@@ -102,7 +102,64 @@
     <t>PRODUCTION  100</t>
   </si>
   <si>
-    <t>PO</t>
+    <t>ITEMID</t>
+  </si>
+  <si>
+    <t>ITEM_DESCRIPTION</t>
+  </si>
+  <si>
+    <t>UOM</t>
+  </si>
+  <si>
+    <t>HSN_CODE</t>
+  </si>
+  <si>
+    <t>TAX</t>
+  </si>
+  <si>
+    <t>WH_DEPTNAME</t>
+  </si>
+  <si>
+    <t>COST_BASIS</t>
+  </si>
+  <si>
+    <t>STOCK_UOM</t>
+  </si>
+  <si>
+    <t>CONVERSION_FACTOR</t>
+  </si>
+  <si>
+    <t>CONTRACT_NO</t>
+  </si>
+  <si>
+    <t>CONTRACT_PRFX</t>
+  </si>
+  <si>
+    <t>CONTRACT_AMEND_NO</t>
+  </si>
+  <si>
+    <t>PO_CLS_QTY</t>
+  </si>
+  <si>
+    <t>RCM_CAT_ID</t>
+  </si>
+  <si>
+    <t>GWL_ITEM_DISSIMILAR_UOM_DESC</t>
+  </si>
+  <si>
+    <t>(740410)-18%</t>
+  </si>
+  <si>
+    <t>User Defined</t>
+  </si>
+  <si>
+    <t>GWL ITEM SERIAL</t>
+  </si>
+  <si>
+    <t>(2022)</t>
+  </si>
+  <si>
+    <t>User Defined Price</t>
   </si>
 </sst>
 </file>
@@ -115,13 +172,25 @@
     <numFmt numFmtId="178" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
     <numFmt numFmtId="179" formatCode="_ &quot;₹&quot;* #,##0_ ;_ &quot;₹&quot;* \-#,##0_ ;_ &quot;₹&quot;* &quot;-&quot;_ ;_ @_ "/>
   </numFmts>
-  <fonts count="24">
+  <fonts count="26">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <charset val="134"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Times New Roman"/>
+      <charset val="134"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF262626"/>
+      <name val="Times New Roman"/>
+      <charset val="134"/>
     </font>
     <font>
       <sz val="8"/>
@@ -635,153 +704,162 @@
     <xf numFmtId="179" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="2" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="4" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="5" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="5" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="6" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="4" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="5" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="5" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="6" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="justify" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -1318,336 +1396,336 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1:J20"/>
-  <sheetFormatPr defaultColWidth="8.72727272727273" defaultRowHeight="14.5"/>
+  <sheetFormatPr defaultColWidth="8.73148148148148" defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="20.7272727272727" customWidth="1"/>
-    <col min="2" max="3" width="12.7272727272727" customWidth="1"/>
-    <col min="4" max="4" width="14.7272727272727" customWidth="1"/>
-    <col min="5" max="5" width="9.81818181818182" customWidth="1"/>
-    <col min="6" max="6" width="14.1818181818182" customWidth="1"/>
-    <col min="7" max="7" width="14.8181818181818" customWidth="1"/>
-    <col min="8" max="8" width="13.8181818181818" customWidth="1"/>
-    <col min="9" max="9" width="14.3636363636364" customWidth="1"/>
+    <col min="1" max="1" width="20.7314814814815" customWidth="1"/>
+    <col min="2" max="3" width="12.7314814814815" customWidth="1"/>
+    <col min="4" max="4" width="14.7314814814815" customWidth="1"/>
+    <col min="5" max="5" width="9.81481481481481" customWidth="1"/>
+    <col min="6" max="6" width="14.1851851851852" customWidth="1"/>
+    <col min="7" max="7" width="14.8148148148148" customWidth="1"/>
+    <col min="8" max="8" width="13.8148148148148" customWidth="1"/>
+    <col min="9" max="9" width="14.3611111111111" customWidth="1"/>
     <col min="10" max="10" width="13" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:10">
-      <c r="A1" s="2" t="s">
+      <c r="A1" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="B1" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="C1" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="D1" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="E1" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="2" t="s">
+      <c r="F1" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="2" t="s">
+      <c r="G1" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="2" t="s">
+      <c r="H1" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="2" t="s">
+      <c r="I1" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="2" t="s">
+      <c r="J1" s="5" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="2" s="1" customFormat="1" ht="21" spans="1:10">
-      <c r="A2" s="3" t="s">
+    <row r="2" s="4" customFormat="1" ht="20.4" spans="1:10">
+      <c r="A2" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="B2" s="4" t="s">
+      <c r="B2" s="7" t="s">
         <v>11</v>
       </c>
-      <c r="C2" s="4" t="s">
+      <c r="C2" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="D2" s="3" t="s">
+      <c r="D2" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="E2" s="3">
+      <c r="E2" s="6">
         <v>1</v>
       </c>
-      <c r="F2" s="3" t="s">
+      <c r="F2" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="G2" s="3">
+      <c r="G2" s="6">
         <v>1010301033</v>
       </c>
-      <c r="H2" s="3" t="s">
+      <c r="H2" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="I2" s="3" t="s">
+      <c r="I2" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="J2" s="3" t="s">
+      <c r="J2" s="6" t="s">
         <v>17</v>
       </c>
     </row>
     <row r="3" ht="15" customHeight="1" spans="1:10">
-      <c r="A3" s="3" t="s">
+      <c r="A3" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="B3" s="4" t="s">
+      <c r="B3" s="7" t="s">
         <v>11</v>
       </c>
-      <c r="C3" s="4" t="s">
+      <c r="C3" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="D3" s="3" t="s">
+      <c r="D3" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="E3" s="3">
+      <c r="E3" s="6">
         <v>6</v>
       </c>
-      <c r="F3" s="4" t="s">
+      <c r="F3" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="G3" s="3">
+      <c r="G3" s="6">
         <v>1010301033</v>
       </c>
-      <c r="H3" s="3" t="s">
+      <c r="H3" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="I3" s="3" t="s">
+      <c r="I3" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="J3" s="3" t="s">
+      <c r="J3" s="6" t="s">
         <v>17</v>
       </c>
     </row>
     <row r="4" spans="1:10">
-      <c r="A4" s="3" t="s">
+      <c r="A4" s="6" t="s">
         <v>21</v>
       </c>
-      <c r="B4" s="4" t="s">
+      <c r="B4" s="7" t="s">
         <v>22</v>
       </c>
-      <c r="C4" s="4" t="s">
+      <c r="C4" s="7" t="s">
         <v>22</v>
       </c>
-      <c r="D4" s="3" t="s">
+      <c r="D4" s="6" t="s">
         <v>23</v>
       </c>
-      <c r="E4" s="3">
+      <c r="E4" s="6">
         <v>1</v>
       </c>
-      <c r="F4" s="4" t="s">
+      <c r="F4" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="G4" s="3">
+      <c r="G4" s="6">
         <v>1000000001</v>
       </c>
-      <c r="H4" s="3"/>
-      <c r="I4" s="3" t="s">
+      <c r="H4" s="6"/>
+      <c r="I4" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="J4" s="3" t="s">
+      <c r="J4" s="6" t="s">
         <v>17</v>
       </c>
     </row>
     <row r="5" spans="1:10">
-      <c r="A5" s="5"/>
-      <c r="B5" s="5"/>
-      <c r="C5" s="5"/>
-      <c r="D5" s="5"/>
-      <c r="E5" s="5"/>
-      <c r="F5" s="5"/>
-      <c r="G5" s="5"/>
-      <c r="H5" s="5"/>
-      <c r="I5" s="5"/>
-      <c r="J5" s="5"/>
+      <c r="A5" s="8"/>
+      <c r="B5" s="8"/>
+      <c r="C5" s="8"/>
+      <c r="D5" s="8"/>
+      <c r="E5" s="8"/>
+      <c r="F5" s="8"/>
+      <c r="G5" s="8"/>
+      <c r="H5" s="8"/>
+      <c r="I5" s="8"/>
+      <c r="J5" s="8"/>
     </row>
     <row r="6" spans="1:10">
-      <c r="A6" s="5"/>
-      <c r="B6" s="5"/>
-      <c r="C6" s="5"/>
-      <c r="D6" s="5"/>
-      <c r="E6" s="5"/>
-      <c r="F6" s="5"/>
-      <c r="G6" s="5"/>
-      <c r="H6" s="5"/>
-      <c r="I6" s="5"/>
-      <c r="J6" s="5"/>
+      <c r="A6" s="8"/>
+      <c r="B6" s="8"/>
+      <c r="C6" s="8"/>
+      <c r="D6" s="8"/>
+      <c r="E6" s="8"/>
+      <c r="F6" s="8"/>
+      <c r="G6" s="8"/>
+      <c r="H6" s="8"/>
+      <c r="I6" s="8"/>
+      <c r="J6" s="8"/>
     </row>
     <row r="7" spans="1:10">
-      <c r="A7" s="5"/>
-      <c r="B7" s="5"/>
-      <c r="C7" s="5"/>
-      <c r="D7" s="5"/>
-      <c r="E7" s="5"/>
-      <c r="F7" s="5"/>
-      <c r="G7" s="5"/>
-      <c r="H7" s="5"/>
-      <c r="I7" s="5"/>
-      <c r="J7" s="5"/>
+      <c r="A7" s="8"/>
+      <c r="B7" s="8"/>
+      <c r="C7" s="8"/>
+      <c r="D7" s="8"/>
+      <c r="E7" s="8"/>
+      <c r="F7" s="8"/>
+      <c r="G7" s="8"/>
+      <c r="H7" s="8"/>
+      <c r="I7" s="8"/>
+      <c r="J7" s="8"/>
     </row>
     <row r="8" spans="1:10">
-      <c r="A8" s="5"/>
-      <c r="B8" s="5"/>
-      <c r="C8" s="5"/>
-      <c r="D8" s="5"/>
-      <c r="E8" s="5"/>
-      <c r="F8" s="5"/>
-      <c r="G8" s="5"/>
-      <c r="H8" s="5"/>
-      <c r="I8" s="5"/>
-      <c r="J8" s="5"/>
+      <c r="A8" s="8"/>
+      <c r="B8" s="8"/>
+      <c r="C8" s="8"/>
+      <c r="D8" s="8"/>
+      <c r="E8" s="8"/>
+      <c r="F8" s="8"/>
+      <c r="G8" s="8"/>
+      <c r="H8" s="8"/>
+      <c r="I8" s="8"/>
+      <c r="J8" s="8"/>
     </row>
     <row r="9" spans="1:10">
-      <c r="A9" s="5"/>
-      <c r="B9" s="5"/>
-      <c r="C9" s="5"/>
-      <c r="D9" s="5"/>
-      <c r="E9" s="5"/>
-      <c r="F9" s="5"/>
-      <c r="G9" s="5"/>
-      <c r="H9" s="5"/>
-      <c r="I9" s="5"/>
-      <c r="J9" s="5"/>
+      <c r="A9" s="8"/>
+      <c r="B9" s="8"/>
+      <c r="C9" s="8"/>
+      <c r="D9" s="8"/>
+      <c r="E9" s="8"/>
+      <c r="F9" s="8"/>
+      <c r="G9" s="8"/>
+      <c r="H9" s="8"/>
+      <c r="I9" s="8"/>
+      <c r="J9" s="8"/>
     </row>
     <row r="10" spans="1:10">
-      <c r="A10" s="5"/>
-      <c r="B10" s="5"/>
-      <c r="C10" s="5"/>
-      <c r="D10" s="5"/>
-      <c r="E10" s="5"/>
-      <c r="F10" s="5"/>
-      <c r="G10" s="5"/>
-      <c r="H10" s="5"/>
-      <c r="I10" s="5"/>
-      <c r="J10" s="5"/>
+      <c r="A10" s="8"/>
+      <c r="B10" s="8"/>
+      <c r="C10" s="8"/>
+      <c r="D10" s="8"/>
+      <c r="E10" s="8"/>
+      <c r="F10" s="8"/>
+      <c r="G10" s="8"/>
+      <c r="H10" s="8"/>
+      <c r="I10" s="8"/>
+      <c r="J10" s="8"/>
     </row>
     <row r="11" spans="1:10">
-      <c r="A11" s="5"/>
-      <c r="B11" s="5"/>
-      <c r="C11" s="5"/>
-      <c r="D11" s="5"/>
-      <c r="E11" s="5"/>
-      <c r="F11" s="5"/>
-      <c r="G11" s="5"/>
-      <c r="H11" s="5"/>
-      <c r="I11" s="5"/>
-      <c r="J11" s="5"/>
+      <c r="A11" s="8"/>
+      <c r="B11" s="8"/>
+      <c r="C11" s="8"/>
+      <c r="D11" s="8"/>
+      <c r="E11" s="8"/>
+      <c r="F11" s="8"/>
+      <c r="G11" s="8"/>
+      <c r="H11" s="8"/>
+      <c r="I11" s="8"/>
+      <c r="J11" s="8"/>
     </row>
     <row r="12" spans="1:10">
-      <c r="A12" s="5"/>
-      <c r="B12" s="5"/>
-      <c r="C12" s="5"/>
-      <c r="D12" s="5"/>
-      <c r="E12" s="5"/>
-      <c r="F12" s="5"/>
-      <c r="G12" s="5"/>
-      <c r="H12" s="5"/>
-      <c r="I12" s="5"/>
-      <c r="J12" s="5"/>
+      <c r="A12" s="8"/>
+      <c r="B12" s="8"/>
+      <c r="C12" s="8"/>
+      <c r="D12" s="8"/>
+      <c r="E12" s="8"/>
+      <c r="F12" s="8"/>
+      <c r="G12" s="8"/>
+      <c r="H12" s="8"/>
+      <c r="I12" s="8"/>
+      <c r="J12" s="8"/>
     </row>
     <row r="13" spans="1:10">
-      <c r="A13" s="5"/>
-      <c r="B13" s="5"/>
-      <c r="C13" s="5"/>
-      <c r="D13" s="5"/>
-      <c r="E13" s="5"/>
-      <c r="F13" s="5"/>
-      <c r="G13" s="5"/>
-      <c r="H13" s="5"/>
-      <c r="I13" s="5"/>
-      <c r="J13" s="5"/>
+      <c r="A13" s="8"/>
+      <c r="B13" s="8"/>
+      <c r="C13" s="8"/>
+      <c r="D13" s="8"/>
+      <c r="E13" s="8"/>
+      <c r="F13" s="8"/>
+      <c r="G13" s="8"/>
+      <c r="H13" s="8"/>
+      <c r="I13" s="8"/>
+      <c r="J13" s="8"/>
     </row>
     <row r="14" spans="1:10">
-      <c r="A14" s="5"/>
-      <c r="B14" s="5"/>
-      <c r="C14" s="5"/>
-      <c r="D14" s="5"/>
-      <c r="E14" s="5"/>
-      <c r="F14" s="5"/>
-      <c r="G14" s="5"/>
-      <c r="H14" s="5"/>
-      <c r="I14" s="5"/>
-      <c r="J14" s="5"/>
+      <c r="A14" s="8"/>
+      <c r="B14" s="8"/>
+      <c r="C14" s="8"/>
+      <c r="D14" s="8"/>
+      <c r="E14" s="8"/>
+      <c r="F14" s="8"/>
+      <c r="G14" s="8"/>
+      <c r="H14" s="8"/>
+      <c r="I14" s="8"/>
+      <c r="J14" s="8"/>
     </row>
     <row r="15" spans="1:10">
-      <c r="A15" s="5"/>
-      <c r="B15" s="5"/>
-      <c r="C15" s="5"/>
-      <c r="D15" s="5"/>
-      <c r="E15" s="5"/>
-      <c r="F15" s="5"/>
-      <c r="G15" s="5"/>
-      <c r="H15" s="5"/>
-      <c r="I15" s="5"/>
-      <c r="J15" s="5"/>
+      <c r="A15" s="8"/>
+      <c r="B15" s="8"/>
+      <c r="C15" s="8"/>
+      <c r="D15" s="8"/>
+      <c r="E15" s="8"/>
+      <c r="F15" s="8"/>
+      <c r="G15" s="8"/>
+      <c r="H15" s="8"/>
+      <c r="I15" s="8"/>
+      <c r="J15" s="8"/>
     </row>
     <row r="16" spans="1:10">
-      <c r="A16" s="5"/>
-      <c r="B16" s="5"/>
-      <c r="C16" s="5"/>
-      <c r="D16" s="5"/>
-      <c r="E16" s="5"/>
-      <c r="F16" s="5"/>
-      <c r="G16" s="5"/>
-      <c r="H16" s="5"/>
-      <c r="I16" s="5"/>
-      <c r="J16" s="5"/>
+      <c r="A16" s="8"/>
+      <c r="B16" s="8"/>
+      <c r="C16" s="8"/>
+      <c r="D16" s="8"/>
+      <c r="E16" s="8"/>
+      <c r="F16" s="8"/>
+      <c r="G16" s="8"/>
+      <c r="H16" s="8"/>
+      <c r="I16" s="8"/>
+      <c r="J16" s="8"/>
     </row>
     <row r="17" spans="1:10">
-      <c r="A17" s="5"/>
-      <c r="B17" s="5"/>
-      <c r="C17" s="5"/>
-      <c r="D17" s="5"/>
-      <c r="E17" s="5"/>
-      <c r="F17" s="5"/>
-      <c r="G17" s="5"/>
-      <c r="H17" s="5"/>
-      <c r="I17" s="5"/>
-      <c r="J17" s="5"/>
+      <c r="A17" s="8"/>
+      <c r="B17" s="8"/>
+      <c r="C17" s="8"/>
+      <c r="D17" s="8"/>
+      <c r="E17" s="8"/>
+      <c r="F17" s="8"/>
+      <c r="G17" s="8"/>
+      <c r="H17" s="8"/>
+      <c r="I17" s="8"/>
+      <c r="J17" s="8"/>
     </row>
     <row r="18" spans="1:10">
-      <c r="A18" s="5"/>
-      <c r="B18" s="5"/>
-      <c r="C18" s="5"/>
-      <c r="D18" s="5"/>
-      <c r="E18" s="5"/>
-      <c r="F18" s="5"/>
-      <c r="G18" s="5"/>
-      <c r="H18" s="5"/>
-      <c r="I18" s="5"/>
-      <c r="J18" s="5"/>
+      <c r="A18" s="8"/>
+      <c r="B18" s="8"/>
+      <c r="C18" s="8"/>
+      <c r="D18" s="8"/>
+      <c r="E18" s="8"/>
+      <c r="F18" s="8"/>
+      <c r="G18" s="8"/>
+      <c r="H18" s="8"/>
+      <c r="I18" s="8"/>
+      <c r="J18" s="8"/>
     </row>
     <row r="19" spans="1:10">
-      <c r="A19" s="5"/>
-      <c r="B19" s="5"/>
-      <c r="C19" s="5"/>
-      <c r="D19" s="5"/>
-      <c r="E19" s="5"/>
-      <c r="F19" s="5"/>
-      <c r="G19" s="5"/>
-      <c r="H19" s="5"/>
-      <c r="I19" s="5"/>
-      <c r="J19" s="5"/>
+      <c r="A19" s="8"/>
+      <c r="B19" s="8"/>
+      <c r="C19" s="8"/>
+      <c r="D19" s="8"/>
+      <c r="E19" s="8"/>
+      <c r="F19" s="8"/>
+      <c r="G19" s="8"/>
+      <c r="H19" s="8"/>
+      <c r="I19" s="8"/>
+      <c r="J19" s="8"/>
     </row>
     <row r="20" spans="1:10">
-      <c r="A20" s="5"/>
-      <c r="B20" s="5"/>
-      <c r="C20" s="5"/>
-      <c r="D20" s="5"/>
-      <c r="E20" s="5"/>
-      <c r="F20" s="5"/>
-      <c r="G20" s="5"/>
-      <c r="H20" s="5"/>
-      <c r="I20" s="5"/>
-      <c r="J20" s="5"/>
+      <c r="A20" s="8"/>
+      <c r="B20" s="8"/>
+      <c r="C20" s="8"/>
+      <c r="D20" s="8"/>
+      <c r="E20" s="8"/>
+      <c r="F20" s="8"/>
+      <c r="G20" s="8"/>
+      <c r="H20" s="8"/>
+      <c r="I20" s="8"/>
+      <c r="J20" s="8"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1658,13 +1736,222 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultColWidth="8.72727272727273" defaultRowHeight="14.5"/>
+  <dimension ref="A1:T4"/>
+  <sheetFormatPr defaultColWidth="8.73148148148148" defaultRowHeight="14.4" outlineLevelRow="3"/>
+  <cols>
+    <col min="1" max="1" width="30" customWidth="1"/>
+    <col min="2" max="2" width="36.4444444444444" customWidth="1"/>
+    <col min="3" max="3" width="6" customWidth="1"/>
+    <col min="4" max="4" width="13.6666666666667" customWidth="1"/>
+    <col min="5" max="5" width="5.22222222222222" customWidth="1"/>
+    <col min="6" max="6" width="17.2222222222222" customWidth="1"/>
+    <col min="7" max="7" width="16.1111111111111" customWidth="1"/>
+    <col min="8" max="8" width="26.8888888888889" customWidth="1"/>
+    <col min="9" max="9" width="17.2222222222222" customWidth="1"/>
+    <col min="10" max="10" width="13.2222222222222" customWidth="1"/>
+    <col min="11" max="11" width="22.7777777777778" customWidth="1"/>
+    <col min="12" max="12" width="12.7777777777778" customWidth="1"/>
+    <col min="13" max="13" width="17.5555555555556" customWidth="1"/>
+    <col min="14" max="14" width="15.5555555555556" customWidth="1"/>
+    <col min="15" max="15" width="16.2222222222222" customWidth="1"/>
+    <col min="16" max="16" width="15.5555555555556" customWidth="1"/>
+    <col min="17" max="17" width="17.7777777777778" customWidth="1"/>
+    <col min="18" max="18" width="24.1111111111111" customWidth="1"/>
+    <col min="19" max="19" width="13.4444444444444" customWidth="1"/>
+    <col min="20" max="20" width="13.5555555555556" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:1">
-      <c r="A1" t="s">
+    <row r="1" spans="1:20">
+      <c r="A1" s="1" t="s">
         <v>24</v>
       </c>
+      <c r="B1" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="L1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="M1" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="N1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="O1" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="P1" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="Q1" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="R1" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="S1" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="T1" s="1" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="2" spans="1:20">
+      <c r="A2" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="E2" s="1">
+        <v>12</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="G2" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="H2" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="I2" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="J2" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="K2" s="1">
+        <v>6</v>
+      </c>
+      <c r="L2" s="1">
+        <v>1010301033</v>
+      </c>
+      <c r="M2" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="N2" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="O2" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="P2" s="1"/>
+      <c r="Q2" s="1"/>
+      <c r="R2" s="1"/>
+      <c r="S2" s="1">
+        <v>0</v>
+      </c>
+      <c r="T2" s="1"/>
+    </row>
+    <row r="3" spans="1:20">
+      <c r="A3" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="D3" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="E3" s="1">
+        <v>5</v>
+      </c>
+      <c r="F3" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="G3" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="H3" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="I3" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="J3" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="K3" s="1">
+        <v>1</v>
+      </c>
+      <c r="L3" s="1">
+        <v>1010301033</v>
+      </c>
+      <c r="M3" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="N3" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="O3" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="P3" s="1"/>
+      <c r="Q3" s="1"/>
+      <c r="R3" s="1"/>
+      <c r="S3" s="1">
+        <v>0</v>
+      </c>
+      <c r="T3" s="1"/>
+    </row>
+    <row r="4" spans="1:20">
+      <c r="A4" s="1"/>
+      <c r="B4" s="1"/>
+      <c r="C4" s="1"/>
+      <c r="D4" s="1"/>
+      <c r="E4" s="1"/>
+      <c r="F4" s="1"/>
+      <c r="G4" s="1"/>
+      <c r="H4" s="1"/>
+      <c r="I4" s="1"/>
+      <c r="J4" s="1"/>
+      <c r="K4" s="1"/>
+      <c r="L4" s="1"/>
+      <c r="M4" s="1"/>
+      <c r="N4" s="1"/>
+      <c r="O4" s="1"/>
+      <c r="P4" s="1"/>
+      <c r="Q4" s="1"/>
+      <c r="R4" s="1"/>
+      <c r="S4" s="1"/>
+      <c r="T4" s="1"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Added Validation And Calculation In Direct PO Test Scenarios
Added Validation And Calculation In Direct PO Test Scenarios
</commit_message>
<xml_diff>
--- a/testdata/ItemDetails.xlsx
+++ b/testdata/ItemDetails.xlsx
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="77" uniqueCount="44">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="100" uniqueCount="53">
   <si>
     <t>ITEM_NAME</t>
   </si>
@@ -160,6 +160,33 @@
   </si>
   <si>
     <t>User Defined Price</t>
+  </si>
+  <si>
+    <t>GWL_SERVICES_02_DESCRIPTION</t>
+  </si>
+  <si>
+    <t>GENERAL EXPENSE</t>
+  </si>
+  <si>
+    <t>GWL_CHECKING_ST</t>
+  </si>
+  <si>
+    <t>BICYCLES VARIANTS</t>
+  </si>
+  <si>
+    <t>TWO WHEELER - AUTOMOBILES</t>
+  </si>
+  <si>
+    <t>AURANGABAD DEPOT</t>
+  </si>
+  <si>
+    <t>INVENTORY - FG</t>
+  </si>
+  <si>
+    <t>U2L1L2L3L4L5L601</t>
+  </si>
+  <si>
+    <t>GENERAL U2</t>
   </si>
 </sst>
 </file>
@@ -834,7 +861,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -845,6 +872,9 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="49" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -1410,322 +1440,322 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10">
-      <c r="A1" s="5" t="s">
+      <c r="A1" s="6" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="5" t="s">
+      <c r="B1" s="6" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="5" t="s">
+      <c r="C1" s="6" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="5" t="s">
+      <c r="D1" s="6" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="5" t="s">
+      <c r="E1" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="5" t="s">
+      <c r="F1" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="5" t="s">
+      <c r="G1" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="5" t="s">
+      <c r="H1" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="5" t="s">
+      <c r="I1" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="5" t="s">
+      <c r="J1" s="6" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="2" s="4" customFormat="1" ht="20.4" spans="1:10">
-      <c r="A2" s="6" t="s">
+    <row r="2" s="5" customFormat="1" ht="20.4" spans="1:10">
+      <c r="A2" s="7" t="s">
         <v>10</v>
       </c>
-      <c r="B2" s="7" t="s">
+      <c r="B2" s="8" t="s">
         <v>11</v>
       </c>
-      <c r="C2" s="7" t="s">
+      <c r="C2" s="8" t="s">
         <v>12</v>
       </c>
-      <c r="D2" s="6" t="s">
+      <c r="D2" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="E2" s="6">
+      <c r="E2" s="7">
         <v>1</v>
       </c>
-      <c r="F2" s="6" t="s">
+      <c r="F2" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="G2" s="6">
+      <c r="G2" s="7">
         <v>1010301033</v>
       </c>
-      <c r="H2" s="6" t="s">
+      <c r="H2" s="7" t="s">
         <v>15</v>
       </c>
-      <c r="I2" s="6" t="s">
+      <c r="I2" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="J2" s="6" t="s">
+      <c r="J2" s="7" t="s">
         <v>17</v>
       </c>
     </row>
     <row r="3" ht="15" customHeight="1" spans="1:10">
-      <c r="A3" s="6" t="s">
+      <c r="A3" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="B3" s="7" t="s">
+      <c r="B3" s="8" t="s">
         <v>11</v>
       </c>
-      <c r="C3" s="7" t="s">
+      <c r="C3" s="8" t="s">
         <v>12</v>
       </c>
-      <c r="D3" s="6" t="s">
+      <c r="D3" s="7" t="s">
         <v>19</v>
       </c>
-      <c r="E3" s="6">
+      <c r="E3" s="7">
         <v>6</v>
       </c>
-      <c r="F3" s="7" t="s">
+      <c r="F3" s="8" t="s">
         <v>20</v>
       </c>
-      <c r="G3" s="6">
+      <c r="G3" s="7">
         <v>1010301033</v>
       </c>
-      <c r="H3" s="6" t="s">
+      <c r="H3" s="7" t="s">
         <v>15</v>
       </c>
-      <c r="I3" s="6" t="s">
+      <c r="I3" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="J3" s="6" t="s">
+      <c r="J3" s="7" t="s">
         <v>17</v>
       </c>
     </row>
     <row r="4" spans="1:10">
-      <c r="A4" s="6" t="s">
+      <c r="A4" s="7" t="s">
         <v>21</v>
       </c>
-      <c r="B4" s="7" t="s">
+      <c r="B4" s="8" t="s">
         <v>22</v>
       </c>
-      <c r="C4" s="7" t="s">
+      <c r="C4" s="8" t="s">
         <v>22</v>
       </c>
-      <c r="D4" s="6" t="s">
+      <c r="D4" s="7" t="s">
         <v>23</v>
       </c>
-      <c r="E4" s="6">
+      <c r="E4" s="7">
         <v>1</v>
       </c>
-      <c r="F4" s="7" t="s">
+      <c r="F4" s="8" t="s">
         <v>14</v>
       </c>
-      <c r="G4" s="6">
+      <c r="G4" s="7">
         <v>1000000001</v>
       </c>
-      <c r="H4" s="6"/>
-      <c r="I4" s="6" t="s">
+      <c r="H4" s="7"/>
+      <c r="I4" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="J4" s="6" t="s">
+      <c r="J4" s="7" t="s">
         <v>17</v>
       </c>
     </row>
     <row r="5" spans="1:10">
-      <c r="A5" s="8"/>
-      <c r="B5" s="8"/>
-      <c r="C5" s="8"/>
-      <c r="D5" s="8"/>
-      <c r="E5" s="8"/>
-      <c r="F5" s="8"/>
-      <c r="G5" s="8"/>
-      <c r="H5" s="8"/>
-      <c r="I5" s="8"/>
-      <c r="J5" s="8"/>
+      <c r="A5" s="9"/>
+      <c r="B5" s="9"/>
+      <c r="C5" s="9"/>
+      <c r="D5" s="9"/>
+      <c r="E5" s="9"/>
+      <c r="F5" s="9"/>
+      <c r="G5" s="9"/>
+      <c r="H5" s="9"/>
+      <c r="I5" s="9"/>
+      <c r="J5" s="9"/>
     </row>
     <row r="6" spans="1:10">
-      <c r="A6" s="8"/>
-      <c r="B6" s="8"/>
-      <c r="C6" s="8"/>
-      <c r="D6" s="8"/>
-      <c r="E6" s="8"/>
-      <c r="F6" s="8"/>
-      <c r="G6" s="8"/>
-      <c r="H6" s="8"/>
-      <c r="I6" s="8"/>
-      <c r="J6" s="8"/>
+      <c r="A6" s="9"/>
+      <c r="B6" s="9"/>
+      <c r="C6" s="9"/>
+      <c r="D6" s="9"/>
+      <c r="E6" s="9"/>
+      <c r="F6" s="9"/>
+      <c r="G6" s="9"/>
+      <c r="H6" s="9"/>
+      <c r="I6" s="9"/>
+      <c r="J6" s="9"/>
     </row>
     <row r="7" spans="1:10">
-      <c r="A7" s="8"/>
-      <c r="B7" s="8"/>
-      <c r="C7" s="8"/>
-      <c r="D7" s="8"/>
-      <c r="E7" s="8"/>
-      <c r="F7" s="8"/>
-      <c r="G7" s="8"/>
-      <c r="H7" s="8"/>
-      <c r="I7" s="8"/>
-      <c r="J7" s="8"/>
+      <c r="A7" s="9"/>
+      <c r="B7" s="9"/>
+      <c r="C7" s="9"/>
+      <c r="D7" s="9"/>
+      <c r="E7" s="9"/>
+      <c r="F7" s="9"/>
+      <c r="G7" s="9"/>
+      <c r="H7" s="9"/>
+      <c r="I7" s="9"/>
+      <c r="J7" s="9"/>
     </row>
     <row r="8" spans="1:10">
-      <c r="A8" s="8"/>
-      <c r="B8" s="8"/>
-      <c r="C8" s="8"/>
-      <c r="D8" s="8"/>
-      <c r="E8" s="8"/>
-      <c r="F8" s="8"/>
-      <c r="G8" s="8"/>
-      <c r="H8" s="8"/>
-      <c r="I8" s="8"/>
-      <c r="J8" s="8"/>
+      <c r="A8" s="9"/>
+      <c r="B8" s="9"/>
+      <c r="C8" s="9"/>
+      <c r="D8" s="9"/>
+      <c r="E8" s="9"/>
+      <c r="F8" s="9"/>
+      <c r="G8" s="9"/>
+      <c r="H8" s="9"/>
+      <c r="I8" s="9"/>
+      <c r="J8" s="9"/>
     </row>
     <row r="9" spans="1:10">
-      <c r="A9" s="8"/>
-      <c r="B9" s="8"/>
-      <c r="C9" s="8"/>
-      <c r="D9" s="8"/>
-      <c r="E9" s="8"/>
-      <c r="F9" s="8"/>
-      <c r="G9" s="8"/>
-      <c r="H9" s="8"/>
-      <c r="I9" s="8"/>
-      <c r="J9" s="8"/>
+      <c r="A9" s="9"/>
+      <c r="B9" s="9"/>
+      <c r="C9" s="9"/>
+      <c r="D9" s="9"/>
+      <c r="E9" s="9"/>
+      <c r="F9" s="9"/>
+      <c r="G9" s="9"/>
+      <c r="H9" s="9"/>
+      <c r="I9" s="9"/>
+      <c r="J9" s="9"/>
     </row>
     <row r="10" spans="1:10">
-      <c r="A10" s="8"/>
-      <c r="B10" s="8"/>
-      <c r="C10" s="8"/>
-      <c r="D10" s="8"/>
-      <c r="E10" s="8"/>
-      <c r="F10" s="8"/>
-      <c r="G10" s="8"/>
-      <c r="H10" s="8"/>
-      <c r="I10" s="8"/>
-      <c r="J10" s="8"/>
+      <c r="A10" s="9"/>
+      <c r="B10" s="9"/>
+      <c r="C10" s="9"/>
+      <c r="D10" s="9"/>
+      <c r="E10" s="9"/>
+      <c r="F10" s="9"/>
+      <c r="G10" s="9"/>
+      <c r="H10" s="9"/>
+      <c r="I10" s="9"/>
+      <c r="J10" s="9"/>
     </row>
     <row r="11" spans="1:10">
-      <c r="A11" s="8"/>
-      <c r="B11" s="8"/>
-      <c r="C11" s="8"/>
-      <c r="D11" s="8"/>
-      <c r="E11" s="8"/>
-      <c r="F11" s="8"/>
-      <c r="G11" s="8"/>
-      <c r="H11" s="8"/>
-      <c r="I11" s="8"/>
-      <c r="J11" s="8"/>
+      <c r="A11" s="9"/>
+      <c r="B11" s="9"/>
+      <c r="C11" s="9"/>
+      <c r="D11" s="9"/>
+      <c r="E11" s="9"/>
+      <c r="F11" s="9"/>
+      <c r="G11" s="9"/>
+      <c r="H11" s="9"/>
+      <c r="I11" s="9"/>
+      <c r="J11" s="9"/>
     </row>
     <row r="12" spans="1:10">
-      <c r="A12" s="8"/>
-      <c r="B12" s="8"/>
-      <c r="C12" s="8"/>
-      <c r="D12" s="8"/>
-      <c r="E12" s="8"/>
-      <c r="F12" s="8"/>
-      <c r="G12" s="8"/>
-      <c r="H12" s="8"/>
-      <c r="I12" s="8"/>
-      <c r="J12" s="8"/>
+      <c r="A12" s="9"/>
+      <c r="B12" s="9"/>
+      <c r="C12" s="9"/>
+      <c r="D12" s="9"/>
+      <c r="E12" s="9"/>
+      <c r="F12" s="9"/>
+      <c r="G12" s="9"/>
+      <c r="H12" s="9"/>
+      <c r="I12" s="9"/>
+      <c r="J12" s="9"/>
     </row>
     <row r="13" spans="1:10">
-      <c r="A13" s="8"/>
-      <c r="B13" s="8"/>
-      <c r="C13" s="8"/>
-      <c r="D13" s="8"/>
-      <c r="E13" s="8"/>
-      <c r="F13" s="8"/>
-      <c r="G13" s="8"/>
-      <c r="H13" s="8"/>
-      <c r="I13" s="8"/>
-      <c r="J13" s="8"/>
+      <c r="A13" s="9"/>
+      <c r="B13" s="9"/>
+      <c r="C13" s="9"/>
+      <c r="D13" s="9"/>
+      <c r="E13" s="9"/>
+      <c r="F13" s="9"/>
+      <c r="G13" s="9"/>
+      <c r="H13" s="9"/>
+      <c r="I13" s="9"/>
+      <c r="J13" s="9"/>
     </row>
     <row r="14" spans="1:10">
-      <c r="A14" s="8"/>
-      <c r="B14" s="8"/>
-      <c r="C14" s="8"/>
-      <c r="D14" s="8"/>
-      <c r="E14" s="8"/>
-      <c r="F14" s="8"/>
-      <c r="G14" s="8"/>
-      <c r="H14" s="8"/>
-      <c r="I14" s="8"/>
-      <c r="J14" s="8"/>
+      <c r="A14" s="9"/>
+      <c r="B14" s="9"/>
+      <c r="C14" s="9"/>
+      <c r="D14" s="9"/>
+      <c r="E14" s="9"/>
+      <c r="F14" s="9"/>
+      <c r="G14" s="9"/>
+      <c r="H14" s="9"/>
+      <c r="I14" s="9"/>
+      <c r="J14" s="9"/>
     </row>
     <row r="15" spans="1:10">
-      <c r="A15" s="8"/>
-      <c r="B15" s="8"/>
-      <c r="C15" s="8"/>
-      <c r="D15" s="8"/>
-      <c r="E15" s="8"/>
-      <c r="F15" s="8"/>
-      <c r="G15" s="8"/>
-      <c r="H15" s="8"/>
-      <c r="I15" s="8"/>
-      <c r="J15" s="8"/>
+      <c r="A15" s="9"/>
+      <c r="B15" s="9"/>
+      <c r="C15" s="9"/>
+      <c r="D15" s="9"/>
+      <c r="E15" s="9"/>
+      <c r="F15" s="9"/>
+      <c r="G15" s="9"/>
+      <c r="H15" s="9"/>
+      <c r="I15" s="9"/>
+      <c r="J15" s="9"/>
     </row>
     <row r="16" spans="1:10">
-      <c r="A16" s="8"/>
-      <c r="B16" s="8"/>
-      <c r="C16" s="8"/>
-      <c r="D16" s="8"/>
-      <c r="E16" s="8"/>
-      <c r="F16" s="8"/>
-      <c r="G16" s="8"/>
-      <c r="H16" s="8"/>
-      <c r="I16" s="8"/>
-      <c r="J16" s="8"/>
+      <c r="A16" s="9"/>
+      <c r="B16" s="9"/>
+      <c r="C16" s="9"/>
+      <c r="D16" s="9"/>
+      <c r="E16" s="9"/>
+      <c r="F16" s="9"/>
+      <c r="G16" s="9"/>
+      <c r="H16" s="9"/>
+      <c r="I16" s="9"/>
+      <c r="J16" s="9"/>
     </row>
     <row r="17" spans="1:10">
-      <c r="A17" s="8"/>
-      <c r="B17" s="8"/>
-      <c r="C17" s="8"/>
-      <c r="D17" s="8"/>
-      <c r="E17" s="8"/>
-      <c r="F17" s="8"/>
-      <c r="G17" s="8"/>
-      <c r="H17" s="8"/>
-      <c r="I17" s="8"/>
-      <c r="J17" s="8"/>
+      <c r="A17" s="9"/>
+      <c r="B17" s="9"/>
+      <c r="C17" s="9"/>
+      <c r="D17" s="9"/>
+      <c r="E17" s="9"/>
+      <c r="F17" s="9"/>
+      <c r="G17" s="9"/>
+      <c r="H17" s="9"/>
+      <c r="I17" s="9"/>
+      <c r="J17" s="9"/>
     </row>
     <row r="18" spans="1:10">
-      <c r="A18" s="8"/>
-      <c r="B18" s="8"/>
-      <c r="C18" s="8"/>
-      <c r="D18" s="8"/>
-      <c r="E18" s="8"/>
-      <c r="F18" s="8"/>
-      <c r="G18" s="8"/>
-      <c r="H18" s="8"/>
-      <c r="I18" s="8"/>
-      <c r="J18" s="8"/>
+      <c r="A18" s="9"/>
+      <c r="B18" s="9"/>
+      <c r="C18" s="9"/>
+      <c r="D18" s="9"/>
+      <c r="E18" s="9"/>
+      <c r="F18" s="9"/>
+      <c r="G18" s="9"/>
+      <c r="H18" s="9"/>
+      <c r="I18" s="9"/>
+      <c r="J18" s="9"/>
     </row>
     <row r="19" spans="1:10">
-      <c r="A19" s="8"/>
-      <c r="B19" s="8"/>
-      <c r="C19" s="8"/>
-      <c r="D19" s="8"/>
-      <c r="E19" s="8"/>
-      <c r="F19" s="8"/>
-      <c r="G19" s="8"/>
-      <c r="H19" s="8"/>
-      <c r="I19" s="8"/>
-      <c r="J19" s="8"/>
+      <c r="A19" s="9"/>
+      <c r="B19" s="9"/>
+      <c r="C19" s="9"/>
+      <c r="D19" s="9"/>
+      <c r="E19" s="9"/>
+      <c r="F19" s="9"/>
+      <c r="G19" s="9"/>
+      <c r="H19" s="9"/>
+      <c r="I19" s="9"/>
+      <c r="J19" s="9"/>
     </row>
     <row r="20" spans="1:10">
-      <c r="A20" s="8"/>
-      <c r="B20" s="8"/>
-      <c r="C20" s="8"/>
-      <c r="D20" s="8"/>
-      <c r="E20" s="8"/>
-      <c r="F20" s="8"/>
-      <c r="G20" s="8"/>
-      <c r="H20" s="8"/>
-      <c r="I20" s="8"/>
-      <c r="J20" s="8"/>
+      <c r="A20" s="9"/>
+      <c r="B20" s="9"/>
+      <c r="C20" s="9"/>
+      <c r="D20" s="9"/>
+      <c r="E20" s="9"/>
+      <c r="F20" s="9"/>
+      <c r="G20" s="9"/>
+      <c r="H20" s="9"/>
+      <c r="I20" s="9"/>
+      <c r="J20" s="9"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1736,8 +1766,8 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:T4"/>
-  <sheetFormatPr defaultColWidth="8.73148148148148" defaultRowHeight="14.4" outlineLevelRow="3"/>
+  <dimension ref="A1:T5"/>
+  <sheetFormatPr defaultColWidth="8.73148148148148" defaultRowHeight="14.4" outlineLevelRow="4"/>
   <cols>
     <col min="1" max="1" width="30" customWidth="1"/>
     <col min="2" max="2" width="36.4444444444444" customWidth="1"/>
@@ -1745,14 +1775,14 @@
     <col min="4" max="4" width="13.6666666666667" customWidth="1"/>
     <col min="5" max="5" width="5.22222222222222" customWidth="1"/>
     <col min="6" max="6" width="17.2222222222222" customWidth="1"/>
-    <col min="7" max="7" width="16.1111111111111" customWidth="1"/>
+    <col min="7" max="7" width="30.2222222222222" customWidth="1"/>
     <col min="8" max="8" width="26.8888888888889" customWidth="1"/>
     <col min="9" max="9" width="17.2222222222222" customWidth="1"/>
     <col min="10" max="10" width="13.2222222222222" customWidth="1"/>
     <col min="11" max="11" width="22.7777777777778" customWidth="1"/>
     <col min="12" max="12" width="12.7777777777778" customWidth="1"/>
     <col min="13" max="13" width="17.5555555555556" customWidth="1"/>
-    <col min="14" max="14" width="15.5555555555556" customWidth="1"/>
+    <col min="14" max="14" width="18.2222222222222" customWidth="1"/>
     <col min="15" max="15" width="16.2222222222222" customWidth="1"/>
     <col min="16" max="16" width="15.5555555555556" customWidth="1"/>
     <col min="17" max="17" width="17.7777777777778" customWidth="1"/>
@@ -1932,26 +1962,112 @@
       <c r="T3" s="1"/>
     </row>
     <row r="4" spans="1:20">
-      <c r="A4" s="1"/>
-      <c r="B4" s="1"/>
-      <c r="C4" s="1"/>
-      <c r="D4" s="1"/>
-      <c r="E4" s="1"/>
-      <c r="F4" s="1"/>
-      <c r="G4" s="1"/>
-      <c r="H4" s="1"/>
-      <c r="I4" s="1"/>
-      <c r="J4" s="1"/>
-      <c r="K4" s="1"/>
-      <c r="L4" s="1"/>
-      <c r="M4" s="1"/>
-      <c r="N4" s="1"/>
-      <c r="O4" s="1"/>
+      <c r="A4" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="D4" s="1">
+        <v>123562</v>
+      </c>
+      <c r="E4" s="1">
+        <v>18</v>
+      </c>
+      <c r="F4" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="G4" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="H4" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="I4" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="J4" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="K4" s="1">
+        <v>1</v>
+      </c>
+      <c r="L4" s="1">
+        <v>1000000792</v>
+      </c>
+      <c r="M4" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="N4" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="O4" s="1" t="s">
+        <v>17</v>
+      </c>
       <c r="P4" s="1"/>
       <c r="Q4" s="1"/>
       <c r="R4" s="1"/>
-      <c r="S4" s="1"/>
+      <c r="S4" s="1">
+        <v>0</v>
+      </c>
       <c r="T4" s="1"/>
+    </row>
+    <row r="5" spans="1:20">
+      <c r="A5" s="4" t="s">
+        <v>46</v>
+      </c>
+      <c r="B5" s="4" t="s">
+        <v>46</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="D5" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="E5" s="4">
+        <v>12</v>
+      </c>
+      <c r="F5" s="4" t="s">
+        <v>47</v>
+      </c>
+      <c r="G5" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="H5" s="4" t="s">
+        <v>49</v>
+      </c>
+      <c r="I5" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="J5" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="K5" s="4">
+        <v>1</v>
+      </c>
+      <c r="L5" s="4">
+        <v>1010301001</v>
+      </c>
+      <c r="M5" s="4" t="s">
+        <v>50</v>
+      </c>
+      <c r="N5" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="O5" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="P5" s="4"/>
+      <c r="Q5" s="4"/>
+      <c r="R5" s="4"/>
+      <c r="S5" s="1">
+        <v>0</v>
+      </c>
+      <c r="T5" s="4"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Updated PO Amendment Test Scenarios
Updated PO Amendment Test Scenarios (General And Material)
</commit_message>
<xml_diff>
--- a/testdata/ItemDetails.xlsx
+++ b/testdata/ItemDetails.xlsx
@@ -4,11 +4,12 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="23040" windowHeight="9120" activeTab="1"/>
+    <workbookView windowWidth="23040" windowHeight="9120" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="PR Details" sheetId="1" r:id="rId1"/>
     <sheet name="PO Details" sheetId="2" r:id="rId2"/>
+    <sheet name="POA Details" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -28,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="100" uniqueCount="53">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="134" uniqueCount="55">
   <si>
     <t>ITEM_NAME</t>
   </si>
@@ -187,6 +188,12 @@
   </si>
   <si>
     <t>GENERAL U2</t>
+  </si>
+  <si>
+    <t>GWL_Item_Similar_02</t>
+  </si>
+  <si>
+    <t>SUPL_UOM</t>
   </si>
 </sst>
 </file>
@@ -199,7 +206,7 @@
     <numFmt numFmtId="178" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
     <numFmt numFmtId="179" formatCode="_ &quot;₹&quot;* #,##0_ ;_ &quot;₹&quot;* \-#,##0_ ;_ &quot;₹&quot;* &quot;-&quot;_ ;_ @_ "/>
   </numFmts>
-  <fonts count="26">
+  <fonts count="27">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -217,6 +224,12 @@
       <sz val="10"/>
       <color rgb="FF262626"/>
       <name val="Times New Roman"/>
+      <charset val="134"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color rgb="FF262626"/>
+      <name val="Arial"/>
       <charset val="134"/>
     </font>
     <font>
@@ -731,165 +744,171 @@
     <xf numFmtId="179" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="2" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="4" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="5" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="5" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="6" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="4" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="5" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="5" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="6" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="49" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="justify" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -1440,322 +1459,322 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10">
-      <c r="A1" s="6" t="s">
+      <c r="A1" s="8" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="6" t="s">
+      <c r="B1" s="8" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="6" t="s">
+      <c r="C1" s="8" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="6" t="s">
+      <c r="D1" s="8" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="6" t="s">
+      <c r="E1" s="8" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="6" t="s">
+      <c r="F1" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="6" t="s">
+      <c r="G1" s="8" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="6" t="s">
+      <c r="H1" s="8" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="6" t="s">
+      <c r="I1" s="8" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="6" t="s">
+      <c r="J1" s="8" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="2" s="5" customFormat="1" ht="20.4" spans="1:10">
-      <c r="A2" s="7" t="s">
+    <row r="2" s="7" customFormat="1" ht="20.4" spans="1:10">
+      <c r="A2" s="9" t="s">
         <v>10</v>
       </c>
-      <c r="B2" s="8" t="s">
+      <c r="B2" s="10" t="s">
         <v>11</v>
       </c>
-      <c r="C2" s="8" t="s">
+      <c r="C2" s="10" t="s">
         <v>12</v>
       </c>
-      <c r="D2" s="7" t="s">
+      <c r="D2" s="9" t="s">
         <v>13</v>
       </c>
-      <c r="E2" s="7">
+      <c r="E2" s="9">
         <v>1</v>
       </c>
-      <c r="F2" s="7" t="s">
+      <c r="F2" s="9" t="s">
         <v>14</v>
       </c>
-      <c r="G2" s="7">
+      <c r="G2" s="9">
         <v>1010301033</v>
       </c>
-      <c r="H2" s="7" t="s">
+      <c r="H2" s="9" t="s">
         <v>15</v>
       </c>
-      <c r="I2" s="7" t="s">
+      <c r="I2" s="9" t="s">
         <v>16</v>
       </c>
-      <c r="J2" s="7" t="s">
+      <c r="J2" s="9" t="s">
         <v>17</v>
       </c>
     </row>
     <row r="3" ht="15" customHeight="1" spans="1:10">
-      <c r="A3" s="7" t="s">
+      <c r="A3" s="9" t="s">
         <v>18</v>
       </c>
-      <c r="B3" s="8" t="s">
+      <c r="B3" s="10" t="s">
         <v>11</v>
       </c>
-      <c r="C3" s="8" t="s">
+      <c r="C3" s="10" t="s">
         <v>12</v>
       </c>
-      <c r="D3" s="7" t="s">
+      <c r="D3" s="9" t="s">
         <v>19</v>
       </c>
-      <c r="E3" s="7">
+      <c r="E3" s="9">
         <v>6</v>
       </c>
-      <c r="F3" s="8" t="s">
+      <c r="F3" s="10" t="s">
         <v>20</v>
       </c>
-      <c r="G3" s="7">
+      <c r="G3" s="9">
         <v>1010301033</v>
       </c>
-      <c r="H3" s="7" t="s">
+      <c r="H3" s="9" t="s">
         <v>15</v>
       </c>
-      <c r="I3" s="7" t="s">
+      <c r="I3" s="9" t="s">
         <v>16</v>
       </c>
-      <c r="J3" s="7" t="s">
+      <c r="J3" s="9" t="s">
         <v>17</v>
       </c>
     </row>
     <row r="4" spans="1:10">
-      <c r="A4" s="7" t="s">
+      <c r="A4" s="9" t="s">
         <v>21</v>
       </c>
-      <c r="B4" s="8" t="s">
+      <c r="B4" s="10" t="s">
         <v>22</v>
       </c>
-      <c r="C4" s="8" t="s">
+      <c r="C4" s="10" t="s">
         <v>22</v>
       </c>
-      <c r="D4" s="7" t="s">
+      <c r="D4" s="9" t="s">
         <v>23</v>
       </c>
-      <c r="E4" s="7">
+      <c r="E4" s="9">
         <v>1</v>
       </c>
-      <c r="F4" s="8" t="s">
+      <c r="F4" s="10" t="s">
         <v>14</v>
       </c>
-      <c r="G4" s="7">
+      <c r="G4" s="9">
         <v>1000000001</v>
       </c>
-      <c r="H4" s="7"/>
-      <c r="I4" s="7" t="s">
+      <c r="H4" s="9"/>
+      <c r="I4" s="9" t="s">
         <v>16</v>
       </c>
-      <c r="J4" s="7" t="s">
+      <c r="J4" s="9" t="s">
         <v>17</v>
       </c>
     </row>
     <row r="5" spans="1:10">
-      <c r="A5" s="9"/>
-      <c r="B5" s="9"/>
-      <c r="C5" s="9"/>
-      <c r="D5" s="9"/>
-      <c r="E5" s="9"/>
-      <c r="F5" s="9"/>
-      <c r="G5" s="9"/>
-      <c r="H5" s="9"/>
-      <c r="I5" s="9"/>
-      <c r="J5" s="9"/>
+      <c r="A5" s="11"/>
+      <c r="B5" s="11"/>
+      <c r="C5" s="11"/>
+      <c r="D5" s="11"/>
+      <c r="E5" s="11"/>
+      <c r="F5" s="11"/>
+      <c r="G5" s="11"/>
+      <c r="H5" s="11"/>
+      <c r="I5" s="11"/>
+      <c r="J5" s="11"/>
     </row>
     <row r="6" spans="1:10">
-      <c r="A6" s="9"/>
-      <c r="B6" s="9"/>
-      <c r="C6" s="9"/>
-      <c r="D6" s="9"/>
-      <c r="E6" s="9"/>
-      <c r="F6" s="9"/>
-      <c r="G6" s="9"/>
-      <c r="H6" s="9"/>
-      <c r="I6" s="9"/>
-      <c r="J6" s="9"/>
+      <c r="A6" s="11"/>
+      <c r="B6" s="11"/>
+      <c r="C6" s="11"/>
+      <c r="D6" s="11"/>
+      <c r="E6" s="11"/>
+      <c r="F6" s="11"/>
+      <c r="G6" s="11"/>
+      <c r="H6" s="11"/>
+      <c r="I6" s="11"/>
+      <c r="J6" s="11"/>
     </row>
     <row r="7" spans="1:10">
-      <c r="A7" s="9"/>
-      <c r="B7" s="9"/>
-      <c r="C7" s="9"/>
-      <c r="D7" s="9"/>
-      <c r="E7" s="9"/>
-      <c r="F7" s="9"/>
-      <c r="G7" s="9"/>
-      <c r="H7" s="9"/>
-      <c r="I7" s="9"/>
-      <c r="J7" s="9"/>
+      <c r="A7" s="11"/>
+      <c r="B7" s="11"/>
+      <c r="C7" s="11"/>
+      <c r="D7" s="11"/>
+      <c r="E7" s="11"/>
+      <c r="F7" s="11"/>
+      <c r="G7" s="11"/>
+      <c r="H7" s="11"/>
+      <c r="I7" s="11"/>
+      <c r="J7" s="11"/>
     </row>
     <row r="8" spans="1:10">
-      <c r="A8" s="9"/>
-      <c r="B8" s="9"/>
-      <c r="C8" s="9"/>
-      <c r="D8" s="9"/>
-      <c r="E8" s="9"/>
-      <c r="F8" s="9"/>
-      <c r="G8" s="9"/>
-      <c r="H8" s="9"/>
-      <c r="I8" s="9"/>
-      <c r="J8" s="9"/>
+      <c r="A8" s="11"/>
+      <c r="B8" s="11"/>
+      <c r="C8" s="11"/>
+      <c r="D8" s="11"/>
+      <c r="E8" s="11"/>
+      <c r="F8" s="11"/>
+      <c r="G8" s="11"/>
+      <c r="H8" s="11"/>
+      <c r="I8" s="11"/>
+      <c r="J8" s="11"/>
     </row>
     <row r="9" spans="1:10">
-      <c r="A9" s="9"/>
-      <c r="B9" s="9"/>
-      <c r="C9" s="9"/>
-      <c r="D9" s="9"/>
-      <c r="E9" s="9"/>
-      <c r="F9" s="9"/>
-      <c r="G9" s="9"/>
-      <c r="H9" s="9"/>
-      <c r="I9" s="9"/>
-      <c r="J9" s="9"/>
+      <c r="A9" s="11"/>
+      <c r="B9" s="11"/>
+      <c r="C9" s="11"/>
+      <c r="D9" s="11"/>
+      <c r="E9" s="11"/>
+      <c r="F9" s="11"/>
+      <c r="G9" s="11"/>
+      <c r="H9" s="11"/>
+      <c r="I9" s="11"/>
+      <c r="J9" s="11"/>
     </row>
     <row r="10" spans="1:10">
-      <c r="A10" s="9"/>
-      <c r="B10" s="9"/>
-      <c r="C10" s="9"/>
-      <c r="D10" s="9"/>
-      <c r="E10" s="9"/>
-      <c r="F10" s="9"/>
-      <c r="G10" s="9"/>
-      <c r="H10" s="9"/>
-      <c r="I10" s="9"/>
-      <c r="J10" s="9"/>
+      <c r="A10" s="11"/>
+      <c r="B10" s="11"/>
+      <c r="C10" s="11"/>
+      <c r="D10" s="11"/>
+      <c r="E10" s="11"/>
+      <c r="F10" s="11"/>
+      <c r="G10" s="11"/>
+      <c r="H10" s="11"/>
+      <c r="I10" s="11"/>
+      <c r="J10" s="11"/>
     </row>
     <row r="11" spans="1:10">
-      <c r="A11" s="9"/>
-      <c r="B11" s="9"/>
-      <c r="C11" s="9"/>
-      <c r="D11" s="9"/>
-      <c r="E11" s="9"/>
-      <c r="F11" s="9"/>
-      <c r="G11" s="9"/>
-      <c r="H11" s="9"/>
-      <c r="I11" s="9"/>
-      <c r="J11" s="9"/>
+      <c r="A11" s="11"/>
+      <c r="B11" s="11"/>
+      <c r="C11" s="11"/>
+      <c r="D11" s="11"/>
+      <c r="E11" s="11"/>
+      <c r="F11" s="11"/>
+      <c r="G11" s="11"/>
+      <c r="H11" s="11"/>
+      <c r="I11" s="11"/>
+      <c r="J11" s="11"/>
     </row>
     <row r="12" spans="1:10">
-      <c r="A12" s="9"/>
-      <c r="B12" s="9"/>
-      <c r="C12" s="9"/>
-      <c r="D12" s="9"/>
-      <c r="E12" s="9"/>
-      <c r="F12" s="9"/>
-      <c r="G12" s="9"/>
-      <c r="H12" s="9"/>
-      <c r="I12" s="9"/>
-      <c r="J12" s="9"/>
+      <c r="A12" s="11"/>
+      <c r="B12" s="11"/>
+      <c r="C12" s="11"/>
+      <c r="D12" s="11"/>
+      <c r="E12" s="11"/>
+      <c r="F12" s="11"/>
+      <c r="G12" s="11"/>
+      <c r="H12" s="11"/>
+      <c r="I12" s="11"/>
+      <c r="J12" s="11"/>
     </row>
     <row r="13" spans="1:10">
-      <c r="A13" s="9"/>
-      <c r="B13" s="9"/>
-      <c r="C13" s="9"/>
-      <c r="D13" s="9"/>
-      <c r="E13" s="9"/>
-      <c r="F13" s="9"/>
-      <c r="G13" s="9"/>
-      <c r="H13" s="9"/>
-      <c r="I13" s="9"/>
-      <c r="J13" s="9"/>
+      <c r="A13" s="11"/>
+      <c r="B13" s="11"/>
+      <c r="C13" s="11"/>
+      <c r="D13" s="11"/>
+      <c r="E13" s="11"/>
+      <c r="F13" s="11"/>
+      <c r="G13" s="11"/>
+      <c r="H13" s="11"/>
+      <c r="I13" s="11"/>
+      <c r="J13" s="11"/>
     </row>
     <row r="14" spans="1:10">
-      <c r="A14" s="9"/>
-      <c r="B14" s="9"/>
-      <c r="C14" s="9"/>
-      <c r="D14" s="9"/>
-      <c r="E14" s="9"/>
-      <c r="F14" s="9"/>
-      <c r="G14" s="9"/>
-      <c r="H14" s="9"/>
-      <c r="I14" s="9"/>
-      <c r="J14" s="9"/>
+      <c r="A14" s="11"/>
+      <c r="B14" s="11"/>
+      <c r="C14" s="11"/>
+      <c r="D14" s="11"/>
+      <c r="E14" s="11"/>
+      <c r="F14" s="11"/>
+      <c r="G14" s="11"/>
+      <c r="H14" s="11"/>
+      <c r="I14" s="11"/>
+      <c r="J14" s="11"/>
     </row>
     <row r="15" spans="1:10">
-      <c r="A15" s="9"/>
-      <c r="B15" s="9"/>
-      <c r="C15" s="9"/>
-      <c r="D15" s="9"/>
-      <c r="E15" s="9"/>
-      <c r="F15" s="9"/>
-      <c r="G15" s="9"/>
-      <c r="H15" s="9"/>
-      <c r="I15" s="9"/>
-      <c r="J15" s="9"/>
+      <c r="A15" s="11"/>
+      <c r="B15" s="11"/>
+      <c r="C15" s="11"/>
+      <c r="D15" s="11"/>
+      <c r="E15" s="11"/>
+      <c r="F15" s="11"/>
+      <c r="G15" s="11"/>
+      <c r="H15" s="11"/>
+      <c r="I15" s="11"/>
+      <c r="J15" s="11"/>
     </row>
     <row r="16" spans="1:10">
-      <c r="A16" s="9"/>
-      <c r="B16" s="9"/>
-      <c r="C16" s="9"/>
-      <c r="D16" s="9"/>
-      <c r="E16" s="9"/>
-      <c r="F16" s="9"/>
-      <c r="G16" s="9"/>
-      <c r="H16" s="9"/>
-      <c r="I16" s="9"/>
-      <c r="J16" s="9"/>
+      <c r="A16" s="11"/>
+      <c r="B16" s="11"/>
+      <c r="C16" s="11"/>
+      <c r="D16" s="11"/>
+      <c r="E16" s="11"/>
+      <c r="F16" s="11"/>
+      <c r="G16" s="11"/>
+      <c r="H16" s="11"/>
+      <c r="I16" s="11"/>
+      <c r="J16" s="11"/>
     </row>
     <row r="17" spans="1:10">
-      <c r="A17" s="9"/>
-      <c r="B17" s="9"/>
-      <c r="C17" s="9"/>
-      <c r="D17" s="9"/>
-      <c r="E17" s="9"/>
-      <c r="F17" s="9"/>
-      <c r="G17" s="9"/>
-      <c r="H17" s="9"/>
-      <c r="I17" s="9"/>
-      <c r="J17" s="9"/>
+      <c r="A17" s="11"/>
+      <c r="B17" s="11"/>
+      <c r="C17" s="11"/>
+      <c r="D17" s="11"/>
+      <c r="E17" s="11"/>
+      <c r="F17" s="11"/>
+      <c r="G17" s="11"/>
+      <c r="H17" s="11"/>
+      <c r="I17" s="11"/>
+      <c r="J17" s="11"/>
     </row>
     <row r="18" spans="1:10">
-      <c r="A18" s="9"/>
-      <c r="B18" s="9"/>
-      <c r="C18" s="9"/>
-      <c r="D18" s="9"/>
-      <c r="E18" s="9"/>
-      <c r="F18" s="9"/>
-      <c r="G18" s="9"/>
-      <c r="H18" s="9"/>
-      <c r="I18" s="9"/>
-      <c r="J18" s="9"/>
+      <c r="A18" s="11"/>
+      <c r="B18" s="11"/>
+      <c r="C18" s="11"/>
+      <c r="D18" s="11"/>
+      <c r="E18" s="11"/>
+      <c r="F18" s="11"/>
+      <c r="G18" s="11"/>
+      <c r="H18" s="11"/>
+      <c r="I18" s="11"/>
+      <c r="J18" s="11"/>
     </row>
     <row r="19" spans="1:10">
-      <c r="A19" s="9"/>
-      <c r="B19" s="9"/>
-      <c r="C19" s="9"/>
-      <c r="D19" s="9"/>
-      <c r="E19" s="9"/>
-      <c r="F19" s="9"/>
-      <c r="G19" s="9"/>
-      <c r="H19" s="9"/>
-      <c r="I19" s="9"/>
-      <c r="J19" s="9"/>
+      <c r="A19" s="11"/>
+      <c r="B19" s="11"/>
+      <c r="C19" s="11"/>
+      <c r="D19" s="11"/>
+      <c r="E19" s="11"/>
+      <c r="F19" s="11"/>
+      <c r="G19" s="11"/>
+      <c r="H19" s="11"/>
+      <c r="I19" s="11"/>
+      <c r="J19" s="11"/>
     </row>
     <row r="20" spans="1:10">
-      <c r="A20" s="9"/>
-      <c r="B20" s="9"/>
-      <c r="C20" s="9"/>
-      <c r="D20" s="9"/>
-      <c r="E20" s="9"/>
-      <c r="F20" s="9"/>
-      <c r="G20" s="9"/>
-      <c r="H20" s="9"/>
-      <c r="I20" s="9"/>
-      <c r="J20" s="9"/>
+      <c r="A20" s="11"/>
+      <c r="B20" s="11"/>
+      <c r="C20" s="11"/>
+      <c r="D20" s="11"/>
+      <c r="E20" s="11"/>
+      <c r="F20" s="11"/>
+      <c r="G20" s="11"/>
+      <c r="H20" s="11"/>
+      <c r="I20" s="11"/>
+      <c r="J20" s="11"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1766,8 +1785,8 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:T5"/>
-  <sheetFormatPr defaultColWidth="8.73148148148148" defaultRowHeight="14.4" outlineLevelRow="4"/>
+  <dimension ref="A1:T6"/>
+  <sheetFormatPr defaultColWidth="8.73148148148148" defaultRowHeight="14.4" outlineLevelRow="5"/>
   <cols>
     <col min="1" max="1" width="30" customWidth="1"/>
     <col min="2" max="2" width="36.4444444444444" customWidth="1"/>
@@ -1792,6 +1811,363 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:20">
+      <c r="A1" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="H1" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="I1" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="J1" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="K1" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="L1" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="M1" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="N1" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="O1" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="P1" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="Q1" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="R1" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="S1" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="T1" s="2" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="2" spans="1:20">
+      <c r="A2" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="E2" s="2">
+        <v>12</v>
+      </c>
+      <c r="F2" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="G2" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="H2" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="I2" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="J2" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="K2" s="2">
+        <v>6</v>
+      </c>
+      <c r="L2" s="2">
+        <v>1010301033</v>
+      </c>
+      <c r="M2" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="N2" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="O2" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="P2" s="2"/>
+      <c r="Q2" s="2"/>
+      <c r="R2" s="2"/>
+      <c r="S2" s="2">
+        <v>0</v>
+      </c>
+      <c r="T2" s="2"/>
+    </row>
+    <row r="3" spans="1:20">
+      <c r="A3" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="D3" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="E3" s="2">
+        <v>5</v>
+      </c>
+      <c r="F3" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="G3" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="H3" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="I3" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="J3" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="K3" s="2">
+        <v>1</v>
+      </c>
+      <c r="L3" s="2">
+        <v>1010301033</v>
+      </c>
+      <c r="M3" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="N3" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="O3" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="P3" s="2"/>
+      <c r="Q3" s="2"/>
+      <c r="R3" s="2"/>
+      <c r="S3" s="2">
+        <v>0</v>
+      </c>
+      <c r="T3" s="2"/>
+    </row>
+    <row r="4" spans="1:20">
+      <c r="A4" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="D4" s="2">
+        <v>123562</v>
+      </c>
+      <c r="E4" s="2">
+        <v>18</v>
+      </c>
+      <c r="F4" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="G4" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="H4" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="I4" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="J4" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="K4" s="2">
+        <v>1</v>
+      </c>
+      <c r="L4" s="2">
+        <v>1000000792</v>
+      </c>
+      <c r="M4" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="N4" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="O4" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="P4" s="2"/>
+      <c r="Q4" s="2"/>
+      <c r="R4" s="2"/>
+      <c r="S4" s="2">
+        <v>0</v>
+      </c>
+      <c r="T4" s="2"/>
+    </row>
+    <row r="5" spans="1:20">
+      <c r="A5" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="D5" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="E5" s="1">
+        <v>12</v>
+      </c>
+      <c r="F5" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="G5" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="H5" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="I5" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="J5" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="K5" s="1">
+        <v>1</v>
+      </c>
+      <c r="L5" s="1">
+        <v>1010301001</v>
+      </c>
+      <c r="M5" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="N5" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="O5" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="P5" s="1"/>
+      <c r="Q5" s="1"/>
+      <c r="R5" s="1"/>
+      <c r="S5" s="2">
+        <v>0</v>
+      </c>
+      <c r="T5" s="1"/>
+    </row>
+    <row r="6" spans="1:20">
+      <c r="A6" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="D6" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="E6">
+        <v>5</v>
+      </c>
+      <c r="F6" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="G6" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="H6" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="I6" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="J6" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="K6" s="1">
+        <v>1</v>
+      </c>
+      <c r="L6" s="1">
+        <v>1010301033</v>
+      </c>
+      <c r="M6" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="N6" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="O6" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="P6" s="1"/>
+      <c r="Q6" s="1"/>
+      <c r="R6" s="1"/>
+      <c r="S6" s="2">
+        <v>0</v>
+      </c>
+      <c r="T6" s="1"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <headerFooter/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
+  <dimension ref="A1:R2"/>
+  <sheetFormatPr defaultColWidth="8.88888888888889" defaultRowHeight="14.4" outlineLevelRow="1"/>
+  <cols>
+    <col min="1" max="2" width="21" customWidth="1"/>
+    <col min="3" max="3" width="6" customWidth="1"/>
+    <col min="4" max="4" width="12.7777777777778" customWidth="1"/>
+    <col min="5" max="5" width="16.5555555555556" customWidth="1"/>
+    <col min="6" max="6" width="15.1111111111111" customWidth="1"/>
+    <col min="7" max="7" width="15.4444444444444" customWidth="1"/>
+    <col min="8" max="8" width="19.5555555555556" customWidth="1"/>
+    <col min="9" max="9" width="10.8888888888889" customWidth="1"/>
+    <col min="10" max="10" width="17.5555555555556" customWidth="1"/>
+    <col min="11" max="11" width="11.2222222222222" customWidth="1"/>
+    <col min="12" max="12" width="21.6666666666667" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:18">
       <c r="A1" s="1" t="s">
         <v>24</v>
       </c>
@@ -1801,273 +2177,83 @@
       <c r="C1" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="D1" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>1</v>
+      <c r="D1" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>9</v>
       </c>
       <c r="H1" s="1" t="s">
         <v>29</v>
       </c>
       <c r="I1" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="J1" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="J1" s="1" t="s">
-        <v>31</v>
-      </c>
       <c r="K1" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="L1" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="L1" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="M1" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="N1" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="O1" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="P1" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="Q1" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="R1" s="1" t="s">
-        <v>35</v>
-      </c>
-      <c r="S1" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="T1" s="1" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="2" spans="1:20">
+      <c r="M1" s="1"/>
+      <c r="N1" s="1"/>
+      <c r="O1" s="1"/>
+      <c r="P1" s="1"/>
+      <c r="Q1" s="1"/>
+      <c r="R1" s="1"/>
+    </row>
+    <row r="2" spans="1:18">
       <c r="A2" s="1" t="s">
-        <v>18</v>
+        <v>53</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>38</v>
+        <v>53</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="D2" s="1" t="s">
-        <v>39</v>
-      </c>
-      <c r="E2" s="1">
-        <v>12</v>
-      </c>
-      <c r="F2" s="2" t="s">
-        <v>12</v>
+        <v>14</v>
+      </c>
+      <c r="D2" s="1">
+        <v>1010301033</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="F2" s="1" t="s">
+        <v>16</v>
       </c>
       <c r="G2" s="1" t="s">
-        <v>11</v>
+        <v>17</v>
       </c>
       <c r="H2" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="I2" s="1" t="s">
-        <v>40</v>
+      <c r="I2" s="3" t="s">
+        <v>42</v>
       </c>
       <c r="J2" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="K2" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="K2" s="1">
-        <v>6</v>
-      </c>
       <c r="L2" s="1">
-        <v>1010301033</v>
-      </c>
-      <c r="M2" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="N2" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="O2" s="1" t="s">
-        <v>17</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="M2" s="1"/>
+      <c r="N2" s="1"/>
+      <c r="O2" s="1"/>
       <c r="P2" s="1"/>
       <c r="Q2" s="1"/>
       <c r="R2" s="1"/>
-      <c r="S2" s="1">
-        <v>0</v>
-      </c>
-      <c r="T2" s="1"/>
-    </row>
-    <row r="3" spans="1:20">
-      <c r="A3" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="B3" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="C3" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="D3" s="3" t="s">
-        <v>42</v>
-      </c>
-      <c r="E3" s="1">
-        <v>5</v>
-      </c>
-      <c r="F3" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="G3" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="H3" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="I3" s="1" t="s">
-        <v>43</v>
-      </c>
-      <c r="J3" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="K3" s="1">
-        <v>1</v>
-      </c>
-      <c r="L3" s="1">
-        <v>1010301033</v>
-      </c>
-      <c r="M3" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="N3" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="O3" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="P3" s="1"/>
-      <c r="Q3" s="1"/>
-      <c r="R3" s="1"/>
-      <c r="S3" s="1">
-        <v>0</v>
-      </c>
-      <c r="T3" s="1"/>
-    </row>
-    <row r="4" spans="1:20">
-      <c r="A4" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="B4" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="C4" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="D4" s="1">
-        <v>123562</v>
-      </c>
-      <c r="E4" s="1">
-        <v>18</v>
-      </c>
-      <c r="F4" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="G4" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="H4" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="I4" s="1" t="s">
-        <v>43</v>
-      </c>
-      <c r="J4" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="K4" s="1">
-        <v>1</v>
-      </c>
-      <c r="L4" s="1">
-        <v>1000000792</v>
-      </c>
-      <c r="M4" s="1" t="s">
-        <v>45</v>
-      </c>
-      <c r="N4" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="O4" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="P4" s="1"/>
-      <c r="Q4" s="1"/>
-      <c r="R4" s="1"/>
-      <c r="S4" s="1">
-        <v>0</v>
-      </c>
-      <c r="T4" s="1"/>
-    </row>
-    <row r="5" spans="1:20">
-      <c r="A5" s="4" t="s">
-        <v>46</v>
-      </c>
-      <c r="B5" s="4" t="s">
-        <v>46</v>
-      </c>
-      <c r="C5" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="D5" s="4" t="s">
-        <v>39</v>
-      </c>
-      <c r="E5" s="4">
-        <v>12</v>
-      </c>
-      <c r="F5" s="4" t="s">
-        <v>47</v>
-      </c>
-      <c r="G5" s="4" t="s">
-        <v>48</v>
-      </c>
-      <c r="H5" s="4" t="s">
-        <v>49</v>
-      </c>
-      <c r="I5" s="4" t="s">
-        <v>43</v>
-      </c>
-      <c r="J5" s="4" t="s">
-        <v>14</v>
-      </c>
-      <c r="K5" s="4">
-        <v>1</v>
-      </c>
-      <c r="L5" s="4">
-        <v>1010301001</v>
-      </c>
-      <c r="M5" s="4" t="s">
-        <v>50</v>
-      </c>
-      <c r="N5" s="4" t="s">
-        <v>51</v>
-      </c>
-      <c r="O5" s="4" t="s">
-        <v>52</v>
-      </c>
-      <c r="P5" s="4"/>
-      <c r="Q5" s="4"/>
-      <c r="R5" s="4"/>
-      <c r="S5" s="1">
-        <v>0</v>
-      </c>
-      <c r="T5" s="4"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Updated Open So, PriceList, Po Amendment Test Scenarios
Updated Open So, PriceList, Po Amendment Test Scenarios
</commit_message>
<xml_diff>
--- a/testdata/ItemDetails.xlsx
+++ b/testdata/ItemDetails.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="23040" windowHeight="9120" activeTab="2"/>
+    <workbookView windowWidth="23040" windowHeight="9120"/>
   </bookViews>
   <sheets>
     <sheet name="PR Details" sheetId="1" r:id="rId1"/>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="134" uniqueCount="55">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="193" uniqueCount="66">
   <si>
     <t>ITEM_NAME</t>
   </si>
@@ -103,6 +103,9 @@
     <t>PRODUCTION  100</t>
   </si>
   <si>
+    <t>CUSTOMS DUTY - RM</t>
+  </si>
+  <si>
     <t>ITEMID</t>
   </si>
   <si>
@@ -166,7 +169,7 @@
     <t>GWL_SERVICES_02_DESCRIPTION</t>
   </si>
   <si>
-    <t>GENERAL EXPENSE</t>
+    <t>EXPENSE DOCUMENT 3</t>
   </si>
   <si>
     <t>GWL_CHECKING_ST</t>
@@ -191,6 +194,37 @@
   </si>
   <si>
     <t>GWL_Item_Similar_02</t>
+  </si>
+  <si>
+    <t xml:space="preserve">HK-NA-MAC-10001
+</t>
+  </si>
+  <si>
+    <t>HK-NOTAPPLICABLE-MAC-10001</t>
+  </si>
+  <si>
+    <t>RAW MATERIAL WH U100</t>
+  </si>
+  <si>
+    <t>INVENTORY - RAW MATERIAL</t>
+  </si>
+  <si>
+    <t>HK-FIFO-SER-BATCH-10001</t>
+  </si>
+  <si>
+    <t>HK-FIFO-SERIAL-BATCH-10001</t>
+  </si>
+  <si>
+    <t>HK-LOT-FIFO-LOT-10001</t>
+  </si>
+  <si>
+    <t>GWL_ITem_service_03</t>
+  </si>
+  <si>
+    <t>PRODUCTION 100</t>
+  </si>
+  <si>
+    <t>SBI CC 30498311798</t>
   </si>
   <si>
     <t>SUPL_UOM</t>
@@ -221,15 +255,15 @@
       <charset val="134"/>
     </font>
     <font>
+      <sz val="9"/>
+      <color rgb="FF262626"/>
+      <name val="Arial"/>
+      <charset val="134"/>
+    </font>
+    <font>
       <sz val="10"/>
       <color rgb="FF262626"/>
       <name val="Times New Roman"/>
-      <charset val="134"/>
-    </font>
-    <font>
-      <sz val="9"/>
-      <color rgb="FF262626"/>
-      <name val="Arial"/>
       <charset val="134"/>
     </font>
     <font>
@@ -725,7 +759,7 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="49">
+  <cellStyleXfs count="50">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
@@ -873,8 +907,11 @@
     <xf numFmtId="0" fontId="25" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -884,16 +921,28 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="49" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="49" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="49" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -912,7 +961,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
-  <cellStyles count="49">
+  <cellStyles count="50">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Comma" xfId="1" builtinId="3"/>
     <cellStyle name="Currency" xfId="2" builtinId="4"/>
@@ -962,6 +1011,7 @@
     <cellStyle name="20% - Accent6" xfId="46" builtinId="50"/>
     <cellStyle name="40% - Accent6" xfId="47" builtinId="51"/>
     <cellStyle name="60% - Accent6" xfId="48" builtinId="52"/>
+    <cellStyle name="Normal 2" xfId="49"/>
   </cellStyles>
   <dxfs count="17">
     <dxf>
@@ -1453,328 +1503,330 @@
     <col min="5" max="5" width="9.81481481481481" customWidth="1"/>
     <col min="6" max="6" width="14.1851851851852" customWidth="1"/>
     <col min="7" max="7" width="14.8148148148148" customWidth="1"/>
-    <col min="8" max="8" width="13.8148148148148" customWidth="1"/>
+    <col min="8" max="8" width="22.2222222222222" customWidth="1"/>
     <col min="9" max="9" width="14.3611111111111" customWidth="1"/>
     <col min="10" max="10" width="13" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:10">
-      <c r="A1" s="8" t="s">
+      <c r="A1" s="12" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="8" t="s">
+      <c r="B1" s="12" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="8" t="s">
+      <c r="C1" s="12" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="8" t="s">
+      <c r="D1" s="12" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="8" t="s">
+      <c r="E1" s="12" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="8" t="s">
+      <c r="F1" s="12" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="8" t="s">
+      <c r="G1" s="12" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="8" t="s">
+      <c r="H1" s="12" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="8" t="s">
+      <c r="I1" s="12" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="8" t="s">
+      <c r="J1" s="12" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="2" s="7" customFormat="1" ht="20.4" spans="1:10">
-      <c r="A2" s="9" t="s">
+    <row r="2" s="11" customFormat="1" ht="20.4" spans="1:10">
+      <c r="A2" s="13" t="s">
         <v>10</v>
       </c>
-      <c r="B2" s="10" t="s">
+      <c r="B2" s="14" t="s">
         <v>11</v>
       </c>
-      <c r="C2" s="10" t="s">
+      <c r="C2" s="14" t="s">
         <v>12</v>
       </c>
-      <c r="D2" s="9" t="s">
+      <c r="D2" s="13" t="s">
         <v>13</v>
       </c>
-      <c r="E2" s="9">
+      <c r="E2" s="13">
         <v>1</v>
       </c>
-      <c r="F2" s="9" t="s">
+      <c r="F2" s="13" t="s">
         <v>14</v>
       </c>
-      <c r="G2" s="9">
+      <c r="G2" s="13">
         <v>1010301033</v>
       </c>
-      <c r="H2" s="9" t="s">
+      <c r="H2" s="13" t="s">
         <v>15</v>
       </c>
-      <c r="I2" s="9" t="s">
+      <c r="I2" s="13" t="s">
         <v>16</v>
       </c>
-      <c r="J2" s="9" t="s">
+      <c r="J2" s="13" t="s">
         <v>17</v>
       </c>
     </row>
     <row r="3" ht="15" customHeight="1" spans="1:10">
-      <c r="A3" s="9" t="s">
+      <c r="A3" s="13" t="s">
         <v>18</v>
       </c>
-      <c r="B3" s="10" t="s">
+      <c r="B3" s="14" t="s">
         <v>11</v>
       </c>
-      <c r="C3" s="10" t="s">
+      <c r="C3" s="14" t="s">
         <v>12</v>
       </c>
-      <c r="D3" s="9" t="s">
+      <c r="D3" s="13" t="s">
         <v>19</v>
       </c>
-      <c r="E3" s="9">
+      <c r="E3" s="13">
         <v>6</v>
       </c>
-      <c r="F3" s="10" t="s">
+      <c r="F3" s="14" t="s">
         <v>20</v>
       </c>
-      <c r="G3" s="9">
+      <c r="G3" s="13">
         <v>1010301033</v>
       </c>
-      <c r="H3" s="9" t="s">
+      <c r="H3" s="13" t="s">
         <v>15</v>
       </c>
-      <c r="I3" s="9" t="s">
+      <c r="I3" s="13" t="s">
         <v>16</v>
       </c>
-      <c r="J3" s="9" t="s">
+      <c r="J3" s="13" t="s">
         <v>17</v>
       </c>
     </row>
     <row r="4" spans="1:10">
-      <c r="A4" s="9" t="s">
+      <c r="A4" s="13" t="s">
         <v>21</v>
       </c>
-      <c r="B4" s="10" t="s">
+      <c r="B4" s="14" t="s">
         <v>22</v>
       </c>
-      <c r="C4" s="10" t="s">
+      <c r="C4" s="14" t="s">
         <v>22</v>
       </c>
-      <c r="D4" s="9" t="s">
+      <c r="D4" s="13" t="s">
         <v>23</v>
       </c>
-      <c r="E4" s="9">
+      <c r="E4" s="13">
         <v>1</v>
       </c>
-      <c r="F4" s="10" t="s">
+      <c r="F4" s="14" t="s">
         <v>14</v>
       </c>
-      <c r="G4" s="9">
-        <v>1000000001</v>
-      </c>
-      <c r="H4" s="9"/>
-      <c r="I4" s="9" t="s">
+      <c r="G4" s="13">
+        <v>5010101060</v>
+      </c>
+      <c r="H4" s="13" t="s">
+        <v>24</v>
+      </c>
+      <c r="I4" s="13" t="s">
         <v>16</v>
       </c>
-      <c r="J4" s="9" t="s">
+      <c r="J4" s="13" t="s">
         <v>17</v>
       </c>
     </row>
     <row r="5" spans="1:10">
-      <c r="A5" s="11"/>
-      <c r="B5" s="11"/>
-      <c r="C5" s="11"/>
-      <c r="D5" s="11"/>
-      <c r="E5" s="11"/>
-      <c r="F5" s="11"/>
-      <c r="G5" s="11"/>
-      <c r="H5" s="11"/>
-      <c r="I5" s="11"/>
-      <c r="J5" s="11"/>
+      <c r="A5" s="15"/>
+      <c r="B5" s="15"/>
+      <c r="C5" s="15"/>
+      <c r="D5" s="15"/>
+      <c r="E5" s="15"/>
+      <c r="F5" s="15"/>
+      <c r="G5" s="15"/>
+      <c r="H5" s="15"/>
+      <c r="I5" s="15"/>
+      <c r="J5" s="15"/>
     </row>
     <row r="6" spans="1:10">
-      <c r="A6" s="11"/>
-      <c r="B6" s="11"/>
-      <c r="C6" s="11"/>
-      <c r="D6" s="11"/>
-      <c r="E6" s="11"/>
-      <c r="F6" s="11"/>
-      <c r="G6" s="11"/>
-      <c r="H6" s="11"/>
-      <c r="I6" s="11"/>
-      <c r="J6" s="11"/>
+      <c r="A6" s="15"/>
+      <c r="B6" s="15"/>
+      <c r="C6" s="15"/>
+      <c r="D6" s="15"/>
+      <c r="E6" s="15"/>
+      <c r="F6" s="15"/>
+      <c r="G6" s="15"/>
+      <c r="H6" s="15"/>
+      <c r="I6" s="15"/>
+      <c r="J6" s="15"/>
     </row>
     <row r="7" spans="1:10">
-      <c r="A7" s="11"/>
-      <c r="B7" s="11"/>
-      <c r="C7" s="11"/>
-      <c r="D7" s="11"/>
-      <c r="E7" s="11"/>
-      <c r="F7" s="11"/>
-      <c r="G7" s="11"/>
-      <c r="H7" s="11"/>
-      <c r="I7" s="11"/>
-      <c r="J7" s="11"/>
+      <c r="A7" s="15"/>
+      <c r="B7" s="15"/>
+      <c r="C7" s="15"/>
+      <c r="D7" s="15"/>
+      <c r="E7" s="15"/>
+      <c r="F7" s="15"/>
+      <c r="G7" s="15"/>
+      <c r="H7" s="15"/>
+      <c r="I7" s="15"/>
+      <c r="J7" s="15"/>
     </row>
     <row r="8" spans="1:10">
-      <c r="A8" s="11"/>
-      <c r="B8" s="11"/>
-      <c r="C8" s="11"/>
-      <c r="D8" s="11"/>
-      <c r="E8" s="11"/>
-      <c r="F8" s="11"/>
-      <c r="G8" s="11"/>
-      <c r="H8" s="11"/>
-      <c r="I8" s="11"/>
-      <c r="J8" s="11"/>
+      <c r="A8" s="15"/>
+      <c r="B8" s="15"/>
+      <c r="C8" s="15"/>
+      <c r="D8" s="15"/>
+      <c r="E8" s="15"/>
+      <c r="F8" s="15"/>
+      <c r="G8" s="15"/>
+      <c r="H8" s="15"/>
+      <c r="I8" s="15"/>
+      <c r="J8" s="15"/>
     </row>
     <row r="9" spans="1:10">
-      <c r="A9" s="11"/>
-      <c r="B9" s="11"/>
-      <c r="C9" s="11"/>
-      <c r="D9" s="11"/>
-      <c r="E9" s="11"/>
-      <c r="F9" s="11"/>
-      <c r="G9" s="11"/>
-      <c r="H9" s="11"/>
-      <c r="I9" s="11"/>
-      <c r="J9" s="11"/>
+      <c r="A9" s="15"/>
+      <c r="B9" s="15"/>
+      <c r="C9" s="15"/>
+      <c r="D9" s="15"/>
+      <c r="E9" s="15"/>
+      <c r="F9" s="15"/>
+      <c r="G9" s="15"/>
+      <c r="H9" s="15"/>
+      <c r="I9" s="15"/>
+      <c r="J9" s="15"/>
     </row>
     <row r="10" spans="1:10">
-      <c r="A10" s="11"/>
-      <c r="B10" s="11"/>
-      <c r="C10" s="11"/>
-      <c r="D10" s="11"/>
-      <c r="E10" s="11"/>
-      <c r="F10" s="11"/>
-      <c r="G10" s="11"/>
-      <c r="H10" s="11"/>
-      <c r="I10" s="11"/>
-      <c r="J10" s="11"/>
+      <c r="A10" s="15"/>
+      <c r="B10" s="15"/>
+      <c r="C10" s="15"/>
+      <c r="D10" s="15"/>
+      <c r="E10" s="15"/>
+      <c r="F10" s="15"/>
+      <c r="G10" s="15"/>
+      <c r="H10" s="15"/>
+      <c r="I10" s="15"/>
+      <c r="J10" s="15"/>
     </row>
     <row r="11" spans="1:10">
-      <c r="A11" s="11"/>
-      <c r="B11" s="11"/>
-      <c r="C11" s="11"/>
-      <c r="D11" s="11"/>
-      <c r="E11" s="11"/>
-      <c r="F11" s="11"/>
-      <c r="G11" s="11"/>
-      <c r="H11" s="11"/>
-      <c r="I11" s="11"/>
-      <c r="J11" s="11"/>
+      <c r="A11" s="15"/>
+      <c r="B11" s="15"/>
+      <c r="C11" s="15"/>
+      <c r="D11" s="15"/>
+      <c r="E11" s="15"/>
+      <c r="F11" s="15"/>
+      <c r="G11" s="15"/>
+      <c r="H11" s="15"/>
+      <c r="I11" s="15"/>
+      <c r="J11" s="15"/>
     </row>
     <row r="12" spans="1:10">
-      <c r="A12" s="11"/>
-      <c r="B12" s="11"/>
-      <c r="C12" s="11"/>
-      <c r="D12" s="11"/>
-      <c r="E12" s="11"/>
-      <c r="F12" s="11"/>
-      <c r="G12" s="11"/>
-      <c r="H12" s="11"/>
-      <c r="I12" s="11"/>
-      <c r="J12" s="11"/>
+      <c r="A12" s="15"/>
+      <c r="B12" s="15"/>
+      <c r="C12" s="15"/>
+      <c r="D12" s="15"/>
+      <c r="E12" s="15"/>
+      <c r="F12" s="15"/>
+      <c r="G12" s="15"/>
+      <c r="H12" s="15"/>
+      <c r="I12" s="15"/>
+      <c r="J12" s="15"/>
     </row>
     <row r="13" spans="1:10">
-      <c r="A13" s="11"/>
-      <c r="B13" s="11"/>
-      <c r="C13" s="11"/>
-      <c r="D13" s="11"/>
-      <c r="E13" s="11"/>
-      <c r="F13" s="11"/>
-      <c r="G13" s="11"/>
-      <c r="H13" s="11"/>
-      <c r="I13" s="11"/>
-      <c r="J13" s="11"/>
+      <c r="A13" s="15"/>
+      <c r="B13" s="15"/>
+      <c r="C13" s="15"/>
+      <c r="D13" s="15"/>
+      <c r="E13" s="15"/>
+      <c r="F13" s="15"/>
+      <c r="G13" s="15"/>
+      <c r="H13" s="15"/>
+      <c r="I13" s="15"/>
+      <c r="J13" s="15"/>
     </row>
     <row r="14" spans="1:10">
-      <c r="A14" s="11"/>
-      <c r="B14" s="11"/>
-      <c r="C14" s="11"/>
-      <c r="D14" s="11"/>
-      <c r="E14" s="11"/>
-      <c r="F14" s="11"/>
-      <c r="G14" s="11"/>
-      <c r="H14" s="11"/>
-      <c r="I14" s="11"/>
-      <c r="J14" s="11"/>
+      <c r="A14" s="15"/>
+      <c r="B14" s="15"/>
+      <c r="C14" s="15"/>
+      <c r="D14" s="15"/>
+      <c r="E14" s="15"/>
+      <c r="F14" s="15"/>
+      <c r="G14" s="15"/>
+      <c r="H14" s="15"/>
+      <c r="I14" s="15"/>
+      <c r="J14" s="15"/>
     </row>
     <row r="15" spans="1:10">
-      <c r="A15" s="11"/>
-      <c r="B15" s="11"/>
-      <c r="C15" s="11"/>
-      <c r="D15" s="11"/>
-      <c r="E15" s="11"/>
-      <c r="F15" s="11"/>
-      <c r="G15" s="11"/>
-      <c r="H15" s="11"/>
-      <c r="I15" s="11"/>
-      <c r="J15" s="11"/>
+      <c r="A15" s="15"/>
+      <c r="B15" s="15"/>
+      <c r="C15" s="15"/>
+      <c r="D15" s="15"/>
+      <c r="E15" s="15"/>
+      <c r="F15" s="15"/>
+      <c r="G15" s="15"/>
+      <c r="H15" s="15"/>
+      <c r="I15" s="15"/>
+      <c r="J15" s="15"/>
     </row>
     <row r="16" spans="1:10">
-      <c r="A16" s="11"/>
-      <c r="B16" s="11"/>
-      <c r="C16" s="11"/>
-      <c r="D16" s="11"/>
-      <c r="E16" s="11"/>
-      <c r="F16" s="11"/>
-      <c r="G16" s="11"/>
-      <c r="H16" s="11"/>
-      <c r="I16" s="11"/>
-      <c r="J16" s="11"/>
+      <c r="A16" s="15"/>
+      <c r="B16" s="15"/>
+      <c r="C16" s="15"/>
+      <c r="D16" s="15"/>
+      <c r="E16" s="15"/>
+      <c r="F16" s="15"/>
+      <c r="G16" s="15"/>
+      <c r="H16" s="15"/>
+      <c r="I16" s="15"/>
+      <c r="J16" s="15"/>
     </row>
     <row r="17" spans="1:10">
-      <c r="A17" s="11"/>
-      <c r="B17" s="11"/>
-      <c r="C17" s="11"/>
-      <c r="D17" s="11"/>
-      <c r="E17" s="11"/>
-      <c r="F17" s="11"/>
-      <c r="G17" s="11"/>
-      <c r="H17" s="11"/>
-      <c r="I17" s="11"/>
-      <c r="J17" s="11"/>
+      <c r="A17" s="15"/>
+      <c r="B17" s="15"/>
+      <c r="C17" s="15"/>
+      <c r="D17" s="15"/>
+      <c r="E17" s="15"/>
+      <c r="F17" s="15"/>
+      <c r="G17" s="15"/>
+      <c r="H17" s="15"/>
+      <c r="I17" s="15"/>
+      <c r="J17" s="15"/>
     </row>
     <row r="18" spans="1:10">
-      <c r="A18" s="11"/>
-      <c r="B18" s="11"/>
-      <c r="C18" s="11"/>
-      <c r="D18" s="11"/>
-      <c r="E18" s="11"/>
-      <c r="F18" s="11"/>
-      <c r="G18" s="11"/>
-      <c r="H18" s="11"/>
-      <c r="I18" s="11"/>
-      <c r="J18" s="11"/>
+      <c r="A18" s="15"/>
+      <c r="B18" s="15"/>
+      <c r="C18" s="15"/>
+      <c r="D18" s="15"/>
+      <c r="E18" s="15"/>
+      <c r="F18" s="15"/>
+      <c r="G18" s="15"/>
+      <c r="H18" s="15"/>
+      <c r="I18" s="15"/>
+      <c r="J18" s="15"/>
     </row>
     <row r="19" spans="1:10">
-      <c r="A19" s="11"/>
-      <c r="B19" s="11"/>
-      <c r="C19" s="11"/>
-      <c r="D19" s="11"/>
-      <c r="E19" s="11"/>
-      <c r="F19" s="11"/>
-      <c r="G19" s="11"/>
-      <c r="H19" s="11"/>
-      <c r="I19" s="11"/>
-      <c r="J19" s="11"/>
+      <c r="A19" s="15"/>
+      <c r="B19" s="15"/>
+      <c r="C19" s="15"/>
+      <c r="D19" s="15"/>
+      <c r="E19" s="15"/>
+      <c r="F19" s="15"/>
+      <c r="G19" s="15"/>
+      <c r="H19" s="15"/>
+      <c r="I19" s="15"/>
+      <c r="J19" s="15"/>
     </row>
     <row r="20" spans="1:10">
-      <c r="A20" s="11"/>
-      <c r="B20" s="11"/>
-      <c r="C20" s="11"/>
-      <c r="D20" s="11"/>
-      <c r="E20" s="11"/>
-      <c r="F20" s="11"/>
-      <c r="G20" s="11"/>
-      <c r="H20" s="11"/>
-      <c r="I20" s="11"/>
-      <c r="J20" s="11"/>
+      <c r="A20" s="15"/>
+      <c r="B20" s="15"/>
+      <c r="C20" s="15"/>
+      <c r="D20" s="15"/>
+      <c r="E20" s="15"/>
+      <c r="F20" s="15"/>
+      <c r="G20" s="15"/>
+      <c r="H20" s="15"/>
+      <c r="I20" s="15"/>
+      <c r="J20" s="15"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1785,8 +1837,8 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:T6"/>
-  <sheetFormatPr defaultColWidth="8.73148148148148" defaultRowHeight="14.4" outlineLevelRow="5"/>
+  <dimension ref="A1:T10"/>
+  <sheetFormatPr defaultColWidth="8.73148148148148" defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="30" customWidth="1"/>
     <col min="2" max="2" width="36.4444444444444" customWidth="1"/>
@@ -1800,7 +1852,7 @@
     <col min="10" max="10" width="13.2222222222222" customWidth="1"/>
     <col min="11" max="11" width="22.7777777777778" customWidth="1"/>
     <col min="12" max="12" width="12.7777777777778" customWidth="1"/>
-    <col min="13" max="13" width="17.5555555555556" customWidth="1"/>
+    <col min="13" max="13" width="29.5555555555556" customWidth="1"/>
     <col min="14" max="14" width="18.2222222222222" customWidth="1"/>
     <col min="15" max="15" width="16.2222222222222" customWidth="1"/>
     <col min="16" max="16" width="15.5555555555556" customWidth="1"/>
@@ -1812,19 +1864,19 @@
   <sheetData>
     <row r="1" spans="1:20">
       <c r="A1" s="2" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F1" s="2" t="s">
         <v>2</v>
@@ -1833,16 +1885,16 @@
         <v>1</v>
       </c>
       <c r="H1" s="2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="I1" s="2" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="K1" s="2" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="L1" s="2" t="s">
         <v>6</v>
@@ -1857,19 +1909,19 @@
         <v>9</v>
       </c>
       <c r="P1" s="2" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="Q1" s="2" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="R1" s="2" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="S1" s="2" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="T1" s="2" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
     </row>
     <row r="2" spans="1:20">
@@ -1877,18 +1929,18 @@
         <v>18</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C2" s="2" t="s">
         <v>20</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="E2" s="2">
         <v>12</v>
       </c>
-      <c r="F2" s="4" t="s">
+      <c r="F2" s="6" t="s">
         <v>12</v>
       </c>
       <c r="G2" s="2" t="s">
@@ -1898,7 +1950,7 @@
         <v>19</v>
       </c>
       <c r="I2" s="2" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="J2" s="2" t="s">
         <v>14</v>
@@ -1931,13 +1983,13 @@
         <v>10</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C3" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="D3" s="5" t="s">
-        <v>42</v>
+      <c r="D3" s="7" t="s">
+        <v>43</v>
       </c>
       <c r="E3" s="2">
         <v>5</v>
@@ -1952,7 +2004,7 @@
         <v>13</v>
       </c>
       <c r="I3" s="2" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="J3" s="2" t="s">
         <v>14</v>
@@ -1985,7 +2037,7 @@
         <v>21</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="C4" s="2" t="s">
         <v>14</v>
@@ -2006,7 +2058,7 @@
         <v>23</v>
       </c>
       <c r="I4" s="2" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="J4" s="2" t="s">
         <v>14</v>
@@ -2015,10 +2067,10 @@
         <v>1</v>
       </c>
       <c r="L4" s="2">
-        <v>1000000792</v>
+        <v>1011134888</v>
       </c>
       <c r="M4" s="2" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="N4" s="2" t="s">
         <v>16</v>
@@ -2036,31 +2088,31 @@
     </row>
     <row r="5" spans="1:20">
       <c r="A5" s="1" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="C5" s="2" t="s">
         <v>14</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="E5" s="1">
         <v>12</v>
       </c>
       <c r="F5" s="1" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="G5" s="1" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="H5" s="1" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="I5" s="1" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="J5" s="1" t="s">
         <v>14</v>
@@ -2072,13 +2124,13 @@
         <v>1010301001</v>
       </c>
       <c r="M5" s="1" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="N5" s="1" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="O5" s="1" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="P5" s="1"/>
       <c r="Q5" s="1"/>
@@ -2090,31 +2142,31 @@
     </row>
     <row r="6" spans="1:20">
       <c r="A6" s="1" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="C6" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="D6" s="3" t="s">
-        <v>42</v>
+      <c r="D6" s="5" t="s">
+        <v>43</v>
       </c>
       <c r="E6">
         <v>5</v>
       </c>
-      <c r="F6" s="6" t="s">
+      <c r="F6" s="8" t="s">
         <v>12</v>
       </c>
-      <c r="G6" s="6" t="s">
+      <c r="G6" s="8" t="s">
         <v>11</v>
       </c>
       <c r="H6" s="1" t="s">
         <v>19</v>
       </c>
       <c r="I6" s="1" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="J6" s="1" t="s">
         <v>14</v>
@@ -2141,6 +2193,222 @@
         <v>0</v>
       </c>
       <c r="T6" s="1"/>
+    </row>
+    <row r="7" spans="1:20">
+      <c r="A7" s="9" t="s">
+        <v>55</v>
+      </c>
+      <c r="B7" s="9" t="s">
+        <v>56</v>
+      </c>
+      <c r="C7" s="9" t="s">
+        <v>20</v>
+      </c>
+      <c r="D7" s="9" t="s">
+        <v>40</v>
+      </c>
+      <c r="E7" s="9">
+        <v>12</v>
+      </c>
+      <c r="F7" s="10" t="s">
+        <v>12</v>
+      </c>
+      <c r="G7" s="9" t="s">
+        <v>11</v>
+      </c>
+      <c r="H7" s="9" t="s">
+        <v>57</v>
+      </c>
+      <c r="I7" s="9" t="s">
+        <v>41</v>
+      </c>
+      <c r="J7" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="K7" s="9">
+        <v>3</v>
+      </c>
+      <c r="L7" s="9">
+        <v>1010301003</v>
+      </c>
+      <c r="M7" s="9" t="s">
+        <v>58</v>
+      </c>
+      <c r="N7" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="O7" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="P7" s="9"/>
+      <c r="Q7" s="9"/>
+      <c r="R7" s="9"/>
+      <c r="S7" s="9">
+        <v>0</v>
+      </c>
+      <c r="T7" s="9"/>
+    </row>
+    <row r="8" spans="1:20">
+      <c r="A8" s="9" t="s">
+        <v>59</v>
+      </c>
+      <c r="B8" s="9" t="s">
+        <v>60</v>
+      </c>
+      <c r="C8" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="D8" s="9" t="s">
+        <v>43</v>
+      </c>
+      <c r="E8" s="9">
+        <v>5</v>
+      </c>
+      <c r="F8" s="10" t="s">
+        <v>12</v>
+      </c>
+      <c r="G8" s="9" t="s">
+        <v>11</v>
+      </c>
+      <c r="H8" s="9" t="s">
+        <v>57</v>
+      </c>
+      <c r="I8" s="9" t="s">
+        <v>41</v>
+      </c>
+      <c r="J8" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="K8" s="9">
+        <v>0</v>
+      </c>
+      <c r="L8" s="9">
+        <v>1010301003</v>
+      </c>
+      <c r="M8" s="9" t="s">
+        <v>58</v>
+      </c>
+      <c r="N8" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="O8" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="P8" s="9"/>
+      <c r="Q8" s="9"/>
+      <c r="R8" s="9"/>
+      <c r="S8" s="9">
+        <v>0</v>
+      </c>
+      <c r="T8" s="9"/>
+    </row>
+    <row r="9" spans="1:20">
+      <c r="A9" s="9" t="s">
+        <v>61</v>
+      </c>
+      <c r="B9" s="9" t="s">
+        <v>61</v>
+      </c>
+      <c r="C9" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="D9" s="9" t="s">
+        <v>43</v>
+      </c>
+      <c r="E9" s="9">
+        <v>5</v>
+      </c>
+      <c r="F9" s="10" t="s">
+        <v>12</v>
+      </c>
+      <c r="G9" s="9" t="s">
+        <v>11</v>
+      </c>
+      <c r="H9" s="9" t="s">
+        <v>57</v>
+      </c>
+      <c r="I9" s="9" t="s">
+        <v>41</v>
+      </c>
+      <c r="J9" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="K9" s="9">
+        <v>0</v>
+      </c>
+      <c r="L9" s="9">
+        <v>1010301003</v>
+      </c>
+      <c r="M9" s="9" t="s">
+        <v>58</v>
+      </c>
+      <c r="N9" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="O9" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="P9" s="9"/>
+      <c r="Q9" s="9"/>
+      <c r="R9" s="9"/>
+      <c r="S9" s="9">
+        <v>0</v>
+      </c>
+      <c r="T9" s="9"/>
+    </row>
+    <row r="10" spans="1:20">
+      <c r="A10" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="B10" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="C10" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="D10" s="9" t="s">
+        <v>43</v>
+      </c>
+      <c r="E10" s="9">
+        <v>5</v>
+      </c>
+      <c r="F10" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="G10" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="H10" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="I10" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="J10" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="K10" s="2">
+        <v>1</v>
+      </c>
+      <c r="L10" s="3">
+        <v>1000000001</v>
+      </c>
+      <c r="M10" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="N10" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="O10" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="P10" s="9"/>
+      <c r="Q10" s="9"/>
+      <c r="R10" s="9"/>
+      <c r="S10" s="9">
+        <v>0</v>
+      </c>
+      <c r="T10" s="9"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2151,13 +2419,13 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:R2"/>
-  <sheetFormatPr defaultColWidth="8.88888888888889" defaultRowHeight="14.4" outlineLevelRow="1"/>
+  <dimension ref="A1:R3"/>
+  <sheetFormatPr defaultColWidth="8.88888888888889" defaultRowHeight="14.4" outlineLevelRow="2"/>
   <cols>
     <col min="1" max="2" width="21" customWidth="1"/>
     <col min="3" max="3" width="6" customWidth="1"/>
     <col min="4" max="4" width="12.7777777777778" customWidth="1"/>
-    <col min="5" max="5" width="16.5555555555556" customWidth="1"/>
+    <col min="5" max="5" width="19.4444444444444" customWidth="1"/>
     <col min="6" max="6" width="15.1111111111111" customWidth="1"/>
     <col min="7" max="7" width="15.4444444444444" customWidth="1"/>
     <col min="8" max="8" width="19.5555555555556" customWidth="1"/>
@@ -2169,13 +2437,13 @@
   <sheetData>
     <row r="1" spans="1:18">
       <c r="A1" s="1" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="D1" s="2" t="s">
         <v>6</v>
@@ -2190,33 +2458,33 @@
         <v>9</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>54</v>
+        <v>65</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="M1" s="1"/>
-      <c r="N1" s="1"/>
-      <c r="O1" s="1"/>
-      <c r="P1" s="1"/>
-      <c r="Q1" s="1"/>
-      <c r="R1" s="1"/>
+        <v>33</v>
+      </c>
+      <c r="M1" s="4"/>
+      <c r="N1" s="4"/>
+      <c r="O1" s="4"/>
+      <c r="P1" s="4"/>
+      <c r="Q1" s="4"/>
+      <c r="R1" s="4"/>
     </row>
     <row r="2" spans="1:18">
       <c r="A2" s="1" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="C2" s="1" t="s">
         <v>14</v>
@@ -2236,11 +2504,11 @@
       <c r="H2" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="I2" s="3" t="s">
-        <v>42</v>
+      <c r="I2" s="5" t="s">
+        <v>43</v>
       </c>
       <c r="J2" s="1" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="K2" s="1" t="s">
         <v>14</v>
@@ -2248,12 +2516,50 @@
       <c r="L2" s="1">
         <v>1</v>
       </c>
-      <c r="M2" s="1"/>
-      <c r="N2" s="1"/>
-      <c r="O2" s="1"/>
-      <c r="P2" s="1"/>
-      <c r="Q2" s="1"/>
-      <c r="R2" s="1"/>
+      <c r="M2" s="4"/>
+      <c r="N2" s="4"/>
+      <c r="O2" s="4"/>
+      <c r="P2" s="4"/>
+      <c r="Q2" s="4"/>
+      <c r="R2" s="4"/>
+    </row>
+    <row r="3" spans="1:12">
+      <c r="A3" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="D3" s="3">
+        <v>1000000001</v>
+      </c>
+      <c r="E3" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="F3" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="G3" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="H3" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="I3" s="5" t="s">
+        <v>43</v>
+      </c>
+      <c r="J3" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="K3" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="L3" s="1">
+        <v>1</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Added PR To Payment Receipt E2E Test Scenario
Added PR To Payment Receipt E2E Test Scenario
</commit_message>
<xml_diff>
--- a/testdata/ItemDetails.xlsx
+++ b/testdata/ItemDetails.xlsx
@@ -4,12 +4,13 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="23040" windowHeight="9120"/>
+    <workbookView windowWidth="23040" windowHeight="9120" activeTab="3"/>
   </bookViews>
   <sheets>
     <sheet name="PR Details" sheetId="1" r:id="rId1"/>
     <sheet name="PO Details" sheetId="2" r:id="rId2"/>
     <sheet name="POA Details" sheetId="3" r:id="rId3"/>
+    <sheet name="PO MULTIPLE ITEM" sheetId="4" r:id="rId4"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -29,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="193" uniqueCount="66">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="199" uniqueCount="68">
   <si>
     <t>ITEM_NAME</t>
   </si>
@@ -228,6 +229,12 @@
   </si>
   <si>
     <t>SUPL_UOM</t>
+  </si>
+  <si>
+    <t>QUANTITY</t>
+  </si>
+  <si>
+    <t>UNIT_COST</t>
   </si>
 </sst>
 </file>
@@ -240,13 +247,19 @@
     <numFmt numFmtId="178" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
     <numFmt numFmtId="179" formatCode="_ &quot;₹&quot;* #,##0_ ;_ &quot;₹&quot;* \-#,##0_ ;_ &quot;₹&quot;* &quot;-&quot;_ ;_ @_ "/>
   </numFmts>
-  <fonts count="27">
+  <fonts count="28">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <charset val="134"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Times New Roman"/>
+      <charset val="134"/>
     </font>
     <font>
       <sz val="10"/>
@@ -778,150 +791,156 @@
     <xf numFmtId="179" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="2" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="4" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="5" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="5" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="6" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="4" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="5" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="5" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="6" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1">
@@ -930,34 +949,34 @@
     <xf numFmtId="49" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="49" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="49" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="49" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="49" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="justify" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -1509,324 +1528,324 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10">
-      <c r="A1" s="12" t="s">
+      <c r="A1" s="14" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="12" t="s">
+      <c r="B1" s="14" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="12" t="s">
+      <c r="C1" s="14" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="12" t="s">
+      <c r="D1" s="14" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="12" t="s">
+      <c r="E1" s="14" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="12" t="s">
+      <c r="F1" s="14" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="12" t="s">
+      <c r="G1" s="14" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="12" t="s">
+      <c r="H1" s="14" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="12" t="s">
+      <c r="I1" s="14" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="12" t="s">
+      <c r="J1" s="14" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="2" s="11" customFormat="1" ht="20.4" spans="1:10">
-      <c r="A2" s="13" t="s">
+    <row r="2" s="13" customFormat="1" ht="20.4" spans="1:10">
+      <c r="A2" s="15" t="s">
         <v>10</v>
       </c>
-      <c r="B2" s="14" t="s">
+      <c r="B2" s="16" t="s">
         <v>11</v>
       </c>
-      <c r="C2" s="14" t="s">
+      <c r="C2" s="16" t="s">
         <v>12</v>
       </c>
-      <c r="D2" s="13" t="s">
+      <c r="D2" s="15" t="s">
         <v>13</v>
       </c>
-      <c r="E2" s="13">
+      <c r="E2" s="15">
         <v>1</v>
       </c>
-      <c r="F2" s="13" t="s">
+      <c r="F2" s="15" t="s">
         <v>14</v>
       </c>
-      <c r="G2" s="13">
+      <c r="G2" s="15">
         <v>1010301033</v>
       </c>
-      <c r="H2" s="13" t="s">
+      <c r="H2" s="15" t="s">
         <v>15</v>
       </c>
-      <c r="I2" s="13" t="s">
+      <c r="I2" s="15" t="s">
         <v>16</v>
       </c>
-      <c r="J2" s="13" t="s">
+      <c r="J2" s="15" t="s">
         <v>17</v>
       </c>
     </row>
     <row r="3" ht="15" customHeight="1" spans="1:10">
-      <c r="A3" s="13" t="s">
+      <c r="A3" s="15" t="s">
         <v>18</v>
       </c>
-      <c r="B3" s="14" t="s">
+      <c r="B3" s="16" t="s">
         <v>11</v>
       </c>
-      <c r="C3" s="14" t="s">
+      <c r="C3" s="16" t="s">
         <v>12</v>
       </c>
-      <c r="D3" s="13" t="s">
+      <c r="D3" s="15" t="s">
         <v>19</v>
       </c>
-      <c r="E3" s="13">
+      <c r="E3" s="15">
         <v>6</v>
       </c>
-      <c r="F3" s="14" t="s">
+      <c r="F3" s="16" t="s">
         <v>20</v>
       </c>
-      <c r="G3" s="13">
+      <c r="G3" s="15">
         <v>1010301033</v>
       </c>
-      <c r="H3" s="13" t="s">
+      <c r="H3" s="15" t="s">
         <v>15</v>
       </c>
-      <c r="I3" s="13" t="s">
+      <c r="I3" s="15" t="s">
         <v>16</v>
       </c>
-      <c r="J3" s="13" t="s">
+      <c r="J3" s="15" t="s">
         <v>17</v>
       </c>
     </row>
     <row r="4" spans="1:10">
-      <c r="A4" s="13" t="s">
+      <c r="A4" s="15" t="s">
         <v>21</v>
       </c>
-      <c r="B4" s="14" t="s">
+      <c r="B4" s="16" t="s">
         <v>22</v>
       </c>
-      <c r="C4" s="14" t="s">
+      <c r="C4" s="16" t="s">
         <v>22</v>
       </c>
-      <c r="D4" s="13" t="s">
+      <c r="D4" s="15" t="s">
         <v>23</v>
       </c>
-      <c r="E4" s="13">
+      <c r="E4" s="15">
         <v>1</v>
       </c>
-      <c r="F4" s="14" t="s">
+      <c r="F4" s="16" t="s">
         <v>14</v>
       </c>
-      <c r="G4" s="13">
+      <c r="G4" s="15">
         <v>5010101060</v>
       </c>
-      <c r="H4" s="13" t="s">
+      <c r="H4" s="15" t="s">
         <v>24</v>
       </c>
-      <c r="I4" s="13" t="s">
+      <c r="I4" s="15" t="s">
         <v>16</v>
       </c>
-      <c r="J4" s="13" t="s">
+      <c r="J4" s="15" t="s">
         <v>17</v>
       </c>
     </row>
     <row r="5" spans="1:10">
-      <c r="A5" s="15"/>
-      <c r="B5" s="15"/>
-      <c r="C5" s="15"/>
-      <c r="D5" s="15"/>
-      <c r="E5" s="15"/>
-      <c r="F5" s="15"/>
-      <c r="G5" s="15"/>
-      <c r="H5" s="15"/>
-      <c r="I5" s="15"/>
-      <c r="J5" s="15"/>
+      <c r="A5" s="17"/>
+      <c r="B5" s="17"/>
+      <c r="C5" s="17"/>
+      <c r="D5" s="17"/>
+      <c r="E5" s="17"/>
+      <c r="F5" s="17"/>
+      <c r="G5" s="17"/>
+      <c r="H5" s="17"/>
+      <c r="I5" s="17"/>
+      <c r="J5" s="17"/>
     </row>
     <row r="6" spans="1:10">
-      <c r="A6" s="15"/>
-      <c r="B6" s="15"/>
-      <c r="C6" s="15"/>
-      <c r="D6" s="15"/>
-      <c r="E6" s="15"/>
-      <c r="F6" s="15"/>
-      <c r="G6" s="15"/>
-      <c r="H6" s="15"/>
-      <c r="I6" s="15"/>
-      <c r="J6" s="15"/>
+      <c r="A6" s="17"/>
+      <c r="B6" s="17"/>
+      <c r="C6" s="17"/>
+      <c r="D6" s="17"/>
+      <c r="E6" s="17"/>
+      <c r="F6" s="17"/>
+      <c r="G6" s="17"/>
+      <c r="H6" s="17"/>
+      <c r="I6" s="17"/>
+      <c r="J6" s="17"/>
     </row>
     <row r="7" spans="1:10">
-      <c r="A7" s="15"/>
-      <c r="B7" s="15"/>
-      <c r="C7" s="15"/>
-      <c r="D7" s="15"/>
-      <c r="E7" s="15"/>
-      <c r="F7" s="15"/>
-      <c r="G7" s="15"/>
-      <c r="H7" s="15"/>
-      <c r="I7" s="15"/>
-      <c r="J7" s="15"/>
+      <c r="A7" s="17"/>
+      <c r="B7" s="17"/>
+      <c r="C7" s="17"/>
+      <c r="D7" s="17"/>
+      <c r="E7" s="17"/>
+      <c r="F7" s="17"/>
+      <c r="G7" s="17"/>
+      <c r="H7" s="17"/>
+      <c r="I7" s="17"/>
+      <c r="J7" s="17"/>
     </row>
     <row r="8" spans="1:10">
-      <c r="A8" s="15"/>
-      <c r="B8" s="15"/>
-      <c r="C8" s="15"/>
-      <c r="D8" s="15"/>
-      <c r="E8" s="15"/>
-      <c r="F8" s="15"/>
-      <c r="G8" s="15"/>
-      <c r="H8" s="15"/>
-      <c r="I8" s="15"/>
-      <c r="J8" s="15"/>
+      <c r="A8" s="17"/>
+      <c r="B8" s="17"/>
+      <c r="C8" s="17"/>
+      <c r="D8" s="17"/>
+      <c r="E8" s="17"/>
+      <c r="F8" s="17"/>
+      <c r="G8" s="17"/>
+      <c r="H8" s="17"/>
+      <c r="I8" s="17"/>
+      <c r="J8" s="17"/>
     </row>
     <row r="9" spans="1:10">
-      <c r="A9" s="15"/>
-      <c r="B9" s="15"/>
-      <c r="C9" s="15"/>
-      <c r="D9" s="15"/>
-      <c r="E9" s="15"/>
-      <c r="F9" s="15"/>
-      <c r="G9" s="15"/>
-      <c r="H9" s="15"/>
-      <c r="I9" s="15"/>
-      <c r="J9" s="15"/>
+      <c r="A9" s="17"/>
+      <c r="B9" s="17"/>
+      <c r="C9" s="17"/>
+      <c r="D9" s="17"/>
+      <c r="E9" s="17"/>
+      <c r="F9" s="17"/>
+      <c r="G9" s="17"/>
+      <c r="H9" s="17"/>
+      <c r="I9" s="17"/>
+      <c r="J9" s="17"/>
     </row>
     <row r="10" spans="1:10">
-      <c r="A10" s="15"/>
-      <c r="B10" s="15"/>
-      <c r="C10" s="15"/>
-      <c r="D10" s="15"/>
-      <c r="E10" s="15"/>
-      <c r="F10" s="15"/>
-      <c r="G10" s="15"/>
-      <c r="H10" s="15"/>
-      <c r="I10" s="15"/>
-      <c r="J10" s="15"/>
+      <c r="A10" s="17"/>
+      <c r="B10" s="17"/>
+      <c r="C10" s="17"/>
+      <c r="D10" s="17"/>
+      <c r="E10" s="17"/>
+      <c r="F10" s="17"/>
+      <c r="G10" s="17"/>
+      <c r="H10" s="17"/>
+      <c r="I10" s="17"/>
+      <c r="J10" s="17"/>
     </row>
     <row r="11" spans="1:10">
-      <c r="A11" s="15"/>
-      <c r="B11" s="15"/>
-      <c r="C11" s="15"/>
-      <c r="D11" s="15"/>
-      <c r="E11" s="15"/>
-      <c r="F11" s="15"/>
-      <c r="G11" s="15"/>
-      <c r="H11" s="15"/>
-      <c r="I11" s="15"/>
-      <c r="J11" s="15"/>
+      <c r="A11" s="17"/>
+      <c r="B11" s="17"/>
+      <c r="C11" s="17"/>
+      <c r="D11" s="17"/>
+      <c r="E11" s="17"/>
+      <c r="F11" s="17"/>
+      <c r="G11" s="17"/>
+      <c r="H11" s="17"/>
+      <c r="I11" s="17"/>
+      <c r="J11" s="17"/>
     </row>
     <row r="12" spans="1:10">
-      <c r="A12" s="15"/>
-      <c r="B12" s="15"/>
-      <c r="C12" s="15"/>
-      <c r="D12" s="15"/>
-      <c r="E12" s="15"/>
-      <c r="F12" s="15"/>
-      <c r="G12" s="15"/>
-      <c r="H12" s="15"/>
-      <c r="I12" s="15"/>
-      <c r="J12" s="15"/>
+      <c r="A12" s="17"/>
+      <c r="B12" s="17"/>
+      <c r="C12" s="17"/>
+      <c r="D12" s="17"/>
+      <c r="E12" s="17"/>
+      <c r="F12" s="17"/>
+      <c r="G12" s="17"/>
+      <c r="H12" s="17"/>
+      <c r="I12" s="17"/>
+      <c r="J12" s="17"/>
     </row>
     <row r="13" spans="1:10">
-      <c r="A13" s="15"/>
-      <c r="B13" s="15"/>
-      <c r="C13" s="15"/>
-      <c r="D13" s="15"/>
-      <c r="E13" s="15"/>
-      <c r="F13" s="15"/>
-      <c r="G13" s="15"/>
-      <c r="H13" s="15"/>
-      <c r="I13" s="15"/>
-      <c r="J13" s="15"/>
+      <c r="A13" s="17"/>
+      <c r="B13" s="17"/>
+      <c r="C13" s="17"/>
+      <c r="D13" s="17"/>
+      <c r="E13" s="17"/>
+      <c r="F13" s="17"/>
+      <c r="G13" s="17"/>
+      <c r="H13" s="17"/>
+      <c r="I13" s="17"/>
+      <c r="J13" s="17"/>
     </row>
     <row r="14" spans="1:10">
-      <c r="A14" s="15"/>
-      <c r="B14" s="15"/>
-      <c r="C14" s="15"/>
-      <c r="D14" s="15"/>
-      <c r="E14" s="15"/>
-      <c r="F14" s="15"/>
-      <c r="G14" s="15"/>
-      <c r="H14" s="15"/>
-      <c r="I14" s="15"/>
-      <c r="J14" s="15"/>
+      <c r="A14" s="17"/>
+      <c r="B14" s="17"/>
+      <c r="C14" s="17"/>
+      <c r="D14" s="17"/>
+      <c r="E14" s="17"/>
+      <c r="F14" s="17"/>
+      <c r="G14" s="17"/>
+      <c r="H14" s="17"/>
+      <c r="I14" s="17"/>
+      <c r="J14" s="17"/>
     </row>
     <row r="15" spans="1:10">
-      <c r="A15" s="15"/>
-      <c r="B15" s="15"/>
-      <c r="C15" s="15"/>
-      <c r="D15" s="15"/>
-      <c r="E15" s="15"/>
-      <c r="F15" s="15"/>
-      <c r="G15" s="15"/>
-      <c r="H15" s="15"/>
-      <c r="I15" s="15"/>
-      <c r="J15" s="15"/>
+      <c r="A15" s="17"/>
+      <c r="B15" s="17"/>
+      <c r="C15" s="17"/>
+      <c r="D15" s="17"/>
+      <c r="E15" s="17"/>
+      <c r="F15" s="17"/>
+      <c r="G15" s="17"/>
+      <c r="H15" s="17"/>
+      <c r="I15" s="17"/>
+      <c r="J15" s="17"/>
     </row>
     <row r="16" spans="1:10">
-      <c r="A16" s="15"/>
-      <c r="B16" s="15"/>
-      <c r="C16" s="15"/>
-      <c r="D16" s="15"/>
-      <c r="E16" s="15"/>
-      <c r="F16" s="15"/>
-      <c r="G16" s="15"/>
-      <c r="H16" s="15"/>
-      <c r="I16" s="15"/>
-      <c r="J16" s="15"/>
+      <c r="A16" s="17"/>
+      <c r="B16" s="17"/>
+      <c r="C16" s="17"/>
+      <c r="D16" s="17"/>
+      <c r="E16" s="17"/>
+      <c r="F16" s="17"/>
+      <c r="G16" s="17"/>
+      <c r="H16" s="17"/>
+      <c r="I16" s="17"/>
+      <c r="J16" s="17"/>
     </row>
     <row r="17" spans="1:10">
-      <c r="A17" s="15"/>
-      <c r="B17" s="15"/>
-      <c r="C17" s="15"/>
-      <c r="D17" s="15"/>
-      <c r="E17" s="15"/>
-      <c r="F17" s="15"/>
-      <c r="G17" s="15"/>
-      <c r="H17" s="15"/>
-      <c r="I17" s="15"/>
-      <c r="J17" s="15"/>
+      <c r="A17" s="17"/>
+      <c r="B17" s="17"/>
+      <c r="C17" s="17"/>
+      <c r="D17" s="17"/>
+      <c r="E17" s="17"/>
+      <c r="F17" s="17"/>
+      <c r="G17" s="17"/>
+      <c r="H17" s="17"/>
+      <c r="I17" s="17"/>
+      <c r="J17" s="17"/>
     </row>
     <row r="18" spans="1:10">
-      <c r="A18" s="15"/>
-      <c r="B18" s="15"/>
-      <c r="C18" s="15"/>
-      <c r="D18" s="15"/>
-      <c r="E18" s="15"/>
-      <c r="F18" s="15"/>
-      <c r="G18" s="15"/>
-      <c r="H18" s="15"/>
-      <c r="I18" s="15"/>
-      <c r="J18" s="15"/>
+      <c r="A18" s="17"/>
+      <c r="B18" s="17"/>
+      <c r="C18" s="17"/>
+      <c r="D18" s="17"/>
+      <c r="E18" s="17"/>
+      <c r="F18" s="17"/>
+      <c r="G18" s="17"/>
+      <c r="H18" s="17"/>
+      <c r="I18" s="17"/>
+      <c r="J18" s="17"/>
     </row>
     <row r="19" spans="1:10">
-      <c r="A19" s="15"/>
-      <c r="B19" s="15"/>
-      <c r="C19" s="15"/>
-      <c r="D19" s="15"/>
-      <c r="E19" s="15"/>
-      <c r="F19" s="15"/>
-      <c r="G19" s="15"/>
-      <c r="H19" s="15"/>
-      <c r="I19" s="15"/>
-      <c r="J19" s="15"/>
+      <c r="A19" s="17"/>
+      <c r="B19" s="17"/>
+      <c r="C19" s="17"/>
+      <c r="D19" s="17"/>
+      <c r="E19" s="17"/>
+      <c r="F19" s="17"/>
+      <c r="G19" s="17"/>
+      <c r="H19" s="17"/>
+      <c r="I19" s="17"/>
+      <c r="J19" s="17"/>
     </row>
     <row r="20" spans="1:10">
-      <c r="A20" s="15"/>
-      <c r="B20" s="15"/>
-      <c r="C20" s="15"/>
-      <c r="D20" s="15"/>
-      <c r="E20" s="15"/>
-      <c r="F20" s="15"/>
-      <c r="G20" s="15"/>
-      <c r="H20" s="15"/>
-      <c r="I20" s="15"/>
-      <c r="J20" s="15"/>
+      <c r="A20" s="17"/>
+      <c r="B20" s="17"/>
+      <c r="C20" s="17"/>
+      <c r="D20" s="17"/>
+      <c r="E20" s="17"/>
+      <c r="F20" s="17"/>
+      <c r="G20" s="17"/>
+      <c r="H20" s="17"/>
+      <c r="I20" s="17"/>
+      <c r="J20" s="17"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1863,552 +1882,552 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:20">
-      <c r="A1" s="2" t="s">
+      <c r="A1" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="B1" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="C1" s="4" t="s">
         <v>27</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="D1" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="E1" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="F1" s="2" t="s">
+      <c r="F1" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="G1" s="2" t="s">
+      <c r="G1" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="H1" s="2" t="s">
+      <c r="H1" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="I1" s="2" t="s">
+      <c r="I1" s="4" t="s">
         <v>31</v>
       </c>
-      <c r="J1" s="2" t="s">
+      <c r="J1" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="K1" s="2" t="s">
+      <c r="K1" s="4" t="s">
         <v>33</v>
       </c>
-      <c r="L1" s="2" t="s">
+      <c r="L1" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="M1" s="2" t="s">
+      <c r="M1" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="N1" s="2" t="s">
+      <c r="N1" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="O1" s="2" t="s">
+      <c r="O1" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="P1" s="2" t="s">
+      <c r="P1" s="4" t="s">
         <v>34</v>
       </c>
-      <c r="Q1" s="2" t="s">
+      <c r="Q1" s="4" t="s">
         <v>35</v>
       </c>
-      <c r="R1" s="2" t="s">
+      <c r="R1" s="4" t="s">
         <v>36</v>
       </c>
-      <c r="S1" s="2" t="s">
+      <c r="S1" s="4" t="s">
         <v>37</v>
       </c>
-      <c r="T1" s="2" t="s">
+      <c r="T1" s="4" t="s">
         <v>38</v>
       </c>
     </row>
     <row r="2" spans="1:20">
-      <c r="A2" s="2" t="s">
+      <c r="A2" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="B2" s="4" t="s">
         <v>39</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="C2" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="D2" s="2" t="s">
+      <c r="D2" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="E2" s="2">
+      <c r="E2" s="4">
         <v>12</v>
       </c>
-      <c r="F2" s="6" t="s">
+      <c r="F2" s="8" t="s">
         <v>12</v>
       </c>
-      <c r="G2" s="2" t="s">
+      <c r="G2" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="H2" s="2" t="s">
+      <c r="H2" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="I2" s="2" t="s">
+      <c r="I2" s="4" t="s">
         <v>41</v>
       </c>
-      <c r="J2" s="2" t="s">
+      <c r="J2" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="K2" s="2">
+      <c r="K2" s="4">
         <v>6</v>
       </c>
-      <c r="L2" s="2">
+      <c r="L2" s="4">
         <v>1010301033</v>
       </c>
-      <c r="M2" s="2" t="s">
+      <c r="M2" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="N2" s="2" t="s">
+      <c r="N2" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="O2" s="2" t="s">
+      <c r="O2" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="P2" s="2"/>
-      <c r="Q2" s="2"/>
-      <c r="R2" s="2"/>
-      <c r="S2" s="2">
+      <c r="P2" s="4"/>
+      <c r="Q2" s="4"/>
+      <c r="R2" s="4"/>
+      <c r="S2" s="4">
         <v>0</v>
       </c>
-      <c r="T2" s="2"/>
+      <c r="T2" s="4"/>
     </row>
     <row r="3" spans="1:20">
-      <c r="A3" s="2" t="s">
+      <c r="A3" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="B3" s="2" t="s">
+      <c r="B3" s="4" t="s">
         <v>42</v>
       </c>
-      <c r="C3" s="2" t="s">
+      <c r="C3" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="D3" s="7" t="s">
+      <c r="D3" s="9" t="s">
         <v>43</v>
       </c>
-      <c r="E3" s="2">
+      <c r="E3" s="4">
         <v>5</v>
       </c>
-      <c r="F3" s="2" t="s">
+      <c r="F3" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="G3" s="2" t="s">
+      <c r="G3" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="H3" s="2" t="s">
+      <c r="H3" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="I3" s="2" t="s">
+      <c r="I3" s="4" t="s">
         <v>44</v>
       </c>
-      <c r="J3" s="2" t="s">
+      <c r="J3" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="K3" s="2">
+      <c r="K3" s="4">
         <v>1</v>
       </c>
-      <c r="L3" s="2">
+      <c r="L3" s="4">
         <v>1010301033</v>
       </c>
-      <c r="M3" s="2" t="s">
+      <c r="M3" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="N3" s="2" t="s">
+      <c r="N3" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="O3" s="2" t="s">
+      <c r="O3" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="P3" s="2"/>
-      <c r="Q3" s="2"/>
-      <c r="R3" s="2"/>
-      <c r="S3" s="2">
+      <c r="P3" s="4"/>
+      <c r="Q3" s="4"/>
+      <c r="R3" s="4"/>
+      <c r="S3" s="4">
         <v>0</v>
       </c>
-      <c r="T3" s="2"/>
+      <c r="T3" s="4"/>
     </row>
     <row r="4" spans="1:20">
-      <c r="A4" s="2" t="s">
+      <c r="A4" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="B4" s="2" t="s">
+      <c r="B4" s="4" t="s">
         <v>45</v>
       </c>
-      <c r="C4" s="2" t="s">
+      <c r="C4" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="D4" s="2">
+      <c r="D4" s="4">
         <v>123562</v>
       </c>
-      <c r="E4" s="2">
+      <c r="E4" s="4">
         <v>18</v>
       </c>
-      <c r="F4" s="2" t="s">
+      <c r="F4" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="G4" s="2" t="s">
+      <c r="G4" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="H4" s="2" t="s">
+      <c r="H4" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="I4" s="2" t="s">
+      <c r="I4" s="4" t="s">
         <v>44</v>
       </c>
-      <c r="J4" s="2" t="s">
+      <c r="J4" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="K4" s="2">
+      <c r="K4" s="4">
         <v>1</v>
       </c>
-      <c r="L4" s="2">
+      <c r="L4" s="4">
         <v>1011134888</v>
       </c>
-      <c r="M4" s="2" t="s">
+      <c r="M4" s="4" t="s">
         <v>46</v>
       </c>
-      <c r="N4" s="2" t="s">
+      <c r="N4" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="O4" s="2" t="s">
+      <c r="O4" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="P4" s="2"/>
-      <c r="Q4" s="2"/>
-      <c r="R4" s="2"/>
-      <c r="S4" s="2">
+      <c r="P4" s="4"/>
+      <c r="Q4" s="4"/>
+      <c r="R4" s="4"/>
+      <c r="S4" s="4">
         <v>0</v>
       </c>
-      <c r="T4" s="2"/>
+      <c r="T4" s="4"/>
     </row>
     <row r="5" spans="1:20">
-      <c r="A5" s="1" t="s">
+      <c r="A5" s="3" t="s">
         <v>47</v>
       </c>
-      <c r="B5" s="1" t="s">
+      <c r="B5" s="3" t="s">
         <v>47</v>
       </c>
-      <c r="C5" s="2" t="s">
+      <c r="C5" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="D5" s="1" t="s">
+      <c r="D5" s="3" t="s">
         <v>40</v>
       </c>
-      <c r="E5" s="1">
+      <c r="E5" s="3">
         <v>12</v>
       </c>
-      <c r="F5" s="1" t="s">
+      <c r="F5" s="3" t="s">
         <v>48</v>
       </c>
-      <c r="G5" s="1" t="s">
+      <c r="G5" s="3" t="s">
         <v>49</v>
       </c>
-      <c r="H5" s="1" t="s">
+      <c r="H5" s="3" t="s">
         <v>50</v>
       </c>
-      <c r="I5" s="1" t="s">
+      <c r="I5" s="3" t="s">
         <v>44</v>
       </c>
-      <c r="J5" s="1" t="s">
+      <c r="J5" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="K5" s="1">
+      <c r="K5" s="3">
         <v>1</v>
       </c>
-      <c r="L5" s="1">
+      <c r="L5" s="3">
         <v>1010301001</v>
       </c>
-      <c r="M5" s="1" t="s">
+      <c r="M5" s="3" t="s">
         <v>51</v>
       </c>
-      <c r="N5" s="1" t="s">
+      <c r="N5" s="3" t="s">
         <v>52</v>
       </c>
-      <c r="O5" s="1" t="s">
+      <c r="O5" s="3" t="s">
         <v>53</v>
       </c>
-      <c r="P5" s="1"/>
-      <c r="Q5" s="1"/>
-      <c r="R5" s="1"/>
-      <c r="S5" s="2">
+      <c r="P5" s="3"/>
+      <c r="Q5" s="3"/>
+      <c r="R5" s="3"/>
+      <c r="S5" s="4">
         <v>0</v>
       </c>
-      <c r="T5" s="1"/>
+      <c r="T5" s="3"/>
     </row>
     <row r="6" spans="1:20">
-      <c r="A6" s="1" t="s">
+      <c r="A6" s="3" t="s">
         <v>54</v>
       </c>
-      <c r="B6" s="1" t="s">
+      <c r="B6" s="3" t="s">
         <v>54</v>
       </c>
-      <c r="C6" s="1" t="s">
+      <c r="C6" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="D6" s="5" t="s">
+      <c r="D6" s="7" t="s">
         <v>43</v>
       </c>
       <c r="E6">
         <v>5</v>
       </c>
-      <c r="F6" s="8" t="s">
+      <c r="F6" s="10" t="s">
         <v>12</v>
       </c>
-      <c r="G6" s="8" t="s">
+      <c r="G6" s="10" t="s">
         <v>11</v>
       </c>
-      <c r="H6" s="1" t="s">
+      <c r="H6" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="I6" s="1" t="s">
+      <c r="I6" s="3" t="s">
         <v>44</v>
       </c>
-      <c r="J6" s="1" t="s">
+      <c r="J6" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="K6" s="1">
+      <c r="K6" s="3">
         <v>1</v>
       </c>
-      <c r="L6" s="1">
+      <c r="L6" s="3">
         <v>1010301033</v>
       </c>
-      <c r="M6" s="1" t="s">
+      <c r="M6" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="N6" s="1" t="s">
+      <c r="N6" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="O6" s="1" t="s">
+      <c r="O6" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="P6" s="1"/>
-      <c r="Q6" s="1"/>
-      <c r="R6" s="1"/>
-      <c r="S6" s="2">
+      <c r="P6" s="3"/>
+      <c r="Q6" s="3"/>
+      <c r="R6" s="3"/>
+      <c r="S6" s="4">
         <v>0</v>
       </c>
-      <c r="T6" s="1"/>
+      <c r="T6" s="3"/>
     </row>
     <row r="7" spans="1:20">
-      <c r="A7" s="9" t="s">
+      <c r="A7" s="11" t="s">
         <v>55</v>
       </c>
-      <c r="B7" s="9" t="s">
+      <c r="B7" s="11" t="s">
         <v>56</v>
       </c>
-      <c r="C7" s="9" t="s">
+      <c r="C7" s="11" t="s">
         <v>20</v>
       </c>
-      <c r="D7" s="9" t="s">
+      <c r="D7" s="11" t="s">
         <v>40</v>
       </c>
-      <c r="E7" s="9">
+      <c r="E7" s="11">
         <v>12</v>
       </c>
-      <c r="F7" s="10" t="s">
+      <c r="F7" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="G7" s="9" t="s">
+      <c r="G7" s="11" t="s">
         <v>11</v>
       </c>
-      <c r="H7" s="9" t="s">
+      <c r="H7" s="11" t="s">
         <v>57</v>
       </c>
-      <c r="I7" s="9" t="s">
+      <c r="I7" s="11" t="s">
         <v>41</v>
       </c>
-      <c r="J7" s="9" t="s">
+      <c r="J7" s="11" t="s">
         <v>14</v>
       </c>
-      <c r="K7" s="9">
+      <c r="K7" s="11">
         <v>3</v>
       </c>
-      <c r="L7" s="9">
+      <c r="L7" s="11">
         <v>1010301003</v>
       </c>
-      <c r="M7" s="9" t="s">
+      <c r="M7" s="11" t="s">
         <v>58</v>
       </c>
-      <c r="N7" s="9" t="s">
+      <c r="N7" s="11" t="s">
         <v>16</v>
       </c>
-      <c r="O7" s="9" t="s">
+      <c r="O7" s="11" t="s">
         <v>17</v>
       </c>
-      <c r="P7" s="9"/>
-      <c r="Q7" s="9"/>
-      <c r="R7" s="9"/>
-      <c r="S7" s="9">
+      <c r="P7" s="11"/>
+      <c r="Q7" s="11"/>
+      <c r="R7" s="11"/>
+      <c r="S7" s="11">
         <v>0</v>
       </c>
-      <c r="T7" s="9"/>
+      <c r="T7" s="11"/>
     </row>
     <row r="8" spans="1:20">
-      <c r="A8" s="9" t="s">
+      <c r="A8" s="11" t="s">
         <v>59</v>
       </c>
-      <c r="B8" s="9" t="s">
+      <c r="B8" s="11" t="s">
         <v>60</v>
       </c>
-      <c r="C8" s="9" t="s">
+      <c r="C8" s="11" t="s">
         <v>14</v>
       </c>
-      <c r="D8" s="9" t="s">
+      <c r="D8" s="11" t="s">
         <v>43</v>
       </c>
-      <c r="E8" s="9">
+      <c r="E8" s="11">
         <v>5</v>
       </c>
-      <c r="F8" s="10" t="s">
+      <c r="F8" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="G8" s="9" t="s">
+      <c r="G8" s="11" t="s">
         <v>11</v>
       </c>
-      <c r="H8" s="9" t="s">
+      <c r="H8" s="11" t="s">
         <v>57</v>
       </c>
-      <c r="I8" s="9" t="s">
+      <c r="I8" s="11" t="s">
         <v>41</v>
       </c>
-      <c r="J8" s="9" t="s">
+      <c r="J8" s="11" t="s">
         <v>14</v>
       </c>
-      <c r="K8" s="9">
+      <c r="K8" s="11">
         <v>0</v>
       </c>
-      <c r="L8" s="9">
+      <c r="L8" s="11">
         <v>1010301003</v>
       </c>
-      <c r="M8" s="9" t="s">
+      <c r="M8" s="11" t="s">
         <v>58</v>
       </c>
-      <c r="N8" s="9" t="s">
+      <c r="N8" s="11" t="s">
         <v>16</v>
       </c>
-      <c r="O8" s="9" t="s">
+      <c r="O8" s="11" t="s">
         <v>17</v>
       </c>
-      <c r="P8" s="9"/>
-      <c r="Q8" s="9"/>
-      <c r="R8" s="9"/>
-      <c r="S8" s="9">
+      <c r="P8" s="11"/>
+      <c r="Q8" s="11"/>
+      <c r="R8" s="11"/>
+      <c r="S8" s="11">
         <v>0</v>
       </c>
-      <c r="T8" s="9"/>
+      <c r="T8" s="11"/>
     </row>
     <row r="9" spans="1:20">
-      <c r="A9" s="9" t="s">
+      <c r="A9" s="11" t="s">
         <v>61</v>
       </c>
-      <c r="B9" s="9" t="s">
+      <c r="B9" s="11" t="s">
         <v>61</v>
       </c>
-      <c r="C9" s="9" t="s">
+      <c r="C9" s="11" t="s">
         <v>14</v>
       </c>
-      <c r="D9" s="9" t="s">
+      <c r="D9" s="11" t="s">
         <v>43</v>
       </c>
-      <c r="E9" s="9">
+      <c r="E9" s="11">
         <v>5</v>
       </c>
-      <c r="F9" s="10" t="s">
+      <c r="F9" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="G9" s="9" t="s">
+      <c r="G9" s="11" t="s">
         <v>11</v>
       </c>
-      <c r="H9" s="9" t="s">
+      <c r="H9" s="11" t="s">
         <v>57</v>
       </c>
-      <c r="I9" s="9" t="s">
+      <c r="I9" s="11" t="s">
         <v>41</v>
       </c>
-      <c r="J9" s="9" t="s">
+      <c r="J9" s="11" t="s">
         <v>14</v>
       </c>
-      <c r="K9" s="9">
+      <c r="K9" s="11">
         <v>0</v>
       </c>
-      <c r="L9" s="9">
+      <c r="L9" s="11">
         <v>1010301003</v>
       </c>
-      <c r="M9" s="9" t="s">
+      <c r="M9" s="11" t="s">
         <v>58</v>
       </c>
-      <c r="N9" s="9" t="s">
+      <c r="N9" s="11" t="s">
         <v>16</v>
       </c>
-      <c r="O9" s="9" t="s">
+      <c r="O9" s="11" t="s">
         <v>17</v>
       </c>
-      <c r="P9" s="9"/>
-      <c r="Q9" s="9"/>
-      <c r="R9" s="9"/>
-      <c r="S9" s="9">
+      <c r="P9" s="11"/>
+      <c r="Q9" s="11"/>
+      <c r="R9" s="11"/>
+      <c r="S9" s="11">
         <v>0</v>
       </c>
-      <c r="T9" s="9"/>
+      <c r="T9" s="11"/>
     </row>
     <row r="10" spans="1:20">
-      <c r="A10" s="1" t="s">
+      <c r="A10" s="3" t="s">
         <v>62</v>
       </c>
-      <c r="B10" s="1" t="s">
+      <c r="B10" s="3" t="s">
         <v>62</v>
       </c>
-      <c r="C10" s="1" t="s">
+      <c r="C10" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="D10" s="9" t="s">
+      <c r="D10" s="11" t="s">
         <v>43</v>
       </c>
-      <c r="E10" s="9">
+      <c r="E10" s="11">
         <v>5</v>
       </c>
-      <c r="F10" s="2" t="s">
+      <c r="F10" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="G10" s="2" t="s">
+      <c r="G10" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="H10" s="2" t="s">
+      <c r="H10" s="4" t="s">
         <v>63</v>
       </c>
-      <c r="I10" s="2" t="s">
+      <c r="I10" s="4" t="s">
         <v>44</v>
       </c>
-      <c r="J10" s="2" t="s">
+      <c r="J10" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="K10" s="2">
+      <c r="K10" s="4">
         <v>1</v>
       </c>
-      <c r="L10" s="3">
+      <c r="L10" s="5">
         <v>1000000001</v>
       </c>
-      <c r="M10" s="1" t="s">
+      <c r="M10" s="3" t="s">
         <v>64</v>
       </c>
-      <c r="N10" s="1" t="s">
+      <c r="N10" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="O10" s="1" t="s">
+      <c r="O10" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="P10" s="9"/>
-      <c r="Q10" s="9"/>
-      <c r="R10" s="9"/>
-      <c r="S10" s="9">
+      <c r="P10" s="11"/>
+      <c r="Q10" s="11"/>
+      <c r="R10" s="11"/>
+      <c r="S10" s="11">
         <v>0</v>
       </c>
-      <c r="T10" s="9"/>
+      <c r="T10" s="11"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2436,129 +2455,190 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:18">
+      <c r="A1" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="D1" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="E1" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="F1" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="G1" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="H1" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="I1" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="J1" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="K1" s="3" t="s">
+        <v>65</v>
+      </c>
+      <c r="L1" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="M1" s="6"/>
+      <c r="N1" s="6"/>
+      <c r="O1" s="6"/>
+      <c r="P1" s="6"/>
+      <c r="Q1" s="6"/>
+      <c r="R1" s="6"/>
+    </row>
+    <row r="2" spans="1:18">
+      <c r="A2" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="D2" s="3">
+        <v>1010301033</v>
+      </c>
+      <c r="E2" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="F2" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="G2" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="H2" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="I2" s="7" t="s">
+        <v>43</v>
+      </c>
+      <c r="J2" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="K2" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="L2" s="3">
+        <v>1</v>
+      </c>
+      <c r="M2" s="6"/>
+      <c r="N2" s="6"/>
+      <c r="O2" s="6"/>
+      <c r="P2" s="6"/>
+      <c r="Q2" s="6"/>
+      <c r="R2" s="6"/>
+    </row>
+    <row r="3" spans="1:12">
+      <c r="A3" s="3" t="s">
+        <v>62</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>62</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="D3" s="5">
+        <v>1000000001</v>
+      </c>
+      <c r="E3" s="3" t="s">
+        <v>64</v>
+      </c>
+      <c r="F3" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="G3" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="H3" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="I3" s="7" t="s">
+        <v>43</v>
+      </c>
+      <c r="J3" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="K3" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="L3" s="3">
+        <v>1</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <headerFooter/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
+  <dimension ref="A1:C4"/>
+  <sheetFormatPr defaultColWidth="8.88888888888889" defaultRowHeight="14.4" outlineLevelRow="3" outlineLevelCol="2"/>
+  <cols>
+    <col min="1" max="1" width="27.1111111111111" customWidth="1"/>
+    <col min="2" max="2" width="10.4444444444444" customWidth="1"/>
+    <col min="3" max="3" width="11.4444444444444" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3">
       <c r="A1" s="1" t="s">
-        <v>25</v>
+        <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3">
+      <c r="A2" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="B2" s="3">
+        <v>30</v>
+      </c>
+      <c r="C2" s="3">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3">
+      <c r="A3" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="B3" s="3">
+        <v>40</v>
+      </c>
+      <c r="C3" s="3">
         <v>26</v>
       </c>
-      <c r="C1" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="D1" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="E1" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="F1" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="G1" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="I1" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="J1" s="1" t="s">
-        <v>31</v>
-      </c>
-      <c r="K1" s="1" t="s">
-        <v>65</v>
-      </c>
-      <c r="L1" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="M1" s="4"/>
-      <c r="N1" s="4"/>
-      <c r="O1" s="4"/>
-      <c r="P1" s="4"/>
-      <c r="Q1" s="4"/>
-      <c r="R1" s="4"/>
-    </row>
-    <row r="2" spans="1:18">
-      <c r="A2" s="1" t="s">
-        <v>54</v>
-      </c>
-      <c r="B2" s="1" t="s">
-        <v>54</v>
-      </c>
-      <c r="C2" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="D2" s="1">
-        <v>1010301033</v>
-      </c>
-      <c r="E2" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="F2" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="G2" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="H2" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="I2" s="5" t="s">
-        <v>43</v>
-      </c>
-      <c r="J2" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="K2" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="L2" s="1">
-        <v>1</v>
-      </c>
-      <c r="M2" s="4"/>
-      <c r="N2" s="4"/>
-      <c r="O2" s="4"/>
-      <c r="P2" s="4"/>
-      <c r="Q2" s="4"/>
-      <c r="R2" s="4"/>
-    </row>
-    <row r="3" spans="1:12">
-      <c r="A3" s="1" t="s">
-        <v>62</v>
-      </c>
-      <c r="B3" s="1" t="s">
-        <v>62</v>
-      </c>
-      <c r="C3" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="D3" s="3">
-        <v>1000000001</v>
-      </c>
-      <c r="E3" s="1" t="s">
-        <v>64</v>
-      </c>
-      <c r="F3" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="G3" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="H3" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="I3" s="5" t="s">
-        <v>43</v>
-      </c>
-      <c r="J3" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="K3" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="L3" s="1">
-        <v>1</v>
+    </row>
+    <row r="4" spans="1:3">
+      <c r="A4" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="B4" s="3">
+        <v>50</v>
+      </c>
+      <c r="C4" s="3">
+        <v>70</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Added Price List And GRN Test Scenarios And Fixed PO Test Scenarios
Added Price List And GRN Test Scenarios And Fixed PO Test Scenarios
</commit_message>
<xml_diff>
--- a/testdata/ItemDetails.xlsx
+++ b/testdata/ItemDetails.xlsx
@@ -4,13 +4,17 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="23040" windowHeight="9120" activeTab="3"/>
+    <workbookView windowWidth="23040" windowHeight="9120" firstSheet="3" activeTab="4"/>
   </bookViews>
   <sheets>
     <sheet name="PR Details" sheetId="1" r:id="rId1"/>
     <sheet name="PO Details" sheetId="2" r:id="rId2"/>
     <sheet name="POA Details" sheetId="3" r:id="rId3"/>
-    <sheet name="PO MULTIPLE ITEM" sheetId="4" r:id="rId4"/>
+    <sheet name="PO _ITEM_MATERIAL" sheetId="4" r:id="rId4"/>
+    <sheet name="PO _ITEM_GEN" sheetId="8" r:id="rId5"/>
+    <sheet name="StockTransferItem" sheetId="5" r:id="rId6"/>
+    <sheet name="POwithRateContractItem" sheetId="6" r:id="rId7"/>
+    <sheet name="POwithRateContractItem_Mat" sheetId="7" r:id="rId8"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -30,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="199" uniqueCount="68">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="257" uniqueCount="91">
   <si>
     <t>ITEM_NAME</t>
   </si>
@@ -235,6 +239,75 @@
   </si>
   <si>
     <t>UNIT_COST</t>
+  </si>
+  <si>
+    <t>LOT_SERIAL</t>
+  </si>
+  <si>
+    <t>LOT_NUMBER</t>
+  </si>
+  <si>
+    <t>SERIAL_NUMBER</t>
+  </si>
+  <si>
+    <t>SERIAL</t>
+  </si>
+  <si>
+    <t>RM1</t>
+  </si>
+  <si>
+    <t>LOT</t>
+  </si>
+  <si>
+    <t>RM</t>
+  </si>
+  <si>
+    <t>RMG</t>
+  </si>
+  <si>
+    <t>HK-NA-MAC-10001</t>
+  </si>
+  <si>
+    <t>NA</t>
+  </si>
+  <si>
+    <t>Stock_Transfer_Item</t>
+  </si>
+  <si>
+    <t>QTY</t>
+  </si>
+  <si>
+    <t>UnitCost</t>
+  </si>
+  <si>
+    <t>TVS FG-MAC-NA-USER DEFINED</t>
+  </si>
+  <si>
+    <t>TVS-FG-00015</t>
+  </si>
+  <si>
+    <t>RateContractItem</t>
+  </si>
+  <si>
+    <t>Quantity</t>
+  </si>
+  <si>
+    <t>DiscountPercentage</t>
+  </si>
+  <si>
+    <t>PK-SER-MAC-10001</t>
+  </si>
+  <si>
+    <t>RMS</t>
+  </si>
+  <si>
+    <t>PK-LOT-MAC-10001</t>
+  </si>
+  <si>
+    <t>RML</t>
+  </si>
+  <si>
+    <t>PK-NA-MAC-10001</t>
   </si>
 </sst>
 </file>
@@ -247,19 +320,13 @@
     <numFmt numFmtId="178" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
     <numFmt numFmtId="179" formatCode="_ &quot;₹&quot;* #,##0_ ;_ &quot;₹&quot;* \-#,##0_ ;_ &quot;₹&quot;* &quot;-&quot;_ ;_ @_ "/>
   </numFmts>
-  <fonts count="28">
+  <fonts count="27">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <charset val="134"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <color theme="1"/>
-      <name val="Times New Roman"/>
-      <charset val="134"/>
     </font>
     <font>
       <sz val="10"/>
@@ -791,156 +858,159 @@
     <xf numFmtId="179" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="2" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="2" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="4" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="5" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="5" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="6" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="4" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="5" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="5" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="6" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1">
@@ -949,34 +1019,34 @@
     <xf numFmtId="49" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="49" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="49" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="49" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="49" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="justify" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -1528,324 +1598,324 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10">
-      <c r="A1" s="14" t="s">
+      <c r="A1" s="15" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="14" t="s">
+      <c r="B1" s="15" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="14" t="s">
+      <c r="C1" s="15" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="14" t="s">
+      <c r="D1" s="15" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="14" t="s">
+      <c r="E1" s="15" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="14" t="s">
+      <c r="F1" s="15" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="14" t="s">
+      <c r="G1" s="15" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="14" t="s">
+      <c r="H1" s="15" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="14" t="s">
+      <c r="I1" s="15" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="14" t="s">
+      <c r="J1" s="15" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="2" s="13" customFormat="1" ht="20.4" spans="1:10">
-      <c r="A2" s="15" t="s">
+    <row r="2" s="14" customFormat="1" ht="20.4" spans="1:10">
+      <c r="A2" s="16" t="s">
         <v>10</v>
       </c>
-      <c r="B2" s="16" t="s">
+      <c r="B2" s="17" t="s">
         <v>11</v>
       </c>
-      <c r="C2" s="16" t="s">
+      <c r="C2" s="17" t="s">
         <v>12</v>
       </c>
-      <c r="D2" s="15" t="s">
+      <c r="D2" s="16" t="s">
         <v>13</v>
       </c>
-      <c r="E2" s="15">
+      <c r="E2" s="16">
         <v>1</v>
       </c>
-      <c r="F2" s="15" t="s">
+      <c r="F2" s="16" t="s">
         <v>14</v>
       </c>
-      <c r="G2" s="15">
+      <c r="G2" s="16">
         <v>1010301033</v>
       </c>
-      <c r="H2" s="15" t="s">
+      <c r="H2" s="16" t="s">
         <v>15</v>
       </c>
-      <c r="I2" s="15" t="s">
+      <c r="I2" s="16" t="s">
         <v>16</v>
       </c>
-      <c r="J2" s="15" t="s">
+      <c r="J2" s="16" t="s">
         <v>17</v>
       </c>
     </row>
     <row r="3" ht="15" customHeight="1" spans="1:10">
-      <c r="A3" s="15" t="s">
+      <c r="A3" s="16" t="s">
         <v>18</v>
       </c>
-      <c r="B3" s="16" t="s">
+      <c r="B3" s="17" t="s">
         <v>11</v>
       </c>
-      <c r="C3" s="16" t="s">
+      <c r="C3" s="17" t="s">
         <v>12</v>
       </c>
-      <c r="D3" s="15" t="s">
+      <c r="D3" s="16" t="s">
         <v>19</v>
       </c>
-      <c r="E3" s="15">
+      <c r="E3" s="16">
         <v>6</v>
       </c>
-      <c r="F3" s="16" t="s">
+      <c r="F3" s="17" t="s">
         <v>20</v>
       </c>
-      <c r="G3" s="15">
+      <c r="G3" s="16">
         <v>1010301033</v>
       </c>
-      <c r="H3" s="15" t="s">
+      <c r="H3" s="16" t="s">
         <v>15</v>
       </c>
-      <c r="I3" s="15" t="s">
+      <c r="I3" s="16" t="s">
         <v>16</v>
       </c>
-      <c r="J3" s="15" t="s">
+      <c r="J3" s="16" t="s">
         <v>17</v>
       </c>
     </row>
     <row r="4" spans="1:10">
-      <c r="A4" s="15" t="s">
+      <c r="A4" s="16" t="s">
         <v>21</v>
       </c>
-      <c r="B4" s="16" t="s">
+      <c r="B4" s="17" t="s">
         <v>22</v>
       </c>
-      <c r="C4" s="16" t="s">
+      <c r="C4" s="17" t="s">
         <v>22</v>
       </c>
-      <c r="D4" s="15" t="s">
+      <c r="D4" s="16" t="s">
         <v>23</v>
       </c>
-      <c r="E4" s="15">
+      <c r="E4" s="16">
         <v>1</v>
       </c>
-      <c r="F4" s="16" t="s">
+      <c r="F4" s="17" t="s">
         <v>14</v>
       </c>
-      <c r="G4" s="15">
+      <c r="G4" s="16">
         <v>5010101060</v>
       </c>
-      <c r="H4" s="15" t="s">
+      <c r="H4" s="16" t="s">
         <v>24</v>
       </c>
-      <c r="I4" s="15" t="s">
+      <c r="I4" s="16" t="s">
         <v>16</v>
       </c>
-      <c r="J4" s="15" t="s">
+      <c r="J4" s="16" t="s">
         <v>17</v>
       </c>
     </row>
     <row r="5" spans="1:10">
-      <c r="A5" s="17"/>
-      <c r="B5" s="17"/>
-      <c r="C5" s="17"/>
-      <c r="D5" s="17"/>
-      <c r="E5" s="17"/>
-      <c r="F5" s="17"/>
-      <c r="G5" s="17"/>
-      <c r="H5" s="17"/>
-      <c r="I5" s="17"/>
-      <c r="J5" s="17"/>
+      <c r="A5" s="18"/>
+      <c r="B5" s="18"/>
+      <c r="C5" s="18"/>
+      <c r="D5" s="18"/>
+      <c r="E5" s="18"/>
+      <c r="F5" s="18"/>
+      <c r="G5" s="18"/>
+      <c r="H5" s="18"/>
+      <c r="I5" s="18"/>
+      <c r="J5" s="18"/>
     </row>
     <row r="6" spans="1:10">
-      <c r="A6" s="17"/>
-      <c r="B6" s="17"/>
-      <c r="C6" s="17"/>
-      <c r="D6" s="17"/>
-      <c r="E6" s="17"/>
-      <c r="F6" s="17"/>
-      <c r="G6" s="17"/>
-      <c r="H6" s="17"/>
-      <c r="I6" s="17"/>
-      <c r="J6" s="17"/>
+      <c r="A6" s="18"/>
+      <c r="B6" s="18"/>
+      <c r="C6" s="18"/>
+      <c r="D6" s="18"/>
+      <c r="E6" s="18"/>
+      <c r="F6" s="18"/>
+      <c r="G6" s="18"/>
+      <c r="H6" s="18"/>
+      <c r="I6" s="18"/>
+      <c r="J6" s="18"/>
     </row>
     <row r="7" spans="1:10">
-      <c r="A7" s="17"/>
-      <c r="B7" s="17"/>
-      <c r="C7" s="17"/>
-      <c r="D7" s="17"/>
-      <c r="E7" s="17"/>
-      <c r="F7" s="17"/>
-      <c r="G7" s="17"/>
-      <c r="H7" s="17"/>
-      <c r="I7" s="17"/>
-      <c r="J7" s="17"/>
+      <c r="A7" s="18"/>
+      <c r="B7" s="18"/>
+      <c r="C7" s="18"/>
+      <c r="D7" s="18"/>
+      <c r="E7" s="18"/>
+      <c r="F7" s="18"/>
+      <c r="G7" s="18"/>
+      <c r="H7" s="18"/>
+      <c r="I7" s="18"/>
+      <c r="J7" s="18"/>
     </row>
     <row r="8" spans="1:10">
-      <c r="A8" s="17"/>
-      <c r="B8" s="17"/>
-      <c r="C8" s="17"/>
-      <c r="D8" s="17"/>
-      <c r="E8" s="17"/>
-      <c r="F8" s="17"/>
-      <c r="G8" s="17"/>
-      <c r="H8" s="17"/>
-      <c r="I8" s="17"/>
-      <c r="J8" s="17"/>
+      <c r="A8" s="18"/>
+      <c r="B8" s="18"/>
+      <c r="C8" s="18"/>
+      <c r="D8" s="18"/>
+      <c r="E8" s="18"/>
+      <c r="F8" s="18"/>
+      <c r="G8" s="18"/>
+      <c r="H8" s="18"/>
+      <c r="I8" s="18"/>
+      <c r="J8" s="18"/>
     </row>
     <row r="9" spans="1:10">
-      <c r="A9" s="17"/>
-      <c r="B9" s="17"/>
-      <c r="C9" s="17"/>
-      <c r="D9" s="17"/>
-      <c r="E9" s="17"/>
-      <c r="F9" s="17"/>
-      <c r="G9" s="17"/>
-      <c r="H9" s="17"/>
-      <c r="I9" s="17"/>
-      <c r="J9" s="17"/>
+      <c r="A9" s="18"/>
+      <c r="B9" s="18"/>
+      <c r="C9" s="18"/>
+      <c r="D9" s="18"/>
+      <c r="E9" s="18"/>
+      <c r="F9" s="18"/>
+      <c r="G9" s="18"/>
+      <c r="H9" s="18"/>
+      <c r="I9" s="18"/>
+      <c r="J9" s="18"/>
     </row>
     <row r="10" spans="1:10">
-      <c r="A10" s="17"/>
-      <c r="B10" s="17"/>
-      <c r="C10" s="17"/>
-      <c r="D10" s="17"/>
-      <c r="E10" s="17"/>
-      <c r="F10" s="17"/>
-      <c r="G10" s="17"/>
-      <c r="H10" s="17"/>
-      <c r="I10" s="17"/>
-      <c r="J10" s="17"/>
+      <c r="A10" s="18"/>
+      <c r="B10" s="18"/>
+      <c r="C10" s="18"/>
+      <c r="D10" s="18"/>
+      <c r="E10" s="18"/>
+      <c r="F10" s="18"/>
+      <c r="G10" s="18"/>
+      <c r="H10" s="18"/>
+      <c r="I10" s="18"/>
+      <c r="J10" s="18"/>
     </row>
     <row r="11" spans="1:10">
-      <c r="A11" s="17"/>
-      <c r="B11" s="17"/>
-      <c r="C11" s="17"/>
-      <c r="D11" s="17"/>
-      <c r="E11" s="17"/>
-      <c r="F11" s="17"/>
-      <c r="G11" s="17"/>
-      <c r="H11" s="17"/>
-      <c r="I11" s="17"/>
-      <c r="J11" s="17"/>
+      <c r="A11" s="18"/>
+      <c r="B11" s="18"/>
+      <c r="C11" s="18"/>
+      <c r="D11" s="18"/>
+      <c r="E11" s="18"/>
+      <c r="F11" s="18"/>
+      <c r="G11" s="18"/>
+      <c r="H11" s="18"/>
+      <c r="I11" s="18"/>
+      <c r="J11" s="18"/>
     </row>
     <row r="12" spans="1:10">
-      <c r="A12" s="17"/>
-      <c r="B12" s="17"/>
-      <c r="C12" s="17"/>
-      <c r="D12" s="17"/>
-      <c r="E12" s="17"/>
-      <c r="F12" s="17"/>
-      <c r="G12" s="17"/>
-      <c r="H12" s="17"/>
-      <c r="I12" s="17"/>
-      <c r="J12" s="17"/>
+      <c r="A12" s="18"/>
+      <c r="B12" s="18"/>
+      <c r="C12" s="18"/>
+      <c r="D12" s="18"/>
+      <c r="E12" s="18"/>
+      <c r="F12" s="18"/>
+      <c r="G12" s="18"/>
+      <c r="H12" s="18"/>
+      <c r="I12" s="18"/>
+      <c r="J12" s="18"/>
     </row>
     <row r="13" spans="1:10">
-      <c r="A13" s="17"/>
-      <c r="B13" s="17"/>
-      <c r="C13" s="17"/>
-      <c r="D13" s="17"/>
-      <c r="E13" s="17"/>
-      <c r="F13" s="17"/>
-      <c r="G13" s="17"/>
-      <c r="H13" s="17"/>
-      <c r="I13" s="17"/>
-      <c r="J13" s="17"/>
+      <c r="A13" s="18"/>
+      <c r="B13" s="18"/>
+      <c r="C13" s="18"/>
+      <c r="D13" s="18"/>
+      <c r="E13" s="18"/>
+      <c r="F13" s="18"/>
+      <c r="G13" s="18"/>
+      <c r="H13" s="18"/>
+      <c r="I13" s="18"/>
+      <c r="J13" s="18"/>
     </row>
     <row r="14" spans="1:10">
-      <c r="A14" s="17"/>
-      <c r="B14" s="17"/>
-      <c r="C14" s="17"/>
-      <c r="D14" s="17"/>
-      <c r="E14" s="17"/>
-      <c r="F14" s="17"/>
-      <c r="G14" s="17"/>
-      <c r="H14" s="17"/>
-      <c r="I14" s="17"/>
-      <c r="J14" s="17"/>
+      <c r="A14" s="18"/>
+      <c r="B14" s="18"/>
+      <c r="C14" s="18"/>
+      <c r="D14" s="18"/>
+      <c r="E14" s="18"/>
+      <c r="F14" s="18"/>
+      <c r="G14" s="18"/>
+      <c r="H14" s="18"/>
+      <c r="I14" s="18"/>
+      <c r="J14" s="18"/>
     </row>
     <row r="15" spans="1:10">
-      <c r="A15" s="17"/>
-      <c r="B15" s="17"/>
-      <c r="C15" s="17"/>
-      <c r="D15" s="17"/>
-      <c r="E15" s="17"/>
-      <c r="F15" s="17"/>
-      <c r="G15" s="17"/>
-      <c r="H15" s="17"/>
-      <c r="I15" s="17"/>
-      <c r="J15" s="17"/>
+      <c r="A15" s="18"/>
+      <c r="B15" s="18"/>
+      <c r="C15" s="18"/>
+      <c r="D15" s="18"/>
+      <c r="E15" s="18"/>
+      <c r="F15" s="18"/>
+      <c r="G15" s="18"/>
+      <c r="H15" s="18"/>
+      <c r="I15" s="18"/>
+      <c r="J15" s="18"/>
     </row>
     <row r="16" spans="1:10">
-      <c r="A16" s="17"/>
-      <c r="B16" s="17"/>
-      <c r="C16" s="17"/>
-      <c r="D16" s="17"/>
-      <c r="E16" s="17"/>
-      <c r="F16" s="17"/>
-      <c r="G16" s="17"/>
-      <c r="H16" s="17"/>
-      <c r="I16" s="17"/>
-      <c r="J16" s="17"/>
+      <c r="A16" s="18"/>
+      <c r="B16" s="18"/>
+      <c r="C16" s="18"/>
+      <c r="D16" s="18"/>
+      <c r="E16" s="18"/>
+      <c r="F16" s="18"/>
+      <c r="G16" s="18"/>
+      <c r="H16" s="18"/>
+      <c r="I16" s="18"/>
+      <c r="J16" s="18"/>
     </row>
     <row r="17" spans="1:10">
-      <c r="A17" s="17"/>
-      <c r="B17" s="17"/>
-      <c r="C17" s="17"/>
-      <c r="D17" s="17"/>
-      <c r="E17" s="17"/>
-      <c r="F17" s="17"/>
-      <c r="G17" s="17"/>
-      <c r="H17" s="17"/>
-      <c r="I17" s="17"/>
-      <c r="J17" s="17"/>
+      <c r="A17" s="18"/>
+      <c r="B17" s="18"/>
+      <c r="C17" s="18"/>
+      <c r="D17" s="18"/>
+      <c r="E17" s="18"/>
+      <c r="F17" s="18"/>
+      <c r="G17" s="18"/>
+      <c r="H17" s="18"/>
+      <c r="I17" s="18"/>
+      <c r="J17" s="18"/>
     </row>
     <row r="18" spans="1:10">
-      <c r="A18" s="17"/>
-      <c r="B18" s="17"/>
-      <c r="C18" s="17"/>
-      <c r="D18" s="17"/>
-      <c r="E18" s="17"/>
-      <c r="F18" s="17"/>
-      <c r="G18" s="17"/>
-      <c r="H18" s="17"/>
-      <c r="I18" s="17"/>
-      <c r="J18" s="17"/>
+      <c r="A18" s="18"/>
+      <c r="B18" s="18"/>
+      <c r="C18" s="18"/>
+      <c r="D18" s="18"/>
+      <c r="E18" s="18"/>
+      <c r="F18" s="18"/>
+      <c r="G18" s="18"/>
+      <c r="H18" s="18"/>
+      <c r="I18" s="18"/>
+      <c r="J18" s="18"/>
     </row>
     <row r="19" spans="1:10">
-      <c r="A19" s="17"/>
-      <c r="B19" s="17"/>
-      <c r="C19" s="17"/>
-      <c r="D19" s="17"/>
-      <c r="E19" s="17"/>
-      <c r="F19" s="17"/>
-      <c r="G19" s="17"/>
-      <c r="H19" s="17"/>
-      <c r="I19" s="17"/>
-      <c r="J19" s="17"/>
+      <c r="A19" s="18"/>
+      <c r="B19" s="18"/>
+      <c r="C19" s="18"/>
+      <c r="D19" s="18"/>
+      <c r="E19" s="18"/>
+      <c r="F19" s="18"/>
+      <c r="G19" s="18"/>
+      <c r="H19" s="18"/>
+      <c r="I19" s="18"/>
+      <c r="J19" s="18"/>
     </row>
     <row r="20" spans="1:10">
-      <c r="A20" s="17"/>
-      <c r="B20" s="17"/>
-      <c r="C20" s="17"/>
-      <c r="D20" s="17"/>
-      <c r="E20" s="17"/>
-      <c r="F20" s="17"/>
-      <c r="G20" s="17"/>
-      <c r="H20" s="17"/>
-      <c r="I20" s="17"/>
-      <c r="J20" s="17"/>
+      <c r="A20" s="18"/>
+      <c r="B20" s="18"/>
+      <c r="C20" s="18"/>
+      <c r="D20" s="18"/>
+      <c r="E20" s="18"/>
+      <c r="F20" s="18"/>
+      <c r="G20" s="18"/>
+      <c r="H20" s="18"/>
+      <c r="I20" s="18"/>
+      <c r="J20" s="18"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1882,228 +1952,228 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:20">
-      <c r="A1" s="4" t="s">
+      <c r="A1" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="B1" s="4" t="s">
+      <c r="B1" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="C1" s="4" t="s">
+      <c r="C1" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="D1" s="4" t="s">
+      <c r="D1" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="E1" s="4" t="s">
+      <c r="E1" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="F1" s="4" t="s">
+      <c r="F1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="G1" s="4" t="s">
+      <c r="G1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="H1" s="4" t="s">
+      <c r="H1" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="I1" s="4" t="s">
+      <c r="I1" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="J1" s="4" t="s">
+      <c r="J1" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="K1" s="4" t="s">
+      <c r="K1" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="L1" s="4" t="s">
+      <c r="L1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="M1" s="4" t="s">
+      <c r="M1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="N1" s="4" t="s">
+      <c r="N1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="O1" s="4" t="s">
+      <c r="O1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="P1" s="4" t="s">
+      <c r="P1" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="Q1" s="4" t="s">
+      <c r="Q1" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="R1" s="4" t="s">
+      <c r="R1" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="S1" s="4" t="s">
+      <c r="S1" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="T1" s="4" t="s">
+      <c r="T1" s="1" t="s">
         <v>38</v>
       </c>
     </row>
     <row r="2" spans="1:20">
-      <c r="A2" s="4" t="s">
+      <c r="A2" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="B2" s="4" t="s">
+      <c r="B2" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="C2" s="4" t="s">
+      <c r="C2" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="D2" s="4" t="s">
+      <c r="D2" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="E2" s="4">
+      <c r="E2" s="1">
         <v>12</v>
       </c>
-      <c r="F2" s="8" t="s">
+      <c r="F2" s="9" t="s">
         <v>12</v>
       </c>
-      <c r="G2" s="4" t="s">
+      <c r="G2" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="H2" s="4" t="s">
+      <c r="H2" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="I2" s="4" t="s">
+      <c r="I2" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="J2" s="4" t="s">
+      <c r="J2" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="K2" s="4">
+      <c r="K2" s="1">
         <v>6</v>
       </c>
-      <c r="L2" s="4">
+      <c r="L2" s="1">
         <v>1010301033</v>
       </c>
-      <c r="M2" s="4" t="s">
+      <c r="M2" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="N2" s="4" t="s">
+      <c r="N2" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="O2" s="4" t="s">
+      <c r="O2" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="P2" s="4"/>
-      <c r="Q2" s="4"/>
-      <c r="R2" s="4"/>
-      <c r="S2" s="4">
+      <c r="P2" s="1"/>
+      <c r="Q2" s="1"/>
+      <c r="R2" s="1"/>
+      <c r="S2" s="1">
         <v>0</v>
       </c>
-      <c r="T2" s="4"/>
+      <c r="T2" s="1"/>
     </row>
     <row r="3" spans="1:20">
-      <c r="A3" s="4" t="s">
+      <c r="A3" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="B3" s="4" t="s">
+      <c r="B3" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="C3" s="4" t="s">
+      <c r="C3" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="D3" s="9" t="s">
+      <c r="D3" s="10" t="s">
         <v>43</v>
       </c>
-      <c r="E3" s="4">
+      <c r="E3" s="1">
         <v>5</v>
       </c>
-      <c r="F3" s="4" t="s">
+      <c r="F3" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="G3" s="4" t="s">
+      <c r="G3" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="H3" s="4" t="s">
+      <c r="H3" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="I3" s="4" t="s">
+      <c r="I3" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="J3" s="4" t="s">
+      <c r="J3" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="K3" s="4">
+      <c r="K3" s="1">
         <v>1</v>
       </c>
-      <c r="L3" s="4">
+      <c r="L3" s="1">
         <v>1010301033</v>
       </c>
-      <c r="M3" s="4" t="s">
+      <c r="M3" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="N3" s="4" t="s">
+      <c r="N3" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="O3" s="4" t="s">
+      <c r="O3" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="P3" s="4"/>
-      <c r="Q3" s="4"/>
-      <c r="R3" s="4"/>
-      <c r="S3" s="4">
+      <c r="P3" s="1"/>
+      <c r="Q3" s="1"/>
+      <c r="R3" s="1"/>
+      <c r="S3" s="1">
         <v>0</v>
       </c>
-      <c r="T3" s="4"/>
+      <c r="T3" s="1"/>
     </row>
     <row r="4" spans="1:20">
-      <c r="A4" s="4" t="s">
+      <c r="A4" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="B4" s="4" t="s">
+      <c r="B4" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="C4" s="4" t="s">
+      <c r="C4" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="D4" s="4">
+      <c r="D4" s="1">
         <v>123562</v>
       </c>
-      <c r="E4" s="4">
+      <c r="E4" s="1">
         <v>18</v>
       </c>
-      <c r="F4" s="4" t="s">
+      <c r="F4" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="G4" s="4" t="s">
+      <c r="G4" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="H4" s="4" t="s">
+      <c r="H4" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="I4" s="4" t="s">
+      <c r="I4" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="J4" s="4" t="s">
+      <c r="J4" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="K4" s="4">
+      <c r="K4" s="1">
         <v>1</v>
       </c>
-      <c r="L4" s="4">
+      <c r="L4" s="1">
         <v>1011134888</v>
       </c>
-      <c r="M4" s="4" t="s">
+      <c r="M4" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="N4" s="4" t="s">
+      <c r="N4" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="O4" s="4" t="s">
+      <c r="O4" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="P4" s="4"/>
-      <c r="Q4" s="4"/>
-      <c r="R4" s="4"/>
-      <c r="S4" s="4">
+      <c r="P4" s="1"/>
+      <c r="Q4" s="1"/>
+      <c r="R4" s="1"/>
+      <c r="S4" s="1">
         <v>0</v>
       </c>
-      <c r="T4" s="4"/>
+      <c r="T4" s="1"/>
     </row>
     <row r="5" spans="1:20">
       <c r="A5" s="3" t="s">
@@ -2112,7 +2182,7 @@
       <c r="B5" s="3" t="s">
         <v>47</v>
       </c>
-      <c r="C5" s="4" t="s">
+      <c r="C5" s="1" t="s">
         <v>14</v>
       </c>
       <c r="D5" s="3" t="s">
@@ -2154,7 +2224,7 @@
       <c r="P5" s="3"/>
       <c r="Q5" s="3"/>
       <c r="R5" s="3"/>
-      <c r="S5" s="4">
+      <c r="S5" s="1">
         <v>0</v>
       </c>
       <c r="T5" s="3"/>
@@ -2169,16 +2239,16 @@
       <c r="C6" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="D6" s="7" t="s">
+      <c r="D6" s="8" t="s">
         <v>43</v>
       </c>
       <c r="E6">
         <v>5</v>
       </c>
-      <c r="F6" s="10" t="s">
+      <c r="F6" s="11" t="s">
         <v>12</v>
       </c>
-      <c r="G6" s="10" t="s">
+      <c r="G6" s="11" t="s">
         <v>11</v>
       </c>
       <c r="H6" s="3" t="s">
@@ -2208,172 +2278,172 @@
       <c r="P6" s="3"/>
       <c r="Q6" s="3"/>
       <c r="R6" s="3"/>
-      <c r="S6" s="4">
+      <c r="S6" s="1">
         <v>0</v>
       </c>
       <c r="T6" s="3"/>
     </row>
     <row r="7" spans="1:20">
-      <c r="A7" s="11" t="s">
+      <c r="A7" s="12" t="s">
         <v>55</v>
       </c>
-      <c r="B7" s="11" t="s">
+      <c r="B7" s="12" t="s">
         <v>56</v>
       </c>
-      <c r="C7" s="11" t="s">
+      <c r="C7" s="12" t="s">
         <v>20</v>
       </c>
-      <c r="D7" s="11" t="s">
+      <c r="D7" s="12" t="s">
         <v>40</v>
       </c>
-      <c r="E7" s="11">
+      <c r="E7" s="12">
         <v>12</v>
       </c>
-      <c r="F7" s="12" t="s">
+      <c r="F7" s="13" t="s">
         <v>12</v>
       </c>
-      <c r="G7" s="11" t="s">
+      <c r="G7" s="12" t="s">
         <v>11</v>
       </c>
-      <c r="H7" s="11" t="s">
+      <c r="H7" s="12" t="s">
         <v>57</v>
       </c>
-      <c r="I7" s="11" t="s">
+      <c r="I7" s="12" t="s">
         <v>41</v>
       </c>
-      <c r="J7" s="11" t="s">
+      <c r="J7" s="12" t="s">
         <v>14</v>
       </c>
-      <c r="K7" s="11">
+      <c r="K7" s="12">
         <v>3</v>
       </c>
-      <c r="L7" s="11">
+      <c r="L7" s="12">
         <v>1010301003</v>
       </c>
-      <c r="M7" s="11" t="s">
+      <c r="M7" s="12" t="s">
         <v>58</v>
       </c>
-      <c r="N7" s="11" t="s">
+      <c r="N7" s="12" t="s">
         <v>16</v>
       </c>
-      <c r="O7" s="11" t="s">
+      <c r="O7" s="12" t="s">
         <v>17</v>
       </c>
-      <c r="P7" s="11"/>
-      <c r="Q7" s="11"/>
-      <c r="R7" s="11"/>
-      <c r="S7" s="11">
+      <c r="P7" s="12"/>
+      <c r="Q7" s="12"/>
+      <c r="R7" s="12"/>
+      <c r="S7" s="12">
         <v>0</v>
       </c>
-      <c r="T7" s="11"/>
+      <c r="T7" s="12"/>
     </row>
     <row r="8" spans="1:20">
-      <c r="A8" s="11" t="s">
+      <c r="A8" s="12" t="s">
         <v>59</v>
       </c>
-      <c r="B8" s="11" t="s">
+      <c r="B8" s="12" t="s">
         <v>60</v>
       </c>
-      <c r="C8" s="11" t="s">
+      <c r="C8" s="12" t="s">
         <v>14</v>
       </c>
-      <c r="D8" s="11" t="s">
+      <c r="D8" s="12" t="s">
         <v>43</v>
       </c>
-      <c r="E8" s="11">
+      <c r="E8" s="12">
         <v>5</v>
       </c>
-      <c r="F8" s="12" t="s">
+      <c r="F8" s="13" t="s">
         <v>12</v>
       </c>
-      <c r="G8" s="11" t="s">
+      <c r="G8" s="12" t="s">
         <v>11</v>
       </c>
-      <c r="H8" s="11" t="s">
+      <c r="H8" s="12" t="s">
         <v>57</v>
       </c>
-      <c r="I8" s="11" t="s">
+      <c r="I8" s="12" t="s">
         <v>41</v>
       </c>
-      <c r="J8" s="11" t="s">
+      <c r="J8" s="12" t="s">
         <v>14</v>
       </c>
-      <c r="K8" s="11">
+      <c r="K8" s="12">
         <v>0</v>
       </c>
-      <c r="L8" s="11">
+      <c r="L8" s="12">
         <v>1010301003</v>
       </c>
-      <c r="M8" s="11" t="s">
+      <c r="M8" s="12" t="s">
         <v>58</v>
       </c>
-      <c r="N8" s="11" t="s">
+      <c r="N8" s="12" t="s">
         <v>16</v>
       </c>
-      <c r="O8" s="11" t="s">
+      <c r="O8" s="12" t="s">
         <v>17</v>
       </c>
-      <c r="P8" s="11"/>
-      <c r="Q8" s="11"/>
-      <c r="R8" s="11"/>
-      <c r="S8" s="11">
+      <c r="P8" s="12"/>
+      <c r="Q8" s="12"/>
+      <c r="R8" s="12"/>
+      <c r="S8" s="12">
         <v>0</v>
       </c>
-      <c r="T8" s="11"/>
+      <c r="T8" s="12"/>
     </row>
     <row r="9" spans="1:20">
-      <c r="A9" s="11" t="s">
+      <c r="A9" s="12" t="s">
         <v>61</v>
       </c>
-      <c r="B9" s="11" t="s">
+      <c r="B9" s="12" t="s">
         <v>61</v>
       </c>
-      <c r="C9" s="11" t="s">
+      <c r="C9" s="12" t="s">
         <v>14</v>
       </c>
-      <c r="D9" s="11" t="s">
+      <c r="D9" s="12" t="s">
         <v>43</v>
       </c>
-      <c r="E9" s="11">
+      <c r="E9" s="12">
         <v>5</v>
       </c>
-      <c r="F9" s="12" t="s">
+      <c r="F9" s="13" t="s">
         <v>12</v>
       </c>
-      <c r="G9" s="11" t="s">
+      <c r="G9" s="12" t="s">
         <v>11</v>
       </c>
-      <c r="H9" s="11" t="s">
+      <c r="H9" s="12" t="s">
         <v>57</v>
       </c>
-      <c r="I9" s="11" t="s">
+      <c r="I9" s="12" t="s">
         <v>41</v>
       </c>
-      <c r="J9" s="11" t="s">
+      <c r="J9" s="12" t="s">
         <v>14</v>
       </c>
-      <c r="K9" s="11">
+      <c r="K9" s="12">
         <v>0</v>
       </c>
-      <c r="L9" s="11">
+      <c r="L9" s="12">
         <v>1010301003</v>
       </c>
-      <c r="M9" s="11" t="s">
+      <c r="M9" s="12" t="s">
         <v>58</v>
       </c>
-      <c r="N9" s="11" t="s">
+      <c r="N9" s="12" t="s">
         <v>16</v>
       </c>
-      <c r="O9" s="11" t="s">
+      <c r="O9" s="12" t="s">
         <v>17</v>
       </c>
-      <c r="P9" s="11"/>
-      <c r="Q9" s="11"/>
-      <c r="R9" s="11"/>
-      <c r="S9" s="11">
+      <c r="P9" s="12"/>
+      <c r="Q9" s="12"/>
+      <c r="R9" s="12"/>
+      <c r="S9" s="12">
         <v>0</v>
       </c>
-      <c r="T9" s="11"/>
+      <c r="T9" s="12"/>
     </row>
     <row r="10" spans="1:20">
       <c r="A10" s="3" t="s">
@@ -2385,31 +2455,31 @@
       <c r="C10" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="D10" s="11" t="s">
+      <c r="D10" s="12" t="s">
         <v>43</v>
       </c>
-      <c r="E10" s="11">
+      <c r="E10" s="12">
         <v>5</v>
       </c>
-      <c r="F10" s="4" t="s">
+      <c r="F10" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="G10" s="4" t="s">
+      <c r="G10" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="H10" s="4" t="s">
+      <c r="H10" s="1" t="s">
         <v>63</v>
       </c>
-      <c r="I10" s="4" t="s">
+      <c r="I10" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="J10" s="4" t="s">
+      <c r="J10" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="K10" s="4">
+      <c r="K10" s="1">
         <v>1</v>
       </c>
-      <c r="L10" s="5">
+      <c r="L10" s="6">
         <v>1000000001</v>
       </c>
       <c r="M10" s="3" t="s">
@@ -2421,13 +2491,13 @@
       <c r="O10" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="P10" s="11"/>
-      <c r="Q10" s="11"/>
-      <c r="R10" s="11"/>
-      <c r="S10" s="11">
+      <c r="P10" s="12"/>
+      <c r="Q10" s="12"/>
+      <c r="R10" s="12"/>
+      <c r="S10" s="12">
         <v>0</v>
       </c>
-      <c r="T10" s="11"/>
+      <c r="T10" s="12"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2464,16 +2534,16 @@
       <c r="C1" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="D1" s="4" t="s">
+      <c r="D1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="E1" s="4" t="s">
+      <c r="E1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="F1" s="4" t="s">
+      <c r="F1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="G1" s="4" t="s">
+      <c r="G1" s="1" t="s">
         <v>9</v>
       </c>
       <c r="H1" s="3" t="s">
@@ -2491,12 +2561,12 @@
       <c r="L1" s="3" t="s">
         <v>33</v>
       </c>
-      <c r="M1" s="6"/>
-      <c r="N1" s="6"/>
-      <c r="O1" s="6"/>
-      <c r="P1" s="6"/>
-      <c r="Q1" s="6"/>
-      <c r="R1" s="6"/>
+      <c r="M1" s="7"/>
+      <c r="N1" s="7"/>
+      <c r="O1" s="7"/>
+      <c r="P1" s="7"/>
+      <c r="Q1" s="7"/>
+      <c r="R1" s="7"/>
     </row>
     <row r="2" spans="1:18">
       <c r="A2" s="3" t="s">
@@ -2523,7 +2593,7 @@
       <c r="H2" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="I2" s="7" t="s">
+      <c r="I2" s="8" t="s">
         <v>43</v>
       </c>
       <c r="J2" s="3" t="s">
@@ -2535,12 +2605,12 @@
       <c r="L2" s="3">
         <v>1</v>
       </c>
-      <c r="M2" s="6"/>
-      <c r="N2" s="6"/>
-      <c r="O2" s="6"/>
-      <c r="P2" s="6"/>
-      <c r="Q2" s="6"/>
-      <c r="R2" s="6"/>
+      <c r="M2" s="7"/>
+      <c r="N2" s="7"/>
+      <c r="O2" s="7"/>
+      <c r="P2" s="7"/>
+      <c r="Q2" s="7"/>
+      <c r="R2" s="7"/>
     </row>
     <row r="3" spans="1:12">
       <c r="A3" s="3" t="s">
@@ -2552,7 +2622,7 @@
       <c r="C3" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="D3" s="5">
+      <c r="D3" s="6">
         <v>1000000001</v>
       </c>
       <c r="E3" s="3" t="s">
@@ -2567,7 +2637,7 @@
       <c r="H3" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="I3" s="7" t="s">
+      <c r="I3" s="8" t="s">
         <v>43</v>
       </c>
       <c r="J3" s="3" t="s">
@@ -2589,57 +2659,432 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:C4"/>
-  <sheetFormatPr defaultColWidth="8.88888888888889" defaultRowHeight="14.4" outlineLevelRow="3" outlineLevelCol="2"/>
+  <dimension ref="A1:F3"/>
+  <sheetFormatPr defaultColWidth="8.88888888888889" defaultRowHeight="14.4" outlineLevelRow="2" outlineLevelCol="5"/>
   <cols>
     <col min="1" max="1" width="27.1111111111111" customWidth="1"/>
     <col min="2" max="2" width="10.4444444444444" customWidth="1"/>
     <col min="3" max="3" width="11.4444444444444" customWidth="1"/>
+    <col min="4" max="4" width="11.6666666666667" customWidth="1"/>
+    <col min="5" max="5" width="14.5555555555556" customWidth="1"/>
+    <col min="6" max="6" width="17.6666666666667" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6">
+      <c r="A1" s="4" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="4" t="s">
+        <v>66</v>
+      </c>
+      <c r="C1" s="4" t="s">
+        <v>67</v>
+      </c>
+      <c r="D1" s="5" t="s">
+        <v>68</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6">
+      <c r="A2" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="B2" s="3">
+        <v>50</v>
+      </c>
+      <c r="C2" s="3">
+        <v>70</v>
+      </c>
+      <c r="D2" s="3" t="s">
+        <v>71</v>
+      </c>
+      <c r="E2" s="3"/>
+      <c r="F2" s="2" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6">
+      <c r="A3" s="3" t="s">
+        <v>61</v>
+      </c>
+      <c r="B3" s="3">
+        <v>40</v>
+      </c>
+      <c r="C3" s="3">
+        <v>26</v>
+      </c>
+      <c r="D3" s="3" t="s">
+        <v>73</v>
+      </c>
+      <c r="E3" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="F3" s="2">
+        <v>2</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <headerFooter/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
+  <dimension ref="A1:F4"/>
+  <sheetFormatPr defaultColWidth="8.88888888888889" defaultRowHeight="14.4" outlineLevelRow="3" outlineLevelCol="5"/>
+  <cols>
+    <col min="1" max="1" width="27.1111111111111" customWidth="1"/>
+    <col min="2" max="2" width="10.4444444444444" customWidth="1"/>
+    <col min="3" max="3" width="11.4444444444444" customWidth="1"/>
+    <col min="4" max="4" width="11.6666666666667" customWidth="1"/>
+    <col min="5" max="5" width="14.5555555555556" customWidth="1"/>
+    <col min="6" max="6" width="17.6666666666667" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6">
+      <c r="A1" s="4" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="4" t="s">
+        <v>66</v>
+      </c>
+      <c r="C1" s="4" t="s">
+        <v>67</v>
+      </c>
+      <c r="D1" s="5" t="s">
+        <v>68</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6">
+      <c r="A2" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="B2" s="3">
+        <v>150</v>
+      </c>
+      <c r="C2" s="3">
+        <v>45</v>
+      </c>
+      <c r="D2" s="3" t="s">
+        <v>71</v>
+      </c>
+      <c r="E2" s="3"/>
+      <c r="F2" s="2" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6">
+      <c r="A3" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="B3" s="3">
+        <v>40</v>
+      </c>
+      <c r="C3" s="3">
+        <v>26</v>
+      </c>
+      <c r="D3" s="3" t="s">
+        <v>77</v>
+      </c>
+      <c r="E3" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="F3" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6">
+      <c r="A4" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="B4" s="3">
+        <v>50</v>
+      </c>
+      <c r="C4" s="3">
+        <v>70</v>
+      </c>
+      <c r="D4" s="3" t="s">
+        <v>73</v>
+      </c>
+      <c r="E4" s="3" t="s">
+        <v>75</v>
+      </c>
+      <c r="F4" s="2"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <headerFooter/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
+  <dimension ref="A1:C3"/>
+  <sheetFormatPr defaultColWidth="8.88888888888889" defaultRowHeight="14.4" outlineLevelRow="2" outlineLevelCol="2"/>
+  <cols>
+    <col min="1" max="1" width="28.6666666666667" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3">
+      <c r="A1" t="s">
+        <v>78</v>
+      </c>
+      <c r="B1" t="s">
+        <v>79</v>
+      </c>
+      <c r="C1" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3">
+      <c r="A2" t="s">
+        <v>81</v>
+      </c>
+      <c r="B2">
+        <v>100</v>
+      </c>
+      <c r="C2">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3">
+      <c r="A3" t="s">
+        <v>82</v>
+      </c>
+      <c r="B3">
+        <v>50</v>
+      </c>
+      <c r="C3">
+        <v>30</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <headerFooter/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
+  <dimension ref="A1:G4"/>
+  <sheetFormatPr defaultColWidth="8.88888888888889" defaultRowHeight="14.4" outlineLevelRow="3" outlineLevelCol="6"/>
+  <cols>
+    <col min="1" max="1" width="19.7777777777778" customWidth="1"/>
+    <col min="2" max="2" width="8.11111111111111" customWidth="1"/>
+    <col min="3" max="3" width="8.55555555555556" customWidth="1"/>
+    <col min="4" max="4" width="17.8888888888889" customWidth="1"/>
+    <col min="5" max="5" width="12.6666666666667" customWidth="1"/>
+    <col min="6" max="6" width="14.5555555555556" customWidth="1"/>
+    <col min="7" max="7" width="17.6666666666667" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7">
       <c r="A1" s="1" t="s">
-        <v>0</v>
+        <v>83</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>66</v>
+        <v>84</v>
       </c>
       <c r="C1" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>85</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7">
+      <c r="A2" s="1" t="s">
+        <v>86</v>
+      </c>
+      <c r="B2" s="1">
+        <v>524</v>
+      </c>
+      <c r="C2" s="1">
+        <v>524</v>
+      </c>
+      <c r="D2" s="1">
+        <v>2</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="G2" s="2" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7">
+      <c r="A3" s="1" t="s">
+        <v>88</v>
+      </c>
+      <c r="B3" s="1">
+        <v>232</v>
+      </c>
+      <c r="C3" s="1">
+        <v>232</v>
+      </c>
+      <c r="D3" s="1">
+        <v>7.9</v>
+      </c>
+      <c r="E3" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="F3" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="G3" s="3"/>
+    </row>
+    <row r="4" spans="1:7">
+      <c r="A4" s="3" t="s">
+        <v>90</v>
+      </c>
+      <c r="B4" s="3">
+        <v>232</v>
+      </c>
+      <c r="C4" s="3">
+        <v>232</v>
+      </c>
+      <c r="D4" s="3">
+        <v>2.32</v>
+      </c>
+      <c r="E4" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="F4" s="3"/>
+      <c r="G4" s="3"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <headerFooter/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
+  <dimension ref="A1:G4"/>
+  <sheetFormatPr defaultColWidth="8.88888888888889" defaultRowHeight="14.4" outlineLevelRow="3" outlineLevelCol="6"/>
+  <cols>
+    <col min="1" max="1" width="19.7777777777778" customWidth="1"/>
+    <col min="2" max="2" width="8.11111111111111" customWidth="1"/>
+    <col min="3" max="3" width="8.55555555555556" customWidth="1"/>
+    <col min="4" max="4" width="17.8888888888889" customWidth="1"/>
+    <col min="5" max="5" width="12.6666666666667" customWidth="1"/>
+    <col min="6" max="6" width="14.5555555555556" customWidth="1"/>
+    <col min="7" max="7" width="17.6666666666667" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7">
+      <c r="A1" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>84</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>85</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7">
+      <c r="A2" s="1" t="s">
+        <v>86</v>
+      </c>
+      <c r="B2" s="1">
+        <v>22</v>
+      </c>
+      <c r="C2" s="1">
+        <v>524</v>
+      </c>
+      <c r="D2" s="1">
+        <v>2</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="G2" s="2" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7">
+      <c r="A3" s="1" t="s">
+        <v>88</v>
+      </c>
+      <c r="B3" s="1">
+        <v>34</v>
+      </c>
+      <c r="C3" s="1">
+        <v>232</v>
+      </c>
+      <c r="D3" s="1">
+        <v>7.9</v>
+      </c>
+      <c r="E3" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="F3" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="G3" s="3"/>
+    </row>
+    <row r="4" spans="1:7">
+      <c r="A4" s="3" t="s">
+        <v>90</v>
+      </c>
+      <c r="B4" s="3">
         <v>67</v>
       </c>
-    </row>
-    <row r="2" spans="1:3">
-      <c r="A2" s="2" t="s">
-        <v>55</v>
-      </c>
-      <c r="B2" s="3">
-        <v>30</v>
-      </c>
-      <c r="C2" s="3">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3">
-      <c r="A3" s="2" t="s">
-        <v>59</v>
-      </c>
-      <c r="B3" s="3">
-        <v>40</v>
-      </c>
-      <c r="C3" s="3">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3">
-      <c r="A4" s="2" t="s">
-        <v>61</v>
-      </c>
-      <c r="B4" s="3">
-        <v>50</v>
-      </c>
       <c r="C4" s="3">
-        <v>70</v>
-      </c>
+        <v>232</v>
+      </c>
+      <c r="D4" s="3">
+        <v>2.32</v>
+      </c>
+      <c r="E4" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="F4" s="3"/>
+      <c r="G4" s="3"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Updated TestDatas And Item Details Sheets
Updated TestDatas And Item Details Sheets
</commit_message>
<xml_diff>
--- a/testdata/ItemDetails.xlsx
+++ b/testdata/ItemDetails.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="23040" windowHeight="9120" firstSheet="3" activeTab="4"/>
+    <workbookView windowWidth="23040" windowHeight="9120" firstSheet="6" activeTab="10"/>
   </bookViews>
   <sheets>
     <sheet name="PR Details" sheetId="1" r:id="rId1"/>
@@ -15,6 +15,9 @@
     <sheet name="StockTransferItem" sheetId="5" r:id="rId6"/>
     <sheet name="POwithRateContractItem" sheetId="6" r:id="rId7"/>
     <sheet name="POwithRateContractItem_Mat" sheetId="7" r:id="rId8"/>
+    <sheet name="SO Details" sheetId="9" r:id="rId9"/>
+    <sheet name="Customer SO Details" sheetId="10" r:id="rId10"/>
+    <sheet name="Open Sales" sheetId="11" r:id="rId11"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -34,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="257" uniqueCount="91">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="427" uniqueCount="158">
   <si>
     <t>ITEM_NAME</t>
   </si>
@@ -308,6 +311,207 @@
   </si>
   <si>
     <t>PK-NA-MAC-10001</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ITEM_ID </t>
+  </si>
+  <si>
+    <t>ITEM_REV</t>
+  </si>
+  <si>
+    <t>ITEM_DESC</t>
+  </si>
+  <si>
+    <t>SALE_UOM</t>
+  </si>
+  <si>
+    <t>TAX_PCT</t>
+  </si>
+  <si>
+    <t>PRICE_BASIS_TYPE</t>
+  </si>
+  <si>
+    <t>CATALOG_PRICELIST_NO</t>
+  </si>
+  <si>
+    <t>CONV_FACT</t>
+  </si>
+  <si>
+    <t>TOLERANCE_TYPE</t>
+  </si>
+  <si>
+    <t>CUST_ITEM_ID</t>
+  </si>
+  <si>
+    <t>CUST_ITEM_DESC</t>
+  </si>
+  <si>
+    <t>WAREHOUSE_DESC</t>
+  </si>
+  <si>
+    <t>SUB_CLASS</t>
+  </si>
+  <si>
+    <t>PRICECLASS</t>
+  </si>
+  <si>
+    <t>PROMOTIONAL</t>
+  </si>
+  <si>
+    <t>HK-FIFO-LOT-BATCH-10001(FG)</t>
+  </si>
+  <si>
+    <t>Item Level</t>
+  </si>
+  <si>
+    <t>DOMESTIC</t>
+  </si>
+  <si>
+    <t>Sales Regular</t>
+  </si>
+  <si>
+    <t>HK-FG-DISSIMILAR-10001</t>
+  </si>
+  <si>
+    <t>HK-SER-MAC-10001(FG)</t>
+  </si>
+  <si>
+    <t>Standard Price</t>
+  </si>
+  <si>
+    <t>HK-FG-STD-PRICE-DISSIMILAR ITEM-10001</t>
+  </si>
+  <si>
+    <t>GENERAL</t>
+  </si>
+  <si>
+    <t>HK-LOT-MAC-10001(FG)</t>
+  </si>
+  <si>
+    <t>Open Order</t>
+  </si>
+  <si>
+    <t>OPSO1/00094/24-25</t>
+  </si>
+  <si>
+    <t>HK-FG-RC-DISSIMILAR ITEM-10001</t>
+  </si>
+  <si>
+    <t>OPSO1/00114/24-25</t>
+  </si>
+  <si>
+    <t>HK-FIFO-SER-BATCH-10001(FG)</t>
+  </si>
+  <si>
+    <t>(2022)5%</t>
+  </si>
+  <si>
+    <t>Catalog</t>
+  </si>
+  <si>
+    <t>HK-FG-CATALOG-DISSIMILAR-10001</t>
+  </si>
+  <si>
+    <t>CUST_ID</t>
+  </si>
+  <si>
+    <t>CUST_DESC</t>
+  </si>
+  <si>
+    <t>GST_TYPE</t>
+  </si>
+  <si>
+    <t>SALES_GST_TYPE</t>
+  </si>
+  <si>
+    <t>GST_CLASSIFICATION</t>
+  </si>
+  <si>
+    <t>CUST_PRINT_NAME</t>
+  </si>
+  <si>
+    <t>SALES_ZONE</t>
+  </si>
+  <si>
+    <t>SALES_REGION</t>
+  </si>
+  <si>
+    <t>CUST_SUB_GRP</t>
+  </si>
+  <si>
+    <t>CUST_GRP</t>
+  </si>
+  <si>
+    <t>SALES_PERSON</t>
+  </si>
+  <si>
+    <t>CUS0015</t>
+  </si>
+  <si>
+    <t>MURUGAN TRADERS</t>
+  </si>
+  <si>
+    <t>Unregistered</t>
+  </si>
+  <si>
+    <t>Inter-State</t>
+  </si>
+  <si>
+    <t>Union Territory</t>
+  </si>
+  <si>
+    <t>NORTH</t>
+  </si>
+  <si>
+    <t>INTERSTATE</t>
+  </si>
+  <si>
+    <t>BPCL</t>
+  </si>
+  <si>
+    <t>SUNDRY DEBTORS-PART</t>
+  </si>
+  <si>
+    <t>VIJAIKUMAR</t>
+  </si>
+  <si>
+    <t>CU0060</t>
+  </si>
+  <si>
+    <t>FRANCE FOREIGN TRADERS</t>
+  </si>
+  <si>
+    <t>Export</t>
+  </si>
+  <si>
+    <t>EXPORT</t>
+  </si>
+  <si>
+    <t>AASHIRVAD AUTOTECH - PART</t>
+  </si>
+  <si>
+    <t>LOCATION_ID</t>
+  </si>
+  <si>
+    <t>UNIT</t>
+  </si>
+  <si>
+    <t>CUSTOMER_ID</t>
+  </si>
+  <si>
+    <t>CUSTOMER_NAME</t>
+  </si>
+  <si>
+    <t>OSO_NO</t>
+  </si>
+  <si>
+    <t>L100</t>
+  </si>
+  <si>
+    <t>U100</t>
+  </si>
+  <si>
+    <t>OPSO1/00092/24-25</t>
   </si>
 </sst>
 </file>
@@ -320,13 +524,19 @@
     <numFmt numFmtId="178" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
     <numFmt numFmtId="179" formatCode="_ &quot;₹&quot;* #,##0_ ;_ &quot;₹&quot;* \-#,##0_ ;_ &quot;₹&quot;* &quot;-&quot;_ ;_ @_ "/>
   </numFmts>
-  <fonts count="27">
+  <fonts count="28">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <charset val="134"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
+      <charset val="134"/>
     </font>
     <font>
       <sz val="10"/>
@@ -517,12 +727,18 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="34">
+  <fills count="35">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFFF"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
@@ -717,12 +933,27 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="10">
+  <borders count="11">
     <border>
       <left/>
       <right/>
       <top/>
       <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="medium">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="medium">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FF000000"/>
+      </bottom>
       <diagonal/>
     </border>
     <border>
@@ -858,55 +1089,52 @@
     <xf numFmtId="179" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="2" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="3" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="4" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="5" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="17" fillId="5" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="5" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="6" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="18" fillId="6" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="6" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="7" borderId="8" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="21" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="10" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="23" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -921,132 +1149,151 @@
     <xf numFmtId="0" fontId="26" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="27" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="26" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="27" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="26" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="27" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="26" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="27" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="26" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="27" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="26" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="27" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="25">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFill="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="49" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="49" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="2" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="49" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="49" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="justify" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -1598,324 +1845,507 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10">
-      <c r="A1" s="15" t="s">
+      <c r="A1" s="21" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="15" t="s">
+      <c r="B1" s="21" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="15" t="s">
+      <c r="C1" s="21" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="15" t="s">
+      <c r="D1" s="21" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="15" t="s">
+      <c r="E1" s="21" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="15" t="s">
+      <c r="F1" s="21" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="15" t="s">
+      <c r="G1" s="21" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="15" t="s">
+      <c r="H1" s="21" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="15" t="s">
+      <c r="I1" s="21" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="15" t="s">
+      <c r="J1" s="21" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="2" s="14" customFormat="1" ht="20.4" spans="1:10">
-      <c r="A2" s="16" t="s">
+    <row r="2" s="20" customFormat="1" ht="20.4" spans="1:10">
+      <c r="A2" s="22" t="s">
         <v>10</v>
       </c>
-      <c r="B2" s="17" t="s">
+      <c r="B2" s="23" t="s">
         <v>11</v>
       </c>
-      <c r="C2" s="17" t="s">
+      <c r="C2" s="23" t="s">
         <v>12</v>
       </c>
-      <c r="D2" s="16" t="s">
+      <c r="D2" s="22" t="s">
         <v>13</v>
       </c>
-      <c r="E2" s="16">
+      <c r="E2" s="22">
         <v>1</v>
       </c>
-      <c r="F2" s="16" t="s">
+      <c r="F2" s="22" t="s">
         <v>14</v>
       </c>
-      <c r="G2" s="16">
+      <c r="G2" s="22">
         <v>1010301033</v>
       </c>
-      <c r="H2" s="16" t="s">
+      <c r="H2" s="22" t="s">
         <v>15</v>
       </c>
-      <c r="I2" s="16" t="s">
+      <c r="I2" s="22" t="s">
         <v>16</v>
       </c>
-      <c r="J2" s="16" t="s">
+      <c r="J2" s="22" t="s">
         <v>17</v>
       </c>
     </row>
     <row r="3" ht="15" customHeight="1" spans="1:10">
-      <c r="A3" s="16" t="s">
+      <c r="A3" s="22" t="s">
         <v>18</v>
       </c>
-      <c r="B3" s="17" t="s">
+      <c r="B3" s="23" t="s">
         <v>11</v>
       </c>
-      <c r="C3" s="17" t="s">
+      <c r="C3" s="23" t="s">
         <v>12</v>
       </c>
-      <c r="D3" s="16" t="s">
+      <c r="D3" s="22" t="s">
         <v>19</v>
       </c>
-      <c r="E3" s="16">
+      <c r="E3" s="22">
         <v>6</v>
       </c>
-      <c r="F3" s="17" t="s">
+      <c r="F3" s="23" t="s">
         <v>20</v>
       </c>
-      <c r="G3" s="16">
+      <c r="G3" s="22">
         <v>1010301033</v>
       </c>
-      <c r="H3" s="16" t="s">
+      <c r="H3" s="22" t="s">
         <v>15</v>
       </c>
-      <c r="I3" s="16" t="s">
+      <c r="I3" s="22" t="s">
         <v>16</v>
       </c>
-      <c r="J3" s="16" t="s">
+      <c r="J3" s="22" t="s">
         <v>17</v>
       </c>
     </row>
     <row r="4" spans="1:10">
-      <c r="A4" s="16" t="s">
+      <c r="A4" s="22" t="s">
         <v>21</v>
       </c>
-      <c r="B4" s="17" t="s">
+      <c r="B4" s="23" t="s">
         <v>22</v>
       </c>
-      <c r="C4" s="17" t="s">
+      <c r="C4" s="23" t="s">
         <v>22</v>
       </c>
-      <c r="D4" s="16" t="s">
+      <c r="D4" s="22" t="s">
         <v>23</v>
       </c>
-      <c r="E4" s="16">
+      <c r="E4" s="22">
         <v>1</v>
       </c>
-      <c r="F4" s="17" t="s">
+      <c r="F4" s="23" t="s">
         <v>14</v>
       </c>
-      <c r="G4" s="16">
+      <c r="G4" s="22">
         <v>5010101060</v>
       </c>
-      <c r="H4" s="16" t="s">
+      <c r="H4" s="22" t="s">
         <v>24</v>
       </c>
-      <c r="I4" s="16" t="s">
+      <c r="I4" s="22" t="s">
         <v>16</v>
       </c>
-      <c r="J4" s="16" t="s">
+      <c r="J4" s="22" t="s">
         <v>17</v>
       </c>
     </row>
     <row r="5" spans="1:10">
-      <c r="A5" s="18"/>
-      <c r="B5" s="18"/>
-      <c r="C5" s="18"/>
-      <c r="D5" s="18"/>
-      <c r="E5" s="18"/>
-      <c r="F5" s="18"/>
-      <c r="G5" s="18"/>
-      <c r="H5" s="18"/>
-      <c r="I5" s="18"/>
-      <c r="J5" s="18"/>
+      <c r="A5" s="24"/>
+      <c r="B5" s="24"/>
+      <c r="C5" s="24"/>
+      <c r="D5" s="24"/>
+      <c r="E5" s="24"/>
+      <c r="F5" s="24"/>
+      <c r="G5" s="24"/>
+      <c r="H5" s="24"/>
+      <c r="I5" s="24"/>
+      <c r="J5" s="24"/>
     </row>
     <row r="6" spans="1:10">
-      <c r="A6" s="18"/>
-      <c r="B6" s="18"/>
-      <c r="C6" s="18"/>
-      <c r="D6" s="18"/>
-      <c r="E6" s="18"/>
-      <c r="F6" s="18"/>
-      <c r="G6" s="18"/>
-      <c r="H6" s="18"/>
-      <c r="I6" s="18"/>
-      <c r="J6" s="18"/>
+      <c r="A6" s="24"/>
+      <c r="B6" s="24"/>
+      <c r="C6" s="24"/>
+      <c r="D6" s="24"/>
+      <c r="E6" s="24"/>
+      <c r="F6" s="24"/>
+      <c r="G6" s="24"/>
+      <c r="H6" s="24"/>
+      <c r="I6" s="24"/>
+      <c r="J6" s="24"/>
     </row>
     <row r="7" spans="1:10">
-      <c r="A7" s="18"/>
-      <c r="B7" s="18"/>
-      <c r="C7" s="18"/>
-      <c r="D7" s="18"/>
-      <c r="E7" s="18"/>
-      <c r="F7" s="18"/>
-      <c r="G7" s="18"/>
-      <c r="H7" s="18"/>
-      <c r="I7" s="18"/>
-      <c r="J7" s="18"/>
+      <c r="A7" s="24"/>
+      <c r="B7" s="24"/>
+      <c r="C7" s="24"/>
+      <c r="D7" s="24"/>
+      <c r="E7" s="24"/>
+      <c r="F7" s="24"/>
+      <c r="G7" s="24"/>
+      <c r="H7" s="24"/>
+      <c r="I7" s="24"/>
+      <c r="J7" s="24"/>
     </row>
     <row r="8" spans="1:10">
-      <c r="A8" s="18"/>
-      <c r="B8" s="18"/>
-      <c r="C8" s="18"/>
-      <c r="D8" s="18"/>
-      <c r="E8" s="18"/>
-      <c r="F8" s="18"/>
-      <c r="G8" s="18"/>
-      <c r="H8" s="18"/>
-      <c r="I8" s="18"/>
-      <c r="J8" s="18"/>
+      <c r="A8" s="24"/>
+      <c r="B8" s="24"/>
+      <c r="C8" s="24"/>
+      <c r="D8" s="24"/>
+      <c r="E8" s="24"/>
+      <c r="F8" s="24"/>
+      <c r="G8" s="24"/>
+      <c r="H8" s="24"/>
+      <c r="I8" s="24"/>
+      <c r="J8" s="24"/>
     </row>
     <row r="9" spans="1:10">
-      <c r="A9" s="18"/>
-      <c r="B9" s="18"/>
-      <c r="C9" s="18"/>
-      <c r="D9" s="18"/>
-      <c r="E9" s="18"/>
-      <c r="F9" s="18"/>
-      <c r="G9" s="18"/>
-      <c r="H9" s="18"/>
-      <c r="I9" s="18"/>
-      <c r="J9" s="18"/>
+      <c r="A9" s="24"/>
+      <c r="B9" s="24"/>
+      <c r="C9" s="24"/>
+      <c r="D9" s="24"/>
+      <c r="E9" s="24"/>
+      <c r="F9" s="24"/>
+      <c r="G9" s="24"/>
+      <c r="H9" s="24"/>
+      <c r="I9" s="24"/>
+      <c r="J9" s="24"/>
     </row>
     <row r="10" spans="1:10">
-      <c r="A10" s="18"/>
-      <c r="B10" s="18"/>
-      <c r="C10" s="18"/>
-      <c r="D10" s="18"/>
-      <c r="E10" s="18"/>
-      <c r="F10" s="18"/>
-      <c r="G10" s="18"/>
-      <c r="H10" s="18"/>
-      <c r="I10" s="18"/>
-      <c r="J10" s="18"/>
+      <c r="A10" s="24"/>
+      <c r="B10" s="24"/>
+      <c r="C10" s="24"/>
+      <c r="D10" s="24"/>
+      <c r="E10" s="24"/>
+      <c r="F10" s="24"/>
+      <c r="G10" s="24"/>
+      <c r="H10" s="24"/>
+      <c r="I10" s="24"/>
+      <c r="J10" s="24"/>
     </row>
     <row r="11" spans="1:10">
-      <c r="A11" s="18"/>
-      <c r="B11" s="18"/>
-      <c r="C11" s="18"/>
-      <c r="D11" s="18"/>
-      <c r="E11" s="18"/>
-      <c r="F11" s="18"/>
-      <c r="G11" s="18"/>
-      <c r="H11" s="18"/>
-      <c r="I11" s="18"/>
-      <c r="J11" s="18"/>
+      <c r="A11" s="24"/>
+      <c r="B11" s="24"/>
+      <c r="C11" s="24"/>
+      <c r="D11" s="24"/>
+      <c r="E11" s="24"/>
+      <c r="F11" s="24"/>
+      <c r="G11" s="24"/>
+      <c r="H11" s="24"/>
+      <c r="I11" s="24"/>
+      <c r="J11" s="24"/>
     </row>
     <row r="12" spans="1:10">
-      <c r="A12" s="18"/>
-      <c r="B12" s="18"/>
-      <c r="C12" s="18"/>
-      <c r="D12" s="18"/>
-      <c r="E12" s="18"/>
-      <c r="F12" s="18"/>
-      <c r="G12" s="18"/>
-      <c r="H12" s="18"/>
-      <c r="I12" s="18"/>
-      <c r="J12" s="18"/>
+      <c r="A12" s="24"/>
+      <c r="B12" s="24"/>
+      <c r="C12" s="24"/>
+      <c r="D12" s="24"/>
+      <c r="E12" s="24"/>
+      <c r="F12" s="24"/>
+      <c r="G12" s="24"/>
+      <c r="H12" s="24"/>
+      <c r="I12" s="24"/>
+      <c r="J12" s="24"/>
     </row>
     <row r="13" spans="1:10">
-      <c r="A13" s="18"/>
-      <c r="B13" s="18"/>
-      <c r="C13" s="18"/>
-      <c r="D13" s="18"/>
-      <c r="E13" s="18"/>
-      <c r="F13" s="18"/>
-      <c r="G13" s="18"/>
-      <c r="H13" s="18"/>
-      <c r="I13" s="18"/>
-      <c r="J13" s="18"/>
+      <c r="A13" s="24"/>
+      <c r="B13" s="24"/>
+      <c r="C13" s="24"/>
+      <c r="D13" s="24"/>
+      <c r="E13" s="24"/>
+      <c r="F13" s="24"/>
+      <c r="G13" s="24"/>
+      <c r="H13" s="24"/>
+      <c r="I13" s="24"/>
+      <c r="J13" s="24"/>
     </row>
     <row r="14" spans="1:10">
-      <c r="A14" s="18"/>
-      <c r="B14" s="18"/>
-      <c r="C14" s="18"/>
-      <c r="D14" s="18"/>
-      <c r="E14" s="18"/>
-      <c r="F14" s="18"/>
-      <c r="G14" s="18"/>
-      <c r="H14" s="18"/>
-      <c r="I14" s="18"/>
-      <c r="J14" s="18"/>
+      <c r="A14" s="24"/>
+      <c r="B14" s="24"/>
+      <c r="C14" s="24"/>
+      <c r="D14" s="24"/>
+      <c r="E14" s="24"/>
+      <c r="F14" s="24"/>
+      <c r="G14" s="24"/>
+      <c r="H14" s="24"/>
+      <c r="I14" s="24"/>
+      <c r="J14" s="24"/>
     </row>
     <row r="15" spans="1:10">
-      <c r="A15" s="18"/>
-      <c r="B15" s="18"/>
-      <c r="C15" s="18"/>
-      <c r="D15" s="18"/>
-      <c r="E15" s="18"/>
-      <c r="F15" s="18"/>
-      <c r="G15" s="18"/>
-      <c r="H15" s="18"/>
-      <c r="I15" s="18"/>
-      <c r="J15" s="18"/>
+      <c r="A15" s="24"/>
+      <c r="B15" s="24"/>
+      <c r="C15" s="24"/>
+      <c r="D15" s="24"/>
+      <c r="E15" s="24"/>
+      <c r="F15" s="24"/>
+      <c r="G15" s="24"/>
+      <c r="H15" s="24"/>
+      <c r="I15" s="24"/>
+      <c r="J15" s="24"/>
     </row>
     <row r="16" spans="1:10">
-      <c r="A16" s="18"/>
-      <c r="B16" s="18"/>
-      <c r="C16" s="18"/>
-      <c r="D16" s="18"/>
-      <c r="E16" s="18"/>
-      <c r="F16" s="18"/>
-      <c r="G16" s="18"/>
-      <c r="H16" s="18"/>
-      <c r="I16" s="18"/>
-      <c r="J16" s="18"/>
+      <c r="A16" s="24"/>
+      <c r="B16" s="24"/>
+      <c r="C16" s="24"/>
+      <c r="D16" s="24"/>
+      <c r="E16" s="24"/>
+      <c r="F16" s="24"/>
+      <c r="G16" s="24"/>
+      <c r="H16" s="24"/>
+      <c r="I16" s="24"/>
+      <c r="J16" s="24"/>
     </row>
     <row r="17" spans="1:10">
-      <c r="A17" s="18"/>
-      <c r="B17" s="18"/>
-      <c r="C17" s="18"/>
-      <c r="D17" s="18"/>
-      <c r="E17" s="18"/>
-      <c r="F17" s="18"/>
-      <c r="G17" s="18"/>
-      <c r="H17" s="18"/>
-      <c r="I17" s="18"/>
-      <c r="J17" s="18"/>
+      <c r="A17" s="24"/>
+      <c r="B17" s="24"/>
+      <c r="C17" s="24"/>
+      <c r="D17" s="24"/>
+      <c r="E17" s="24"/>
+      <c r="F17" s="24"/>
+      <c r="G17" s="24"/>
+      <c r="H17" s="24"/>
+      <c r="I17" s="24"/>
+      <c r="J17" s="24"/>
     </row>
     <row r="18" spans="1:10">
-      <c r="A18" s="18"/>
-      <c r="B18" s="18"/>
-      <c r="C18" s="18"/>
-      <c r="D18" s="18"/>
-      <c r="E18" s="18"/>
-      <c r="F18" s="18"/>
-      <c r="G18" s="18"/>
-      <c r="H18" s="18"/>
-      <c r="I18" s="18"/>
-      <c r="J18" s="18"/>
+      <c r="A18" s="24"/>
+      <c r="B18" s="24"/>
+      <c r="C18" s="24"/>
+      <c r="D18" s="24"/>
+      <c r="E18" s="24"/>
+      <c r="F18" s="24"/>
+      <c r="G18" s="24"/>
+      <c r="H18" s="24"/>
+      <c r="I18" s="24"/>
+      <c r="J18" s="24"/>
     </row>
     <row r="19" spans="1:10">
-      <c r="A19" s="18"/>
-      <c r="B19" s="18"/>
-      <c r="C19" s="18"/>
-      <c r="D19" s="18"/>
-      <c r="E19" s="18"/>
-      <c r="F19" s="18"/>
-      <c r="G19" s="18"/>
-      <c r="H19" s="18"/>
-      <c r="I19" s="18"/>
-      <c r="J19" s="18"/>
+      <c r="A19" s="24"/>
+      <c r="B19" s="24"/>
+      <c r="C19" s="24"/>
+      <c r="D19" s="24"/>
+      <c r="E19" s="24"/>
+      <c r="F19" s="24"/>
+      <c r="G19" s="24"/>
+      <c r="H19" s="24"/>
+      <c r="I19" s="24"/>
+      <c r="J19" s="24"/>
     </row>
     <row r="20" spans="1:10">
-      <c r="A20" s="18"/>
-      <c r="B20" s="18"/>
-      <c r="C20" s="18"/>
-      <c r="D20" s="18"/>
-      <c r="E20" s="18"/>
-      <c r="F20" s="18"/>
-      <c r="G20" s="18"/>
-      <c r="H20" s="18"/>
-      <c r="I20" s="18"/>
-      <c r="J20" s="18"/>
+      <c r="A20" s="24"/>
+      <c r="B20" s="24"/>
+      <c r="C20" s="24"/>
+      <c r="D20" s="24"/>
+      <c r="E20" s="24"/>
+      <c r="F20" s="24"/>
+      <c r="G20" s="24"/>
+      <c r="H20" s="24"/>
+      <c r="I20" s="24"/>
+      <c r="J20" s="24"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <headerFooter/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
+  <dimension ref="A1:K3"/>
+  <sheetFormatPr defaultColWidth="8.88888888888889" defaultRowHeight="14.4" outlineLevelRow="2"/>
+  <cols>
+    <col min="1" max="1" width="9" customWidth="1"/>
+    <col min="2" max="2" width="25.7777777777778" customWidth="1"/>
+    <col min="3" max="3" width="12.4444444444444" customWidth="1"/>
+    <col min="4" max="4" width="16.2222222222222" customWidth="1"/>
+    <col min="5" max="5" width="20.2222222222222" customWidth="1"/>
+    <col min="6" max="6" width="25.7777777777778" customWidth="1"/>
+    <col min="7" max="7" width="12.2222222222222" customWidth="1"/>
+    <col min="8" max="8" width="14.5555555555556" customWidth="1"/>
+    <col min="9" max="9" width="28.5555555555556" customWidth="1"/>
+    <col min="10" max="10" width="23" customWidth="1"/>
+    <col min="11" max="11" width="14.6666666666667" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:11">
+      <c r="A1" s="4" t="s">
+        <v>124</v>
+      </c>
+      <c r="B1" s="4" t="s">
+        <v>125</v>
+      </c>
+      <c r="C1" s="4" t="s">
+        <v>126</v>
+      </c>
+      <c r="D1" s="4" t="s">
+        <v>127</v>
+      </c>
+      <c r="E1" s="4" t="s">
+        <v>128</v>
+      </c>
+      <c r="F1" s="5" t="s">
+        <v>129</v>
+      </c>
+      <c r="G1" s="5" t="s">
+        <v>130</v>
+      </c>
+      <c r="H1" s="5" t="s">
+        <v>131</v>
+      </c>
+      <c r="I1" s="5" t="s">
+        <v>132</v>
+      </c>
+      <c r="J1" s="5" t="s">
+        <v>133</v>
+      </c>
+      <c r="K1" s="5" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11">
+      <c r="A2" s="4" t="s">
+        <v>135</v>
+      </c>
+      <c r="B2" s="4" t="s">
+        <v>136</v>
+      </c>
+      <c r="C2" s="4" t="s">
+        <v>137</v>
+      </c>
+      <c r="D2" s="4" t="s">
+        <v>138</v>
+      </c>
+      <c r="E2" s="4" t="s">
+        <v>139</v>
+      </c>
+      <c r="F2" s="6" t="s">
+        <v>136</v>
+      </c>
+      <c r="G2" s="6" t="s">
+        <v>140</v>
+      </c>
+      <c r="H2" s="6" t="s">
+        <v>141</v>
+      </c>
+      <c r="I2" s="6" t="s">
+        <v>142</v>
+      </c>
+      <c r="J2" s="6" t="s">
+        <v>143</v>
+      </c>
+      <c r="K2" s="6" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11">
+      <c r="A3" s="7" t="s">
+        <v>145</v>
+      </c>
+      <c r="B3" s="6" t="s">
+        <v>146</v>
+      </c>
+      <c r="C3" s="4" t="s">
+        <v>137</v>
+      </c>
+      <c r="D3" s="6" t="s">
+        <v>147</v>
+      </c>
+      <c r="E3" s="6" t="s">
+        <v>147</v>
+      </c>
+      <c r="F3" s="6" t="s">
+        <v>146</v>
+      </c>
+      <c r="G3" s="6" t="s">
+        <v>148</v>
+      </c>
+      <c r="H3" s="6" t="s">
+        <v>148</v>
+      </c>
+      <c r="I3" s="6" t="s">
+        <v>149</v>
+      </c>
+      <c r="J3" s="6" t="s">
+        <v>143</v>
+      </c>
+      <c r="K3" s="6" t="s">
+        <v>144</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <headerFooter/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
+  <dimension ref="A1:E2"/>
+  <sheetFormatPr defaultColWidth="8.88888888888889" defaultRowHeight="14.4" outlineLevelRow="1" outlineLevelCol="4"/>
+  <cols>
+    <col min="1" max="1" width="13.5555555555556" customWidth="1"/>
+    <col min="2" max="2" width="6" customWidth="1"/>
+    <col min="3" max="3" width="14.4444444444444" customWidth="1"/>
+    <col min="4" max="4" width="18.1111111111111" customWidth="1"/>
+    <col min="5" max="5" width="19.5555555555556" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="15.15" spans="1:5">
+      <c r="A1" s="1" t="s">
+        <v>150</v>
+      </c>
+      <c r="B1" t="s">
+        <v>151</v>
+      </c>
+      <c r="C1" t="s">
+        <v>152</v>
+      </c>
+      <c r="D1" t="s">
+        <v>153</v>
+      </c>
+      <c r="E1" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="2" ht="15.15" spans="1:5">
+      <c r="A2" s="1" t="s">
+        <v>155</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>156</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>135</v>
+      </c>
+      <c r="D2" s="3" t="s">
+        <v>136</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>157</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1952,552 +2382,552 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:20">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="9" t="s">
         <v>25</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="9" t="s">
         <v>26</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="9" t="s">
         <v>27</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="9" t="s">
         <v>28</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" s="9" t="s">
         <v>29</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" s="9" t="s">
         <v>2</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" s="9" t="s">
         <v>1</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" s="9" t="s">
         <v>30</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" s="9" t="s">
         <v>31</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" s="9" t="s">
         <v>32</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" s="9" t="s">
         <v>33</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" s="9" t="s">
         <v>6</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="M1" s="9" t="s">
         <v>7</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="N1" s="9" t="s">
         <v>8</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="O1" s="9" t="s">
         <v>9</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="P1" s="9" t="s">
         <v>34</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="Q1" s="9" t="s">
         <v>35</v>
       </c>
-      <c r="R1" s="1" t="s">
+      <c r="R1" s="9" t="s">
         <v>36</v>
       </c>
-      <c r="S1" s="1" t="s">
+      <c r="S1" s="9" t="s">
         <v>37</v>
       </c>
-      <c r="T1" s="1" t="s">
+      <c r="T1" s="9" t="s">
         <v>38</v>
       </c>
     </row>
     <row r="2" spans="1:20">
-      <c r="A2" s="1" t="s">
+      <c r="A2" s="9" t="s">
         <v>18</v>
       </c>
-      <c r="B2" s="1" t="s">
+      <c r="B2" s="9" t="s">
         <v>39</v>
       </c>
-      <c r="C2" s="1" t="s">
+      <c r="C2" s="9" t="s">
         <v>20</v>
       </c>
-      <c r="D2" s="1" t="s">
+      <c r="D2" s="9" t="s">
         <v>40</v>
       </c>
-      <c r="E2" s="1">
+      <c r="E2" s="9">
         <v>12</v>
       </c>
-      <c r="F2" s="9" t="s">
+      <c r="F2" s="15" t="s">
         <v>12</v>
       </c>
-      <c r="G2" s="1" t="s">
+      <c r="G2" s="9" t="s">
         <v>11</v>
       </c>
-      <c r="H2" s="1" t="s">
+      <c r="H2" s="9" t="s">
         <v>19</v>
       </c>
-      <c r="I2" s="1" t="s">
+      <c r="I2" s="9" t="s">
         <v>41</v>
       </c>
-      <c r="J2" s="1" t="s">
+      <c r="J2" s="9" t="s">
         <v>14</v>
       </c>
-      <c r="K2" s="1">
+      <c r="K2" s="9">
         <v>6</v>
       </c>
-      <c r="L2" s="1">
+      <c r="L2" s="9">
         <v>1010301033</v>
       </c>
-      <c r="M2" s="1" t="s">
+      <c r="M2" s="9" t="s">
         <v>15</v>
       </c>
-      <c r="N2" s="1" t="s">
+      <c r="N2" s="9" t="s">
         <v>16</v>
       </c>
-      <c r="O2" s="1" t="s">
+      <c r="O2" s="9" t="s">
         <v>17</v>
       </c>
-      <c r="P2" s="1"/>
-      <c r="Q2" s="1"/>
-      <c r="R2" s="1"/>
-      <c r="S2" s="1">
+      <c r="P2" s="9"/>
+      <c r="Q2" s="9"/>
+      <c r="R2" s="9"/>
+      <c r="S2" s="9">
         <v>0</v>
       </c>
-      <c r="T2" s="1"/>
+      <c r="T2" s="9"/>
     </row>
     <row r="3" spans="1:20">
-      <c r="A3" s="1" t="s">
+      <c r="A3" s="9" t="s">
         <v>10</v>
       </c>
-      <c r="B3" s="1" t="s">
+      <c r="B3" s="9" t="s">
         <v>42</v>
       </c>
-      <c r="C3" s="1" t="s">
+      <c r="C3" s="9" t="s">
         <v>14</v>
       </c>
-      <c r="D3" s="10" t="s">
+      <c r="D3" s="16" t="s">
         <v>43</v>
       </c>
-      <c r="E3" s="1">
+      <c r="E3" s="9">
         <v>5</v>
       </c>
-      <c r="F3" s="1" t="s">
+      <c r="F3" s="9" t="s">
         <v>12</v>
       </c>
-      <c r="G3" s="1" t="s">
+      <c r="G3" s="9" t="s">
         <v>11</v>
       </c>
-      <c r="H3" s="1" t="s">
+      <c r="H3" s="9" t="s">
         <v>13</v>
       </c>
-      <c r="I3" s="1" t="s">
+      <c r="I3" s="9" t="s">
         <v>44</v>
       </c>
-      <c r="J3" s="1" t="s">
+      <c r="J3" s="9" t="s">
         <v>14</v>
       </c>
-      <c r="K3" s="1">
+      <c r="K3" s="9">
         <v>1</v>
       </c>
-      <c r="L3" s="1">
+      <c r="L3" s="9">
         <v>1010301033</v>
       </c>
-      <c r="M3" s="1" t="s">
+      <c r="M3" s="9" t="s">
         <v>15</v>
       </c>
-      <c r="N3" s="1" t="s">
+      <c r="N3" s="9" t="s">
         <v>16</v>
       </c>
-      <c r="O3" s="1" t="s">
+      <c r="O3" s="9" t="s">
         <v>17</v>
       </c>
-      <c r="P3" s="1"/>
-      <c r="Q3" s="1"/>
-      <c r="R3" s="1"/>
-      <c r="S3" s="1">
+      <c r="P3" s="9"/>
+      <c r="Q3" s="9"/>
+      <c r="R3" s="9"/>
+      <c r="S3" s="9">
         <v>0</v>
       </c>
-      <c r="T3" s="1"/>
+      <c r="T3" s="9"/>
     </row>
     <row r="4" spans="1:20">
-      <c r="A4" s="1" t="s">
+      <c r="A4" s="9" t="s">
         <v>21</v>
       </c>
-      <c r="B4" s="1" t="s">
+      <c r="B4" s="9" t="s">
         <v>45</v>
       </c>
-      <c r="C4" s="1" t="s">
+      <c r="C4" s="9" t="s">
         <v>14</v>
       </c>
-      <c r="D4" s="1">
+      <c r="D4" s="9">
         <v>123562</v>
       </c>
-      <c r="E4" s="1">
+      <c r="E4" s="9">
         <v>18</v>
       </c>
-      <c r="F4" s="1" t="s">
+      <c r="F4" s="9" t="s">
         <v>22</v>
       </c>
-      <c r="G4" s="1" t="s">
+      <c r="G4" s="9" t="s">
         <v>22</v>
       </c>
-      <c r="H4" s="1" t="s">
+      <c r="H4" s="9" t="s">
         <v>23</v>
       </c>
-      <c r="I4" s="1" t="s">
+      <c r="I4" s="9" t="s">
         <v>44</v>
       </c>
-      <c r="J4" s="1" t="s">
+      <c r="J4" s="9" t="s">
         <v>14</v>
       </c>
-      <c r="K4" s="1">
+      <c r="K4" s="9">
         <v>1</v>
       </c>
-      <c r="L4" s="1">
+      <c r="L4" s="9">
         <v>1011134888</v>
       </c>
-      <c r="M4" s="1" t="s">
+      <c r="M4" s="9" t="s">
         <v>46</v>
       </c>
-      <c r="N4" s="1" t="s">
+      <c r="N4" s="9" t="s">
         <v>16</v>
       </c>
-      <c r="O4" s="1" t="s">
+      <c r="O4" s="9" t="s">
         <v>17</v>
       </c>
-      <c r="P4" s="1"/>
-      <c r="Q4" s="1"/>
-      <c r="R4" s="1"/>
-      <c r="S4" s="1">
+      <c r="P4" s="9"/>
+      <c r="Q4" s="9"/>
+      <c r="R4" s="9"/>
+      <c r="S4" s="9">
         <v>0</v>
       </c>
-      <c r="T4" s="1"/>
+      <c r="T4" s="9"/>
     </row>
     <row r="5" spans="1:20">
-      <c r="A5" s="3" t="s">
+      <c r="A5" s="6" t="s">
         <v>47</v>
       </c>
-      <c r="B5" s="3" t="s">
+      <c r="B5" s="6" t="s">
         <v>47</v>
       </c>
-      <c r="C5" s="1" t="s">
+      <c r="C5" s="9" t="s">
         <v>14</v>
       </c>
-      <c r="D5" s="3" t="s">
+      <c r="D5" s="6" t="s">
         <v>40</v>
       </c>
-      <c r="E5" s="3">
+      <c r="E5" s="6">
         <v>12</v>
       </c>
-      <c r="F5" s="3" t="s">
+      <c r="F5" s="6" t="s">
         <v>48</v>
       </c>
-      <c r="G5" s="3" t="s">
+      <c r="G5" s="6" t="s">
         <v>49</v>
       </c>
-      <c r="H5" s="3" t="s">
+      <c r="H5" s="6" t="s">
         <v>50</v>
       </c>
-      <c r="I5" s="3" t="s">
+      <c r="I5" s="6" t="s">
         <v>44</v>
       </c>
-      <c r="J5" s="3" t="s">
+      <c r="J5" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="K5" s="3">
+      <c r="K5" s="6">
         <v>1</v>
       </c>
-      <c r="L5" s="3">
+      <c r="L5" s="6">
         <v>1010301001</v>
       </c>
-      <c r="M5" s="3" t="s">
+      <c r="M5" s="6" t="s">
         <v>51</v>
       </c>
-      <c r="N5" s="3" t="s">
+      <c r="N5" s="6" t="s">
         <v>52</v>
       </c>
-      <c r="O5" s="3" t="s">
+      <c r="O5" s="6" t="s">
         <v>53</v>
       </c>
-      <c r="P5" s="3"/>
-      <c r="Q5" s="3"/>
-      <c r="R5" s="3"/>
-      <c r="S5" s="1">
+      <c r="P5" s="6"/>
+      <c r="Q5" s="6"/>
+      <c r="R5" s="6"/>
+      <c r="S5" s="9">
         <v>0</v>
       </c>
-      <c r="T5" s="3"/>
+      <c r="T5" s="6"/>
     </row>
     <row r="6" spans="1:20">
-      <c r="A6" s="3" t="s">
+      <c r="A6" s="6" t="s">
         <v>54</v>
       </c>
-      <c r="B6" s="3" t="s">
+      <c r="B6" s="6" t="s">
         <v>54</v>
       </c>
-      <c r="C6" s="3" t="s">
+      <c r="C6" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="D6" s="8" t="s">
+      <c r="D6" s="14" t="s">
         <v>43</v>
       </c>
       <c r="E6">
         <v>5</v>
       </c>
-      <c r="F6" s="11" t="s">
+      <c r="F6" s="17" t="s">
         <v>12</v>
       </c>
-      <c r="G6" s="11" t="s">
+      <c r="G6" s="17" t="s">
         <v>11</v>
       </c>
-      <c r="H6" s="3" t="s">
+      <c r="H6" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="I6" s="3" t="s">
+      <c r="I6" s="6" t="s">
         <v>44</v>
       </c>
-      <c r="J6" s="3" t="s">
+      <c r="J6" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="K6" s="3">
+      <c r="K6" s="6">
         <v>1</v>
       </c>
-      <c r="L6" s="3">
+      <c r="L6" s="6">
         <v>1010301033</v>
       </c>
-      <c r="M6" s="3" t="s">
+      <c r="M6" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="N6" s="3" t="s">
+      <c r="N6" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="O6" s="3" t="s">
+      <c r="O6" s="6" t="s">
         <v>17</v>
       </c>
-      <c r="P6" s="3"/>
-      <c r="Q6" s="3"/>
-      <c r="R6" s="3"/>
-      <c r="S6" s="1">
+      <c r="P6" s="6"/>
+      <c r="Q6" s="6"/>
+      <c r="R6" s="6"/>
+      <c r="S6" s="9">
         <v>0</v>
       </c>
-      <c r="T6" s="3"/>
+      <c r="T6" s="6"/>
     </row>
     <row r="7" spans="1:20">
-      <c r="A7" s="12" t="s">
+      <c r="A7" s="18" t="s">
         <v>55</v>
       </c>
-      <c r="B7" s="12" t="s">
+      <c r="B7" s="18" t="s">
         <v>56</v>
       </c>
-      <c r="C7" s="12" t="s">
+      <c r="C7" s="18" t="s">
         <v>20</v>
       </c>
-      <c r="D7" s="12" t="s">
+      <c r="D7" s="18" t="s">
         <v>40</v>
       </c>
-      <c r="E7" s="12">
+      <c r="E7" s="18">
         <v>12</v>
       </c>
-      <c r="F7" s="13" t="s">
+      <c r="F7" s="19" t="s">
         <v>12</v>
       </c>
-      <c r="G7" s="12" t="s">
+      <c r="G7" s="18" t="s">
         <v>11</v>
       </c>
-      <c r="H7" s="12" t="s">
+      <c r="H7" s="18" t="s">
         <v>57</v>
       </c>
-      <c r="I7" s="12" t="s">
+      <c r="I7" s="18" t="s">
         <v>41</v>
       </c>
-      <c r="J7" s="12" t="s">
+      <c r="J7" s="18" t="s">
         <v>14</v>
       </c>
-      <c r="K7" s="12">
+      <c r="K7" s="18">
         <v>3</v>
       </c>
-      <c r="L7" s="12">
+      <c r="L7" s="18">
         <v>1010301003</v>
       </c>
-      <c r="M7" s="12" t="s">
+      <c r="M7" s="18" t="s">
         <v>58</v>
       </c>
-      <c r="N7" s="12" t="s">
+      <c r="N7" s="18" t="s">
         <v>16</v>
       </c>
-      <c r="O7" s="12" t="s">
+      <c r="O7" s="18" t="s">
         <v>17</v>
       </c>
-      <c r="P7" s="12"/>
-      <c r="Q7" s="12"/>
-      <c r="R7" s="12"/>
-      <c r="S7" s="12">
+      <c r="P7" s="18"/>
+      <c r="Q7" s="18"/>
+      <c r="R7" s="18"/>
+      <c r="S7" s="18">
         <v>0</v>
       </c>
-      <c r="T7" s="12"/>
+      <c r="T7" s="18"/>
     </row>
     <row r="8" spans="1:20">
-      <c r="A8" s="12" t="s">
+      <c r="A8" s="18" t="s">
         <v>59</v>
       </c>
-      <c r="B8" s="12" t="s">
+      <c r="B8" s="18" t="s">
         <v>60</v>
       </c>
-      <c r="C8" s="12" t="s">
+      <c r="C8" s="18" t="s">
         <v>14</v>
       </c>
-      <c r="D8" s="12" t="s">
+      <c r="D8" s="18" t="s">
         <v>43</v>
       </c>
-      <c r="E8" s="12">
+      <c r="E8" s="18">
         <v>5</v>
       </c>
-      <c r="F8" s="13" t="s">
+      <c r="F8" s="19" t="s">
         <v>12</v>
       </c>
-      <c r="G8" s="12" t="s">
+      <c r="G8" s="18" t="s">
         <v>11</v>
       </c>
-      <c r="H8" s="12" t="s">
+      <c r="H8" s="18" t="s">
         <v>57</v>
       </c>
-      <c r="I8" s="12" t="s">
+      <c r="I8" s="18" t="s">
         <v>41</v>
       </c>
-      <c r="J8" s="12" t="s">
+      <c r="J8" s="18" t="s">
         <v>14</v>
       </c>
-      <c r="K8" s="12">
+      <c r="K8" s="18">
         <v>0</v>
       </c>
-      <c r="L8" s="12">
+      <c r="L8" s="18">
         <v>1010301003</v>
       </c>
-      <c r="M8" s="12" t="s">
+      <c r="M8" s="18" t="s">
         <v>58</v>
       </c>
-      <c r="N8" s="12" t="s">
+      <c r="N8" s="18" t="s">
         <v>16</v>
       </c>
-      <c r="O8" s="12" t="s">
+      <c r="O8" s="18" t="s">
         <v>17</v>
       </c>
-      <c r="P8" s="12"/>
-      <c r="Q8" s="12"/>
-      <c r="R8" s="12"/>
-      <c r="S8" s="12">
+      <c r="P8" s="18"/>
+      <c r="Q8" s="18"/>
+      <c r="R8" s="18"/>
+      <c r="S8" s="18">
         <v>0</v>
       </c>
-      <c r="T8" s="12"/>
+      <c r="T8" s="18"/>
     </row>
     <row r="9" spans="1:20">
-      <c r="A9" s="12" t="s">
+      <c r="A9" s="18" t="s">
         <v>61</v>
       </c>
-      <c r="B9" s="12" t="s">
+      <c r="B9" s="18" t="s">
         <v>61</v>
       </c>
-      <c r="C9" s="12" t="s">
+      <c r="C9" s="18" t="s">
         <v>14</v>
       </c>
-      <c r="D9" s="12" t="s">
+      <c r="D9" s="18" t="s">
         <v>43</v>
       </c>
-      <c r="E9" s="12">
+      <c r="E9" s="18">
         <v>5</v>
       </c>
-      <c r="F9" s="13" t="s">
+      <c r="F9" s="19" t="s">
         <v>12</v>
       </c>
-      <c r="G9" s="12" t="s">
+      <c r="G9" s="18" t="s">
         <v>11</v>
       </c>
-      <c r="H9" s="12" t="s">
+      <c r="H9" s="18" t="s">
         <v>57</v>
       </c>
-      <c r="I9" s="12" t="s">
+      <c r="I9" s="18" t="s">
         <v>41</v>
       </c>
-      <c r="J9" s="12" t="s">
+      <c r="J9" s="18" t="s">
         <v>14</v>
       </c>
-      <c r="K9" s="12">
+      <c r="K9" s="18">
         <v>0</v>
       </c>
-      <c r="L9" s="12">
+      <c r="L9" s="18">
         <v>1010301003</v>
       </c>
-      <c r="M9" s="12" t="s">
+      <c r="M9" s="18" t="s">
         <v>58</v>
       </c>
-      <c r="N9" s="12" t="s">
+      <c r="N9" s="18" t="s">
         <v>16</v>
       </c>
-      <c r="O9" s="12" t="s">
+      <c r="O9" s="18" t="s">
         <v>17</v>
       </c>
-      <c r="P9" s="12"/>
-      <c r="Q9" s="12"/>
-      <c r="R9" s="12"/>
-      <c r="S9" s="12">
+      <c r="P9" s="18"/>
+      <c r="Q9" s="18"/>
+      <c r="R9" s="18"/>
+      <c r="S9" s="18">
         <v>0</v>
       </c>
-      <c r="T9" s="12"/>
+      <c r="T9" s="18"/>
     </row>
     <row r="10" spans="1:20">
-      <c r="A10" s="3" t="s">
+      <c r="A10" s="6" t="s">
         <v>62</v>
       </c>
-      <c r="B10" s="3" t="s">
+      <c r="B10" s="6" t="s">
         <v>62</v>
       </c>
-      <c r="C10" s="3" t="s">
+      <c r="C10" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="D10" s="12" t="s">
+      <c r="D10" s="18" t="s">
         <v>43</v>
       </c>
-      <c r="E10" s="12">
+      <c r="E10" s="18">
         <v>5</v>
       </c>
-      <c r="F10" s="1" t="s">
+      <c r="F10" s="9" t="s">
         <v>22</v>
       </c>
-      <c r="G10" s="1" t="s">
+      <c r="G10" s="9" t="s">
         <v>22</v>
       </c>
-      <c r="H10" s="1" t="s">
+      <c r="H10" s="9" t="s">
         <v>63</v>
       </c>
-      <c r="I10" s="1" t="s">
+      <c r="I10" s="9" t="s">
         <v>44</v>
       </c>
-      <c r="J10" s="1" t="s">
+      <c r="J10" s="9" t="s">
         <v>14</v>
       </c>
-      <c r="K10" s="1">
+      <c r="K10" s="9">
         <v>1</v>
       </c>
-      <c r="L10" s="6">
+      <c r="L10" s="12">
         <v>1000000001</v>
       </c>
-      <c r="M10" s="3" t="s">
+      <c r="M10" s="6" t="s">
         <v>64</v>
       </c>
-      <c r="N10" s="3" t="s">
+      <c r="N10" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="O10" s="3" t="s">
+      <c r="O10" s="6" t="s">
         <v>17</v>
       </c>
-      <c r="P10" s="12"/>
-      <c r="Q10" s="12"/>
-      <c r="R10" s="12"/>
-      <c r="S10" s="12">
+      <c r="P10" s="18"/>
+      <c r="Q10" s="18"/>
+      <c r="R10" s="18"/>
+      <c r="S10" s="18">
         <v>0</v>
       </c>
-      <c r="T10" s="12"/>
+      <c r="T10" s="18"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2525,128 +2955,128 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:18">
-      <c r="A1" s="3" t="s">
+      <c r="A1" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="B1" s="3" t="s">
+      <c r="B1" s="6" t="s">
         <v>26</v>
       </c>
-      <c r="C1" s="3" t="s">
+      <c r="C1" s="6" t="s">
         <v>27</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="9" t="s">
         <v>6</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" s="9" t="s">
         <v>7</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" s="9" t="s">
         <v>8</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" s="9" t="s">
         <v>9</v>
       </c>
-      <c r="H1" s="3" t="s">
+      <c r="H1" s="6" t="s">
         <v>30</v>
       </c>
-      <c r="I1" s="3" t="s">
+      <c r="I1" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="J1" s="3" t="s">
+      <c r="J1" s="6" t="s">
         <v>31</v>
       </c>
-      <c r="K1" s="3" t="s">
+      <c r="K1" s="6" t="s">
         <v>65</v>
       </c>
-      <c r="L1" s="3" t="s">
+      <c r="L1" s="6" t="s">
         <v>33</v>
       </c>
-      <c r="M1" s="7"/>
-      <c r="N1" s="7"/>
-      <c r="O1" s="7"/>
-      <c r="P1" s="7"/>
-      <c r="Q1" s="7"/>
-      <c r="R1" s="7"/>
+      <c r="M1" s="13"/>
+      <c r="N1" s="13"/>
+      <c r="O1" s="13"/>
+      <c r="P1" s="13"/>
+      <c r="Q1" s="13"/>
+      <c r="R1" s="13"/>
     </row>
     <row r="2" spans="1:18">
-      <c r="A2" s="3" t="s">
+      <c r="A2" s="6" t="s">
         <v>54</v>
       </c>
-      <c r="B2" s="3" t="s">
+      <c r="B2" s="6" t="s">
         <v>54</v>
       </c>
-      <c r="C2" s="3" t="s">
+      <c r="C2" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="D2" s="3">
+      <c r="D2" s="6">
         <v>1010301033</v>
       </c>
-      <c r="E2" s="3" t="s">
+      <c r="E2" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="F2" s="3" t="s">
+      <c r="F2" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="G2" s="3" t="s">
+      <c r="G2" s="6" t="s">
         <v>17</v>
       </c>
-      <c r="H2" s="3" t="s">
+      <c r="H2" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="I2" s="8" t="s">
+      <c r="I2" s="14" t="s">
         <v>43</v>
       </c>
-      <c r="J2" s="3" t="s">
+      <c r="J2" s="6" t="s">
         <v>44</v>
       </c>
-      <c r="K2" s="3" t="s">
+      <c r="K2" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="L2" s="3">
+      <c r="L2" s="6">
         <v>1</v>
       </c>
-      <c r="M2" s="7"/>
-      <c r="N2" s="7"/>
-      <c r="O2" s="7"/>
-      <c r="P2" s="7"/>
-      <c r="Q2" s="7"/>
-      <c r="R2" s="7"/>
+      <c r="M2" s="13"/>
+      <c r="N2" s="13"/>
+      <c r="O2" s="13"/>
+      <c r="P2" s="13"/>
+      <c r="Q2" s="13"/>
+      <c r="R2" s="13"/>
     </row>
     <row r="3" spans="1:12">
-      <c r="A3" s="3" t="s">
+      <c r="A3" s="6" t="s">
         <v>62</v>
       </c>
-      <c r="B3" s="3" t="s">
+      <c r="B3" s="6" t="s">
         <v>62</v>
       </c>
-      <c r="C3" s="3" t="s">
+      <c r="C3" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="D3" s="6">
+      <c r="D3" s="12">
         <v>1000000001</v>
       </c>
-      <c r="E3" s="3" t="s">
+      <c r="E3" s="6" t="s">
         <v>64</v>
       </c>
-      <c r="F3" s="3" t="s">
+      <c r="F3" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="G3" s="3" t="s">
+      <c r="G3" s="6" t="s">
         <v>17</v>
       </c>
-      <c r="H3" s="3" t="s">
+      <c r="H3" s="6" t="s">
         <v>23</v>
       </c>
-      <c r="I3" s="8" t="s">
+      <c r="I3" s="14" t="s">
         <v>43</v>
       </c>
-      <c r="J3" s="3" t="s">
+      <c r="J3" s="6" t="s">
         <v>44</v>
       </c>
-      <c r="K3" s="3" t="s">
+      <c r="K3" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="L3" s="3">
+      <c r="L3" s="6">
         <v>1</v>
       </c>
     </row>
@@ -2671,60 +3101,60 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6">
-      <c r="A1" s="4" t="s">
+      <c r="A1" s="10" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="4" t="s">
+      <c r="B1" s="10" t="s">
         <v>66</v>
       </c>
-      <c r="C1" s="4" t="s">
+      <c r="C1" s="10" t="s">
         <v>67</v>
       </c>
-      <c r="D1" s="5" t="s">
+      <c r="D1" s="11" t="s">
         <v>68</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" s="9" t="s">
         <v>69</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" s="9" t="s">
         <v>70</v>
       </c>
     </row>
     <row r="2" spans="1:6">
-      <c r="A2" s="3" t="s">
+      <c r="A2" s="6" t="s">
         <v>59</v>
       </c>
-      <c r="B2" s="3">
+      <c r="B2" s="6">
         <v>50</v>
       </c>
-      <c r="C2" s="3">
+      <c r="C2" s="6">
         <v>70</v>
       </c>
-      <c r="D2" s="3" t="s">
+      <c r="D2" s="6" t="s">
         <v>71</v>
       </c>
-      <c r="E2" s="3"/>
-      <c r="F2" s="2" t="s">
+      <c r="E2" s="6"/>
+      <c r="F2" s="4" t="s">
         <v>72</v>
       </c>
     </row>
     <row r="3" spans="1:6">
-      <c r="A3" s="3" t="s">
+      <c r="A3" s="6" t="s">
         <v>61</v>
       </c>
-      <c r="B3" s="3">
+      <c r="B3" s="6">
         <v>40</v>
       </c>
-      <c r="C3" s="3">
+      <c r="C3" s="6">
         <v>26</v>
       </c>
-      <c r="D3" s="3" t="s">
+      <c r="D3" s="6" t="s">
         <v>73</v>
       </c>
-      <c r="E3" s="2" t="s">
+      <c r="E3" s="4" t="s">
         <v>74</v>
       </c>
-      <c r="F3" s="2">
+      <c r="F3" s="4">
         <v>2</v>
       </c>
     </row>
@@ -2749,80 +3179,80 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6">
-      <c r="A1" s="4" t="s">
+      <c r="A1" s="10" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="4" t="s">
+      <c r="B1" s="10" t="s">
         <v>66</v>
       </c>
-      <c r="C1" s="4" t="s">
+      <c r="C1" s="10" t="s">
         <v>67</v>
       </c>
-      <c r="D1" s="5" t="s">
+      <c r="D1" s="11" t="s">
         <v>68</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" s="9" t="s">
         <v>69</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" s="9" t="s">
         <v>70</v>
       </c>
     </row>
     <row r="2" spans="1:6">
-      <c r="A2" s="1" t="s">
+      <c r="A2" s="9" t="s">
         <v>59</v>
       </c>
-      <c r="B2" s="3">
+      <c r="B2" s="6">
         <v>150</v>
       </c>
-      <c r="C2" s="3">
+      <c r="C2" s="6">
         <v>45</v>
       </c>
-      <c r="D2" s="3" t="s">
+      <c r="D2" s="6" t="s">
         <v>71</v>
       </c>
-      <c r="E2" s="3"/>
-      <c r="F2" s="2" t="s">
+      <c r="E2" s="6"/>
+      <c r="F2" s="4" t="s">
         <v>75</v>
       </c>
     </row>
     <row r="3" spans="1:6">
-      <c r="A3" s="1" t="s">
+      <c r="A3" s="9" t="s">
         <v>76</v>
       </c>
-      <c r="B3" s="3">
+      <c r="B3" s="6">
         <v>40</v>
       </c>
-      <c r="C3" s="3">
+      <c r="C3" s="6">
         <v>26</v>
       </c>
-      <c r="D3" s="3" t="s">
+      <c r="D3" s="6" t="s">
         <v>77</v>
       </c>
-      <c r="E3" s="2" t="s">
+      <c r="E3" s="4" t="s">
         <v>74</v>
       </c>
-      <c r="F3" s="2">
+      <c r="F3" s="4">
         <v>2</v>
       </c>
     </row>
     <row r="4" spans="1:6">
-      <c r="A4" s="1" t="s">
+      <c r="A4" s="9" t="s">
         <v>61</v>
       </c>
-      <c r="B4" s="3">
+      <c r="B4" s="6">
         <v>50</v>
       </c>
-      <c r="C4" s="3">
+      <c r="C4" s="6">
         <v>70</v>
       </c>
-      <c r="D4" s="3" t="s">
+      <c r="D4" s="6" t="s">
         <v>73</v>
       </c>
-      <c r="E4" s="3" t="s">
+      <c r="E4" s="6" t="s">
         <v>75</v>
       </c>
-      <c r="F4" s="2"/>
+      <c r="F4" s="4"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2894,90 +3324,90 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="9" t="s">
         <v>83</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="9" t="s">
         <v>84</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="9" t="s">
         <v>80</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="9" t="s">
         <v>85</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" s="9" t="s">
         <v>68</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" s="9" t="s">
         <v>69</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" s="9" t="s">
         <v>70</v>
       </c>
     </row>
     <row r="2" spans="1:7">
-      <c r="A2" s="1" t="s">
+      <c r="A2" s="9" t="s">
         <v>86</v>
       </c>
-      <c r="B2" s="1">
+      <c r="B2" s="9">
         <v>524</v>
       </c>
-      <c r="C2" s="1">
+      <c r="C2" s="9">
         <v>524</v>
       </c>
-      <c r="D2" s="1">
+      <c r="D2" s="9">
         <v>2</v>
       </c>
-      <c r="E2" s="2" t="s">
+      <c r="E2" s="4" t="s">
         <v>71</v>
       </c>
-      <c r="F2" s="2" t="s">
+      <c r="F2" s="4" t="s">
         <v>74</v>
       </c>
-      <c r="G2" s="2" t="s">
+      <c r="G2" s="4" t="s">
         <v>87</v>
       </c>
     </row>
     <row r="3" spans="1:7">
-      <c r="A3" s="1" t="s">
+      <c r="A3" s="9" t="s">
         <v>88</v>
       </c>
-      <c r="B3" s="1">
+      <c r="B3" s="9">
         <v>232</v>
       </c>
-      <c r="C3" s="1">
+      <c r="C3" s="9">
         <v>232</v>
       </c>
-      <c r="D3" s="1">
+      <c r="D3" s="9">
         <v>7.9</v>
       </c>
-      <c r="E3" s="2" t="s">
+      <c r="E3" s="4" t="s">
         <v>73</v>
       </c>
-      <c r="F3" s="2" t="s">
+      <c r="F3" s="4" t="s">
         <v>89</v>
       </c>
-      <c r="G3" s="3"/>
+      <c r="G3" s="6"/>
     </row>
     <row r="4" spans="1:7">
-      <c r="A4" s="3" t="s">
+      <c r="A4" s="6" t="s">
         <v>90</v>
       </c>
-      <c r="B4" s="3">
+      <c r="B4" s="6">
         <v>232</v>
       </c>
-      <c r="C4" s="3">
+      <c r="C4" s="6">
         <v>232</v>
       </c>
-      <c r="D4" s="3">
+      <c r="D4" s="6">
         <v>2.32</v>
       </c>
-      <c r="E4" s="2" t="s">
+      <c r="E4" s="4" t="s">
         <v>77</v>
       </c>
-      <c r="F4" s="3"/>
-      <c r="G4" s="3"/>
+      <c r="F4" s="6"/>
+      <c r="G4" s="6"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -3001,90 +3431,620 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="9" t="s">
         <v>83</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="9" t="s">
         <v>84</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="9" t="s">
         <v>80</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="9" t="s">
         <v>85</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" s="9" t="s">
         <v>68</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" s="9" t="s">
         <v>69</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" s="9" t="s">
         <v>70</v>
       </c>
     </row>
     <row r="2" spans="1:7">
-      <c r="A2" s="1" t="s">
+      <c r="A2" s="9" t="s">
         <v>86</v>
       </c>
-      <c r="B2" s="1">
+      <c r="B2" s="9">
         <v>22</v>
       </c>
-      <c r="C2" s="1">
+      <c r="C2" s="9">
         <v>524</v>
       </c>
-      <c r="D2" s="1">
+      <c r="D2" s="9">
         <v>2</v>
       </c>
-      <c r="E2" s="2" t="s">
+      <c r="E2" s="4" t="s">
         <v>71</v>
       </c>
-      <c r="F2" s="2" t="s">
+      <c r="F2" s="4" t="s">
         <v>74</v>
       </c>
-      <c r="G2" s="2" t="s">
+      <c r="G2" s="4" t="s">
         <v>87</v>
       </c>
     </row>
     <row r="3" spans="1:7">
-      <c r="A3" s="1" t="s">
+      <c r="A3" s="9" t="s">
         <v>88</v>
       </c>
-      <c r="B3" s="1">
+      <c r="B3" s="9">
         <v>34</v>
       </c>
-      <c r="C3" s="1">
+      <c r="C3" s="9">
         <v>232</v>
       </c>
-      <c r="D3" s="1">
+      <c r="D3" s="9">
         <v>7.9</v>
       </c>
-      <c r="E3" s="2" t="s">
+      <c r="E3" s="4" t="s">
         <v>73</v>
       </c>
-      <c r="F3" s="2" t="s">
+      <c r="F3" s="4" t="s">
         <v>89</v>
       </c>
-      <c r="G3" s="3"/>
+      <c r="G3" s="6"/>
     </row>
     <row r="4" spans="1:7">
-      <c r="A4" s="3" t="s">
+      <c r="A4" s="6" t="s">
         <v>90</v>
       </c>
-      <c r="B4" s="3">
+      <c r="B4" s="6">
         <v>67</v>
       </c>
-      <c r="C4" s="3">
+      <c r="C4" s="6">
         <v>232</v>
       </c>
-      <c r="D4" s="3">
+      <c r="D4" s="6">
         <v>2.32</v>
       </c>
-      <c r="E4" s="2" t="s">
+      <c r="E4" s="4" t="s">
         <v>77</v>
       </c>
-      <c r="F4" s="3"/>
-      <c r="G4" s="3"/>
+      <c r="F4" s="6"/>
+      <c r="G4" s="6"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <headerFooter/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
+  <dimension ref="A1:S9"/>
+  <sheetFormatPr defaultColWidth="8.88888888888889" defaultRowHeight="14.4"/>
+  <cols>
+    <col min="1" max="1" width="39.6666666666667" customWidth="1"/>
+    <col min="2" max="2" width="10.1111111111111" customWidth="1"/>
+    <col min="3" max="3" width="39.6666666666667" customWidth="1"/>
+    <col min="4" max="4" width="11" customWidth="1"/>
+    <col min="5" max="5" width="13.2222222222222" customWidth="1"/>
+    <col min="6" max="6" width="8.88888888888889" customWidth="1"/>
+    <col min="7" max="7" width="17.8888888888889" customWidth="1"/>
+    <col min="8" max="8" width="19.5555555555556" customWidth="1"/>
+    <col min="9" max="9" width="23.7777777777778" customWidth="1"/>
+    <col min="10" max="10" width="12.6666666666667" customWidth="1"/>
+    <col min="11" max="11" width="11.8888888888889" customWidth="1"/>
+    <col min="12" max="12" width="17.4444444444444" customWidth="1"/>
+    <col min="13" max="14" width="39.6666666666667" customWidth="1"/>
+    <col min="15" max="15" width="25.7777777777778" customWidth="1"/>
+    <col min="16" max="17" width="16.5555555555556" customWidth="1"/>
+    <col min="18" max="18" width="11.5555555555556" customWidth="1"/>
+    <col min="19" max="19" width="14.8888888888889" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:19">
+      <c r="A1" s="6" t="s">
+        <v>91</v>
+      </c>
+      <c r="B1" s="6" t="s">
+        <v>92</v>
+      </c>
+      <c r="C1" s="6" t="s">
+        <v>93</v>
+      </c>
+      <c r="D1" s="6" t="s">
+        <v>94</v>
+      </c>
+      <c r="E1" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="F1" s="6" t="s">
+        <v>95</v>
+      </c>
+      <c r="G1" s="6" t="s">
+        <v>96</v>
+      </c>
+      <c r="H1" s="6" t="s">
+        <v>34</v>
+      </c>
+      <c r="I1" s="6" t="s">
+        <v>97</v>
+      </c>
+      <c r="J1" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="K1" s="6" t="s">
+        <v>98</v>
+      </c>
+      <c r="L1" s="6" t="s">
+        <v>99</v>
+      </c>
+      <c r="M1" s="6" t="s">
+        <v>100</v>
+      </c>
+      <c r="N1" s="6" t="s">
+        <v>101</v>
+      </c>
+      <c r="O1" s="6" t="s">
+        <v>102</v>
+      </c>
+      <c r="P1" s="6" t="s">
+        <v>103</v>
+      </c>
+      <c r="Q1" s="6" t="s">
+        <v>1</v>
+      </c>
+      <c r="R1" s="6" t="s">
+        <v>104</v>
+      </c>
+      <c r="S1" s="8" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="2" spans="1:19">
+      <c r="A2" s="7" t="s">
+        <v>106</v>
+      </c>
+      <c r="B2" s="6">
+        <v>0</v>
+      </c>
+      <c r="C2" s="7" t="s">
+        <v>106</v>
+      </c>
+      <c r="D2" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="E2" s="6" t="s">
+        <v>40</v>
+      </c>
+      <c r="F2" s="6">
+        <v>12</v>
+      </c>
+      <c r="G2" s="6" t="s">
+        <v>41</v>
+      </c>
+      <c r="H2" s="6"/>
+      <c r="I2" s="6"/>
+      <c r="J2" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="K2" s="6">
+        <v>1</v>
+      </c>
+      <c r="L2" s="6" t="s">
+        <v>107</v>
+      </c>
+      <c r="M2" s="6"/>
+      <c r="N2" s="6"/>
+      <c r="O2" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="P2" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="Q2" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="R2" s="6" t="s">
+        <v>108</v>
+      </c>
+      <c r="S2" s="5" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="3" spans="1:19">
+      <c r="A3" s="7" t="s">
+        <v>110</v>
+      </c>
+      <c r="B3" s="6">
+        <v>0</v>
+      </c>
+      <c r="C3" s="7" t="s">
+        <v>110</v>
+      </c>
+      <c r="D3" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="E3" s="7">
+        <v>772213</v>
+      </c>
+      <c r="F3" s="6">
+        <v>5</v>
+      </c>
+      <c r="G3" s="6" t="s">
+        <v>41</v>
+      </c>
+      <c r="H3" s="6"/>
+      <c r="I3" s="6"/>
+      <c r="J3" s="6" t="s">
+        <v>20</v>
+      </c>
+      <c r="K3" s="6">
+        <v>3</v>
+      </c>
+      <c r="L3" s="6" t="s">
+        <v>107</v>
+      </c>
+      <c r="M3" s="6"/>
+      <c r="N3" s="6"/>
+      <c r="O3" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="P3" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="Q3" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="R3" s="6" t="s">
+        <v>108</v>
+      </c>
+      <c r="S3" s="5" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="4" spans="1:19">
+      <c r="A4" s="6" t="s">
+        <v>111</v>
+      </c>
+      <c r="B4" s="6">
+        <v>0</v>
+      </c>
+      <c r="C4" s="6" t="s">
+        <v>111</v>
+      </c>
+      <c r="D4" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="E4" s="6" t="s">
+        <v>40</v>
+      </c>
+      <c r="F4" s="6">
+        <v>12</v>
+      </c>
+      <c r="G4" s="8" t="s">
+        <v>112</v>
+      </c>
+      <c r="H4" s="6"/>
+      <c r="I4" s="6"/>
+      <c r="J4" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="K4" s="6">
+        <v>1</v>
+      </c>
+      <c r="L4" s="6" t="s">
+        <v>107</v>
+      </c>
+      <c r="M4" s="6" t="s">
+        <v>111</v>
+      </c>
+      <c r="N4" s="6" t="s">
+        <v>111</v>
+      </c>
+      <c r="O4" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="P4" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="Q4" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="R4" s="6" t="s">
+        <v>108</v>
+      </c>
+      <c r="S4" s="5" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="5" spans="1:19">
+      <c r="A5" s="6" t="s">
+        <v>113</v>
+      </c>
+      <c r="B5" s="8">
+        <v>0</v>
+      </c>
+      <c r="C5" s="6" t="s">
+        <v>113</v>
+      </c>
+      <c r="D5" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="E5" s="6">
+        <v>75052200</v>
+      </c>
+      <c r="F5" s="8">
+        <v>5</v>
+      </c>
+      <c r="G5" s="8" t="s">
+        <v>112</v>
+      </c>
+      <c r="H5" s="6"/>
+      <c r="I5" s="6"/>
+      <c r="J5" s="8" t="s">
+        <v>20</v>
+      </c>
+      <c r="K5" s="8">
+        <v>2</v>
+      </c>
+      <c r="L5" s="6" t="s">
+        <v>107</v>
+      </c>
+      <c r="M5" s="6" t="s">
+        <v>113</v>
+      </c>
+      <c r="N5" s="6" t="s">
+        <v>113</v>
+      </c>
+      <c r="O5" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="P5" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="Q5" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="R5" s="6" t="s">
+        <v>114</v>
+      </c>
+      <c r="S5" s="5" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="6" spans="1:19">
+      <c r="A6" s="8" t="s">
+        <v>115</v>
+      </c>
+      <c r="B6" s="8">
+        <v>0</v>
+      </c>
+      <c r="C6" s="6" t="s">
+        <v>115</v>
+      </c>
+      <c r="D6" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="E6" s="8" t="s">
+        <v>40</v>
+      </c>
+      <c r="F6" s="8">
+        <v>12</v>
+      </c>
+      <c r="G6" s="8" t="s">
+        <v>116</v>
+      </c>
+      <c r="H6" s="8" t="s">
+        <v>117</v>
+      </c>
+      <c r="I6" s="6"/>
+      <c r="J6" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="K6" s="8">
+        <v>1</v>
+      </c>
+      <c r="L6" s="6" t="s">
+        <v>107</v>
+      </c>
+      <c r="M6" s="8" t="s">
+        <v>115</v>
+      </c>
+      <c r="N6" s="8" t="s">
+        <v>115</v>
+      </c>
+      <c r="O6" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="P6" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="Q6" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="R6" s="6" t="s">
+        <v>108</v>
+      </c>
+      <c r="S6" s="5" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="7" spans="1:19">
+      <c r="A7" s="8" t="s">
+        <v>118</v>
+      </c>
+      <c r="B7" s="8">
+        <v>0</v>
+      </c>
+      <c r="C7" s="6" t="s">
+        <v>118</v>
+      </c>
+      <c r="D7" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="E7" s="8" t="s">
+        <v>40</v>
+      </c>
+      <c r="F7" s="8">
+        <v>12</v>
+      </c>
+      <c r="G7" s="8" t="s">
+        <v>116</v>
+      </c>
+      <c r="H7" s="8" t="s">
+        <v>119</v>
+      </c>
+      <c r="I7" s="6"/>
+      <c r="J7" s="8" t="s">
+        <v>20</v>
+      </c>
+      <c r="K7" s="8">
+        <v>4</v>
+      </c>
+      <c r="L7" s="6" t="s">
+        <v>107</v>
+      </c>
+      <c r="M7" s="8" t="s">
+        <v>118</v>
+      </c>
+      <c r="N7" s="8" t="s">
+        <v>118</v>
+      </c>
+      <c r="O7" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="P7" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="Q7" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="R7" s="6" t="s">
+        <v>108</v>
+      </c>
+      <c r="S7" s="5" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="8" spans="1:19">
+      <c r="A8" s="6" t="s">
+        <v>120</v>
+      </c>
+      <c r="B8" s="8">
+        <v>0</v>
+      </c>
+      <c r="C8" s="6" t="s">
+        <v>120</v>
+      </c>
+      <c r="D8" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="E8" s="6" t="s">
+        <v>121</v>
+      </c>
+      <c r="F8" s="8">
+        <v>5</v>
+      </c>
+      <c r="G8" s="8" t="s">
+        <v>122</v>
+      </c>
+      <c r="H8" s="6"/>
+      <c r="I8" s="6">
+        <v>95</v>
+      </c>
+      <c r="J8" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="K8" s="8">
+        <v>1</v>
+      </c>
+      <c r="L8" s="6" t="s">
+        <v>107</v>
+      </c>
+      <c r="M8" s="6" t="s">
+        <v>120</v>
+      </c>
+      <c r="N8" s="6" t="s">
+        <v>120</v>
+      </c>
+      <c r="O8" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="P8" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="Q8" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="R8" s="6" t="s">
+        <v>108</v>
+      </c>
+      <c r="S8" s="5" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="9" spans="1:19">
+      <c r="A9" s="8" t="s">
+        <v>123</v>
+      </c>
+      <c r="B9" s="8">
+        <v>0</v>
+      </c>
+      <c r="C9" s="6" t="s">
+        <v>123</v>
+      </c>
+      <c r="D9" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="E9" s="8" t="s">
+        <v>40</v>
+      </c>
+      <c r="F9" s="8">
+        <v>12</v>
+      </c>
+      <c r="G9" s="8" t="s">
+        <v>122</v>
+      </c>
+      <c r="H9" s="6"/>
+      <c r="I9" s="6">
+        <v>97</v>
+      </c>
+      <c r="J9" s="8" t="s">
+        <v>20</v>
+      </c>
+      <c r="K9" s="8">
+        <v>4</v>
+      </c>
+      <c r="L9" s="6" t="s">
+        <v>107</v>
+      </c>
+      <c r="M9" s="8" t="s">
+        <v>123</v>
+      </c>
+      <c r="N9" s="8" t="s">
+        <v>123</v>
+      </c>
+      <c r="O9" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="P9" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="Q9" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="R9" s="6" t="s">
+        <v>108</v>
+      </c>
+      <c r="S9" s="5" t="s">
+        <v>109</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Added Item Details, TestDatas And Item Details Handler
Added Item Details, TestDatas And Item Details Handler
</commit_message>
<xml_diff>
--- a/testdata/ItemDetails.xlsx
+++ b/testdata/ItemDetails.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="23040" windowHeight="9120" firstSheet="6" activeTab="10"/>
+    <workbookView windowWidth="23040" windowHeight="9120" firstSheet="6" activeTab="11"/>
   </bookViews>
   <sheets>
     <sheet name="PR Details" sheetId="1" r:id="rId1"/>
@@ -18,6 +18,7 @@
     <sheet name="SO Details" sheetId="9" r:id="rId9"/>
     <sheet name="Customer SO Details" sheetId="10" r:id="rId10"/>
     <sheet name="Open Sales" sheetId="11" r:id="rId11"/>
+    <sheet name="SI Details" sheetId="12" r:id="rId12"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -37,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="427" uniqueCount="158">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="483" uniqueCount="176">
   <si>
     <t>ITEM_NAME</t>
   </si>
@@ -512,6 +513,60 @@
   </si>
   <si>
     <t>OPSO1/00092/24-25</t>
+  </si>
+  <si>
+    <t>Customer_Name</t>
+  </si>
+  <si>
+    <t>Currency</t>
+  </si>
+  <si>
+    <t>SI_Type</t>
+  </si>
+  <si>
+    <t>Loc_Id</t>
+  </si>
+  <si>
+    <t>Unit</t>
+  </si>
+  <si>
+    <t>GST_Classification</t>
+  </si>
+  <si>
+    <t>GST_Type</t>
+  </si>
+  <si>
+    <t>ARUN PVT LTD.</t>
+  </si>
+  <si>
+    <t>INR</t>
+  </si>
+  <si>
+    <t>SI - GENERAL</t>
+  </si>
+  <si>
+    <t>Local</t>
+  </si>
+  <si>
+    <t>Registered</t>
+  </si>
+  <si>
+    <t>USD</t>
+  </si>
+  <si>
+    <t>AJK ENTERPRISES</t>
+  </si>
+  <si>
+    <t>PANDI PVT. LTD</t>
+  </si>
+  <si>
+    <t>PRAKASH PVT. LTD.</t>
+  </si>
+  <si>
+    <t>CHENNAI SEZ</t>
+  </si>
+  <si>
+    <t>SEZ-Unit</t>
   </si>
 </sst>
 </file>
@@ -524,13 +579,26 @@
     <numFmt numFmtId="178" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
     <numFmt numFmtId="179" formatCode="_ &quot;₹&quot;* #,##0_ ;_ &quot;₹&quot;* \-#,##0_ ;_ &quot;₹&quot;* &quot;-&quot;_ ;_ @_ "/>
   </numFmts>
-  <fonts count="28">
+  <fonts count="30">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <charset val="134"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
+      <charset val="134"/>
     </font>
     <font>
       <sz val="9"/>
@@ -727,12 +795,18 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="35">
+  <fills count="36">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
@@ -942,6 +1016,21 @@
       <diagonal/>
     </border>
     <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
       <left style="medium">
         <color rgb="FF000000"/>
       </left>
@@ -953,21 +1042,6 @@
       </top>
       <bottom style="medium">
         <color rgb="FF000000"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
       </bottom>
       <diagonal/>
     </border>
@@ -1089,211 +1163,220 @@
     <xf numFmtId="179" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="3" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="3" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="5" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="5" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="6" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="5" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="19" fillId="6" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="7" borderId="8" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="10" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="7" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="7" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="8" borderId="8" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="10" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="35" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="28">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFill="1" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="2" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="49" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="49" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="49" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="49" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="justify" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -1845,324 +1928,324 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10">
-      <c r="A1" s="21" t="s">
+      <c r="A1" s="24" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="21" t="s">
+      <c r="B1" s="24" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="21" t="s">
+      <c r="C1" s="24" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="21" t="s">
+      <c r="D1" s="24" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="21" t="s">
+      <c r="E1" s="24" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="21" t="s">
+      <c r="F1" s="24" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="21" t="s">
+      <c r="G1" s="24" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="21" t="s">
+      <c r="H1" s="24" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="21" t="s">
+      <c r="I1" s="24" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="21" t="s">
+      <c r="J1" s="24" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="2" s="20" customFormat="1" ht="20.4" spans="1:10">
-      <c r="A2" s="22" t="s">
+    <row r="2" s="23" customFormat="1" ht="20.4" spans="1:10">
+      <c r="A2" s="25" t="s">
         <v>10</v>
       </c>
-      <c r="B2" s="23" t="s">
+      <c r="B2" s="26" t="s">
         <v>11</v>
       </c>
-      <c r="C2" s="23" t="s">
+      <c r="C2" s="26" t="s">
         <v>12</v>
       </c>
-      <c r="D2" s="22" t="s">
+      <c r="D2" s="25" t="s">
         <v>13</v>
       </c>
-      <c r="E2" s="22">
+      <c r="E2" s="25">
         <v>1</v>
       </c>
-      <c r="F2" s="22" t="s">
+      <c r="F2" s="25" t="s">
         <v>14</v>
       </c>
-      <c r="G2" s="22">
+      <c r="G2" s="25">
         <v>1010301033</v>
       </c>
-      <c r="H2" s="22" t="s">
+      <c r="H2" s="25" t="s">
         <v>15</v>
       </c>
-      <c r="I2" s="22" t="s">
+      <c r="I2" s="25" t="s">
         <v>16</v>
       </c>
-      <c r="J2" s="22" t="s">
+      <c r="J2" s="25" t="s">
         <v>17</v>
       </c>
     </row>
     <row r="3" ht="15" customHeight="1" spans="1:10">
-      <c r="A3" s="22" t="s">
+      <c r="A3" s="25" t="s">
         <v>18</v>
       </c>
-      <c r="B3" s="23" t="s">
+      <c r="B3" s="26" t="s">
         <v>11</v>
       </c>
-      <c r="C3" s="23" t="s">
+      <c r="C3" s="26" t="s">
         <v>12</v>
       </c>
-      <c r="D3" s="22" t="s">
+      <c r="D3" s="25" t="s">
         <v>19</v>
       </c>
-      <c r="E3" s="22">
+      <c r="E3" s="25">
         <v>6</v>
       </c>
-      <c r="F3" s="23" t="s">
+      <c r="F3" s="26" t="s">
         <v>20</v>
       </c>
-      <c r="G3" s="22">
+      <c r="G3" s="25">
         <v>1010301033</v>
       </c>
-      <c r="H3" s="22" t="s">
+      <c r="H3" s="25" t="s">
         <v>15</v>
       </c>
-      <c r="I3" s="22" t="s">
+      <c r="I3" s="25" t="s">
         <v>16</v>
       </c>
-      <c r="J3" s="22" t="s">
+      <c r="J3" s="25" t="s">
         <v>17</v>
       </c>
     </row>
     <row r="4" spans="1:10">
-      <c r="A4" s="22" t="s">
+      <c r="A4" s="25" t="s">
         <v>21</v>
       </c>
-      <c r="B4" s="23" t="s">
+      <c r="B4" s="26" t="s">
         <v>22</v>
       </c>
-      <c r="C4" s="23" t="s">
+      <c r="C4" s="26" t="s">
         <v>22</v>
       </c>
-      <c r="D4" s="22" t="s">
+      <c r="D4" s="25" t="s">
         <v>23</v>
       </c>
-      <c r="E4" s="22">
+      <c r="E4" s="25">
         <v>1</v>
       </c>
-      <c r="F4" s="23" t="s">
+      <c r="F4" s="26" t="s">
         <v>14</v>
       </c>
-      <c r="G4" s="22">
+      <c r="G4" s="25">
         <v>5010101060</v>
       </c>
-      <c r="H4" s="22" t="s">
+      <c r="H4" s="25" t="s">
         <v>24</v>
       </c>
-      <c r="I4" s="22" t="s">
+      <c r="I4" s="25" t="s">
         <v>16</v>
       </c>
-      <c r="J4" s="22" t="s">
+      <c r="J4" s="25" t="s">
         <v>17</v>
       </c>
     </row>
     <row r="5" spans="1:10">
-      <c r="A5" s="24"/>
-      <c r="B5" s="24"/>
-      <c r="C5" s="24"/>
-      <c r="D5" s="24"/>
-      <c r="E5" s="24"/>
-      <c r="F5" s="24"/>
-      <c r="G5" s="24"/>
-      <c r="H5" s="24"/>
-      <c r="I5" s="24"/>
-      <c r="J5" s="24"/>
+      <c r="A5" s="27"/>
+      <c r="B5" s="27"/>
+      <c r="C5" s="27"/>
+      <c r="D5" s="27"/>
+      <c r="E5" s="27"/>
+      <c r="F5" s="27"/>
+      <c r="G5" s="27"/>
+      <c r="H5" s="27"/>
+      <c r="I5" s="27"/>
+      <c r="J5" s="27"/>
     </row>
     <row r="6" spans="1:10">
-      <c r="A6" s="24"/>
-      <c r="B6" s="24"/>
-      <c r="C6" s="24"/>
-      <c r="D6" s="24"/>
-      <c r="E6" s="24"/>
-      <c r="F6" s="24"/>
-      <c r="G6" s="24"/>
-      <c r="H6" s="24"/>
-      <c r="I6" s="24"/>
-      <c r="J6" s="24"/>
+      <c r="A6" s="27"/>
+      <c r="B6" s="27"/>
+      <c r="C6" s="27"/>
+      <c r="D6" s="27"/>
+      <c r="E6" s="27"/>
+      <c r="F6" s="27"/>
+      <c r="G6" s="27"/>
+      <c r="H6" s="27"/>
+      <c r="I6" s="27"/>
+      <c r="J6" s="27"/>
     </row>
     <row r="7" spans="1:10">
-      <c r="A7" s="24"/>
-      <c r="B7" s="24"/>
-      <c r="C7" s="24"/>
-      <c r="D7" s="24"/>
-      <c r="E7" s="24"/>
-      <c r="F7" s="24"/>
-      <c r="G7" s="24"/>
-      <c r="H7" s="24"/>
-      <c r="I7" s="24"/>
-      <c r="J7" s="24"/>
+      <c r="A7" s="27"/>
+      <c r="B7" s="27"/>
+      <c r="C7" s="27"/>
+      <c r="D7" s="27"/>
+      <c r="E7" s="27"/>
+      <c r="F7" s="27"/>
+      <c r="G7" s="27"/>
+      <c r="H7" s="27"/>
+      <c r="I7" s="27"/>
+      <c r="J7" s="27"/>
     </row>
     <row r="8" spans="1:10">
-      <c r="A8" s="24"/>
-      <c r="B8" s="24"/>
-      <c r="C8" s="24"/>
-      <c r="D8" s="24"/>
-      <c r="E8" s="24"/>
-      <c r="F8" s="24"/>
-      <c r="G8" s="24"/>
-      <c r="H8" s="24"/>
-      <c r="I8" s="24"/>
-      <c r="J8" s="24"/>
+      <c r="A8" s="27"/>
+      <c r="B8" s="27"/>
+      <c r="C8" s="27"/>
+      <c r="D8" s="27"/>
+      <c r="E8" s="27"/>
+      <c r="F8" s="27"/>
+      <c r="G8" s="27"/>
+      <c r="H8" s="27"/>
+      <c r="I8" s="27"/>
+      <c r="J8" s="27"/>
     </row>
     <row r="9" spans="1:10">
-      <c r="A9" s="24"/>
-      <c r="B9" s="24"/>
-      <c r="C9" s="24"/>
-      <c r="D9" s="24"/>
-      <c r="E9" s="24"/>
-      <c r="F9" s="24"/>
-      <c r="G9" s="24"/>
-      <c r="H9" s="24"/>
-      <c r="I9" s="24"/>
-      <c r="J9" s="24"/>
+      <c r="A9" s="27"/>
+      <c r="B9" s="27"/>
+      <c r="C9" s="27"/>
+      <c r="D9" s="27"/>
+      <c r="E9" s="27"/>
+      <c r="F9" s="27"/>
+      <c r="G9" s="27"/>
+      <c r="H9" s="27"/>
+      <c r="I9" s="27"/>
+      <c r="J9" s="27"/>
     </row>
     <row r="10" spans="1:10">
-      <c r="A10" s="24"/>
-      <c r="B10" s="24"/>
-      <c r="C10" s="24"/>
-      <c r="D10" s="24"/>
-      <c r="E10" s="24"/>
-      <c r="F10" s="24"/>
-      <c r="G10" s="24"/>
-      <c r="H10" s="24"/>
-      <c r="I10" s="24"/>
-      <c r="J10" s="24"/>
+      <c r="A10" s="27"/>
+      <c r="B10" s="27"/>
+      <c r="C10" s="27"/>
+      <c r="D10" s="27"/>
+      <c r="E10" s="27"/>
+      <c r="F10" s="27"/>
+      <c r="G10" s="27"/>
+      <c r="H10" s="27"/>
+      <c r="I10" s="27"/>
+      <c r="J10" s="27"/>
     </row>
     <row r="11" spans="1:10">
-      <c r="A11" s="24"/>
-      <c r="B11" s="24"/>
-      <c r="C11" s="24"/>
-      <c r="D11" s="24"/>
-      <c r="E11" s="24"/>
-      <c r="F11" s="24"/>
-      <c r="G11" s="24"/>
-      <c r="H11" s="24"/>
-      <c r="I11" s="24"/>
-      <c r="J11" s="24"/>
+      <c r="A11" s="27"/>
+      <c r="B11" s="27"/>
+      <c r="C11" s="27"/>
+      <c r="D11" s="27"/>
+      <c r="E11" s="27"/>
+      <c r="F11" s="27"/>
+      <c r="G11" s="27"/>
+      <c r="H11" s="27"/>
+      <c r="I11" s="27"/>
+      <c r="J11" s="27"/>
     </row>
     <row r="12" spans="1:10">
-      <c r="A12" s="24"/>
-      <c r="B12" s="24"/>
-      <c r="C12" s="24"/>
-      <c r="D12" s="24"/>
-      <c r="E12" s="24"/>
-      <c r="F12" s="24"/>
-      <c r="G12" s="24"/>
-      <c r="H12" s="24"/>
-      <c r="I12" s="24"/>
-      <c r="J12" s="24"/>
+      <c r="A12" s="27"/>
+      <c r="B12" s="27"/>
+      <c r="C12" s="27"/>
+      <c r="D12" s="27"/>
+      <c r="E12" s="27"/>
+      <c r="F12" s="27"/>
+      <c r="G12" s="27"/>
+      <c r="H12" s="27"/>
+      <c r="I12" s="27"/>
+      <c r="J12" s="27"/>
     </row>
     <row r="13" spans="1:10">
-      <c r="A13" s="24"/>
-      <c r="B13" s="24"/>
-      <c r="C13" s="24"/>
-      <c r="D13" s="24"/>
-      <c r="E13" s="24"/>
-      <c r="F13" s="24"/>
-      <c r="G13" s="24"/>
-      <c r="H13" s="24"/>
-      <c r="I13" s="24"/>
-      <c r="J13" s="24"/>
+      <c r="A13" s="27"/>
+      <c r="B13" s="27"/>
+      <c r="C13" s="27"/>
+      <c r="D13" s="27"/>
+      <c r="E13" s="27"/>
+      <c r="F13" s="27"/>
+      <c r="G13" s="27"/>
+      <c r="H13" s="27"/>
+      <c r="I13" s="27"/>
+      <c r="J13" s="27"/>
     </row>
     <row r="14" spans="1:10">
-      <c r="A14" s="24"/>
-      <c r="B14" s="24"/>
-      <c r="C14" s="24"/>
-      <c r="D14" s="24"/>
-      <c r="E14" s="24"/>
-      <c r="F14" s="24"/>
-      <c r="G14" s="24"/>
-      <c r="H14" s="24"/>
-      <c r="I14" s="24"/>
-      <c r="J14" s="24"/>
+      <c r="A14" s="27"/>
+      <c r="B14" s="27"/>
+      <c r="C14" s="27"/>
+      <c r="D14" s="27"/>
+      <c r="E14" s="27"/>
+      <c r="F14" s="27"/>
+      <c r="G14" s="27"/>
+      <c r="H14" s="27"/>
+      <c r="I14" s="27"/>
+      <c r="J14" s="27"/>
     </row>
     <row r="15" spans="1:10">
-      <c r="A15" s="24"/>
-      <c r="B15" s="24"/>
-      <c r="C15" s="24"/>
-      <c r="D15" s="24"/>
-      <c r="E15" s="24"/>
-      <c r="F15" s="24"/>
-      <c r="G15" s="24"/>
-      <c r="H15" s="24"/>
-      <c r="I15" s="24"/>
-      <c r="J15" s="24"/>
+      <c r="A15" s="27"/>
+      <c r="B15" s="27"/>
+      <c r="C15" s="27"/>
+      <c r="D15" s="27"/>
+      <c r="E15" s="27"/>
+      <c r="F15" s="27"/>
+      <c r="G15" s="27"/>
+      <c r="H15" s="27"/>
+      <c r="I15" s="27"/>
+      <c r="J15" s="27"/>
     </row>
     <row r="16" spans="1:10">
-      <c r="A16" s="24"/>
-      <c r="B16" s="24"/>
-      <c r="C16" s="24"/>
-      <c r="D16" s="24"/>
-      <c r="E16" s="24"/>
-      <c r="F16" s="24"/>
-      <c r="G16" s="24"/>
-      <c r="H16" s="24"/>
-      <c r="I16" s="24"/>
-      <c r="J16" s="24"/>
+      <c r="A16" s="27"/>
+      <c r="B16" s="27"/>
+      <c r="C16" s="27"/>
+      <c r="D16" s="27"/>
+      <c r="E16" s="27"/>
+      <c r="F16" s="27"/>
+      <c r="G16" s="27"/>
+      <c r="H16" s="27"/>
+      <c r="I16" s="27"/>
+      <c r="J16" s="27"/>
     </row>
     <row r="17" spans="1:10">
-      <c r="A17" s="24"/>
-      <c r="B17" s="24"/>
-      <c r="C17" s="24"/>
-      <c r="D17" s="24"/>
-      <c r="E17" s="24"/>
-      <c r="F17" s="24"/>
-      <c r="G17" s="24"/>
-      <c r="H17" s="24"/>
-      <c r="I17" s="24"/>
-      <c r="J17" s="24"/>
+      <c r="A17" s="27"/>
+      <c r="B17" s="27"/>
+      <c r="C17" s="27"/>
+      <c r="D17" s="27"/>
+      <c r="E17" s="27"/>
+      <c r="F17" s="27"/>
+      <c r="G17" s="27"/>
+      <c r="H17" s="27"/>
+      <c r="I17" s="27"/>
+      <c r="J17" s="27"/>
     </row>
     <row r="18" spans="1:10">
-      <c r="A18" s="24"/>
-      <c r="B18" s="24"/>
-      <c r="C18" s="24"/>
-      <c r="D18" s="24"/>
-      <c r="E18" s="24"/>
-      <c r="F18" s="24"/>
-      <c r="G18" s="24"/>
-      <c r="H18" s="24"/>
-      <c r="I18" s="24"/>
-      <c r="J18" s="24"/>
+      <c r="A18" s="27"/>
+      <c r="B18" s="27"/>
+      <c r="C18" s="27"/>
+      <c r="D18" s="27"/>
+      <c r="E18" s="27"/>
+      <c r="F18" s="27"/>
+      <c r="G18" s="27"/>
+      <c r="H18" s="27"/>
+      <c r="I18" s="27"/>
+      <c r="J18" s="27"/>
     </row>
     <row r="19" spans="1:10">
-      <c r="A19" s="24"/>
-      <c r="B19" s="24"/>
-      <c r="C19" s="24"/>
-      <c r="D19" s="24"/>
-      <c r="E19" s="24"/>
-      <c r="F19" s="24"/>
-      <c r="G19" s="24"/>
-      <c r="H19" s="24"/>
-      <c r="I19" s="24"/>
-      <c r="J19" s="24"/>
+      <c r="A19" s="27"/>
+      <c r="B19" s="27"/>
+      <c r="C19" s="27"/>
+      <c r="D19" s="27"/>
+      <c r="E19" s="27"/>
+      <c r="F19" s="27"/>
+      <c r="G19" s="27"/>
+      <c r="H19" s="27"/>
+      <c r="I19" s="27"/>
+      <c r="J19" s="27"/>
     </row>
     <row r="20" spans="1:10">
-      <c r="A20" s="24"/>
-      <c r="B20" s="24"/>
-      <c r="C20" s="24"/>
-      <c r="D20" s="24"/>
-      <c r="E20" s="24"/>
-      <c r="F20" s="24"/>
-      <c r="G20" s="24"/>
-      <c r="H20" s="24"/>
-      <c r="I20" s="24"/>
-      <c r="J20" s="24"/>
+      <c r="A20" s="27"/>
+      <c r="B20" s="27"/>
+      <c r="C20" s="27"/>
+      <c r="D20" s="27"/>
+      <c r="E20" s="27"/>
+      <c r="F20" s="27"/>
+      <c r="G20" s="27"/>
+      <c r="H20" s="27"/>
+      <c r="I20" s="27"/>
+      <c r="J20" s="27"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2190,107 +2273,107 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11">
-      <c r="A1" s="4" t="s">
+      <c r="A1" s="9" t="s">
         <v>124</v>
       </c>
-      <c r="B1" s="4" t="s">
+      <c r="B1" s="9" t="s">
         <v>125</v>
       </c>
-      <c r="C1" s="4" t="s">
+      <c r="C1" s="9" t="s">
         <v>126</v>
       </c>
-      <c r="D1" s="4" t="s">
+      <c r="D1" s="9" t="s">
         <v>127</v>
       </c>
-      <c r="E1" s="4" t="s">
+      <c r="E1" s="9" t="s">
         <v>128</v>
       </c>
-      <c r="F1" s="5" t="s">
+      <c r="F1" s="10" t="s">
         <v>129</v>
       </c>
-      <c r="G1" s="5" t="s">
+      <c r="G1" s="10" t="s">
         <v>130</v>
       </c>
-      <c r="H1" s="5" t="s">
+      <c r="H1" s="10" t="s">
         <v>131</v>
       </c>
-      <c r="I1" s="5" t="s">
+      <c r="I1" s="10" t="s">
         <v>132</v>
       </c>
-      <c r="J1" s="5" t="s">
+      <c r="J1" s="10" t="s">
         <v>133</v>
       </c>
-      <c r="K1" s="5" t="s">
+      <c r="K1" s="10" t="s">
         <v>134</v>
       </c>
     </row>
     <row r="2" spans="1:11">
-      <c r="A2" s="4" t="s">
+      <c r="A2" s="9" t="s">
         <v>135</v>
       </c>
-      <c r="B2" s="4" t="s">
+      <c r="B2" s="9" t="s">
         <v>136</v>
       </c>
-      <c r="C2" s="4" t="s">
+      <c r="C2" s="9" t="s">
         <v>137</v>
       </c>
-      <c r="D2" s="4" t="s">
+      <c r="D2" s="9" t="s">
         <v>138</v>
       </c>
-      <c r="E2" s="4" t="s">
+      <c r="E2" s="9" t="s">
         <v>139</v>
       </c>
-      <c r="F2" s="6" t="s">
+      <c r="F2" s="3" t="s">
         <v>136</v>
       </c>
-      <c r="G2" s="6" t="s">
+      <c r="G2" s="3" t="s">
         <v>140</v>
       </c>
-      <c r="H2" s="6" t="s">
+      <c r="H2" s="3" t="s">
         <v>141</v>
       </c>
-      <c r="I2" s="6" t="s">
+      <c r="I2" s="3" t="s">
         <v>142</v>
       </c>
-      <c r="J2" s="6" t="s">
+      <c r="J2" s="3" t="s">
         <v>143</v>
       </c>
-      <c r="K2" s="6" t="s">
+      <c r="K2" s="3" t="s">
         <v>144</v>
       </c>
     </row>
     <row r="3" spans="1:11">
-      <c r="A3" s="7" t="s">
+      <c r="A3" s="11" t="s">
         <v>145</v>
       </c>
-      <c r="B3" s="6" t="s">
+      <c r="B3" s="3" t="s">
         <v>146</v>
       </c>
-      <c r="C3" s="4" t="s">
+      <c r="C3" s="9" t="s">
         <v>137</v>
       </c>
-      <c r="D3" s="6" t="s">
+      <c r="D3" s="3" t="s">
         <v>147</v>
       </c>
-      <c r="E3" s="6" t="s">
+      <c r="E3" s="3" t="s">
         <v>147</v>
       </c>
-      <c r="F3" s="6" t="s">
+      <c r="F3" s="3" t="s">
         <v>146</v>
       </c>
-      <c r="G3" s="6" t="s">
+      <c r="G3" s="3" t="s">
         <v>148</v>
       </c>
-      <c r="H3" s="6" t="s">
+      <c r="H3" s="3" t="s">
         <v>148</v>
       </c>
-      <c r="I3" s="6" t="s">
+      <c r="I3" s="3" t="s">
         <v>149</v>
       </c>
-      <c r="J3" s="6" t="s">
+      <c r="J3" s="3" t="s">
         <v>143</v>
       </c>
-      <c r="K3" s="6" t="s">
+      <c r="K3" s="3" t="s">
         <v>144</v>
       </c>
     </row>
@@ -2314,7 +2397,7 @@
   </cols>
   <sheetData>
     <row r="1" ht="15.15" spans="1:5">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="6" t="s">
         <v>150</v>
       </c>
       <c r="B1" t="s">
@@ -2331,20 +2414,225 @@
       </c>
     </row>
     <row r="2" ht="15.15" spans="1:5">
-      <c r="A2" s="1" t="s">
+      <c r="A2" s="6" t="s">
         <v>155</v>
       </c>
-      <c r="B2" s="1" t="s">
+      <c r="B2" s="6" t="s">
         <v>156</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="C2" s="7" t="s">
         <v>135</v>
       </c>
-      <c r="D2" s="3" t="s">
+      <c r="D2" s="8" t="s">
         <v>136</v>
       </c>
-      <c r="E2" s="1" t="s">
+      <c r="E2" s="6" t="s">
         <v>157</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <headerFooter/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
+  <dimension ref="A1:G8"/>
+  <sheetFormatPr defaultColWidth="8.88888888888889" defaultRowHeight="14.4" outlineLevelRow="7" outlineLevelCol="6"/>
+  <cols>
+    <col min="1" max="1" width="25.7777777777778" customWidth="1"/>
+    <col min="2" max="2" width="8.88888888888889" customWidth="1"/>
+    <col min="3" max="3" width="12.2222222222222" customWidth="1"/>
+    <col min="4" max="4" width="7.11111111111111" customWidth="1"/>
+    <col min="5" max="5" width="5.22222222222222" customWidth="1"/>
+    <col min="6" max="6" width="17.4444444444444" customWidth="1"/>
+    <col min="7" max="7" width="12.4444444444444" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7">
+      <c r="A1" s="1" t="s">
+        <v>158</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>159</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>160</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>161</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>162</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>163</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7">
+      <c r="A2" s="3" t="s">
+        <v>165</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>166</v>
+      </c>
+      <c r="C2" s="4" t="s">
+        <v>167</v>
+      </c>
+      <c r="D2" s="4" t="s">
+        <v>155</v>
+      </c>
+      <c r="E2" s="4" t="s">
+        <v>156</v>
+      </c>
+      <c r="F2" s="3" t="s">
+        <v>168</v>
+      </c>
+      <c r="G2" s="3" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7">
+      <c r="A3" s="3" t="s">
+        <v>146</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>170</v>
+      </c>
+      <c r="C3" s="4" t="s">
+        <v>167</v>
+      </c>
+      <c r="D3" s="4" t="s">
+        <v>155</v>
+      </c>
+      <c r="E3" s="4" t="s">
+        <v>156</v>
+      </c>
+      <c r="F3" s="3" t="s">
+        <v>147</v>
+      </c>
+      <c r="G3" s="3" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7">
+      <c r="A4" s="3" t="s">
+        <v>171</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>166</v>
+      </c>
+      <c r="C4" s="4" t="s">
+        <v>167</v>
+      </c>
+      <c r="D4" s="4" t="s">
+        <v>155</v>
+      </c>
+      <c r="E4" s="4" t="s">
+        <v>156</v>
+      </c>
+      <c r="F4" s="3" t="s">
+        <v>168</v>
+      </c>
+      <c r="G4" s="3" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7">
+      <c r="A5" s="3" t="s">
+        <v>136</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>166</v>
+      </c>
+      <c r="C5" s="4" t="s">
+        <v>167</v>
+      </c>
+      <c r="D5" s="4" t="s">
+        <v>155</v>
+      </c>
+      <c r="E5" s="4" t="s">
+        <v>156</v>
+      </c>
+      <c r="F5" s="5" t="s">
+        <v>138</v>
+      </c>
+      <c r="G5" s="3" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7">
+      <c r="A6" s="3" t="s">
+        <v>172</v>
+      </c>
+      <c r="B6" s="3" t="s">
+        <v>166</v>
+      </c>
+      <c r="C6" s="4" t="s">
+        <v>167</v>
+      </c>
+      <c r="D6" s="4" t="s">
+        <v>155</v>
+      </c>
+      <c r="E6" s="4" t="s">
+        <v>156</v>
+      </c>
+      <c r="F6" s="3" t="s">
+        <v>138</v>
+      </c>
+      <c r="G6" s="3" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7">
+      <c r="A7" s="3" t="s">
+        <v>173</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>166</v>
+      </c>
+      <c r="C7" s="4" t="s">
+        <v>167</v>
+      </c>
+      <c r="D7" s="4" t="s">
+        <v>155</v>
+      </c>
+      <c r="E7" s="4" t="s">
+        <v>156</v>
+      </c>
+      <c r="F7" s="3" t="s">
+        <v>138</v>
+      </c>
+      <c r="G7" s="3" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7">
+      <c r="A8" s="3" t="s">
+        <v>174</v>
+      </c>
+      <c r="B8" s="3" t="s">
+        <v>166</v>
+      </c>
+      <c r="C8" s="4" t="s">
+        <v>167</v>
+      </c>
+      <c r="D8" s="4" t="s">
+        <v>155</v>
+      </c>
+      <c r="E8" s="4" t="s">
+        <v>156</v>
+      </c>
+      <c r="F8" s="3" t="s">
+        <v>175</v>
+      </c>
+      <c r="G8" s="3" t="s">
+        <v>169</v>
       </c>
     </row>
   </sheetData>
@@ -2382,552 +2670,552 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:20">
-      <c r="A1" s="9" t="s">
+      <c r="A1" s="12" t="s">
         <v>25</v>
       </c>
-      <c r="B1" s="9" t="s">
+      <c r="B1" s="12" t="s">
         <v>26</v>
       </c>
-      <c r="C1" s="9" t="s">
+      <c r="C1" s="12" t="s">
         <v>27</v>
       </c>
-      <c r="D1" s="9" t="s">
+      <c r="D1" s="12" t="s">
         <v>28</v>
       </c>
-      <c r="E1" s="9" t="s">
+      <c r="E1" s="12" t="s">
         <v>29</v>
       </c>
-      <c r="F1" s="9" t="s">
+      <c r="F1" s="12" t="s">
         <v>2</v>
       </c>
-      <c r="G1" s="9" t="s">
+      <c r="G1" s="12" t="s">
         <v>1</v>
       </c>
-      <c r="H1" s="9" t="s">
+      <c r="H1" s="12" t="s">
         <v>30</v>
       </c>
-      <c r="I1" s="9" t="s">
+      <c r="I1" s="12" t="s">
         <v>31</v>
       </c>
-      <c r="J1" s="9" t="s">
+      <c r="J1" s="12" t="s">
         <v>32</v>
       </c>
-      <c r="K1" s="9" t="s">
+      <c r="K1" s="12" t="s">
         <v>33</v>
       </c>
-      <c r="L1" s="9" t="s">
+      <c r="L1" s="12" t="s">
         <v>6</v>
       </c>
-      <c r="M1" s="9" t="s">
+      <c r="M1" s="12" t="s">
         <v>7</v>
       </c>
-      <c r="N1" s="9" t="s">
+      <c r="N1" s="12" t="s">
         <v>8</v>
       </c>
-      <c r="O1" s="9" t="s">
+      <c r="O1" s="12" t="s">
         <v>9</v>
       </c>
-      <c r="P1" s="9" t="s">
+      <c r="P1" s="12" t="s">
         <v>34</v>
       </c>
-      <c r="Q1" s="9" t="s">
+      <c r="Q1" s="12" t="s">
         <v>35</v>
       </c>
-      <c r="R1" s="9" t="s">
+      <c r="R1" s="12" t="s">
         <v>36</v>
       </c>
-      <c r="S1" s="9" t="s">
+      <c r="S1" s="12" t="s">
         <v>37</v>
       </c>
-      <c r="T1" s="9" t="s">
+      <c r="T1" s="12" t="s">
         <v>38</v>
       </c>
     </row>
     <row r="2" spans="1:20">
-      <c r="A2" s="9" t="s">
+      <c r="A2" s="12" t="s">
         <v>18</v>
       </c>
-      <c r="B2" s="9" t="s">
+      <c r="B2" s="12" t="s">
         <v>39</v>
       </c>
-      <c r="C2" s="9" t="s">
+      <c r="C2" s="12" t="s">
         <v>20</v>
       </c>
-      <c r="D2" s="9" t="s">
+      <c r="D2" s="12" t="s">
         <v>40</v>
       </c>
-      <c r="E2" s="9">
+      <c r="E2" s="12">
         <v>12</v>
       </c>
-      <c r="F2" s="15" t="s">
+      <c r="F2" s="18" t="s">
         <v>12</v>
       </c>
-      <c r="G2" s="9" t="s">
+      <c r="G2" s="12" t="s">
         <v>11</v>
       </c>
-      <c r="H2" s="9" t="s">
+      <c r="H2" s="12" t="s">
         <v>19</v>
       </c>
-      <c r="I2" s="9" t="s">
+      <c r="I2" s="12" t="s">
         <v>41</v>
       </c>
-      <c r="J2" s="9" t="s">
+      <c r="J2" s="12" t="s">
         <v>14</v>
       </c>
-      <c r="K2" s="9">
+      <c r="K2" s="12">
         <v>6</v>
       </c>
-      <c r="L2" s="9">
+      <c r="L2" s="12">
         <v>1010301033</v>
       </c>
-      <c r="M2" s="9" t="s">
+      <c r="M2" s="12" t="s">
         <v>15</v>
       </c>
-      <c r="N2" s="9" t="s">
+      <c r="N2" s="12" t="s">
         <v>16</v>
       </c>
-      <c r="O2" s="9" t="s">
+      <c r="O2" s="12" t="s">
         <v>17</v>
       </c>
-      <c r="P2" s="9"/>
-      <c r="Q2" s="9"/>
-      <c r="R2" s="9"/>
-      <c r="S2" s="9">
+      <c r="P2" s="12"/>
+      <c r="Q2" s="12"/>
+      <c r="R2" s="12"/>
+      <c r="S2" s="12">
         <v>0</v>
       </c>
-      <c r="T2" s="9"/>
+      <c r="T2" s="12"/>
     </row>
     <row r="3" spans="1:20">
-      <c r="A3" s="9" t="s">
+      <c r="A3" s="12" t="s">
         <v>10</v>
       </c>
-      <c r="B3" s="9" t="s">
+      <c r="B3" s="12" t="s">
         <v>42</v>
       </c>
-      <c r="C3" s="9" t="s">
+      <c r="C3" s="12" t="s">
         <v>14</v>
       </c>
-      <c r="D3" s="16" t="s">
+      <c r="D3" s="19" t="s">
         <v>43</v>
       </c>
-      <c r="E3" s="9">
+      <c r="E3" s="12">
         <v>5</v>
       </c>
-      <c r="F3" s="9" t="s">
+      <c r="F3" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="G3" s="9" t="s">
+      <c r="G3" s="12" t="s">
         <v>11</v>
       </c>
-      <c r="H3" s="9" t="s">
+      <c r="H3" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="I3" s="9" t="s">
+      <c r="I3" s="12" t="s">
         <v>44</v>
       </c>
-      <c r="J3" s="9" t="s">
+      <c r="J3" s="12" t="s">
         <v>14</v>
       </c>
-      <c r="K3" s="9">
+      <c r="K3" s="12">
         <v>1</v>
       </c>
-      <c r="L3" s="9">
+      <c r="L3" s="12">
         <v>1010301033</v>
       </c>
-      <c r="M3" s="9" t="s">
+      <c r="M3" s="12" t="s">
         <v>15</v>
       </c>
-      <c r="N3" s="9" t="s">
+      <c r="N3" s="12" t="s">
         <v>16</v>
       </c>
-      <c r="O3" s="9" t="s">
+      <c r="O3" s="12" t="s">
         <v>17</v>
       </c>
-      <c r="P3" s="9"/>
-      <c r="Q3" s="9"/>
-      <c r="R3" s="9"/>
-      <c r="S3" s="9">
+      <c r="P3" s="12"/>
+      <c r="Q3" s="12"/>
+      <c r="R3" s="12"/>
+      <c r="S3" s="12">
         <v>0</v>
       </c>
-      <c r="T3" s="9"/>
+      <c r="T3" s="12"/>
     </row>
     <row r="4" spans="1:20">
-      <c r="A4" s="9" t="s">
+      <c r="A4" s="12" t="s">
         <v>21</v>
       </c>
-      <c r="B4" s="9" t="s">
+      <c r="B4" s="12" t="s">
         <v>45</v>
       </c>
-      <c r="C4" s="9" t="s">
+      <c r="C4" s="12" t="s">
         <v>14</v>
       </c>
-      <c r="D4" s="9">
+      <c r="D4" s="12">
         <v>123562</v>
       </c>
-      <c r="E4" s="9">
+      <c r="E4" s="12">
         <v>18</v>
       </c>
-      <c r="F4" s="9" t="s">
+      <c r="F4" s="12" t="s">
         <v>22</v>
       </c>
-      <c r="G4" s="9" t="s">
+      <c r="G4" s="12" t="s">
         <v>22</v>
       </c>
-      <c r="H4" s="9" t="s">
+      <c r="H4" s="12" t="s">
         <v>23</v>
       </c>
-      <c r="I4" s="9" t="s">
+      <c r="I4" s="12" t="s">
         <v>44</v>
       </c>
-      <c r="J4" s="9" t="s">
+      <c r="J4" s="12" t="s">
         <v>14</v>
       </c>
-      <c r="K4" s="9">
+      <c r="K4" s="12">
         <v>1</v>
       </c>
-      <c r="L4" s="9">
+      <c r="L4" s="12">
         <v>1011134888</v>
       </c>
-      <c r="M4" s="9" t="s">
+      <c r="M4" s="12" t="s">
         <v>46</v>
       </c>
-      <c r="N4" s="9" t="s">
+      <c r="N4" s="12" t="s">
         <v>16</v>
       </c>
-      <c r="O4" s="9" t="s">
+      <c r="O4" s="12" t="s">
         <v>17</v>
       </c>
-      <c r="P4" s="9"/>
-      <c r="Q4" s="9"/>
-      <c r="R4" s="9"/>
-      <c r="S4" s="9">
+      <c r="P4" s="12"/>
+      <c r="Q4" s="12"/>
+      <c r="R4" s="12"/>
+      <c r="S4" s="12">
         <v>0</v>
       </c>
-      <c r="T4" s="9"/>
+      <c r="T4" s="12"/>
     </row>
     <row r="5" spans="1:20">
-      <c r="A5" s="6" t="s">
+      <c r="A5" s="3" t="s">
         <v>47</v>
       </c>
-      <c r="B5" s="6" t="s">
+      <c r="B5" s="3" t="s">
         <v>47</v>
       </c>
-      <c r="C5" s="9" t="s">
+      <c r="C5" s="12" t="s">
         <v>14</v>
       </c>
-      <c r="D5" s="6" t="s">
+      <c r="D5" s="3" t="s">
         <v>40</v>
       </c>
-      <c r="E5" s="6">
+      <c r="E5" s="3">
         <v>12</v>
       </c>
-      <c r="F5" s="6" t="s">
+      <c r="F5" s="3" t="s">
         <v>48</v>
       </c>
-      <c r="G5" s="6" t="s">
+      <c r="G5" s="3" t="s">
         <v>49</v>
       </c>
-      <c r="H5" s="6" t="s">
+      <c r="H5" s="3" t="s">
         <v>50</v>
       </c>
-      <c r="I5" s="6" t="s">
+      <c r="I5" s="3" t="s">
         <v>44</v>
       </c>
-      <c r="J5" s="6" t="s">
+      <c r="J5" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="K5" s="6">
+      <c r="K5" s="3">
         <v>1</v>
       </c>
-      <c r="L5" s="6">
+      <c r="L5" s="3">
         <v>1010301001</v>
       </c>
-      <c r="M5" s="6" t="s">
+      <c r="M5" s="3" t="s">
         <v>51</v>
       </c>
-      <c r="N5" s="6" t="s">
+      <c r="N5" s="3" t="s">
         <v>52</v>
       </c>
-      <c r="O5" s="6" t="s">
+      <c r="O5" s="3" t="s">
         <v>53</v>
       </c>
-      <c r="P5" s="6"/>
-      <c r="Q5" s="6"/>
-      <c r="R5" s="6"/>
-      <c r="S5" s="9">
+      <c r="P5" s="3"/>
+      <c r="Q5" s="3"/>
+      <c r="R5" s="3"/>
+      <c r="S5" s="12">
         <v>0</v>
       </c>
-      <c r="T5" s="6"/>
+      <c r="T5" s="3"/>
     </row>
     <row r="6" spans="1:20">
-      <c r="A6" s="6" t="s">
+      <c r="A6" s="3" t="s">
         <v>54</v>
       </c>
-      <c r="B6" s="6" t="s">
+      <c r="B6" s="3" t="s">
         <v>54</v>
       </c>
-      <c r="C6" s="6" t="s">
+      <c r="C6" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="D6" s="14" t="s">
+      <c r="D6" s="17" t="s">
         <v>43</v>
       </c>
       <c r="E6">
         <v>5</v>
       </c>
-      <c r="F6" s="17" t="s">
+      <c r="F6" s="20" t="s">
         <v>12</v>
       </c>
-      <c r="G6" s="17" t="s">
+      <c r="G6" s="20" t="s">
         <v>11</v>
       </c>
-      <c r="H6" s="6" t="s">
+      <c r="H6" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="I6" s="6" t="s">
+      <c r="I6" s="3" t="s">
         <v>44</v>
       </c>
-      <c r="J6" s="6" t="s">
+      <c r="J6" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="K6" s="6">
+      <c r="K6" s="3">
         <v>1</v>
       </c>
-      <c r="L6" s="6">
+      <c r="L6" s="3">
         <v>1010301033</v>
       </c>
-      <c r="M6" s="6" t="s">
+      <c r="M6" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="N6" s="6" t="s">
+      <c r="N6" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="O6" s="6" t="s">
+      <c r="O6" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="P6" s="6"/>
-      <c r="Q6" s="6"/>
-      <c r="R6" s="6"/>
-      <c r="S6" s="9">
+      <c r="P6" s="3"/>
+      <c r="Q6" s="3"/>
+      <c r="R6" s="3"/>
+      <c r="S6" s="12">
         <v>0</v>
       </c>
-      <c r="T6" s="6"/>
+      <c r="T6" s="3"/>
     </row>
     <row r="7" spans="1:20">
-      <c r="A7" s="18" t="s">
+      <c r="A7" s="21" t="s">
         <v>55</v>
       </c>
-      <c r="B7" s="18" t="s">
+      <c r="B7" s="21" t="s">
         <v>56</v>
       </c>
-      <c r="C7" s="18" t="s">
+      <c r="C7" s="21" t="s">
         <v>20</v>
       </c>
-      <c r="D7" s="18" t="s">
+      <c r="D7" s="21" t="s">
         <v>40</v>
       </c>
-      <c r="E7" s="18">
+      <c r="E7" s="21">
         <v>12</v>
       </c>
-      <c r="F7" s="19" t="s">
+      <c r="F7" s="22" t="s">
         <v>12</v>
       </c>
-      <c r="G7" s="18" t="s">
+      <c r="G7" s="21" t="s">
         <v>11</v>
       </c>
-      <c r="H7" s="18" t="s">
+      <c r="H7" s="21" t="s">
         <v>57</v>
       </c>
-      <c r="I7" s="18" t="s">
+      <c r="I7" s="21" t="s">
         <v>41</v>
       </c>
-      <c r="J7" s="18" t="s">
+      <c r="J7" s="21" t="s">
         <v>14</v>
       </c>
-      <c r="K7" s="18">
+      <c r="K7" s="21">
         <v>3</v>
       </c>
-      <c r="L7" s="18">
+      <c r="L7" s="21">
         <v>1010301003</v>
       </c>
-      <c r="M7" s="18" t="s">
+      <c r="M7" s="21" t="s">
         <v>58</v>
       </c>
-      <c r="N7" s="18" t="s">
+      <c r="N7" s="21" t="s">
         <v>16</v>
       </c>
-      <c r="O7" s="18" t="s">
+      <c r="O7" s="21" t="s">
         <v>17</v>
       </c>
-      <c r="P7" s="18"/>
-      <c r="Q7" s="18"/>
-      <c r="R7" s="18"/>
-      <c r="S7" s="18">
+      <c r="P7" s="21"/>
+      <c r="Q7" s="21"/>
+      <c r="R7" s="21"/>
+      <c r="S7" s="21">
         <v>0</v>
       </c>
-      <c r="T7" s="18"/>
+      <c r="T7" s="21"/>
     </row>
     <row r="8" spans="1:20">
-      <c r="A8" s="18" t="s">
+      <c r="A8" s="21" t="s">
         <v>59</v>
       </c>
-      <c r="B8" s="18" t="s">
+      <c r="B8" s="21" t="s">
         <v>60</v>
       </c>
-      <c r="C8" s="18" t="s">
+      <c r="C8" s="21" t="s">
         <v>14</v>
       </c>
-      <c r="D8" s="18" t="s">
+      <c r="D8" s="21" t="s">
         <v>43</v>
       </c>
-      <c r="E8" s="18">
+      <c r="E8" s="21">
         <v>5</v>
       </c>
-      <c r="F8" s="19" t="s">
+      <c r="F8" s="22" t="s">
         <v>12</v>
       </c>
-      <c r="G8" s="18" t="s">
+      <c r="G8" s="21" t="s">
         <v>11</v>
       </c>
-      <c r="H8" s="18" t="s">
+      <c r="H8" s="21" t="s">
         <v>57</v>
       </c>
-      <c r="I8" s="18" t="s">
+      <c r="I8" s="21" t="s">
         <v>41</v>
       </c>
-      <c r="J8" s="18" t="s">
+      <c r="J8" s="21" t="s">
         <v>14</v>
       </c>
-      <c r="K8" s="18">
+      <c r="K8" s="21">
         <v>0</v>
       </c>
-      <c r="L8" s="18">
+      <c r="L8" s="21">
         <v>1010301003</v>
       </c>
-      <c r="M8" s="18" t="s">
+      <c r="M8" s="21" t="s">
         <v>58</v>
       </c>
-      <c r="N8" s="18" t="s">
+      <c r="N8" s="21" t="s">
         <v>16</v>
       </c>
-      <c r="O8" s="18" t="s">
+      <c r="O8" s="21" t="s">
         <v>17</v>
       </c>
-      <c r="P8" s="18"/>
-      <c r="Q8" s="18"/>
-      <c r="R8" s="18"/>
-      <c r="S8" s="18">
+      <c r="P8" s="21"/>
+      <c r="Q8" s="21"/>
+      <c r="R8" s="21"/>
+      <c r="S8" s="21">
         <v>0</v>
       </c>
-      <c r="T8" s="18"/>
+      <c r="T8" s="21"/>
     </row>
     <row r="9" spans="1:20">
-      <c r="A9" s="18" t="s">
+      <c r="A9" s="21" t="s">
         <v>61</v>
       </c>
-      <c r="B9" s="18" t="s">
+      <c r="B9" s="21" t="s">
         <v>61</v>
       </c>
-      <c r="C9" s="18" t="s">
+      <c r="C9" s="21" t="s">
         <v>14</v>
       </c>
-      <c r="D9" s="18" t="s">
+      <c r="D9" s="21" t="s">
         <v>43</v>
       </c>
-      <c r="E9" s="18">
+      <c r="E9" s="21">
         <v>5</v>
       </c>
-      <c r="F9" s="19" t="s">
+      <c r="F9" s="22" t="s">
         <v>12</v>
       </c>
-      <c r="G9" s="18" t="s">
+      <c r="G9" s="21" t="s">
         <v>11</v>
       </c>
-      <c r="H9" s="18" t="s">
+      <c r="H9" s="21" t="s">
         <v>57</v>
       </c>
-      <c r="I9" s="18" t="s">
+      <c r="I9" s="21" t="s">
         <v>41</v>
       </c>
-      <c r="J9" s="18" t="s">
+      <c r="J9" s="21" t="s">
         <v>14</v>
       </c>
-      <c r="K9" s="18">
+      <c r="K9" s="21">
         <v>0</v>
       </c>
-      <c r="L9" s="18">
+      <c r="L9" s="21">
         <v>1010301003</v>
       </c>
-      <c r="M9" s="18" t="s">
+      <c r="M9" s="21" t="s">
         <v>58</v>
       </c>
-      <c r="N9" s="18" t="s">
+      <c r="N9" s="21" t="s">
         <v>16</v>
       </c>
-      <c r="O9" s="18" t="s">
+      <c r="O9" s="21" t="s">
         <v>17</v>
       </c>
-      <c r="P9" s="18"/>
-      <c r="Q9" s="18"/>
-      <c r="R9" s="18"/>
-      <c r="S9" s="18">
+      <c r="P9" s="21"/>
+      <c r="Q9" s="21"/>
+      <c r="R9" s="21"/>
+      <c r="S9" s="21">
         <v>0</v>
       </c>
-      <c r="T9" s="18"/>
+      <c r="T9" s="21"/>
     </row>
     <row r="10" spans="1:20">
-      <c r="A10" s="6" t="s">
+      <c r="A10" s="3" t="s">
         <v>62</v>
       </c>
-      <c r="B10" s="6" t="s">
+      <c r="B10" s="3" t="s">
         <v>62</v>
       </c>
-      <c r="C10" s="6" t="s">
+      <c r="C10" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="D10" s="18" t="s">
+      <c r="D10" s="21" t="s">
         <v>43</v>
       </c>
-      <c r="E10" s="18">
+      <c r="E10" s="21">
         <v>5</v>
       </c>
-      <c r="F10" s="9" t="s">
+      <c r="F10" s="12" t="s">
         <v>22</v>
       </c>
-      <c r="G10" s="9" t="s">
+      <c r="G10" s="12" t="s">
         <v>22</v>
       </c>
-      <c r="H10" s="9" t="s">
+      <c r="H10" s="12" t="s">
         <v>63</v>
       </c>
-      <c r="I10" s="9" t="s">
+      <c r="I10" s="12" t="s">
         <v>44</v>
       </c>
-      <c r="J10" s="9" t="s">
+      <c r="J10" s="12" t="s">
         <v>14</v>
       </c>
-      <c r="K10" s="9">
+      <c r="K10" s="12">
         <v>1</v>
       </c>
-      <c r="L10" s="12">
+      <c r="L10" s="15">
         <v>1000000001</v>
       </c>
-      <c r="M10" s="6" t="s">
+      <c r="M10" s="3" t="s">
         <v>64</v>
       </c>
-      <c r="N10" s="6" t="s">
+      <c r="N10" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="O10" s="6" t="s">
+      <c r="O10" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="P10" s="18"/>
-      <c r="Q10" s="18"/>
-      <c r="R10" s="18"/>
-      <c r="S10" s="18">
+      <c r="P10" s="21"/>
+      <c r="Q10" s="21"/>
+      <c r="R10" s="21"/>
+      <c r="S10" s="21">
         <v>0</v>
       </c>
-      <c r="T10" s="18"/>
+      <c r="T10" s="21"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2955,128 +3243,128 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:18">
-      <c r="A1" s="6" t="s">
+      <c r="A1" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="B1" s="6" t="s">
+      <c r="B1" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="C1" s="6" t="s">
+      <c r="C1" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="D1" s="9" t="s">
+      <c r="D1" s="12" t="s">
         <v>6</v>
       </c>
-      <c r="E1" s="9" t="s">
+      <c r="E1" s="12" t="s">
         <v>7</v>
       </c>
-      <c r="F1" s="9" t="s">
+      <c r="F1" s="12" t="s">
         <v>8</v>
       </c>
-      <c r="G1" s="9" t="s">
+      <c r="G1" s="12" t="s">
         <v>9</v>
       </c>
-      <c r="H1" s="6" t="s">
+      <c r="H1" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="I1" s="6" t="s">
+      <c r="I1" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="J1" s="6" t="s">
+      <c r="J1" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="K1" s="6" t="s">
+      <c r="K1" s="3" t="s">
         <v>65</v>
       </c>
-      <c r="L1" s="6" t="s">
+      <c r="L1" s="3" t="s">
         <v>33</v>
       </c>
-      <c r="M1" s="13"/>
-      <c r="N1" s="13"/>
-      <c r="O1" s="13"/>
-      <c r="P1" s="13"/>
-      <c r="Q1" s="13"/>
-      <c r="R1" s="13"/>
+      <c r="M1" s="16"/>
+      <c r="N1" s="16"/>
+      <c r="O1" s="16"/>
+      <c r="P1" s="16"/>
+      <c r="Q1" s="16"/>
+      <c r="R1" s="16"/>
     </row>
     <row r="2" spans="1:18">
-      <c r="A2" s="6" t="s">
+      <c r="A2" s="3" t="s">
         <v>54</v>
       </c>
-      <c r="B2" s="6" t="s">
+      <c r="B2" s="3" t="s">
         <v>54</v>
       </c>
-      <c r="C2" s="6" t="s">
+      <c r="C2" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="D2" s="6">
+      <c r="D2" s="3">
         <v>1010301033</v>
       </c>
-      <c r="E2" s="6" t="s">
+      <c r="E2" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="F2" s="6" t="s">
+      <c r="F2" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="G2" s="6" t="s">
+      <c r="G2" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="H2" s="6" t="s">
+      <c r="H2" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="I2" s="14" t="s">
+      <c r="I2" s="17" t="s">
         <v>43</v>
       </c>
-      <c r="J2" s="6" t="s">
+      <c r="J2" s="3" t="s">
         <v>44</v>
       </c>
-      <c r="K2" s="6" t="s">
+      <c r="K2" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="L2" s="6">
+      <c r="L2" s="3">
         <v>1</v>
       </c>
-      <c r="M2" s="13"/>
-      <c r="N2" s="13"/>
-      <c r="O2" s="13"/>
-      <c r="P2" s="13"/>
-      <c r="Q2" s="13"/>
-      <c r="R2" s="13"/>
+      <c r="M2" s="16"/>
+      <c r="N2" s="16"/>
+      <c r="O2" s="16"/>
+      <c r="P2" s="16"/>
+      <c r="Q2" s="16"/>
+      <c r="R2" s="16"/>
     </row>
     <row r="3" spans="1:12">
-      <c r="A3" s="6" t="s">
+      <c r="A3" s="3" t="s">
         <v>62</v>
       </c>
-      <c r="B3" s="6" t="s">
+      <c r="B3" s="3" t="s">
         <v>62</v>
       </c>
-      <c r="C3" s="6" t="s">
+      <c r="C3" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="D3" s="12">
+      <c r="D3" s="15">
         <v>1000000001</v>
       </c>
-      <c r="E3" s="6" t="s">
+      <c r="E3" s="3" t="s">
         <v>64</v>
       </c>
-      <c r="F3" s="6" t="s">
+      <c r="F3" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="G3" s="6" t="s">
+      <c r="G3" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="H3" s="6" t="s">
+      <c r="H3" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="I3" s="14" t="s">
+      <c r="I3" s="17" t="s">
         <v>43</v>
       </c>
-      <c r="J3" s="6" t="s">
+      <c r="J3" s="3" t="s">
         <v>44</v>
       </c>
-      <c r="K3" s="6" t="s">
+      <c r="K3" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="L3" s="6">
+      <c r="L3" s="3">
         <v>1</v>
       </c>
     </row>
@@ -3101,60 +3389,60 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6">
-      <c r="A1" s="10" t="s">
+      <c r="A1" s="13" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="10" t="s">
+      <c r="B1" s="13" t="s">
         <v>66</v>
       </c>
-      <c r="C1" s="10" t="s">
+      <c r="C1" s="13" t="s">
         <v>67</v>
       </c>
-      <c r="D1" s="11" t="s">
+      <c r="D1" s="14" t="s">
         <v>68</v>
       </c>
-      <c r="E1" s="9" t="s">
+      <c r="E1" s="12" t="s">
         <v>69</v>
       </c>
-      <c r="F1" s="9" t="s">
+      <c r="F1" s="12" t="s">
         <v>70</v>
       </c>
     </row>
     <row r="2" spans="1:6">
-      <c r="A2" s="6" t="s">
+      <c r="A2" s="3" t="s">
         <v>59</v>
       </c>
-      <c r="B2" s="6">
+      <c r="B2" s="3">
         <v>50</v>
       </c>
-      <c r="C2" s="6">
+      <c r="C2" s="3">
         <v>70</v>
       </c>
-      <c r="D2" s="6" t="s">
+      <c r="D2" s="3" t="s">
         <v>71</v>
       </c>
-      <c r="E2" s="6"/>
-      <c r="F2" s="4" t="s">
+      <c r="E2" s="3"/>
+      <c r="F2" s="9" t="s">
         <v>72</v>
       </c>
     </row>
     <row r="3" spans="1:6">
-      <c r="A3" s="6" t="s">
+      <c r="A3" s="3" t="s">
         <v>61</v>
       </c>
-      <c r="B3" s="6">
+      <c r="B3" s="3">
         <v>40</v>
       </c>
-      <c r="C3" s="6">
+      <c r="C3" s="3">
         <v>26</v>
       </c>
-      <c r="D3" s="6" t="s">
+      <c r="D3" s="3" t="s">
         <v>73</v>
       </c>
-      <c r="E3" s="4" t="s">
+      <c r="E3" s="9" t="s">
         <v>74</v>
       </c>
-      <c r="F3" s="4">
+      <c r="F3" s="9">
         <v>2</v>
       </c>
     </row>
@@ -3179,80 +3467,80 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6">
-      <c r="A1" s="10" t="s">
+      <c r="A1" s="13" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="10" t="s">
+      <c r="B1" s="13" t="s">
         <v>66</v>
       </c>
-      <c r="C1" s="10" t="s">
+      <c r="C1" s="13" t="s">
         <v>67</v>
       </c>
-      <c r="D1" s="11" t="s">
+      <c r="D1" s="14" t="s">
         <v>68</v>
       </c>
-      <c r="E1" s="9" t="s">
+      <c r="E1" s="12" t="s">
         <v>69</v>
       </c>
-      <c r="F1" s="9" t="s">
+      <c r="F1" s="12" t="s">
         <v>70</v>
       </c>
     </row>
     <row r="2" spans="1:6">
-      <c r="A2" s="9" t="s">
+      <c r="A2" s="12" t="s">
         <v>59</v>
       </c>
-      <c r="B2" s="6">
+      <c r="B2" s="3">
         <v>150</v>
       </c>
-      <c r="C2" s="6">
+      <c r="C2" s="3">
         <v>45</v>
       </c>
-      <c r="D2" s="6" t="s">
+      <c r="D2" s="3" t="s">
         <v>71</v>
       </c>
-      <c r="E2" s="6"/>
-      <c r="F2" s="4" t="s">
+      <c r="E2" s="3"/>
+      <c r="F2" s="9" t="s">
         <v>75</v>
       </c>
     </row>
     <row r="3" spans="1:6">
-      <c r="A3" s="9" t="s">
+      <c r="A3" s="12" t="s">
         <v>76</v>
       </c>
-      <c r="B3" s="6">
+      <c r="B3" s="3">
         <v>40</v>
       </c>
-      <c r="C3" s="6">
+      <c r="C3" s="3">
         <v>26</v>
       </c>
-      <c r="D3" s="6" t="s">
+      <c r="D3" s="3" t="s">
         <v>77</v>
       </c>
-      <c r="E3" s="4" t="s">
+      <c r="E3" s="9" t="s">
         <v>74</v>
       </c>
-      <c r="F3" s="4">
+      <c r="F3" s="9">
         <v>2</v>
       </c>
     </row>
     <row r="4" spans="1:6">
-      <c r="A4" s="9" t="s">
+      <c r="A4" s="12" t="s">
         <v>61</v>
       </c>
-      <c r="B4" s="6">
+      <c r="B4" s="3">
         <v>50</v>
       </c>
-      <c r="C4" s="6">
+      <c r="C4" s="3">
         <v>70</v>
       </c>
-      <c r="D4" s="6" t="s">
+      <c r="D4" s="3" t="s">
         <v>73</v>
       </c>
-      <c r="E4" s="6" t="s">
+      <c r="E4" s="3" t="s">
         <v>75</v>
       </c>
-      <c r="F4" s="4"/>
+      <c r="F4" s="9"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -3324,90 +3612,90 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7">
-      <c r="A1" s="9" t="s">
+      <c r="A1" s="12" t="s">
         <v>83</v>
       </c>
-      <c r="B1" s="9" t="s">
+      <c r="B1" s="12" t="s">
         <v>84</v>
       </c>
-      <c r="C1" s="9" t="s">
+      <c r="C1" s="12" t="s">
         <v>80</v>
       </c>
-      <c r="D1" s="9" t="s">
+      <c r="D1" s="12" t="s">
         <v>85</v>
       </c>
-      <c r="E1" s="9" t="s">
+      <c r="E1" s="12" t="s">
         <v>68</v>
       </c>
-      <c r="F1" s="9" t="s">
+      <c r="F1" s="12" t="s">
         <v>69</v>
       </c>
-      <c r="G1" s="9" t="s">
+      <c r="G1" s="12" t="s">
         <v>70</v>
       </c>
     </row>
     <row r="2" spans="1:7">
-      <c r="A2" s="9" t="s">
+      <c r="A2" s="12" t="s">
         <v>86</v>
       </c>
-      <c r="B2" s="9">
+      <c r="B2" s="12">
         <v>524</v>
       </c>
-      <c r="C2" s="9">
+      <c r="C2" s="12">
         <v>524</v>
       </c>
-      <c r="D2" s="9">
+      <c r="D2" s="12">
         <v>2</v>
       </c>
-      <c r="E2" s="4" t="s">
+      <c r="E2" s="9" t="s">
         <v>71</v>
       </c>
-      <c r="F2" s="4" t="s">
+      <c r="F2" s="9" t="s">
         <v>74</v>
       </c>
-      <c r="G2" s="4" t="s">
+      <c r="G2" s="9" t="s">
         <v>87</v>
       </c>
     </row>
     <row r="3" spans="1:7">
-      <c r="A3" s="9" t="s">
+      <c r="A3" s="12" t="s">
         <v>88</v>
       </c>
-      <c r="B3" s="9">
+      <c r="B3" s="12">
         <v>232</v>
       </c>
-      <c r="C3" s="9">
+      <c r="C3" s="12">
         <v>232</v>
       </c>
-      <c r="D3" s="9">
+      <c r="D3" s="12">
         <v>7.9</v>
       </c>
-      <c r="E3" s="4" t="s">
+      <c r="E3" s="9" t="s">
         <v>73</v>
       </c>
-      <c r="F3" s="4" t="s">
+      <c r="F3" s="9" t="s">
         <v>89</v>
       </c>
-      <c r="G3" s="6"/>
+      <c r="G3" s="3"/>
     </row>
     <row r="4" spans="1:7">
-      <c r="A4" s="6" t="s">
+      <c r="A4" s="3" t="s">
         <v>90</v>
       </c>
-      <c r="B4" s="6">
+      <c r="B4" s="3">
         <v>232</v>
       </c>
-      <c r="C4" s="6">
+      <c r="C4" s="3">
         <v>232</v>
       </c>
-      <c r="D4" s="6">
+      <c r="D4" s="3">
         <v>2.32</v>
       </c>
-      <c r="E4" s="4" t="s">
+      <c r="E4" s="9" t="s">
         <v>77</v>
       </c>
-      <c r="F4" s="6"/>
-      <c r="G4" s="6"/>
+      <c r="F4" s="3"/>
+      <c r="G4" s="3"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -3431,90 +3719,90 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7">
-      <c r="A1" s="9" t="s">
+      <c r="A1" s="12" t="s">
         <v>83</v>
       </c>
-      <c r="B1" s="9" t="s">
+      <c r="B1" s="12" t="s">
         <v>84</v>
       </c>
-      <c r="C1" s="9" t="s">
+      <c r="C1" s="12" t="s">
         <v>80</v>
       </c>
-      <c r="D1" s="9" t="s">
+      <c r="D1" s="12" t="s">
         <v>85</v>
       </c>
-      <c r="E1" s="9" t="s">
+      <c r="E1" s="12" t="s">
         <v>68</v>
       </c>
-      <c r="F1" s="9" t="s">
+      <c r="F1" s="12" t="s">
         <v>69</v>
       </c>
-      <c r="G1" s="9" t="s">
+      <c r="G1" s="12" t="s">
         <v>70</v>
       </c>
     </row>
     <row r="2" spans="1:7">
-      <c r="A2" s="9" t="s">
+      <c r="A2" s="12" t="s">
         <v>86</v>
       </c>
-      <c r="B2" s="9">
+      <c r="B2" s="12">
         <v>22</v>
       </c>
-      <c r="C2" s="9">
+      <c r="C2" s="12">
         <v>524</v>
       </c>
-      <c r="D2" s="9">
+      <c r="D2" s="12">
         <v>2</v>
       </c>
-      <c r="E2" s="4" t="s">
+      <c r="E2" s="9" t="s">
         <v>71</v>
       </c>
-      <c r="F2" s="4" t="s">
+      <c r="F2" s="9" t="s">
         <v>74</v>
       </c>
-      <c r="G2" s="4" t="s">
+      <c r="G2" s="9" t="s">
         <v>87</v>
       </c>
     </row>
     <row r="3" spans="1:7">
-      <c r="A3" s="9" t="s">
+      <c r="A3" s="12" t="s">
         <v>88</v>
       </c>
-      <c r="B3" s="9">
+      <c r="B3" s="12">
         <v>34</v>
       </c>
-      <c r="C3" s="9">
+      <c r="C3" s="12">
         <v>232</v>
       </c>
-      <c r="D3" s="9">
+      <c r="D3" s="12">
         <v>7.9</v>
       </c>
-      <c r="E3" s="4" t="s">
+      <c r="E3" s="9" t="s">
         <v>73</v>
       </c>
-      <c r="F3" s="4" t="s">
+      <c r="F3" s="9" t="s">
         <v>89</v>
       </c>
-      <c r="G3" s="6"/>
+      <c r="G3" s="3"/>
     </row>
     <row r="4" spans="1:7">
-      <c r="A4" s="6" t="s">
+      <c r="A4" s="3" t="s">
         <v>90</v>
       </c>
-      <c r="B4" s="6">
+      <c r="B4" s="3">
         <v>67</v>
       </c>
-      <c r="C4" s="6">
+      <c r="C4" s="3">
         <v>232</v>
       </c>
-      <c r="D4" s="6">
+      <c r="D4" s="3">
         <v>2.32</v>
       </c>
-      <c r="E4" s="4" t="s">
+      <c r="E4" s="9" t="s">
         <v>77</v>
       </c>
-      <c r="F4" s="6"/>
-      <c r="G4" s="6"/>
+      <c r="F4" s="3"/>
+      <c r="G4" s="3"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -3548,501 +3836,501 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:19">
-      <c r="A1" s="6" t="s">
+      <c r="A1" s="3" t="s">
         <v>91</v>
       </c>
-      <c r="B1" s="6" t="s">
+      <c r="B1" s="3" t="s">
         <v>92</v>
       </c>
-      <c r="C1" s="6" t="s">
+      <c r="C1" s="3" t="s">
         <v>93</v>
       </c>
-      <c r="D1" s="6" t="s">
+      <c r="D1" s="3" t="s">
         <v>94</v>
       </c>
-      <c r="E1" s="6" t="s">
+      <c r="E1" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="F1" s="6" t="s">
+      <c r="F1" s="3" t="s">
         <v>95</v>
       </c>
-      <c r="G1" s="6" t="s">
+      <c r="G1" s="3" t="s">
         <v>96</v>
       </c>
-      <c r="H1" s="6" t="s">
+      <c r="H1" s="3" t="s">
         <v>34</v>
       </c>
-      <c r="I1" s="6" t="s">
+      <c r="I1" s="3" t="s">
         <v>97</v>
       </c>
-      <c r="J1" s="6" t="s">
+      <c r="J1" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="K1" s="6" t="s">
+      <c r="K1" s="3" t="s">
         <v>98</v>
       </c>
-      <c r="L1" s="6" t="s">
+      <c r="L1" s="3" t="s">
         <v>99</v>
       </c>
-      <c r="M1" s="6" t="s">
+      <c r="M1" s="3" t="s">
         <v>100</v>
       </c>
-      <c r="N1" s="6" t="s">
+      <c r="N1" s="3" t="s">
         <v>101</v>
       </c>
-      <c r="O1" s="6" t="s">
+      <c r="O1" s="3" t="s">
         <v>102</v>
       </c>
-      <c r="P1" s="6" t="s">
+      <c r="P1" s="3" t="s">
         <v>103</v>
       </c>
-      <c r="Q1" s="6" t="s">
+      <c r="Q1" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="R1" s="6" t="s">
+      <c r="R1" s="3" t="s">
         <v>104</v>
       </c>
-      <c r="S1" s="8" t="s">
+      <c r="S1" s="5" t="s">
         <v>105</v>
       </c>
     </row>
     <row r="2" spans="1:19">
-      <c r="A2" s="7" t="s">
+      <c r="A2" s="11" t="s">
         <v>106</v>
       </c>
-      <c r="B2" s="6">
+      <c r="B2" s="3">
         <v>0</v>
       </c>
-      <c r="C2" s="7" t="s">
+      <c r="C2" s="11" t="s">
         <v>106</v>
       </c>
-      <c r="D2" s="6" t="s">
+      <c r="D2" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="E2" s="6" t="s">
+      <c r="E2" s="3" t="s">
         <v>40</v>
       </c>
-      <c r="F2" s="6">
+      <c r="F2" s="3">
         <v>12</v>
       </c>
-      <c r="G2" s="6" t="s">
+      <c r="G2" s="3" t="s">
         <v>41</v>
       </c>
-      <c r="H2" s="6"/>
-      <c r="I2" s="6"/>
-      <c r="J2" s="6" t="s">
+      <c r="H2" s="3"/>
+      <c r="I2" s="3"/>
+      <c r="J2" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="K2" s="6">
+      <c r="K2" s="3">
         <v>1</v>
       </c>
-      <c r="L2" s="6" t="s">
+      <c r="L2" s="3" t="s">
         <v>107</v>
       </c>
-      <c r="M2" s="6"/>
-      <c r="N2" s="6"/>
-      <c r="O2" s="4" t="s">
+      <c r="M2" s="3"/>
+      <c r="N2" s="3"/>
+      <c r="O2" s="9" t="s">
         <v>13</v>
       </c>
-      <c r="P2" s="4" t="s">
+      <c r="P2" s="9" t="s">
         <v>15</v>
       </c>
-      <c r="Q2" s="4" t="s">
+      <c r="Q2" s="9" t="s">
         <v>15</v>
       </c>
-      <c r="R2" s="6" t="s">
+      <c r="R2" s="3" t="s">
         <v>108</v>
       </c>
-      <c r="S2" s="5" t="s">
+      <c r="S2" s="10" t="s">
         <v>109</v>
       </c>
     </row>
     <row r="3" spans="1:19">
-      <c r="A3" s="7" t="s">
+      <c r="A3" s="11" t="s">
         <v>110</v>
       </c>
-      <c r="B3" s="6">
+      <c r="B3" s="3">
         <v>0</v>
       </c>
-      <c r="C3" s="7" t="s">
+      <c r="C3" s="11" t="s">
         <v>110</v>
       </c>
-      <c r="D3" s="6" t="s">
+      <c r="D3" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="E3" s="7">
+      <c r="E3" s="11">
         <v>772213</v>
       </c>
-      <c r="F3" s="6">
+      <c r="F3" s="3">
         <v>5</v>
       </c>
-      <c r="G3" s="6" t="s">
+      <c r="G3" s="3" t="s">
         <v>41</v>
       </c>
-      <c r="H3" s="6"/>
-      <c r="I3" s="6"/>
-      <c r="J3" s="6" t="s">
+      <c r="H3" s="3"/>
+      <c r="I3" s="3"/>
+      <c r="J3" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="K3" s="6">
+      <c r="K3" s="3">
         <v>3</v>
       </c>
-      <c r="L3" s="6" t="s">
+      <c r="L3" s="3" t="s">
         <v>107</v>
       </c>
-      <c r="M3" s="6"/>
-      <c r="N3" s="6"/>
-      <c r="O3" s="4" t="s">
+      <c r="M3" s="3"/>
+      <c r="N3" s="3"/>
+      <c r="O3" s="9" t="s">
         <v>13</v>
       </c>
-      <c r="P3" s="4" t="s">
+      <c r="P3" s="9" t="s">
         <v>15</v>
       </c>
-      <c r="Q3" s="4" t="s">
+      <c r="Q3" s="9" t="s">
         <v>15</v>
       </c>
-      <c r="R3" s="6" t="s">
+      <c r="R3" s="3" t="s">
         <v>108</v>
       </c>
-      <c r="S3" s="5" t="s">
+      <c r="S3" s="10" t="s">
         <v>109</v>
       </c>
     </row>
     <row r="4" spans="1:19">
-      <c r="A4" s="6" t="s">
+      <c r="A4" s="3" t="s">
         <v>111</v>
       </c>
-      <c r="B4" s="6">
+      <c r="B4" s="3">
         <v>0</v>
       </c>
-      <c r="C4" s="6" t="s">
+      <c r="C4" s="3" t="s">
         <v>111</v>
       </c>
-      <c r="D4" s="8" t="s">
+      <c r="D4" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="E4" s="6" t="s">
+      <c r="E4" s="3" t="s">
         <v>40</v>
       </c>
-      <c r="F4" s="6">
+      <c r="F4" s="3">
         <v>12</v>
       </c>
-      <c r="G4" s="8" t="s">
+      <c r="G4" s="5" t="s">
         <v>112</v>
       </c>
-      <c r="H4" s="6"/>
-      <c r="I4" s="6"/>
-      <c r="J4" s="6" t="s">
+      <c r="H4" s="3"/>
+      <c r="I4" s="3"/>
+      <c r="J4" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="K4" s="6">
+      <c r="K4" s="3">
         <v>1</v>
       </c>
-      <c r="L4" s="6" t="s">
+      <c r="L4" s="3" t="s">
         <v>107</v>
       </c>
-      <c r="M4" s="6" t="s">
+      <c r="M4" s="3" t="s">
         <v>111</v>
       </c>
-      <c r="N4" s="6" t="s">
+      <c r="N4" s="3" t="s">
         <v>111</v>
       </c>
-      <c r="O4" s="4" t="s">
+      <c r="O4" s="9" t="s">
         <v>13</v>
       </c>
-      <c r="P4" s="4" t="s">
+      <c r="P4" s="9" t="s">
         <v>15</v>
       </c>
-      <c r="Q4" s="4" t="s">
+      <c r="Q4" s="9" t="s">
         <v>15</v>
       </c>
-      <c r="R4" s="6" t="s">
+      <c r="R4" s="3" t="s">
         <v>108</v>
       </c>
-      <c r="S4" s="5" t="s">
+      <c r="S4" s="10" t="s">
         <v>109</v>
       </c>
     </row>
     <row r="5" spans="1:19">
-      <c r="A5" s="6" t="s">
+      <c r="A5" s="3" t="s">
         <v>113</v>
       </c>
-      <c r="B5" s="8">
+      <c r="B5" s="5">
         <v>0</v>
       </c>
-      <c r="C5" s="6" t="s">
+      <c r="C5" s="3" t="s">
         <v>113</v>
       </c>
-      <c r="D5" s="8" t="s">
+      <c r="D5" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="E5" s="6">
+      <c r="E5" s="3">
         <v>75052200</v>
       </c>
-      <c r="F5" s="8">
+      <c r="F5" s="5">
         <v>5</v>
       </c>
-      <c r="G5" s="8" t="s">
+      <c r="G5" s="5" t="s">
         <v>112</v>
       </c>
-      <c r="H5" s="6"/>
-      <c r="I5" s="6"/>
-      <c r="J5" s="8" t="s">
+      <c r="H5" s="3"/>
+      <c r="I5" s="3"/>
+      <c r="J5" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="K5" s="8">
+      <c r="K5" s="5">
         <v>2</v>
       </c>
-      <c r="L5" s="6" t="s">
+      <c r="L5" s="3" t="s">
         <v>107</v>
       </c>
-      <c r="M5" s="6" t="s">
+      <c r="M5" s="3" t="s">
         <v>113</v>
       </c>
-      <c r="N5" s="6" t="s">
+      <c r="N5" s="3" t="s">
         <v>113</v>
       </c>
-      <c r="O5" s="4" t="s">
+      <c r="O5" s="9" t="s">
         <v>13</v>
       </c>
-      <c r="P5" s="4" t="s">
+      <c r="P5" s="9" t="s">
         <v>15</v>
       </c>
-      <c r="Q5" s="4" t="s">
+      <c r="Q5" s="9" t="s">
         <v>15</v>
       </c>
-      <c r="R5" s="6" t="s">
+      <c r="R5" s="3" t="s">
         <v>114</v>
       </c>
-      <c r="S5" s="5" t="s">
+      <c r="S5" s="10" t="s">
         <v>109</v>
       </c>
     </row>
     <row r="6" spans="1:19">
-      <c r="A6" s="8" t="s">
+      <c r="A6" s="5" t="s">
         <v>115</v>
       </c>
-      <c r="B6" s="8">
+      <c r="B6" s="5">
         <v>0</v>
       </c>
-      <c r="C6" s="6" t="s">
+      <c r="C6" s="3" t="s">
         <v>115</v>
       </c>
-      <c r="D6" s="8" t="s">
+      <c r="D6" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="E6" s="8" t="s">
+      <c r="E6" s="5" t="s">
         <v>40</v>
       </c>
-      <c r="F6" s="8">
+      <c r="F6" s="5">
         <v>12</v>
       </c>
-      <c r="G6" s="8" t="s">
+      <c r="G6" s="5" t="s">
         <v>116</v>
       </c>
-      <c r="H6" s="8" t="s">
+      <c r="H6" s="5" t="s">
         <v>117</v>
       </c>
-      <c r="I6" s="6"/>
-      <c r="J6" s="8" t="s">
+      <c r="I6" s="3"/>
+      <c r="J6" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="K6" s="8">
+      <c r="K6" s="5">
         <v>1</v>
       </c>
-      <c r="L6" s="6" t="s">
+      <c r="L6" s="3" t="s">
         <v>107</v>
       </c>
-      <c r="M6" s="8" t="s">
+      <c r="M6" s="5" t="s">
         <v>115</v>
       </c>
-      <c r="N6" s="8" t="s">
+      <c r="N6" s="5" t="s">
         <v>115</v>
       </c>
-      <c r="O6" s="4" t="s">
+      <c r="O6" s="9" t="s">
         <v>13</v>
       </c>
-      <c r="P6" s="4" t="s">
+      <c r="P6" s="9" t="s">
         <v>15</v>
       </c>
-      <c r="Q6" s="4" t="s">
+      <c r="Q6" s="9" t="s">
         <v>15</v>
       </c>
-      <c r="R6" s="6" t="s">
+      <c r="R6" s="3" t="s">
         <v>108</v>
       </c>
-      <c r="S6" s="5" t="s">
+      <c r="S6" s="10" t="s">
         <v>109</v>
       </c>
     </row>
     <row r="7" spans="1:19">
-      <c r="A7" s="8" t="s">
+      <c r="A7" s="5" t="s">
         <v>118</v>
       </c>
-      <c r="B7" s="8">
+      <c r="B7" s="5">
         <v>0</v>
       </c>
-      <c r="C7" s="6" t="s">
+      <c r="C7" s="3" t="s">
         <v>118</v>
       </c>
-      <c r="D7" s="8" t="s">
+      <c r="D7" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="E7" s="8" t="s">
+      <c r="E7" s="5" t="s">
         <v>40</v>
       </c>
-      <c r="F7" s="8">
+      <c r="F7" s="5">
         <v>12</v>
       </c>
-      <c r="G7" s="8" t="s">
+      <c r="G7" s="5" t="s">
         <v>116</v>
       </c>
-      <c r="H7" s="8" t="s">
+      <c r="H7" s="5" t="s">
         <v>119</v>
       </c>
-      <c r="I7" s="6"/>
-      <c r="J7" s="8" t="s">
+      <c r="I7" s="3"/>
+      <c r="J7" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="K7" s="8">
+      <c r="K7" s="5">
         <v>4</v>
       </c>
-      <c r="L7" s="6" t="s">
+      <c r="L7" s="3" t="s">
         <v>107</v>
       </c>
-      <c r="M7" s="8" t="s">
+      <c r="M7" s="5" t="s">
         <v>118</v>
       </c>
-      <c r="N7" s="8" t="s">
+      <c r="N7" s="5" t="s">
         <v>118</v>
       </c>
-      <c r="O7" s="4" t="s">
+      <c r="O7" s="9" t="s">
         <v>13</v>
       </c>
-      <c r="P7" s="4" t="s">
+      <c r="P7" s="9" t="s">
         <v>15</v>
       </c>
-      <c r="Q7" s="4" t="s">
+      <c r="Q7" s="9" t="s">
         <v>15</v>
       </c>
-      <c r="R7" s="6" t="s">
+      <c r="R7" s="3" t="s">
         <v>108</v>
       </c>
-      <c r="S7" s="5" t="s">
+      <c r="S7" s="10" t="s">
         <v>109</v>
       </c>
     </row>
     <row r="8" spans="1:19">
-      <c r="A8" s="6" t="s">
+      <c r="A8" s="3" t="s">
         <v>120</v>
       </c>
-      <c r="B8" s="8">
+      <c r="B8" s="5">
         <v>0</v>
       </c>
-      <c r="C8" s="6" t="s">
+      <c r="C8" s="3" t="s">
         <v>120</v>
       </c>
-      <c r="D8" s="8" t="s">
+      <c r="D8" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="E8" s="6" t="s">
+      <c r="E8" s="3" t="s">
         <v>121</v>
       </c>
-      <c r="F8" s="8">
+      <c r="F8" s="5">
         <v>5</v>
       </c>
-      <c r="G8" s="8" t="s">
+      <c r="G8" s="5" t="s">
         <v>122</v>
       </c>
-      <c r="H8" s="6"/>
-      <c r="I8" s="6">
+      <c r="H8" s="3"/>
+      <c r="I8" s="3">
         <v>95</v>
       </c>
-      <c r="J8" s="8" t="s">
+      <c r="J8" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="K8" s="8">
+      <c r="K8" s="5">
         <v>1</v>
       </c>
-      <c r="L8" s="6" t="s">
+      <c r="L8" s="3" t="s">
         <v>107</v>
       </c>
-      <c r="M8" s="6" t="s">
+      <c r="M8" s="3" t="s">
         <v>120</v>
       </c>
-      <c r="N8" s="6" t="s">
+      <c r="N8" s="3" t="s">
         <v>120</v>
       </c>
-      <c r="O8" s="4" t="s">
+      <c r="O8" s="9" t="s">
         <v>13</v>
       </c>
-      <c r="P8" s="4" t="s">
+      <c r="P8" s="9" t="s">
         <v>15</v>
       </c>
-      <c r="Q8" s="4" t="s">
+      <c r="Q8" s="9" t="s">
         <v>15</v>
       </c>
-      <c r="R8" s="6" t="s">
+      <c r="R8" s="3" t="s">
         <v>108</v>
       </c>
-      <c r="S8" s="5" t="s">
+      <c r="S8" s="10" t="s">
         <v>109</v>
       </c>
     </row>
     <row r="9" spans="1:19">
-      <c r="A9" s="8" t="s">
+      <c r="A9" s="5" t="s">
         <v>123</v>
       </c>
-      <c r="B9" s="8">
+      <c r="B9" s="5">
         <v>0</v>
       </c>
-      <c r="C9" s="6" t="s">
+      <c r="C9" s="3" t="s">
         <v>123</v>
       </c>
-      <c r="D9" s="8" t="s">
+      <c r="D9" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="E9" s="8" t="s">
+      <c r="E9" s="5" t="s">
         <v>40</v>
       </c>
-      <c r="F9" s="8">
+      <c r="F9" s="5">
         <v>12</v>
       </c>
-      <c r="G9" s="8" t="s">
+      <c r="G9" s="5" t="s">
         <v>122</v>
       </c>
-      <c r="H9" s="6"/>
-      <c r="I9" s="6">
+      <c r="H9" s="3"/>
+      <c r="I9" s="3">
         <v>97</v>
       </c>
-      <c r="J9" s="8" t="s">
+      <c r="J9" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="K9" s="8">
+      <c r="K9" s="5">
         <v>4</v>
       </c>
-      <c r="L9" s="6" t="s">
+      <c r="L9" s="3" t="s">
         <v>107</v>
       </c>
-      <c r="M9" s="8" t="s">
+      <c r="M9" s="5" t="s">
         <v>123</v>
       </c>
-      <c r="N9" s="8" t="s">
+      <c r="N9" s="5" t="s">
         <v>123</v>
       </c>
-      <c r="O9" s="4" t="s">
+      <c r="O9" s="9" t="s">
         <v>13</v>
       </c>
-      <c r="P9" s="4" t="s">
+      <c r="P9" s="9" t="s">
         <v>15</v>
       </c>
-      <c r="Q9" s="4" t="s">
+      <c r="Q9" s="9" t="s">
         <v>15</v>
       </c>
-      <c r="R9" s="6" t="s">
+      <c r="R9" s="3" t="s">
         <v>108</v>
       </c>
-      <c r="S9" s="5" t="s">
+      <c r="S9" s="10" t="s">
         <v>109</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Added New Test Scenarios for the Sales Order Screen
Added New Test Scenarios for the Sales Order Screen And then Modify The Existing Test Scenarios methods
</commit_message>
<xml_diff>
--- a/testdata/ItemDetails.xlsx
+++ b/testdata/ItemDetails.xlsx
@@ -1,10 +1,10 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
+  <fileVersion appName="xl" lastEdited="4" lowestEdited="5" rupBuild="4505"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="23040" windowHeight="9120" firstSheet="6" activeTab="11"/>
+    <workbookView xWindow="-15" yWindow="2355" windowWidth="15030" windowHeight="6540" firstSheet="7" activeTab="8"/>
   </bookViews>
   <sheets>
     <sheet name="PR Details" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,8 @@
     <sheet name="Open Sales" sheetId="11" r:id="rId11"/>
     <sheet name="SI Details" sheetId="12" r:id="rId12"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="124519"/>
+  <oleSize ref="A1:G20"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -572,14 +573,8 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="xr9">
-  <numFmts count="4">
-    <numFmt numFmtId="176" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
-    <numFmt numFmtId="177" formatCode="_ &quot;₹&quot;* #,##0.00_ ;_ &quot;₹&quot;* \-#,##0.00_ ;_ &quot;₹&quot;* &quot;-&quot;??_ ;_ @_ "/>
-    <numFmt numFmtId="178" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
-    <numFmt numFmtId="179" formatCode="_ &quot;₹&quot;* #,##0_ ;_ &quot;₹&quot;* \-#,##0_ ;_ &quot;₹&quot;* &quot;-&quot;_ ;_ @_ "/>
-  </numFmts>
-  <fonts count="30">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <fonts count="11">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -650,152 +645,8 @@
       <name val="Times New Roman"/>
       <charset val="134"/>
     </font>
-    <font>
-      <u/>
-      <sz val="11"/>
-      <color rgb="FF0000FF"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <u/>
-      <sz val="11"/>
-      <color rgb="FF800080"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FFFF0000"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="18"/>
-      <color theme="3"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <i/>
-      <sz val="11"/>
-      <color rgb="FF7F7F7F"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="15"/>
-      <color theme="3"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="13"/>
-      <color theme="3"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="3"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF3F3F76"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FF3F3F3F"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FFFA7D00"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FFFFFFFF"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FFFA7D00"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF006100"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF9C0006"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF9C6500"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="0"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
   </fonts>
-  <fills count="36">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -804,7 +655,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.599993896298105"/>
+        <fgColor theme="9" tint="0.59999389629810485"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -820,194 +671,8 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFFCC"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFCC99"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFF2F2F2"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFA5A5A5"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFC6EFCE"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFC7CE"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFEB9C"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
   </fills>
-  <borders count="11">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -1045,254 +710,12 @@
       </bottom>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color rgb="FFB2B2B2"/>
-      </left>
-      <right style="thin">
-        <color rgb="FFB2B2B2"/>
-      </right>
-      <top style="thin">
-        <color rgb="FFB2B2B2"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FFB2B2B2"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="medium">
-        <color theme="4"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="medium">
-        <color theme="4" tint="0.499984740745262"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF7F7F7F"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF7F7F7F"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF7F7F7F"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF7F7F7F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF3F3F3F"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF3F3F3F"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF3F3F3F"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF3F3F3F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="double">
-        <color rgb="FF3F3F3F"/>
-      </left>
-      <right style="double">
-        <color rgb="FF3F3F3F"/>
-      </right>
-      <top style="double">
-        <color rgb="FF3F3F3F"/>
-      </top>
-      <bottom style="double">
-        <color rgb="FF3F3F3F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="double">
-        <color rgb="FFFF8001"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color theme="4"/>
-      </top>
-      <bottom style="double">
-        <color theme="4"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
-  <cellStyleXfs count="50">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="176" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="177" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="178" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="179" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="3" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="5" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="6" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="7" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="7" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="8" borderId="8" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="10" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="35" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
@@ -1358,10 +781,10 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="49" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="49" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -1380,90 +803,159 @@
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
-  <cellStyles count="50">
+  <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Comma" xfId="1" builtinId="3"/>
-    <cellStyle name="Currency" xfId="2" builtinId="4"/>
-    <cellStyle name="Percent" xfId="3" builtinId="5"/>
-    <cellStyle name="Comma [0]" xfId="4" builtinId="6"/>
-    <cellStyle name="Currency [0]" xfId="5" builtinId="7"/>
-    <cellStyle name="Hyperlink" xfId="6" builtinId="8"/>
-    <cellStyle name="Followed Hyperlink" xfId="7" builtinId="9"/>
-    <cellStyle name="Note" xfId="8" builtinId="10"/>
-    <cellStyle name="Warning Text" xfId="9" builtinId="11"/>
-    <cellStyle name="Title" xfId="10" builtinId="15"/>
-    <cellStyle name="CExplanatory Text" xfId="11" builtinId="53"/>
-    <cellStyle name="Heading 1" xfId="12" builtinId="16"/>
-    <cellStyle name="Heading 2" xfId="13" builtinId="17"/>
-    <cellStyle name="Heading 3" xfId="14" builtinId="18"/>
-    <cellStyle name="Heading 4" xfId="15" builtinId="19"/>
-    <cellStyle name="Input" xfId="16" builtinId="20"/>
-    <cellStyle name="Output" xfId="17" builtinId="21"/>
-    <cellStyle name="Calculation" xfId="18" builtinId="22"/>
-    <cellStyle name="Check Cell" xfId="19" builtinId="23"/>
-    <cellStyle name="Linked Cell" xfId="20" builtinId="24"/>
-    <cellStyle name="Total" xfId="21" builtinId="25"/>
-    <cellStyle name="Good" xfId="22" builtinId="26"/>
-    <cellStyle name="Bad" xfId="23" builtinId="27"/>
-    <cellStyle name="Neutral" xfId="24" builtinId="28"/>
-    <cellStyle name="Accent1" xfId="25" builtinId="29"/>
-    <cellStyle name="20% - Accent1" xfId="26" builtinId="30"/>
-    <cellStyle name="40% - Accent1" xfId="27" builtinId="31"/>
-    <cellStyle name="60% - Accent1" xfId="28" builtinId="32"/>
-    <cellStyle name="Accent2" xfId="29" builtinId="33"/>
-    <cellStyle name="20% - Accent2" xfId="30" builtinId="34"/>
-    <cellStyle name="40% - Accent2" xfId="31" builtinId="35"/>
-    <cellStyle name="60% - Accent2" xfId="32" builtinId="36"/>
-    <cellStyle name="Accent3" xfId="33" builtinId="37"/>
-    <cellStyle name="20% - Accent3" xfId="34" builtinId="38"/>
-    <cellStyle name="40% - Accent3" xfId="35" builtinId="39"/>
-    <cellStyle name="60% - Accent3" xfId="36" builtinId="40"/>
-    <cellStyle name="Accent4" xfId="37" builtinId="41"/>
-    <cellStyle name="20% - Accent4" xfId="38" builtinId="42"/>
-    <cellStyle name="40% - Accent4" xfId="39" builtinId="43"/>
-    <cellStyle name="60% - Accent4" xfId="40" builtinId="44"/>
-    <cellStyle name="Accent5" xfId="41" builtinId="45"/>
-    <cellStyle name="20% - Accent5" xfId="42" builtinId="46"/>
-    <cellStyle name="40% - Accent5" xfId="43" builtinId="47"/>
-    <cellStyle name="60% - Accent5" xfId="44" builtinId="48"/>
-    <cellStyle name="Accent6" xfId="45" builtinId="49"/>
-    <cellStyle name="20% - Accent6" xfId="46" builtinId="50"/>
-    <cellStyle name="40% - Accent6" xfId="47" builtinId="51"/>
-    <cellStyle name="60% - Accent6" xfId="48" builtinId="52"/>
-    <cellStyle name="Normal 2" xfId="49"/>
+    <cellStyle name="Normal 2" xfId="1"/>
   </cellStyles>
   <dxfs count="17">
     <dxf>
       <fill>
         <patternFill patternType="solid">
-          <fgColor theme="4" tint="0.799981688894314"/>
-          <bgColor theme="4" tint="0.799981688894314"/>
+          <fgColor theme="4" tint="0.79995117038483843"/>
+          <bgColor theme="4" tint="0.79995117038483843"/>
+        </patternFill>
+      </fill>
+      <border>
+        <bottom style="thin">
+          <color theme="4" tint="0.39994506668294322"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor theme="4" tint="0.79995117038483843"/>
+          <bgColor theme="4" tint="0.79995117038483843"/>
+        </patternFill>
+      </fill>
+      <border>
+        <bottom style="thin">
+          <color theme="4" tint="0.39994506668294322"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="1"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="1"/>
+      </font>
+      <border>
+        <bottom style="thin">
+          <color theme="4" tint="0.39994506668294322"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <color theme="1"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <color theme="1"/>
+      </font>
+      <border>
+        <top style="thin">
+          <color theme="4"/>
+        </top>
+        <bottom style="thin">
+          <color theme="4"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor theme="4" tint="0.79995117038483843"/>
+          <bgColor theme="4" tint="0.79995117038483843"/>
         </patternFill>
       </fill>
     </dxf>
     <dxf>
       <fill>
         <patternFill patternType="solid">
-          <fgColor theme="4" tint="0.799981688894314"/>
-          <bgColor theme="4" tint="0.799981688894314"/>
+          <fgColor theme="4" tint="0.79995117038483843"/>
+          <bgColor theme="4" tint="0.79995117038483843"/>
         </patternFill>
       </fill>
     </dxf>
     <dxf>
       <font>
-        <b val="1"/>
+        <b/>
+        <color theme="1"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor theme="4" tint="0.79995117038483843"/>
+          <bgColor theme="4" tint="0.79995117038483843"/>
+        </patternFill>
+      </fill>
+      <border>
+        <top style="thin">
+          <color theme="4" tint="0.39994506668294322"/>
+        </top>
+        <bottom style="thin">
+          <color theme="4" tint="0.39994506668294322"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <color theme="1"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor theme="4" tint="0.79995117038483843"/>
+          <bgColor theme="4" tint="0.79995117038483843"/>
+        </patternFill>
+      </fill>
+      <border>
+        <bottom style="thin">
+          <color theme="4" tint="0.39994506668294322"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor theme="4" tint="0.79995117038483843"/>
+          <bgColor theme="4" tint="0.79995117038483843"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor theme="4" tint="0.79995117038483843"/>
+          <bgColor theme="4" tint="0.79995117038483843"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
         <color theme="1"/>
       </font>
     </dxf>
     <dxf>
       <font>
-        <b val="1"/>
+        <b/>
         <color theme="1"/>
       </font>
     </dxf>
     <dxf>
       <font>
-        <b val="1"/>
+        <b/>
         <color theme="1"/>
       </font>
       <border>
@@ -1474,7 +966,7 @@
     </dxf>
     <dxf>
       <font>
-        <b val="1"/>
+        <b/>
         <color theme="0"/>
       </font>
       <fill>
@@ -1502,149 +994,32 @@
           <color theme="4"/>
         </bottom>
         <horizontal style="thin">
-          <color theme="4" tint="0.399975585192419"/>
+          <color theme="4" tint="0.39994506668294322"/>
         </horizontal>
-      </border>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor theme="4" tint="0.799981688894314"/>
-          <bgColor theme="4" tint="0.799981688894314"/>
-        </patternFill>
-      </fill>
-      <border>
-        <bottom style="thin">
-          <color theme="4" tint="0.399975585192419"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="1"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor theme="4" tint="0.799981688894314"/>
-          <bgColor theme="4" tint="0.799981688894314"/>
-        </patternFill>
-      </fill>
-      <border>
-        <bottom style="thin">
-          <color theme="4" tint="0.399975585192419"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="1"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="1"/>
-      </font>
-      <border>
-        <bottom style="thin">
-          <color theme="4" tint="0.399975585192419"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="1"/>
-        <color theme="1"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="1"/>
-        <color theme="1"/>
-      </font>
-      <border>
-        <top style="thin">
-          <color theme="4"/>
-        </top>
-        <bottom style="thin">
-          <color theme="4"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor theme="4" tint="0.799981688894314"/>
-          <bgColor theme="4" tint="0.799981688894314"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor theme="4" tint="0.799981688894314"/>
-          <bgColor theme="4" tint="0.799981688894314"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="1"/>
-        <color theme="1"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor theme="4" tint="0.799981688894314"/>
-          <bgColor theme="4" tint="0.799981688894314"/>
-        </patternFill>
-      </fill>
-      <border>
-        <top style="thin">
-          <color theme="4" tint="0.399975585192419"/>
-        </top>
-        <bottom style="thin">
-          <color theme="4" tint="0.399975585192419"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="1"/>
-        <color theme="1"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor theme="4" tint="0.799981688894314"/>
-          <bgColor theme="4" tint="0.799981688894314"/>
-        </patternFill>
-      </fill>
-      <border>
-        <bottom style="thin">
-          <color theme="4" tint="0.399975585192419"/>
-        </bottom>
       </border>
     </dxf>
   </dxfs>
   <tableStyles count="2" defaultTableStyle="TableStylePreset3_Accent1" defaultPivotStyle="PivotStylePreset2_Accent1">
-    <tableStyle name="TableStylePreset3_Accent1" pivot="0" count="7" xr9:uid="{59DB682C-5494-4EDE-A608-00C9E5F0F923}">
-      <tableStyleElement type="wholeTable" dxfId="6"/>
-      <tableStyleElement type="headerRow" dxfId="5"/>
-      <tableStyleElement type="totalRow" dxfId="4"/>
-      <tableStyleElement type="firstColumn" dxfId="3"/>
-      <tableStyleElement type="lastColumn" dxfId="2"/>
-      <tableStyleElement type="firstRowStripe" dxfId="1"/>
-      <tableStyleElement type="firstColumnStripe" dxfId="0"/>
+    <tableStyle name="TableStylePreset3_Accent1" pivot="0" count="7">
+      <tableStyleElement type="wholeTable" dxfId="16"/>
+      <tableStyleElement type="headerRow" dxfId="15"/>
+      <tableStyleElement type="totalRow" dxfId="14"/>
+      <tableStyleElement type="firstColumn" dxfId="13"/>
+      <tableStyleElement type="lastColumn" dxfId="12"/>
+      <tableStyleElement type="firstRowStripe" dxfId="11"/>
+      <tableStyleElement type="firstColumnStripe" dxfId="10"/>
     </tableStyle>
-    <tableStyle name="PivotStylePreset2_Accent1" table="0" count="10" xr9:uid="{267968C8-6FFD-4C36-ACC1-9EA1FD1885CA}">
-      <tableStyleElement type="headerRow" dxfId="16"/>
-      <tableStyleElement type="totalRow" dxfId="15"/>
-      <tableStyleElement type="firstRowStripe" dxfId="14"/>
-      <tableStyleElement type="firstColumnStripe" dxfId="13"/>
-      <tableStyleElement type="firstSubtotalRow" dxfId="12"/>
-      <tableStyleElement type="secondSubtotalRow" dxfId="11"/>
-      <tableStyleElement type="firstRowSubheading" dxfId="10"/>
-      <tableStyleElement type="secondRowSubheading" dxfId="9"/>
-      <tableStyleElement type="pageFieldLabels" dxfId="8"/>
-      <tableStyleElement type="pageFieldValues" dxfId="7"/>
+    <tableStyle name="PivotStylePreset2_Accent1" table="0" count="10">
+      <tableStyleElement type="headerRow" dxfId="9"/>
+      <tableStyleElement type="totalRow" dxfId="8"/>
+      <tableStyleElement type="firstRowStripe" dxfId="7"/>
+      <tableStyleElement type="firstColumnStripe" dxfId="6"/>
+      <tableStyleElement type="firstSubtotalRow" dxfId="5"/>
+      <tableStyleElement type="secondSubtotalRow" dxfId="4"/>
+      <tableStyleElement type="firstRowSubheading" dxfId="3"/>
+      <tableStyleElement type="secondRowSubheading" dxfId="2"/>
+      <tableStyleElement type="pageFieldLabels" dxfId="1"/>
+      <tableStyleElement type="pageFieldValues" dxfId="0"/>
     </tableStyle>
   </tableStyles>
   <extLst>
@@ -1907,23 +1282,23 @@
     </a:fmtScheme>
   </a:themeElements>
   <a:objectDefaults/>
+  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
-  <sheetPr/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:J20"/>
-  <sheetFormatPr defaultColWidth="8.73148148148148" defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="20.7314814814815" customWidth="1"/>
-    <col min="2" max="3" width="12.7314814814815" customWidth="1"/>
-    <col min="4" max="4" width="14.7314814814815" customWidth="1"/>
-    <col min="5" max="5" width="9.81481481481481" customWidth="1"/>
-    <col min="6" max="6" width="14.1851851851852" customWidth="1"/>
-    <col min="7" max="7" width="14.8148148148148" customWidth="1"/>
-    <col min="8" max="8" width="22.2222222222222" customWidth="1"/>
-    <col min="9" max="9" width="14.3611111111111" customWidth="1"/>
+    <col min="1" max="1" width="20.7109375" customWidth="1"/>
+    <col min="2" max="3" width="12.7109375" customWidth="1"/>
+    <col min="4" max="4" width="14.7109375" customWidth="1"/>
+    <col min="5" max="5" width="9.85546875" customWidth="1"/>
+    <col min="6" max="6" width="14.140625" customWidth="1"/>
+    <col min="7" max="7" width="14.85546875" customWidth="1"/>
+    <col min="8" max="8" width="22.28515625" customWidth="1"/>
+    <col min="9" max="9" width="14.42578125" customWidth="1"/>
     <col min="10" max="10" width="13" customWidth="1"/>
   </cols>
   <sheetData>
@@ -1959,7 +1334,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="2" s="23" customFormat="1" ht="20.4" spans="1:10">
+    <row r="2" spans="1:10" s="23" customFormat="1" ht="22.5">
       <c r="A2" s="25" t="s">
         <v>10</v>
       </c>
@@ -1991,7 +1366,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="3" ht="15" customHeight="1" spans="1:10">
+    <row r="3" spans="1:10" ht="15" customHeight="1">
       <c r="A3" s="25" t="s">
         <v>18</v>
       </c>
@@ -2023,7 +1398,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="4" spans="1:10">
+    <row r="4" spans="1:10" ht="22.5">
       <c r="A4" s="25" t="s">
         <v>21</v>
       </c>
@@ -2249,27 +1624,25 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
-  <sheetPr/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:K3"/>
-  <sheetFormatPr defaultColWidth="8.88888888888889" defaultRowHeight="14.4" outlineLevelRow="2"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="9" customWidth="1"/>
-    <col min="2" max="2" width="25.7777777777778" customWidth="1"/>
-    <col min="3" max="3" width="12.4444444444444" customWidth="1"/>
-    <col min="4" max="4" width="16.2222222222222" customWidth="1"/>
-    <col min="5" max="5" width="20.2222222222222" customWidth="1"/>
-    <col min="6" max="6" width="25.7777777777778" customWidth="1"/>
-    <col min="7" max="7" width="12.2222222222222" customWidth="1"/>
-    <col min="8" max="8" width="14.5555555555556" customWidth="1"/>
-    <col min="9" max="9" width="28.5555555555556" customWidth="1"/>
+    <col min="2" max="2" width="25.7109375" customWidth="1"/>
+    <col min="3" max="3" width="12.42578125" customWidth="1"/>
+    <col min="4" max="4" width="16.28515625" customWidth="1"/>
+    <col min="5" max="5" width="20.28515625" customWidth="1"/>
+    <col min="6" max="6" width="25.7109375" customWidth="1"/>
+    <col min="7" max="7" width="12.28515625" customWidth="1"/>
+    <col min="8" max="8" width="14.5703125" customWidth="1"/>
+    <col min="9" max="9" width="28.5703125" customWidth="1"/>
     <col min="10" max="10" width="23" customWidth="1"/>
-    <col min="11" max="11" width="14.6666666666667" customWidth="1"/>
+    <col min="11" max="11" width="14.7109375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:11">
@@ -2379,24 +1752,22 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
-  <sheetPr/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:E2"/>
-  <sheetFormatPr defaultColWidth="8.88888888888889" defaultRowHeight="14.4" outlineLevelRow="1" outlineLevelCol="4"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="13.5555555555556" customWidth="1"/>
+    <col min="1" max="1" width="13.5703125" customWidth="1"/>
     <col min="2" max="2" width="6" customWidth="1"/>
-    <col min="3" max="3" width="14.4444444444444" customWidth="1"/>
-    <col min="4" max="4" width="18.1111111111111" customWidth="1"/>
-    <col min="5" max="5" width="19.5555555555556" customWidth="1"/>
+    <col min="3" max="3" width="14.42578125" customWidth="1"/>
+    <col min="4" max="4" width="18.140625" customWidth="1"/>
+    <col min="5" max="5" width="19.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="15.15" spans="1:5">
+    <row r="1" spans="1:5">
       <c r="A1" s="6" t="s">
         <v>150</v>
       </c>
@@ -2413,7 +1784,7 @@
         <v>154</v>
       </c>
     </row>
-    <row r="2" ht="15.15" spans="1:5">
+    <row r="2" spans="1:5" ht="30">
       <c r="A2" s="6" t="s">
         <v>155</v>
       </c>
@@ -2432,23 +1803,21 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
-  <sheetPr/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:G8"/>
-  <sheetFormatPr defaultColWidth="8.88888888888889" defaultRowHeight="14.4" outlineLevelRow="7" outlineLevelCol="6"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="25.7777777777778" customWidth="1"/>
-    <col min="2" max="2" width="8.88888888888889" customWidth="1"/>
-    <col min="3" max="3" width="12.2222222222222" customWidth="1"/>
-    <col min="4" max="4" width="7.11111111111111" customWidth="1"/>
-    <col min="5" max="5" width="5.22222222222222" customWidth="1"/>
-    <col min="6" max="6" width="17.4444444444444" customWidth="1"/>
-    <col min="7" max="7" width="12.4444444444444" customWidth="1"/>
+    <col min="1" max="1" width="25.7109375" customWidth="1"/>
+    <col min="2" max="2" width="8.85546875" customWidth="1"/>
+    <col min="3" max="3" width="12.28515625" customWidth="1"/>
+    <col min="4" max="4" width="7.140625" customWidth="1"/>
+    <col min="5" max="5" width="5.28515625" customWidth="1"/>
+    <col min="6" max="6" width="17.42578125" customWidth="1"/>
+    <col min="7" max="7" width="12.42578125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7">
@@ -2637,36 +2006,34 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
-  <sheetPr/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:T10"/>
-  <sheetFormatPr defaultColWidth="8.73148148148148" defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="30" customWidth="1"/>
-    <col min="2" max="2" width="36.4444444444444" customWidth="1"/>
+    <col min="2" max="2" width="36.42578125" customWidth="1"/>
     <col min="3" max="3" width="6" customWidth="1"/>
-    <col min="4" max="4" width="13.6666666666667" customWidth="1"/>
-    <col min="5" max="5" width="5.22222222222222" customWidth="1"/>
-    <col min="6" max="6" width="17.2222222222222" customWidth="1"/>
-    <col min="7" max="7" width="30.2222222222222" customWidth="1"/>
-    <col min="8" max="8" width="26.8888888888889" customWidth="1"/>
-    <col min="9" max="9" width="17.2222222222222" customWidth="1"/>
-    <col min="10" max="10" width="13.2222222222222" customWidth="1"/>
-    <col min="11" max="11" width="22.7777777777778" customWidth="1"/>
-    <col min="12" max="12" width="12.7777777777778" customWidth="1"/>
-    <col min="13" max="13" width="29.5555555555556" customWidth="1"/>
-    <col min="14" max="14" width="18.2222222222222" customWidth="1"/>
-    <col min="15" max="15" width="16.2222222222222" customWidth="1"/>
-    <col min="16" max="16" width="15.5555555555556" customWidth="1"/>
-    <col min="17" max="17" width="17.7777777777778" customWidth="1"/>
-    <col min="18" max="18" width="24.1111111111111" customWidth="1"/>
-    <col min="19" max="19" width="13.4444444444444" customWidth="1"/>
-    <col min="20" max="20" width="13.5555555555556" customWidth="1"/>
+    <col min="4" max="4" width="13.7109375" customWidth="1"/>
+    <col min="5" max="5" width="5.28515625" customWidth="1"/>
+    <col min="6" max="6" width="17.28515625" customWidth="1"/>
+    <col min="7" max="7" width="30.28515625" customWidth="1"/>
+    <col min="8" max="8" width="26.85546875" customWidth="1"/>
+    <col min="9" max="9" width="17.28515625" customWidth="1"/>
+    <col min="10" max="10" width="13.28515625" customWidth="1"/>
+    <col min="11" max="11" width="22.7109375" customWidth="1"/>
+    <col min="12" max="12" width="12.7109375" customWidth="1"/>
+    <col min="13" max="13" width="29.5703125" customWidth="1"/>
+    <col min="14" max="14" width="18.28515625" customWidth="1"/>
+    <col min="15" max="15" width="16.28515625" customWidth="1"/>
+    <col min="16" max="16" width="15.5703125" customWidth="1"/>
+    <col min="17" max="17" width="17.7109375" customWidth="1"/>
+    <col min="18" max="18" width="24.140625" customWidth="1"/>
+    <col min="19" max="19" width="13.42578125" customWidth="1"/>
+    <col min="20" max="20" width="13.5703125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:20">
@@ -3219,27 +2586,25 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
-  <sheetPr/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:R3"/>
-  <sheetFormatPr defaultColWidth="8.88888888888889" defaultRowHeight="14.4" outlineLevelRow="2"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="2" width="21" customWidth="1"/>
     <col min="3" max="3" width="6" customWidth="1"/>
-    <col min="4" max="4" width="12.7777777777778" customWidth="1"/>
-    <col min="5" max="5" width="19.4444444444444" customWidth="1"/>
-    <col min="6" max="6" width="15.1111111111111" customWidth="1"/>
-    <col min="7" max="7" width="15.4444444444444" customWidth="1"/>
-    <col min="8" max="8" width="19.5555555555556" customWidth="1"/>
-    <col min="9" max="9" width="10.8888888888889" customWidth="1"/>
-    <col min="10" max="10" width="17.5555555555556" customWidth="1"/>
-    <col min="11" max="11" width="11.2222222222222" customWidth="1"/>
-    <col min="12" max="12" width="21.6666666666667" customWidth="1"/>
+    <col min="4" max="4" width="12.7109375" customWidth="1"/>
+    <col min="5" max="5" width="19.42578125" customWidth="1"/>
+    <col min="6" max="6" width="15.140625" customWidth="1"/>
+    <col min="7" max="7" width="15.42578125" customWidth="1"/>
+    <col min="8" max="8" width="19.5703125" customWidth="1"/>
+    <col min="9" max="9" width="10.85546875" customWidth="1"/>
+    <col min="10" max="10" width="17.5703125" customWidth="1"/>
+    <col min="11" max="11" width="11.28515625" customWidth="1"/>
+    <col min="12" max="12" width="21.7109375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:18">
@@ -3330,7 +2695,7 @@
       <c r="Q2" s="16"/>
       <c r="R2" s="16"/>
     </row>
-    <row r="3" spans="1:12">
+    <row r="3" spans="1:18">
       <c r="A3" s="3" t="s">
         <v>62</v>
       </c>
@@ -3370,22 +2735,20 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
-  <sheetPr/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:F3"/>
-  <sheetFormatPr defaultColWidth="8.88888888888889" defaultRowHeight="14.4" outlineLevelRow="2" outlineLevelCol="5"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="27.1111111111111" customWidth="1"/>
-    <col min="2" max="2" width="10.4444444444444" customWidth="1"/>
-    <col min="3" max="3" width="11.4444444444444" customWidth="1"/>
-    <col min="4" max="4" width="11.6666666666667" customWidth="1"/>
-    <col min="5" max="5" width="14.5555555555556" customWidth="1"/>
-    <col min="6" max="6" width="17.6666666666667" customWidth="1"/>
+    <col min="1" max="1" width="27.140625" customWidth="1"/>
+    <col min="2" max="2" width="10.42578125" customWidth="1"/>
+    <col min="3" max="3" width="11.42578125" customWidth="1"/>
+    <col min="4" max="4" width="11.7109375" customWidth="1"/>
+    <col min="5" max="5" width="14.5703125" customWidth="1"/>
+    <col min="6" max="6" width="17.7109375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6">
@@ -3448,22 +2811,20 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
-  <sheetPr/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:F4"/>
-  <sheetFormatPr defaultColWidth="8.88888888888889" defaultRowHeight="14.4" outlineLevelRow="3" outlineLevelCol="5"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="27.1111111111111" customWidth="1"/>
-    <col min="2" max="2" width="10.4444444444444" customWidth="1"/>
-    <col min="3" max="3" width="11.4444444444444" customWidth="1"/>
-    <col min="4" max="4" width="11.6666666666667" customWidth="1"/>
-    <col min="5" max="5" width="14.5555555555556" customWidth="1"/>
-    <col min="6" max="6" width="17.6666666666667" customWidth="1"/>
+    <col min="1" max="1" width="27.140625" customWidth="1"/>
+    <col min="2" max="2" width="10.42578125" customWidth="1"/>
+    <col min="3" max="3" width="11.42578125" customWidth="1"/>
+    <col min="4" max="4" width="11.7109375" customWidth="1"/>
+    <col min="5" max="5" width="14.5703125" customWidth="1"/>
+    <col min="6" max="6" width="17.7109375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6">
@@ -3544,17 +2905,15 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
-  <sheetPr/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:C3"/>
-  <sheetFormatPr defaultColWidth="8.88888888888889" defaultRowHeight="14.4" outlineLevelRow="2" outlineLevelCol="2"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="28.6666666666667" customWidth="1"/>
+    <col min="1" max="1" width="28.7109375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3">
@@ -3592,23 +2951,21 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
-  <sheetPr/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:G4"/>
-  <sheetFormatPr defaultColWidth="8.88888888888889" defaultRowHeight="14.4" outlineLevelRow="3" outlineLevelCol="6"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="19.7777777777778" customWidth="1"/>
-    <col min="2" max="2" width="8.11111111111111" customWidth="1"/>
-    <col min="3" max="3" width="8.55555555555556" customWidth="1"/>
-    <col min="4" max="4" width="17.8888888888889" customWidth="1"/>
-    <col min="5" max="5" width="12.6666666666667" customWidth="1"/>
-    <col min="6" max="6" width="14.5555555555556" customWidth="1"/>
-    <col min="7" max="7" width="17.6666666666667" customWidth="1"/>
+    <col min="1" max="1" width="19.7109375" customWidth="1"/>
+    <col min="2" max="2" width="8.140625" customWidth="1"/>
+    <col min="3" max="3" width="8.5703125" customWidth="1"/>
+    <col min="4" max="4" width="17.85546875" customWidth="1"/>
+    <col min="5" max="5" width="12.7109375" customWidth="1"/>
+    <col min="6" max="6" width="14.5703125" customWidth="1"/>
+    <col min="7" max="7" width="17.7109375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7">
@@ -3689,7 +3046,7 @@
         <v>232</v>
       </c>
       <c r="D4" s="3">
-        <v>2.32</v>
+        <v>2.3199999999999998</v>
       </c>
       <c r="E4" s="9" t="s">
         <v>77</v>
@@ -3699,23 +3056,21 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
-  <sheetPr/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:G4"/>
-  <sheetFormatPr defaultColWidth="8.88888888888889" defaultRowHeight="14.4" outlineLevelRow="3" outlineLevelCol="6"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="19.7777777777778" customWidth="1"/>
-    <col min="2" max="2" width="8.11111111111111" customWidth="1"/>
-    <col min="3" max="3" width="8.55555555555556" customWidth="1"/>
-    <col min="4" max="4" width="17.8888888888889" customWidth="1"/>
-    <col min="5" max="5" width="12.6666666666667" customWidth="1"/>
-    <col min="6" max="6" width="14.5555555555556" customWidth="1"/>
-    <col min="7" max="7" width="17.6666666666667" customWidth="1"/>
+    <col min="1" max="1" width="19.7109375" customWidth="1"/>
+    <col min="2" max="2" width="8.140625" customWidth="1"/>
+    <col min="3" max="3" width="8.5703125" customWidth="1"/>
+    <col min="4" max="4" width="17.85546875" customWidth="1"/>
+    <col min="5" max="5" width="12.7109375" customWidth="1"/>
+    <col min="6" max="6" width="14.5703125" customWidth="1"/>
+    <col min="7" max="7" width="17.7109375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7">
@@ -3796,7 +3151,7 @@
         <v>232</v>
       </c>
       <c r="D4" s="3">
-        <v>2.32</v>
+        <v>2.3199999999999998</v>
       </c>
       <c r="E4" s="9" t="s">
         <v>77</v>
@@ -3806,33 +3161,31 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
-  <sheetPr/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:S9"/>
-  <sheetFormatPr defaultColWidth="8.88888888888889" defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="39.6666666666667" customWidth="1"/>
-    <col min="2" max="2" width="10.1111111111111" customWidth="1"/>
-    <col min="3" max="3" width="39.6666666666667" customWidth="1"/>
+    <col min="1" max="1" width="39.7109375" customWidth="1"/>
+    <col min="2" max="2" width="10.140625" customWidth="1"/>
+    <col min="3" max="3" width="39.7109375" customWidth="1"/>
     <col min="4" max="4" width="11" customWidth="1"/>
-    <col min="5" max="5" width="13.2222222222222" customWidth="1"/>
-    <col min="6" max="6" width="8.88888888888889" customWidth="1"/>
-    <col min="7" max="7" width="17.8888888888889" customWidth="1"/>
-    <col min="8" max="8" width="19.5555555555556" customWidth="1"/>
-    <col min="9" max="9" width="23.7777777777778" customWidth="1"/>
-    <col min="10" max="10" width="12.6666666666667" customWidth="1"/>
-    <col min="11" max="11" width="11.8888888888889" customWidth="1"/>
-    <col min="12" max="12" width="17.4444444444444" customWidth="1"/>
-    <col min="13" max="14" width="39.6666666666667" customWidth="1"/>
-    <col min="15" max="15" width="25.7777777777778" customWidth="1"/>
-    <col min="16" max="17" width="16.5555555555556" customWidth="1"/>
-    <col min="18" max="18" width="11.5555555555556" customWidth="1"/>
-    <col min="19" max="19" width="14.8888888888889" customWidth="1"/>
+    <col min="5" max="5" width="13.28515625" customWidth="1"/>
+    <col min="6" max="6" width="8.85546875" customWidth="1"/>
+    <col min="7" max="7" width="17.85546875" customWidth="1"/>
+    <col min="8" max="8" width="19.5703125" customWidth="1"/>
+    <col min="9" max="9" width="23.7109375" customWidth="1"/>
+    <col min="10" max="10" width="12.7109375" customWidth="1"/>
+    <col min="11" max="11" width="11.85546875" customWidth="1"/>
+    <col min="12" max="12" width="17.42578125" customWidth="1"/>
+    <col min="13" max="14" width="39.7109375" customWidth="1"/>
+    <col min="15" max="15" width="25.7109375" customWidth="1"/>
+    <col min="16" max="17" width="16.5703125" customWidth="1"/>
+    <col min="18" max="18" width="11.5703125" customWidth="1"/>
+    <col min="19" max="19" width="14.85546875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:19">
@@ -4336,6 +3689,5 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <headerFooter/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Fixed Employee Creation Scenarios and Added Open Sale Order Amendment Scenario
Fixed Employee Creation Scenarios in Payroll and Added Open Sale Order Amendment Scenario
</commit_message>
<xml_diff>
--- a/testdata/ItemDetails.xlsx
+++ b/testdata/ItemDetails.xlsx
@@ -1,10 +1,10 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="4" lowestEdited="5" rupBuild="4505"/>
+  <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView xWindow="-15" yWindow="2355" windowWidth="15030" windowHeight="6540" firstSheet="7" activeTab="8"/>
+    <workbookView windowWidth="19200" windowHeight="6920" firstSheet="7" activeTab="10"/>
   </bookViews>
   <sheets>
     <sheet name="PR Details" sheetId="1" r:id="rId1"/>
@@ -20,8 +20,7 @@
     <sheet name="Open Sales" sheetId="11" r:id="rId11"/>
     <sheet name="SI Details" sheetId="12" r:id="rId12"/>
   </sheets>
-  <calcPr calcId="124519"/>
-  <oleSize ref="A1:G20"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -39,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="483" uniqueCount="176">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="521" uniqueCount="189">
   <si>
     <t>ITEM_NAME</t>
   </si>
@@ -414,6 +413,15 @@
     <t>HK-FG-CATALOG-DISSIMILAR-10001</t>
   </si>
   <si>
+    <t>HK-LOT-FIFO-LOT-10001(FG)</t>
+  </si>
+  <si>
+    <t>Price List</t>
+  </si>
+  <si>
+    <t>HK-FG-PRICELIST-DISSIMILAR UOM-10001</t>
+  </si>
+  <si>
     <t>CUST_ID</t>
   </si>
   <si>
@@ -514,6 +522,36 @@
   </si>
   <si>
     <t>OPSO1/00092/24-25</t>
+  </si>
+  <si>
+    <t>L0001</t>
+  </si>
+  <si>
+    <t>U1</t>
+  </si>
+  <si>
+    <t>C010</t>
+  </si>
+  <si>
+    <t>MAHESH TRADERS</t>
+  </si>
+  <si>
+    <t>OSOD-2425-00240</t>
+  </si>
+  <si>
+    <t>L30</t>
+  </si>
+  <si>
+    <t>U30</t>
+  </si>
+  <si>
+    <t>CUS0007</t>
+  </si>
+  <si>
+    <t>ARGOMM S.P.A -EXPORT</t>
+  </si>
+  <si>
+    <t>OSO30-2425-00005</t>
   </si>
   <si>
     <t>Customer_Name</t>
@@ -573,27 +611,20 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="11">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="xr9">
+  <numFmts count="4">
+    <numFmt numFmtId="176" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
+    <numFmt numFmtId="177" formatCode="_ &quot;₹&quot;* #,##0.00_ ;_ &quot;₹&quot;* \-#,##0.00_ ;_ &quot;₹&quot;* &quot;-&quot;??_ ;_ @_ "/>
+    <numFmt numFmtId="178" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
+    <numFmt numFmtId="179" formatCode="_ &quot;₹&quot;* #,##0_ ;_ &quot;₹&quot;* \-#,##0_ ;_ &quot;₹&quot;* &quot;-&quot;_ ;_ @_ "/>
+  </numFmts>
+  <fonts count="28">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <charset val="134"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="9"/>
-      <color rgb="FF000000"/>
-      <name val="Arial"/>
-      <charset val="134"/>
     </font>
     <font>
       <sz val="9"/>
@@ -645,8 +676,152 @@
       <name val="Times New Roman"/>
       <charset val="134"/>
     </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color rgb="FF0000FF"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color rgb="FF800080"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="18"/>
+      <color theme="3"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="11"/>
+      <color rgb="FF7F7F7F"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="15"/>
+      <color theme="3"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="13"/>
+      <color theme="3"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="3"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF3F3F76"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF3F3F3F"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFA7D00"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFA7D00"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF006100"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF9C0006"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF9C6500"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="0"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="5">
+  <fills count="35">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -655,7 +830,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.59999389629810485"/>
+        <fgColor theme="9" tint="0.599993896298105"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -671,8 +846,188 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFCC"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFCC99"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF2F2F2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFA5A5A5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC6EFCE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC7CE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFEB9C"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="3">
+  <borders count="10">
     <border>
       <left/>
       <right/>
@@ -696,55 +1051,285 @@
       <diagonal/>
     </border>
     <border>
-      <left style="medium">
-        <color rgb="FF000000"/>
+      <left style="thin">
+        <color rgb="FFB2B2B2"/>
       </left>
-      <right style="medium">
-        <color rgb="FF000000"/>
+      <right style="thin">
+        <color rgb="FFB2B2B2"/>
       </right>
-      <top style="medium">
-        <color rgb="FF000000"/>
+      <top style="thin">
+        <color rgb="FFB2B2B2"/>
       </top>
+      <bottom style="thin">
+        <color rgb="FFB2B2B2"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
       <bottom style="medium">
-        <color rgb="FF000000"/>
+        <color theme="4"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color theme="4" tint="0.499984740745262"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF7F7F7F"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF7F7F7F"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF7F7F7F"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF7F7F7F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF3F3F3F"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF3F3F3F"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF3F3F3F"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF3F3F3F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="double">
+        <color rgb="FF3F3F3F"/>
+      </left>
+      <right style="double">
+        <color rgb="FF3F3F3F"/>
+      </right>
+      <top style="double">
+        <color rgb="FF3F3F3F"/>
+      </top>
+      <bottom style="double">
+        <color rgb="FF3F3F3F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="double">
+        <color rgb="FFFF8001"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color theme="4"/>
+      </top>
+      <bottom style="double">
+        <color theme="4"/>
       </bottom>
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="2">
+  <cellStyleXfs count="50">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0">
+    <xf numFmtId="176" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="177" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="178" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="179" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="2" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="6" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="7" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="7" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="8" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="28">
+  <cellXfs count="29">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1">
@@ -754,7 +1339,7 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
@@ -763,7 +1348,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1">
@@ -772,190 +1357,121 @@
     <xf numFmtId="49" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="49" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="49" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="justify" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
-  <cellStyles count="2">
+  <cellStyles count="50">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Normal 2" xfId="1"/>
+    <cellStyle name="Comma" xfId="1" builtinId="3"/>
+    <cellStyle name="Currency" xfId="2" builtinId="4"/>
+    <cellStyle name="Percent" xfId="3" builtinId="5"/>
+    <cellStyle name="Comma [0]" xfId="4" builtinId="6"/>
+    <cellStyle name="Currency [0]" xfId="5" builtinId="7"/>
+    <cellStyle name="Hyperlink" xfId="6" builtinId="8"/>
+    <cellStyle name="Followed Hyperlink" xfId="7" builtinId="9"/>
+    <cellStyle name="Note" xfId="8" builtinId="10"/>
+    <cellStyle name="Warning Text" xfId="9" builtinId="11"/>
+    <cellStyle name="Title" xfId="10" builtinId="15"/>
+    <cellStyle name="CExplanatory Text" xfId="11" builtinId="53"/>
+    <cellStyle name="Heading 1" xfId="12" builtinId="16"/>
+    <cellStyle name="Heading 2" xfId="13" builtinId="17"/>
+    <cellStyle name="Heading 3" xfId="14" builtinId="18"/>
+    <cellStyle name="Heading 4" xfId="15" builtinId="19"/>
+    <cellStyle name="Input" xfId="16" builtinId="20"/>
+    <cellStyle name="Output" xfId="17" builtinId="21"/>
+    <cellStyle name="Calculation" xfId="18" builtinId="22"/>
+    <cellStyle name="Check Cell" xfId="19" builtinId="23"/>
+    <cellStyle name="Linked Cell" xfId="20" builtinId="24"/>
+    <cellStyle name="Total" xfId="21" builtinId="25"/>
+    <cellStyle name="Good" xfId="22" builtinId="26"/>
+    <cellStyle name="Bad" xfId="23" builtinId="27"/>
+    <cellStyle name="Neutral" xfId="24" builtinId="28"/>
+    <cellStyle name="Accent1" xfId="25" builtinId="29"/>
+    <cellStyle name="20% - Accent1" xfId="26" builtinId="30"/>
+    <cellStyle name="40% - Accent1" xfId="27" builtinId="31"/>
+    <cellStyle name="60% - Accent1" xfId="28" builtinId="32"/>
+    <cellStyle name="Accent2" xfId="29" builtinId="33"/>
+    <cellStyle name="20% - Accent2" xfId="30" builtinId="34"/>
+    <cellStyle name="40% - Accent2" xfId="31" builtinId="35"/>
+    <cellStyle name="60% - Accent2" xfId="32" builtinId="36"/>
+    <cellStyle name="Accent3" xfId="33" builtinId="37"/>
+    <cellStyle name="20% - Accent3" xfId="34" builtinId="38"/>
+    <cellStyle name="40% - Accent3" xfId="35" builtinId="39"/>
+    <cellStyle name="60% - Accent3" xfId="36" builtinId="40"/>
+    <cellStyle name="Accent4" xfId="37" builtinId="41"/>
+    <cellStyle name="20% - Accent4" xfId="38" builtinId="42"/>
+    <cellStyle name="40% - Accent4" xfId="39" builtinId="43"/>
+    <cellStyle name="60% - Accent4" xfId="40" builtinId="44"/>
+    <cellStyle name="Accent5" xfId="41" builtinId="45"/>
+    <cellStyle name="20% - Accent5" xfId="42" builtinId="46"/>
+    <cellStyle name="40% - Accent5" xfId="43" builtinId="47"/>
+    <cellStyle name="60% - Accent5" xfId="44" builtinId="48"/>
+    <cellStyle name="Accent6" xfId="45" builtinId="49"/>
+    <cellStyle name="20% - Accent6" xfId="46" builtinId="50"/>
+    <cellStyle name="40% - Accent6" xfId="47" builtinId="51"/>
+    <cellStyle name="60% - Accent6" xfId="48" builtinId="52"/>
+    <cellStyle name="Normal 2" xfId="49"/>
   </cellStyles>
   <dxfs count="17">
     <dxf>
       <fill>
         <patternFill patternType="solid">
-          <fgColor theme="4" tint="0.79995117038483843"/>
-          <bgColor theme="4" tint="0.79995117038483843"/>
-        </patternFill>
-      </fill>
-      <border>
-        <bottom style="thin">
-          <color theme="4" tint="0.39994506668294322"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor theme="4" tint="0.79995117038483843"/>
-          <bgColor theme="4" tint="0.79995117038483843"/>
-        </patternFill>
-      </fill>
-      <border>
-        <bottom style="thin">
-          <color theme="4" tint="0.39994506668294322"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="1"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="1"/>
-      </font>
-      <border>
-        <bottom style="thin">
-          <color theme="4" tint="0.39994506668294322"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <color theme="1"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <color theme="1"/>
-      </font>
-      <border>
-        <top style="thin">
-          <color theme="4"/>
-        </top>
-        <bottom style="thin">
-          <color theme="4"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor theme="4" tint="0.79995117038483843"/>
-          <bgColor theme="4" tint="0.79995117038483843"/>
+          <fgColor theme="4" tint="0.799981688894314"/>
+          <bgColor theme="4" tint="0.799981688894314"/>
         </patternFill>
       </fill>
     </dxf>
     <dxf>
       <fill>
         <patternFill patternType="solid">
-          <fgColor theme="4" tint="0.79995117038483843"/>
-          <bgColor theme="4" tint="0.79995117038483843"/>
+          <fgColor theme="4" tint="0.799981688894314"/>
+          <bgColor theme="4" tint="0.799981688894314"/>
         </patternFill>
       </fill>
     </dxf>
     <dxf>
       <font>
-        <b/>
-        <color theme="1"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor theme="4" tint="0.79995117038483843"/>
-          <bgColor theme="4" tint="0.79995117038483843"/>
-        </patternFill>
-      </fill>
-      <border>
-        <top style="thin">
-          <color theme="4" tint="0.39994506668294322"/>
-        </top>
-        <bottom style="thin">
-          <color theme="4" tint="0.39994506668294322"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <color theme="1"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor theme="4" tint="0.79995117038483843"/>
-          <bgColor theme="4" tint="0.79995117038483843"/>
-        </patternFill>
-      </fill>
-      <border>
-        <bottom style="thin">
-          <color theme="4" tint="0.39994506668294322"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor theme="4" tint="0.79995117038483843"/>
-          <bgColor theme="4" tint="0.79995117038483843"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor theme="4" tint="0.79995117038483843"/>
-          <bgColor theme="4" tint="0.79995117038483843"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
+        <b val="1"/>
         <color theme="1"/>
       </font>
     </dxf>
     <dxf>
       <font>
-        <b/>
+        <b val="1"/>
         <color theme="1"/>
       </font>
     </dxf>
     <dxf>
       <font>
-        <b/>
+        <b val="1"/>
         <color theme="1"/>
       </font>
       <border>
@@ -966,7 +1482,7 @@
     </dxf>
     <dxf>
       <font>
-        <b/>
+        <b val="1"/>
         <color theme="0"/>
       </font>
       <fill>
@@ -994,32 +1510,149 @@
           <color theme="4"/>
         </bottom>
         <horizontal style="thin">
-          <color theme="4" tint="0.39994506668294322"/>
+          <color theme="4" tint="0.399975585192419"/>
         </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor theme="4" tint="0.799981688894314"/>
+          <bgColor theme="4" tint="0.799981688894314"/>
+        </patternFill>
+      </fill>
+      <border>
+        <bottom style="thin">
+          <color theme="4" tint="0.399975585192419"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor theme="4" tint="0.799981688894314"/>
+          <bgColor theme="4" tint="0.799981688894314"/>
+        </patternFill>
+      </fill>
+      <border>
+        <bottom style="thin">
+          <color theme="4" tint="0.399975585192419"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="1"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="1"/>
+      </font>
+      <border>
+        <bottom style="thin">
+          <color theme="4" tint="0.399975585192419"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <color theme="1"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <color theme="1"/>
+      </font>
+      <border>
+        <top style="thin">
+          <color theme="4"/>
+        </top>
+        <bottom style="thin">
+          <color theme="4"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor theme="4" tint="0.799981688894314"/>
+          <bgColor theme="4" tint="0.799981688894314"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor theme="4" tint="0.799981688894314"/>
+          <bgColor theme="4" tint="0.799981688894314"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <color theme="1"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor theme="4" tint="0.799981688894314"/>
+          <bgColor theme="4" tint="0.799981688894314"/>
+        </patternFill>
+      </fill>
+      <border>
+        <top style="thin">
+          <color theme="4" tint="0.399975585192419"/>
+        </top>
+        <bottom style="thin">
+          <color theme="4" tint="0.399975585192419"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <color theme="1"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor theme="4" tint="0.799981688894314"/>
+          <bgColor theme="4" tint="0.799981688894314"/>
+        </patternFill>
+      </fill>
+      <border>
+        <bottom style="thin">
+          <color theme="4" tint="0.399975585192419"/>
+        </bottom>
       </border>
     </dxf>
   </dxfs>
   <tableStyles count="2" defaultTableStyle="TableStylePreset3_Accent1" defaultPivotStyle="PivotStylePreset2_Accent1">
-    <tableStyle name="TableStylePreset3_Accent1" pivot="0" count="7">
-      <tableStyleElement type="wholeTable" dxfId="16"/>
-      <tableStyleElement type="headerRow" dxfId="15"/>
-      <tableStyleElement type="totalRow" dxfId="14"/>
-      <tableStyleElement type="firstColumn" dxfId="13"/>
-      <tableStyleElement type="lastColumn" dxfId="12"/>
-      <tableStyleElement type="firstRowStripe" dxfId="11"/>
-      <tableStyleElement type="firstColumnStripe" dxfId="10"/>
+    <tableStyle name="TableStylePreset3_Accent1" pivot="0" count="7" xr9:uid="{59DB682C-5494-4EDE-A608-00C9E5F0F923}">
+      <tableStyleElement type="wholeTable" dxfId="6"/>
+      <tableStyleElement type="headerRow" dxfId="5"/>
+      <tableStyleElement type="totalRow" dxfId="4"/>
+      <tableStyleElement type="firstColumn" dxfId="3"/>
+      <tableStyleElement type="lastColumn" dxfId="2"/>
+      <tableStyleElement type="firstRowStripe" dxfId="1"/>
+      <tableStyleElement type="firstColumnStripe" dxfId="0"/>
     </tableStyle>
-    <tableStyle name="PivotStylePreset2_Accent1" table="0" count="10">
-      <tableStyleElement type="headerRow" dxfId="9"/>
-      <tableStyleElement type="totalRow" dxfId="8"/>
-      <tableStyleElement type="firstRowStripe" dxfId="7"/>
-      <tableStyleElement type="firstColumnStripe" dxfId="6"/>
-      <tableStyleElement type="firstSubtotalRow" dxfId="5"/>
-      <tableStyleElement type="secondSubtotalRow" dxfId="4"/>
-      <tableStyleElement type="firstRowSubheading" dxfId="3"/>
-      <tableStyleElement type="secondRowSubheading" dxfId="2"/>
-      <tableStyleElement type="pageFieldLabels" dxfId="1"/>
-      <tableStyleElement type="pageFieldValues" dxfId="0"/>
+    <tableStyle name="PivotStylePreset2_Accent1" table="0" count="10" xr9:uid="{267968C8-6FFD-4C36-ACC1-9EA1FD1885CA}">
+      <tableStyleElement type="headerRow" dxfId="16"/>
+      <tableStyleElement type="totalRow" dxfId="15"/>
+      <tableStyleElement type="firstRowStripe" dxfId="14"/>
+      <tableStyleElement type="firstColumnStripe" dxfId="13"/>
+      <tableStyleElement type="firstSubtotalRow" dxfId="12"/>
+      <tableStyleElement type="secondSubtotalRow" dxfId="11"/>
+      <tableStyleElement type="firstRowSubheading" dxfId="10"/>
+      <tableStyleElement type="secondRowSubheading" dxfId="9"/>
+      <tableStyleElement type="pageFieldLabels" dxfId="8"/>
+      <tableStyleElement type="pageFieldValues" dxfId="7"/>
     </tableStyle>
   </tableStyles>
   <extLst>
@@ -1282,983 +1915,1025 @@
     </a:fmtScheme>
   </a:themeElements>
   <a:objectDefaults/>
-  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
   <dimension ref="A1:J20"/>
-  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="8.70909090909091" defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="20.7109375" customWidth="1"/>
-    <col min="2" max="3" width="12.7109375" customWidth="1"/>
-    <col min="4" max="4" width="14.7109375" customWidth="1"/>
-    <col min="5" max="5" width="9.85546875" customWidth="1"/>
-    <col min="6" max="6" width="14.140625" customWidth="1"/>
-    <col min="7" max="7" width="14.85546875" customWidth="1"/>
-    <col min="8" max="8" width="22.28515625" customWidth="1"/>
-    <col min="9" max="9" width="14.42578125" customWidth="1"/>
+    <col min="1" max="1" width="20.7090909090909" customWidth="1"/>
+    <col min="2" max="3" width="12.7090909090909" customWidth="1"/>
+    <col min="4" max="4" width="14.7090909090909" customWidth="1"/>
+    <col min="5" max="5" width="9.85454545454546" customWidth="1"/>
+    <col min="6" max="6" width="14.1363636363636" customWidth="1"/>
+    <col min="7" max="7" width="14.8545454545455" customWidth="1"/>
+    <col min="8" max="8" width="22.2818181818182" customWidth="1"/>
+    <col min="9" max="9" width="14.4272727272727" customWidth="1"/>
     <col min="10" max="10" width="13" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:10">
-      <c r="A1" s="24" t="s">
+      <c r="A1" s="25" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="24" t="s">
+      <c r="B1" s="25" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="24" t="s">
+      <c r="C1" s="25" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="24" t="s">
+      <c r="D1" s="25" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="24" t="s">
+      <c r="E1" s="25" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="24" t="s">
+      <c r="F1" s="25" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="24" t="s">
+      <c r="G1" s="25" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="24" t="s">
+      <c r="H1" s="25" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="24" t="s">
+      <c r="I1" s="25" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="24" t="s">
+      <c r="J1" s="25" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="2" spans="1:10" s="23" customFormat="1" ht="22.5">
-      <c r="A2" s="25" t="s">
+    <row r="2" s="24" customFormat="1" ht="21" spans="1:10">
+      <c r="A2" s="26" t="s">
         <v>10</v>
       </c>
-      <c r="B2" s="26" t="s">
+      <c r="B2" s="27" t="s">
         <v>11</v>
       </c>
-      <c r="C2" s="26" t="s">
+      <c r="C2" s="27" t="s">
         <v>12</v>
       </c>
-      <c r="D2" s="25" t="s">
+      <c r="D2" s="26" t="s">
         <v>13</v>
       </c>
-      <c r="E2" s="25">
+      <c r="E2" s="26">
         <v>1</v>
       </c>
-      <c r="F2" s="25" t="s">
+      <c r="F2" s="26" t="s">
         <v>14</v>
       </c>
-      <c r="G2" s="25">
+      <c r="G2" s="26">
         <v>1010301033</v>
       </c>
-      <c r="H2" s="25" t="s">
+      <c r="H2" s="26" t="s">
         <v>15</v>
       </c>
-      <c r="I2" s="25" t="s">
+      <c r="I2" s="26" t="s">
         <v>16</v>
       </c>
-      <c r="J2" s="25" t="s">
+      <c r="J2" s="26" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="3" spans="1:10" ht="15" customHeight="1">
-      <c r="A3" s="25" t="s">
+    <row r="3" ht="15" customHeight="1" spans="1:10">
+      <c r="A3" s="26" t="s">
         <v>18</v>
       </c>
-      <c r="B3" s="26" t="s">
+      <c r="B3" s="27" t="s">
         <v>11</v>
       </c>
-      <c r="C3" s="26" t="s">
+      <c r="C3" s="27" t="s">
         <v>12</v>
       </c>
-      <c r="D3" s="25" t="s">
+      <c r="D3" s="26" t="s">
         <v>19</v>
       </c>
-      <c r="E3" s="25">
+      <c r="E3" s="26">
         <v>6</v>
       </c>
-      <c r="F3" s="26" t="s">
+      <c r="F3" s="27" t="s">
         <v>20</v>
       </c>
-      <c r="G3" s="25">
+      <c r="G3" s="26">
         <v>1010301033</v>
       </c>
-      <c r="H3" s="25" t="s">
+      <c r="H3" s="26" t="s">
         <v>15</v>
       </c>
-      <c r="I3" s="25" t="s">
+      <c r="I3" s="26" t="s">
         <v>16</v>
       </c>
-      <c r="J3" s="25" t="s">
+      <c r="J3" s="26" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="4" spans="1:10" ht="22.5">
-      <c r="A4" s="25" t="s">
+    <row r="4" spans="1:10">
+      <c r="A4" s="26" t="s">
         <v>21</v>
       </c>
-      <c r="B4" s="26" t="s">
+      <c r="B4" s="27" t="s">
         <v>22</v>
       </c>
-      <c r="C4" s="26" t="s">
+      <c r="C4" s="27" t="s">
         <v>22</v>
       </c>
-      <c r="D4" s="25" t="s">
+      <c r="D4" s="26" t="s">
         <v>23</v>
       </c>
-      <c r="E4" s="25">
+      <c r="E4" s="26">
         <v>1</v>
       </c>
-      <c r="F4" s="26" t="s">
+      <c r="F4" s="27" t="s">
         <v>14</v>
       </c>
-      <c r="G4" s="25">
+      <c r="G4" s="26">
         <v>5010101060</v>
       </c>
-      <c r="H4" s="25" t="s">
+      <c r="H4" s="26" t="s">
         <v>24</v>
       </c>
-      <c r="I4" s="25" t="s">
+      <c r="I4" s="26" t="s">
         <v>16</v>
       </c>
-      <c r="J4" s="25" t="s">
+      <c r="J4" s="26" t="s">
         <v>17</v>
       </c>
     </row>
     <row r="5" spans="1:10">
-      <c r="A5" s="27"/>
-      <c r="B5" s="27"/>
-      <c r="C5" s="27"/>
-      <c r="D5" s="27"/>
-      <c r="E5" s="27"/>
-      <c r="F5" s="27"/>
-      <c r="G5" s="27"/>
-      <c r="H5" s="27"/>
-      <c r="I5" s="27"/>
-      <c r="J5" s="27"/>
+      <c r="A5" s="28"/>
+      <c r="B5" s="28"/>
+      <c r="C5" s="28"/>
+      <c r="D5" s="28"/>
+      <c r="E5" s="28"/>
+      <c r="F5" s="28"/>
+      <c r="G5" s="28"/>
+      <c r="H5" s="28"/>
+      <c r="I5" s="28"/>
+      <c r="J5" s="28"/>
     </row>
     <row r="6" spans="1:10">
-      <c r="A6" s="27"/>
-      <c r="B6" s="27"/>
-      <c r="C6" s="27"/>
-      <c r="D6" s="27"/>
-      <c r="E6" s="27"/>
-      <c r="F6" s="27"/>
-      <c r="G6" s="27"/>
-      <c r="H6" s="27"/>
-      <c r="I6" s="27"/>
-      <c r="J6" s="27"/>
+      <c r="A6" s="28"/>
+      <c r="B6" s="28"/>
+      <c r="C6" s="28"/>
+      <c r="D6" s="28"/>
+      <c r="E6" s="28"/>
+      <c r="F6" s="28"/>
+      <c r="G6" s="28"/>
+      <c r="H6" s="28"/>
+      <c r="I6" s="28"/>
+      <c r="J6" s="28"/>
     </row>
     <row r="7" spans="1:10">
-      <c r="A7" s="27"/>
-      <c r="B7" s="27"/>
-      <c r="C7" s="27"/>
-      <c r="D7" s="27"/>
-      <c r="E7" s="27"/>
-      <c r="F7" s="27"/>
-      <c r="G7" s="27"/>
-      <c r="H7" s="27"/>
-      <c r="I7" s="27"/>
-      <c r="J7" s="27"/>
+      <c r="A7" s="28"/>
+      <c r="B7" s="28"/>
+      <c r="C7" s="28"/>
+      <c r="D7" s="28"/>
+      <c r="E7" s="28"/>
+      <c r="F7" s="28"/>
+      <c r="G7" s="28"/>
+      <c r="H7" s="28"/>
+      <c r="I7" s="28"/>
+      <c r="J7" s="28"/>
     </row>
     <row r="8" spans="1:10">
-      <c r="A8" s="27"/>
-      <c r="B8" s="27"/>
-      <c r="C8" s="27"/>
-      <c r="D8" s="27"/>
-      <c r="E8" s="27"/>
-      <c r="F8" s="27"/>
-      <c r="G8" s="27"/>
-      <c r="H8" s="27"/>
-      <c r="I8" s="27"/>
-      <c r="J8" s="27"/>
+      <c r="A8" s="28"/>
+      <c r="B8" s="28"/>
+      <c r="C8" s="28"/>
+      <c r="D8" s="28"/>
+      <c r="E8" s="28"/>
+      <c r="F8" s="28"/>
+      <c r="G8" s="28"/>
+      <c r="H8" s="28"/>
+      <c r="I8" s="28"/>
+      <c r="J8" s="28"/>
     </row>
     <row r="9" spans="1:10">
-      <c r="A9" s="27"/>
-      <c r="B9" s="27"/>
-      <c r="C9" s="27"/>
-      <c r="D9" s="27"/>
-      <c r="E9" s="27"/>
-      <c r="F9" s="27"/>
-      <c r="G9" s="27"/>
-      <c r="H9" s="27"/>
-      <c r="I9" s="27"/>
-      <c r="J9" s="27"/>
+      <c r="A9" s="28"/>
+      <c r="B9" s="28"/>
+      <c r="C9" s="28"/>
+      <c r="D9" s="28"/>
+      <c r="E9" s="28"/>
+      <c r="F9" s="28"/>
+      <c r="G9" s="28"/>
+      <c r="H9" s="28"/>
+      <c r="I9" s="28"/>
+      <c r="J9" s="28"/>
     </row>
     <row r="10" spans="1:10">
-      <c r="A10" s="27"/>
-      <c r="B10" s="27"/>
-      <c r="C10" s="27"/>
-      <c r="D10" s="27"/>
-      <c r="E10" s="27"/>
-      <c r="F10" s="27"/>
-      <c r="G10" s="27"/>
-      <c r="H10" s="27"/>
-      <c r="I10" s="27"/>
-      <c r="J10" s="27"/>
+      <c r="A10" s="28"/>
+      <c r="B10" s="28"/>
+      <c r="C10" s="28"/>
+      <c r="D10" s="28"/>
+      <c r="E10" s="28"/>
+      <c r="F10" s="28"/>
+      <c r="G10" s="28"/>
+      <c r="H10" s="28"/>
+      <c r="I10" s="28"/>
+      <c r="J10" s="28"/>
     </row>
     <row r="11" spans="1:10">
-      <c r="A11" s="27"/>
-      <c r="B11" s="27"/>
-      <c r="C11" s="27"/>
-      <c r="D11" s="27"/>
-      <c r="E11" s="27"/>
-      <c r="F11" s="27"/>
-      <c r="G11" s="27"/>
-      <c r="H11" s="27"/>
-      <c r="I11" s="27"/>
-      <c r="J11" s="27"/>
+      <c r="A11" s="28"/>
+      <c r="B11" s="28"/>
+      <c r="C11" s="28"/>
+      <c r="D11" s="28"/>
+      <c r="E11" s="28"/>
+      <c r="F11" s="28"/>
+      <c r="G11" s="28"/>
+      <c r="H11" s="28"/>
+      <c r="I11" s="28"/>
+      <c r="J11" s="28"/>
     </row>
     <row r="12" spans="1:10">
-      <c r="A12" s="27"/>
-      <c r="B12" s="27"/>
-      <c r="C12" s="27"/>
-      <c r="D12" s="27"/>
-      <c r="E12" s="27"/>
-      <c r="F12" s="27"/>
-      <c r="G12" s="27"/>
-      <c r="H12" s="27"/>
-      <c r="I12" s="27"/>
-      <c r="J12" s="27"/>
+      <c r="A12" s="28"/>
+      <c r="B12" s="28"/>
+      <c r="C12" s="28"/>
+      <c r="D12" s="28"/>
+      <c r="E12" s="28"/>
+      <c r="F12" s="28"/>
+      <c r="G12" s="28"/>
+      <c r="H12" s="28"/>
+      <c r="I12" s="28"/>
+      <c r="J12" s="28"/>
     </row>
     <row r="13" spans="1:10">
-      <c r="A13" s="27"/>
-      <c r="B13" s="27"/>
-      <c r="C13" s="27"/>
-      <c r="D13" s="27"/>
-      <c r="E13" s="27"/>
-      <c r="F13" s="27"/>
-      <c r="G13" s="27"/>
-      <c r="H13" s="27"/>
-      <c r="I13" s="27"/>
-      <c r="J13" s="27"/>
+      <c r="A13" s="28"/>
+      <c r="B13" s="28"/>
+      <c r="C13" s="28"/>
+      <c r="D13" s="28"/>
+      <c r="E13" s="28"/>
+      <c r="F13" s="28"/>
+      <c r="G13" s="28"/>
+      <c r="H13" s="28"/>
+      <c r="I13" s="28"/>
+      <c r="J13" s="28"/>
     </row>
     <row r="14" spans="1:10">
-      <c r="A14" s="27"/>
-      <c r="B14" s="27"/>
-      <c r="C14" s="27"/>
-      <c r="D14" s="27"/>
-      <c r="E14" s="27"/>
-      <c r="F14" s="27"/>
-      <c r="G14" s="27"/>
-      <c r="H14" s="27"/>
-      <c r="I14" s="27"/>
-      <c r="J14" s="27"/>
+      <c r="A14" s="28"/>
+      <c r="B14" s="28"/>
+      <c r="C14" s="28"/>
+      <c r="D14" s="28"/>
+      <c r="E14" s="28"/>
+      <c r="F14" s="28"/>
+      <c r="G14" s="28"/>
+      <c r="H14" s="28"/>
+      <c r="I14" s="28"/>
+      <c r="J14" s="28"/>
     </row>
     <row r="15" spans="1:10">
-      <c r="A15" s="27"/>
-      <c r="B15" s="27"/>
-      <c r="C15" s="27"/>
-      <c r="D15" s="27"/>
-      <c r="E15" s="27"/>
-      <c r="F15" s="27"/>
-      <c r="G15" s="27"/>
-      <c r="H15" s="27"/>
-      <c r="I15" s="27"/>
-      <c r="J15" s="27"/>
+      <c r="A15" s="28"/>
+      <c r="B15" s="28"/>
+      <c r="C15" s="28"/>
+      <c r="D15" s="28"/>
+      <c r="E15" s="28"/>
+      <c r="F15" s="28"/>
+      <c r="G15" s="28"/>
+      <c r="H15" s="28"/>
+      <c r="I15" s="28"/>
+      <c r="J15" s="28"/>
     </row>
     <row r="16" spans="1:10">
-      <c r="A16" s="27"/>
-      <c r="B16" s="27"/>
-      <c r="C16" s="27"/>
-      <c r="D16" s="27"/>
-      <c r="E16" s="27"/>
-      <c r="F16" s="27"/>
-      <c r="G16" s="27"/>
-      <c r="H16" s="27"/>
-      <c r="I16" s="27"/>
-      <c r="J16" s="27"/>
+      <c r="A16" s="28"/>
+      <c r="B16" s="28"/>
+      <c r="C16" s="28"/>
+      <c r="D16" s="28"/>
+      <c r="E16" s="28"/>
+      <c r="F16" s="28"/>
+      <c r="G16" s="28"/>
+      <c r="H16" s="28"/>
+      <c r="I16" s="28"/>
+      <c r="J16" s="28"/>
     </row>
     <row r="17" spans="1:10">
-      <c r="A17" s="27"/>
-      <c r="B17" s="27"/>
-      <c r="C17" s="27"/>
-      <c r="D17" s="27"/>
-      <c r="E17" s="27"/>
-      <c r="F17" s="27"/>
-      <c r="G17" s="27"/>
-      <c r="H17" s="27"/>
-      <c r="I17" s="27"/>
-      <c r="J17" s="27"/>
+      <c r="A17" s="28"/>
+      <c r="B17" s="28"/>
+      <c r="C17" s="28"/>
+      <c r="D17" s="28"/>
+      <c r="E17" s="28"/>
+      <c r="F17" s="28"/>
+      <c r="G17" s="28"/>
+      <c r="H17" s="28"/>
+      <c r="I17" s="28"/>
+      <c r="J17" s="28"/>
     </row>
     <row r="18" spans="1:10">
-      <c r="A18" s="27"/>
-      <c r="B18" s="27"/>
-      <c r="C18" s="27"/>
-      <c r="D18" s="27"/>
-      <c r="E18" s="27"/>
-      <c r="F18" s="27"/>
-      <c r="G18" s="27"/>
-      <c r="H18" s="27"/>
-      <c r="I18" s="27"/>
-      <c r="J18" s="27"/>
+      <c r="A18" s="28"/>
+      <c r="B18" s="28"/>
+      <c r="C18" s="28"/>
+      <c r="D18" s="28"/>
+      <c r="E18" s="28"/>
+      <c r="F18" s="28"/>
+      <c r="G18" s="28"/>
+      <c r="H18" s="28"/>
+      <c r="I18" s="28"/>
+      <c r="J18" s="28"/>
     </row>
     <row r="19" spans="1:10">
-      <c r="A19" s="27"/>
-      <c r="B19" s="27"/>
-      <c r="C19" s="27"/>
-      <c r="D19" s="27"/>
-      <c r="E19" s="27"/>
-      <c r="F19" s="27"/>
-      <c r="G19" s="27"/>
-      <c r="H19" s="27"/>
-      <c r="I19" s="27"/>
-      <c r="J19" s="27"/>
+      <c r="A19" s="28"/>
+      <c r="B19" s="28"/>
+      <c r="C19" s="28"/>
+      <c r="D19" s="28"/>
+      <c r="E19" s="28"/>
+      <c r="F19" s="28"/>
+      <c r="G19" s="28"/>
+      <c r="H19" s="28"/>
+      <c r="I19" s="28"/>
+      <c r="J19" s="28"/>
     </row>
     <row r="20" spans="1:10">
-      <c r="A20" s="27"/>
-      <c r="B20" s="27"/>
-      <c r="C20" s="27"/>
-      <c r="D20" s="27"/>
-      <c r="E20" s="27"/>
-      <c r="F20" s="27"/>
-      <c r="G20" s="27"/>
-      <c r="H20" s="27"/>
-      <c r="I20" s="27"/>
-      <c r="J20" s="27"/>
+      <c r="A20" s="28"/>
+      <c r="B20" s="28"/>
+      <c r="C20" s="28"/>
+      <c r="D20" s="28"/>
+      <c r="E20" s="28"/>
+      <c r="F20" s="28"/>
+      <c r="G20" s="28"/>
+      <c r="H20" s="28"/>
+      <c r="I20" s="28"/>
+      <c r="J20" s="28"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
   <dimension ref="A1:K3"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="8.85454545454546" defaultRowHeight="14.5" outlineLevelRow="2"/>
   <cols>
     <col min="1" max="1" width="9" customWidth="1"/>
-    <col min="2" max="2" width="25.7109375" customWidth="1"/>
-    <col min="3" max="3" width="12.42578125" customWidth="1"/>
-    <col min="4" max="4" width="16.28515625" customWidth="1"/>
-    <col min="5" max="5" width="20.28515625" customWidth="1"/>
-    <col min="6" max="6" width="25.7109375" customWidth="1"/>
-    <col min="7" max="7" width="12.28515625" customWidth="1"/>
-    <col min="8" max="8" width="14.5703125" customWidth="1"/>
-    <col min="9" max="9" width="28.5703125" customWidth="1"/>
+    <col min="2" max="2" width="25.7090909090909" customWidth="1"/>
+    <col min="3" max="3" width="12.4272727272727" customWidth="1"/>
+    <col min="4" max="4" width="16.2818181818182" customWidth="1"/>
+    <col min="5" max="5" width="20.2818181818182" customWidth="1"/>
+    <col min="6" max="6" width="25.7090909090909" customWidth="1"/>
+    <col min="7" max="7" width="12.2818181818182" customWidth="1"/>
+    <col min="8" max="8" width="14.5727272727273" customWidth="1"/>
+    <col min="9" max="9" width="28.5727272727273" customWidth="1"/>
     <col min="10" max="10" width="23" customWidth="1"/>
-    <col min="11" max="11" width="14.7109375" customWidth="1"/>
+    <col min="11" max="11" width="14.7090909090909" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:11">
-      <c r="A1" s="9" t="s">
-        <v>124</v>
-      </c>
-      <c r="B1" s="9" t="s">
-        <v>125</v>
-      </c>
-      <c r="C1" s="9" t="s">
-        <v>126</v>
-      </c>
-      <c r="D1" s="9" t="s">
+      <c r="A1" s="10" t="s">
         <v>127</v>
       </c>
-      <c r="E1" s="9" t="s">
+      <c r="B1" s="10" t="s">
         <v>128</v>
       </c>
-      <c r="F1" s="10" t="s">
+      <c r="C1" s="10" t="s">
         <v>129</v>
       </c>
-      <c r="G1" s="10" t="s">
+      <c r="D1" s="10" t="s">
         <v>130</v>
       </c>
-      <c r="H1" s="10" t="s">
+      <c r="E1" s="10" t="s">
         <v>131</v>
       </c>
-      <c r="I1" s="10" t="s">
+      <c r="F1" s="11" t="s">
         <v>132</v>
       </c>
-      <c r="J1" s="10" t="s">
+      <c r="G1" s="11" t="s">
         <v>133</v>
       </c>
-      <c r="K1" s="10" t="s">
+      <c r="H1" s="11" t="s">
         <v>134</v>
       </c>
+      <c r="I1" s="11" t="s">
+        <v>135</v>
+      </c>
+      <c r="J1" s="11" t="s">
+        <v>136</v>
+      </c>
+      <c r="K1" s="11" t="s">
+        <v>137</v>
+      </c>
     </row>
     <row r="2" spans="1:11">
-      <c r="A2" s="9" t="s">
-        <v>135</v>
-      </c>
-      <c r="B2" s="9" t="s">
-        <v>136</v>
-      </c>
-      <c r="C2" s="9" t="s">
-        <v>137</v>
-      </c>
-      <c r="D2" s="9" t="s">
+      <c r="A2" s="10" t="s">
         <v>138</v>
       </c>
-      <c r="E2" s="9" t="s">
+      <c r="B2" s="10" t="s">
         <v>139</v>
       </c>
+      <c r="C2" s="10" t="s">
+        <v>140</v>
+      </c>
+      <c r="D2" s="10" t="s">
+        <v>141</v>
+      </c>
+      <c r="E2" s="10" t="s">
+        <v>142</v>
+      </c>
       <c r="F2" s="3" t="s">
-        <v>136</v>
+        <v>139</v>
       </c>
       <c r="G2" s="3" t="s">
+        <v>143</v>
+      </c>
+      <c r="H2" s="3" t="s">
+        <v>144</v>
+      </c>
+      <c r="I2" s="3" t="s">
+        <v>145</v>
+      </c>
+      <c r="J2" s="3" t="s">
+        <v>146</v>
+      </c>
+      <c r="K2" s="3" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11">
+      <c r="A3" s="12" t="s">
+        <v>148</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>149</v>
+      </c>
+      <c r="C3" s="10" t="s">
         <v>140</v>
       </c>
-      <c r="H2" s="3" t="s">
-        <v>141</v>
-      </c>
-      <c r="I2" s="3" t="s">
-        <v>142</v>
-      </c>
-      <c r="J2" s="3" t="s">
-        <v>143</v>
-      </c>
-      <c r="K2" s="3" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="3" spans="1:11">
-      <c r="A3" s="11" t="s">
-        <v>145</v>
-      </c>
-      <c r="B3" s="3" t="s">
+      <c r="D3" s="3" t="s">
+        <v>150</v>
+      </c>
+      <c r="E3" s="3" t="s">
+        <v>150</v>
+      </c>
+      <c r="F3" s="3" t="s">
+        <v>149</v>
+      </c>
+      <c r="G3" s="3" t="s">
+        <v>151</v>
+      </c>
+      <c r="H3" s="3" t="s">
+        <v>151</v>
+      </c>
+      <c r="I3" s="3" t="s">
+        <v>152</v>
+      </c>
+      <c r="J3" s="3" t="s">
         <v>146</v>
       </c>
-      <c r="C3" s="9" t="s">
-        <v>137</v>
-      </c>
-      <c r="D3" s="3" t="s">
+      <c r="K3" s="3" t="s">
         <v>147</v>
-      </c>
-      <c r="E3" s="3" t="s">
-        <v>147</v>
-      </c>
-      <c r="F3" s="3" t="s">
-        <v>146</v>
-      </c>
-      <c r="G3" s="3" t="s">
-        <v>148</v>
-      </c>
-      <c r="H3" s="3" t="s">
-        <v>148</v>
-      </c>
-      <c r="I3" s="3" t="s">
-        <v>149</v>
-      </c>
-      <c r="J3" s="3" t="s">
-        <v>143</v>
-      </c>
-      <c r="K3" s="3" t="s">
-        <v>144</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E2"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
+  <dimension ref="A1:E4"/>
+  <sheetFormatPr defaultColWidth="8.85454545454546" defaultRowHeight="14.5" outlineLevelRow="3" outlineLevelCol="4"/>
   <cols>
-    <col min="1" max="1" width="13.5703125" customWidth="1"/>
+    <col min="1" max="1" width="13.5727272727273" customWidth="1"/>
     <col min="2" max="2" width="6" customWidth="1"/>
-    <col min="3" max="3" width="14.42578125" customWidth="1"/>
-    <col min="4" max="4" width="18.140625" customWidth="1"/>
-    <col min="5" max="5" width="19.5703125" customWidth="1"/>
+    <col min="3" max="3" width="14.4272727272727" customWidth="1"/>
+    <col min="4" max="4" width="18.1363636363636" customWidth="1"/>
+    <col min="5" max="5" width="19.5727272727273" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5">
       <c r="A1" s="6" t="s">
-        <v>150</v>
-      </c>
-      <c r="B1" t="s">
-        <v>151</v>
-      </c>
-      <c r="C1" t="s">
-        <v>152</v>
-      </c>
-      <c r="D1" t="s">
         <v>153</v>
       </c>
-      <c r="E1" t="s">
+      <c r="B1" s="7" t="s">
         <v>154</v>
       </c>
-    </row>
-    <row r="2" spans="1:5" ht="30">
+      <c r="C1" s="7" t="s">
+        <v>155</v>
+      </c>
+      <c r="D1" s="7" t="s">
+        <v>156</v>
+      </c>
+      <c r="E1" s="7" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5">
       <c r="A2" s="6" t="s">
-        <v>155</v>
+        <v>158</v>
       </c>
       <c r="B2" s="6" t="s">
-        <v>156</v>
-      </c>
-      <c r="C2" s="7" t="s">
-        <v>135</v>
-      </c>
-      <c r="D2" s="8" t="s">
-        <v>136</v>
+        <v>159</v>
+      </c>
+      <c r="C2" s="8" t="s">
+        <v>138</v>
+      </c>
+      <c r="D2" s="9" t="s">
+        <v>139</v>
       </c>
       <c r="E2" s="6" t="s">
-        <v>157</v>
+        <v>160</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5">
+      <c r="A3" s="7" t="s">
+        <v>161</v>
+      </c>
+      <c r="B3" s="7" t="s">
+        <v>162</v>
+      </c>
+      <c r="C3" s="7" t="s">
+        <v>163</v>
+      </c>
+      <c r="D3" s="7" t="s">
+        <v>164</v>
+      </c>
+      <c r="E3" s="7" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5">
+      <c r="A4" s="7" t="s">
+        <v>166</v>
+      </c>
+      <c r="B4" s="7" t="s">
+        <v>167</v>
+      </c>
+      <c r="C4" s="7" t="s">
+        <v>168</v>
+      </c>
+      <c r="D4" s="7" t="s">
+        <v>169</v>
+      </c>
+      <c r="E4" s="7" t="s">
+        <v>170</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
   <dimension ref="A1:G8"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="8.85454545454546" defaultRowHeight="14.5" outlineLevelRow="7" outlineLevelCol="6"/>
   <cols>
-    <col min="1" max="1" width="25.7109375" customWidth="1"/>
-    <col min="2" max="2" width="8.85546875" customWidth="1"/>
-    <col min="3" max="3" width="12.28515625" customWidth="1"/>
-    <col min="4" max="4" width="7.140625" customWidth="1"/>
-    <col min="5" max="5" width="5.28515625" customWidth="1"/>
-    <col min="6" max="6" width="17.42578125" customWidth="1"/>
-    <col min="7" max="7" width="12.42578125" customWidth="1"/>
+    <col min="1" max="1" width="25.7090909090909" customWidth="1"/>
+    <col min="2" max="2" width="8.85454545454546" customWidth="1"/>
+    <col min="3" max="3" width="12.2818181818182" customWidth="1"/>
+    <col min="4" max="4" width="7.13636363636364" customWidth="1"/>
+    <col min="5" max="5" width="5.28181818181818" customWidth="1"/>
+    <col min="6" max="6" width="17.4272727272727" customWidth="1"/>
+    <col min="7" max="7" width="12.4272727272727" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7">
       <c r="A1" s="1" t="s">
-        <v>158</v>
+        <v>171</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>159</v>
+        <v>172</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>160</v>
+        <v>173</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>161</v>
+        <v>174</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>162</v>
+        <v>175</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>163</v>
+        <v>176</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>164</v>
+        <v>177</v>
       </c>
     </row>
     <row r="2" spans="1:7">
       <c r="A2" s="3" t="s">
-        <v>165</v>
+        <v>178</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>166</v>
+        <v>179</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>167</v>
+        <v>180</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>155</v>
+        <v>158</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>156</v>
+        <v>159</v>
       </c>
       <c r="F2" s="3" t="s">
-        <v>168</v>
+        <v>181</v>
       </c>
       <c r="G2" s="3" t="s">
-        <v>169</v>
+        <v>182</v>
       </c>
     </row>
     <row r="3" spans="1:7">
       <c r="A3" s="3" t="s">
-        <v>146</v>
+        <v>149</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>170</v>
+        <v>183</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>167</v>
+        <v>180</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>155</v>
+        <v>158</v>
       </c>
       <c r="E3" s="4" t="s">
-        <v>156</v>
+        <v>159</v>
       </c>
       <c r="F3" s="3" t="s">
-        <v>147</v>
+        <v>150</v>
       </c>
       <c r="G3" s="3" t="s">
-        <v>137</v>
+        <v>140</v>
       </c>
     </row>
     <row r="4" spans="1:7">
       <c r="A4" s="3" t="s">
-        <v>171</v>
+        <v>184</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>166</v>
+        <v>179</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>167</v>
+        <v>180</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>155</v>
+        <v>158</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>156</v>
+        <v>159</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>168</v>
+        <v>181</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>169</v>
+        <v>182</v>
       </c>
     </row>
     <row r="5" spans="1:7">
       <c r="A5" s="3" t="s">
-        <v>136</v>
+        <v>139</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>166</v>
+        <v>179</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>167</v>
+        <v>180</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>155</v>
+        <v>158</v>
       </c>
       <c r="E5" s="4" t="s">
-        <v>156</v>
+        <v>159</v>
       </c>
       <c r="F5" s="5" t="s">
-        <v>138</v>
+        <v>141</v>
       </c>
       <c r="G5" s="3" t="s">
-        <v>137</v>
+        <v>140</v>
       </c>
     </row>
     <row r="6" spans="1:7">
       <c r="A6" s="3" t="s">
-        <v>172</v>
+        <v>185</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>166</v>
+        <v>179</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>167</v>
+        <v>180</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>155</v>
+        <v>158</v>
       </c>
       <c r="E6" s="4" t="s">
-        <v>156</v>
+        <v>159</v>
       </c>
       <c r="F6" s="3" t="s">
-        <v>138</v>
+        <v>141</v>
       </c>
       <c r="G6" s="3" t="s">
-        <v>169</v>
+        <v>182</v>
       </c>
     </row>
     <row r="7" spans="1:7">
       <c r="A7" s="3" t="s">
-        <v>173</v>
+        <v>186</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>166</v>
+        <v>179</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>167</v>
+        <v>180</v>
       </c>
       <c r="D7" s="4" t="s">
-        <v>155</v>
+        <v>158</v>
       </c>
       <c r="E7" s="4" t="s">
-        <v>156</v>
+        <v>159</v>
       </c>
       <c r="F7" s="3" t="s">
-        <v>138</v>
+        <v>141</v>
       </c>
       <c r="G7" s="3" t="s">
-        <v>169</v>
+        <v>182</v>
       </c>
     </row>
     <row r="8" spans="1:7">
       <c r="A8" s="3" t="s">
-        <v>174</v>
+        <v>187</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>166</v>
+        <v>179</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>167</v>
+        <v>180</v>
       </c>
       <c r="D8" s="4" t="s">
-        <v>155</v>
+        <v>158</v>
       </c>
       <c r="E8" s="4" t="s">
-        <v>156</v>
+        <v>159</v>
       </c>
       <c r="F8" s="3" t="s">
-        <v>175</v>
+        <v>188</v>
       </c>
       <c r="G8" s="3" t="s">
-        <v>169</v>
+        <v>182</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
   <dimension ref="A1:T10"/>
-  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="8.70909090909091" defaultRowHeight="14.5"/>
   <cols>
     <col min="1" max="1" width="30" customWidth="1"/>
-    <col min="2" max="2" width="36.42578125" customWidth="1"/>
+    <col min="2" max="2" width="36.4272727272727" customWidth="1"/>
     <col min="3" max="3" width="6" customWidth="1"/>
-    <col min="4" max="4" width="13.7109375" customWidth="1"/>
-    <col min="5" max="5" width="5.28515625" customWidth="1"/>
-    <col min="6" max="6" width="17.28515625" customWidth="1"/>
-    <col min="7" max="7" width="30.28515625" customWidth="1"/>
-    <col min="8" max="8" width="26.85546875" customWidth="1"/>
-    <col min="9" max="9" width="17.28515625" customWidth="1"/>
-    <col min="10" max="10" width="13.28515625" customWidth="1"/>
-    <col min="11" max="11" width="22.7109375" customWidth="1"/>
-    <col min="12" max="12" width="12.7109375" customWidth="1"/>
-    <col min="13" max="13" width="29.5703125" customWidth="1"/>
-    <col min="14" max="14" width="18.28515625" customWidth="1"/>
-    <col min="15" max="15" width="16.28515625" customWidth="1"/>
-    <col min="16" max="16" width="15.5703125" customWidth="1"/>
-    <col min="17" max="17" width="17.7109375" customWidth="1"/>
-    <col min="18" max="18" width="24.140625" customWidth="1"/>
-    <col min="19" max="19" width="13.42578125" customWidth="1"/>
-    <col min="20" max="20" width="13.5703125" customWidth="1"/>
+    <col min="4" max="4" width="13.7090909090909" customWidth="1"/>
+    <col min="5" max="5" width="5.28181818181818" customWidth="1"/>
+    <col min="6" max="6" width="17.2818181818182" customWidth="1"/>
+    <col min="7" max="7" width="30.2818181818182" customWidth="1"/>
+    <col min="8" max="8" width="26.8545454545455" customWidth="1"/>
+    <col min="9" max="9" width="17.2818181818182" customWidth="1"/>
+    <col min="10" max="10" width="13.2818181818182" customWidth="1"/>
+    <col min="11" max="11" width="22.7090909090909" customWidth="1"/>
+    <col min="12" max="12" width="12.7090909090909" customWidth="1"/>
+    <col min="13" max="13" width="29.5727272727273" customWidth="1"/>
+    <col min="14" max="14" width="18.2818181818182" customWidth="1"/>
+    <col min="15" max="15" width="16.2818181818182" customWidth="1"/>
+    <col min="16" max="16" width="15.5727272727273" customWidth="1"/>
+    <col min="17" max="17" width="17.7090909090909" customWidth="1"/>
+    <col min="18" max="18" width="24.1363636363636" customWidth="1"/>
+    <col min="19" max="19" width="13.4272727272727" customWidth="1"/>
+    <col min="20" max="20" width="13.5727272727273" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:20">
-      <c r="A1" s="12" t="s">
+      <c r="A1" s="13" t="s">
         <v>25</v>
       </c>
-      <c r="B1" s="12" t="s">
+      <c r="B1" s="13" t="s">
         <v>26</v>
       </c>
-      <c r="C1" s="12" t="s">
+      <c r="C1" s="13" t="s">
         <v>27</v>
       </c>
-      <c r="D1" s="12" t="s">
+      <c r="D1" s="13" t="s">
         <v>28</v>
       </c>
-      <c r="E1" s="12" t="s">
+      <c r="E1" s="13" t="s">
         <v>29</v>
       </c>
-      <c r="F1" s="12" t="s">
+      <c r="F1" s="13" t="s">
         <v>2</v>
       </c>
-      <c r="G1" s="12" t="s">
+      <c r="G1" s="13" t="s">
         <v>1</v>
       </c>
-      <c r="H1" s="12" t="s">
+      <c r="H1" s="13" t="s">
         <v>30</v>
       </c>
-      <c r="I1" s="12" t="s">
+      <c r="I1" s="13" t="s">
         <v>31</v>
       </c>
-      <c r="J1" s="12" t="s">
+      <c r="J1" s="13" t="s">
         <v>32</v>
       </c>
-      <c r="K1" s="12" t="s">
+      <c r="K1" s="13" t="s">
         <v>33</v>
       </c>
-      <c r="L1" s="12" t="s">
+      <c r="L1" s="13" t="s">
         <v>6</v>
       </c>
-      <c r="M1" s="12" t="s">
+      <c r="M1" s="13" t="s">
         <v>7</v>
       </c>
-      <c r="N1" s="12" t="s">
+      <c r="N1" s="13" t="s">
         <v>8</v>
       </c>
-      <c r="O1" s="12" t="s">
+      <c r="O1" s="13" t="s">
         <v>9</v>
       </c>
-      <c r="P1" s="12" t="s">
+      <c r="P1" s="13" t="s">
         <v>34</v>
       </c>
-      <c r="Q1" s="12" t="s">
+      <c r="Q1" s="13" t="s">
         <v>35</v>
       </c>
-      <c r="R1" s="12" t="s">
+      <c r="R1" s="13" t="s">
         <v>36</v>
       </c>
-      <c r="S1" s="12" t="s">
+      <c r="S1" s="13" t="s">
         <v>37</v>
       </c>
-      <c r="T1" s="12" t="s">
+      <c r="T1" s="13" t="s">
         <v>38</v>
       </c>
     </row>
     <row r="2" spans="1:20">
-      <c r="A2" s="12" t="s">
+      <c r="A2" s="13" t="s">
         <v>18</v>
       </c>
-      <c r="B2" s="12" t="s">
+      <c r="B2" s="13" t="s">
         <v>39</v>
       </c>
-      <c r="C2" s="12" t="s">
+      <c r="C2" s="13" t="s">
         <v>20</v>
       </c>
-      <c r="D2" s="12" t="s">
+      <c r="D2" s="13" t="s">
         <v>40</v>
       </c>
-      <c r="E2" s="12">
+      <c r="E2" s="13">
         <v>12</v>
       </c>
-      <c r="F2" s="18" t="s">
+      <c r="F2" s="19" t="s">
         <v>12</v>
       </c>
-      <c r="G2" s="12" t="s">
+      <c r="G2" s="13" t="s">
         <v>11</v>
       </c>
-      <c r="H2" s="12" t="s">
+      <c r="H2" s="13" t="s">
         <v>19</v>
       </c>
-      <c r="I2" s="12" t="s">
+      <c r="I2" s="13" t="s">
         <v>41</v>
       </c>
-      <c r="J2" s="12" t="s">
+      <c r="J2" s="13" t="s">
         <v>14</v>
       </c>
-      <c r="K2" s="12">
+      <c r="K2" s="13">
         <v>6</v>
       </c>
-      <c r="L2" s="12">
+      <c r="L2" s="13">
         <v>1010301033</v>
       </c>
-      <c r="M2" s="12" t="s">
+      <c r="M2" s="13" t="s">
         <v>15</v>
       </c>
-      <c r="N2" s="12" t="s">
+      <c r="N2" s="13" t="s">
         <v>16</v>
       </c>
-      <c r="O2" s="12" t="s">
+      <c r="O2" s="13" t="s">
         <v>17</v>
       </c>
-      <c r="P2" s="12"/>
-      <c r="Q2" s="12"/>
-      <c r="R2" s="12"/>
-      <c r="S2" s="12">
+      <c r="P2" s="13"/>
+      <c r="Q2" s="13"/>
+      <c r="R2" s="13"/>
+      <c r="S2" s="13">
         <v>0</v>
       </c>
-      <c r="T2" s="12"/>
+      <c r="T2" s="13"/>
     </row>
     <row r="3" spans="1:20">
-      <c r="A3" s="12" t="s">
+      <c r="A3" s="13" t="s">
         <v>10</v>
       </c>
-      <c r="B3" s="12" t="s">
+      <c r="B3" s="13" t="s">
         <v>42</v>
       </c>
-      <c r="C3" s="12" t="s">
+      <c r="C3" s="13" t="s">
         <v>14</v>
       </c>
-      <c r="D3" s="19" t="s">
+      <c r="D3" s="20" t="s">
         <v>43</v>
       </c>
-      <c r="E3" s="12">
+      <c r="E3" s="13">
         <v>5</v>
       </c>
-      <c r="F3" s="12" t="s">
+      <c r="F3" s="13" t="s">
         <v>12</v>
       </c>
-      <c r="G3" s="12" t="s">
+      <c r="G3" s="13" t="s">
         <v>11</v>
       </c>
-      <c r="H3" s="12" t="s">
+      <c r="H3" s="13" t="s">
         <v>13</v>
       </c>
-      <c r="I3" s="12" t="s">
+      <c r="I3" s="13" t="s">
         <v>44</v>
       </c>
-      <c r="J3" s="12" t="s">
+      <c r="J3" s="13" t="s">
         <v>14</v>
       </c>
-      <c r="K3" s="12">
+      <c r="K3" s="13">
         <v>1</v>
       </c>
-      <c r="L3" s="12">
+      <c r="L3" s="13">
         <v>1010301033</v>
       </c>
-      <c r="M3" s="12" t="s">
+      <c r="M3" s="13" t="s">
         <v>15</v>
       </c>
-      <c r="N3" s="12" t="s">
+      <c r="N3" s="13" t="s">
         <v>16</v>
       </c>
-      <c r="O3" s="12" t="s">
+      <c r="O3" s="13" t="s">
         <v>17</v>
       </c>
-      <c r="P3" s="12"/>
-      <c r="Q3" s="12"/>
-      <c r="R3" s="12"/>
-      <c r="S3" s="12">
+      <c r="P3" s="13"/>
+      <c r="Q3" s="13"/>
+      <c r="R3" s="13"/>
+      <c r="S3" s="13">
         <v>0</v>
       </c>
-      <c r="T3" s="12"/>
+      <c r="T3" s="13"/>
     </row>
     <row r="4" spans="1:20">
-      <c r="A4" s="12" t="s">
+      <c r="A4" s="13" t="s">
         <v>21</v>
       </c>
-      <c r="B4" s="12" t="s">
+      <c r="B4" s="13" t="s">
         <v>45</v>
       </c>
-      <c r="C4" s="12" t="s">
+      <c r="C4" s="13" t="s">
         <v>14</v>
       </c>
-      <c r="D4" s="12">
+      <c r="D4" s="13">
         <v>123562</v>
       </c>
-      <c r="E4" s="12">
+      <c r="E4" s="13">
         <v>18</v>
       </c>
-      <c r="F4" s="12" t="s">
+      <c r="F4" s="13" t="s">
         <v>22</v>
       </c>
-      <c r="G4" s="12" t="s">
+      <c r="G4" s="13" t="s">
         <v>22</v>
       </c>
-      <c r="H4" s="12" t="s">
+      <c r="H4" s="13" t="s">
         <v>23</v>
       </c>
-      <c r="I4" s="12" t="s">
+      <c r="I4" s="13" t="s">
         <v>44</v>
       </c>
-      <c r="J4" s="12" t="s">
+      <c r="J4" s="13" t="s">
         <v>14</v>
       </c>
-      <c r="K4" s="12">
+      <c r="K4" s="13">
         <v>1</v>
       </c>
-      <c r="L4" s="12">
+      <c r="L4" s="13">
         <v>1011134888</v>
       </c>
-      <c r="M4" s="12" t="s">
+      <c r="M4" s="13" t="s">
         <v>46</v>
       </c>
-      <c r="N4" s="12" t="s">
+      <c r="N4" s="13" t="s">
         <v>16</v>
       </c>
-      <c r="O4" s="12" t="s">
+      <c r="O4" s="13" t="s">
         <v>17</v>
       </c>
-      <c r="P4" s="12"/>
-      <c r="Q4" s="12"/>
-      <c r="R4" s="12"/>
-      <c r="S4" s="12">
+      <c r="P4" s="13"/>
+      <c r="Q4" s="13"/>
+      <c r="R4" s="13"/>
+      <c r="S4" s="13">
         <v>0</v>
       </c>
-      <c r="T4" s="12"/>
+      <c r="T4" s="13"/>
     </row>
     <row r="5" spans="1:20">
       <c r="A5" s="3" t="s">
@@ -2267,7 +2942,7 @@
       <c r="B5" s="3" t="s">
         <v>47</v>
       </c>
-      <c r="C5" s="12" t="s">
+      <c r="C5" s="13" t="s">
         <v>14</v>
       </c>
       <c r="D5" s="3" t="s">
@@ -2309,7 +2984,7 @@
       <c r="P5" s="3"/>
       <c r="Q5" s="3"/>
       <c r="R5" s="3"/>
-      <c r="S5" s="12">
+      <c r="S5" s="13">
         <v>0</v>
       </c>
       <c r="T5" s="3"/>
@@ -2324,16 +2999,16 @@
       <c r="C6" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="D6" s="17" t="s">
+      <c r="D6" s="18" t="s">
         <v>43</v>
       </c>
       <c r="E6">
         <v>5</v>
       </c>
-      <c r="F6" s="20" t="s">
+      <c r="F6" s="21" t="s">
         <v>12</v>
       </c>
-      <c r="G6" s="20" t="s">
+      <c r="G6" s="21" t="s">
         <v>11</v>
       </c>
       <c r="H6" s="3" t="s">
@@ -2363,172 +3038,172 @@
       <c r="P6" s="3"/>
       <c r="Q6" s="3"/>
       <c r="R6" s="3"/>
-      <c r="S6" s="12">
+      <c r="S6" s="13">
         <v>0</v>
       </c>
       <c r="T6" s="3"/>
     </row>
     <row r="7" spans="1:20">
-      <c r="A7" s="21" t="s">
+      <c r="A7" s="22" t="s">
         <v>55</v>
       </c>
-      <c r="B7" s="21" t="s">
+      <c r="B7" s="22" t="s">
         <v>56</v>
       </c>
-      <c r="C7" s="21" t="s">
+      <c r="C7" s="22" t="s">
         <v>20</v>
       </c>
-      <c r="D7" s="21" t="s">
+      <c r="D7" s="22" t="s">
         <v>40</v>
       </c>
-      <c r="E7" s="21">
+      <c r="E7" s="22">
         <v>12</v>
       </c>
-      <c r="F7" s="22" t="s">
+      <c r="F7" s="23" t="s">
         <v>12</v>
       </c>
-      <c r="G7" s="21" t="s">
+      <c r="G7" s="22" t="s">
         <v>11</v>
       </c>
-      <c r="H7" s="21" t="s">
+      <c r="H7" s="22" t="s">
         <v>57</v>
       </c>
-      <c r="I7" s="21" t="s">
+      <c r="I7" s="22" t="s">
         <v>41</v>
       </c>
-      <c r="J7" s="21" t="s">
+      <c r="J7" s="22" t="s">
         <v>14</v>
       </c>
-      <c r="K7" s="21">
+      <c r="K7" s="22">
         <v>3</v>
       </c>
-      <c r="L7" s="21">
+      <c r="L7" s="22">
         <v>1010301003</v>
       </c>
-      <c r="M7" s="21" t="s">
+      <c r="M7" s="22" t="s">
         <v>58</v>
       </c>
-      <c r="N7" s="21" t="s">
+      <c r="N7" s="22" t="s">
         <v>16</v>
       </c>
-      <c r="O7" s="21" t="s">
+      <c r="O7" s="22" t="s">
         <v>17</v>
       </c>
-      <c r="P7" s="21"/>
-      <c r="Q7" s="21"/>
-      <c r="R7" s="21"/>
-      <c r="S7" s="21">
+      <c r="P7" s="22"/>
+      <c r="Q7" s="22"/>
+      <c r="R7" s="22"/>
+      <c r="S7" s="22">
         <v>0</v>
       </c>
-      <c r="T7" s="21"/>
+      <c r="T7" s="22"/>
     </row>
     <row r="8" spans="1:20">
-      <c r="A8" s="21" t="s">
+      <c r="A8" s="22" t="s">
         <v>59</v>
       </c>
-      <c r="B8" s="21" t="s">
+      <c r="B8" s="22" t="s">
         <v>60</v>
       </c>
-      <c r="C8" s="21" t="s">
+      <c r="C8" s="22" t="s">
         <v>14</v>
       </c>
-      <c r="D8" s="21" t="s">
+      <c r="D8" s="22" t="s">
         <v>43</v>
       </c>
-      <c r="E8" s="21">
+      <c r="E8" s="22">
         <v>5</v>
       </c>
-      <c r="F8" s="22" t="s">
+      <c r="F8" s="23" t="s">
         <v>12</v>
       </c>
-      <c r="G8" s="21" t="s">
+      <c r="G8" s="22" t="s">
         <v>11</v>
       </c>
-      <c r="H8" s="21" t="s">
+      <c r="H8" s="22" t="s">
         <v>57</v>
       </c>
-      <c r="I8" s="21" t="s">
+      <c r="I8" s="22" t="s">
         <v>41</v>
       </c>
-      <c r="J8" s="21" t="s">
+      <c r="J8" s="22" t="s">
         <v>14</v>
       </c>
-      <c r="K8" s="21">
+      <c r="K8" s="22">
         <v>0</v>
       </c>
-      <c r="L8" s="21">
+      <c r="L8" s="22">
         <v>1010301003</v>
       </c>
-      <c r="M8" s="21" t="s">
+      <c r="M8" s="22" t="s">
         <v>58</v>
       </c>
-      <c r="N8" s="21" t="s">
+      <c r="N8" s="22" t="s">
         <v>16</v>
       </c>
-      <c r="O8" s="21" t="s">
+      <c r="O8" s="22" t="s">
         <v>17</v>
       </c>
-      <c r="P8" s="21"/>
-      <c r="Q8" s="21"/>
-      <c r="R8" s="21"/>
-      <c r="S8" s="21">
+      <c r="P8" s="22"/>
+      <c r="Q8" s="22"/>
+      <c r="R8" s="22"/>
+      <c r="S8" s="22">
         <v>0</v>
       </c>
-      <c r="T8" s="21"/>
+      <c r="T8" s="22"/>
     </row>
     <row r="9" spans="1:20">
-      <c r="A9" s="21" t="s">
+      <c r="A9" s="22" t="s">
         <v>61</v>
       </c>
-      <c r="B9" s="21" t="s">
+      <c r="B9" s="22" t="s">
         <v>61</v>
       </c>
-      <c r="C9" s="21" t="s">
+      <c r="C9" s="22" t="s">
         <v>14</v>
       </c>
-      <c r="D9" s="21" t="s">
+      <c r="D9" s="22" t="s">
         <v>43</v>
       </c>
-      <c r="E9" s="21">
+      <c r="E9" s="22">
         <v>5</v>
       </c>
-      <c r="F9" s="22" t="s">
+      <c r="F9" s="23" t="s">
         <v>12</v>
       </c>
-      <c r="G9" s="21" t="s">
+      <c r="G9" s="22" t="s">
         <v>11</v>
       </c>
-      <c r="H9" s="21" t="s">
+      <c r="H9" s="22" t="s">
         <v>57</v>
       </c>
-      <c r="I9" s="21" t="s">
+      <c r="I9" s="22" t="s">
         <v>41</v>
       </c>
-      <c r="J9" s="21" t="s">
+      <c r="J9" s="22" t="s">
         <v>14</v>
       </c>
-      <c r="K9" s="21">
+      <c r="K9" s="22">
         <v>0</v>
       </c>
-      <c r="L9" s="21">
+      <c r="L9" s="22">
         <v>1010301003</v>
       </c>
-      <c r="M9" s="21" t="s">
+      <c r="M9" s="22" t="s">
         <v>58</v>
       </c>
-      <c r="N9" s="21" t="s">
+      <c r="N9" s="22" t="s">
         <v>16</v>
       </c>
-      <c r="O9" s="21" t="s">
+      <c r="O9" s="22" t="s">
         <v>17</v>
       </c>
-      <c r="P9" s="21"/>
-      <c r="Q9" s="21"/>
-      <c r="R9" s="21"/>
-      <c r="S9" s="21">
+      <c r="P9" s="22"/>
+      <c r="Q9" s="22"/>
+      <c r="R9" s="22"/>
+      <c r="S9" s="22">
         <v>0</v>
       </c>
-      <c r="T9" s="21"/>
+      <c r="T9" s="22"/>
     </row>
     <row r="10" spans="1:20">
       <c r="A10" s="3" t="s">
@@ -2540,31 +3215,31 @@
       <c r="C10" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="D10" s="21" t="s">
+      <c r="D10" s="22" t="s">
         <v>43</v>
       </c>
-      <c r="E10" s="21">
+      <c r="E10" s="22">
         <v>5</v>
       </c>
-      <c r="F10" s="12" t="s">
+      <c r="F10" s="13" t="s">
         <v>22</v>
       </c>
-      <c r="G10" s="12" t="s">
+      <c r="G10" s="13" t="s">
         <v>22</v>
       </c>
-      <c r="H10" s="12" t="s">
+      <c r="H10" s="13" t="s">
         <v>63</v>
       </c>
-      <c r="I10" s="12" t="s">
+      <c r="I10" s="13" t="s">
         <v>44</v>
       </c>
-      <c r="J10" s="12" t="s">
+      <c r="J10" s="13" t="s">
         <v>14</v>
       </c>
-      <c r="K10" s="12">
+      <c r="K10" s="13">
         <v>1</v>
       </c>
-      <c r="L10" s="15">
+      <c r="L10" s="16">
         <v>1000000001</v>
       </c>
       <c r="M10" s="3" t="s">
@@ -2576,35 +3251,37 @@
       <c r="O10" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="P10" s="21"/>
-      <c r="Q10" s="21"/>
-      <c r="R10" s="21"/>
-      <c r="S10" s="21">
+      <c r="P10" s="22"/>
+      <c r="Q10" s="22"/>
+      <c r="R10" s="22"/>
+      <c r="S10" s="22">
         <v>0</v>
       </c>
-      <c r="T10" s="21"/>
+      <c r="T10" s="22"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
   <dimension ref="A1:R3"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="8.85454545454546" defaultRowHeight="14.5" outlineLevelRow="2"/>
   <cols>
     <col min="1" max="2" width="21" customWidth="1"/>
     <col min="3" max="3" width="6" customWidth="1"/>
-    <col min="4" max="4" width="12.7109375" customWidth="1"/>
-    <col min="5" max="5" width="19.42578125" customWidth="1"/>
-    <col min="6" max="6" width="15.140625" customWidth="1"/>
-    <col min="7" max="7" width="15.42578125" customWidth="1"/>
-    <col min="8" max="8" width="19.5703125" customWidth="1"/>
-    <col min="9" max="9" width="10.85546875" customWidth="1"/>
-    <col min="10" max="10" width="17.5703125" customWidth="1"/>
-    <col min="11" max="11" width="11.28515625" customWidth="1"/>
-    <col min="12" max="12" width="21.7109375" customWidth="1"/>
+    <col min="4" max="4" width="12.7090909090909" customWidth="1"/>
+    <col min="5" max="5" width="19.4272727272727" customWidth="1"/>
+    <col min="6" max="6" width="15.1363636363636" customWidth="1"/>
+    <col min="7" max="7" width="15.4272727272727" customWidth="1"/>
+    <col min="8" max="8" width="19.5727272727273" customWidth="1"/>
+    <col min="9" max="9" width="10.8545454545455" customWidth="1"/>
+    <col min="10" max="10" width="17.5727272727273" customWidth="1"/>
+    <col min="11" max="11" width="11.2818181818182" customWidth="1"/>
+    <col min="12" max="12" width="21.7090909090909" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:18">
@@ -2617,16 +3294,16 @@
       <c r="C1" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="D1" s="12" t="s">
+      <c r="D1" s="13" t="s">
         <v>6</v>
       </c>
-      <c r="E1" s="12" t="s">
+      <c r="E1" s="13" t="s">
         <v>7</v>
       </c>
-      <c r="F1" s="12" t="s">
+      <c r="F1" s="13" t="s">
         <v>8</v>
       </c>
-      <c r="G1" s="12" t="s">
+      <c r="G1" s="13" t="s">
         <v>9</v>
       </c>
       <c r="H1" s="3" t="s">
@@ -2644,12 +3321,12 @@
       <c r="L1" s="3" t="s">
         <v>33</v>
       </c>
-      <c r="M1" s="16"/>
-      <c r="N1" s="16"/>
-      <c r="O1" s="16"/>
-      <c r="P1" s="16"/>
-      <c r="Q1" s="16"/>
-      <c r="R1" s="16"/>
+      <c r="M1" s="17"/>
+      <c r="N1" s="17"/>
+      <c r="O1" s="17"/>
+      <c r="P1" s="17"/>
+      <c r="Q1" s="17"/>
+      <c r="R1" s="17"/>
     </row>
     <row r="2" spans="1:18">
       <c r="A2" s="3" t="s">
@@ -2676,7 +3353,7 @@
       <c r="H2" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="I2" s="17" t="s">
+      <c r="I2" s="18" t="s">
         <v>43</v>
       </c>
       <c r="J2" s="3" t="s">
@@ -2688,14 +3365,14 @@
       <c r="L2" s="3">
         <v>1</v>
       </c>
-      <c r="M2" s="16"/>
-      <c r="N2" s="16"/>
-      <c r="O2" s="16"/>
-      <c r="P2" s="16"/>
-      <c r="Q2" s="16"/>
-      <c r="R2" s="16"/>
-    </row>
-    <row r="3" spans="1:18">
+      <c r="M2" s="17"/>
+      <c r="N2" s="17"/>
+      <c r="O2" s="17"/>
+      <c r="P2" s="17"/>
+      <c r="Q2" s="17"/>
+      <c r="R2" s="17"/>
+    </row>
+    <row r="3" spans="1:12">
       <c r="A3" s="3" t="s">
         <v>62</v>
       </c>
@@ -2705,7 +3382,7 @@
       <c r="C3" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="D3" s="15">
+      <c r="D3" s="16">
         <v>1000000001</v>
       </c>
       <c r="E3" s="3" t="s">
@@ -2720,7 +3397,7 @@
       <c r="H3" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="I3" s="17" t="s">
+      <c r="I3" s="18" t="s">
         <v>43</v>
       </c>
       <c r="J3" s="3" t="s">
@@ -2735,39 +3412,41 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
   <dimension ref="A1:F3"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="8.85454545454546" defaultRowHeight="14.5" outlineLevelRow="2" outlineLevelCol="5"/>
   <cols>
-    <col min="1" max="1" width="27.140625" customWidth="1"/>
-    <col min="2" max="2" width="10.42578125" customWidth="1"/>
-    <col min="3" max="3" width="11.42578125" customWidth="1"/>
-    <col min="4" max="4" width="11.7109375" customWidth="1"/>
-    <col min="5" max="5" width="14.5703125" customWidth="1"/>
-    <col min="6" max="6" width="17.7109375" customWidth="1"/>
+    <col min="1" max="1" width="27.1363636363636" customWidth="1"/>
+    <col min="2" max="2" width="10.4272727272727" customWidth="1"/>
+    <col min="3" max="3" width="11.4272727272727" customWidth="1"/>
+    <col min="4" max="4" width="11.7090909090909" customWidth="1"/>
+    <col min="5" max="5" width="14.5727272727273" customWidth="1"/>
+    <col min="6" max="6" width="17.7090909090909" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6">
-      <c r="A1" s="13" t="s">
+      <c r="A1" s="14" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="13" t="s">
+      <c r="B1" s="14" t="s">
         <v>66</v>
       </c>
-      <c r="C1" s="13" t="s">
+      <c r="C1" s="14" t="s">
         <v>67</v>
       </c>
-      <c r="D1" s="14" t="s">
+      <c r="D1" s="15" t="s">
         <v>68</v>
       </c>
-      <c r="E1" s="12" t="s">
+      <c r="E1" s="13" t="s">
         <v>69</v>
       </c>
-      <c r="F1" s="12" t="s">
+      <c r="F1" s="13" t="s">
         <v>70</v>
       </c>
     </row>
@@ -2785,7 +3464,7 @@
         <v>71</v>
       </c>
       <c r="E2" s="3"/>
-      <c r="F2" s="9" t="s">
+      <c r="F2" s="10" t="s">
         <v>72</v>
       </c>
     </row>
@@ -2802,53 +3481,55 @@
       <c r="D3" s="3" t="s">
         <v>73</v>
       </c>
-      <c r="E3" s="9" t="s">
+      <c r="E3" s="10" t="s">
         <v>74</v>
       </c>
-      <c r="F3" s="9">
+      <c r="F3" s="10">
         <v>2</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
   <dimension ref="A1:F4"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="8.85454545454546" defaultRowHeight="14.5" outlineLevelRow="3" outlineLevelCol="5"/>
   <cols>
-    <col min="1" max="1" width="27.140625" customWidth="1"/>
-    <col min="2" max="2" width="10.42578125" customWidth="1"/>
-    <col min="3" max="3" width="11.42578125" customWidth="1"/>
-    <col min="4" max="4" width="11.7109375" customWidth="1"/>
-    <col min="5" max="5" width="14.5703125" customWidth="1"/>
-    <col min="6" max="6" width="17.7109375" customWidth="1"/>
+    <col min="1" max="1" width="27.1363636363636" customWidth="1"/>
+    <col min="2" max="2" width="10.4272727272727" customWidth="1"/>
+    <col min="3" max="3" width="11.4272727272727" customWidth="1"/>
+    <col min="4" max="4" width="11.7090909090909" customWidth="1"/>
+    <col min="5" max="5" width="14.5727272727273" customWidth="1"/>
+    <col min="6" max="6" width="17.7090909090909" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6">
-      <c r="A1" s="13" t="s">
+      <c r="A1" s="14" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="13" t="s">
+      <c r="B1" s="14" t="s">
         <v>66</v>
       </c>
-      <c r="C1" s="13" t="s">
+      <c r="C1" s="14" t="s">
         <v>67</v>
       </c>
-      <c r="D1" s="14" t="s">
+      <c r="D1" s="15" t="s">
         <v>68</v>
       </c>
-      <c r="E1" s="12" t="s">
+      <c r="E1" s="13" t="s">
         <v>69</v>
       </c>
-      <c r="F1" s="12" t="s">
+      <c r="F1" s="13" t="s">
         <v>70</v>
       </c>
     </row>
     <row r="2" spans="1:6">
-      <c r="A2" s="12" t="s">
+      <c r="A2" s="13" t="s">
         <v>59</v>
       </c>
       <c r="B2" s="3">
@@ -2861,12 +3542,12 @@
         <v>71</v>
       </c>
       <c r="E2" s="3"/>
-      <c r="F2" s="9" t="s">
+      <c r="F2" s="10" t="s">
         <v>75</v>
       </c>
     </row>
     <row r="3" spans="1:6">
-      <c r="A3" s="12" t="s">
+      <c r="A3" s="13" t="s">
         <v>76</v>
       </c>
       <c r="B3" s="3">
@@ -2878,15 +3559,15 @@
       <c r="D3" s="3" t="s">
         <v>77</v>
       </c>
-      <c r="E3" s="9" t="s">
+      <c r="E3" s="10" t="s">
         <v>74</v>
       </c>
-      <c r="F3" s="9">
+      <c r="F3" s="10">
         <v>2</v>
       </c>
     </row>
     <row r="4" spans="1:6">
-      <c r="A4" s="12" t="s">
+      <c r="A4" s="13" t="s">
         <v>61</v>
       </c>
       <c r="B4" s="3">
@@ -2901,19 +3582,21 @@
       <c r="E4" s="3" t="s">
         <v>75</v>
       </c>
-      <c r="F4" s="9"/>
+      <c r="F4" s="10"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
   <dimension ref="A1:C3"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="8.85454545454546" defaultRowHeight="14.5" outlineLevelRow="2" outlineLevelCol="2"/>
   <cols>
-    <col min="1" max="1" width="28.7109375" customWidth="1"/>
+    <col min="1" max="1" width="28.7090909090909" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3">
@@ -2951,86 +3634,88 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
   <dimension ref="A1:G4"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="8.85454545454546" defaultRowHeight="14.5" outlineLevelRow="3" outlineLevelCol="6"/>
   <cols>
-    <col min="1" max="1" width="19.7109375" customWidth="1"/>
-    <col min="2" max="2" width="8.140625" customWidth="1"/>
-    <col min="3" max="3" width="8.5703125" customWidth="1"/>
-    <col min="4" max="4" width="17.85546875" customWidth="1"/>
-    <col min="5" max="5" width="12.7109375" customWidth="1"/>
-    <col min="6" max="6" width="14.5703125" customWidth="1"/>
-    <col min="7" max="7" width="17.7109375" customWidth="1"/>
+    <col min="1" max="1" width="19.7090909090909" customWidth="1"/>
+    <col min="2" max="2" width="8.13636363636364" customWidth="1"/>
+    <col min="3" max="3" width="8.57272727272727" customWidth="1"/>
+    <col min="4" max="4" width="17.8545454545455" customWidth="1"/>
+    <col min="5" max="5" width="12.7090909090909" customWidth="1"/>
+    <col min="6" max="6" width="14.5727272727273" customWidth="1"/>
+    <col min="7" max="7" width="17.7090909090909" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7">
-      <c r="A1" s="12" t="s">
+      <c r="A1" s="13" t="s">
         <v>83</v>
       </c>
-      <c r="B1" s="12" t="s">
+      <c r="B1" s="13" t="s">
         <v>84</v>
       </c>
-      <c r="C1" s="12" t="s">
+      <c r="C1" s="13" t="s">
         <v>80</v>
       </c>
-      <c r="D1" s="12" t="s">
+      <c r="D1" s="13" t="s">
         <v>85</v>
       </c>
-      <c r="E1" s="12" t="s">
+      <c r="E1" s="13" t="s">
         <v>68</v>
       </c>
-      <c r="F1" s="12" t="s">
+      <c r="F1" s="13" t="s">
         <v>69</v>
       </c>
-      <c r="G1" s="12" t="s">
+      <c r="G1" s="13" t="s">
         <v>70</v>
       </c>
     </row>
     <row r="2" spans="1:7">
-      <c r="A2" s="12" t="s">
+      <c r="A2" s="13" t="s">
         <v>86</v>
       </c>
-      <c r="B2" s="12">
+      <c r="B2" s="13">
         <v>524</v>
       </c>
-      <c r="C2" s="12">
+      <c r="C2" s="13">
         <v>524</v>
       </c>
-      <c r="D2" s="12">
+      <c r="D2" s="13">
         <v>2</v>
       </c>
-      <c r="E2" s="9" t="s">
+      <c r="E2" s="10" t="s">
         <v>71</v>
       </c>
-      <c r="F2" s="9" t="s">
+      <c r="F2" s="10" t="s">
         <v>74</v>
       </c>
-      <c r="G2" s="9" t="s">
+      <c r="G2" s="10" t="s">
         <v>87</v>
       </c>
     </row>
     <row r="3" spans="1:7">
-      <c r="A3" s="12" t="s">
+      <c r="A3" s="13" t="s">
         <v>88</v>
       </c>
-      <c r="B3" s="12">
+      <c r="B3" s="13">
         <v>232</v>
       </c>
-      <c r="C3" s="12">
+      <c r="C3" s="13">
         <v>232</v>
       </c>
-      <c r="D3" s="12">
+      <c r="D3" s="13">
         <v>7.9</v>
       </c>
-      <c r="E3" s="9" t="s">
+      <c r="E3" s="10" t="s">
         <v>73</v>
       </c>
-      <c r="F3" s="9" t="s">
+      <c r="F3" s="10" t="s">
         <v>89</v>
       </c>
       <c r="G3" s="3"/>
@@ -3046,9 +3731,9 @@
         <v>232</v>
       </c>
       <c r="D4" s="3">
-        <v>2.3199999999999998</v>
-      </c>
-      <c r="E4" s="9" t="s">
+        <v>2.32</v>
+      </c>
+      <c r="E4" s="10" t="s">
         <v>77</v>
       </c>
       <c r="F4" s="3"/>
@@ -3056,86 +3741,88 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
   <dimension ref="A1:G4"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="8.85454545454546" defaultRowHeight="14.5" outlineLevelRow="3" outlineLevelCol="6"/>
   <cols>
-    <col min="1" max="1" width="19.7109375" customWidth="1"/>
-    <col min="2" max="2" width="8.140625" customWidth="1"/>
-    <col min="3" max="3" width="8.5703125" customWidth="1"/>
-    <col min="4" max="4" width="17.85546875" customWidth="1"/>
-    <col min="5" max="5" width="12.7109375" customWidth="1"/>
-    <col min="6" max="6" width="14.5703125" customWidth="1"/>
-    <col min="7" max="7" width="17.7109375" customWidth="1"/>
+    <col min="1" max="1" width="19.7090909090909" customWidth="1"/>
+    <col min="2" max="2" width="8.13636363636364" customWidth="1"/>
+    <col min="3" max="3" width="8.57272727272727" customWidth="1"/>
+    <col min="4" max="4" width="17.8545454545455" customWidth="1"/>
+    <col min="5" max="5" width="12.7090909090909" customWidth="1"/>
+    <col min="6" max="6" width="14.5727272727273" customWidth="1"/>
+    <col min="7" max="7" width="17.7090909090909" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7">
-      <c r="A1" s="12" t="s">
+      <c r="A1" s="13" t="s">
         <v>83</v>
       </c>
-      <c r="B1" s="12" t="s">
+      <c r="B1" s="13" t="s">
         <v>84</v>
       </c>
-      <c r="C1" s="12" t="s">
+      <c r="C1" s="13" t="s">
         <v>80</v>
       </c>
-      <c r="D1" s="12" t="s">
+      <c r="D1" s="13" t="s">
         <v>85</v>
       </c>
-      <c r="E1" s="12" t="s">
+      <c r="E1" s="13" t="s">
         <v>68</v>
       </c>
-      <c r="F1" s="12" t="s">
+      <c r="F1" s="13" t="s">
         <v>69</v>
       </c>
-      <c r="G1" s="12" t="s">
+      <c r="G1" s="13" t="s">
         <v>70</v>
       </c>
     </row>
     <row r="2" spans="1:7">
-      <c r="A2" s="12" t="s">
+      <c r="A2" s="13" t="s">
         <v>86</v>
       </c>
-      <c r="B2" s="12">
+      <c r="B2" s="13">
         <v>22</v>
       </c>
-      <c r="C2" s="12">
+      <c r="C2" s="13">
         <v>524</v>
       </c>
-      <c r="D2" s="12">
+      <c r="D2" s="13">
         <v>2</v>
       </c>
-      <c r="E2" s="9" t="s">
+      <c r="E2" s="10" t="s">
         <v>71</v>
       </c>
-      <c r="F2" s="9" t="s">
+      <c r="F2" s="10" t="s">
         <v>74</v>
       </c>
-      <c r="G2" s="9" t="s">
+      <c r="G2" s="10" t="s">
         <v>87</v>
       </c>
     </row>
     <row r="3" spans="1:7">
-      <c r="A3" s="12" t="s">
+      <c r="A3" s="13" t="s">
         <v>88</v>
       </c>
-      <c r="B3" s="12">
+      <c r="B3" s="13">
         <v>34</v>
       </c>
-      <c r="C3" s="12">
+      <c r="C3" s="13">
         <v>232</v>
       </c>
-      <c r="D3" s="12">
+      <c r="D3" s="13">
         <v>7.9</v>
       </c>
-      <c r="E3" s="9" t="s">
+      <c r="E3" s="10" t="s">
         <v>73</v>
       </c>
-      <c r="F3" s="9" t="s">
+      <c r="F3" s="10" t="s">
         <v>89</v>
       </c>
       <c r="G3" s="3"/>
@@ -3151,9 +3838,9 @@
         <v>232</v>
       </c>
       <c r="D4" s="3">
-        <v>2.3199999999999998</v>
-      </c>
-      <c r="E4" s="9" t="s">
+        <v>2.32</v>
+      </c>
+      <c r="E4" s="10" t="s">
         <v>77</v>
       </c>
       <c r="F4" s="3"/>
@@ -3161,31 +3848,33 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:S9"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
+  <dimension ref="A1:S11"/>
+  <sheetFormatPr defaultColWidth="8.85454545454546" defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="39.7109375" customWidth="1"/>
-    <col min="2" max="2" width="10.140625" customWidth="1"/>
-    <col min="3" max="3" width="39.7109375" customWidth="1"/>
+    <col min="1" max="1" width="39.7090909090909" customWidth="1"/>
+    <col min="2" max="2" width="10.1363636363636" customWidth="1"/>
+    <col min="3" max="3" width="39.7090909090909" customWidth="1"/>
     <col min="4" max="4" width="11" customWidth="1"/>
-    <col min="5" max="5" width="13.28515625" customWidth="1"/>
-    <col min="6" max="6" width="8.85546875" customWidth="1"/>
-    <col min="7" max="7" width="17.85546875" customWidth="1"/>
-    <col min="8" max="8" width="19.5703125" customWidth="1"/>
-    <col min="9" max="9" width="23.7109375" customWidth="1"/>
-    <col min="10" max="10" width="12.7109375" customWidth="1"/>
-    <col min="11" max="11" width="11.85546875" customWidth="1"/>
-    <col min="12" max="12" width="17.42578125" customWidth="1"/>
-    <col min="13" max="14" width="39.7109375" customWidth="1"/>
-    <col min="15" max="15" width="25.7109375" customWidth="1"/>
-    <col min="16" max="17" width="16.5703125" customWidth="1"/>
-    <col min="18" max="18" width="11.5703125" customWidth="1"/>
-    <col min="19" max="19" width="14.85546875" customWidth="1"/>
+    <col min="5" max="5" width="13.2818181818182" customWidth="1"/>
+    <col min="6" max="6" width="8.85454545454546" customWidth="1"/>
+    <col min="7" max="7" width="17.8545454545455" customWidth="1"/>
+    <col min="8" max="8" width="19.5727272727273" customWidth="1"/>
+    <col min="9" max="9" width="23.7090909090909" customWidth="1"/>
+    <col min="10" max="10" width="12.7090909090909" customWidth="1"/>
+    <col min="11" max="11" width="11.8545454545455" customWidth="1"/>
+    <col min="12" max="12" width="17.4272727272727" customWidth="1"/>
+    <col min="13" max="14" width="39.7090909090909" customWidth="1"/>
+    <col min="15" max="15" width="25.7090909090909" customWidth="1"/>
+    <col min="16" max="17" width="16.5727272727273" customWidth="1"/>
+    <col min="18" max="18" width="11.5727272727273" customWidth="1"/>
+    <col min="19" max="19" width="14.8545454545455" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:19">
@@ -3248,13 +3937,13 @@
       </c>
     </row>
     <row r="2" spans="1:19">
-      <c r="A2" s="11" t="s">
+      <c r="A2" s="12" t="s">
         <v>106</v>
       </c>
       <c r="B2" s="3">
         <v>0</v>
       </c>
-      <c r="C2" s="11" t="s">
+      <c r="C2" s="12" t="s">
         <v>106</v>
       </c>
       <c r="D2" s="3" t="s">
@@ -3282,36 +3971,36 @@
       </c>
       <c r="M2" s="3"/>
       <c r="N2" s="3"/>
-      <c r="O2" s="9" t="s">
+      <c r="O2" s="10" t="s">
         <v>13</v>
       </c>
-      <c r="P2" s="9" t="s">
+      <c r="P2" s="10" t="s">
         <v>15</v>
       </c>
-      <c r="Q2" s="9" t="s">
+      <c r="Q2" s="10" t="s">
         <v>15</v>
       </c>
       <c r="R2" s="3" t="s">
         <v>108</v>
       </c>
-      <c r="S2" s="10" t="s">
+      <c r="S2" s="11" t="s">
         <v>109</v>
       </c>
     </row>
     <row r="3" spans="1:19">
-      <c r="A3" s="11" t="s">
+      <c r="A3" s="12" t="s">
         <v>110</v>
       </c>
       <c r="B3" s="3">
         <v>0</v>
       </c>
-      <c r="C3" s="11" t="s">
+      <c r="C3" s="12" t="s">
         <v>110</v>
       </c>
       <c r="D3" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="E3" s="11">
+      <c r="E3" s="12">
         <v>772213</v>
       </c>
       <c r="F3" s="3">
@@ -3333,19 +4022,19 @@
       </c>
       <c r="M3" s="3"/>
       <c r="N3" s="3"/>
-      <c r="O3" s="9" t="s">
+      <c r="O3" s="10" t="s">
         <v>13</v>
       </c>
-      <c r="P3" s="9" t="s">
+      <c r="P3" s="10" t="s">
         <v>15</v>
       </c>
-      <c r="Q3" s="9" t="s">
+      <c r="Q3" s="10" t="s">
         <v>15</v>
       </c>
       <c r="R3" s="3" t="s">
         <v>108</v>
       </c>
-      <c r="S3" s="10" t="s">
+      <c r="S3" s="11" t="s">
         <v>109</v>
       </c>
     </row>
@@ -3388,19 +4077,19 @@
       <c r="N4" s="3" t="s">
         <v>111</v>
       </c>
-      <c r="O4" s="9" t="s">
+      <c r="O4" s="10" t="s">
         <v>13</v>
       </c>
-      <c r="P4" s="9" t="s">
+      <c r="P4" s="10" t="s">
         <v>15</v>
       </c>
-      <c r="Q4" s="9" t="s">
+      <c r="Q4" s="10" t="s">
         <v>15</v>
       </c>
       <c r="R4" s="3" t="s">
         <v>108</v>
       </c>
-      <c r="S4" s="10" t="s">
+      <c r="S4" s="11" t="s">
         <v>109</v>
       </c>
     </row>
@@ -3443,19 +4132,19 @@
       <c r="N5" s="3" t="s">
         <v>113</v>
       </c>
-      <c r="O5" s="9" t="s">
+      <c r="O5" s="10" t="s">
         <v>13</v>
       </c>
-      <c r="P5" s="9" t="s">
+      <c r="P5" s="10" t="s">
         <v>15</v>
       </c>
-      <c r="Q5" s="9" t="s">
+      <c r="Q5" s="10" t="s">
         <v>15</v>
       </c>
       <c r="R5" s="3" t="s">
         <v>114</v>
       </c>
-      <c r="S5" s="10" t="s">
+      <c r="S5" s="11" t="s">
         <v>109</v>
       </c>
     </row>
@@ -3500,19 +4189,19 @@
       <c r="N6" s="5" t="s">
         <v>115</v>
       </c>
-      <c r="O6" s="9" t="s">
+      <c r="O6" s="10" t="s">
         <v>13</v>
       </c>
-      <c r="P6" s="9" t="s">
+      <c r="P6" s="10" t="s">
         <v>15</v>
       </c>
-      <c r="Q6" s="9" t="s">
+      <c r="Q6" s="10" t="s">
         <v>15</v>
       </c>
       <c r="R6" s="3" t="s">
         <v>108</v>
       </c>
-      <c r="S6" s="10" t="s">
+      <c r="S6" s="11" t="s">
         <v>109</v>
       </c>
     </row>
@@ -3557,19 +4246,19 @@
       <c r="N7" s="5" t="s">
         <v>118</v>
       </c>
-      <c r="O7" s="9" t="s">
+      <c r="O7" s="10" t="s">
         <v>13</v>
       </c>
-      <c r="P7" s="9" t="s">
+      <c r="P7" s="10" t="s">
         <v>15</v>
       </c>
-      <c r="Q7" s="9" t="s">
+      <c r="Q7" s="10" t="s">
         <v>15</v>
       </c>
       <c r="R7" s="3" t="s">
         <v>108</v>
       </c>
-      <c r="S7" s="10" t="s">
+      <c r="S7" s="11" t="s">
         <v>109</v>
       </c>
     </row>
@@ -3614,19 +4303,19 @@
       <c r="N8" s="3" t="s">
         <v>120</v>
       </c>
-      <c r="O8" s="9" t="s">
+      <c r="O8" s="10" t="s">
         <v>13</v>
       </c>
-      <c r="P8" s="9" t="s">
+      <c r="P8" s="10" t="s">
         <v>15</v>
       </c>
-      <c r="Q8" s="9" t="s">
+      <c r="Q8" s="10" t="s">
         <v>15</v>
       </c>
       <c r="R8" s="3" t="s">
         <v>108</v>
       </c>
-      <c r="S8" s="10" t="s">
+      <c r="S8" s="11" t="s">
         <v>109</v>
       </c>
     </row>
@@ -3671,23 +4360,134 @@
       <c r="N9" s="5" t="s">
         <v>123</v>
       </c>
-      <c r="O9" s="9" t="s">
+      <c r="O9" s="10" t="s">
         <v>13</v>
       </c>
-      <c r="P9" s="9" t="s">
+      <c r="P9" s="10" t="s">
         <v>15</v>
       </c>
-      <c r="Q9" s="9" t="s">
+      <c r="Q9" s="10" t="s">
         <v>15</v>
       </c>
       <c r="R9" s="3" t="s">
         <v>108</v>
       </c>
-      <c r="S9" s="10" t="s">
+      <c r="S9" s="11" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="10" spans="1:19">
+      <c r="A10" s="3" t="s">
+        <v>124</v>
+      </c>
+      <c r="B10" s="3">
+        <v>0</v>
+      </c>
+      <c r="C10" s="3" t="s">
+        <v>124</v>
+      </c>
+      <c r="D10" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="E10" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="F10" s="3">
+        <v>12</v>
+      </c>
+      <c r="G10" s="3" t="s">
+        <v>125</v>
+      </c>
+      <c r="H10" s="3"/>
+      <c r="I10" s="3"/>
+      <c r="J10" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="K10" s="3">
+        <v>1</v>
+      </c>
+      <c r="L10" s="3" t="s">
+        <v>107</v>
+      </c>
+      <c r="M10" s="3" t="s">
+        <v>124</v>
+      </c>
+      <c r="N10" s="3" t="s">
+        <v>124</v>
+      </c>
+      <c r="O10" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="P10" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="Q10" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="R10" s="3" t="s">
+        <v>108</v>
+      </c>
+      <c r="S10" s="3" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="11" spans="1:19">
+      <c r="A11" s="3" t="s">
+        <v>126</v>
+      </c>
+      <c r="B11" s="3">
+        <v>0</v>
+      </c>
+      <c r="C11" s="3" t="s">
+        <v>126</v>
+      </c>
+      <c r="D11" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="E11" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="F11" s="3">
+        <v>12</v>
+      </c>
+      <c r="G11" s="3" t="s">
+        <v>125</v>
+      </c>
+      <c r="H11" s="3"/>
+      <c r="I11" s="3"/>
+      <c r="J11" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="K11" s="3">
+        <v>4</v>
+      </c>
+      <c r="L11" s="3" t="s">
+        <v>107</v>
+      </c>
+      <c r="M11" s="3" t="s">
+        <v>126</v>
+      </c>
+      <c r="N11" s="3" t="s">
+        <v>126</v>
+      </c>
+      <c r="O11" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="P11" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="Q11" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="R11" s="3" t="s">
+        <v>108</v>
+      </c>
+      <c r="S11" s="3" t="s">
         <v>109</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <headerFooter/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Fixed Failures In OpenSoAmend SalesInvoices Grn PO PR POA PriceList Functions
Fixed Failures In OpenSoAmend SalesInvoices Grn PO PR POA PriceList Functions
</commit_message>
<xml_diff>
--- a/testdata/ItemDetails.xlsx
+++ b/testdata/ItemDetails.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="19200" windowHeight="6920" firstSheet="7" activeTab="10"/>
+    <workbookView windowWidth="23040" windowHeight="9120"/>
   </bookViews>
   <sheets>
     <sheet name="PR Details" sheetId="1" r:id="rId1"/>
@@ -19,6 +19,7 @@
     <sheet name="Customer SO Details" sheetId="10" r:id="rId10"/>
     <sheet name="Open Sales" sheetId="11" r:id="rId11"/>
     <sheet name="SI Details" sheetId="12" r:id="rId12"/>
+    <sheet name="MRTOMRV Data" sheetId="13" r:id="rId13"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -38,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="521" uniqueCount="189">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="528" uniqueCount="194">
   <si>
     <t>ITEM_NAME</t>
   </si>
@@ -112,7 +113,7 @@
     <t>PRODUCTION  100</t>
   </si>
   <si>
-    <t>CUSTOMS DUTY - RM</t>
+    <t>CHARGES ACCT</t>
   </si>
   <si>
     <t>ITEMID</t>
@@ -606,6 +607,21 @@
   </si>
   <si>
     <t>SEZ-Unit</t>
+  </si>
+  <si>
+    <t>Item</t>
+  </si>
+  <si>
+    <t>WareHouse</t>
+  </si>
+  <si>
+    <t>GWL_ITEM_STOCK_01</t>
+  </si>
+  <si>
+    <t>RM KD</t>
+  </si>
+  <si>
+    <t>GWL_ITEM_STOCK_04</t>
   </si>
 </sst>
 </file>
@@ -618,8 +634,16 @@
     <numFmt numFmtId="178" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
     <numFmt numFmtId="179" formatCode="_ &quot;₹&quot;* #,##0_ ;_ &quot;₹&quot;* \-#,##0_ ;_ &quot;₹&quot;* &quot;-&quot;_ ;_ @_ "/>
   </numFmts>
-  <fonts count="28">
+  <fonts count="29">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -1168,153 +1192,156 @@
     <xf numFmtId="179" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="2" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="6" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="7" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="7" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="8" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="6" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="7" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="7" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="8" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="29">
+  <cellXfs count="28">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1">
@@ -1323,23 +1350,17 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
@@ -1348,7 +1369,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1">
@@ -1357,34 +1378,34 @@
     <xf numFmtId="49" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="49" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="49" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="49" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="49" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="justify" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -1922,338 +1943,338 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1:J20"/>
-  <sheetFormatPr defaultColWidth="8.70909090909091" defaultRowHeight="14.5"/>
+  <sheetFormatPr defaultColWidth="8.71296296296296" defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="20.7090909090909" customWidth="1"/>
-    <col min="2" max="3" width="12.7090909090909" customWidth="1"/>
-    <col min="4" max="4" width="14.7090909090909" customWidth="1"/>
-    <col min="5" max="5" width="9.85454545454546" customWidth="1"/>
-    <col min="6" max="6" width="14.1363636363636" customWidth="1"/>
-    <col min="7" max="7" width="14.8545454545455" customWidth="1"/>
-    <col min="8" max="8" width="22.2818181818182" customWidth="1"/>
-    <col min="9" max="9" width="14.4272727272727" customWidth="1"/>
+    <col min="1" max="1" width="20.712962962963" customWidth="1"/>
+    <col min="2" max="3" width="12.712962962963" customWidth="1"/>
+    <col min="4" max="4" width="14.712962962963" customWidth="1"/>
+    <col min="5" max="5" width="9.85185185185185" customWidth="1"/>
+    <col min="6" max="6" width="14.1388888888889" customWidth="1"/>
+    <col min="7" max="7" width="14.8518518518519" customWidth="1"/>
+    <col min="8" max="8" width="22.2777777777778" customWidth="1"/>
+    <col min="9" max="9" width="14.4259259259259" customWidth="1"/>
     <col min="10" max="10" width="13" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:10">
-      <c r="A1" s="25" t="s">
+      <c r="A1" s="24" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="25" t="s">
+      <c r="B1" s="24" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="25" t="s">
+      <c r="C1" s="24" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="25" t="s">
+      <c r="D1" s="24" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="25" t="s">
+      <c r="E1" s="24" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="25" t="s">
+      <c r="F1" s="24" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="25" t="s">
+      <c r="G1" s="24" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="25" t="s">
+      <c r="H1" s="24" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="25" t="s">
+      <c r="I1" s="24" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="25" t="s">
+      <c r="J1" s="24" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="2" s="24" customFormat="1" ht="21" spans="1:10">
-      <c r="A2" s="26" t="s">
+    <row r="2" s="23" customFormat="1" ht="20.4" spans="1:10">
+      <c r="A2" s="25" t="s">
         <v>10</v>
       </c>
-      <c r="B2" s="27" t="s">
+      <c r="B2" s="26" t="s">
         <v>11</v>
       </c>
-      <c r="C2" s="27" t="s">
+      <c r="C2" s="26" t="s">
         <v>12</v>
       </c>
-      <c r="D2" s="26" t="s">
+      <c r="D2" s="25" t="s">
         <v>13</v>
       </c>
-      <c r="E2" s="26">
+      <c r="E2" s="25">
         <v>1</v>
       </c>
-      <c r="F2" s="26" t="s">
+      <c r="F2" s="25" t="s">
         <v>14</v>
       </c>
-      <c r="G2" s="26">
+      <c r="G2" s="25">
         <v>1010301033</v>
       </c>
-      <c r="H2" s="26" t="s">
+      <c r="H2" s="25" t="s">
         <v>15</v>
       </c>
-      <c r="I2" s="26" t="s">
+      <c r="I2" s="25" t="s">
         <v>16</v>
       </c>
-      <c r="J2" s="26" t="s">
+      <c r="J2" s="25" t="s">
         <v>17</v>
       </c>
     </row>
     <row r="3" ht="15" customHeight="1" spans="1:10">
-      <c r="A3" s="26" t="s">
+      <c r="A3" s="25" t="s">
         <v>18</v>
       </c>
-      <c r="B3" s="27" t="s">
+      <c r="B3" s="26" t="s">
         <v>11</v>
       </c>
-      <c r="C3" s="27" t="s">
+      <c r="C3" s="26" t="s">
         <v>12</v>
       </c>
-      <c r="D3" s="26" t="s">
+      <c r="D3" s="25" t="s">
         <v>19</v>
       </c>
-      <c r="E3" s="26">
+      <c r="E3" s="25">
         <v>6</v>
       </c>
-      <c r="F3" s="27" t="s">
+      <c r="F3" s="26" t="s">
         <v>20</v>
       </c>
-      <c r="G3" s="26">
+      <c r="G3" s="25">
         <v>1010301033</v>
       </c>
-      <c r="H3" s="26" t="s">
+      <c r="H3" s="25" t="s">
         <v>15</v>
       </c>
-      <c r="I3" s="26" t="s">
+      <c r="I3" s="25" t="s">
         <v>16</v>
       </c>
-      <c r="J3" s="26" t="s">
+      <c r="J3" s="25" t="s">
         <v>17</v>
       </c>
     </row>
     <row r="4" spans="1:10">
-      <c r="A4" s="26" t="s">
+      <c r="A4" s="25" t="s">
         <v>21</v>
       </c>
-      <c r="B4" s="27" t="s">
+      <c r="B4" s="26" t="s">
         <v>22</v>
       </c>
-      <c r="C4" s="27" t="s">
+      <c r="C4" s="26" t="s">
         <v>22</v>
       </c>
-      <c r="D4" s="26" t="s">
+      <c r="D4" s="25" t="s">
         <v>23</v>
       </c>
-      <c r="E4" s="26">
+      <c r="E4" s="25">
         <v>1</v>
       </c>
-      <c r="F4" s="27" t="s">
+      <c r="F4" s="26" t="s">
         <v>14</v>
       </c>
-      <c r="G4" s="26">
-        <v>5010101060</v>
-      </c>
-      <c r="H4" s="26" t="s">
+      <c r="G4" s="25">
+        <v>5010100004</v>
+      </c>
+      <c r="H4" s="25" t="s">
         <v>24</v>
       </c>
-      <c r="I4" s="26" t="s">
+      <c r="I4" s="25" t="s">
         <v>16</v>
       </c>
-      <c r="J4" s="26" t="s">
+      <c r="J4" s="25" t="s">
         <v>17</v>
       </c>
     </row>
     <row r="5" spans="1:10">
-      <c r="A5" s="28"/>
-      <c r="B5" s="28"/>
-      <c r="C5" s="28"/>
-      <c r="D5" s="28"/>
-      <c r="E5" s="28"/>
-      <c r="F5" s="28"/>
-      <c r="G5" s="28"/>
-      <c r="H5" s="28"/>
-      <c r="I5" s="28"/>
-      <c r="J5" s="28"/>
+      <c r="A5" s="27"/>
+      <c r="B5" s="27"/>
+      <c r="C5" s="27"/>
+      <c r="D5" s="27"/>
+      <c r="E5" s="27"/>
+      <c r="F5" s="27"/>
+      <c r="G5" s="27"/>
+      <c r="H5" s="27"/>
+      <c r="I5" s="27"/>
+      <c r="J5" s="27"/>
     </row>
     <row r="6" spans="1:10">
-      <c r="A6" s="28"/>
-      <c r="B6" s="28"/>
-      <c r="C6" s="28"/>
-      <c r="D6" s="28"/>
-      <c r="E6" s="28"/>
-      <c r="F6" s="28"/>
-      <c r="G6" s="28"/>
-      <c r="H6" s="28"/>
-      <c r="I6" s="28"/>
-      <c r="J6" s="28"/>
+      <c r="A6" s="27"/>
+      <c r="B6" s="27"/>
+      <c r="C6" s="27"/>
+      <c r="D6" s="27"/>
+      <c r="E6" s="27"/>
+      <c r="F6" s="27"/>
+      <c r="G6" s="27"/>
+      <c r="H6" s="27"/>
+      <c r="I6" s="27"/>
+      <c r="J6" s="27"/>
     </row>
     <row r="7" spans="1:10">
-      <c r="A7" s="28"/>
-      <c r="B7" s="28"/>
-      <c r="C7" s="28"/>
-      <c r="D7" s="28"/>
-      <c r="E7" s="28"/>
-      <c r="F7" s="28"/>
-      <c r="G7" s="28"/>
-      <c r="H7" s="28"/>
-      <c r="I7" s="28"/>
-      <c r="J7" s="28"/>
+      <c r="A7" s="27"/>
+      <c r="B7" s="27"/>
+      <c r="C7" s="27"/>
+      <c r="D7" s="27"/>
+      <c r="E7" s="27"/>
+      <c r="F7" s="27"/>
+      <c r="G7" s="27"/>
+      <c r="H7" s="27"/>
+      <c r="I7" s="27"/>
+      <c r="J7" s="27"/>
     </row>
     <row r="8" spans="1:10">
-      <c r="A8" s="28"/>
-      <c r="B8" s="28"/>
-      <c r="C8" s="28"/>
-      <c r="D8" s="28"/>
-      <c r="E8" s="28"/>
-      <c r="F8" s="28"/>
-      <c r="G8" s="28"/>
-      <c r="H8" s="28"/>
-      <c r="I8" s="28"/>
-      <c r="J8" s="28"/>
+      <c r="A8" s="27"/>
+      <c r="B8" s="27"/>
+      <c r="C8" s="27"/>
+      <c r="D8" s="27"/>
+      <c r="E8" s="27"/>
+      <c r="F8" s="27"/>
+      <c r="G8" s="27"/>
+      <c r="H8" s="27"/>
+      <c r="I8" s="27"/>
+      <c r="J8" s="27"/>
     </row>
     <row r="9" spans="1:10">
-      <c r="A9" s="28"/>
-      <c r="B9" s="28"/>
-      <c r="C9" s="28"/>
-      <c r="D9" s="28"/>
-      <c r="E9" s="28"/>
-      <c r="F9" s="28"/>
-      <c r="G9" s="28"/>
-      <c r="H9" s="28"/>
-      <c r="I9" s="28"/>
-      <c r="J9" s="28"/>
+      <c r="A9" s="27"/>
+      <c r="B9" s="27"/>
+      <c r="C9" s="27"/>
+      <c r="D9" s="27"/>
+      <c r="E9" s="27"/>
+      <c r="F9" s="27"/>
+      <c r="G9" s="27"/>
+      <c r="H9" s="27"/>
+      <c r="I9" s="27"/>
+      <c r="J9" s="27"/>
     </row>
     <row r="10" spans="1:10">
-      <c r="A10" s="28"/>
-      <c r="B10" s="28"/>
-      <c r="C10" s="28"/>
-      <c r="D10" s="28"/>
-      <c r="E10" s="28"/>
-      <c r="F10" s="28"/>
-      <c r="G10" s="28"/>
-      <c r="H10" s="28"/>
-      <c r="I10" s="28"/>
-      <c r="J10" s="28"/>
+      <c r="A10" s="27"/>
+      <c r="B10" s="27"/>
+      <c r="C10" s="27"/>
+      <c r="D10" s="27"/>
+      <c r="E10" s="27"/>
+      <c r="F10" s="27"/>
+      <c r="G10" s="27"/>
+      <c r="H10" s="27"/>
+      <c r="I10" s="27"/>
+      <c r="J10" s="27"/>
     </row>
     <row r="11" spans="1:10">
-      <c r="A11" s="28"/>
-      <c r="B11" s="28"/>
-      <c r="C11" s="28"/>
-      <c r="D11" s="28"/>
-      <c r="E11" s="28"/>
-      <c r="F11" s="28"/>
-      <c r="G11" s="28"/>
-      <c r="H11" s="28"/>
-      <c r="I11" s="28"/>
-      <c r="J11" s="28"/>
+      <c r="A11" s="27"/>
+      <c r="B11" s="27"/>
+      <c r="C11" s="27"/>
+      <c r="D11" s="27"/>
+      <c r="E11" s="27"/>
+      <c r="F11" s="27"/>
+      <c r="G11" s="27"/>
+      <c r="H11" s="27"/>
+      <c r="I11" s="27"/>
+      <c r="J11" s="27"/>
     </row>
     <row r="12" spans="1:10">
-      <c r="A12" s="28"/>
-      <c r="B12" s="28"/>
-      <c r="C12" s="28"/>
-      <c r="D12" s="28"/>
-      <c r="E12" s="28"/>
-      <c r="F12" s="28"/>
-      <c r="G12" s="28"/>
-      <c r="H12" s="28"/>
-      <c r="I12" s="28"/>
-      <c r="J12" s="28"/>
+      <c r="A12" s="27"/>
+      <c r="B12" s="27"/>
+      <c r="C12" s="27"/>
+      <c r="D12" s="27"/>
+      <c r="E12" s="27"/>
+      <c r="F12" s="27"/>
+      <c r="G12" s="27"/>
+      <c r="H12" s="27"/>
+      <c r="I12" s="27"/>
+      <c r="J12" s="27"/>
     </row>
     <row r="13" spans="1:10">
-      <c r="A13" s="28"/>
-      <c r="B13" s="28"/>
-      <c r="C13" s="28"/>
-      <c r="D13" s="28"/>
-      <c r="E13" s="28"/>
-      <c r="F13" s="28"/>
-      <c r="G13" s="28"/>
-      <c r="H13" s="28"/>
-      <c r="I13" s="28"/>
-      <c r="J13" s="28"/>
+      <c r="A13" s="27"/>
+      <c r="B13" s="27"/>
+      <c r="C13" s="27"/>
+      <c r="D13" s="27"/>
+      <c r="E13" s="27"/>
+      <c r="F13" s="27"/>
+      <c r="G13" s="27"/>
+      <c r="H13" s="27"/>
+      <c r="I13" s="27"/>
+      <c r="J13" s="27"/>
     </row>
     <row r="14" spans="1:10">
-      <c r="A14" s="28"/>
-      <c r="B14" s="28"/>
-      <c r="C14" s="28"/>
-      <c r="D14" s="28"/>
-      <c r="E14" s="28"/>
-      <c r="F14" s="28"/>
-      <c r="G14" s="28"/>
-      <c r="H14" s="28"/>
-      <c r="I14" s="28"/>
-      <c r="J14" s="28"/>
+      <c r="A14" s="27"/>
+      <c r="B14" s="27"/>
+      <c r="C14" s="27"/>
+      <c r="D14" s="27"/>
+      <c r="E14" s="27"/>
+      <c r="F14" s="27"/>
+      <c r="G14" s="27"/>
+      <c r="H14" s="27"/>
+      <c r="I14" s="27"/>
+      <c r="J14" s="27"/>
     </row>
     <row r="15" spans="1:10">
-      <c r="A15" s="28"/>
-      <c r="B15" s="28"/>
-      <c r="C15" s="28"/>
-      <c r="D15" s="28"/>
-      <c r="E15" s="28"/>
-      <c r="F15" s="28"/>
-      <c r="G15" s="28"/>
-      <c r="H15" s="28"/>
-      <c r="I15" s="28"/>
-      <c r="J15" s="28"/>
+      <c r="A15" s="27"/>
+      <c r="B15" s="27"/>
+      <c r="C15" s="27"/>
+      <c r="D15" s="27"/>
+      <c r="E15" s="27"/>
+      <c r="F15" s="27"/>
+      <c r="G15" s="27"/>
+      <c r="H15" s="27"/>
+      <c r="I15" s="27"/>
+      <c r="J15" s="27"/>
     </row>
     <row r="16" spans="1:10">
-      <c r="A16" s="28"/>
-      <c r="B16" s="28"/>
-      <c r="C16" s="28"/>
-      <c r="D16" s="28"/>
-      <c r="E16" s="28"/>
-      <c r="F16" s="28"/>
-      <c r="G16" s="28"/>
-      <c r="H16" s="28"/>
-      <c r="I16" s="28"/>
-      <c r="J16" s="28"/>
+      <c r="A16" s="27"/>
+      <c r="B16" s="27"/>
+      <c r="C16" s="27"/>
+      <c r="D16" s="27"/>
+      <c r="E16" s="27"/>
+      <c r="F16" s="27"/>
+      <c r="G16" s="27"/>
+      <c r="H16" s="27"/>
+      <c r="I16" s="27"/>
+      <c r="J16" s="27"/>
     </row>
     <row r="17" spans="1:10">
-      <c r="A17" s="28"/>
-      <c r="B17" s="28"/>
-      <c r="C17" s="28"/>
-      <c r="D17" s="28"/>
-      <c r="E17" s="28"/>
-      <c r="F17" s="28"/>
-      <c r="G17" s="28"/>
-      <c r="H17" s="28"/>
-      <c r="I17" s="28"/>
-      <c r="J17" s="28"/>
+      <c r="A17" s="27"/>
+      <c r="B17" s="27"/>
+      <c r="C17" s="27"/>
+      <c r="D17" s="27"/>
+      <c r="E17" s="27"/>
+      <c r="F17" s="27"/>
+      <c r="G17" s="27"/>
+      <c r="H17" s="27"/>
+      <c r="I17" s="27"/>
+      <c r="J17" s="27"/>
     </row>
     <row r="18" spans="1:10">
-      <c r="A18" s="28"/>
-      <c r="B18" s="28"/>
-      <c r="C18" s="28"/>
-      <c r="D18" s="28"/>
-      <c r="E18" s="28"/>
-      <c r="F18" s="28"/>
-      <c r="G18" s="28"/>
-      <c r="H18" s="28"/>
-      <c r="I18" s="28"/>
-      <c r="J18" s="28"/>
+      <c r="A18" s="27"/>
+      <c r="B18" s="27"/>
+      <c r="C18" s="27"/>
+      <c r="D18" s="27"/>
+      <c r="E18" s="27"/>
+      <c r="F18" s="27"/>
+      <c r="G18" s="27"/>
+      <c r="H18" s="27"/>
+      <c r="I18" s="27"/>
+      <c r="J18" s="27"/>
     </row>
     <row r="19" spans="1:10">
-      <c r="A19" s="28"/>
-      <c r="B19" s="28"/>
-      <c r="C19" s="28"/>
-      <c r="D19" s="28"/>
-      <c r="E19" s="28"/>
-      <c r="F19" s="28"/>
-      <c r="G19" s="28"/>
-      <c r="H19" s="28"/>
-      <c r="I19" s="28"/>
-      <c r="J19" s="28"/>
+      <c r="A19" s="27"/>
+      <c r="B19" s="27"/>
+      <c r="C19" s="27"/>
+      <c r="D19" s="27"/>
+      <c r="E19" s="27"/>
+      <c r="F19" s="27"/>
+      <c r="G19" s="27"/>
+      <c r="H19" s="27"/>
+      <c r="I19" s="27"/>
+      <c r="J19" s="27"/>
     </row>
     <row r="20" spans="1:10">
-      <c r="A20" s="28"/>
-      <c r="B20" s="28"/>
-      <c r="C20" s="28"/>
-      <c r="D20" s="28"/>
-      <c r="E20" s="28"/>
-      <c r="F20" s="28"/>
-      <c r="G20" s="28"/>
-      <c r="H20" s="28"/>
-      <c r="I20" s="28"/>
-      <c r="J20" s="28"/>
+      <c r="A20" s="27"/>
+      <c r="B20" s="27"/>
+      <c r="C20" s="27"/>
+      <c r="D20" s="27"/>
+      <c r="E20" s="27"/>
+      <c r="F20" s="27"/>
+      <c r="G20" s="27"/>
+      <c r="H20" s="27"/>
+      <c r="I20" s="27"/>
+      <c r="J20" s="27"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2265,123 +2286,123 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1:K3"/>
-  <sheetFormatPr defaultColWidth="8.85454545454546" defaultRowHeight="14.5" outlineLevelRow="2"/>
+  <sheetFormatPr defaultColWidth="8.85185185185185" defaultRowHeight="14.4" outlineLevelRow="2"/>
   <cols>
     <col min="1" max="1" width="9" customWidth="1"/>
-    <col min="2" max="2" width="25.7090909090909" customWidth="1"/>
-    <col min="3" max="3" width="12.4272727272727" customWidth="1"/>
-    <col min="4" max="4" width="16.2818181818182" customWidth="1"/>
-    <col min="5" max="5" width="20.2818181818182" customWidth="1"/>
-    <col min="6" max="6" width="25.7090909090909" customWidth="1"/>
-    <col min="7" max="7" width="12.2818181818182" customWidth="1"/>
-    <col min="8" max="8" width="14.5727272727273" customWidth="1"/>
-    <col min="9" max="9" width="28.5727272727273" customWidth="1"/>
+    <col min="2" max="2" width="25.712962962963" customWidth="1"/>
+    <col min="3" max="3" width="12.4259259259259" customWidth="1"/>
+    <col min="4" max="4" width="16.2777777777778" customWidth="1"/>
+    <col min="5" max="5" width="20.2777777777778" customWidth="1"/>
+    <col min="6" max="6" width="25.712962962963" customWidth="1"/>
+    <col min="7" max="7" width="12.2777777777778" customWidth="1"/>
+    <col min="8" max="8" width="14.5740740740741" customWidth="1"/>
+    <col min="9" max="9" width="28.5740740740741" customWidth="1"/>
     <col min="10" max="10" width="23" customWidth="1"/>
-    <col min="11" max="11" width="14.7090909090909" customWidth="1"/>
+    <col min="11" max="11" width="14.712962962963" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:11">
-      <c r="A1" s="10" t="s">
+      <c r="A1" s="7" t="s">
         <v>127</v>
       </c>
-      <c r="B1" s="10" t="s">
+      <c r="B1" s="7" t="s">
         <v>128</v>
       </c>
-      <c r="C1" s="10" t="s">
+      <c r="C1" s="7" t="s">
         <v>129</v>
       </c>
-      <c r="D1" s="10" t="s">
+      <c r="D1" s="7" t="s">
         <v>130</v>
       </c>
-      <c r="E1" s="10" t="s">
+      <c r="E1" s="7" t="s">
         <v>131</v>
       </c>
-      <c r="F1" s="11" t="s">
+      <c r="F1" s="10" t="s">
         <v>132</v>
       </c>
-      <c r="G1" s="11" t="s">
+      <c r="G1" s="10" t="s">
         <v>133</v>
       </c>
-      <c r="H1" s="11" t="s">
+      <c r="H1" s="10" t="s">
         <v>134</v>
       </c>
-      <c r="I1" s="11" t="s">
+      <c r="I1" s="10" t="s">
         <v>135</v>
       </c>
-      <c r="J1" s="11" t="s">
+      <c r="J1" s="10" t="s">
         <v>136</v>
       </c>
-      <c r="K1" s="11" t="s">
+      <c r="K1" s="10" t="s">
         <v>137</v>
       </c>
     </row>
     <row r="2" spans="1:11">
-      <c r="A2" s="10" t="s">
+      <c r="A2" s="7" t="s">
         <v>138</v>
       </c>
-      <c r="B2" s="10" t="s">
+      <c r="B2" s="7" t="s">
         <v>139</v>
       </c>
-      <c r="C2" s="10" t="s">
+      <c r="C2" s="7" t="s">
         <v>140</v>
       </c>
-      <c r="D2" s="10" t="s">
+      <c r="D2" s="7" t="s">
         <v>141</v>
       </c>
-      <c r="E2" s="10" t="s">
+      <c r="E2" s="7" t="s">
         <v>142</v>
       </c>
-      <c r="F2" s="3" t="s">
+      <c r="F2" s="2" t="s">
         <v>139</v>
       </c>
-      <c r="G2" s="3" t="s">
+      <c r="G2" s="2" t="s">
         <v>143</v>
       </c>
-      <c r="H2" s="3" t="s">
+      <c r="H2" s="2" t="s">
         <v>144</v>
       </c>
-      <c r="I2" s="3" t="s">
+      <c r="I2" s="2" t="s">
         <v>145</v>
       </c>
-      <c r="J2" s="3" t="s">
+      <c r="J2" s="2" t="s">
         <v>146</v>
       </c>
-      <c r="K2" s="3" t="s">
+      <c r="K2" s="2" t="s">
         <v>147</v>
       </c>
     </row>
     <row r="3" spans="1:11">
-      <c r="A3" s="12" t="s">
+      <c r="A3" s="11" t="s">
         <v>148</v>
       </c>
-      <c r="B3" s="3" t="s">
+      <c r="B3" s="2" t="s">
         <v>149</v>
       </c>
-      <c r="C3" s="10" t="s">
+      <c r="C3" s="7" t="s">
         <v>140</v>
       </c>
-      <c r="D3" s="3" t="s">
+      <c r="D3" s="2" t="s">
         <v>150</v>
       </c>
-      <c r="E3" s="3" t="s">
+      <c r="E3" s="2" t="s">
         <v>150</v>
       </c>
-      <c r="F3" s="3" t="s">
+      <c r="F3" s="2" t="s">
         <v>149</v>
       </c>
-      <c r="G3" s="3" t="s">
+      <c r="G3" s="2" t="s">
         <v>151</v>
       </c>
-      <c r="H3" s="3" t="s">
+      <c r="H3" s="2" t="s">
         <v>151</v>
       </c>
-      <c r="I3" s="3" t="s">
+      <c r="I3" s="2" t="s">
         <v>152</v>
       </c>
-      <c r="J3" s="3" t="s">
+      <c r="J3" s="2" t="s">
         <v>146</v>
       </c>
-      <c r="K3" s="3" t="s">
+      <c r="K3" s="2" t="s">
         <v>147</v>
       </c>
     </row>
@@ -2395,37 +2416,37 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1:E4"/>
-  <sheetFormatPr defaultColWidth="8.85454545454546" defaultRowHeight="14.5" outlineLevelRow="3" outlineLevelCol="4"/>
+  <sheetFormatPr defaultColWidth="8.85185185185185" defaultRowHeight="14.4" outlineLevelRow="3" outlineLevelCol="4"/>
   <cols>
-    <col min="1" max="1" width="13.5727272727273" customWidth="1"/>
+    <col min="1" max="1" width="13.5740740740741" customWidth="1"/>
     <col min="2" max="2" width="6" customWidth="1"/>
-    <col min="3" max="3" width="14.4272727272727" customWidth="1"/>
-    <col min="4" max="4" width="18.1363636363636" customWidth="1"/>
-    <col min="5" max="5" width="19.5727272727273" customWidth="1"/>
+    <col min="3" max="3" width="14.4259259259259" customWidth="1"/>
+    <col min="4" max="4" width="18.1388888888889" customWidth="1"/>
+    <col min="5" max="5" width="19.5740740740741" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5">
-      <c r="A1" s="6" t="s">
+      <c r="A1" s="7" t="s">
         <v>153</v>
       </c>
-      <c r="B1" s="7" t="s">
+      <c r="B1" s="2" t="s">
         <v>154</v>
       </c>
-      <c r="C1" s="7" t="s">
+      <c r="C1" s="2" t="s">
         <v>155</v>
       </c>
-      <c r="D1" s="7" t="s">
+      <c r="D1" s="2" t="s">
         <v>156</v>
       </c>
-      <c r="E1" s="7" t="s">
+      <c r="E1" s="2" t="s">
         <v>157</v>
       </c>
     </row>
     <row r="2" spans="1:5">
-      <c r="A2" s="6" t="s">
+      <c r="A2" s="7" t="s">
         <v>158</v>
       </c>
-      <c r="B2" s="6" t="s">
+      <c r="B2" s="7" t="s">
         <v>159</v>
       </c>
       <c r="C2" s="8" t="s">
@@ -2434,41 +2455,41 @@
       <c r="D2" s="9" t="s">
         <v>139</v>
       </c>
-      <c r="E2" s="6" t="s">
+      <c r="E2" s="7" t="s">
         <v>160</v>
       </c>
     </row>
     <row r="3" spans="1:5">
-      <c r="A3" s="7" t="s">
+      <c r="A3" s="2" t="s">
         <v>161</v>
       </c>
-      <c r="B3" s="7" t="s">
+      <c r="B3" s="2" t="s">
         <v>162</v>
       </c>
-      <c r="C3" s="7" t="s">
+      <c r="C3" s="2" t="s">
         <v>163</v>
       </c>
-      <c r="D3" s="7" t="s">
+      <c r="D3" s="2" t="s">
         <v>164</v>
       </c>
-      <c r="E3" s="7" t="s">
+      <c r="E3" s="2" t="s">
         <v>165</v>
       </c>
     </row>
     <row r="4" spans="1:5">
-      <c r="A4" s="7" t="s">
+      <c r="A4" s="2" t="s">
         <v>166</v>
       </c>
-      <c r="B4" s="7" t="s">
+      <c r="B4" s="2" t="s">
         <v>167</v>
       </c>
-      <c r="C4" s="7" t="s">
+      <c r="C4" s="2" t="s">
         <v>168</v>
       </c>
-      <c r="D4" s="7" t="s">
+      <c r="D4" s="2" t="s">
         <v>169</v>
       </c>
-      <c r="E4" s="7" t="s">
+      <c r="E4" s="2" t="s">
         <v>170</v>
       </c>
     </row>
@@ -2482,199 +2503,249 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1:G8"/>
-  <sheetFormatPr defaultColWidth="8.85454545454546" defaultRowHeight="14.5" outlineLevelRow="7" outlineLevelCol="6"/>
+  <sheetFormatPr defaultColWidth="8.85185185185185" defaultRowHeight="14.4" outlineLevelRow="7" outlineLevelCol="6"/>
   <cols>
-    <col min="1" max="1" width="25.7090909090909" customWidth="1"/>
-    <col min="2" max="2" width="8.85454545454546" customWidth="1"/>
-    <col min="3" max="3" width="12.2818181818182" customWidth="1"/>
-    <col min="4" max="4" width="7.13636363636364" customWidth="1"/>
-    <col min="5" max="5" width="5.28181818181818" customWidth="1"/>
-    <col min="6" max="6" width="17.4272727272727" customWidth="1"/>
-    <col min="7" max="7" width="12.4272727272727" customWidth="1"/>
+    <col min="1" max="1" width="25.712962962963" customWidth="1"/>
+    <col min="2" max="2" width="8.85185185185185" customWidth="1"/>
+    <col min="3" max="3" width="12.2777777777778" customWidth="1"/>
+    <col min="4" max="4" width="7.13888888888889" customWidth="1"/>
+    <col min="5" max="5" width="5.27777777777778" customWidth="1"/>
+    <col min="6" max="6" width="17.4259259259259" customWidth="1"/>
+    <col min="7" max="7" width="12.4259259259259" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7">
+      <c r="A1" s="3" t="s">
+        <v>171</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>172</v>
+      </c>
+      <c r="C1" s="4" t="s">
+        <v>173</v>
+      </c>
+      <c r="D1" s="4" t="s">
+        <v>174</v>
+      </c>
+      <c r="E1" s="4" t="s">
+        <v>175</v>
+      </c>
+      <c r="F1" s="3" t="s">
+        <v>176</v>
+      </c>
+      <c r="G1" s="3" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7">
+      <c r="A2" s="2" t="s">
+        <v>178</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>179</v>
+      </c>
+      <c r="C2" s="5" t="s">
+        <v>180</v>
+      </c>
+      <c r="D2" s="5" t="s">
+        <v>158</v>
+      </c>
+      <c r="E2" s="5" t="s">
+        <v>159</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>181</v>
+      </c>
+      <c r="G2" s="2" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7">
+      <c r="A3" s="2" t="s">
+        <v>149</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>183</v>
+      </c>
+      <c r="C3" s="5" t="s">
+        <v>180</v>
+      </c>
+      <c r="D3" s="5" t="s">
+        <v>158</v>
+      </c>
+      <c r="E3" s="5" t="s">
+        <v>159</v>
+      </c>
+      <c r="F3" s="2" t="s">
+        <v>150</v>
+      </c>
+      <c r="G3" s="2" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7">
+      <c r="A4" s="2" t="s">
+        <v>184</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>179</v>
+      </c>
+      <c r="C4" s="5" t="s">
+        <v>180</v>
+      </c>
+      <c r="D4" s="5" t="s">
+        <v>158</v>
+      </c>
+      <c r="E4" s="5" t="s">
+        <v>159</v>
+      </c>
+      <c r="F4" s="2" t="s">
+        <v>181</v>
+      </c>
+      <c r="G4" s="2" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7">
+      <c r="A5" s="2" t="s">
+        <v>139</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>179</v>
+      </c>
+      <c r="C5" s="5" t="s">
+        <v>180</v>
+      </c>
+      <c r="D5" s="5" t="s">
+        <v>158</v>
+      </c>
+      <c r="E5" s="5" t="s">
+        <v>159</v>
+      </c>
+      <c r="F5" s="6" t="s">
+        <v>141</v>
+      </c>
+      <c r="G5" s="2" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7">
+      <c r="A6" s="2" t="s">
+        <v>185</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>179</v>
+      </c>
+      <c r="C6" s="5" t="s">
+        <v>180</v>
+      </c>
+      <c r="D6" s="5" t="s">
+        <v>158</v>
+      </c>
+      <c r="E6" s="5" t="s">
+        <v>159</v>
+      </c>
+      <c r="F6" s="2" t="s">
+        <v>141</v>
+      </c>
+      <c r="G6" s="2" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7">
+      <c r="A7" s="2" t="s">
+        <v>186</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>179</v>
+      </c>
+      <c r="C7" s="5" t="s">
+        <v>180</v>
+      </c>
+      <c r="D7" s="5" t="s">
+        <v>158</v>
+      </c>
+      <c r="E7" s="5" t="s">
+        <v>159</v>
+      </c>
+      <c r="F7" s="2" t="s">
+        <v>141</v>
+      </c>
+      <c r="G7" s="2" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7">
+      <c r="A8" s="2" t="s">
+        <v>187</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>179</v>
+      </c>
+      <c r="C8" s="5" t="s">
+        <v>180</v>
+      </c>
+      <c r="D8" s="5" t="s">
+        <v>158</v>
+      </c>
+      <c r="E8" s="5" t="s">
+        <v>159</v>
+      </c>
+      <c r="F8" s="2" t="s">
+        <v>188</v>
+      </c>
+      <c r="G8" s="2" t="s">
+        <v>182</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <headerFooter/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
+  <dimension ref="A1:C3"/>
+  <sheetFormatPr defaultColWidth="8.88888888888889" defaultRowHeight="14.4" outlineLevelRow="2" outlineLevelCol="2"/>
+  <cols>
+    <col min="1" max="1" width="25.5555555555556" customWidth="1"/>
+    <col min="2" max="2" width="15.2222222222222" customWidth="1"/>
+    <col min="3" max="3" width="16.4444444444444" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3">
       <c r="A1" s="1" t="s">
-        <v>171</v>
+        <v>189</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>172</v>
-      </c>
-      <c r="C1" s="2" t="s">
-        <v>173</v>
-      </c>
-      <c r="D1" s="2" t="s">
-        <v>174</v>
-      </c>
-      <c r="E1" s="2" t="s">
-        <v>175</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>176</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>177</v>
-      </c>
-    </row>
-    <row r="2" spans="1:7">
-      <c r="A2" s="3" t="s">
-        <v>178</v>
-      </c>
-      <c r="B2" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="C2" s="4" t="s">
-        <v>180</v>
-      </c>
-      <c r="D2" s="4" t="s">
-        <v>158</v>
-      </c>
-      <c r="E2" s="4" t="s">
-        <v>159</v>
-      </c>
-      <c r="F2" s="3" t="s">
-        <v>181</v>
-      </c>
-      <c r="G2" s="3" t="s">
-        <v>182</v>
-      </c>
-    </row>
-    <row r="3" spans="1:7">
-      <c r="A3" s="3" t="s">
-        <v>149</v>
-      </c>
-      <c r="B3" s="3" t="s">
-        <v>183</v>
-      </c>
-      <c r="C3" s="4" t="s">
-        <v>180</v>
-      </c>
-      <c r="D3" s="4" t="s">
-        <v>158</v>
-      </c>
-      <c r="E3" s="4" t="s">
-        <v>159</v>
-      </c>
-      <c r="F3" s="3" t="s">
-        <v>150</v>
-      </c>
-      <c r="G3" s="3" t="s">
-        <v>140</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7">
-      <c r="A4" s="3" t="s">
-        <v>184</v>
-      </c>
-      <c r="B4" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="C4" s="4" t="s">
-        <v>180</v>
-      </c>
-      <c r="D4" s="4" t="s">
-        <v>158</v>
-      </c>
-      <c r="E4" s="4" t="s">
-        <v>159</v>
-      </c>
-      <c r="F4" s="3" t="s">
-        <v>181</v>
-      </c>
-      <c r="G4" s="3" t="s">
-        <v>182</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7">
-      <c r="A5" s="3" t="s">
-        <v>139</v>
-      </c>
-      <c r="B5" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="C5" s="4" t="s">
-        <v>180</v>
-      </c>
-      <c r="D5" s="4" t="s">
-        <v>158</v>
-      </c>
-      <c r="E5" s="4" t="s">
-        <v>159</v>
-      </c>
-      <c r="F5" s="5" t="s">
-        <v>141</v>
-      </c>
-      <c r="G5" s="3" t="s">
-        <v>140</v>
-      </c>
-    </row>
-    <row r="6" spans="1:7">
-      <c r="A6" s="3" t="s">
-        <v>185</v>
-      </c>
-      <c r="B6" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="C6" s="4" t="s">
-        <v>180</v>
-      </c>
-      <c r="D6" s="4" t="s">
-        <v>158</v>
-      </c>
-      <c r="E6" s="4" t="s">
-        <v>159</v>
-      </c>
-      <c r="F6" s="3" t="s">
-        <v>141</v>
-      </c>
-      <c r="G6" s="3" t="s">
-        <v>182</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7">
-      <c r="A7" s="3" t="s">
-        <v>186</v>
-      </c>
-      <c r="B7" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="C7" s="4" t="s">
-        <v>180</v>
-      </c>
-      <c r="D7" s="4" t="s">
-        <v>158</v>
-      </c>
-      <c r="E7" s="4" t="s">
-        <v>159</v>
-      </c>
-      <c r="F7" s="3" t="s">
-        <v>141</v>
-      </c>
-      <c r="G7" s="3" t="s">
-        <v>182</v>
-      </c>
-    </row>
-    <row r="8" spans="1:7">
-      <c r="A8" s="3" t="s">
-        <v>187</v>
-      </c>
-      <c r="B8" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="C8" s="4" t="s">
-        <v>180</v>
-      </c>
-      <c r="D8" s="4" t="s">
-        <v>158</v>
-      </c>
-      <c r="E8" s="4" t="s">
-        <v>159</v>
-      </c>
-      <c r="F8" s="3" t="s">
-        <v>188</v>
-      </c>
-      <c r="G8" s="3" t="s">
-        <v>182</v>
+        <v>190</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3">
+      <c r="A2" s="2" t="s">
+        <v>191</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>192</v>
+      </c>
+      <c r="C2" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3">
+      <c r="A3" s="2" t="s">
+        <v>193</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>192</v>
+      </c>
+      <c r="C3" s="2">
+        <v>2</v>
       </c>
     </row>
   </sheetData>
@@ -2687,577 +2758,577 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1:T10"/>
-  <sheetFormatPr defaultColWidth="8.70909090909091" defaultRowHeight="14.5"/>
+  <sheetFormatPr defaultColWidth="8.71296296296296" defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="30" customWidth="1"/>
-    <col min="2" max="2" width="36.4272727272727" customWidth="1"/>
+    <col min="2" max="2" width="36.4259259259259" customWidth="1"/>
     <col min="3" max="3" width="6" customWidth="1"/>
-    <col min="4" max="4" width="13.7090909090909" customWidth="1"/>
-    <col min="5" max="5" width="5.28181818181818" customWidth="1"/>
-    <col min="6" max="6" width="17.2818181818182" customWidth="1"/>
-    <col min="7" max="7" width="30.2818181818182" customWidth="1"/>
-    <col min="8" max="8" width="26.8545454545455" customWidth="1"/>
-    <col min="9" max="9" width="17.2818181818182" customWidth="1"/>
-    <col min="10" max="10" width="13.2818181818182" customWidth="1"/>
-    <col min="11" max="11" width="22.7090909090909" customWidth="1"/>
-    <col min="12" max="12" width="12.7090909090909" customWidth="1"/>
-    <col min="13" max="13" width="29.5727272727273" customWidth="1"/>
-    <col min="14" max="14" width="18.2818181818182" customWidth="1"/>
-    <col min="15" max="15" width="16.2818181818182" customWidth="1"/>
-    <col min="16" max="16" width="15.5727272727273" customWidth="1"/>
-    <col min="17" max="17" width="17.7090909090909" customWidth="1"/>
-    <col min="18" max="18" width="24.1363636363636" customWidth="1"/>
-    <col min="19" max="19" width="13.4272727272727" customWidth="1"/>
-    <col min="20" max="20" width="13.5727272727273" customWidth="1"/>
+    <col min="4" max="4" width="13.712962962963" customWidth="1"/>
+    <col min="5" max="5" width="5.27777777777778" customWidth="1"/>
+    <col min="6" max="6" width="17.2777777777778" customWidth="1"/>
+    <col min="7" max="7" width="30.2777777777778" customWidth="1"/>
+    <col min="8" max="8" width="26.8518518518519" customWidth="1"/>
+    <col min="9" max="9" width="17.2777777777778" customWidth="1"/>
+    <col min="10" max="10" width="13.2777777777778" customWidth="1"/>
+    <col min="11" max="11" width="22.712962962963" customWidth="1"/>
+    <col min="12" max="12" width="12.712962962963" customWidth="1"/>
+    <col min="13" max="13" width="29.5740740740741" customWidth="1"/>
+    <col min="14" max="14" width="18.2777777777778" customWidth="1"/>
+    <col min="15" max="15" width="16.2777777777778" customWidth="1"/>
+    <col min="16" max="16" width="15.5740740740741" customWidth="1"/>
+    <col min="17" max="17" width="17.712962962963" customWidth="1"/>
+    <col min="18" max="18" width="24.1388888888889" customWidth="1"/>
+    <col min="19" max="19" width="13.4259259259259" customWidth="1"/>
+    <col min="20" max="20" width="13.5740740740741" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:20">
-      <c r="A1" s="13" t="s">
+      <c r="A1" s="12" t="s">
         <v>25</v>
       </c>
-      <c r="B1" s="13" t="s">
+      <c r="B1" s="12" t="s">
         <v>26</v>
       </c>
-      <c r="C1" s="13" t="s">
+      <c r="C1" s="12" t="s">
         <v>27</v>
       </c>
-      <c r="D1" s="13" t="s">
+      <c r="D1" s="12" t="s">
         <v>28</v>
       </c>
-      <c r="E1" s="13" t="s">
+      <c r="E1" s="12" t="s">
         <v>29</v>
       </c>
-      <c r="F1" s="13" t="s">
+      <c r="F1" s="12" t="s">
         <v>2</v>
       </c>
-      <c r="G1" s="13" t="s">
+      <c r="G1" s="12" t="s">
         <v>1</v>
       </c>
-      <c r="H1" s="13" t="s">
+      <c r="H1" s="12" t="s">
         <v>30</v>
       </c>
-      <c r="I1" s="13" t="s">
+      <c r="I1" s="12" t="s">
         <v>31</v>
       </c>
-      <c r="J1" s="13" t="s">
+      <c r="J1" s="12" t="s">
         <v>32</v>
       </c>
-      <c r="K1" s="13" t="s">
+      <c r="K1" s="12" t="s">
         <v>33</v>
       </c>
-      <c r="L1" s="13" t="s">
+      <c r="L1" s="12" t="s">
         <v>6</v>
       </c>
-      <c r="M1" s="13" t="s">
+      <c r="M1" s="12" t="s">
         <v>7</v>
       </c>
-      <c r="N1" s="13" t="s">
+      <c r="N1" s="12" t="s">
         <v>8</v>
       </c>
-      <c r="O1" s="13" t="s">
+      <c r="O1" s="12" t="s">
         <v>9</v>
       </c>
-      <c r="P1" s="13" t="s">
+      <c r="P1" s="12" t="s">
         <v>34</v>
       </c>
-      <c r="Q1" s="13" t="s">
+      <c r="Q1" s="12" t="s">
         <v>35</v>
       </c>
-      <c r="R1" s="13" t="s">
+      <c r="R1" s="12" t="s">
         <v>36</v>
       </c>
-      <c r="S1" s="13" t="s">
+      <c r="S1" s="12" t="s">
         <v>37</v>
       </c>
-      <c r="T1" s="13" t="s">
+      <c r="T1" s="12" t="s">
         <v>38</v>
       </c>
     </row>
     <row r="2" spans="1:20">
-      <c r="A2" s="13" t="s">
+      <c r="A2" s="12" t="s">
         <v>18</v>
       </c>
-      <c r="B2" s="13" t="s">
+      <c r="B2" s="12" t="s">
         <v>39</v>
       </c>
-      <c r="C2" s="13" t="s">
+      <c r="C2" s="12" t="s">
         <v>20</v>
       </c>
-      <c r="D2" s="13" t="s">
+      <c r="D2" s="12" t="s">
         <v>40</v>
       </c>
-      <c r="E2" s="13">
+      <c r="E2" s="12">
         <v>12</v>
       </c>
-      <c r="F2" s="19" t="s">
+      <c r="F2" s="18" t="s">
         <v>12</v>
       </c>
-      <c r="G2" s="13" t="s">
+      <c r="G2" s="12" t="s">
         <v>11</v>
       </c>
-      <c r="H2" s="13" t="s">
+      <c r="H2" s="12" t="s">
         <v>19</v>
       </c>
-      <c r="I2" s="13" t="s">
+      <c r="I2" s="12" t="s">
         <v>41</v>
       </c>
-      <c r="J2" s="13" t="s">
+      <c r="J2" s="12" t="s">
         <v>14</v>
       </c>
-      <c r="K2" s="13">
+      <c r="K2" s="12">
         <v>6</v>
       </c>
-      <c r="L2" s="13">
+      <c r="L2" s="12">
         <v>1010301033</v>
       </c>
-      <c r="M2" s="13" t="s">
+      <c r="M2" s="12" t="s">
         <v>15</v>
       </c>
-      <c r="N2" s="13" t="s">
+      <c r="N2" s="12" t="s">
         <v>16</v>
       </c>
-      <c r="O2" s="13" t="s">
+      <c r="O2" s="12" t="s">
         <v>17</v>
       </c>
-      <c r="P2" s="13"/>
-      <c r="Q2" s="13"/>
-      <c r="R2" s="13"/>
-      <c r="S2" s="13">
+      <c r="P2" s="12"/>
+      <c r="Q2" s="12"/>
+      <c r="R2" s="12"/>
+      <c r="S2" s="12">
         <v>0</v>
       </c>
-      <c r="T2" s="13"/>
+      <c r="T2" s="12"/>
     </row>
     <row r="3" spans="1:20">
-      <c r="A3" s="13" t="s">
+      <c r="A3" s="12" t="s">
         <v>10</v>
       </c>
-      <c r="B3" s="13" t="s">
+      <c r="B3" s="12" t="s">
         <v>42</v>
       </c>
-      <c r="C3" s="13" t="s">
+      <c r="C3" s="12" t="s">
         <v>14</v>
       </c>
-      <c r="D3" s="20" t="s">
+      <c r="D3" s="19" t="s">
         <v>43</v>
       </c>
-      <c r="E3" s="13">
+      <c r="E3" s="12">
         <v>5</v>
       </c>
-      <c r="F3" s="13" t="s">
+      <c r="F3" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="G3" s="13" t="s">
+      <c r="G3" s="12" t="s">
         <v>11</v>
       </c>
-      <c r="H3" s="13" t="s">
+      <c r="H3" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="I3" s="13" t="s">
+      <c r="I3" s="12" t="s">
         <v>44</v>
       </c>
-      <c r="J3" s="13" t="s">
+      <c r="J3" s="12" t="s">
         <v>14</v>
       </c>
-      <c r="K3" s="13">
+      <c r="K3" s="12">
         <v>1</v>
       </c>
-      <c r="L3" s="13">
+      <c r="L3" s="12">
         <v>1010301033</v>
       </c>
-      <c r="M3" s="13" t="s">
+      <c r="M3" s="12" t="s">
         <v>15</v>
       </c>
-      <c r="N3" s="13" t="s">
+      <c r="N3" s="12" t="s">
         <v>16</v>
       </c>
-      <c r="O3" s="13" t="s">
+      <c r="O3" s="12" t="s">
         <v>17</v>
       </c>
-      <c r="P3" s="13"/>
-      <c r="Q3" s="13"/>
-      <c r="R3" s="13"/>
-      <c r="S3" s="13">
+      <c r="P3" s="12"/>
+      <c r="Q3" s="12"/>
+      <c r="R3" s="12"/>
+      <c r="S3" s="12">
         <v>0</v>
       </c>
-      <c r="T3" s="13"/>
+      <c r="T3" s="12"/>
     </row>
     <row r="4" spans="1:20">
-      <c r="A4" s="13" t="s">
+      <c r="A4" s="12" t="s">
         <v>21</v>
       </c>
-      <c r="B4" s="13" t="s">
+      <c r="B4" s="12" t="s">
         <v>45</v>
       </c>
-      <c r="C4" s="13" t="s">
+      <c r="C4" s="12" t="s">
         <v>14</v>
       </c>
-      <c r="D4" s="13">
+      <c r="D4" s="12">
         <v>123562</v>
       </c>
-      <c r="E4" s="13">
+      <c r="E4" s="12">
         <v>18</v>
       </c>
-      <c r="F4" s="13" t="s">
+      <c r="F4" s="12" t="s">
         <v>22</v>
       </c>
-      <c r="G4" s="13" t="s">
+      <c r="G4" s="12" t="s">
         <v>22</v>
       </c>
-      <c r="H4" s="13" t="s">
+      <c r="H4" s="12" t="s">
         <v>23</v>
       </c>
-      <c r="I4" s="13" t="s">
+      <c r="I4" s="12" t="s">
         <v>44</v>
       </c>
-      <c r="J4" s="13" t="s">
+      <c r="J4" s="12" t="s">
         <v>14</v>
       </c>
-      <c r="K4" s="13">
+      <c r="K4" s="12">
         <v>1</v>
       </c>
-      <c r="L4" s="13">
+      <c r="L4" s="12">
         <v>1011134888</v>
       </c>
-      <c r="M4" s="13" t="s">
+      <c r="M4" s="12" t="s">
         <v>46</v>
       </c>
-      <c r="N4" s="13" t="s">
+      <c r="N4" s="12" t="s">
         <v>16</v>
       </c>
-      <c r="O4" s="13" t="s">
+      <c r="O4" s="12" t="s">
         <v>17</v>
       </c>
-      <c r="P4" s="13"/>
-      <c r="Q4" s="13"/>
-      <c r="R4" s="13"/>
-      <c r="S4" s="13">
+      <c r="P4" s="12"/>
+      <c r="Q4" s="12"/>
+      <c r="R4" s="12"/>
+      <c r="S4" s="12">
         <v>0</v>
       </c>
-      <c r="T4" s="13"/>
+      <c r="T4" s="12"/>
     </row>
     <row r="5" spans="1:20">
-      <c r="A5" s="3" t="s">
+      <c r="A5" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="B5" s="3" t="s">
+      <c r="B5" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="C5" s="13" t="s">
+      <c r="C5" s="12" t="s">
         <v>14</v>
       </c>
-      <c r="D5" s="3" t="s">
+      <c r="D5" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="E5" s="3">
+      <c r="E5" s="2">
         <v>12</v>
       </c>
-      <c r="F5" s="3" t="s">
+      <c r="F5" s="2" t="s">
         <v>48</v>
       </c>
-      <c r="G5" s="3" t="s">
+      <c r="G5" s="2" t="s">
         <v>49</v>
       </c>
-      <c r="H5" s="3" t="s">
+      <c r="H5" s="2" t="s">
         <v>50</v>
       </c>
-      <c r="I5" s="3" t="s">
+      <c r="I5" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="J5" s="3" t="s">
+      <c r="J5" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="K5" s="3">
+      <c r="K5" s="2">
         <v>1</v>
       </c>
-      <c r="L5" s="3">
+      <c r="L5" s="2">
         <v>1010301001</v>
       </c>
-      <c r="M5" s="3" t="s">
+      <c r="M5" s="2" t="s">
         <v>51</v>
       </c>
-      <c r="N5" s="3" t="s">
+      <c r="N5" s="2" t="s">
         <v>52</v>
       </c>
-      <c r="O5" s="3" t="s">
+      <c r="O5" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="P5" s="3"/>
-      <c r="Q5" s="3"/>
-      <c r="R5" s="3"/>
-      <c r="S5" s="13">
+      <c r="P5" s="2"/>
+      <c r="Q5" s="2"/>
+      <c r="R5" s="2"/>
+      <c r="S5" s="12">
         <v>0</v>
       </c>
-      <c r="T5" s="3"/>
+      <c r="T5" s="2"/>
     </row>
     <row r="6" spans="1:20">
-      <c r="A6" s="3" t="s">
+      <c r="A6" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="B6" s="3" t="s">
+      <c r="B6" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="C6" s="3" t="s">
+      <c r="C6" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="D6" s="18" t="s">
+      <c r="D6" s="17" t="s">
         <v>43</v>
       </c>
       <c r="E6">
         <v>5</v>
       </c>
-      <c r="F6" s="21" t="s">
+      <c r="F6" s="20" t="s">
         <v>12</v>
       </c>
-      <c r="G6" s="21" t="s">
+      <c r="G6" s="20" t="s">
         <v>11</v>
       </c>
-      <c r="H6" s="3" t="s">
+      <c r="H6" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="I6" s="3" t="s">
+      <c r="I6" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="J6" s="3" t="s">
+      <c r="J6" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="K6" s="3">
+      <c r="K6" s="2">
         <v>1</v>
       </c>
-      <c r="L6" s="3">
+      <c r="L6" s="2">
         <v>1010301033</v>
       </c>
-      <c r="M6" s="3" t="s">
+      <c r="M6" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="N6" s="3" t="s">
+      <c r="N6" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="O6" s="3" t="s">
+      <c r="O6" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="P6" s="3"/>
-      <c r="Q6" s="3"/>
-      <c r="R6" s="3"/>
-      <c r="S6" s="13">
+      <c r="P6" s="2"/>
+      <c r="Q6" s="2"/>
+      <c r="R6" s="2"/>
+      <c r="S6" s="12">
         <v>0</v>
       </c>
-      <c r="T6" s="3"/>
+      <c r="T6" s="2"/>
     </row>
     <row r="7" spans="1:20">
-      <c r="A7" s="22" t="s">
+      <c r="A7" s="21" t="s">
         <v>55</v>
       </c>
-      <c r="B7" s="22" t="s">
+      <c r="B7" s="21" t="s">
         <v>56</v>
       </c>
-      <c r="C7" s="22" t="s">
+      <c r="C7" s="21" t="s">
         <v>20</v>
       </c>
-      <c r="D7" s="22" t="s">
+      <c r="D7" s="21" t="s">
         <v>40</v>
       </c>
-      <c r="E7" s="22">
+      <c r="E7" s="21">
         <v>12</v>
       </c>
-      <c r="F7" s="23" t="s">
+      <c r="F7" s="22" t="s">
         <v>12</v>
       </c>
-      <c r="G7" s="22" t="s">
+      <c r="G7" s="21" t="s">
         <v>11</v>
       </c>
-      <c r="H7" s="22" t="s">
+      <c r="H7" s="21" t="s">
         <v>57</v>
       </c>
-      <c r="I7" s="22" t="s">
+      <c r="I7" s="21" t="s">
         <v>41</v>
       </c>
-      <c r="J7" s="22" t="s">
+      <c r="J7" s="21" t="s">
         <v>14</v>
       </c>
-      <c r="K7" s="22">
+      <c r="K7" s="21">
         <v>3</v>
       </c>
-      <c r="L7" s="22">
+      <c r="L7" s="21">
         <v>1010301003</v>
       </c>
-      <c r="M7" s="22" t="s">
+      <c r="M7" s="21" t="s">
         <v>58</v>
       </c>
-      <c r="N7" s="22" t="s">
+      <c r="N7" s="21" t="s">
         <v>16</v>
       </c>
-      <c r="O7" s="22" t="s">
+      <c r="O7" s="21" t="s">
         <v>17</v>
       </c>
-      <c r="P7" s="22"/>
-      <c r="Q7" s="22"/>
-      <c r="R7" s="22"/>
-      <c r="S7" s="22">
+      <c r="P7" s="21"/>
+      <c r="Q7" s="21"/>
+      <c r="R7" s="21"/>
+      <c r="S7" s="21">
         <v>0</v>
       </c>
-      <c r="T7" s="22"/>
+      <c r="T7" s="21"/>
     </row>
     <row r="8" spans="1:20">
-      <c r="A8" s="22" t="s">
+      <c r="A8" s="21" t="s">
         <v>59</v>
       </c>
-      <c r="B8" s="22" t="s">
+      <c r="B8" s="21" t="s">
         <v>60</v>
       </c>
-      <c r="C8" s="22" t="s">
+      <c r="C8" s="21" t="s">
         <v>14</v>
       </c>
-      <c r="D8" s="22" t="s">
+      <c r="D8" s="21" t="s">
         <v>43</v>
       </c>
-      <c r="E8" s="22">
+      <c r="E8" s="21">
         <v>5</v>
       </c>
-      <c r="F8" s="23" t="s">
+      <c r="F8" s="22" t="s">
         <v>12</v>
       </c>
-      <c r="G8" s="22" t="s">
+      <c r="G8" s="21" t="s">
         <v>11</v>
       </c>
-      <c r="H8" s="22" t="s">
+      <c r="H8" s="21" t="s">
         <v>57</v>
       </c>
-      <c r="I8" s="22" t="s">
+      <c r="I8" s="21" t="s">
         <v>41</v>
       </c>
-      <c r="J8" s="22" t="s">
+      <c r="J8" s="21" t="s">
         <v>14</v>
       </c>
-      <c r="K8" s="22">
+      <c r="K8" s="21">
         <v>0</v>
       </c>
-      <c r="L8" s="22">
+      <c r="L8" s="21">
         <v>1010301003</v>
       </c>
-      <c r="M8" s="22" t="s">
+      <c r="M8" s="21" t="s">
         <v>58</v>
       </c>
-      <c r="N8" s="22" t="s">
+      <c r="N8" s="21" t="s">
         <v>16</v>
       </c>
-      <c r="O8" s="22" t="s">
+      <c r="O8" s="21" t="s">
         <v>17</v>
       </c>
-      <c r="P8" s="22"/>
-      <c r="Q8" s="22"/>
-      <c r="R8" s="22"/>
-      <c r="S8" s="22">
+      <c r="P8" s="21"/>
+      <c r="Q8" s="21"/>
+      <c r="R8" s="21"/>
+      <c r="S8" s="21">
         <v>0</v>
       </c>
-      <c r="T8" s="22"/>
+      <c r="T8" s="21"/>
     </row>
     <row r="9" spans="1:20">
-      <c r="A9" s="22" t="s">
+      <c r="A9" s="21" t="s">
         <v>61</v>
       </c>
-      <c r="B9" s="22" t="s">
+      <c r="B9" s="21" t="s">
         <v>61</v>
       </c>
-      <c r="C9" s="22" t="s">
+      <c r="C9" s="21" t="s">
         <v>14</v>
       </c>
-      <c r="D9" s="22" t="s">
+      <c r="D9" s="21" t="s">
         <v>43</v>
       </c>
-      <c r="E9" s="22">
+      <c r="E9" s="21">
         <v>5</v>
       </c>
-      <c r="F9" s="23" t="s">
+      <c r="F9" s="22" t="s">
         <v>12</v>
       </c>
-      <c r="G9" s="22" t="s">
+      <c r="G9" s="21" t="s">
         <v>11</v>
       </c>
-      <c r="H9" s="22" t="s">
+      <c r="H9" s="21" t="s">
         <v>57</v>
       </c>
-      <c r="I9" s="22" t="s">
+      <c r="I9" s="21" t="s">
         <v>41</v>
       </c>
-      <c r="J9" s="22" t="s">
+      <c r="J9" s="21" t="s">
         <v>14</v>
       </c>
-      <c r="K9" s="22">
+      <c r="K9" s="21">
         <v>0</v>
       </c>
-      <c r="L9" s="22">
+      <c r="L9" s="21">
         <v>1010301003</v>
       </c>
-      <c r="M9" s="22" t="s">
+      <c r="M9" s="21" t="s">
         <v>58</v>
       </c>
-      <c r="N9" s="22" t="s">
+      <c r="N9" s="21" t="s">
         <v>16</v>
       </c>
-      <c r="O9" s="22" t="s">
+      <c r="O9" s="21" t="s">
         <v>17</v>
       </c>
-      <c r="P9" s="22"/>
-      <c r="Q9" s="22"/>
-      <c r="R9" s="22"/>
-      <c r="S9" s="22">
+      <c r="P9" s="21"/>
+      <c r="Q9" s="21"/>
+      <c r="R9" s="21"/>
+      <c r="S9" s="21">
         <v>0</v>
       </c>
-      <c r="T9" s="22"/>
+      <c r="T9" s="21"/>
     </row>
     <row r="10" spans="1:20">
-      <c r="A10" s="3" t="s">
+      <c r="A10" s="2" t="s">
         <v>62</v>
       </c>
-      <c r="B10" s="3" t="s">
+      <c r="B10" s="2" t="s">
         <v>62</v>
       </c>
-      <c r="C10" s="3" t="s">
+      <c r="C10" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="D10" s="22" t="s">
+      <c r="D10" s="21" t="s">
         <v>43</v>
       </c>
-      <c r="E10" s="22">
+      <c r="E10" s="21">
         <v>5</v>
       </c>
-      <c r="F10" s="13" t="s">
+      <c r="F10" s="12" t="s">
         <v>22</v>
       </c>
-      <c r="G10" s="13" t="s">
+      <c r="G10" s="12" t="s">
         <v>22</v>
       </c>
-      <c r="H10" s="13" t="s">
+      <c r="H10" s="12" t="s">
         <v>63</v>
       </c>
-      <c r="I10" s="13" t="s">
+      <c r="I10" s="12" t="s">
         <v>44</v>
       </c>
-      <c r="J10" s="13" t="s">
+      <c r="J10" s="12" t="s">
         <v>14</v>
       </c>
-      <c r="K10" s="13">
+      <c r="K10" s="12">
         <v>1</v>
       </c>
-      <c r="L10" s="16">
+      <c r="L10" s="15">
         <v>1000000001</v>
       </c>
-      <c r="M10" s="3" t="s">
+      <c r="M10" s="2" t="s">
         <v>64</v>
       </c>
-      <c r="N10" s="3" t="s">
+      <c r="N10" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="O10" s="3" t="s">
+      <c r="O10" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="P10" s="22"/>
-      <c r="Q10" s="22"/>
-      <c r="R10" s="22"/>
-      <c r="S10" s="22">
+      <c r="P10" s="21"/>
+      <c r="Q10" s="21"/>
+      <c r="R10" s="21"/>
+      <c r="S10" s="21">
         <v>0</v>
       </c>
-      <c r="T10" s="22"/>
+      <c r="T10" s="21"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -3269,144 +3340,144 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1:R3"/>
-  <sheetFormatPr defaultColWidth="8.85454545454546" defaultRowHeight="14.5" outlineLevelRow="2"/>
+  <sheetFormatPr defaultColWidth="8.85185185185185" defaultRowHeight="14.4" outlineLevelRow="2"/>
   <cols>
     <col min="1" max="2" width="21" customWidth="1"/>
     <col min="3" max="3" width="6" customWidth="1"/>
-    <col min="4" max="4" width="12.7090909090909" customWidth="1"/>
-    <col min="5" max="5" width="19.4272727272727" customWidth="1"/>
-    <col min="6" max="6" width="15.1363636363636" customWidth="1"/>
-    <col min="7" max="7" width="15.4272727272727" customWidth="1"/>
-    <col min="8" max="8" width="19.5727272727273" customWidth="1"/>
-    <col min="9" max="9" width="10.8545454545455" customWidth="1"/>
-    <col min="10" max="10" width="17.5727272727273" customWidth="1"/>
-    <col min="11" max="11" width="11.2818181818182" customWidth="1"/>
-    <col min="12" max="12" width="21.7090909090909" customWidth="1"/>
+    <col min="4" max="4" width="12.712962962963" customWidth="1"/>
+    <col min="5" max="5" width="19.4259259259259" customWidth="1"/>
+    <col min="6" max="6" width="15.1388888888889" customWidth="1"/>
+    <col min="7" max="7" width="15.4259259259259" customWidth="1"/>
+    <col min="8" max="8" width="19.5740740740741" customWidth="1"/>
+    <col min="9" max="9" width="10.8518518518519" customWidth="1"/>
+    <col min="10" max="10" width="17.5740740740741" customWidth="1"/>
+    <col min="11" max="11" width="11.2777777777778" customWidth="1"/>
+    <col min="12" max="12" width="21.712962962963" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:18">
-      <c r="A1" s="3" t="s">
+      <c r="A1" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="B1" s="3" t="s">
+      <c r="B1" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="C1" s="3" t="s">
+      <c r="C1" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="D1" s="13" t="s">
+      <c r="D1" s="12" t="s">
         <v>6</v>
       </c>
-      <c r="E1" s="13" t="s">
+      <c r="E1" s="12" t="s">
         <v>7</v>
       </c>
-      <c r="F1" s="13" t="s">
+      <c r="F1" s="12" t="s">
         <v>8</v>
       </c>
-      <c r="G1" s="13" t="s">
+      <c r="G1" s="12" t="s">
         <v>9</v>
       </c>
-      <c r="H1" s="3" t="s">
+      <c r="H1" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="I1" s="3" t="s">
+      <c r="I1" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="J1" s="3" t="s">
+      <c r="J1" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="K1" s="3" t="s">
+      <c r="K1" s="2" t="s">
         <v>65</v>
       </c>
-      <c r="L1" s="3" t="s">
+      <c r="L1" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="M1" s="17"/>
-      <c r="N1" s="17"/>
-      <c r="O1" s="17"/>
-      <c r="P1" s="17"/>
-      <c r="Q1" s="17"/>
-      <c r="R1" s="17"/>
+      <c r="M1" s="16"/>
+      <c r="N1" s="16"/>
+      <c r="O1" s="16"/>
+      <c r="P1" s="16"/>
+      <c r="Q1" s="16"/>
+      <c r="R1" s="16"/>
     </row>
     <row r="2" spans="1:18">
-      <c r="A2" s="3" t="s">
+      <c r="A2" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="B2" s="3" t="s">
+      <c r="B2" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="C2" s="3" t="s">
+      <c r="C2" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="D2" s="3">
+      <c r="D2" s="2">
         <v>1010301033</v>
       </c>
-      <c r="E2" s="3" t="s">
+      <c r="E2" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="F2" s="3" t="s">
+      <c r="F2" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="G2" s="3" t="s">
+      <c r="G2" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="H2" s="3" t="s">
+      <c r="H2" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="I2" s="18" t="s">
+      <c r="I2" s="17" t="s">
         <v>43</v>
       </c>
-      <c r="J2" s="3" t="s">
+      <c r="J2" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="K2" s="3" t="s">
+      <c r="K2" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="L2" s="3">
+      <c r="L2" s="2">
         <v>1</v>
       </c>
-      <c r="M2" s="17"/>
-      <c r="N2" s="17"/>
-      <c r="O2" s="17"/>
-      <c r="P2" s="17"/>
-      <c r="Q2" s="17"/>
-      <c r="R2" s="17"/>
+      <c r="M2" s="16"/>
+      <c r="N2" s="16"/>
+      <c r="O2" s="16"/>
+      <c r="P2" s="16"/>
+      <c r="Q2" s="16"/>
+      <c r="R2" s="16"/>
     </row>
     <row r="3" spans="1:12">
-      <c r="A3" s="3" t="s">
+      <c r="A3" s="2" t="s">
         <v>62</v>
       </c>
-      <c r="B3" s="3" t="s">
+      <c r="B3" s="2" t="s">
         <v>62</v>
       </c>
-      <c r="C3" s="3" t="s">
+      <c r="C3" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="D3" s="16">
+      <c r="D3" s="15">
         <v>1000000001</v>
       </c>
-      <c r="E3" s="3" t="s">
+      <c r="E3" s="2" t="s">
         <v>64</v>
       </c>
-      <c r="F3" s="3" t="s">
+      <c r="F3" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="G3" s="3" t="s">
+      <c r="G3" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="H3" s="3" t="s">
+      <c r="H3" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="I3" s="18" t="s">
+      <c r="I3" s="17" t="s">
         <v>43</v>
       </c>
-      <c r="J3" s="3" t="s">
+      <c r="J3" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="K3" s="3" t="s">
+      <c r="K3" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="L3" s="3">
+      <c r="L3" s="2">
         <v>1</v>
       </c>
     </row>
@@ -3420,71 +3491,71 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1:F3"/>
-  <sheetFormatPr defaultColWidth="8.85454545454546" defaultRowHeight="14.5" outlineLevelRow="2" outlineLevelCol="5"/>
+  <sheetFormatPr defaultColWidth="8.85185185185185" defaultRowHeight="14.4" outlineLevelRow="2" outlineLevelCol="5"/>
   <cols>
-    <col min="1" max="1" width="27.1363636363636" customWidth="1"/>
-    <col min="2" max="2" width="10.4272727272727" customWidth="1"/>
-    <col min="3" max="3" width="11.4272727272727" customWidth="1"/>
-    <col min="4" max="4" width="11.7090909090909" customWidth="1"/>
-    <col min="5" max="5" width="14.5727272727273" customWidth="1"/>
-    <col min="6" max="6" width="17.7090909090909" customWidth="1"/>
+    <col min="1" max="1" width="27.1388888888889" customWidth="1"/>
+    <col min="2" max="2" width="10.4259259259259" customWidth="1"/>
+    <col min="3" max="3" width="11.4259259259259" customWidth="1"/>
+    <col min="4" max="4" width="11.712962962963" customWidth="1"/>
+    <col min="5" max="5" width="14.5740740740741" customWidth="1"/>
+    <col min="6" max="6" width="17.712962962963" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6">
-      <c r="A1" s="14" t="s">
+      <c r="A1" s="13" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="14" t="s">
+      <c r="B1" s="13" t="s">
         <v>66</v>
       </c>
-      <c r="C1" s="14" t="s">
+      <c r="C1" s="13" t="s">
         <v>67</v>
       </c>
-      <c r="D1" s="15" t="s">
+      <c r="D1" s="14" t="s">
         <v>68</v>
       </c>
-      <c r="E1" s="13" t="s">
+      <c r="E1" s="12" t="s">
         <v>69</v>
       </c>
-      <c r="F1" s="13" t="s">
+      <c r="F1" s="12" t="s">
         <v>70</v>
       </c>
     </row>
     <row r="2" spans="1:6">
-      <c r="A2" s="3" t="s">
+      <c r="A2" s="2" t="s">
         <v>59</v>
       </c>
-      <c r="B2" s="3">
+      <c r="B2" s="2">
         <v>50</v>
       </c>
-      <c r="C2" s="3">
+      <c r="C2" s="2">
         <v>70</v>
       </c>
-      <c r="D2" s="3" t="s">
+      <c r="D2" s="2" t="s">
         <v>71</v>
       </c>
-      <c r="E2" s="3"/>
-      <c r="F2" s="10" t="s">
+      <c r="E2" s="2"/>
+      <c r="F2" s="7" t="s">
         <v>72</v>
       </c>
     </row>
     <row r="3" spans="1:6">
-      <c r="A3" s="3" t="s">
+      <c r="A3" s="2" t="s">
         <v>61</v>
       </c>
-      <c r="B3" s="3">
+      <c r="B3" s="2">
         <v>40</v>
       </c>
-      <c r="C3" s="3">
+      <c r="C3" s="2">
         <v>26</v>
       </c>
-      <c r="D3" s="3" t="s">
+      <c r="D3" s="2" t="s">
         <v>73</v>
       </c>
-      <c r="E3" s="10" t="s">
+      <c r="E3" s="7" t="s">
         <v>74</v>
       </c>
-      <c r="F3" s="10">
+      <c r="F3" s="7">
         <v>2</v>
       </c>
     </row>
@@ -3498,91 +3569,91 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1:F4"/>
-  <sheetFormatPr defaultColWidth="8.85454545454546" defaultRowHeight="14.5" outlineLevelRow="3" outlineLevelCol="5"/>
+  <sheetFormatPr defaultColWidth="8.85185185185185" defaultRowHeight="14.4" outlineLevelRow="3" outlineLevelCol="5"/>
   <cols>
-    <col min="1" max="1" width="27.1363636363636" customWidth="1"/>
-    <col min="2" max="2" width="10.4272727272727" customWidth="1"/>
-    <col min="3" max="3" width="11.4272727272727" customWidth="1"/>
-    <col min="4" max="4" width="11.7090909090909" customWidth="1"/>
-    <col min="5" max="5" width="14.5727272727273" customWidth="1"/>
-    <col min="6" max="6" width="17.7090909090909" customWidth="1"/>
+    <col min="1" max="1" width="27.1388888888889" customWidth="1"/>
+    <col min="2" max="2" width="10.4259259259259" customWidth="1"/>
+    <col min="3" max="3" width="11.4259259259259" customWidth="1"/>
+    <col min="4" max="4" width="11.712962962963" customWidth="1"/>
+    <col min="5" max="5" width="14.5740740740741" customWidth="1"/>
+    <col min="6" max="6" width="17.712962962963" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6">
-      <c r="A1" s="14" t="s">
+      <c r="A1" s="13" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="14" t="s">
+      <c r="B1" s="13" t="s">
         <v>66</v>
       </c>
-      <c r="C1" s="14" t="s">
+      <c r="C1" s="13" t="s">
         <v>67</v>
       </c>
-      <c r="D1" s="15" t="s">
+      <c r="D1" s="14" t="s">
         <v>68</v>
       </c>
-      <c r="E1" s="13" t="s">
+      <c r="E1" s="12" t="s">
         <v>69</v>
       </c>
-      <c r="F1" s="13" t="s">
+      <c r="F1" s="12" t="s">
         <v>70</v>
       </c>
     </row>
     <row r="2" spans="1:6">
-      <c r="A2" s="13" t="s">
+      <c r="A2" s="12" t="s">
         <v>59</v>
       </c>
-      <c r="B2" s="3">
+      <c r="B2" s="2">
         <v>150</v>
       </c>
-      <c r="C2" s="3">
+      <c r="C2" s="2">
         <v>45</v>
       </c>
-      <c r="D2" s="3" t="s">
+      <c r="D2" s="2" t="s">
         <v>71</v>
       </c>
-      <c r="E2" s="3"/>
-      <c r="F2" s="10" t="s">
+      <c r="E2" s="2"/>
+      <c r="F2" s="7" t="s">
         <v>75</v>
       </c>
     </row>
     <row r="3" spans="1:6">
-      <c r="A3" s="13" t="s">
+      <c r="A3" s="12" t="s">
         <v>76</v>
       </c>
-      <c r="B3" s="3">
+      <c r="B3" s="2">
         <v>40</v>
       </c>
-      <c r="C3" s="3">
+      <c r="C3" s="2">
         <v>26</v>
       </c>
-      <c r="D3" s="3" t="s">
+      <c r="D3" s="2" t="s">
         <v>77</v>
       </c>
-      <c r="E3" s="10" t="s">
+      <c r="E3" s="7" t="s">
         <v>74</v>
       </c>
-      <c r="F3" s="10">
+      <c r="F3" s="7">
         <v>2</v>
       </c>
     </row>
     <row r="4" spans="1:6">
-      <c r="A4" s="13" t="s">
+      <c r="A4" s="12" t="s">
         <v>61</v>
       </c>
-      <c r="B4" s="3">
+      <c r="B4" s="2">
         <v>50</v>
       </c>
-      <c r="C4" s="3">
+      <c r="C4" s="2">
         <v>70</v>
       </c>
-      <c r="D4" s="3" t="s">
+      <c r="D4" s="2" t="s">
         <v>73</v>
       </c>
-      <c r="E4" s="3" t="s">
+      <c r="E4" s="2" t="s">
         <v>75</v>
       </c>
-      <c r="F4" s="10"/>
+      <c r="F4" s="7"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -3594,9 +3665,9 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1:C3"/>
-  <sheetFormatPr defaultColWidth="8.85454545454546" defaultRowHeight="14.5" outlineLevelRow="2" outlineLevelCol="2"/>
+  <sheetFormatPr defaultColWidth="8.85185185185185" defaultRowHeight="14.4" outlineLevelRow="2" outlineLevelCol="2"/>
   <cols>
-    <col min="1" max="1" width="28.7090909090909" customWidth="1"/>
+    <col min="1" max="1" width="28.712962962963" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3">
@@ -3642,102 +3713,102 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1:G4"/>
-  <sheetFormatPr defaultColWidth="8.85454545454546" defaultRowHeight="14.5" outlineLevelRow="3" outlineLevelCol="6"/>
+  <sheetFormatPr defaultColWidth="8.85185185185185" defaultRowHeight="14.4" outlineLevelRow="3" outlineLevelCol="6"/>
   <cols>
-    <col min="1" max="1" width="19.7090909090909" customWidth="1"/>
-    <col min="2" max="2" width="8.13636363636364" customWidth="1"/>
-    <col min="3" max="3" width="8.57272727272727" customWidth="1"/>
-    <col min="4" max="4" width="17.8545454545455" customWidth="1"/>
-    <col min="5" max="5" width="12.7090909090909" customWidth="1"/>
-    <col min="6" max="6" width="14.5727272727273" customWidth="1"/>
-    <col min="7" max="7" width="17.7090909090909" customWidth="1"/>
+    <col min="1" max="1" width="19.712962962963" customWidth="1"/>
+    <col min="2" max="2" width="8.13888888888889" customWidth="1"/>
+    <col min="3" max="3" width="8.57407407407407" customWidth="1"/>
+    <col min="4" max="4" width="17.8518518518519" customWidth="1"/>
+    <col min="5" max="5" width="12.712962962963" customWidth="1"/>
+    <col min="6" max="6" width="14.5740740740741" customWidth="1"/>
+    <col min="7" max="7" width="17.712962962963" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7">
-      <c r="A1" s="13" t="s">
+      <c r="A1" s="12" t="s">
         <v>83</v>
       </c>
-      <c r="B1" s="13" t="s">
+      <c r="B1" s="12" t="s">
         <v>84</v>
       </c>
-      <c r="C1" s="13" t="s">
+      <c r="C1" s="12" t="s">
         <v>80</v>
       </c>
-      <c r="D1" s="13" t="s">
+      <c r="D1" s="12" t="s">
         <v>85</v>
       </c>
-      <c r="E1" s="13" t="s">
+      <c r="E1" s="12" t="s">
         <v>68</v>
       </c>
-      <c r="F1" s="13" t="s">
+      <c r="F1" s="12" t="s">
         <v>69</v>
       </c>
-      <c r="G1" s="13" t="s">
+      <c r="G1" s="12" t="s">
         <v>70</v>
       </c>
     </row>
     <row r="2" spans="1:7">
-      <c r="A2" s="13" t="s">
+      <c r="A2" s="12" t="s">
         <v>86</v>
       </c>
-      <c r="B2" s="13">
+      <c r="B2" s="12">
         <v>524</v>
       </c>
-      <c r="C2" s="13">
+      <c r="C2" s="12">
         <v>524</v>
       </c>
-      <c r="D2" s="13">
+      <c r="D2" s="12">
         <v>2</v>
       </c>
-      <c r="E2" s="10" t="s">
+      <c r="E2" s="7" t="s">
         <v>71</v>
       </c>
-      <c r="F2" s="10" t="s">
+      <c r="F2" s="7" t="s">
         <v>74</v>
       </c>
-      <c r="G2" s="10" t="s">
+      <c r="G2" s="7" t="s">
         <v>87</v>
       </c>
     </row>
     <row r="3" spans="1:7">
-      <c r="A3" s="13" t="s">
+      <c r="A3" s="12" t="s">
         <v>88</v>
       </c>
-      <c r="B3" s="13">
+      <c r="B3" s="12">
         <v>232</v>
       </c>
-      <c r="C3" s="13">
+      <c r="C3" s="12">
         <v>232</v>
       </c>
-      <c r="D3" s="13">
+      <c r="D3" s="12">
         <v>7.9</v>
       </c>
-      <c r="E3" s="10" t="s">
+      <c r="E3" s="7" t="s">
         <v>73</v>
       </c>
-      <c r="F3" s="10" t="s">
+      <c r="F3" s="7" t="s">
         <v>89</v>
       </c>
-      <c r="G3" s="3"/>
+      <c r="G3" s="2"/>
     </row>
     <row r="4" spans="1:7">
-      <c r="A4" s="3" t="s">
+      <c r="A4" s="2" t="s">
         <v>90</v>
       </c>
-      <c r="B4" s="3">
+      <c r="B4" s="2">
         <v>232</v>
       </c>
-      <c r="C4" s="3">
+      <c r="C4" s="2">
         <v>232</v>
       </c>
-      <c r="D4" s="3">
+      <c r="D4" s="2">
         <v>2.32</v>
       </c>
-      <c r="E4" s="10" t="s">
+      <c r="E4" s="7" t="s">
         <v>77</v>
       </c>
-      <c r="F4" s="3"/>
-      <c r="G4" s="3"/>
+      <c r="F4" s="2"/>
+      <c r="G4" s="2"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -3749,102 +3820,102 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1:G4"/>
-  <sheetFormatPr defaultColWidth="8.85454545454546" defaultRowHeight="14.5" outlineLevelRow="3" outlineLevelCol="6"/>
+  <sheetFormatPr defaultColWidth="8.85185185185185" defaultRowHeight="14.4" outlineLevelRow="3" outlineLevelCol="6"/>
   <cols>
-    <col min="1" max="1" width="19.7090909090909" customWidth="1"/>
-    <col min="2" max="2" width="8.13636363636364" customWidth="1"/>
-    <col min="3" max="3" width="8.57272727272727" customWidth="1"/>
-    <col min="4" max="4" width="17.8545454545455" customWidth="1"/>
-    <col min="5" max="5" width="12.7090909090909" customWidth="1"/>
-    <col min="6" max="6" width="14.5727272727273" customWidth="1"/>
-    <col min="7" max="7" width="17.7090909090909" customWidth="1"/>
+    <col min="1" max="1" width="19.712962962963" customWidth="1"/>
+    <col min="2" max="2" width="8.13888888888889" customWidth="1"/>
+    <col min="3" max="3" width="8.57407407407407" customWidth="1"/>
+    <col min="4" max="4" width="17.8518518518519" customWidth="1"/>
+    <col min="5" max="5" width="12.712962962963" customWidth="1"/>
+    <col min="6" max="6" width="14.5740740740741" customWidth="1"/>
+    <col min="7" max="7" width="17.712962962963" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7">
-      <c r="A1" s="13" t="s">
+      <c r="A1" s="12" t="s">
         <v>83</v>
       </c>
-      <c r="B1" s="13" t="s">
+      <c r="B1" s="12" t="s">
         <v>84</v>
       </c>
-      <c r="C1" s="13" t="s">
+      <c r="C1" s="12" t="s">
         <v>80</v>
       </c>
-      <c r="D1" s="13" t="s">
+      <c r="D1" s="12" t="s">
         <v>85</v>
       </c>
-      <c r="E1" s="13" t="s">
+      <c r="E1" s="12" t="s">
         <v>68</v>
       </c>
-      <c r="F1" s="13" t="s">
+      <c r="F1" s="12" t="s">
         <v>69</v>
       </c>
-      <c r="G1" s="13" t="s">
+      <c r="G1" s="12" t="s">
         <v>70</v>
       </c>
     </row>
     <row r="2" spans="1:7">
-      <c r="A2" s="13" t="s">
+      <c r="A2" s="12" t="s">
         <v>86</v>
       </c>
-      <c r="B2" s="13">
+      <c r="B2" s="12">
         <v>22</v>
       </c>
-      <c r="C2" s="13">
+      <c r="C2" s="12">
         <v>524</v>
       </c>
-      <c r="D2" s="13">
+      <c r="D2" s="12">
         <v>2</v>
       </c>
-      <c r="E2" s="10" t="s">
+      <c r="E2" s="7" t="s">
         <v>71</v>
       </c>
-      <c r="F2" s="10" t="s">
+      <c r="F2" s="7" t="s">
         <v>74</v>
       </c>
-      <c r="G2" s="10" t="s">
+      <c r="G2" s="7" t="s">
         <v>87</v>
       </c>
     </row>
     <row r="3" spans="1:7">
-      <c r="A3" s="13" t="s">
+      <c r="A3" s="12" t="s">
         <v>88</v>
       </c>
-      <c r="B3" s="13">
+      <c r="B3" s="12">
         <v>34</v>
       </c>
-      <c r="C3" s="13">
+      <c r="C3" s="12">
         <v>232</v>
       </c>
-      <c r="D3" s="13">
+      <c r="D3" s="12">
         <v>7.9</v>
       </c>
-      <c r="E3" s="10" t="s">
+      <c r="E3" s="7" t="s">
         <v>73</v>
       </c>
-      <c r="F3" s="10" t="s">
+      <c r="F3" s="7" t="s">
         <v>89</v>
       </c>
-      <c r="G3" s="3"/>
+      <c r="G3" s="2"/>
     </row>
     <row r="4" spans="1:7">
-      <c r="A4" s="3" t="s">
+      <c r="A4" s="2" t="s">
         <v>90</v>
       </c>
-      <c r="B4" s="3">
+      <c r="B4" s="2">
         <v>67</v>
       </c>
-      <c r="C4" s="3">
+      <c r="C4" s="2">
         <v>232</v>
       </c>
-      <c r="D4" s="3">
+      <c r="D4" s="2">
         <v>2.32</v>
       </c>
-      <c r="E4" s="10" t="s">
+      <c r="E4" s="7" t="s">
         <v>77</v>
       </c>
-      <c r="F4" s="3"/>
-      <c r="G4" s="3"/>
+      <c r="F4" s="2"/>
+      <c r="G4" s="2"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -3856,633 +3927,633 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1:S11"/>
-  <sheetFormatPr defaultColWidth="8.85454545454546" defaultRowHeight="14.5"/>
+  <sheetFormatPr defaultColWidth="8.85185185185185" defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="39.7090909090909" customWidth="1"/>
-    <col min="2" max="2" width="10.1363636363636" customWidth="1"/>
-    <col min="3" max="3" width="39.7090909090909" customWidth="1"/>
+    <col min="1" max="1" width="39.712962962963" customWidth="1"/>
+    <col min="2" max="2" width="10.1388888888889" customWidth="1"/>
+    <col min="3" max="3" width="39.712962962963" customWidth="1"/>
     <col min="4" max="4" width="11" customWidth="1"/>
-    <col min="5" max="5" width="13.2818181818182" customWidth="1"/>
-    <col min="6" max="6" width="8.85454545454546" customWidth="1"/>
-    <col min="7" max="7" width="17.8545454545455" customWidth="1"/>
-    <col min="8" max="8" width="19.5727272727273" customWidth="1"/>
-    <col min="9" max="9" width="23.7090909090909" customWidth="1"/>
-    <col min="10" max="10" width="12.7090909090909" customWidth="1"/>
-    <col min="11" max="11" width="11.8545454545455" customWidth="1"/>
-    <col min="12" max="12" width="17.4272727272727" customWidth="1"/>
-    <col min="13" max="14" width="39.7090909090909" customWidth="1"/>
-    <col min="15" max="15" width="25.7090909090909" customWidth="1"/>
-    <col min="16" max="17" width="16.5727272727273" customWidth="1"/>
-    <col min="18" max="18" width="11.5727272727273" customWidth="1"/>
-    <col min="19" max="19" width="14.8545454545455" customWidth="1"/>
+    <col min="5" max="5" width="13.2777777777778" customWidth="1"/>
+    <col min="6" max="6" width="8.85185185185185" customWidth="1"/>
+    <col min="7" max="7" width="17.8518518518519" customWidth="1"/>
+    <col min="8" max="8" width="19.5740740740741" customWidth="1"/>
+    <col min="9" max="9" width="23.712962962963" customWidth="1"/>
+    <col min="10" max="10" width="12.712962962963" customWidth="1"/>
+    <col min="11" max="11" width="11.8518518518519" customWidth="1"/>
+    <col min="12" max="12" width="17.4259259259259" customWidth="1"/>
+    <col min="13" max="14" width="39.712962962963" customWidth="1"/>
+    <col min="15" max="15" width="25.712962962963" customWidth="1"/>
+    <col min="16" max="17" width="16.5740740740741" customWidth="1"/>
+    <col min="18" max="18" width="11.5740740740741" customWidth="1"/>
+    <col min="19" max="19" width="14.8518518518519" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:19">
-      <c r="A1" s="3" t="s">
+      <c r="A1" s="2" t="s">
         <v>91</v>
       </c>
-      <c r="B1" s="3" t="s">
+      <c r="B1" s="2" t="s">
         <v>92</v>
       </c>
-      <c r="C1" s="3" t="s">
+      <c r="C1" s="2" t="s">
         <v>93</v>
       </c>
-      <c r="D1" s="3" t="s">
+      <c r="D1" s="2" t="s">
         <v>94</v>
       </c>
-      <c r="E1" s="3" t="s">
+      <c r="E1" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="F1" s="3" t="s">
+      <c r="F1" s="2" t="s">
         <v>95</v>
       </c>
-      <c r="G1" s="3" t="s">
+      <c r="G1" s="2" t="s">
         <v>96</v>
       </c>
-      <c r="H1" s="3" t="s">
+      <c r="H1" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="I1" s="3" t="s">
+      <c r="I1" s="2" t="s">
         <v>97</v>
       </c>
-      <c r="J1" s="3" t="s">
+      <c r="J1" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="K1" s="3" t="s">
+      <c r="K1" s="2" t="s">
         <v>98</v>
       </c>
-      <c r="L1" s="3" t="s">
+      <c r="L1" s="2" t="s">
         <v>99</v>
       </c>
-      <c r="M1" s="3" t="s">
+      <c r="M1" s="2" t="s">
         <v>100</v>
       </c>
-      <c r="N1" s="3" t="s">
+      <c r="N1" s="2" t="s">
         <v>101</v>
       </c>
-      <c r="O1" s="3" t="s">
+      <c r="O1" s="2" t="s">
         <v>102</v>
       </c>
-      <c r="P1" s="3" t="s">
+      <c r="P1" s="2" t="s">
         <v>103</v>
       </c>
-      <c r="Q1" s="3" t="s">
+      <c r="Q1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="R1" s="3" t="s">
+      <c r="R1" s="2" t="s">
         <v>104</v>
       </c>
-      <c r="S1" s="5" t="s">
+      <c r="S1" s="6" t="s">
         <v>105</v>
       </c>
     </row>
     <row r="2" spans="1:19">
-      <c r="A2" s="12" t="s">
+      <c r="A2" s="11" t="s">
         <v>106</v>
       </c>
-      <c r="B2" s="3">
+      <c r="B2" s="2">
         <v>0</v>
       </c>
-      <c r="C2" s="12" t="s">
+      <c r="C2" s="11" t="s">
         <v>106</v>
       </c>
-      <c r="D2" s="3" t="s">
+      <c r="D2" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="E2" s="3" t="s">
+      <c r="E2" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="F2" s="3">
+      <c r="F2" s="2">
         <v>12</v>
       </c>
-      <c r="G2" s="3" t="s">
+      <c r="G2" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="H2" s="3"/>
-      <c r="I2" s="3"/>
-      <c r="J2" s="3" t="s">
+      <c r="H2" s="2"/>
+      <c r="I2" s="2"/>
+      <c r="J2" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="K2" s="3">
+      <c r="K2" s="2">
         <v>1</v>
       </c>
-      <c r="L2" s="3" t="s">
+      <c r="L2" s="2" t="s">
         <v>107</v>
       </c>
-      <c r="M2" s="3"/>
-      <c r="N2" s="3"/>
-      <c r="O2" s="10" t="s">
+      <c r="M2" s="2"/>
+      <c r="N2" s="2"/>
+      <c r="O2" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="P2" s="10" t="s">
+      <c r="P2" s="7" t="s">
         <v>15</v>
       </c>
-      <c r="Q2" s="10" t="s">
+      <c r="Q2" s="7" t="s">
         <v>15</v>
       </c>
-      <c r="R2" s="3" t="s">
+      <c r="R2" s="2" t="s">
         <v>108</v>
       </c>
-      <c r="S2" s="11" t="s">
+      <c r="S2" s="10" t="s">
         <v>109</v>
       </c>
     </row>
     <row r="3" spans="1:19">
-      <c r="A3" s="12" t="s">
+      <c r="A3" s="11" t="s">
         <v>110</v>
       </c>
-      <c r="B3" s="3">
+      <c r="B3" s="2">
         <v>0</v>
       </c>
-      <c r="C3" s="12" t="s">
+      <c r="C3" s="11" t="s">
         <v>110</v>
       </c>
-      <c r="D3" s="3" t="s">
+      <c r="D3" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="E3" s="12">
+      <c r="E3" s="11">
         <v>772213</v>
       </c>
-      <c r="F3" s="3">
+      <c r="F3" s="2">
         <v>5</v>
       </c>
-      <c r="G3" s="3" t="s">
+      <c r="G3" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="H3" s="3"/>
-      <c r="I3" s="3"/>
-      <c r="J3" s="3" t="s">
+      <c r="H3" s="2"/>
+      <c r="I3" s="2"/>
+      <c r="J3" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="K3" s="3">
+      <c r="K3" s="2">
         <v>3</v>
       </c>
-      <c r="L3" s="3" t="s">
+      <c r="L3" s="2" t="s">
         <v>107</v>
       </c>
-      <c r="M3" s="3"/>
-      <c r="N3" s="3"/>
-      <c r="O3" s="10" t="s">
+      <c r="M3" s="2"/>
+      <c r="N3" s="2"/>
+      <c r="O3" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="P3" s="10" t="s">
+      <c r="P3" s="7" t="s">
         <v>15</v>
       </c>
-      <c r="Q3" s="10" t="s">
+      <c r="Q3" s="7" t="s">
         <v>15</v>
       </c>
-      <c r="R3" s="3" t="s">
+      <c r="R3" s="2" t="s">
         <v>108</v>
       </c>
-      <c r="S3" s="11" t="s">
+      <c r="S3" s="10" t="s">
         <v>109</v>
       </c>
     </row>
     <row r="4" spans="1:19">
-      <c r="A4" s="3" t="s">
+      <c r="A4" s="2" t="s">
         <v>111</v>
       </c>
-      <c r="B4" s="3">
+      <c r="B4" s="2">
         <v>0</v>
       </c>
-      <c r="C4" s="3" t="s">
+      <c r="C4" s="2" t="s">
         <v>111</v>
       </c>
-      <c r="D4" s="5" t="s">
+      <c r="D4" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="E4" s="3" t="s">
+      <c r="E4" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="F4" s="3">
+      <c r="F4" s="2">
         <v>12</v>
       </c>
-      <c r="G4" s="5" t="s">
+      <c r="G4" s="6" t="s">
         <v>112</v>
       </c>
-      <c r="H4" s="3"/>
-      <c r="I4" s="3"/>
-      <c r="J4" s="3" t="s">
+      <c r="H4" s="2"/>
+      <c r="I4" s="2"/>
+      <c r="J4" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="K4" s="3">
+      <c r="K4" s="2">
         <v>1</v>
       </c>
-      <c r="L4" s="3" t="s">
+      <c r="L4" s="2" t="s">
         <v>107</v>
       </c>
-      <c r="M4" s="3" t="s">
+      <c r="M4" s="2" t="s">
         <v>111</v>
       </c>
-      <c r="N4" s="3" t="s">
+      <c r="N4" s="2" t="s">
         <v>111</v>
       </c>
-      <c r="O4" s="10" t="s">
+      <c r="O4" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="P4" s="10" t="s">
+      <c r="P4" s="7" t="s">
         <v>15</v>
       </c>
-      <c r="Q4" s="10" t="s">
+      <c r="Q4" s="7" t="s">
         <v>15</v>
       </c>
-      <c r="R4" s="3" t="s">
+      <c r="R4" s="2" t="s">
         <v>108</v>
       </c>
-      <c r="S4" s="11" t="s">
+      <c r="S4" s="10" t="s">
         <v>109</v>
       </c>
     </row>
     <row r="5" spans="1:19">
-      <c r="A5" s="3" t="s">
+      <c r="A5" s="2" t="s">
         <v>113</v>
       </c>
-      <c r="B5" s="5">
+      <c r="B5" s="6">
         <v>0</v>
       </c>
-      <c r="C5" s="3" t="s">
+      <c r="C5" s="2" t="s">
         <v>113</v>
       </c>
-      <c r="D5" s="5" t="s">
+      <c r="D5" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="E5" s="3">
+      <c r="E5" s="2">
         <v>75052200</v>
       </c>
-      <c r="F5" s="5">
+      <c r="F5" s="6">
         <v>5</v>
       </c>
-      <c r="G5" s="5" t="s">
+      <c r="G5" s="6" t="s">
         <v>112</v>
       </c>
-      <c r="H5" s="3"/>
-      <c r="I5" s="3"/>
-      <c r="J5" s="5" t="s">
+      <c r="H5" s="2"/>
+      <c r="I5" s="2"/>
+      <c r="J5" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="K5" s="5">
+      <c r="K5" s="6">
         <v>2</v>
       </c>
-      <c r="L5" s="3" t="s">
+      <c r="L5" s="2" t="s">
         <v>107</v>
       </c>
-      <c r="M5" s="3" t="s">
+      <c r="M5" s="2" t="s">
         <v>113</v>
       </c>
-      <c r="N5" s="3" t="s">
+      <c r="N5" s="2" t="s">
         <v>113</v>
       </c>
-      <c r="O5" s="10" t="s">
+      <c r="O5" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="P5" s="10" t="s">
+      <c r="P5" s="7" t="s">
         <v>15</v>
       </c>
-      <c r="Q5" s="10" t="s">
+      <c r="Q5" s="7" t="s">
         <v>15</v>
       </c>
-      <c r="R5" s="3" t="s">
+      <c r="R5" s="2" t="s">
         <v>114</v>
       </c>
-      <c r="S5" s="11" t="s">
+      <c r="S5" s="10" t="s">
         <v>109</v>
       </c>
     </row>
     <row r="6" spans="1:19">
-      <c r="A6" s="5" t="s">
+      <c r="A6" s="6" t="s">
         <v>115</v>
       </c>
-      <c r="B6" s="5">
+      <c r="B6" s="6">
         <v>0</v>
       </c>
-      <c r="C6" s="3" t="s">
+      <c r="C6" s="2" t="s">
         <v>115</v>
       </c>
-      <c r="D6" s="5" t="s">
+      <c r="D6" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="E6" s="5" t="s">
+      <c r="E6" s="6" t="s">
         <v>40</v>
       </c>
-      <c r="F6" s="5">
+      <c r="F6" s="6">
         <v>12</v>
       </c>
-      <c r="G6" s="5" t="s">
+      <c r="G6" s="6" t="s">
         <v>116</v>
       </c>
-      <c r="H6" s="5" t="s">
+      <c r="H6" s="6" t="s">
         <v>117</v>
       </c>
-      <c r="I6" s="3"/>
-      <c r="J6" s="5" t="s">
+      <c r="I6" s="2"/>
+      <c r="J6" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="K6" s="5">
+      <c r="K6" s="6">
         <v>1</v>
       </c>
-      <c r="L6" s="3" t="s">
+      <c r="L6" s="2" t="s">
         <v>107</v>
       </c>
-      <c r="M6" s="5" t="s">
+      <c r="M6" s="6" t="s">
         <v>115</v>
       </c>
-      <c r="N6" s="5" t="s">
+      <c r="N6" s="6" t="s">
         <v>115</v>
       </c>
-      <c r="O6" s="10" t="s">
+      <c r="O6" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="P6" s="10" t="s">
+      <c r="P6" s="7" t="s">
         <v>15</v>
       </c>
-      <c r="Q6" s="10" t="s">
+      <c r="Q6" s="7" t="s">
         <v>15</v>
       </c>
-      <c r="R6" s="3" t="s">
+      <c r="R6" s="2" t="s">
         <v>108</v>
       </c>
-      <c r="S6" s="11" t="s">
+      <c r="S6" s="10" t="s">
         <v>109</v>
       </c>
     </row>
     <row r="7" spans="1:19">
-      <c r="A7" s="5" t="s">
+      <c r="A7" s="6" t="s">
         <v>118</v>
       </c>
-      <c r="B7" s="5">
+      <c r="B7" s="6">
         <v>0</v>
       </c>
-      <c r="C7" s="3" t="s">
+      <c r="C7" s="2" t="s">
         <v>118</v>
       </c>
-      <c r="D7" s="5" t="s">
+      <c r="D7" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="E7" s="5" t="s">
+      <c r="E7" s="6" t="s">
         <v>40</v>
       </c>
-      <c r="F7" s="5">
+      <c r="F7" s="6">
         <v>12</v>
       </c>
-      <c r="G7" s="5" t="s">
+      <c r="G7" s="6" t="s">
         <v>116</v>
       </c>
-      <c r="H7" s="5" t="s">
+      <c r="H7" s="6" t="s">
         <v>119</v>
       </c>
-      <c r="I7" s="3"/>
-      <c r="J7" s="5" t="s">
+      <c r="I7" s="2"/>
+      <c r="J7" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="K7" s="5">
+      <c r="K7" s="6">
         <v>4</v>
       </c>
-      <c r="L7" s="3" t="s">
+      <c r="L7" s="2" t="s">
         <v>107</v>
       </c>
-      <c r="M7" s="5" t="s">
+      <c r="M7" s="6" t="s">
         <v>118</v>
       </c>
-      <c r="N7" s="5" t="s">
+      <c r="N7" s="6" t="s">
         <v>118</v>
       </c>
-      <c r="O7" s="10" t="s">
+      <c r="O7" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="P7" s="10" t="s">
+      <c r="P7" s="7" t="s">
         <v>15</v>
       </c>
-      <c r="Q7" s="10" t="s">
+      <c r="Q7" s="7" t="s">
         <v>15</v>
       </c>
-      <c r="R7" s="3" t="s">
+      <c r="R7" s="2" t="s">
         <v>108</v>
       </c>
-      <c r="S7" s="11" t="s">
+      <c r="S7" s="10" t="s">
         <v>109</v>
       </c>
     </row>
     <row r="8" spans="1:19">
-      <c r="A8" s="3" t="s">
+      <c r="A8" s="2" t="s">
         <v>120</v>
       </c>
-      <c r="B8" s="5">
+      <c r="B8" s="6">
         <v>0</v>
       </c>
-      <c r="C8" s="3" t="s">
+      <c r="C8" s="2" t="s">
         <v>120</v>
       </c>
-      <c r="D8" s="5" t="s">
+      <c r="D8" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="E8" s="3" t="s">
+      <c r="E8" s="2" t="s">
         <v>121</v>
       </c>
-      <c r="F8" s="5">
+      <c r="F8" s="6">
         <v>5</v>
       </c>
-      <c r="G8" s="5" t="s">
+      <c r="G8" s="6" t="s">
         <v>122</v>
       </c>
-      <c r="H8" s="3"/>
-      <c r="I8" s="3">
+      <c r="H8" s="2"/>
+      <c r="I8" s="2">
         <v>95</v>
       </c>
-      <c r="J8" s="5" t="s">
+      <c r="J8" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="K8" s="5">
+      <c r="K8" s="6">
         <v>1</v>
       </c>
-      <c r="L8" s="3" t="s">
+      <c r="L8" s="2" t="s">
         <v>107</v>
       </c>
-      <c r="M8" s="3" t="s">
+      <c r="M8" s="2" t="s">
         <v>120</v>
       </c>
-      <c r="N8" s="3" t="s">
+      <c r="N8" s="2" t="s">
         <v>120</v>
       </c>
-      <c r="O8" s="10" t="s">
+      <c r="O8" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="P8" s="10" t="s">
+      <c r="P8" s="7" t="s">
         <v>15</v>
       </c>
-      <c r="Q8" s="10" t="s">
+      <c r="Q8" s="7" t="s">
         <v>15</v>
       </c>
-      <c r="R8" s="3" t="s">
+      <c r="R8" s="2" t="s">
         <v>108</v>
       </c>
-      <c r="S8" s="11" t="s">
+      <c r="S8" s="10" t="s">
         <v>109</v>
       </c>
     </row>
     <row r="9" spans="1:19">
-      <c r="A9" s="5" t="s">
+      <c r="A9" s="6" t="s">
         <v>123</v>
       </c>
-      <c r="B9" s="5">
+      <c r="B9" s="6">
         <v>0</v>
       </c>
-      <c r="C9" s="3" t="s">
+      <c r="C9" s="2" t="s">
         <v>123</v>
       </c>
-      <c r="D9" s="5" t="s">
+      <c r="D9" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="E9" s="5" t="s">
+      <c r="E9" s="6" t="s">
         <v>40</v>
       </c>
-      <c r="F9" s="5">
+      <c r="F9" s="6">
         <v>12</v>
       </c>
-      <c r="G9" s="5" t="s">
+      <c r="G9" s="6" t="s">
         <v>122</v>
       </c>
-      <c r="H9" s="3"/>
-      <c r="I9" s="3">
+      <c r="H9" s="2"/>
+      <c r="I9" s="2">
         <v>97</v>
       </c>
-      <c r="J9" s="5" t="s">
+      <c r="J9" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="K9" s="5">
+      <c r="K9" s="6">
         <v>4</v>
       </c>
-      <c r="L9" s="3" t="s">
+      <c r="L9" s="2" t="s">
         <v>107</v>
       </c>
-      <c r="M9" s="5" t="s">
+      <c r="M9" s="6" t="s">
         <v>123</v>
       </c>
-      <c r="N9" s="5" t="s">
+      <c r="N9" s="6" t="s">
         <v>123</v>
       </c>
-      <c r="O9" s="10" t="s">
+      <c r="O9" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="P9" s="10" t="s">
+      <c r="P9" s="7" t="s">
         <v>15</v>
       </c>
-      <c r="Q9" s="10" t="s">
+      <c r="Q9" s="7" t="s">
         <v>15</v>
       </c>
-      <c r="R9" s="3" t="s">
+      <c r="R9" s="2" t="s">
         <v>108</v>
       </c>
-      <c r="S9" s="11" t="s">
+      <c r="S9" s="10" t="s">
         <v>109</v>
       </c>
     </row>
     <row r="10" spans="1:19">
-      <c r="A10" s="3" t="s">
+      <c r="A10" s="2" t="s">
         <v>124</v>
       </c>
-      <c r="B10" s="3">
+      <c r="B10" s="2">
         <v>0</v>
       </c>
-      <c r="C10" s="3" t="s">
+      <c r="C10" s="2" t="s">
         <v>124</v>
       </c>
-      <c r="D10" s="3" t="s">
+      <c r="D10" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="E10" s="3" t="s">
+      <c r="E10" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="F10" s="3">
+      <c r="F10" s="2">
         <v>12</v>
       </c>
-      <c r="G10" s="3" t="s">
+      <c r="G10" s="2" t="s">
         <v>125</v>
       </c>
-      <c r="H10" s="3"/>
-      <c r="I10" s="3"/>
-      <c r="J10" s="3" t="s">
+      <c r="H10" s="2"/>
+      <c r="I10" s="2"/>
+      <c r="J10" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="K10" s="3">
+      <c r="K10" s="2">
         <v>1</v>
       </c>
-      <c r="L10" s="3" t="s">
+      <c r="L10" s="2" t="s">
         <v>107</v>
       </c>
-      <c r="M10" s="3" t="s">
+      <c r="M10" s="2" t="s">
         <v>124</v>
       </c>
-      <c r="N10" s="3" t="s">
+      <c r="N10" s="2" t="s">
         <v>124</v>
       </c>
-      <c r="O10" s="3" t="s">
+      <c r="O10" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="P10" s="3" t="s">
+      <c r="P10" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="Q10" s="3" t="s">
+      <c r="Q10" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="R10" s="3" t="s">
+      <c r="R10" s="2" t="s">
         <v>108</v>
       </c>
-      <c r="S10" s="3" t="s">
+      <c r="S10" s="2" t="s">
         <v>109</v>
       </c>
     </row>
     <row r="11" spans="1:19">
-      <c r="A11" s="3" t="s">
+      <c r="A11" s="2" t="s">
         <v>126</v>
       </c>
-      <c r="B11" s="3">
+      <c r="B11" s="2">
         <v>0</v>
       </c>
-      <c r="C11" s="3" t="s">
+      <c r="C11" s="2" t="s">
         <v>126</v>
       </c>
-      <c r="D11" s="3" t="s">
+      <c r="D11" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="E11" s="3" t="s">
+      <c r="E11" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="F11" s="3">
+      <c r="F11" s="2">
         <v>12</v>
       </c>
-      <c r="G11" s="3" t="s">
+      <c r="G11" s="2" t="s">
         <v>125</v>
       </c>
-      <c r="H11" s="3"/>
-      <c r="I11" s="3"/>
-      <c r="J11" s="3" t="s">
+      <c r="H11" s="2"/>
+      <c r="I11" s="2"/>
+      <c r="J11" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="K11" s="3">
+      <c r="K11" s="2">
         <v>4</v>
       </c>
-      <c r="L11" s="3" t="s">
+      <c r="L11" s="2" t="s">
         <v>107</v>
       </c>
-      <c r="M11" s="3" t="s">
+      <c r="M11" s="2" t="s">
         <v>126</v>
       </c>
-      <c r="N11" s="3" t="s">
+      <c r="N11" s="2" t="s">
         <v>126</v>
       </c>
-      <c r="O11" s="3" t="s">
+      <c r="O11" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="P11" s="3" t="s">
+      <c r="P11" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="Q11" s="3" t="s">
+      <c r="Q11" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="R11" s="3" t="s">
+      <c r="R11" s="2" t="s">
         <v>108</v>
       </c>
-      <c r="S11" s="3" t="s">
+      <c r="S11" s="2" t="s">
         <v>109</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Added Production Order to MRV E2E Scenario and Fixed Failed Test Scenarios
Added Production Order to MRV E2E Scenario and Fixed Failed Test Scenarios in Employee Master, PO, Sales Invoice and Open SO Amendment
</commit_message>
<xml_diff>
--- a/testdata/ItemDetails.xlsx
+++ b/testdata/ItemDetails.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="23040" windowHeight="9120"/>
+    <workbookView windowWidth="19200" windowHeight="6920" firstSheet="7" activeTab="11"/>
   </bookViews>
   <sheets>
     <sheet name="PR Details" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="528" uniqueCount="194">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="549" uniqueCount="200">
   <si>
     <t>ITEM_NAME</t>
   </si>
@@ -607,6 +607,24 @@
   </si>
   <si>
     <t>SEZ-Unit</t>
+  </si>
+  <si>
+    <t>INKSPLASH PRINTING</t>
+  </si>
+  <si>
+    <t>SI - FREE SAMPLE</t>
+  </si>
+  <si>
+    <t>MALAR TRADERS</t>
+  </si>
+  <si>
+    <t>SI - FREE REPLACEMENT</t>
+  </si>
+  <si>
+    <t>URBAN ENTERPRISES</t>
+  </si>
+  <si>
+    <t>SI - SCRAP</t>
   </si>
   <si>
     <t>Item</t>
@@ -634,7 +652,7 @@
     <numFmt numFmtId="178" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
     <numFmt numFmtId="179" formatCode="_ &quot;₹&quot;* #,##0_ ;_ &quot;₹&quot;* \-#,##0_ ;_ &quot;₹&quot;* &quot;-&quot;_ ;_ @_ "/>
   </numFmts>
-  <fonts count="29">
+  <fonts count="30">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -649,6 +667,12 @@
       <name val="Calibri"/>
       <charset val="134"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
+      <charset val="134"/>
     </font>
     <font>
       <sz val="9"/>
@@ -1192,140 +1216,140 @@
     <xf numFmtId="179" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="2" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="6" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="7" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="7" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="8" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="6" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="7" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="7" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="8" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="28">
+  <cellXfs count="31">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -1341,10 +1365,16 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1">
@@ -1360,7 +1390,10 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
@@ -1369,7 +1402,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1">
@@ -1378,34 +1411,34 @@
     <xf numFmtId="49" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="49" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="49" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="49" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="49" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="justify" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -1943,338 +1976,338 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1:J20"/>
-  <sheetFormatPr defaultColWidth="8.71296296296296" defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultColWidth="8.70909090909091" defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="20.712962962963" customWidth="1"/>
-    <col min="2" max="3" width="12.712962962963" customWidth="1"/>
-    <col min="4" max="4" width="14.712962962963" customWidth="1"/>
-    <col min="5" max="5" width="9.85185185185185" customWidth="1"/>
-    <col min="6" max="6" width="14.1388888888889" customWidth="1"/>
-    <col min="7" max="7" width="14.8518518518519" customWidth="1"/>
-    <col min="8" max="8" width="22.2777777777778" customWidth="1"/>
-    <col min="9" max="9" width="14.4259259259259" customWidth="1"/>
+    <col min="1" max="1" width="20.7090909090909" customWidth="1"/>
+    <col min="2" max="3" width="12.7090909090909" customWidth="1"/>
+    <col min="4" max="4" width="14.7090909090909" customWidth="1"/>
+    <col min="5" max="5" width="9.85454545454546" customWidth="1"/>
+    <col min="6" max="6" width="14.1363636363636" customWidth="1"/>
+    <col min="7" max="7" width="14.8545454545455" customWidth="1"/>
+    <col min="8" max="8" width="22.2818181818182" customWidth="1"/>
+    <col min="9" max="9" width="14.4272727272727" customWidth="1"/>
     <col min="10" max="10" width="13" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:10">
-      <c r="A1" s="24" t="s">
+      <c r="A1" s="27" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="24" t="s">
+      <c r="B1" s="27" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="24" t="s">
+      <c r="C1" s="27" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="24" t="s">
+      <c r="D1" s="27" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="24" t="s">
+      <c r="E1" s="27" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="24" t="s">
+      <c r="F1" s="27" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="24" t="s">
+      <c r="G1" s="27" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="24" t="s">
+      <c r="H1" s="27" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="24" t="s">
+      <c r="I1" s="27" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="24" t="s">
+      <c r="J1" s="27" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="2" s="23" customFormat="1" ht="20.4" spans="1:10">
-      <c r="A2" s="25" t="s">
+    <row r="2" s="26" customFormat="1" ht="21" spans="1:10">
+      <c r="A2" s="28" t="s">
         <v>10</v>
       </c>
-      <c r="B2" s="26" t="s">
+      <c r="B2" s="29" t="s">
         <v>11</v>
       </c>
-      <c r="C2" s="26" t="s">
+      <c r="C2" s="29" t="s">
         <v>12</v>
       </c>
-      <c r="D2" s="25" t="s">
+      <c r="D2" s="28" t="s">
         <v>13</v>
       </c>
-      <c r="E2" s="25">
+      <c r="E2" s="28">
         <v>1</v>
       </c>
-      <c r="F2" s="25" t="s">
+      <c r="F2" s="28" t="s">
         <v>14</v>
       </c>
-      <c r="G2" s="25">
+      <c r="G2" s="28">
         <v>1010301033</v>
       </c>
-      <c r="H2" s="25" t="s">
+      <c r="H2" s="28" t="s">
         <v>15</v>
       </c>
-      <c r="I2" s="25" t="s">
+      <c r="I2" s="28" t="s">
         <v>16</v>
       </c>
-      <c r="J2" s="25" t="s">
+      <c r="J2" s="28" t="s">
         <v>17</v>
       </c>
     </row>
     <row r="3" ht="15" customHeight="1" spans="1:10">
-      <c r="A3" s="25" t="s">
+      <c r="A3" s="28" t="s">
         <v>18</v>
       </c>
-      <c r="B3" s="26" t="s">
+      <c r="B3" s="29" t="s">
         <v>11</v>
       </c>
-      <c r="C3" s="26" t="s">
+      <c r="C3" s="29" t="s">
         <v>12</v>
       </c>
-      <c r="D3" s="25" t="s">
+      <c r="D3" s="28" t="s">
         <v>19</v>
       </c>
-      <c r="E3" s="25">
+      <c r="E3" s="28">
         <v>6</v>
       </c>
-      <c r="F3" s="26" t="s">
+      <c r="F3" s="29" t="s">
         <v>20</v>
       </c>
-      <c r="G3" s="25">
+      <c r="G3" s="28">
         <v>1010301033</v>
       </c>
-      <c r="H3" s="25" t="s">
+      <c r="H3" s="28" t="s">
         <v>15</v>
       </c>
-      <c r="I3" s="25" t="s">
+      <c r="I3" s="28" t="s">
         <v>16</v>
       </c>
-      <c r="J3" s="25" t="s">
+      <c r="J3" s="28" t="s">
         <v>17</v>
       </c>
     </row>
     <row r="4" spans="1:10">
-      <c r="A4" s="25" t="s">
+      <c r="A4" s="28" t="s">
         <v>21</v>
       </c>
-      <c r="B4" s="26" t="s">
+      <c r="B4" s="29" t="s">
         <v>22</v>
       </c>
-      <c r="C4" s="26" t="s">
+      <c r="C4" s="29" t="s">
         <v>22</v>
       </c>
-      <c r="D4" s="25" t="s">
+      <c r="D4" s="28" t="s">
         <v>23</v>
       </c>
-      <c r="E4" s="25">
+      <c r="E4" s="28">
         <v>1</v>
       </c>
-      <c r="F4" s="26" t="s">
+      <c r="F4" s="29" t="s">
         <v>14</v>
       </c>
-      <c r="G4" s="25">
+      <c r="G4" s="28">
         <v>5010100004</v>
       </c>
-      <c r="H4" s="25" t="s">
+      <c r="H4" s="28" t="s">
         <v>24</v>
       </c>
-      <c r="I4" s="25" t="s">
+      <c r="I4" s="28" t="s">
         <v>16</v>
       </c>
-      <c r="J4" s="25" t="s">
+      <c r="J4" s="28" t="s">
         <v>17</v>
       </c>
     </row>
     <row r="5" spans="1:10">
-      <c r="A5" s="27"/>
-      <c r="B5" s="27"/>
-      <c r="C5" s="27"/>
-      <c r="D5" s="27"/>
-      <c r="E5" s="27"/>
-      <c r="F5" s="27"/>
-      <c r="G5" s="27"/>
-      <c r="H5" s="27"/>
-      <c r="I5" s="27"/>
-      <c r="J5" s="27"/>
+      <c r="A5" s="30"/>
+      <c r="B5" s="30"/>
+      <c r="C5" s="30"/>
+      <c r="D5" s="30"/>
+      <c r="E5" s="30"/>
+      <c r="F5" s="30"/>
+      <c r="G5" s="30"/>
+      <c r="H5" s="30"/>
+      <c r="I5" s="30"/>
+      <c r="J5" s="30"/>
     </row>
     <row r="6" spans="1:10">
-      <c r="A6" s="27"/>
-      <c r="B6" s="27"/>
-      <c r="C6" s="27"/>
-      <c r="D6" s="27"/>
-      <c r="E6" s="27"/>
-      <c r="F6" s="27"/>
-      <c r="G6" s="27"/>
-      <c r="H6" s="27"/>
-      <c r="I6" s="27"/>
-      <c r="J6" s="27"/>
+      <c r="A6" s="30"/>
+      <c r="B6" s="30"/>
+      <c r="C6" s="30"/>
+      <c r="D6" s="30"/>
+      <c r="E6" s="30"/>
+      <c r="F6" s="30"/>
+      <c r="G6" s="30"/>
+      <c r="H6" s="30"/>
+      <c r="I6" s="30"/>
+      <c r="J6" s="30"/>
     </row>
     <row r="7" spans="1:10">
-      <c r="A7" s="27"/>
-      <c r="B7" s="27"/>
-      <c r="C7" s="27"/>
-      <c r="D7" s="27"/>
-      <c r="E7" s="27"/>
-      <c r="F7" s="27"/>
-      <c r="G7" s="27"/>
-      <c r="H7" s="27"/>
-      <c r="I7" s="27"/>
-      <c r="J7" s="27"/>
+      <c r="A7" s="30"/>
+      <c r="B7" s="30"/>
+      <c r="C7" s="30"/>
+      <c r="D7" s="30"/>
+      <c r="E7" s="30"/>
+      <c r="F7" s="30"/>
+      <c r="G7" s="30"/>
+      <c r="H7" s="30"/>
+      <c r="I7" s="30"/>
+      <c r="J7" s="30"/>
     </row>
     <row r="8" spans="1:10">
-      <c r="A8" s="27"/>
-      <c r="B8" s="27"/>
-      <c r="C8" s="27"/>
-      <c r="D8" s="27"/>
-      <c r="E8" s="27"/>
-      <c r="F8" s="27"/>
-      <c r="G8" s="27"/>
-      <c r="H8" s="27"/>
-      <c r="I8" s="27"/>
-      <c r="J8" s="27"/>
+      <c r="A8" s="30"/>
+      <c r="B8" s="30"/>
+      <c r="C8" s="30"/>
+      <c r="D8" s="30"/>
+      <c r="E8" s="30"/>
+      <c r="F8" s="30"/>
+      <c r="G8" s="30"/>
+      <c r="H8" s="30"/>
+      <c r="I8" s="30"/>
+      <c r="J8" s="30"/>
     </row>
     <row r="9" spans="1:10">
-      <c r="A9" s="27"/>
-      <c r="B9" s="27"/>
-      <c r="C9" s="27"/>
-      <c r="D9" s="27"/>
-      <c r="E9" s="27"/>
-      <c r="F9" s="27"/>
-      <c r="G9" s="27"/>
-      <c r="H9" s="27"/>
-      <c r="I9" s="27"/>
-      <c r="J9" s="27"/>
+      <c r="A9" s="30"/>
+      <c r="B9" s="30"/>
+      <c r="C9" s="30"/>
+      <c r="D9" s="30"/>
+      <c r="E9" s="30"/>
+      <c r="F9" s="30"/>
+      <c r="G9" s="30"/>
+      <c r="H9" s="30"/>
+      <c r="I9" s="30"/>
+      <c r="J9" s="30"/>
     </row>
     <row r="10" spans="1:10">
-      <c r="A10" s="27"/>
-      <c r="B10" s="27"/>
-      <c r="C10" s="27"/>
-      <c r="D10" s="27"/>
-      <c r="E10" s="27"/>
-      <c r="F10" s="27"/>
-      <c r="G10" s="27"/>
-      <c r="H10" s="27"/>
-      <c r="I10" s="27"/>
-      <c r="J10" s="27"/>
+      <c r="A10" s="30"/>
+      <c r="B10" s="30"/>
+      <c r="C10" s="30"/>
+      <c r="D10" s="30"/>
+      <c r="E10" s="30"/>
+      <c r="F10" s="30"/>
+      <c r="G10" s="30"/>
+      <c r="H10" s="30"/>
+      <c r="I10" s="30"/>
+      <c r="J10" s="30"/>
     </row>
     <row r="11" spans="1:10">
-      <c r="A11" s="27"/>
-      <c r="B11" s="27"/>
-      <c r="C11" s="27"/>
-      <c r="D11" s="27"/>
-      <c r="E11" s="27"/>
-      <c r="F11" s="27"/>
-      <c r="G11" s="27"/>
-      <c r="H11" s="27"/>
-      <c r="I11" s="27"/>
-      <c r="J11" s="27"/>
+      <c r="A11" s="30"/>
+      <c r="B11" s="30"/>
+      <c r="C11" s="30"/>
+      <c r="D11" s="30"/>
+      <c r="E11" s="30"/>
+      <c r="F11" s="30"/>
+      <c r="G11" s="30"/>
+      <c r="H11" s="30"/>
+      <c r="I11" s="30"/>
+      <c r="J11" s="30"/>
     </row>
     <row r="12" spans="1:10">
-      <c r="A12" s="27"/>
-      <c r="B12" s="27"/>
-      <c r="C12" s="27"/>
-      <c r="D12" s="27"/>
-      <c r="E12" s="27"/>
-      <c r="F12" s="27"/>
-      <c r="G12" s="27"/>
-      <c r="H12" s="27"/>
-      <c r="I12" s="27"/>
-      <c r="J12" s="27"/>
+      <c r="A12" s="30"/>
+      <c r="B12" s="30"/>
+      <c r="C12" s="30"/>
+      <c r="D12" s="30"/>
+      <c r="E12" s="30"/>
+      <c r="F12" s="30"/>
+      <c r="G12" s="30"/>
+      <c r="H12" s="30"/>
+      <c r="I12" s="30"/>
+      <c r="J12" s="30"/>
     </row>
     <row r="13" spans="1:10">
-      <c r="A13" s="27"/>
-      <c r="B13" s="27"/>
-      <c r="C13" s="27"/>
-      <c r="D13" s="27"/>
-      <c r="E13" s="27"/>
-      <c r="F13" s="27"/>
-      <c r="G13" s="27"/>
-      <c r="H13" s="27"/>
-      <c r="I13" s="27"/>
-      <c r="J13" s="27"/>
+      <c r="A13" s="30"/>
+      <c r="B13" s="30"/>
+      <c r="C13" s="30"/>
+      <c r="D13" s="30"/>
+      <c r="E13" s="30"/>
+      <c r="F13" s="30"/>
+      <c r="G13" s="30"/>
+      <c r="H13" s="30"/>
+      <c r="I13" s="30"/>
+      <c r="J13" s="30"/>
     </row>
     <row r="14" spans="1:10">
-      <c r="A14" s="27"/>
-      <c r="B14" s="27"/>
-      <c r="C14" s="27"/>
-      <c r="D14" s="27"/>
-      <c r="E14" s="27"/>
-      <c r="F14" s="27"/>
-      <c r="G14" s="27"/>
-      <c r="H14" s="27"/>
-      <c r="I14" s="27"/>
-      <c r="J14" s="27"/>
+      <c r="A14" s="30"/>
+      <c r="B14" s="30"/>
+      <c r="C14" s="30"/>
+      <c r="D14" s="30"/>
+      <c r="E14" s="30"/>
+      <c r="F14" s="30"/>
+      <c r="G14" s="30"/>
+      <c r="H14" s="30"/>
+      <c r="I14" s="30"/>
+      <c r="J14" s="30"/>
     </row>
     <row r="15" spans="1:10">
-      <c r="A15" s="27"/>
-      <c r="B15" s="27"/>
-      <c r="C15" s="27"/>
-      <c r="D15" s="27"/>
-      <c r="E15" s="27"/>
-      <c r="F15" s="27"/>
-      <c r="G15" s="27"/>
-      <c r="H15" s="27"/>
-      <c r="I15" s="27"/>
-      <c r="J15" s="27"/>
+      <c r="A15" s="30"/>
+      <c r="B15" s="30"/>
+      <c r="C15" s="30"/>
+      <c r="D15" s="30"/>
+      <c r="E15" s="30"/>
+      <c r="F15" s="30"/>
+      <c r="G15" s="30"/>
+      <c r="H15" s="30"/>
+      <c r="I15" s="30"/>
+      <c r="J15" s="30"/>
     </row>
     <row r="16" spans="1:10">
-      <c r="A16" s="27"/>
-      <c r="B16" s="27"/>
-      <c r="C16" s="27"/>
-      <c r="D16" s="27"/>
-      <c r="E16" s="27"/>
-      <c r="F16" s="27"/>
-      <c r="G16" s="27"/>
-      <c r="H16" s="27"/>
-      <c r="I16" s="27"/>
-      <c r="J16" s="27"/>
+      <c r="A16" s="30"/>
+      <c r="B16" s="30"/>
+      <c r="C16" s="30"/>
+      <c r="D16" s="30"/>
+      <c r="E16" s="30"/>
+      <c r="F16" s="30"/>
+      <c r="G16" s="30"/>
+      <c r="H16" s="30"/>
+      <c r="I16" s="30"/>
+      <c r="J16" s="30"/>
     </row>
     <row r="17" spans="1:10">
-      <c r="A17" s="27"/>
-      <c r="B17" s="27"/>
-      <c r="C17" s="27"/>
-      <c r="D17" s="27"/>
-      <c r="E17" s="27"/>
-      <c r="F17" s="27"/>
-      <c r="G17" s="27"/>
-      <c r="H17" s="27"/>
-      <c r="I17" s="27"/>
-      <c r="J17" s="27"/>
+      <c r="A17" s="30"/>
+      <c r="B17" s="30"/>
+      <c r="C17" s="30"/>
+      <c r="D17" s="30"/>
+      <c r="E17" s="30"/>
+      <c r="F17" s="30"/>
+      <c r="G17" s="30"/>
+      <c r="H17" s="30"/>
+      <c r="I17" s="30"/>
+      <c r="J17" s="30"/>
     </row>
     <row r="18" spans="1:10">
-      <c r="A18" s="27"/>
-      <c r="B18" s="27"/>
-      <c r="C18" s="27"/>
-      <c r="D18" s="27"/>
-      <c r="E18" s="27"/>
-      <c r="F18" s="27"/>
-      <c r="G18" s="27"/>
-      <c r="H18" s="27"/>
-      <c r="I18" s="27"/>
-      <c r="J18" s="27"/>
+      <c r="A18" s="30"/>
+      <c r="B18" s="30"/>
+      <c r="C18" s="30"/>
+      <c r="D18" s="30"/>
+      <c r="E18" s="30"/>
+      <c r="F18" s="30"/>
+      <c r="G18" s="30"/>
+      <c r="H18" s="30"/>
+      <c r="I18" s="30"/>
+      <c r="J18" s="30"/>
     </row>
     <row r="19" spans="1:10">
-      <c r="A19" s="27"/>
-      <c r="B19" s="27"/>
-      <c r="C19" s="27"/>
-      <c r="D19" s="27"/>
-      <c r="E19" s="27"/>
-      <c r="F19" s="27"/>
-      <c r="G19" s="27"/>
-      <c r="H19" s="27"/>
-      <c r="I19" s="27"/>
-      <c r="J19" s="27"/>
+      <c r="A19" s="30"/>
+      <c r="B19" s="30"/>
+      <c r="C19" s="30"/>
+      <c r="D19" s="30"/>
+      <c r="E19" s="30"/>
+      <c r="F19" s="30"/>
+      <c r="G19" s="30"/>
+      <c r="H19" s="30"/>
+      <c r="I19" s="30"/>
+      <c r="J19" s="30"/>
     </row>
     <row r="20" spans="1:10">
-      <c r="A20" s="27"/>
-      <c r="B20" s="27"/>
-      <c r="C20" s="27"/>
-      <c r="D20" s="27"/>
-      <c r="E20" s="27"/>
-      <c r="F20" s="27"/>
-      <c r="G20" s="27"/>
-      <c r="H20" s="27"/>
-      <c r="I20" s="27"/>
-      <c r="J20" s="27"/>
+      <c r="A20" s="30"/>
+      <c r="B20" s="30"/>
+      <c r="C20" s="30"/>
+      <c r="D20" s="30"/>
+      <c r="E20" s="30"/>
+      <c r="F20" s="30"/>
+      <c r="G20" s="30"/>
+      <c r="H20" s="30"/>
+      <c r="I20" s="30"/>
+      <c r="J20" s="30"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2286,70 +2319,70 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1:K3"/>
-  <sheetFormatPr defaultColWidth="8.85185185185185" defaultRowHeight="14.4" outlineLevelRow="2"/>
+  <sheetFormatPr defaultColWidth="8.85454545454546" defaultRowHeight="14.5" outlineLevelRow="2"/>
   <cols>
     <col min="1" max="1" width="9" customWidth="1"/>
-    <col min="2" max="2" width="25.712962962963" customWidth="1"/>
-    <col min="3" max="3" width="12.4259259259259" customWidth="1"/>
-    <col min="4" max="4" width="16.2777777777778" customWidth="1"/>
-    <col min="5" max="5" width="20.2777777777778" customWidth="1"/>
-    <col min="6" max="6" width="25.712962962963" customWidth="1"/>
-    <col min="7" max="7" width="12.2777777777778" customWidth="1"/>
-    <col min="8" max="8" width="14.5740740740741" customWidth="1"/>
-    <col min="9" max="9" width="28.5740740740741" customWidth="1"/>
+    <col min="2" max="2" width="25.7090909090909" customWidth="1"/>
+    <col min="3" max="3" width="12.4272727272727" customWidth="1"/>
+    <col min="4" max="4" width="16.2818181818182" customWidth="1"/>
+    <col min="5" max="5" width="20.2818181818182" customWidth="1"/>
+    <col min="6" max="6" width="25.7090909090909" customWidth="1"/>
+    <col min="7" max="7" width="12.2818181818182" customWidth="1"/>
+    <col min="8" max="8" width="14.5727272727273" customWidth="1"/>
+    <col min="9" max="9" width="28.5727272727273" customWidth="1"/>
     <col min="10" max="10" width="23" customWidth="1"/>
-    <col min="11" max="11" width="14.712962962963" customWidth="1"/>
+    <col min="11" max="11" width="14.7090909090909" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:11">
-      <c r="A1" s="7" t="s">
+      <c r="A1" s="9" t="s">
         <v>127</v>
       </c>
-      <c r="B1" s="7" t="s">
+      <c r="B1" s="9" t="s">
         <v>128</v>
       </c>
-      <c r="C1" s="7" t="s">
+      <c r="C1" s="9" t="s">
         <v>129</v>
       </c>
-      <c r="D1" s="7" t="s">
+      <c r="D1" s="9" t="s">
         <v>130</v>
       </c>
-      <c r="E1" s="7" t="s">
+      <c r="E1" s="9" t="s">
         <v>131</v>
       </c>
-      <c r="F1" s="10" t="s">
+      <c r="F1" s="12" t="s">
         <v>132</v>
       </c>
-      <c r="G1" s="10" t="s">
+      <c r="G1" s="12" t="s">
         <v>133</v>
       </c>
-      <c r="H1" s="10" t="s">
+      <c r="H1" s="12" t="s">
         <v>134</v>
       </c>
-      <c r="I1" s="10" t="s">
+      <c r="I1" s="12" t="s">
         <v>135</v>
       </c>
-      <c r="J1" s="10" t="s">
+      <c r="J1" s="12" t="s">
         <v>136</v>
       </c>
-      <c r="K1" s="10" t="s">
+      <c r="K1" s="12" t="s">
         <v>137</v>
       </c>
     </row>
     <row r="2" spans="1:11">
-      <c r="A2" s="7" t="s">
+      <c r="A2" s="9" t="s">
         <v>138</v>
       </c>
-      <c r="B2" s="7" t="s">
+      <c r="B2" s="9" t="s">
         <v>139</v>
       </c>
-      <c r="C2" s="7" t="s">
+      <c r="C2" s="9" t="s">
         <v>140</v>
       </c>
-      <c r="D2" s="7" t="s">
+      <c r="D2" s="9" t="s">
         <v>141</v>
       </c>
-      <c r="E2" s="7" t="s">
+      <c r="E2" s="9" t="s">
         <v>142</v>
       </c>
       <c r="F2" s="2" t="s">
@@ -2372,13 +2405,13 @@
       </c>
     </row>
     <row r="3" spans="1:11">
-      <c r="A3" s="11" t="s">
+      <c r="A3" s="13" t="s">
         <v>148</v>
       </c>
       <c r="B3" s="2" t="s">
         <v>149</v>
       </c>
-      <c r="C3" s="7" t="s">
+      <c r="C3" s="9" t="s">
         <v>140</v>
       </c>
       <c r="D3" s="2" t="s">
@@ -2416,17 +2449,17 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1:E4"/>
-  <sheetFormatPr defaultColWidth="8.85185185185185" defaultRowHeight="14.4" outlineLevelRow="3" outlineLevelCol="4"/>
+  <sheetFormatPr defaultColWidth="8.85454545454546" defaultRowHeight="14.5" outlineLevelRow="3" outlineLevelCol="4"/>
   <cols>
-    <col min="1" max="1" width="13.5740740740741" customWidth="1"/>
+    <col min="1" max="1" width="13.5727272727273" customWidth="1"/>
     <col min="2" max="2" width="6" customWidth="1"/>
-    <col min="3" max="3" width="14.4259259259259" customWidth="1"/>
-    <col min="4" max="4" width="18.1388888888889" customWidth="1"/>
-    <col min="5" max="5" width="19.5740740740741" customWidth="1"/>
+    <col min="3" max="3" width="14.4272727272727" customWidth="1"/>
+    <col min="4" max="4" width="18.1363636363636" customWidth="1"/>
+    <col min="5" max="5" width="19.5727272727273" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5">
-      <c r="A1" s="7" t="s">
+      <c r="A1" s="9" t="s">
         <v>153</v>
       </c>
       <c r="B1" s="2" t="s">
@@ -2443,19 +2476,19 @@
       </c>
     </row>
     <row r="2" spans="1:5">
-      <c r="A2" s="7" t="s">
+      <c r="A2" s="9" t="s">
         <v>158</v>
       </c>
-      <c r="B2" s="7" t="s">
+      <c r="B2" s="9" t="s">
         <v>159</v>
       </c>
-      <c r="C2" s="8" t="s">
+      <c r="C2" s="10" t="s">
         <v>138</v>
       </c>
-      <c r="D2" s="9" t="s">
+      <c r="D2" s="11" t="s">
         <v>139</v>
       </c>
-      <c r="E2" s="7" t="s">
+      <c r="E2" s="9" t="s">
         <v>160</v>
       </c>
     </row>
@@ -2502,16 +2535,16 @@
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:G8"/>
-  <sheetFormatPr defaultColWidth="8.85185185185185" defaultRowHeight="14.4" outlineLevelRow="7" outlineLevelCol="6"/>
+  <dimension ref="A1:G11"/>
+  <sheetFormatPr defaultColWidth="8.85454545454546" defaultRowHeight="14.5" outlineLevelCol="6"/>
   <cols>
-    <col min="1" max="1" width="25.712962962963" customWidth="1"/>
-    <col min="2" max="2" width="8.85185185185185" customWidth="1"/>
-    <col min="3" max="3" width="12.2777777777778" customWidth="1"/>
-    <col min="4" max="4" width="7.13888888888889" customWidth="1"/>
-    <col min="5" max="5" width="5.27777777777778" customWidth="1"/>
-    <col min="6" max="6" width="17.4259259259259" customWidth="1"/>
-    <col min="7" max="7" width="12.4259259259259" customWidth="1"/>
+    <col min="1" max="1" width="25.7090909090909" customWidth="1"/>
+    <col min="2" max="2" width="8.85454545454546" customWidth="1"/>
+    <col min="3" max="3" width="12.2818181818182" customWidth="1"/>
+    <col min="4" max="4" width="7.13636363636364" customWidth="1"/>
+    <col min="5" max="5" width="5.28181818181818" customWidth="1"/>
+    <col min="6" max="6" width="17.4272727272727" customWidth="1"/>
+    <col min="7" max="7" width="12.4272727272727" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7">
@@ -2538,163 +2571,232 @@
       </c>
     </row>
     <row r="2" spans="1:7">
-      <c r="A2" s="2" t="s">
+      <c r="A2" s="5" t="s">
         <v>178</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="B2" s="5" t="s">
         <v>179</v>
       </c>
-      <c r="C2" s="5" t="s">
+      <c r="C2" s="6" t="s">
         <v>180</v>
       </c>
-      <c r="D2" s="5" t="s">
+      <c r="D2" s="6" t="s">
         <v>158</v>
       </c>
-      <c r="E2" s="5" t="s">
+      <c r="E2" s="6" t="s">
         <v>159</v>
       </c>
-      <c r="F2" s="2" t="s">
+      <c r="F2" s="5" t="s">
         <v>181</v>
       </c>
-      <c r="G2" s="2" t="s">
+      <c r="G2" s="5" t="s">
         <v>182</v>
       </c>
     </row>
     <row r="3" spans="1:7">
-      <c r="A3" s="2" t="s">
+      <c r="A3" s="5" t="s">
         <v>149</v>
       </c>
-      <c r="B3" s="2" t="s">
+      <c r="B3" s="5" t="s">
         <v>183</v>
       </c>
-      <c r="C3" s="5" t="s">
+      <c r="C3" s="6" t="s">
         <v>180</v>
       </c>
-      <c r="D3" s="5" t="s">
+      <c r="D3" s="6" t="s">
         <v>158</v>
       </c>
-      <c r="E3" s="5" t="s">
+      <c r="E3" s="6" t="s">
         <v>159</v>
       </c>
-      <c r="F3" s="2" t="s">
+      <c r="F3" s="5" t="s">
         <v>150</v>
       </c>
-      <c r="G3" s="2" t="s">
+      <c r="G3" s="5" t="s">
         <v>140</v>
       </c>
     </row>
     <row r="4" spans="1:7">
-      <c r="A4" s="2" t="s">
+      <c r="A4" s="5" t="s">
         <v>184</v>
       </c>
-      <c r="B4" s="2" t="s">
+      <c r="B4" s="5" t="s">
         <v>179</v>
       </c>
-      <c r="C4" s="5" t="s">
+      <c r="C4" s="6" t="s">
         <v>180</v>
       </c>
-      <c r="D4" s="5" t="s">
+      <c r="D4" s="6" t="s">
         <v>158</v>
       </c>
-      <c r="E4" s="5" t="s">
+      <c r="E4" s="6" t="s">
         <v>159</v>
       </c>
-      <c r="F4" s="2" t="s">
+      <c r="F4" s="5" t="s">
         <v>181</v>
       </c>
-      <c r="G4" s="2" t="s">
+      <c r="G4" s="5" t="s">
         <v>182</v>
       </c>
     </row>
     <row r="5" spans="1:7">
-      <c r="A5" s="2" t="s">
+      <c r="A5" s="5" t="s">
         <v>139</v>
       </c>
-      <c r="B5" s="2" t="s">
+      <c r="B5" s="5" t="s">
         <v>179</v>
       </c>
-      <c r="C5" s="5" t="s">
+      <c r="C5" s="6" t="s">
         <v>180</v>
       </c>
-      <c r="D5" s="5" t="s">
+      <c r="D5" s="6" t="s">
         <v>158</v>
       </c>
-      <c r="E5" s="5" t="s">
+      <c r="E5" s="6" t="s">
         <v>159</v>
       </c>
-      <c r="F5" s="6" t="s">
+      <c r="F5" s="5" t="s">
         <v>141</v>
       </c>
-      <c r="G5" s="2" t="s">
+      <c r="G5" s="5" t="s">
         <v>140</v>
       </c>
     </row>
     <row r="6" spans="1:7">
-      <c r="A6" s="2" t="s">
+      <c r="A6" s="5" t="s">
         <v>185</v>
       </c>
-      <c r="B6" s="2" t="s">
+      <c r="B6" s="5" t="s">
         <v>179</v>
       </c>
-      <c r="C6" s="5" t="s">
+      <c r="C6" s="6" t="s">
         <v>180</v>
       </c>
-      <c r="D6" s="5" t="s">
+      <c r="D6" s="6" t="s">
         <v>158</v>
       </c>
-      <c r="E6" s="5" t="s">
+      <c r="E6" s="6" t="s">
         <v>159</v>
       </c>
-      <c r="F6" s="2" t="s">
+      <c r="F6" s="5" t="s">
         <v>141</v>
       </c>
-      <c r="G6" s="2" t="s">
+      <c r="G6" s="5" t="s">
         <v>182</v>
       </c>
     </row>
     <row r="7" spans="1:7">
-      <c r="A7" s="2" t="s">
+      <c r="A7" s="5" t="s">
         <v>186</v>
       </c>
-      <c r="B7" s="2" t="s">
+      <c r="B7" s="5" t="s">
         <v>179</v>
       </c>
-      <c r="C7" s="5" t="s">
+      <c r="C7" s="6" t="s">
         <v>180</v>
       </c>
-      <c r="D7" s="5" t="s">
+      <c r="D7" s="6" t="s">
         <v>158</v>
       </c>
-      <c r="E7" s="5" t="s">
+      <c r="E7" s="6" t="s">
         <v>159</v>
       </c>
-      <c r="F7" s="2" t="s">
+      <c r="F7" s="5" t="s">
         <v>141</v>
       </c>
-      <c r="G7" s="2" t="s">
+      <c r="G7" s="5" t="s">
         <v>182</v>
       </c>
     </row>
     <row r="8" spans="1:7">
-      <c r="A8" s="2" t="s">
+      <c r="A8" s="5" t="s">
         <v>187</v>
       </c>
-      <c r="B8" s="2" t="s">
+      <c r="B8" s="5" t="s">
         <v>179</v>
       </c>
-      <c r="C8" s="5" t="s">
+      <c r="C8" s="6" t="s">
         <v>180</v>
       </c>
-      <c r="D8" s="5" t="s">
+      <c r="D8" s="6" t="s">
         <v>158</v>
       </c>
-      <c r="E8" s="5" t="s">
+      <c r="E8" s="6" t="s">
         <v>159</v>
       </c>
-      <c r="F8" s="2" t="s">
+      <c r="F8" s="5" t="s">
         <v>188</v>
       </c>
-      <c r="G8" s="2" t="s">
+      <c r="G8" s="5" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7">
+      <c r="A9" s="7" t="s">
+        <v>189</v>
+      </c>
+      <c r="B9" s="7" t="s">
+        <v>179</v>
+      </c>
+      <c r="C9" s="8" t="s">
+        <v>190</v>
+      </c>
+      <c r="D9" s="8" t="s">
+        <v>158</v>
+      </c>
+      <c r="E9" s="8" t="s">
+        <v>159</v>
+      </c>
+      <c r="F9" s="7" t="s">
+        <v>181</v>
+      </c>
+      <c r="G9" s="7" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7">
+      <c r="A10" s="7" t="s">
+        <v>191</v>
+      </c>
+      <c r="B10" s="7" t="s">
+        <v>179</v>
+      </c>
+      <c r="C10" s="8" t="s">
+        <v>192</v>
+      </c>
+      <c r="D10" s="8" t="s">
+        <v>158</v>
+      </c>
+      <c r="E10" s="8" t="s">
+        <v>159</v>
+      </c>
+      <c r="F10" s="7" t="s">
+        <v>181</v>
+      </c>
+      <c r="G10" s="7" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7">
+      <c r="A11" s="7" t="s">
+        <v>193</v>
+      </c>
+      <c r="B11" s="7" t="s">
+        <v>179</v>
+      </c>
+      <c r="C11" s="8" t="s">
+        <v>194</v>
+      </c>
+      <c r="D11" s="8" t="s">
+        <v>158</v>
+      </c>
+      <c r="E11" s="8" t="s">
+        <v>159</v>
+      </c>
+      <c r="F11" s="7" t="s">
+        <v>181</v>
+      </c>
+      <c r="G11" s="7" t="s">
         <v>182</v>
       </c>
     </row>
@@ -2708,19 +2810,19 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1:C3"/>
-  <sheetFormatPr defaultColWidth="8.88888888888889" defaultRowHeight="14.4" outlineLevelRow="2" outlineLevelCol="2"/>
+  <sheetFormatPr defaultColWidth="8.89090909090909" defaultRowHeight="14.5" outlineLevelRow="2" outlineLevelCol="2"/>
   <cols>
-    <col min="1" max="1" width="25.5555555555556" customWidth="1"/>
-    <col min="2" max="2" width="15.2222222222222" customWidth="1"/>
-    <col min="3" max="3" width="16.4444444444444" customWidth="1"/>
+    <col min="1" max="1" width="25.5545454545455" customWidth="1"/>
+    <col min="2" max="2" width="15.2181818181818" customWidth="1"/>
+    <col min="3" max="3" width="16.4454545454545" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3">
       <c r="A1" s="1" t="s">
-        <v>189</v>
+        <v>195</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>190</v>
+        <v>196</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>84</v>
@@ -2728,10 +2830,10 @@
     </row>
     <row r="2" spans="1:3">
       <c r="A2" s="2" t="s">
-        <v>191</v>
+        <v>197</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>192</v>
+        <v>198</v>
       </c>
       <c r="C2" s="2">
         <v>2</v>
@@ -2739,10 +2841,10 @@
     </row>
     <row r="3" spans="1:3">
       <c r="A3" s="2" t="s">
-        <v>193</v>
+        <v>199</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>192</v>
+        <v>198</v>
       </c>
       <c r="C3" s="2">
         <v>2</v>
@@ -2758,253 +2860,253 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1:T10"/>
-  <sheetFormatPr defaultColWidth="8.71296296296296" defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultColWidth="8.70909090909091" defaultRowHeight="14.5"/>
   <cols>
     <col min="1" max="1" width="30" customWidth="1"/>
-    <col min="2" max="2" width="36.4259259259259" customWidth="1"/>
+    <col min="2" max="2" width="36.4272727272727" customWidth="1"/>
     <col min="3" max="3" width="6" customWidth="1"/>
-    <col min="4" max="4" width="13.712962962963" customWidth="1"/>
-    <col min="5" max="5" width="5.27777777777778" customWidth="1"/>
-    <col min="6" max="6" width="17.2777777777778" customWidth="1"/>
-    <col min="7" max="7" width="30.2777777777778" customWidth="1"/>
-    <col min="8" max="8" width="26.8518518518519" customWidth="1"/>
-    <col min="9" max="9" width="17.2777777777778" customWidth="1"/>
-    <col min="10" max="10" width="13.2777777777778" customWidth="1"/>
-    <col min="11" max="11" width="22.712962962963" customWidth="1"/>
-    <col min="12" max="12" width="12.712962962963" customWidth="1"/>
-    <col min="13" max="13" width="29.5740740740741" customWidth="1"/>
-    <col min="14" max="14" width="18.2777777777778" customWidth="1"/>
-    <col min="15" max="15" width="16.2777777777778" customWidth="1"/>
-    <col min="16" max="16" width="15.5740740740741" customWidth="1"/>
-    <col min="17" max="17" width="17.712962962963" customWidth="1"/>
-    <col min="18" max="18" width="24.1388888888889" customWidth="1"/>
-    <col min="19" max="19" width="13.4259259259259" customWidth="1"/>
-    <col min="20" max="20" width="13.5740740740741" customWidth="1"/>
+    <col min="4" max="4" width="13.7090909090909" customWidth="1"/>
+    <col min="5" max="5" width="5.28181818181818" customWidth="1"/>
+    <col min="6" max="6" width="17.2818181818182" customWidth="1"/>
+    <col min="7" max="7" width="30.2818181818182" customWidth="1"/>
+    <col min="8" max="8" width="26.8545454545455" customWidth="1"/>
+    <col min="9" max="9" width="17.2818181818182" customWidth="1"/>
+    <col min="10" max="10" width="13.2818181818182" customWidth="1"/>
+    <col min="11" max="11" width="22.7090909090909" customWidth="1"/>
+    <col min="12" max="12" width="12.7090909090909" customWidth="1"/>
+    <col min="13" max="13" width="29.5727272727273" customWidth="1"/>
+    <col min="14" max="14" width="18.2818181818182" customWidth="1"/>
+    <col min="15" max="15" width="16.2818181818182" customWidth="1"/>
+    <col min="16" max="16" width="15.5727272727273" customWidth="1"/>
+    <col min="17" max="17" width="17.7090909090909" customWidth="1"/>
+    <col min="18" max="18" width="24.1363636363636" customWidth="1"/>
+    <col min="19" max="19" width="13.4272727272727" customWidth="1"/>
+    <col min="20" max="20" width="13.5727272727273" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:20">
-      <c r="A1" s="12" t="s">
+      <c r="A1" s="15" t="s">
         <v>25</v>
       </c>
-      <c r="B1" s="12" t="s">
+      <c r="B1" s="15" t="s">
         <v>26</v>
       </c>
-      <c r="C1" s="12" t="s">
+      <c r="C1" s="15" t="s">
         <v>27</v>
       </c>
-      <c r="D1" s="12" t="s">
+      <c r="D1" s="15" t="s">
         <v>28</v>
       </c>
-      <c r="E1" s="12" t="s">
+      <c r="E1" s="15" t="s">
         <v>29</v>
       </c>
-      <c r="F1" s="12" t="s">
+      <c r="F1" s="15" t="s">
         <v>2</v>
       </c>
-      <c r="G1" s="12" t="s">
+      <c r="G1" s="15" t="s">
         <v>1</v>
       </c>
-      <c r="H1" s="12" t="s">
+      <c r="H1" s="15" t="s">
         <v>30</v>
       </c>
-      <c r="I1" s="12" t="s">
+      <c r="I1" s="15" t="s">
         <v>31</v>
       </c>
-      <c r="J1" s="12" t="s">
+      <c r="J1" s="15" t="s">
         <v>32</v>
       </c>
-      <c r="K1" s="12" t="s">
+      <c r="K1" s="15" t="s">
         <v>33</v>
       </c>
-      <c r="L1" s="12" t="s">
+      <c r="L1" s="15" t="s">
         <v>6</v>
       </c>
-      <c r="M1" s="12" t="s">
+      <c r="M1" s="15" t="s">
         <v>7</v>
       </c>
-      <c r="N1" s="12" t="s">
+      <c r="N1" s="15" t="s">
         <v>8</v>
       </c>
-      <c r="O1" s="12" t="s">
+      <c r="O1" s="15" t="s">
         <v>9</v>
       </c>
-      <c r="P1" s="12" t="s">
+      <c r="P1" s="15" t="s">
         <v>34</v>
       </c>
-      <c r="Q1" s="12" t="s">
+      <c r="Q1" s="15" t="s">
         <v>35</v>
       </c>
-      <c r="R1" s="12" t="s">
+      <c r="R1" s="15" t="s">
         <v>36</v>
       </c>
-      <c r="S1" s="12" t="s">
+      <c r="S1" s="15" t="s">
         <v>37</v>
       </c>
-      <c r="T1" s="12" t="s">
+      <c r="T1" s="15" t="s">
         <v>38</v>
       </c>
     </row>
     <row r="2" spans="1:20">
-      <c r="A2" s="12" t="s">
+      <c r="A2" s="15" t="s">
         <v>18</v>
       </c>
-      <c r="B2" s="12" t="s">
+      <c r="B2" s="15" t="s">
         <v>39</v>
       </c>
-      <c r="C2" s="12" t="s">
+      <c r="C2" s="15" t="s">
         <v>20</v>
       </c>
-      <c r="D2" s="12" t="s">
+      <c r="D2" s="15" t="s">
         <v>40</v>
       </c>
-      <c r="E2" s="12">
+      <c r="E2" s="15">
         <v>12</v>
       </c>
-      <c r="F2" s="18" t="s">
+      <c r="F2" s="21" t="s">
         <v>12</v>
       </c>
-      <c r="G2" s="12" t="s">
+      <c r="G2" s="15" t="s">
         <v>11</v>
       </c>
-      <c r="H2" s="12" t="s">
+      <c r="H2" s="15" t="s">
         <v>19</v>
       </c>
-      <c r="I2" s="12" t="s">
+      <c r="I2" s="15" t="s">
         <v>41</v>
       </c>
-      <c r="J2" s="12" t="s">
+      <c r="J2" s="15" t="s">
         <v>14</v>
       </c>
-      <c r="K2" s="12">
+      <c r="K2" s="15">
         <v>6</v>
       </c>
-      <c r="L2" s="12">
+      <c r="L2" s="15">
         <v>1010301033</v>
       </c>
-      <c r="M2" s="12" t="s">
+      <c r="M2" s="15" t="s">
         <v>15</v>
       </c>
-      <c r="N2" s="12" t="s">
+      <c r="N2" s="15" t="s">
         <v>16</v>
       </c>
-      <c r="O2" s="12" t="s">
+      <c r="O2" s="15" t="s">
         <v>17</v>
       </c>
-      <c r="P2" s="12"/>
-      <c r="Q2" s="12"/>
-      <c r="R2" s="12"/>
-      <c r="S2" s="12">
+      <c r="P2" s="15"/>
+      <c r="Q2" s="15"/>
+      <c r="R2" s="15"/>
+      <c r="S2" s="15">
         <v>0</v>
       </c>
-      <c r="T2" s="12"/>
+      <c r="T2" s="15"/>
     </row>
     <row r="3" spans="1:20">
-      <c r="A3" s="12" t="s">
+      <c r="A3" s="15" t="s">
         <v>10</v>
       </c>
-      <c r="B3" s="12" t="s">
+      <c r="B3" s="15" t="s">
         <v>42</v>
       </c>
-      <c r="C3" s="12" t="s">
+      <c r="C3" s="15" t="s">
         <v>14</v>
       </c>
-      <c r="D3" s="19" t="s">
+      <c r="D3" s="22" t="s">
         <v>43</v>
       </c>
-      <c r="E3" s="12">
+      <c r="E3" s="15">
         <v>5</v>
       </c>
-      <c r="F3" s="12" t="s">
+      <c r="F3" s="15" t="s">
         <v>12</v>
       </c>
-      <c r="G3" s="12" t="s">
+      <c r="G3" s="15" t="s">
         <v>11</v>
       </c>
-      <c r="H3" s="12" t="s">
+      <c r="H3" s="15" t="s">
         <v>13</v>
       </c>
-      <c r="I3" s="12" t="s">
+      <c r="I3" s="15" t="s">
         <v>44</v>
       </c>
-      <c r="J3" s="12" t="s">
+      <c r="J3" s="15" t="s">
         <v>14</v>
       </c>
-      <c r="K3" s="12">
+      <c r="K3" s="15">
         <v>1</v>
       </c>
-      <c r="L3" s="12">
+      <c r="L3" s="15">
         <v>1010301033</v>
       </c>
-      <c r="M3" s="12" t="s">
+      <c r="M3" s="15" t="s">
         <v>15</v>
       </c>
-      <c r="N3" s="12" t="s">
+      <c r="N3" s="15" t="s">
         <v>16</v>
       </c>
-      <c r="O3" s="12" t="s">
+      <c r="O3" s="15" t="s">
         <v>17</v>
       </c>
-      <c r="P3" s="12"/>
-      <c r="Q3" s="12"/>
-      <c r="R3" s="12"/>
-      <c r="S3" s="12">
+      <c r="P3" s="15"/>
+      <c r="Q3" s="15"/>
+      <c r="R3" s="15"/>
+      <c r="S3" s="15">
         <v>0</v>
       </c>
-      <c r="T3" s="12"/>
+      <c r="T3" s="15"/>
     </row>
     <row r="4" spans="1:20">
-      <c r="A4" s="12" t="s">
+      <c r="A4" s="15" t="s">
         <v>21</v>
       </c>
-      <c r="B4" s="12" t="s">
+      <c r="B4" s="15" t="s">
         <v>45</v>
       </c>
-      <c r="C4" s="12" t="s">
+      <c r="C4" s="15" t="s">
         <v>14</v>
       </c>
-      <c r="D4" s="12">
+      <c r="D4" s="15">
         <v>123562</v>
       </c>
-      <c r="E4" s="12">
+      <c r="E4" s="15">
         <v>18</v>
       </c>
-      <c r="F4" s="12" t="s">
+      <c r="F4" s="15" t="s">
         <v>22</v>
       </c>
-      <c r="G4" s="12" t="s">
+      <c r="G4" s="15" t="s">
         <v>22</v>
       </c>
-      <c r="H4" s="12" t="s">
+      <c r="H4" s="15" t="s">
         <v>23</v>
       </c>
-      <c r="I4" s="12" t="s">
+      <c r="I4" s="15" t="s">
         <v>44</v>
       </c>
-      <c r="J4" s="12" t="s">
+      <c r="J4" s="15" t="s">
         <v>14</v>
       </c>
-      <c r="K4" s="12">
+      <c r="K4" s="15">
         <v>1</v>
       </c>
-      <c r="L4" s="12">
+      <c r="L4" s="15">
         <v>1011134888</v>
       </c>
-      <c r="M4" s="12" t="s">
+      <c r="M4" s="15" t="s">
         <v>46</v>
       </c>
-      <c r="N4" s="12" t="s">
+      <c r="N4" s="15" t="s">
         <v>16</v>
       </c>
-      <c r="O4" s="12" t="s">
+      <c r="O4" s="15" t="s">
         <v>17</v>
       </c>
-      <c r="P4" s="12"/>
-      <c r="Q4" s="12"/>
-      <c r="R4" s="12"/>
-      <c r="S4" s="12">
+      <c r="P4" s="15"/>
+      <c r="Q4" s="15"/>
+      <c r="R4" s="15"/>
+      <c r="S4" s="15">
         <v>0</v>
       </c>
-      <c r="T4" s="12"/>
+      <c r="T4" s="15"/>
     </row>
     <row r="5" spans="1:20">
       <c r="A5" s="2" t="s">
@@ -3013,7 +3115,7 @@
       <c r="B5" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="C5" s="12" t="s">
+      <c r="C5" s="15" t="s">
         <v>14</v>
       </c>
       <c r="D5" s="2" t="s">
@@ -3055,7 +3157,7 @@
       <c r="P5" s="2"/>
       <c r="Q5" s="2"/>
       <c r="R5" s="2"/>
-      <c r="S5" s="12">
+      <c r="S5" s="15">
         <v>0</v>
       </c>
       <c r="T5" s="2"/>
@@ -3070,16 +3172,16 @@
       <c r="C6" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="D6" s="17" t="s">
+      <c r="D6" s="20" t="s">
         <v>43</v>
       </c>
       <c r="E6">
         <v>5</v>
       </c>
-      <c r="F6" s="20" t="s">
+      <c r="F6" s="23" t="s">
         <v>12</v>
       </c>
-      <c r="G6" s="20" t="s">
+      <c r="G6" s="23" t="s">
         <v>11</v>
       </c>
       <c r="H6" s="2" t="s">
@@ -3109,172 +3211,172 @@
       <c r="P6" s="2"/>
       <c r="Q6" s="2"/>
       <c r="R6" s="2"/>
-      <c r="S6" s="12">
+      <c r="S6" s="15">
         <v>0</v>
       </c>
       <c r="T6" s="2"/>
     </row>
     <row r="7" spans="1:20">
-      <c r="A7" s="21" t="s">
+      <c r="A7" s="24" t="s">
         <v>55</v>
       </c>
-      <c r="B7" s="21" t="s">
+      <c r="B7" s="24" t="s">
         <v>56</v>
       </c>
-      <c r="C7" s="21" t="s">
+      <c r="C7" s="24" t="s">
         <v>20</v>
       </c>
-      <c r="D7" s="21" t="s">
+      <c r="D7" s="24" t="s">
         <v>40</v>
       </c>
-      <c r="E7" s="21">
+      <c r="E7" s="24">
         <v>12</v>
       </c>
-      <c r="F7" s="22" t="s">
+      <c r="F7" s="25" t="s">
         <v>12</v>
       </c>
-      <c r="G7" s="21" t="s">
+      <c r="G7" s="24" t="s">
         <v>11</v>
       </c>
-      <c r="H7" s="21" t="s">
+      <c r="H7" s="24" t="s">
         <v>57</v>
       </c>
-      <c r="I7" s="21" t="s">
+      <c r="I7" s="24" t="s">
         <v>41</v>
       </c>
-      <c r="J7" s="21" t="s">
+      <c r="J7" s="24" t="s">
         <v>14</v>
       </c>
-      <c r="K7" s="21">
+      <c r="K7" s="24">
         <v>3</v>
       </c>
-      <c r="L7" s="21">
+      <c r="L7" s="24">
         <v>1010301003</v>
       </c>
-      <c r="M7" s="21" t="s">
+      <c r="M7" s="24" t="s">
         <v>58</v>
       </c>
-      <c r="N7" s="21" t="s">
+      <c r="N7" s="24" t="s">
         <v>16</v>
       </c>
-      <c r="O7" s="21" t="s">
+      <c r="O7" s="24" t="s">
         <v>17</v>
       </c>
-      <c r="P7" s="21"/>
-      <c r="Q7" s="21"/>
-      <c r="R7" s="21"/>
-      <c r="S7" s="21">
+      <c r="P7" s="24"/>
+      <c r="Q7" s="24"/>
+      <c r="R7" s="24"/>
+      <c r="S7" s="24">
         <v>0</v>
       </c>
-      <c r="T7" s="21"/>
+      <c r="T7" s="24"/>
     </row>
     <row r="8" spans="1:20">
-      <c r="A8" s="21" t="s">
+      <c r="A8" s="24" t="s">
         <v>59</v>
       </c>
-      <c r="B8" s="21" t="s">
+      <c r="B8" s="24" t="s">
         <v>60</v>
       </c>
-      <c r="C8" s="21" t="s">
+      <c r="C8" s="24" t="s">
         <v>14</v>
       </c>
-      <c r="D8" s="21" t="s">
+      <c r="D8" s="24" t="s">
         <v>43</v>
       </c>
-      <c r="E8" s="21">
+      <c r="E8" s="24">
         <v>5</v>
       </c>
-      <c r="F8" s="22" t="s">
+      <c r="F8" s="25" t="s">
         <v>12</v>
       </c>
-      <c r="G8" s="21" t="s">
+      <c r="G8" s="24" t="s">
         <v>11</v>
       </c>
-      <c r="H8" s="21" t="s">
+      <c r="H8" s="24" t="s">
         <v>57</v>
       </c>
-      <c r="I8" s="21" t="s">
+      <c r="I8" s="24" t="s">
         <v>41</v>
       </c>
-      <c r="J8" s="21" t="s">
+      <c r="J8" s="24" t="s">
         <v>14</v>
       </c>
-      <c r="K8" s="21">
+      <c r="K8" s="24">
         <v>0</v>
       </c>
-      <c r="L8" s="21">
+      <c r="L8" s="24">
         <v>1010301003</v>
       </c>
-      <c r="M8" s="21" t="s">
+      <c r="M8" s="24" t="s">
         <v>58</v>
       </c>
-      <c r="N8" s="21" t="s">
+      <c r="N8" s="24" t="s">
         <v>16</v>
       </c>
-      <c r="O8" s="21" t="s">
+      <c r="O8" s="24" t="s">
         <v>17</v>
       </c>
-      <c r="P8" s="21"/>
-      <c r="Q8" s="21"/>
-      <c r="R8" s="21"/>
-      <c r="S8" s="21">
+      <c r="P8" s="24"/>
+      <c r="Q8" s="24"/>
+      <c r="R8" s="24"/>
+      <c r="S8" s="24">
         <v>0</v>
       </c>
-      <c r="T8" s="21"/>
+      <c r="T8" s="24"/>
     </row>
     <row r="9" spans="1:20">
-      <c r="A9" s="21" t="s">
+      <c r="A9" s="24" t="s">
         <v>61</v>
       </c>
-      <c r="B9" s="21" t="s">
+      <c r="B9" s="24" t="s">
         <v>61</v>
       </c>
-      <c r="C9" s="21" t="s">
+      <c r="C9" s="24" t="s">
         <v>14</v>
       </c>
-      <c r="D9" s="21" t="s">
+      <c r="D9" s="24" t="s">
         <v>43</v>
       </c>
-      <c r="E9" s="21">
+      <c r="E9" s="24">
         <v>5</v>
       </c>
-      <c r="F9" s="22" t="s">
+      <c r="F9" s="25" t="s">
         <v>12</v>
       </c>
-      <c r="G9" s="21" t="s">
+      <c r="G9" s="24" t="s">
         <v>11</v>
       </c>
-      <c r="H9" s="21" t="s">
+      <c r="H9" s="24" t="s">
         <v>57</v>
       </c>
-      <c r="I9" s="21" t="s">
+      <c r="I9" s="24" t="s">
         <v>41</v>
       </c>
-      <c r="J9" s="21" t="s">
+      <c r="J9" s="24" t="s">
         <v>14</v>
       </c>
-      <c r="K9" s="21">
+      <c r="K9" s="24">
         <v>0</v>
       </c>
-      <c r="L9" s="21">
+      <c r="L9" s="24">
         <v>1010301003</v>
       </c>
-      <c r="M9" s="21" t="s">
+      <c r="M9" s="24" t="s">
         <v>58</v>
       </c>
-      <c r="N9" s="21" t="s">
+      <c r="N9" s="24" t="s">
         <v>16</v>
       </c>
-      <c r="O9" s="21" t="s">
+      <c r="O9" s="24" t="s">
         <v>17</v>
       </c>
-      <c r="P9" s="21"/>
-      <c r="Q9" s="21"/>
-      <c r="R9" s="21"/>
-      <c r="S9" s="21">
+      <c r="P9" s="24"/>
+      <c r="Q9" s="24"/>
+      <c r="R9" s="24"/>
+      <c r="S9" s="24">
         <v>0</v>
       </c>
-      <c r="T9" s="21"/>
+      <c r="T9" s="24"/>
     </row>
     <row r="10" spans="1:20">
       <c r="A10" s="2" t="s">
@@ -3286,31 +3388,31 @@
       <c r="C10" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="D10" s="21" t="s">
+      <c r="D10" s="24" t="s">
         <v>43</v>
       </c>
-      <c r="E10" s="21">
+      <c r="E10" s="24">
         <v>5</v>
       </c>
-      <c r="F10" s="12" t="s">
+      <c r="F10" s="15" t="s">
         <v>22</v>
       </c>
-      <c r="G10" s="12" t="s">
+      <c r="G10" s="15" t="s">
         <v>22</v>
       </c>
-      <c r="H10" s="12" t="s">
+      <c r="H10" s="15" t="s">
         <v>63</v>
       </c>
-      <c r="I10" s="12" t="s">
+      <c r="I10" s="15" t="s">
         <v>44</v>
       </c>
-      <c r="J10" s="12" t="s">
+      <c r="J10" s="15" t="s">
         <v>14</v>
       </c>
-      <c r="K10" s="12">
+      <c r="K10" s="15">
         <v>1</v>
       </c>
-      <c r="L10" s="15">
+      <c r="L10" s="18">
         <v>1000000001</v>
       </c>
       <c r="M10" s="2" t="s">
@@ -3322,13 +3424,13 @@
       <c r="O10" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="P10" s="21"/>
-      <c r="Q10" s="21"/>
-      <c r="R10" s="21"/>
-      <c r="S10" s="21">
+      <c r="P10" s="24"/>
+      <c r="Q10" s="24"/>
+      <c r="R10" s="24"/>
+      <c r="S10" s="24">
         <v>0</v>
       </c>
-      <c r="T10" s="21"/>
+      <c r="T10" s="24"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -3340,19 +3442,19 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1:R3"/>
-  <sheetFormatPr defaultColWidth="8.85185185185185" defaultRowHeight="14.4" outlineLevelRow="2"/>
+  <sheetFormatPr defaultColWidth="8.85454545454546" defaultRowHeight="14.5" outlineLevelRow="2"/>
   <cols>
     <col min="1" max="2" width="21" customWidth="1"/>
     <col min="3" max="3" width="6" customWidth="1"/>
-    <col min="4" max="4" width="12.712962962963" customWidth="1"/>
-    <col min="5" max="5" width="19.4259259259259" customWidth="1"/>
-    <col min="6" max="6" width="15.1388888888889" customWidth="1"/>
-    <col min="7" max="7" width="15.4259259259259" customWidth="1"/>
-    <col min="8" max="8" width="19.5740740740741" customWidth="1"/>
-    <col min="9" max="9" width="10.8518518518519" customWidth="1"/>
-    <col min="10" max="10" width="17.5740740740741" customWidth="1"/>
-    <col min="11" max="11" width="11.2777777777778" customWidth="1"/>
-    <col min="12" max="12" width="21.712962962963" customWidth="1"/>
+    <col min="4" max="4" width="12.7090909090909" customWidth="1"/>
+    <col min="5" max="5" width="19.4272727272727" customWidth="1"/>
+    <col min="6" max="6" width="15.1363636363636" customWidth="1"/>
+    <col min="7" max="7" width="15.4272727272727" customWidth="1"/>
+    <col min="8" max="8" width="19.5727272727273" customWidth="1"/>
+    <col min="9" max="9" width="10.8545454545455" customWidth="1"/>
+    <col min="10" max="10" width="17.5727272727273" customWidth="1"/>
+    <col min="11" max="11" width="11.2818181818182" customWidth="1"/>
+    <col min="12" max="12" width="21.7090909090909" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:18">
@@ -3365,16 +3467,16 @@
       <c r="C1" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="D1" s="12" t="s">
+      <c r="D1" s="15" t="s">
         <v>6</v>
       </c>
-      <c r="E1" s="12" t="s">
+      <c r="E1" s="15" t="s">
         <v>7</v>
       </c>
-      <c r="F1" s="12" t="s">
+      <c r="F1" s="15" t="s">
         <v>8</v>
       </c>
-      <c r="G1" s="12" t="s">
+      <c r="G1" s="15" t="s">
         <v>9</v>
       </c>
       <c r="H1" s="2" t="s">
@@ -3392,12 +3494,12 @@
       <c r="L1" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="M1" s="16"/>
-      <c r="N1" s="16"/>
-      <c r="O1" s="16"/>
-      <c r="P1" s="16"/>
-      <c r="Q1" s="16"/>
-      <c r="R1" s="16"/>
+      <c r="M1" s="19"/>
+      <c r="N1" s="19"/>
+      <c r="O1" s="19"/>
+      <c r="P1" s="19"/>
+      <c r="Q1" s="19"/>
+      <c r="R1" s="19"/>
     </row>
     <row r="2" spans="1:18">
       <c r="A2" s="2" t="s">
@@ -3424,7 +3526,7 @@
       <c r="H2" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="I2" s="17" t="s">
+      <c r="I2" s="20" t="s">
         <v>43</v>
       </c>
       <c r="J2" s="2" t="s">
@@ -3436,12 +3538,12 @@
       <c r="L2" s="2">
         <v>1</v>
       </c>
-      <c r="M2" s="16"/>
-      <c r="N2" s="16"/>
-      <c r="O2" s="16"/>
-      <c r="P2" s="16"/>
-      <c r="Q2" s="16"/>
-      <c r="R2" s="16"/>
+      <c r="M2" s="19"/>
+      <c r="N2" s="19"/>
+      <c r="O2" s="19"/>
+      <c r="P2" s="19"/>
+      <c r="Q2" s="19"/>
+      <c r="R2" s="19"/>
     </row>
     <row r="3" spans="1:12">
       <c r="A3" s="2" t="s">
@@ -3453,7 +3555,7 @@
       <c r="C3" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="D3" s="15">
+      <c r="D3" s="18">
         <v>1000000001</v>
       </c>
       <c r="E3" s="2" t="s">
@@ -3468,7 +3570,7 @@
       <c r="H3" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="I3" s="17" t="s">
+      <c r="I3" s="20" t="s">
         <v>43</v>
       </c>
       <c r="J3" s="2" t="s">
@@ -3491,33 +3593,33 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1:F3"/>
-  <sheetFormatPr defaultColWidth="8.85185185185185" defaultRowHeight="14.4" outlineLevelRow="2" outlineLevelCol="5"/>
+  <sheetFormatPr defaultColWidth="8.85454545454546" defaultRowHeight="14.5" outlineLevelRow="2" outlineLevelCol="5"/>
   <cols>
-    <col min="1" max="1" width="27.1388888888889" customWidth="1"/>
-    <col min="2" max="2" width="10.4259259259259" customWidth="1"/>
-    <col min="3" max="3" width="11.4259259259259" customWidth="1"/>
-    <col min="4" max="4" width="11.712962962963" customWidth="1"/>
-    <col min="5" max="5" width="14.5740740740741" customWidth="1"/>
-    <col min="6" max="6" width="17.712962962963" customWidth="1"/>
+    <col min="1" max="1" width="27.1363636363636" customWidth="1"/>
+    <col min="2" max="2" width="10.4272727272727" customWidth="1"/>
+    <col min="3" max="3" width="11.4272727272727" customWidth="1"/>
+    <col min="4" max="4" width="11.7090909090909" customWidth="1"/>
+    <col min="5" max="5" width="14.5727272727273" customWidth="1"/>
+    <col min="6" max="6" width="17.7090909090909" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6">
-      <c r="A1" s="13" t="s">
+      <c r="A1" s="16" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="13" t="s">
+      <c r="B1" s="16" t="s">
         <v>66</v>
       </c>
-      <c r="C1" s="13" t="s">
+      <c r="C1" s="16" t="s">
         <v>67</v>
       </c>
-      <c r="D1" s="14" t="s">
+      <c r="D1" s="17" t="s">
         <v>68</v>
       </c>
-      <c r="E1" s="12" t="s">
+      <c r="E1" s="15" t="s">
         <v>69</v>
       </c>
-      <c r="F1" s="12" t="s">
+      <c r="F1" s="15" t="s">
         <v>70</v>
       </c>
     </row>
@@ -3535,7 +3637,7 @@
         <v>71</v>
       </c>
       <c r="E2" s="2"/>
-      <c r="F2" s="7" t="s">
+      <c r="F2" s="9" t="s">
         <v>72</v>
       </c>
     </row>
@@ -3552,10 +3654,10 @@
       <c r="D3" s="2" t="s">
         <v>73</v>
       </c>
-      <c r="E3" s="7" t="s">
+      <c r="E3" s="9" t="s">
         <v>74</v>
       </c>
-      <c r="F3" s="7">
+      <c r="F3" s="9">
         <v>2</v>
       </c>
     </row>
@@ -3569,38 +3671,38 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1:F4"/>
-  <sheetFormatPr defaultColWidth="8.85185185185185" defaultRowHeight="14.4" outlineLevelRow="3" outlineLevelCol="5"/>
+  <sheetFormatPr defaultColWidth="8.85454545454546" defaultRowHeight="14.5" outlineLevelRow="3" outlineLevelCol="5"/>
   <cols>
-    <col min="1" max="1" width="27.1388888888889" customWidth="1"/>
-    <col min="2" max="2" width="10.4259259259259" customWidth="1"/>
-    <col min="3" max="3" width="11.4259259259259" customWidth="1"/>
-    <col min="4" max="4" width="11.712962962963" customWidth="1"/>
-    <col min="5" max="5" width="14.5740740740741" customWidth="1"/>
-    <col min="6" max="6" width="17.712962962963" customWidth="1"/>
+    <col min="1" max="1" width="27.1363636363636" customWidth="1"/>
+    <col min="2" max="2" width="10.4272727272727" customWidth="1"/>
+    <col min="3" max="3" width="11.4272727272727" customWidth="1"/>
+    <col min="4" max="4" width="11.7090909090909" customWidth="1"/>
+    <col min="5" max="5" width="14.5727272727273" customWidth="1"/>
+    <col min="6" max="6" width="17.7090909090909" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6">
-      <c r="A1" s="13" t="s">
+      <c r="A1" s="16" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="13" t="s">
+      <c r="B1" s="16" t="s">
         <v>66</v>
       </c>
-      <c r="C1" s="13" t="s">
+      <c r="C1" s="16" t="s">
         <v>67</v>
       </c>
-      <c r="D1" s="14" t="s">
+      <c r="D1" s="17" t="s">
         <v>68</v>
       </c>
-      <c r="E1" s="12" t="s">
+      <c r="E1" s="15" t="s">
         <v>69</v>
       </c>
-      <c r="F1" s="12" t="s">
+      <c r="F1" s="15" t="s">
         <v>70</v>
       </c>
     </row>
     <row r="2" spans="1:6">
-      <c r="A2" s="12" t="s">
+      <c r="A2" s="15" t="s">
         <v>59</v>
       </c>
       <c r="B2" s="2">
@@ -3613,12 +3715,12 @@
         <v>71</v>
       </c>
       <c r="E2" s="2"/>
-      <c r="F2" s="7" t="s">
+      <c r="F2" s="9" t="s">
         <v>75</v>
       </c>
     </row>
     <row r="3" spans="1:6">
-      <c r="A3" s="12" t="s">
+      <c r="A3" s="15" t="s">
         <v>76</v>
       </c>
       <c r="B3" s="2">
@@ -3630,15 +3732,15 @@
       <c r="D3" s="2" t="s">
         <v>77</v>
       </c>
-      <c r="E3" s="7" t="s">
+      <c r="E3" s="9" t="s">
         <v>74</v>
       </c>
-      <c r="F3" s="7">
+      <c r="F3" s="9">
         <v>2</v>
       </c>
     </row>
     <row r="4" spans="1:6">
-      <c r="A4" s="12" t="s">
+      <c r="A4" s="15" t="s">
         <v>61</v>
       </c>
       <c r="B4" s="2">
@@ -3653,7 +3755,7 @@
       <c r="E4" s="2" t="s">
         <v>75</v>
       </c>
-      <c r="F4" s="7"/>
+      <c r="F4" s="9"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -3665,9 +3767,9 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1:C3"/>
-  <sheetFormatPr defaultColWidth="8.85185185185185" defaultRowHeight="14.4" outlineLevelRow="2" outlineLevelCol="2"/>
+  <sheetFormatPr defaultColWidth="8.85454545454546" defaultRowHeight="14.5" outlineLevelRow="2" outlineLevelCol="2"/>
   <cols>
-    <col min="1" max="1" width="28.712962962963" customWidth="1"/>
+    <col min="1" max="1" width="28.7090909090909" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3">
@@ -3713,80 +3815,80 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1:G4"/>
-  <sheetFormatPr defaultColWidth="8.85185185185185" defaultRowHeight="14.4" outlineLevelRow="3" outlineLevelCol="6"/>
+  <sheetFormatPr defaultColWidth="8.85454545454546" defaultRowHeight="14.5" outlineLevelRow="3" outlineLevelCol="6"/>
   <cols>
-    <col min="1" max="1" width="19.712962962963" customWidth="1"/>
-    <col min="2" max="2" width="8.13888888888889" customWidth="1"/>
-    <col min="3" max="3" width="8.57407407407407" customWidth="1"/>
-    <col min="4" max="4" width="17.8518518518519" customWidth="1"/>
-    <col min="5" max="5" width="12.712962962963" customWidth="1"/>
-    <col min="6" max="6" width="14.5740740740741" customWidth="1"/>
-    <col min="7" max="7" width="17.712962962963" customWidth="1"/>
+    <col min="1" max="1" width="19.7090909090909" customWidth="1"/>
+    <col min="2" max="2" width="8.13636363636364" customWidth="1"/>
+    <col min="3" max="3" width="8.57272727272727" customWidth="1"/>
+    <col min="4" max="4" width="17.8545454545455" customWidth="1"/>
+    <col min="5" max="5" width="12.7090909090909" customWidth="1"/>
+    <col min="6" max="6" width="14.5727272727273" customWidth="1"/>
+    <col min="7" max="7" width="17.7090909090909" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7">
-      <c r="A1" s="12" t="s">
+      <c r="A1" s="15" t="s">
         <v>83</v>
       </c>
-      <c r="B1" s="12" t="s">
+      <c r="B1" s="15" t="s">
         <v>84</v>
       </c>
-      <c r="C1" s="12" t="s">
+      <c r="C1" s="15" t="s">
         <v>80</v>
       </c>
-      <c r="D1" s="12" t="s">
+      <c r="D1" s="15" t="s">
         <v>85</v>
       </c>
-      <c r="E1" s="12" t="s">
+      <c r="E1" s="15" t="s">
         <v>68</v>
       </c>
-      <c r="F1" s="12" t="s">
+      <c r="F1" s="15" t="s">
         <v>69</v>
       </c>
-      <c r="G1" s="12" t="s">
+      <c r="G1" s="15" t="s">
         <v>70</v>
       </c>
     </row>
     <row r="2" spans="1:7">
-      <c r="A2" s="12" t="s">
+      <c r="A2" s="15" t="s">
         <v>86</v>
       </c>
-      <c r="B2" s="12">
+      <c r="B2" s="15">
         <v>524</v>
       </c>
-      <c r="C2" s="12">
+      <c r="C2" s="15">
         <v>524</v>
       </c>
-      <c r="D2" s="12">
+      <c r="D2" s="15">
         <v>2</v>
       </c>
-      <c r="E2" s="7" t="s">
+      <c r="E2" s="9" t="s">
         <v>71</v>
       </c>
-      <c r="F2" s="7" t="s">
+      <c r="F2" s="9" t="s">
         <v>74</v>
       </c>
-      <c r="G2" s="7" t="s">
+      <c r="G2" s="9" t="s">
         <v>87</v>
       </c>
     </row>
     <row r="3" spans="1:7">
-      <c r="A3" s="12" t="s">
+      <c r="A3" s="15" t="s">
         <v>88</v>
       </c>
-      <c r="B3" s="12">
+      <c r="B3" s="15">
         <v>232</v>
       </c>
-      <c r="C3" s="12">
+      <c r="C3" s="15">
         <v>232</v>
       </c>
-      <c r="D3" s="12">
+      <c r="D3" s="15">
         <v>7.9</v>
       </c>
-      <c r="E3" s="7" t="s">
+      <c r="E3" s="9" t="s">
         <v>73</v>
       </c>
-      <c r="F3" s="7" t="s">
+      <c r="F3" s="9" t="s">
         <v>89</v>
       </c>
       <c r="G3" s="2"/>
@@ -3804,7 +3906,7 @@
       <c r="D4" s="2">
         <v>2.32</v>
       </c>
-      <c r="E4" s="7" t="s">
+      <c r="E4" s="9" t="s">
         <v>77</v>
       </c>
       <c r="F4" s="2"/>
@@ -3820,80 +3922,80 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1:G4"/>
-  <sheetFormatPr defaultColWidth="8.85185185185185" defaultRowHeight="14.4" outlineLevelRow="3" outlineLevelCol="6"/>
+  <sheetFormatPr defaultColWidth="8.85454545454546" defaultRowHeight="14.5" outlineLevelRow="3" outlineLevelCol="6"/>
   <cols>
-    <col min="1" max="1" width="19.712962962963" customWidth="1"/>
-    <col min="2" max="2" width="8.13888888888889" customWidth="1"/>
-    <col min="3" max="3" width="8.57407407407407" customWidth="1"/>
-    <col min="4" max="4" width="17.8518518518519" customWidth="1"/>
-    <col min="5" max="5" width="12.712962962963" customWidth="1"/>
-    <col min="6" max="6" width="14.5740740740741" customWidth="1"/>
-    <col min="7" max="7" width="17.712962962963" customWidth="1"/>
+    <col min="1" max="1" width="19.7090909090909" customWidth="1"/>
+    <col min="2" max="2" width="8.13636363636364" customWidth="1"/>
+    <col min="3" max="3" width="8.57272727272727" customWidth="1"/>
+    <col min="4" max="4" width="17.8545454545455" customWidth="1"/>
+    <col min="5" max="5" width="12.7090909090909" customWidth="1"/>
+    <col min="6" max="6" width="14.5727272727273" customWidth="1"/>
+    <col min="7" max="7" width="17.7090909090909" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7">
-      <c r="A1" s="12" t="s">
+      <c r="A1" s="15" t="s">
         <v>83</v>
       </c>
-      <c r="B1" s="12" t="s">
+      <c r="B1" s="15" t="s">
         <v>84</v>
       </c>
-      <c r="C1" s="12" t="s">
+      <c r="C1" s="15" t="s">
         <v>80</v>
       </c>
-      <c r="D1" s="12" t="s">
+      <c r="D1" s="15" t="s">
         <v>85</v>
       </c>
-      <c r="E1" s="12" t="s">
+      <c r="E1" s="15" t="s">
         <v>68</v>
       </c>
-      <c r="F1" s="12" t="s">
+      <c r="F1" s="15" t="s">
         <v>69</v>
       </c>
-      <c r="G1" s="12" t="s">
+      <c r="G1" s="15" t="s">
         <v>70</v>
       </c>
     </row>
     <row r="2" spans="1:7">
-      <c r="A2" s="12" t="s">
+      <c r="A2" s="15" t="s">
         <v>86</v>
       </c>
-      <c r="B2" s="12">
+      <c r="B2" s="15">
         <v>22</v>
       </c>
-      <c r="C2" s="12">
+      <c r="C2" s="15">
         <v>524</v>
       </c>
-      <c r="D2" s="12">
+      <c r="D2" s="15">
         <v>2</v>
       </c>
-      <c r="E2" s="7" t="s">
+      <c r="E2" s="9" t="s">
         <v>71</v>
       </c>
-      <c r="F2" s="7" t="s">
+      <c r="F2" s="9" t="s">
         <v>74</v>
       </c>
-      <c r="G2" s="7" t="s">
+      <c r="G2" s="9" t="s">
         <v>87</v>
       </c>
     </row>
     <row r="3" spans="1:7">
-      <c r="A3" s="12" t="s">
+      <c r="A3" s="15" t="s">
         <v>88</v>
       </c>
-      <c r="B3" s="12">
+      <c r="B3" s="15">
         <v>34</v>
       </c>
-      <c r="C3" s="12">
+      <c r="C3" s="15">
         <v>232</v>
       </c>
-      <c r="D3" s="12">
+      <c r="D3" s="15">
         <v>7.9</v>
       </c>
-      <c r="E3" s="7" t="s">
+      <c r="E3" s="9" t="s">
         <v>73</v>
       </c>
-      <c r="F3" s="7" t="s">
+      <c r="F3" s="9" t="s">
         <v>89</v>
       </c>
       <c r="G3" s="2"/>
@@ -3911,7 +4013,7 @@
       <c r="D4" s="2">
         <v>2.32</v>
       </c>
-      <c r="E4" s="7" t="s">
+      <c r="E4" s="9" t="s">
         <v>77</v>
       </c>
       <c r="F4" s="2"/>
@@ -3927,25 +4029,25 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1:S11"/>
-  <sheetFormatPr defaultColWidth="8.85185185185185" defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultColWidth="8.85454545454546" defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="39.712962962963" customWidth="1"/>
-    <col min="2" max="2" width="10.1388888888889" customWidth="1"/>
-    <col min="3" max="3" width="39.712962962963" customWidth="1"/>
+    <col min="1" max="1" width="39.7090909090909" customWidth="1"/>
+    <col min="2" max="2" width="10.1363636363636" customWidth="1"/>
+    <col min="3" max="3" width="39.7090909090909" customWidth="1"/>
     <col min="4" max="4" width="11" customWidth="1"/>
-    <col min="5" max="5" width="13.2777777777778" customWidth="1"/>
-    <col min="6" max="6" width="8.85185185185185" customWidth="1"/>
-    <col min="7" max="7" width="17.8518518518519" customWidth="1"/>
-    <col min="8" max="8" width="19.5740740740741" customWidth="1"/>
-    <col min="9" max="9" width="23.712962962963" customWidth="1"/>
-    <col min="10" max="10" width="12.712962962963" customWidth="1"/>
-    <col min="11" max="11" width="11.8518518518519" customWidth="1"/>
-    <col min="12" max="12" width="17.4259259259259" customWidth="1"/>
-    <col min="13" max="14" width="39.712962962963" customWidth="1"/>
-    <col min="15" max="15" width="25.712962962963" customWidth="1"/>
-    <col min="16" max="17" width="16.5740740740741" customWidth="1"/>
-    <col min="18" max="18" width="11.5740740740741" customWidth="1"/>
-    <col min="19" max="19" width="14.8518518518519" customWidth="1"/>
+    <col min="5" max="5" width="13.2818181818182" customWidth="1"/>
+    <col min="6" max="6" width="8.85454545454546" customWidth="1"/>
+    <col min="7" max="7" width="17.8545454545455" customWidth="1"/>
+    <col min="8" max="8" width="19.5727272727273" customWidth="1"/>
+    <col min="9" max="9" width="23.7090909090909" customWidth="1"/>
+    <col min="10" max="10" width="12.7090909090909" customWidth="1"/>
+    <col min="11" max="11" width="11.8545454545455" customWidth="1"/>
+    <col min="12" max="12" width="17.4272727272727" customWidth="1"/>
+    <col min="13" max="14" width="39.7090909090909" customWidth="1"/>
+    <col min="15" max="15" width="25.7090909090909" customWidth="1"/>
+    <col min="16" max="17" width="16.5727272727273" customWidth="1"/>
+    <col min="18" max="18" width="11.5727272727273" customWidth="1"/>
+    <col min="19" max="19" width="14.8545454545455" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:19">
@@ -4003,18 +4105,18 @@
       <c r="R1" s="2" t="s">
         <v>104</v>
       </c>
-      <c r="S1" s="6" t="s">
+      <c r="S1" s="14" t="s">
         <v>105</v>
       </c>
     </row>
     <row r="2" spans="1:19">
-      <c r="A2" s="11" t="s">
+      <c r="A2" s="13" t="s">
         <v>106</v>
       </c>
       <c r="B2" s="2">
         <v>0</v>
       </c>
-      <c r="C2" s="11" t="s">
+      <c r="C2" s="13" t="s">
         <v>106</v>
       </c>
       <c r="D2" s="2" t="s">
@@ -4042,36 +4144,36 @@
       </c>
       <c r="M2" s="2"/>
       <c r="N2" s="2"/>
-      <c r="O2" s="7" t="s">
+      <c r="O2" s="9" t="s">
         <v>13</v>
       </c>
-      <c r="P2" s="7" t="s">
+      <c r="P2" s="9" t="s">
         <v>15</v>
       </c>
-      <c r="Q2" s="7" t="s">
+      <c r="Q2" s="9" t="s">
         <v>15</v>
       </c>
       <c r="R2" s="2" t="s">
         <v>108</v>
       </c>
-      <c r="S2" s="10" t="s">
+      <c r="S2" s="12" t="s">
         <v>109</v>
       </c>
     </row>
     <row r="3" spans="1:19">
-      <c r="A3" s="11" t="s">
+      <c r="A3" s="13" t="s">
         <v>110</v>
       </c>
       <c r="B3" s="2">
         <v>0</v>
       </c>
-      <c r="C3" s="11" t="s">
+      <c r="C3" s="13" t="s">
         <v>110</v>
       </c>
       <c r="D3" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="E3" s="11">
+      <c r="E3" s="13">
         <v>772213</v>
       </c>
       <c r="F3" s="2">
@@ -4093,19 +4195,19 @@
       </c>
       <c r="M3" s="2"/>
       <c r="N3" s="2"/>
-      <c r="O3" s="7" t="s">
+      <c r="O3" s="9" t="s">
         <v>13</v>
       </c>
-      <c r="P3" s="7" t="s">
+      <c r="P3" s="9" t="s">
         <v>15</v>
       </c>
-      <c r="Q3" s="7" t="s">
+      <c r="Q3" s="9" t="s">
         <v>15</v>
       </c>
       <c r="R3" s="2" t="s">
         <v>108</v>
       </c>
-      <c r="S3" s="10" t="s">
+      <c r="S3" s="12" t="s">
         <v>109</v>
       </c>
     </row>
@@ -4119,7 +4221,7 @@
       <c r="C4" s="2" t="s">
         <v>111</v>
       </c>
-      <c r="D4" s="6" t="s">
+      <c r="D4" s="14" t="s">
         <v>14</v>
       </c>
       <c r="E4" s="2" t="s">
@@ -4128,7 +4230,7 @@
       <c r="F4" s="2">
         <v>12</v>
       </c>
-      <c r="G4" s="6" t="s">
+      <c r="G4" s="14" t="s">
         <v>112</v>
       </c>
       <c r="H4" s="2"/>
@@ -4148,19 +4250,19 @@
       <c r="N4" s="2" t="s">
         <v>111</v>
       </c>
-      <c r="O4" s="7" t="s">
+      <c r="O4" s="9" t="s">
         <v>13</v>
       </c>
-      <c r="P4" s="7" t="s">
+      <c r="P4" s="9" t="s">
         <v>15</v>
       </c>
-      <c r="Q4" s="7" t="s">
+      <c r="Q4" s="9" t="s">
         <v>15</v>
       </c>
       <c r="R4" s="2" t="s">
         <v>108</v>
       </c>
-      <c r="S4" s="10" t="s">
+      <c r="S4" s="12" t="s">
         <v>109</v>
       </c>
     </row>
@@ -4168,30 +4270,30 @@
       <c r="A5" s="2" t="s">
         <v>113</v>
       </c>
-      <c r="B5" s="6">
+      <c r="B5" s="14">
         <v>0</v>
       </c>
       <c r="C5" s="2" t="s">
         <v>113</v>
       </c>
-      <c r="D5" s="6" t="s">
+      <c r="D5" s="14" t="s">
         <v>14</v>
       </c>
       <c r="E5" s="2">
         <v>75052200</v>
       </c>
-      <c r="F5" s="6">
+      <c r="F5" s="14">
         <v>5</v>
       </c>
-      <c r="G5" s="6" t="s">
+      <c r="G5" s="14" t="s">
         <v>112</v>
       </c>
       <c r="H5" s="2"/>
       <c r="I5" s="2"/>
-      <c r="J5" s="6" t="s">
+      <c r="J5" s="14" t="s">
         <v>20</v>
       </c>
-      <c r="K5" s="6">
+      <c r="K5" s="14">
         <v>2</v>
       </c>
       <c r="L5" s="2" t="s">
@@ -4203,133 +4305,133 @@
       <c r="N5" s="2" t="s">
         <v>113</v>
       </c>
-      <c r="O5" s="7" t="s">
+      <c r="O5" s="9" t="s">
         <v>13</v>
       </c>
-      <c r="P5" s="7" t="s">
+      <c r="P5" s="9" t="s">
         <v>15</v>
       </c>
-      <c r="Q5" s="7" t="s">
+      <c r="Q5" s="9" t="s">
         <v>15</v>
       </c>
       <c r="R5" s="2" t="s">
         <v>114</v>
       </c>
-      <c r="S5" s="10" t="s">
+      <c r="S5" s="12" t="s">
         <v>109</v>
       </c>
     </row>
     <row r="6" spans="1:19">
-      <c r="A6" s="6" t="s">
+      <c r="A6" s="14" t="s">
         <v>115</v>
       </c>
-      <c r="B6" s="6">
+      <c r="B6" s="14">
         <v>0</v>
       </c>
       <c r="C6" s="2" t="s">
         <v>115</v>
       </c>
-      <c r="D6" s="6" t="s">
+      <c r="D6" s="14" t="s">
         <v>14</v>
       </c>
-      <c r="E6" s="6" t="s">
+      <c r="E6" s="14" t="s">
         <v>40</v>
       </c>
-      <c r="F6" s="6">
+      <c r="F6" s="14">
         <v>12</v>
       </c>
-      <c r="G6" s="6" t="s">
+      <c r="G6" s="14" t="s">
         <v>116</v>
       </c>
-      <c r="H6" s="6" t="s">
+      <c r="H6" s="14" t="s">
         <v>117</v>
       </c>
       <c r="I6" s="2"/>
-      <c r="J6" s="6" t="s">
+      <c r="J6" s="14" t="s">
         <v>14</v>
       </c>
-      <c r="K6" s="6">
+      <c r="K6" s="14">
         <v>1</v>
       </c>
       <c r="L6" s="2" t="s">
         <v>107</v>
       </c>
-      <c r="M6" s="6" t="s">
+      <c r="M6" s="14" t="s">
         <v>115</v>
       </c>
-      <c r="N6" s="6" t="s">
+      <c r="N6" s="14" t="s">
         <v>115</v>
       </c>
-      <c r="O6" s="7" t="s">
+      <c r="O6" s="9" t="s">
         <v>13</v>
       </c>
-      <c r="P6" s="7" t="s">
+      <c r="P6" s="9" t="s">
         <v>15</v>
       </c>
-      <c r="Q6" s="7" t="s">
+      <c r="Q6" s="9" t="s">
         <v>15</v>
       </c>
       <c r="R6" s="2" t="s">
         <v>108</v>
       </c>
-      <c r="S6" s="10" t="s">
+      <c r="S6" s="12" t="s">
         <v>109</v>
       </c>
     </row>
     <row r="7" spans="1:19">
-      <c r="A7" s="6" t="s">
+      <c r="A7" s="14" t="s">
         <v>118</v>
       </c>
-      <c r="B7" s="6">
+      <c r="B7" s="14">
         <v>0</v>
       </c>
       <c r="C7" s="2" t="s">
         <v>118</v>
       </c>
-      <c r="D7" s="6" t="s">
+      <c r="D7" s="14" t="s">
         <v>14</v>
       </c>
-      <c r="E7" s="6" t="s">
+      <c r="E7" s="14" t="s">
         <v>40</v>
       </c>
-      <c r="F7" s="6">
+      <c r="F7" s="14">
         <v>12</v>
       </c>
-      <c r="G7" s="6" t="s">
+      <c r="G7" s="14" t="s">
         <v>116</v>
       </c>
-      <c r="H7" s="6" t="s">
+      <c r="H7" s="14" t="s">
         <v>119</v>
       </c>
       <c r="I7" s="2"/>
-      <c r="J7" s="6" t="s">
+      <c r="J7" s="14" t="s">
         <v>20</v>
       </c>
-      <c r="K7" s="6">
+      <c r="K7" s="14">
         <v>4</v>
       </c>
       <c r="L7" s="2" t="s">
         <v>107</v>
       </c>
-      <c r="M7" s="6" t="s">
+      <c r="M7" s="14" t="s">
         <v>118</v>
       </c>
-      <c r="N7" s="6" t="s">
+      <c r="N7" s="14" t="s">
         <v>118</v>
       </c>
-      <c r="O7" s="7" t="s">
+      <c r="O7" s="9" t="s">
         <v>13</v>
       </c>
-      <c r="P7" s="7" t="s">
+      <c r="P7" s="9" t="s">
         <v>15</v>
       </c>
-      <c r="Q7" s="7" t="s">
+      <c r="Q7" s="9" t="s">
         <v>15</v>
       </c>
       <c r="R7" s="2" t="s">
         <v>108</v>
       </c>
-      <c r="S7" s="10" t="s">
+      <c r="S7" s="12" t="s">
         <v>109</v>
       </c>
     </row>
@@ -4337,32 +4439,32 @@
       <c r="A8" s="2" t="s">
         <v>120</v>
       </c>
-      <c r="B8" s="6">
+      <c r="B8" s="14">
         <v>0</v>
       </c>
       <c r="C8" s="2" t="s">
         <v>120</v>
       </c>
-      <c r="D8" s="6" t="s">
+      <c r="D8" s="14" t="s">
         <v>14</v>
       </c>
       <c r="E8" s="2" t="s">
         <v>121</v>
       </c>
-      <c r="F8" s="6">
+      <c r="F8" s="14">
         <v>5</v>
       </c>
-      <c r="G8" s="6" t="s">
+      <c r="G8" s="14" t="s">
         <v>122</v>
       </c>
       <c r="H8" s="2"/>
       <c r="I8" s="2">
         <v>95</v>
       </c>
-      <c r="J8" s="6" t="s">
+      <c r="J8" s="14" t="s">
         <v>14</v>
       </c>
-      <c r="K8" s="6">
+      <c r="K8" s="14">
         <v>1</v>
       </c>
       <c r="L8" s="2" t="s">
@@ -4374,76 +4476,76 @@
       <c r="N8" s="2" t="s">
         <v>120</v>
       </c>
-      <c r="O8" s="7" t="s">
+      <c r="O8" s="9" t="s">
         <v>13</v>
       </c>
-      <c r="P8" s="7" t="s">
+      <c r="P8" s="9" t="s">
         <v>15</v>
       </c>
-      <c r="Q8" s="7" t="s">
+      <c r="Q8" s="9" t="s">
         <v>15</v>
       </c>
       <c r="R8" s="2" t="s">
         <v>108</v>
       </c>
-      <c r="S8" s="10" t="s">
+      <c r="S8" s="12" t="s">
         <v>109</v>
       </c>
     </row>
     <row r="9" spans="1:19">
-      <c r="A9" s="6" t="s">
+      <c r="A9" s="14" t="s">
         <v>123</v>
       </c>
-      <c r="B9" s="6">
+      <c r="B9" s="14">
         <v>0</v>
       </c>
       <c r="C9" s="2" t="s">
         <v>123</v>
       </c>
-      <c r="D9" s="6" t="s">
+      <c r="D9" s="14" t="s">
         <v>14</v>
       </c>
-      <c r="E9" s="6" t="s">
+      <c r="E9" s="14" t="s">
         <v>40</v>
       </c>
-      <c r="F9" s="6">
+      <c r="F9" s="14">
         <v>12</v>
       </c>
-      <c r="G9" s="6" t="s">
+      <c r="G9" s="14" t="s">
         <v>122</v>
       </c>
       <c r="H9" s="2"/>
       <c r="I9" s="2">
         <v>97</v>
       </c>
-      <c r="J9" s="6" t="s">
+      <c r="J9" s="14" t="s">
         <v>20</v>
       </c>
-      <c r="K9" s="6">
+      <c r="K9" s="14">
         <v>4</v>
       </c>
       <c r="L9" s="2" t="s">
         <v>107</v>
       </c>
-      <c r="M9" s="6" t="s">
+      <c r="M9" s="14" t="s">
         <v>123</v>
       </c>
-      <c r="N9" s="6" t="s">
+      <c r="N9" s="14" t="s">
         <v>123</v>
       </c>
-      <c r="O9" s="7" t="s">
+      <c r="O9" s="9" t="s">
         <v>13</v>
       </c>
-      <c r="P9" s="7" t="s">
+      <c r="P9" s="9" t="s">
         <v>15</v>
       </c>
-      <c r="Q9" s="7" t="s">
+      <c r="Q9" s="9" t="s">
         <v>15</v>
       </c>
       <c r="R9" s="2" t="s">
         <v>108</v>
       </c>
-      <c r="S9" s="10" t="s">
+      <c r="S9" s="12" t="s">
         <v>109</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Added DB Validations In Existing Methods Of Sales Order Functions
Added DB Validations In Existing Methods Of Sales Order Functions
</commit_message>
<xml_diff>
--- a/testdata/ItemDetails.xlsx
+++ b/testdata/ItemDetails.xlsx
@@ -1,10 +1,10 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
+  <fileVersion appName="xl" lastEdited="4" lowestEdited="5" rupBuild="4505"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="19200" windowHeight="6920" firstSheet="7" activeTab="11"/>
+    <workbookView xWindow="0" yWindow="2520" windowWidth="15150" windowHeight="5535" firstSheet="7" activeTab="8"/>
   </bookViews>
   <sheets>
     <sheet name="PR Details" sheetId="1" r:id="rId1"/>
@@ -21,7 +21,8 @@
     <sheet name="SI Details" sheetId="12" r:id="rId12"/>
     <sheet name="MRTOMRV Data" sheetId="13" r:id="rId13"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="124519"/>
+  <oleSize ref="N1:T7"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -645,14 +646,8 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="xr9">
-  <numFmts count="4">
-    <numFmt numFmtId="176" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
-    <numFmt numFmtId="177" formatCode="_ &quot;₹&quot;* #,##0.00_ ;_ &quot;₹&quot;* \-#,##0.00_ ;_ &quot;₹&quot;* &quot;-&quot;??_ ;_ @_ "/>
-    <numFmt numFmtId="178" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
-    <numFmt numFmtId="179" formatCode="_ &quot;₹&quot;* #,##0_ ;_ &quot;₹&quot;* \-#,##0_ ;_ &quot;₹&quot;* &quot;-&quot;_ ;_ @_ "/>
-  </numFmts>
-  <fonts count="30">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <fonts count="12">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -725,151 +720,14 @@
       <charset val="134"/>
     </font>
     <font>
-      <u/>
       <sz val="11"/>
-      <color rgb="FF0000FF"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <u/>
-      <sz val="11"/>
-      <color rgb="FF800080"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FFFF0000"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="18"/>
-      <color theme="3"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <charset val="134"/>
       <scheme val="minor"/>
     </font>
-    <font>
-      <i/>
-      <sz val="11"/>
-      <color rgb="FF7F7F7F"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="15"/>
-      <color theme="3"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="13"/>
-      <color theme="3"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="3"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF3F3F76"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FF3F3F3F"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FFFA7D00"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FFFFFFFF"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FFFA7D00"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF006100"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF9C0006"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF9C6500"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="0"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
   </fonts>
-  <fills count="35">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -878,7 +736,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.599993896298105"/>
+        <fgColor theme="9" tint="0.59999389629810485"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -894,188 +752,8 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFFCC"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFCC99"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFF2F2F2"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFA5A5A5"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFC6EFCE"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFC7CE"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFEB9C"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
   </fills>
-  <borders count="10">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -1098,254 +776,12 @@
       </bottom>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color rgb="FFB2B2B2"/>
-      </left>
-      <right style="thin">
-        <color rgb="FFB2B2B2"/>
-      </right>
-      <top style="thin">
-        <color rgb="FFB2B2B2"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FFB2B2B2"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="medium">
-        <color theme="4"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="medium">
-        <color theme="4" tint="0.499984740745262"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF7F7F7F"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF7F7F7F"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF7F7F7F"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF7F7F7F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF3F3F3F"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF3F3F3F"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF3F3F3F"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF3F3F3F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="double">
-        <color rgb="FF3F3F3F"/>
-      </left>
-      <right style="double">
-        <color rgb="FF3F3F3F"/>
-      </right>
-      <top style="double">
-        <color rgb="FF3F3F3F"/>
-      </top>
-      <bottom style="double">
-        <color rgb="FF3F3F3F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="double">
-        <color rgb="FFFF8001"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color theme="4"/>
-      </top>
-      <bottom style="double">
-        <color theme="4"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
-  <cellStyleXfs count="50">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="176" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="177" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="178" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="179" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="2" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="6" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="7" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="7" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="8" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
@@ -1420,10 +856,10 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="49" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="49" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -1442,90 +878,159 @@
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
-  <cellStyles count="50">
+  <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Comma" xfId="1" builtinId="3"/>
-    <cellStyle name="Currency" xfId="2" builtinId="4"/>
-    <cellStyle name="Percent" xfId="3" builtinId="5"/>
-    <cellStyle name="Comma [0]" xfId="4" builtinId="6"/>
-    <cellStyle name="Currency [0]" xfId="5" builtinId="7"/>
-    <cellStyle name="Hyperlink" xfId="6" builtinId="8"/>
-    <cellStyle name="Followed Hyperlink" xfId="7" builtinId="9"/>
-    <cellStyle name="Note" xfId="8" builtinId="10"/>
-    <cellStyle name="Warning Text" xfId="9" builtinId="11"/>
-    <cellStyle name="Title" xfId="10" builtinId="15"/>
-    <cellStyle name="CExplanatory Text" xfId="11" builtinId="53"/>
-    <cellStyle name="Heading 1" xfId="12" builtinId="16"/>
-    <cellStyle name="Heading 2" xfId="13" builtinId="17"/>
-    <cellStyle name="Heading 3" xfId="14" builtinId="18"/>
-    <cellStyle name="Heading 4" xfId="15" builtinId="19"/>
-    <cellStyle name="Input" xfId="16" builtinId="20"/>
-    <cellStyle name="Output" xfId="17" builtinId="21"/>
-    <cellStyle name="Calculation" xfId="18" builtinId="22"/>
-    <cellStyle name="Check Cell" xfId="19" builtinId="23"/>
-    <cellStyle name="Linked Cell" xfId="20" builtinId="24"/>
-    <cellStyle name="Total" xfId="21" builtinId="25"/>
-    <cellStyle name="Good" xfId="22" builtinId="26"/>
-    <cellStyle name="Bad" xfId="23" builtinId="27"/>
-    <cellStyle name="Neutral" xfId="24" builtinId="28"/>
-    <cellStyle name="Accent1" xfId="25" builtinId="29"/>
-    <cellStyle name="20% - Accent1" xfId="26" builtinId="30"/>
-    <cellStyle name="40% - Accent1" xfId="27" builtinId="31"/>
-    <cellStyle name="60% - Accent1" xfId="28" builtinId="32"/>
-    <cellStyle name="Accent2" xfId="29" builtinId="33"/>
-    <cellStyle name="20% - Accent2" xfId="30" builtinId="34"/>
-    <cellStyle name="40% - Accent2" xfId="31" builtinId="35"/>
-    <cellStyle name="60% - Accent2" xfId="32" builtinId="36"/>
-    <cellStyle name="Accent3" xfId="33" builtinId="37"/>
-    <cellStyle name="20% - Accent3" xfId="34" builtinId="38"/>
-    <cellStyle name="40% - Accent3" xfId="35" builtinId="39"/>
-    <cellStyle name="60% - Accent3" xfId="36" builtinId="40"/>
-    <cellStyle name="Accent4" xfId="37" builtinId="41"/>
-    <cellStyle name="20% - Accent4" xfId="38" builtinId="42"/>
-    <cellStyle name="40% - Accent4" xfId="39" builtinId="43"/>
-    <cellStyle name="60% - Accent4" xfId="40" builtinId="44"/>
-    <cellStyle name="Accent5" xfId="41" builtinId="45"/>
-    <cellStyle name="20% - Accent5" xfId="42" builtinId="46"/>
-    <cellStyle name="40% - Accent5" xfId="43" builtinId="47"/>
-    <cellStyle name="60% - Accent5" xfId="44" builtinId="48"/>
-    <cellStyle name="Accent6" xfId="45" builtinId="49"/>
-    <cellStyle name="20% - Accent6" xfId="46" builtinId="50"/>
-    <cellStyle name="40% - Accent6" xfId="47" builtinId="51"/>
-    <cellStyle name="60% - Accent6" xfId="48" builtinId="52"/>
-    <cellStyle name="Normal 2" xfId="49"/>
+    <cellStyle name="Normal 2" xfId="1"/>
   </cellStyles>
   <dxfs count="17">
     <dxf>
       <fill>
         <patternFill patternType="solid">
-          <fgColor theme="4" tint="0.799981688894314"/>
-          <bgColor theme="4" tint="0.799981688894314"/>
+          <fgColor theme="4" tint="0.79995117038483843"/>
+          <bgColor theme="4" tint="0.79995117038483843"/>
+        </patternFill>
+      </fill>
+      <border>
+        <bottom style="thin">
+          <color theme="4" tint="0.39994506668294322"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor theme="4" tint="0.79995117038483843"/>
+          <bgColor theme="4" tint="0.79995117038483843"/>
+        </patternFill>
+      </fill>
+      <border>
+        <bottom style="thin">
+          <color theme="4" tint="0.39994506668294322"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="1"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="1"/>
+      </font>
+      <border>
+        <bottom style="thin">
+          <color theme="4" tint="0.39994506668294322"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <color theme="1"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <color theme="1"/>
+      </font>
+      <border>
+        <top style="thin">
+          <color theme="4"/>
+        </top>
+        <bottom style="thin">
+          <color theme="4"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor theme="4" tint="0.79995117038483843"/>
+          <bgColor theme="4" tint="0.79995117038483843"/>
         </patternFill>
       </fill>
     </dxf>
     <dxf>
       <fill>
         <patternFill patternType="solid">
-          <fgColor theme="4" tint="0.799981688894314"/>
-          <bgColor theme="4" tint="0.799981688894314"/>
+          <fgColor theme="4" tint="0.79995117038483843"/>
+          <bgColor theme="4" tint="0.79995117038483843"/>
         </patternFill>
       </fill>
     </dxf>
     <dxf>
       <font>
-        <b val="1"/>
+        <b/>
+        <color theme="1"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor theme="4" tint="0.79995117038483843"/>
+          <bgColor theme="4" tint="0.79995117038483843"/>
+        </patternFill>
+      </fill>
+      <border>
+        <top style="thin">
+          <color theme="4" tint="0.39994506668294322"/>
+        </top>
+        <bottom style="thin">
+          <color theme="4" tint="0.39994506668294322"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <color theme="1"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor theme="4" tint="0.79995117038483843"/>
+          <bgColor theme="4" tint="0.79995117038483843"/>
+        </patternFill>
+      </fill>
+      <border>
+        <bottom style="thin">
+          <color theme="4" tint="0.39994506668294322"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor theme="4" tint="0.79995117038483843"/>
+          <bgColor theme="4" tint="0.79995117038483843"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor theme="4" tint="0.79995117038483843"/>
+          <bgColor theme="4" tint="0.79995117038483843"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
         <color theme="1"/>
       </font>
     </dxf>
     <dxf>
       <font>
-        <b val="1"/>
+        <b/>
         <color theme="1"/>
       </font>
     </dxf>
     <dxf>
       <font>
-        <b val="1"/>
+        <b/>
         <color theme="1"/>
       </font>
       <border>
@@ -1536,7 +1041,7 @@
     </dxf>
     <dxf>
       <font>
-        <b val="1"/>
+        <b/>
         <color theme="0"/>
       </font>
       <fill>
@@ -1564,149 +1069,32 @@
           <color theme="4"/>
         </bottom>
         <horizontal style="thin">
-          <color theme="4" tint="0.399975585192419"/>
+          <color theme="4" tint="0.39994506668294322"/>
         </horizontal>
-      </border>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor theme="4" tint="0.799981688894314"/>
-          <bgColor theme="4" tint="0.799981688894314"/>
-        </patternFill>
-      </fill>
-      <border>
-        <bottom style="thin">
-          <color theme="4" tint="0.399975585192419"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="1"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor theme="4" tint="0.799981688894314"/>
-          <bgColor theme="4" tint="0.799981688894314"/>
-        </patternFill>
-      </fill>
-      <border>
-        <bottom style="thin">
-          <color theme="4" tint="0.399975585192419"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="1"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="1"/>
-      </font>
-      <border>
-        <bottom style="thin">
-          <color theme="4" tint="0.399975585192419"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="1"/>
-        <color theme="1"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="1"/>
-        <color theme="1"/>
-      </font>
-      <border>
-        <top style="thin">
-          <color theme="4"/>
-        </top>
-        <bottom style="thin">
-          <color theme="4"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor theme="4" tint="0.799981688894314"/>
-          <bgColor theme="4" tint="0.799981688894314"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor theme="4" tint="0.799981688894314"/>
-          <bgColor theme="4" tint="0.799981688894314"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="1"/>
-        <color theme="1"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor theme="4" tint="0.799981688894314"/>
-          <bgColor theme="4" tint="0.799981688894314"/>
-        </patternFill>
-      </fill>
-      <border>
-        <top style="thin">
-          <color theme="4" tint="0.399975585192419"/>
-        </top>
-        <bottom style="thin">
-          <color theme="4" tint="0.399975585192419"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="1"/>
-        <color theme="1"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor theme="4" tint="0.799981688894314"/>
-          <bgColor theme="4" tint="0.799981688894314"/>
-        </patternFill>
-      </fill>
-      <border>
-        <bottom style="thin">
-          <color theme="4" tint="0.399975585192419"/>
-        </bottom>
       </border>
     </dxf>
   </dxfs>
   <tableStyles count="2" defaultTableStyle="TableStylePreset3_Accent1" defaultPivotStyle="PivotStylePreset2_Accent1">
-    <tableStyle name="TableStylePreset3_Accent1" pivot="0" count="7" xr9:uid="{59DB682C-5494-4EDE-A608-00C9E5F0F923}">
-      <tableStyleElement type="wholeTable" dxfId="6"/>
-      <tableStyleElement type="headerRow" dxfId="5"/>
-      <tableStyleElement type="totalRow" dxfId="4"/>
-      <tableStyleElement type="firstColumn" dxfId="3"/>
-      <tableStyleElement type="lastColumn" dxfId="2"/>
-      <tableStyleElement type="firstRowStripe" dxfId="1"/>
-      <tableStyleElement type="firstColumnStripe" dxfId="0"/>
+    <tableStyle name="TableStylePreset3_Accent1" pivot="0" count="7">
+      <tableStyleElement type="wholeTable" dxfId="16"/>
+      <tableStyleElement type="headerRow" dxfId="15"/>
+      <tableStyleElement type="totalRow" dxfId="14"/>
+      <tableStyleElement type="firstColumn" dxfId="13"/>
+      <tableStyleElement type="lastColumn" dxfId="12"/>
+      <tableStyleElement type="firstRowStripe" dxfId="11"/>
+      <tableStyleElement type="firstColumnStripe" dxfId="10"/>
     </tableStyle>
-    <tableStyle name="PivotStylePreset2_Accent1" table="0" count="10" xr9:uid="{267968C8-6FFD-4C36-ACC1-9EA1FD1885CA}">
-      <tableStyleElement type="headerRow" dxfId="16"/>
-      <tableStyleElement type="totalRow" dxfId="15"/>
-      <tableStyleElement type="firstRowStripe" dxfId="14"/>
-      <tableStyleElement type="firstColumnStripe" dxfId="13"/>
-      <tableStyleElement type="firstSubtotalRow" dxfId="12"/>
-      <tableStyleElement type="secondSubtotalRow" dxfId="11"/>
-      <tableStyleElement type="firstRowSubheading" dxfId="10"/>
-      <tableStyleElement type="secondRowSubheading" dxfId="9"/>
-      <tableStyleElement type="pageFieldLabels" dxfId="8"/>
-      <tableStyleElement type="pageFieldValues" dxfId="7"/>
+    <tableStyle name="PivotStylePreset2_Accent1" table="0" count="10">
+      <tableStyleElement type="headerRow" dxfId="9"/>
+      <tableStyleElement type="totalRow" dxfId="8"/>
+      <tableStyleElement type="firstRowStripe" dxfId="7"/>
+      <tableStyleElement type="firstColumnStripe" dxfId="6"/>
+      <tableStyleElement type="firstSubtotalRow" dxfId="5"/>
+      <tableStyleElement type="secondSubtotalRow" dxfId="4"/>
+      <tableStyleElement type="firstRowSubheading" dxfId="3"/>
+      <tableStyleElement type="secondRowSubheading" dxfId="2"/>
+      <tableStyleElement type="pageFieldLabels" dxfId="1"/>
+      <tableStyleElement type="pageFieldValues" dxfId="0"/>
     </tableStyle>
   </tableStyles>
   <extLst>
@@ -1969,23 +1357,23 @@
     </a:fmtScheme>
   </a:themeElements>
   <a:objectDefaults/>
+  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
-  <sheetPr/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:J20"/>
-  <sheetFormatPr defaultColWidth="8.70909090909091" defaultRowHeight="14.5"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="20.7090909090909" customWidth="1"/>
-    <col min="2" max="3" width="12.7090909090909" customWidth="1"/>
-    <col min="4" max="4" width="14.7090909090909" customWidth="1"/>
-    <col min="5" max="5" width="9.85454545454546" customWidth="1"/>
-    <col min="6" max="6" width="14.1363636363636" customWidth="1"/>
-    <col min="7" max="7" width="14.8545454545455" customWidth="1"/>
-    <col min="8" max="8" width="22.2818181818182" customWidth="1"/>
-    <col min="9" max="9" width="14.4272727272727" customWidth="1"/>
+    <col min="1" max="1" width="20.7109375" customWidth="1"/>
+    <col min="2" max="3" width="12.7109375" customWidth="1"/>
+    <col min="4" max="4" width="14.7109375" customWidth="1"/>
+    <col min="5" max="5" width="9.85546875" customWidth="1"/>
+    <col min="6" max="6" width="14.140625" customWidth="1"/>
+    <col min="7" max="7" width="14.85546875" customWidth="1"/>
+    <col min="8" max="8" width="22.28515625" customWidth="1"/>
+    <col min="9" max="9" width="14.42578125" customWidth="1"/>
     <col min="10" max="10" width="13" customWidth="1"/>
   </cols>
   <sheetData>
@@ -2021,7 +1409,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="2" s="26" customFormat="1" ht="21" spans="1:10">
+    <row r="2" spans="1:10" s="26" customFormat="1" ht="22.5">
       <c r="A2" s="28" t="s">
         <v>10</v>
       </c>
@@ -2053,7 +1441,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="3" ht="15" customHeight="1" spans="1:10">
+    <row r="3" spans="1:10" ht="15" customHeight="1">
       <c r="A3" s="28" t="s">
         <v>18</v>
       </c>
@@ -2085,7 +1473,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="4" spans="1:10">
+    <row r="4" spans="1:10" ht="22.5">
       <c r="A4" s="28" t="s">
         <v>21</v>
       </c>
@@ -2311,27 +1699,25 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
-  <sheetPr/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:K3"/>
-  <sheetFormatPr defaultColWidth="8.85454545454546" defaultRowHeight="14.5" outlineLevelRow="2"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="9" customWidth="1"/>
-    <col min="2" max="2" width="25.7090909090909" customWidth="1"/>
-    <col min="3" max="3" width="12.4272727272727" customWidth="1"/>
-    <col min="4" max="4" width="16.2818181818182" customWidth="1"/>
-    <col min="5" max="5" width="20.2818181818182" customWidth="1"/>
-    <col min="6" max="6" width="25.7090909090909" customWidth="1"/>
-    <col min="7" max="7" width="12.2818181818182" customWidth="1"/>
-    <col min="8" max="8" width="14.5727272727273" customWidth="1"/>
-    <col min="9" max="9" width="28.5727272727273" customWidth="1"/>
+    <col min="2" max="2" width="25.7109375" customWidth="1"/>
+    <col min="3" max="3" width="12.42578125" customWidth="1"/>
+    <col min="4" max="4" width="16.28515625" customWidth="1"/>
+    <col min="5" max="5" width="20.28515625" customWidth="1"/>
+    <col min="6" max="6" width="25.7109375" customWidth="1"/>
+    <col min="7" max="7" width="12.28515625" customWidth="1"/>
+    <col min="8" max="8" width="14.5703125" customWidth="1"/>
+    <col min="9" max="9" width="28.5703125" customWidth="1"/>
     <col min="10" max="10" width="23" customWidth="1"/>
-    <col min="11" max="11" width="14.7090909090909" customWidth="1"/>
+    <col min="11" max="11" width="14.7109375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:11">
@@ -2441,21 +1827,19 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
-  <sheetPr/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:E4"/>
-  <sheetFormatPr defaultColWidth="8.85454545454546" defaultRowHeight="14.5" outlineLevelRow="3" outlineLevelCol="4"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="13.5727272727273" customWidth="1"/>
+    <col min="1" max="1" width="13.5703125" customWidth="1"/>
     <col min="2" max="2" width="6" customWidth="1"/>
-    <col min="3" max="3" width="14.4272727272727" customWidth="1"/>
-    <col min="4" max="4" width="18.1363636363636" customWidth="1"/>
-    <col min="5" max="5" width="19.5727272727273" customWidth="1"/>
+    <col min="3" max="3" width="14.42578125" customWidth="1"/>
+    <col min="4" max="4" width="18.140625" customWidth="1"/>
+    <col min="5" max="5" width="19.5703125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5">
@@ -2475,7 +1859,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="2" spans="1:5">
+    <row r="2" spans="1:5" ht="30">
       <c r="A2" s="9" t="s">
         <v>158</v>
       </c>
@@ -2528,23 +1912,21 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
-  <sheetPr/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:G11"/>
-  <sheetFormatPr defaultColWidth="8.85454545454546" defaultRowHeight="14.5" outlineLevelCol="6"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="25.7090909090909" customWidth="1"/>
-    <col min="2" max="2" width="8.85454545454546" customWidth="1"/>
-    <col min="3" max="3" width="12.2818181818182" customWidth="1"/>
-    <col min="4" max="4" width="7.13636363636364" customWidth="1"/>
-    <col min="5" max="5" width="5.28181818181818" customWidth="1"/>
-    <col min="6" max="6" width="17.4272727272727" customWidth="1"/>
-    <col min="7" max="7" width="12.4272727272727" customWidth="1"/>
+    <col min="1" max="1" width="25.7109375" customWidth="1"/>
+    <col min="2" max="2" width="8.85546875" customWidth="1"/>
+    <col min="3" max="3" width="12.28515625" customWidth="1"/>
+    <col min="4" max="4" width="7.140625" customWidth="1"/>
+    <col min="5" max="5" width="5.28515625" customWidth="1"/>
+    <col min="6" max="6" width="17.42578125" customWidth="1"/>
+    <col min="7" max="7" width="12.42578125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7">
@@ -2802,19 +2184,17 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
-  <sheetPr/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:C3"/>
-  <sheetFormatPr defaultColWidth="8.89090909090909" defaultRowHeight="14.5" outlineLevelRow="2" outlineLevelCol="2"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="25.5545454545455" customWidth="1"/>
-    <col min="2" max="2" width="15.2181818181818" customWidth="1"/>
-    <col min="3" max="3" width="16.4454545454545" customWidth="1"/>
+    <col min="1" max="1" width="25.5703125" customWidth="1"/>
+    <col min="2" max="2" width="15.140625" customWidth="1"/>
+    <col min="3" max="3" width="16.42578125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3">
@@ -2852,36 +2232,34 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
-  <sheetPr/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:T10"/>
-  <sheetFormatPr defaultColWidth="8.70909090909091" defaultRowHeight="14.5"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="30" customWidth="1"/>
-    <col min="2" max="2" width="36.4272727272727" customWidth="1"/>
+    <col min="2" max="2" width="36.42578125" customWidth="1"/>
     <col min="3" max="3" width="6" customWidth="1"/>
-    <col min="4" max="4" width="13.7090909090909" customWidth="1"/>
-    <col min="5" max="5" width="5.28181818181818" customWidth="1"/>
-    <col min="6" max="6" width="17.2818181818182" customWidth="1"/>
-    <col min="7" max="7" width="30.2818181818182" customWidth="1"/>
-    <col min="8" max="8" width="26.8545454545455" customWidth="1"/>
-    <col min="9" max="9" width="17.2818181818182" customWidth="1"/>
-    <col min="10" max="10" width="13.2818181818182" customWidth="1"/>
-    <col min="11" max="11" width="22.7090909090909" customWidth="1"/>
-    <col min="12" max="12" width="12.7090909090909" customWidth="1"/>
-    <col min="13" max="13" width="29.5727272727273" customWidth="1"/>
-    <col min="14" max="14" width="18.2818181818182" customWidth="1"/>
-    <col min="15" max="15" width="16.2818181818182" customWidth="1"/>
-    <col min="16" max="16" width="15.5727272727273" customWidth="1"/>
-    <col min="17" max="17" width="17.7090909090909" customWidth="1"/>
-    <col min="18" max="18" width="24.1363636363636" customWidth="1"/>
-    <col min="19" max="19" width="13.4272727272727" customWidth="1"/>
-    <col min="20" max="20" width="13.5727272727273" customWidth="1"/>
+    <col min="4" max="4" width="13.7109375" customWidth="1"/>
+    <col min="5" max="5" width="5.28515625" customWidth="1"/>
+    <col min="6" max="6" width="17.28515625" customWidth="1"/>
+    <col min="7" max="7" width="30.28515625" customWidth="1"/>
+    <col min="8" max="8" width="26.85546875" customWidth="1"/>
+    <col min="9" max="9" width="17.28515625" customWidth="1"/>
+    <col min="10" max="10" width="13.28515625" customWidth="1"/>
+    <col min="11" max="11" width="22.7109375" customWidth="1"/>
+    <col min="12" max="12" width="12.7109375" customWidth="1"/>
+    <col min="13" max="13" width="29.5703125" customWidth="1"/>
+    <col min="14" max="14" width="18.28515625" customWidth="1"/>
+    <col min="15" max="15" width="16.28515625" customWidth="1"/>
+    <col min="16" max="16" width="15.5703125" customWidth="1"/>
+    <col min="17" max="17" width="17.7109375" customWidth="1"/>
+    <col min="18" max="18" width="24.140625" customWidth="1"/>
+    <col min="19" max="19" width="13.42578125" customWidth="1"/>
+    <col min="20" max="20" width="13.5703125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:20">
@@ -3434,27 +2812,25 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
-  <sheetPr/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:R3"/>
-  <sheetFormatPr defaultColWidth="8.85454545454546" defaultRowHeight="14.5" outlineLevelRow="2"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="2" width="21" customWidth="1"/>
     <col min="3" max="3" width="6" customWidth="1"/>
-    <col min="4" max="4" width="12.7090909090909" customWidth="1"/>
-    <col min="5" max="5" width="19.4272727272727" customWidth="1"/>
-    <col min="6" max="6" width="15.1363636363636" customWidth="1"/>
-    <col min="7" max="7" width="15.4272727272727" customWidth="1"/>
-    <col min="8" max="8" width="19.5727272727273" customWidth="1"/>
-    <col min="9" max="9" width="10.8545454545455" customWidth="1"/>
-    <col min="10" max="10" width="17.5727272727273" customWidth="1"/>
-    <col min="11" max="11" width="11.2818181818182" customWidth="1"/>
-    <col min="12" max="12" width="21.7090909090909" customWidth="1"/>
+    <col min="4" max="4" width="12.7109375" customWidth="1"/>
+    <col min="5" max="5" width="19.42578125" customWidth="1"/>
+    <col min="6" max="6" width="15.140625" customWidth="1"/>
+    <col min="7" max="7" width="15.42578125" customWidth="1"/>
+    <col min="8" max="8" width="19.5703125" customWidth="1"/>
+    <col min="9" max="9" width="10.85546875" customWidth="1"/>
+    <col min="10" max="10" width="17.5703125" customWidth="1"/>
+    <col min="11" max="11" width="11.28515625" customWidth="1"/>
+    <col min="12" max="12" width="21.7109375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:18">
@@ -3545,7 +2921,7 @@
       <c r="Q2" s="19"/>
       <c r="R2" s="19"/>
     </row>
-    <row r="3" spans="1:12">
+    <row r="3" spans="1:18">
       <c r="A3" s="2" t="s">
         <v>62</v>
       </c>
@@ -3585,22 +2961,20 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
-  <sheetPr/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:F3"/>
-  <sheetFormatPr defaultColWidth="8.85454545454546" defaultRowHeight="14.5" outlineLevelRow="2" outlineLevelCol="5"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="27.1363636363636" customWidth="1"/>
-    <col min="2" max="2" width="10.4272727272727" customWidth="1"/>
-    <col min="3" max="3" width="11.4272727272727" customWidth="1"/>
-    <col min="4" max="4" width="11.7090909090909" customWidth="1"/>
-    <col min="5" max="5" width="14.5727272727273" customWidth="1"/>
-    <col min="6" max="6" width="17.7090909090909" customWidth="1"/>
+    <col min="1" max="1" width="27.140625" customWidth="1"/>
+    <col min="2" max="2" width="10.42578125" customWidth="1"/>
+    <col min="3" max="3" width="11.42578125" customWidth="1"/>
+    <col min="4" max="4" width="11.7109375" customWidth="1"/>
+    <col min="5" max="5" width="14.5703125" customWidth="1"/>
+    <col min="6" max="6" width="17.7109375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6">
@@ -3663,22 +3037,20 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
-  <sheetPr/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:F4"/>
-  <sheetFormatPr defaultColWidth="8.85454545454546" defaultRowHeight="14.5" outlineLevelRow="3" outlineLevelCol="5"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="27.1363636363636" customWidth="1"/>
-    <col min="2" max="2" width="10.4272727272727" customWidth="1"/>
-    <col min="3" max="3" width="11.4272727272727" customWidth="1"/>
-    <col min="4" max="4" width="11.7090909090909" customWidth="1"/>
-    <col min="5" max="5" width="14.5727272727273" customWidth="1"/>
-    <col min="6" max="6" width="17.7090909090909" customWidth="1"/>
+    <col min="1" max="1" width="27.140625" customWidth="1"/>
+    <col min="2" max="2" width="10.42578125" customWidth="1"/>
+    <col min="3" max="3" width="11.42578125" customWidth="1"/>
+    <col min="4" max="4" width="11.7109375" customWidth="1"/>
+    <col min="5" max="5" width="14.5703125" customWidth="1"/>
+    <col min="6" max="6" width="17.7109375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6">
@@ -3759,17 +3131,15 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
-  <sheetPr/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:C3"/>
-  <sheetFormatPr defaultColWidth="8.85454545454546" defaultRowHeight="14.5" outlineLevelRow="2" outlineLevelCol="2"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="28.7090909090909" customWidth="1"/>
+    <col min="1" max="1" width="28.7109375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3">
@@ -3807,23 +3177,21 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
-  <sheetPr/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:G4"/>
-  <sheetFormatPr defaultColWidth="8.85454545454546" defaultRowHeight="14.5" outlineLevelRow="3" outlineLevelCol="6"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="19.7090909090909" customWidth="1"/>
-    <col min="2" max="2" width="8.13636363636364" customWidth="1"/>
-    <col min="3" max="3" width="8.57272727272727" customWidth="1"/>
-    <col min="4" max="4" width="17.8545454545455" customWidth="1"/>
-    <col min="5" max="5" width="12.7090909090909" customWidth="1"/>
-    <col min="6" max="6" width="14.5727272727273" customWidth="1"/>
-    <col min="7" max="7" width="17.7090909090909" customWidth="1"/>
+    <col min="1" max="1" width="19.7109375" customWidth="1"/>
+    <col min="2" max="2" width="8.140625" customWidth="1"/>
+    <col min="3" max="3" width="8.5703125" customWidth="1"/>
+    <col min="4" max="4" width="17.85546875" customWidth="1"/>
+    <col min="5" max="5" width="12.7109375" customWidth="1"/>
+    <col min="6" max="6" width="14.5703125" customWidth="1"/>
+    <col min="7" max="7" width="17.7109375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7">
@@ -3904,7 +3272,7 @@
         <v>232</v>
       </c>
       <c r="D4" s="2">
-        <v>2.32</v>
+        <v>2.3199999999999998</v>
       </c>
       <c r="E4" s="9" t="s">
         <v>77</v>
@@ -3914,23 +3282,21 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
-  <sheetPr/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:G4"/>
-  <sheetFormatPr defaultColWidth="8.85454545454546" defaultRowHeight="14.5" outlineLevelRow="3" outlineLevelCol="6"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="19.7090909090909" customWidth="1"/>
-    <col min="2" max="2" width="8.13636363636364" customWidth="1"/>
-    <col min="3" max="3" width="8.57272727272727" customWidth="1"/>
-    <col min="4" max="4" width="17.8545454545455" customWidth="1"/>
-    <col min="5" max="5" width="12.7090909090909" customWidth="1"/>
-    <col min="6" max="6" width="14.5727272727273" customWidth="1"/>
-    <col min="7" max="7" width="17.7090909090909" customWidth="1"/>
+    <col min="1" max="1" width="19.7109375" customWidth="1"/>
+    <col min="2" max="2" width="8.140625" customWidth="1"/>
+    <col min="3" max="3" width="8.5703125" customWidth="1"/>
+    <col min="4" max="4" width="17.85546875" customWidth="1"/>
+    <col min="5" max="5" width="12.7109375" customWidth="1"/>
+    <col min="6" max="6" width="14.5703125" customWidth="1"/>
+    <col min="7" max="7" width="17.7109375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7">
@@ -4011,7 +3377,7 @@
         <v>232</v>
       </c>
       <c r="D4" s="2">
-        <v>2.32</v>
+        <v>2.3199999999999998</v>
       </c>
       <c r="E4" s="9" t="s">
         <v>77</v>
@@ -4021,33 +3387,31 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
-  <sheetPr/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:S11"/>
-  <sheetFormatPr defaultColWidth="8.85454545454546" defaultRowHeight="14.5"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="39.7090909090909" customWidth="1"/>
-    <col min="2" max="2" width="10.1363636363636" customWidth="1"/>
-    <col min="3" max="3" width="39.7090909090909" customWidth="1"/>
+    <col min="1" max="1" width="39.7109375" customWidth="1"/>
+    <col min="2" max="2" width="10.140625" customWidth="1"/>
+    <col min="3" max="3" width="39.7109375" customWidth="1"/>
     <col min="4" max="4" width="11" customWidth="1"/>
-    <col min="5" max="5" width="13.2818181818182" customWidth="1"/>
-    <col min="6" max="6" width="8.85454545454546" customWidth="1"/>
-    <col min="7" max="7" width="17.8545454545455" customWidth="1"/>
-    <col min="8" max="8" width="19.5727272727273" customWidth="1"/>
-    <col min="9" max="9" width="23.7090909090909" customWidth="1"/>
-    <col min="10" max="10" width="12.7090909090909" customWidth="1"/>
-    <col min="11" max="11" width="11.8545454545455" customWidth="1"/>
-    <col min="12" max="12" width="17.4272727272727" customWidth="1"/>
-    <col min="13" max="14" width="39.7090909090909" customWidth="1"/>
-    <col min="15" max="15" width="25.7090909090909" customWidth="1"/>
-    <col min="16" max="17" width="16.5727272727273" customWidth="1"/>
-    <col min="18" max="18" width="11.5727272727273" customWidth="1"/>
-    <col min="19" max="19" width="14.8545454545455" customWidth="1"/>
+    <col min="5" max="5" width="13.28515625" customWidth="1"/>
+    <col min="6" max="6" width="8.85546875" customWidth="1"/>
+    <col min="7" max="7" width="17.85546875" customWidth="1"/>
+    <col min="8" max="8" width="19.5703125" customWidth="1"/>
+    <col min="9" max="9" width="23.7109375" customWidth="1"/>
+    <col min="10" max="10" width="12.7109375" customWidth="1"/>
+    <col min="11" max="11" width="11.85546875" customWidth="1"/>
+    <col min="12" max="12" width="17.42578125" customWidth="1"/>
+    <col min="13" max="14" width="39.7109375" customWidth="1"/>
+    <col min="15" max="15" width="25.7109375" customWidth="1"/>
+    <col min="16" max="17" width="16.5703125" customWidth="1"/>
+    <col min="18" max="18" width="11.5703125" customWidth="1"/>
+    <col min="19" max="19" width="14.85546875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:19">
@@ -4661,6 +4025,5 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <headerFooter/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Added MR To MRV Test Scenarios & Updated Fixes
Added MR To MRV Test Scenarios & Updated Fixes
</commit_message>
<xml_diff>
--- a/testdata/ItemDetails.xlsx
+++ b/testdata/ItemDetails.xlsx
@@ -1,10 +1,10 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="4" lowestEdited="5" rupBuild="4505"/>
+  <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="2520" windowWidth="15150" windowHeight="5535" firstSheet="7" activeTab="8"/>
+    <workbookView windowWidth="23040" windowHeight="9120" firstSheet="7" activeTab="13"/>
   </bookViews>
   <sheets>
     <sheet name="PR Details" sheetId="1" r:id="rId1"/>
@@ -20,9 +20,9 @@
     <sheet name="Open Sales" sheetId="11" r:id="rId11"/>
     <sheet name="SI Details" sheetId="12" r:id="rId12"/>
     <sheet name="MRTOMRV Data" sheetId="13" r:id="rId13"/>
+    <sheet name="MRTOMRVWip Data" sheetId="14" r:id="rId14"/>
   </sheets>
-  <calcPr calcId="124519"/>
-  <oleSize ref="N1:T7"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="549" uniqueCount="200">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="556" uniqueCount="202">
   <si>
     <t>ITEM_NAME</t>
   </si>
@@ -641,13 +641,25 @@
   </si>
   <si>
     <t>GWL_ITEM_STOCK_04</t>
+  </si>
+  <si>
+    <t>GWL_ITEM_STOCK_06</t>
+  </si>
+  <si>
+    <t>GWL_ITEM_STOCK_07</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="12">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="xr9">
+  <numFmts count="4">
+    <numFmt numFmtId="176" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
+    <numFmt numFmtId="177" formatCode="_ &quot;₹&quot;* #,##0.00_ ;_ &quot;₹&quot;* \-#,##0.00_ ;_ &quot;₹&quot;* &quot;-&quot;??_ ;_ @_ "/>
+    <numFmt numFmtId="178" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
+    <numFmt numFmtId="179" formatCode="_ &quot;₹&quot;* #,##0_ ;_ &quot;₹&quot;* \-#,##0_ ;_ &quot;₹&quot;* &quot;-&quot;_ ;_ @_ "/>
+  </numFmts>
+  <fonts count="29">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -662,12 +674,6 @@
       <name val="Calibri"/>
       <charset val="134"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="9"/>
-      <color rgb="FF000000"/>
-      <name val="Arial"/>
-      <charset val="134"/>
     </font>
     <font>
       <sz val="9"/>
@@ -720,14 +726,151 @@
       <charset val="134"/>
     </font>
     <font>
+      <u/>
       <sz val="11"/>
-      <color theme="1"/>
+      <color rgb="FF0000FF"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color rgb="FF800080"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="18"/>
+      <color theme="3"/>
       <name val="Calibri"/>
       <charset val="134"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <i/>
+      <sz val="11"/>
+      <color rgb="FF7F7F7F"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="15"/>
+      <color theme="3"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="13"/>
+      <color theme="3"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="3"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF3F3F76"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF3F3F3F"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFA7D00"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFA7D00"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF006100"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF9C0006"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF9C6500"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="0"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="5">
+  <fills count="36">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -736,7 +879,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.59999389629810485"/>
+        <fgColor theme="9" tint="0.599993896298105"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -752,8 +895,194 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFCC"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFCC99"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF2F2F2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFA5A5A5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC6EFCE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC7CE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFEB9C"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="10">
     <border>
       <left/>
       <right/>
@@ -776,16 +1105,258 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFB2B2B2"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFB2B2B2"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFB2B2B2"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFB2B2B2"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color theme="4"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color theme="4" tint="0.499984740745262"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF7F7F7F"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF7F7F7F"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF7F7F7F"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF7F7F7F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF3F3F3F"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF3F3F3F"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF3F3F3F"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF3F3F3F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="double">
+        <color rgb="FF3F3F3F"/>
+      </left>
+      <right style="double">
+        <color rgb="FF3F3F3F"/>
+      </right>
+      <top style="double">
+        <color rgb="FF3F3F3F"/>
+      </top>
+      <bottom style="double">
+        <color rgb="FF3F3F3F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="double">
+        <color rgb="FFFF8001"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color theme="4"/>
+      </top>
+      <bottom style="double">
+        <color theme="4"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
-  <cellStyleXfs count="2">
+  <cellStyleXfs count="50">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0">
+    <xf numFmtId="176" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="177" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="178" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="179" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="2" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="6" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="7" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="7" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="8" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="35" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="31">
+  <cellXfs count="28">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -807,12 +1378,6 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
@@ -826,10 +1391,7 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
@@ -838,7 +1400,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1">
@@ -847,190 +1409,121 @@
     <xf numFmtId="49" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="49" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="49" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="justify" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
-  <cellStyles count="2">
+  <cellStyles count="50">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Normal 2" xfId="1"/>
+    <cellStyle name="Comma" xfId="1" builtinId="3"/>
+    <cellStyle name="Currency" xfId="2" builtinId="4"/>
+    <cellStyle name="Percent" xfId="3" builtinId="5"/>
+    <cellStyle name="Comma [0]" xfId="4" builtinId="6"/>
+    <cellStyle name="Currency [0]" xfId="5" builtinId="7"/>
+    <cellStyle name="Hyperlink" xfId="6" builtinId="8"/>
+    <cellStyle name="Followed Hyperlink" xfId="7" builtinId="9"/>
+    <cellStyle name="Note" xfId="8" builtinId="10"/>
+    <cellStyle name="Warning Text" xfId="9" builtinId="11"/>
+    <cellStyle name="Title" xfId="10" builtinId="15"/>
+    <cellStyle name="CExplanatory Text" xfId="11" builtinId="53"/>
+    <cellStyle name="Heading 1" xfId="12" builtinId="16"/>
+    <cellStyle name="Heading 2" xfId="13" builtinId="17"/>
+    <cellStyle name="Heading 3" xfId="14" builtinId="18"/>
+    <cellStyle name="Heading 4" xfId="15" builtinId="19"/>
+    <cellStyle name="Input" xfId="16" builtinId="20"/>
+    <cellStyle name="Output" xfId="17" builtinId="21"/>
+    <cellStyle name="Calculation" xfId="18" builtinId="22"/>
+    <cellStyle name="Check Cell" xfId="19" builtinId="23"/>
+    <cellStyle name="Linked Cell" xfId="20" builtinId="24"/>
+    <cellStyle name="Total" xfId="21" builtinId="25"/>
+    <cellStyle name="Good" xfId="22" builtinId="26"/>
+    <cellStyle name="Bad" xfId="23" builtinId="27"/>
+    <cellStyle name="Neutral" xfId="24" builtinId="28"/>
+    <cellStyle name="Accent1" xfId="25" builtinId="29"/>
+    <cellStyle name="20% - Accent1" xfId="26" builtinId="30"/>
+    <cellStyle name="40% - Accent1" xfId="27" builtinId="31"/>
+    <cellStyle name="60% - Accent1" xfId="28" builtinId="32"/>
+    <cellStyle name="Accent2" xfId="29" builtinId="33"/>
+    <cellStyle name="20% - Accent2" xfId="30" builtinId="34"/>
+    <cellStyle name="40% - Accent2" xfId="31" builtinId="35"/>
+    <cellStyle name="60% - Accent2" xfId="32" builtinId="36"/>
+    <cellStyle name="Accent3" xfId="33" builtinId="37"/>
+    <cellStyle name="20% - Accent3" xfId="34" builtinId="38"/>
+    <cellStyle name="40% - Accent3" xfId="35" builtinId="39"/>
+    <cellStyle name="60% - Accent3" xfId="36" builtinId="40"/>
+    <cellStyle name="Accent4" xfId="37" builtinId="41"/>
+    <cellStyle name="20% - Accent4" xfId="38" builtinId="42"/>
+    <cellStyle name="40% - Accent4" xfId="39" builtinId="43"/>
+    <cellStyle name="60% - Accent4" xfId="40" builtinId="44"/>
+    <cellStyle name="Accent5" xfId="41" builtinId="45"/>
+    <cellStyle name="20% - Accent5" xfId="42" builtinId="46"/>
+    <cellStyle name="40% - Accent5" xfId="43" builtinId="47"/>
+    <cellStyle name="60% - Accent5" xfId="44" builtinId="48"/>
+    <cellStyle name="Accent6" xfId="45" builtinId="49"/>
+    <cellStyle name="20% - Accent6" xfId="46" builtinId="50"/>
+    <cellStyle name="40% - Accent6" xfId="47" builtinId="51"/>
+    <cellStyle name="60% - Accent6" xfId="48" builtinId="52"/>
+    <cellStyle name="Normal 2" xfId="49"/>
   </cellStyles>
   <dxfs count="17">
     <dxf>
       <fill>
         <patternFill patternType="solid">
-          <fgColor theme="4" tint="0.79995117038483843"/>
-          <bgColor theme="4" tint="0.79995117038483843"/>
-        </patternFill>
-      </fill>
-      <border>
-        <bottom style="thin">
-          <color theme="4" tint="0.39994506668294322"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor theme="4" tint="0.79995117038483843"/>
-          <bgColor theme="4" tint="0.79995117038483843"/>
-        </patternFill>
-      </fill>
-      <border>
-        <bottom style="thin">
-          <color theme="4" tint="0.39994506668294322"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="1"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="1"/>
-      </font>
-      <border>
-        <bottom style="thin">
-          <color theme="4" tint="0.39994506668294322"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <color theme="1"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <color theme="1"/>
-      </font>
-      <border>
-        <top style="thin">
-          <color theme="4"/>
-        </top>
-        <bottom style="thin">
-          <color theme="4"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor theme="4" tint="0.79995117038483843"/>
-          <bgColor theme="4" tint="0.79995117038483843"/>
+          <fgColor theme="4" tint="0.799981688894314"/>
+          <bgColor theme="4" tint="0.799981688894314"/>
         </patternFill>
       </fill>
     </dxf>
     <dxf>
       <fill>
         <patternFill patternType="solid">
-          <fgColor theme="4" tint="0.79995117038483843"/>
-          <bgColor theme="4" tint="0.79995117038483843"/>
+          <fgColor theme="4" tint="0.799981688894314"/>
+          <bgColor theme="4" tint="0.799981688894314"/>
         </patternFill>
       </fill>
     </dxf>
     <dxf>
       <font>
-        <b/>
-        <color theme="1"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor theme="4" tint="0.79995117038483843"/>
-          <bgColor theme="4" tint="0.79995117038483843"/>
-        </patternFill>
-      </fill>
-      <border>
-        <top style="thin">
-          <color theme="4" tint="0.39994506668294322"/>
-        </top>
-        <bottom style="thin">
-          <color theme="4" tint="0.39994506668294322"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <color theme="1"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor theme="4" tint="0.79995117038483843"/>
-          <bgColor theme="4" tint="0.79995117038483843"/>
-        </patternFill>
-      </fill>
-      <border>
-        <bottom style="thin">
-          <color theme="4" tint="0.39994506668294322"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor theme="4" tint="0.79995117038483843"/>
-          <bgColor theme="4" tint="0.79995117038483843"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor theme="4" tint="0.79995117038483843"/>
-          <bgColor theme="4" tint="0.79995117038483843"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
+        <b val="1"/>
         <color theme="1"/>
       </font>
     </dxf>
     <dxf>
       <font>
-        <b/>
+        <b val="1"/>
         <color theme="1"/>
       </font>
     </dxf>
     <dxf>
       <font>
-        <b/>
+        <b val="1"/>
         <color theme="1"/>
       </font>
       <border>
@@ -1041,7 +1534,7 @@
     </dxf>
     <dxf>
       <font>
-        <b/>
+        <b val="1"/>
         <color theme="0"/>
       </font>
       <fill>
@@ -1069,32 +1562,149 @@
           <color theme="4"/>
         </bottom>
         <horizontal style="thin">
-          <color theme="4" tint="0.39994506668294322"/>
+          <color theme="4" tint="0.399975585192419"/>
         </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor theme="4" tint="0.799981688894314"/>
+          <bgColor theme="4" tint="0.799981688894314"/>
+        </patternFill>
+      </fill>
+      <border>
+        <bottom style="thin">
+          <color theme="4" tint="0.399975585192419"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor theme="4" tint="0.799981688894314"/>
+          <bgColor theme="4" tint="0.799981688894314"/>
+        </patternFill>
+      </fill>
+      <border>
+        <bottom style="thin">
+          <color theme="4" tint="0.399975585192419"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="1"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="1"/>
+      </font>
+      <border>
+        <bottom style="thin">
+          <color theme="4" tint="0.399975585192419"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <color theme="1"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <color theme="1"/>
+      </font>
+      <border>
+        <top style="thin">
+          <color theme="4"/>
+        </top>
+        <bottom style="thin">
+          <color theme="4"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor theme="4" tint="0.799981688894314"/>
+          <bgColor theme="4" tint="0.799981688894314"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor theme="4" tint="0.799981688894314"/>
+          <bgColor theme="4" tint="0.799981688894314"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <color theme="1"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor theme="4" tint="0.799981688894314"/>
+          <bgColor theme="4" tint="0.799981688894314"/>
+        </patternFill>
+      </fill>
+      <border>
+        <top style="thin">
+          <color theme="4" tint="0.399975585192419"/>
+        </top>
+        <bottom style="thin">
+          <color theme="4" tint="0.399975585192419"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <color theme="1"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor theme="4" tint="0.799981688894314"/>
+          <bgColor theme="4" tint="0.799981688894314"/>
+        </patternFill>
+      </fill>
+      <border>
+        <bottom style="thin">
+          <color theme="4" tint="0.399975585192419"/>
+        </bottom>
       </border>
     </dxf>
   </dxfs>
   <tableStyles count="2" defaultTableStyle="TableStylePreset3_Accent1" defaultPivotStyle="PivotStylePreset2_Accent1">
-    <tableStyle name="TableStylePreset3_Accent1" pivot="0" count="7">
-      <tableStyleElement type="wholeTable" dxfId="16"/>
-      <tableStyleElement type="headerRow" dxfId="15"/>
-      <tableStyleElement type="totalRow" dxfId="14"/>
-      <tableStyleElement type="firstColumn" dxfId="13"/>
-      <tableStyleElement type="lastColumn" dxfId="12"/>
-      <tableStyleElement type="firstRowStripe" dxfId="11"/>
-      <tableStyleElement type="firstColumnStripe" dxfId="10"/>
+    <tableStyle name="TableStylePreset3_Accent1" pivot="0" count="7" xr9:uid="{59DB682C-5494-4EDE-A608-00C9E5F0F923}">
+      <tableStyleElement type="wholeTable" dxfId="6"/>
+      <tableStyleElement type="headerRow" dxfId="5"/>
+      <tableStyleElement type="totalRow" dxfId="4"/>
+      <tableStyleElement type="firstColumn" dxfId="3"/>
+      <tableStyleElement type="lastColumn" dxfId="2"/>
+      <tableStyleElement type="firstRowStripe" dxfId="1"/>
+      <tableStyleElement type="firstColumnStripe" dxfId="0"/>
     </tableStyle>
-    <tableStyle name="PivotStylePreset2_Accent1" table="0" count="10">
-      <tableStyleElement type="headerRow" dxfId="9"/>
-      <tableStyleElement type="totalRow" dxfId="8"/>
-      <tableStyleElement type="firstRowStripe" dxfId="7"/>
-      <tableStyleElement type="firstColumnStripe" dxfId="6"/>
-      <tableStyleElement type="firstSubtotalRow" dxfId="5"/>
-      <tableStyleElement type="secondSubtotalRow" dxfId="4"/>
-      <tableStyleElement type="firstRowSubheading" dxfId="3"/>
-      <tableStyleElement type="secondRowSubheading" dxfId="2"/>
-      <tableStyleElement type="pageFieldLabels" dxfId="1"/>
-      <tableStyleElement type="pageFieldValues" dxfId="0"/>
+    <tableStyle name="PivotStylePreset2_Accent1" table="0" count="10" xr9:uid="{267968C8-6FFD-4C36-ACC1-9EA1FD1885CA}">
+      <tableStyleElement type="headerRow" dxfId="16"/>
+      <tableStyleElement type="totalRow" dxfId="15"/>
+      <tableStyleElement type="firstRowStripe" dxfId="14"/>
+      <tableStyleElement type="firstColumnStripe" dxfId="13"/>
+      <tableStyleElement type="firstSubtotalRow" dxfId="12"/>
+      <tableStyleElement type="secondSubtotalRow" dxfId="11"/>
+      <tableStyleElement type="firstRowSubheading" dxfId="10"/>
+      <tableStyleElement type="secondRowSubheading" dxfId="9"/>
+      <tableStyleElement type="pageFieldLabels" dxfId="8"/>
+      <tableStyleElement type="pageFieldValues" dxfId="7"/>
     </tableStyle>
   </tableStyles>
   <extLst>
@@ -1357,418 +1967,420 @@
     </a:fmtScheme>
   </a:themeElements>
   <a:objectDefaults/>
-  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
   <dimension ref="A1:J20"/>
-  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="8.71296296296296" defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="20.7109375" customWidth="1"/>
-    <col min="2" max="3" width="12.7109375" customWidth="1"/>
-    <col min="4" max="4" width="14.7109375" customWidth="1"/>
-    <col min="5" max="5" width="9.85546875" customWidth="1"/>
-    <col min="6" max="6" width="14.140625" customWidth="1"/>
-    <col min="7" max="7" width="14.85546875" customWidth="1"/>
-    <col min="8" max="8" width="22.28515625" customWidth="1"/>
-    <col min="9" max="9" width="14.42578125" customWidth="1"/>
+    <col min="1" max="1" width="20.712962962963" customWidth="1"/>
+    <col min="2" max="3" width="12.712962962963" customWidth="1"/>
+    <col min="4" max="4" width="14.712962962963" customWidth="1"/>
+    <col min="5" max="5" width="9.85185185185185" customWidth="1"/>
+    <col min="6" max="6" width="14.1388888888889" customWidth="1"/>
+    <col min="7" max="7" width="14.8518518518519" customWidth="1"/>
+    <col min="8" max="8" width="22.287037037037" customWidth="1"/>
+    <col min="9" max="9" width="14.4259259259259" customWidth="1"/>
     <col min="10" max="10" width="13" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:10">
-      <c r="A1" s="27" t="s">
+      <c r="A1" s="24" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="27" t="s">
+      <c r="B1" s="24" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="27" t="s">
+      <c r="C1" s="24" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="27" t="s">
+      <c r="D1" s="24" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="27" t="s">
+      <c r="E1" s="24" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="27" t="s">
+      <c r="F1" s="24" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="27" t="s">
+      <c r="G1" s="24" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="27" t="s">
+      <c r="H1" s="24" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="27" t="s">
+      <c r="I1" s="24" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="27" t="s">
+      <c r="J1" s="24" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="2" spans="1:10" s="26" customFormat="1" ht="22.5">
-      <c r="A2" s="28" t="s">
+    <row r="2" s="23" customFormat="1" ht="20.4" spans="1:10">
+      <c r="A2" s="25" t="s">
         <v>10</v>
       </c>
-      <c r="B2" s="29" t="s">
+      <c r="B2" s="26" t="s">
         <v>11</v>
       </c>
-      <c r="C2" s="29" t="s">
+      <c r="C2" s="26" t="s">
         <v>12</v>
       </c>
-      <c r="D2" s="28" t="s">
+      <c r="D2" s="25" t="s">
         <v>13</v>
       </c>
-      <c r="E2" s="28">
+      <c r="E2" s="25">
         <v>1</v>
       </c>
-      <c r="F2" s="28" t="s">
+      <c r="F2" s="25" t="s">
         <v>14</v>
       </c>
-      <c r="G2" s="28">
+      <c r="G2" s="25">
         <v>1010301033</v>
       </c>
-      <c r="H2" s="28" t="s">
+      <c r="H2" s="25" t="s">
         <v>15</v>
       </c>
-      <c r="I2" s="28" t="s">
+      <c r="I2" s="25" t="s">
         <v>16</v>
       </c>
-      <c r="J2" s="28" t="s">
+      <c r="J2" s="25" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="3" spans="1:10" ht="15" customHeight="1">
-      <c r="A3" s="28" t="s">
+    <row r="3" ht="15" customHeight="1" spans="1:10">
+      <c r="A3" s="25" t="s">
         <v>18</v>
       </c>
-      <c r="B3" s="29" t="s">
+      <c r="B3" s="26" t="s">
         <v>11</v>
       </c>
-      <c r="C3" s="29" t="s">
+      <c r="C3" s="26" t="s">
         <v>12</v>
       </c>
-      <c r="D3" s="28" t="s">
+      <c r="D3" s="25" t="s">
         <v>19</v>
       </c>
-      <c r="E3" s="28">
+      <c r="E3" s="25">
         <v>6</v>
       </c>
-      <c r="F3" s="29" t="s">
+      <c r="F3" s="26" t="s">
         <v>20</v>
       </c>
-      <c r="G3" s="28">
+      <c r="G3" s="25">
         <v>1010301033</v>
       </c>
-      <c r="H3" s="28" t="s">
+      <c r="H3" s="25" t="s">
         <v>15</v>
       </c>
-      <c r="I3" s="28" t="s">
+      <c r="I3" s="25" t="s">
         <v>16</v>
       </c>
-      <c r="J3" s="28" t="s">
+      <c r="J3" s="25" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="4" spans="1:10" ht="22.5">
-      <c r="A4" s="28" t="s">
+    <row r="4" spans="1:10">
+      <c r="A4" s="25" t="s">
         <v>21</v>
       </c>
-      <c r="B4" s="29" t="s">
+      <c r="B4" s="26" t="s">
         <v>22</v>
       </c>
-      <c r="C4" s="29" t="s">
+      <c r="C4" s="26" t="s">
         <v>22</v>
       </c>
-      <c r="D4" s="28" t="s">
+      <c r="D4" s="25" t="s">
         <v>23</v>
       </c>
-      <c r="E4" s="28">
+      <c r="E4" s="25">
         <v>1</v>
       </c>
-      <c r="F4" s="29" t="s">
+      <c r="F4" s="26" t="s">
         <v>14</v>
       </c>
-      <c r="G4" s="28">
+      <c r="G4" s="25">
         <v>5010100004</v>
       </c>
-      <c r="H4" s="28" t="s">
+      <c r="H4" s="25" t="s">
         <v>24</v>
       </c>
-      <c r="I4" s="28" t="s">
+      <c r="I4" s="25" t="s">
         <v>16</v>
       </c>
-      <c r="J4" s="28" t="s">
+      <c r="J4" s="25" t="s">
         <v>17</v>
       </c>
     </row>
     <row r="5" spans="1:10">
-      <c r="A5" s="30"/>
-      <c r="B5" s="30"/>
-      <c r="C5" s="30"/>
-      <c r="D5" s="30"/>
-      <c r="E5" s="30"/>
-      <c r="F5" s="30"/>
-      <c r="G5" s="30"/>
-      <c r="H5" s="30"/>
-      <c r="I5" s="30"/>
-      <c r="J5" s="30"/>
+      <c r="A5" s="27"/>
+      <c r="B5" s="27"/>
+      <c r="C5" s="27"/>
+      <c r="D5" s="27"/>
+      <c r="E5" s="27"/>
+      <c r="F5" s="27"/>
+      <c r="G5" s="27"/>
+      <c r="H5" s="27"/>
+      <c r="I5" s="27"/>
+      <c r="J5" s="27"/>
     </row>
     <row r="6" spans="1:10">
-      <c r="A6" s="30"/>
-      <c r="B6" s="30"/>
-      <c r="C6" s="30"/>
-      <c r="D6" s="30"/>
-      <c r="E6" s="30"/>
-      <c r="F6" s="30"/>
-      <c r="G6" s="30"/>
-      <c r="H6" s="30"/>
-      <c r="I6" s="30"/>
-      <c r="J6" s="30"/>
+      <c r="A6" s="27"/>
+      <c r="B6" s="27"/>
+      <c r="C6" s="27"/>
+      <c r="D6" s="27"/>
+      <c r="E6" s="27"/>
+      <c r="F6" s="27"/>
+      <c r="G6" s="27"/>
+      <c r="H6" s="27"/>
+      <c r="I6" s="27"/>
+      <c r="J6" s="27"/>
     </row>
     <row r="7" spans="1:10">
-      <c r="A7" s="30"/>
-      <c r="B7" s="30"/>
-      <c r="C7" s="30"/>
-      <c r="D7" s="30"/>
-      <c r="E7" s="30"/>
-      <c r="F7" s="30"/>
-      <c r="G7" s="30"/>
-      <c r="H7" s="30"/>
-      <c r="I7" s="30"/>
-      <c r="J7" s="30"/>
+      <c r="A7" s="27"/>
+      <c r="B7" s="27"/>
+      <c r="C7" s="27"/>
+      <c r="D7" s="27"/>
+      <c r="E7" s="27"/>
+      <c r="F7" s="27"/>
+      <c r="G7" s="27"/>
+      <c r="H7" s="27"/>
+      <c r="I7" s="27"/>
+      <c r="J7" s="27"/>
     </row>
     <row r="8" spans="1:10">
-      <c r="A8" s="30"/>
-      <c r="B8" s="30"/>
-      <c r="C8" s="30"/>
-      <c r="D8" s="30"/>
-      <c r="E8" s="30"/>
-      <c r="F8" s="30"/>
-      <c r="G8" s="30"/>
-      <c r="H8" s="30"/>
-      <c r="I8" s="30"/>
-      <c r="J8" s="30"/>
+      <c r="A8" s="27"/>
+      <c r="B8" s="27"/>
+      <c r="C8" s="27"/>
+      <c r="D8" s="27"/>
+      <c r="E8" s="27"/>
+      <c r="F8" s="27"/>
+      <c r="G8" s="27"/>
+      <c r="H8" s="27"/>
+      <c r="I8" s="27"/>
+      <c r="J8" s="27"/>
     </row>
     <row r="9" spans="1:10">
-      <c r="A9" s="30"/>
-      <c r="B9" s="30"/>
-      <c r="C9" s="30"/>
-      <c r="D9" s="30"/>
-      <c r="E9" s="30"/>
-      <c r="F9" s="30"/>
-      <c r="G9" s="30"/>
-      <c r="H9" s="30"/>
-      <c r="I9" s="30"/>
-      <c r="J9" s="30"/>
+      <c r="A9" s="27"/>
+      <c r="B9" s="27"/>
+      <c r="C9" s="27"/>
+      <c r="D9" s="27"/>
+      <c r="E9" s="27"/>
+      <c r="F9" s="27"/>
+      <c r="G9" s="27"/>
+      <c r="H9" s="27"/>
+      <c r="I9" s="27"/>
+      <c r="J9" s="27"/>
     </row>
     <row r="10" spans="1:10">
-      <c r="A10" s="30"/>
-      <c r="B10" s="30"/>
-      <c r="C10" s="30"/>
-      <c r="D10" s="30"/>
-      <c r="E10" s="30"/>
-      <c r="F10" s="30"/>
-      <c r="G10" s="30"/>
-      <c r="H10" s="30"/>
-      <c r="I10" s="30"/>
-      <c r="J10" s="30"/>
+      <c r="A10" s="27"/>
+      <c r="B10" s="27"/>
+      <c r="C10" s="27"/>
+      <c r="D10" s="27"/>
+      <c r="E10" s="27"/>
+      <c r="F10" s="27"/>
+      <c r="G10" s="27"/>
+      <c r="H10" s="27"/>
+      <c r="I10" s="27"/>
+      <c r="J10" s="27"/>
     </row>
     <row r="11" spans="1:10">
-      <c r="A11" s="30"/>
-      <c r="B11" s="30"/>
-      <c r="C11" s="30"/>
-      <c r="D11" s="30"/>
-      <c r="E11" s="30"/>
-      <c r="F11" s="30"/>
-      <c r="G11" s="30"/>
-      <c r="H11" s="30"/>
-      <c r="I11" s="30"/>
-      <c r="J11" s="30"/>
+      <c r="A11" s="27"/>
+      <c r="B11" s="27"/>
+      <c r="C11" s="27"/>
+      <c r="D11" s="27"/>
+      <c r="E11" s="27"/>
+      <c r="F11" s="27"/>
+      <c r="G11" s="27"/>
+      <c r="H11" s="27"/>
+      <c r="I11" s="27"/>
+      <c r="J11" s="27"/>
     </row>
     <row r="12" spans="1:10">
-      <c r="A12" s="30"/>
-      <c r="B12" s="30"/>
-      <c r="C12" s="30"/>
-      <c r="D12" s="30"/>
-      <c r="E12" s="30"/>
-      <c r="F12" s="30"/>
-      <c r="G12" s="30"/>
-      <c r="H12" s="30"/>
-      <c r="I12" s="30"/>
-      <c r="J12" s="30"/>
+      <c r="A12" s="27"/>
+      <c r="B12" s="27"/>
+      <c r="C12" s="27"/>
+      <c r="D12" s="27"/>
+      <c r="E12" s="27"/>
+      <c r="F12" s="27"/>
+      <c r="G12" s="27"/>
+      <c r="H12" s="27"/>
+      <c r="I12" s="27"/>
+      <c r="J12" s="27"/>
     </row>
     <row r="13" spans="1:10">
-      <c r="A13" s="30"/>
-      <c r="B13" s="30"/>
-      <c r="C13" s="30"/>
-      <c r="D13" s="30"/>
-      <c r="E13" s="30"/>
-      <c r="F13" s="30"/>
-      <c r="G13" s="30"/>
-      <c r="H13" s="30"/>
-      <c r="I13" s="30"/>
-      <c r="J13" s="30"/>
+      <c r="A13" s="27"/>
+      <c r="B13" s="27"/>
+      <c r="C13" s="27"/>
+      <c r="D13" s="27"/>
+      <c r="E13" s="27"/>
+      <c r="F13" s="27"/>
+      <c r="G13" s="27"/>
+      <c r="H13" s="27"/>
+      <c r="I13" s="27"/>
+      <c r="J13" s="27"/>
     </row>
     <row r="14" spans="1:10">
-      <c r="A14" s="30"/>
-      <c r="B14" s="30"/>
-      <c r="C14" s="30"/>
-      <c r="D14" s="30"/>
-      <c r="E14" s="30"/>
-      <c r="F14" s="30"/>
-      <c r="G14" s="30"/>
-      <c r="H14" s="30"/>
-      <c r="I14" s="30"/>
-      <c r="J14" s="30"/>
+      <c r="A14" s="27"/>
+      <c r="B14" s="27"/>
+      <c r="C14" s="27"/>
+      <c r="D14" s="27"/>
+      <c r="E14" s="27"/>
+      <c r="F14" s="27"/>
+      <c r="G14" s="27"/>
+      <c r="H14" s="27"/>
+      <c r="I14" s="27"/>
+      <c r="J14" s="27"/>
     </row>
     <row r="15" spans="1:10">
-      <c r="A15" s="30"/>
-      <c r="B15" s="30"/>
-      <c r="C15" s="30"/>
-      <c r="D15" s="30"/>
-      <c r="E15" s="30"/>
-      <c r="F15" s="30"/>
-      <c r="G15" s="30"/>
-      <c r="H15" s="30"/>
-      <c r="I15" s="30"/>
-      <c r="J15" s="30"/>
+      <c r="A15" s="27"/>
+      <c r="B15" s="27"/>
+      <c r="C15" s="27"/>
+      <c r="D15" s="27"/>
+      <c r="E15" s="27"/>
+      <c r="F15" s="27"/>
+      <c r="G15" s="27"/>
+      <c r="H15" s="27"/>
+      <c r="I15" s="27"/>
+      <c r="J15" s="27"/>
     </row>
     <row r="16" spans="1:10">
-      <c r="A16" s="30"/>
-      <c r="B16" s="30"/>
-      <c r="C16" s="30"/>
-      <c r="D16" s="30"/>
-      <c r="E16" s="30"/>
-      <c r="F16" s="30"/>
-      <c r="G16" s="30"/>
-      <c r="H16" s="30"/>
-      <c r="I16" s="30"/>
-      <c r="J16" s="30"/>
+      <c r="A16" s="27"/>
+      <c r="B16" s="27"/>
+      <c r="C16" s="27"/>
+      <c r="D16" s="27"/>
+      <c r="E16" s="27"/>
+      <c r="F16" s="27"/>
+      <c r="G16" s="27"/>
+      <c r="H16" s="27"/>
+      <c r="I16" s="27"/>
+      <c r="J16" s="27"/>
     </row>
     <row r="17" spans="1:10">
-      <c r="A17" s="30"/>
-      <c r="B17" s="30"/>
-      <c r="C17" s="30"/>
-      <c r="D17" s="30"/>
-      <c r="E17" s="30"/>
-      <c r="F17" s="30"/>
-      <c r="G17" s="30"/>
-      <c r="H17" s="30"/>
-      <c r="I17" s="30"/>
-      <c r="J17" s="30"/>
+      <c r="A17" s="27"/>
+      <c r="B17" s="27"/>
+      <c r="C17" s="27"/>
+      <c r="D17" s="27"/>
+      <c r="E17" s="27"/>
+      <c r="F17" s="27"/>
+      <c r="G17" s="27"/>
+      <c r="H17" s="27"/>
+      <c r="I17" s="27"/>
+      <c r="J17" s="27"/>
     </row>
     <row r="18" spans="1:10">
-      <c r="A18" s="30"/>
-      <c r="B18" s="30"/>
-      <c r="C18" s="30"/>
-      <c r="D18" s="30"/>
-      <c r="E18" s="30"/>
-      <c r="F18" s="30"/>
-      <c r="G18" s="30"/>
-      <c r="H18" s="30"/>
-      <c r="I18" s="30"/>
-      <c r="J18" s="30"/>
+      <c r="A18" s="27"/>
+      <c r="B18" s="27"/>
+      <c r="C18" s="27"/>
+      <c r="D18" s="27"/>
+      <c r="E18" s="27"/>
+      <c r="F18" s="27"/>
+      <c r="G18" s="27"/>
+      <c r="H18" s="27"/>
+      <c r="I18" s="27"/>
+      <c r="J18" s="27"/>
     </row>
     <row r="19" spans="1:10">
-      <c r="A19" s="30"/>
-      <c r="B19" s="30"/>
-      <c r="C19" s="30"/>
-      <c r="D19" s="30"/>
-      <c r="E19" s="30"/>
-      <c r="F19" s="30"/>
-      <c r="G19" s="30"/>
-      <c r="H19" s="30"/>
-      <c r="I19" s="30"/>
-      <c r="J19" s="30"/>
+      <c r="A19" s="27"/>
+      <c r="B19" s="27"/>
+      <c r="C19" s="27"/>
+      <c r="D19" s="27"/>
+      <c r="E19" s="27"/>
+      <c r="F19" s="27"/>
+      <c r="G19" s="27"/>
+      <c r="H19" s="27"/>
+      <c r="I19" s="27"/>
+      <c r="J19" s="27"/>
     </row>
     <row r="20" spans="1:10">
-      <c r="A20" s="30"/>
-      <c r="B20" s="30"/>
-      <c r="C20" s="30"/>
-      <c r="D20" s="30"/>
-      <c r="E20" s="30"/>
-      <c r="F20" s="30"/>
-      <c r="G20" s="30"/>
-      <c r="H20" s="30"/>
-      <c r="I20" s="30"/>
-      <c r="J20" s="30"/>
+      <c r="A20" s="27"/>
+      <c r="B20" s="27"/>
+      <c r="C20" s="27"/>
+      <c r="D20" s="27"/>
+      <c r="E20" s="27"/>
+      <c r="F20" s="27"/>
+      <c r="G20" s="27"/>
+      <c r="H20" s="27"/>
+      <c r="I20" s="27"/>
+      <c r="J20" s="27"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
   <dimension ref="A1:K3"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="8.85185185185185" defaultRowHeight="14.4" outlineLevelRow="2"/>
   <cols>
     <col min="1" max="1" width="9" customWidth="1"/>
-    <col min="2" max="2" width="25.7109375" customWidth="1"/>
-    <col min="3" max="3" width="12.42578125" customWidth="1"/>
-    <col min="4" max="4" width="16.28515625" customWidth="1"/>
-    <col min="5" max="5" width="20.28515625" customWidth="1"/>
-    <col min="6" max="6" width="25.7109375" customWidth="1"/>
-    <col min="7" max="7" width="12.28515625" customWidth="1"/>
-    <col min="8" max="8" width="14.5703125" customWidth="1"/>
-    <col min="9" max="9" width="28.5703125" customWidth="1"/>
+    <col min="2" max="2" width="25.712962962963" customWidth="1"/>
+    <col min="3" max="3" width="12.4259259259259" customWidth="1"/>
+    <col min="4" max="4" width="16.287037037037" customWidth="1"/>
+    <col min="5" max="5" width="20.287037037037" customWidth="1"/>
+    <col min="6" max="6" width="25.712962962963" customWidth="1"/>
+    <col min="7" max="7" width="12.287037037037" customWidth="1"/>
+    <col min="8" max="8" width="14.5740740740741" customWidth="1"/>
+    <col min="9" max="9" width="28.5740740740741" customWidth="1"/>
     <col min="10" max="10" width="23" customWidth="1"/>
-    <col min="11" max="11" width="14.7109375" customWidth="1"/>
+    <col min="11" max="11" width="14.712962962963" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:11">
-      <c r="A1" s="9" t="s">
+      <c r="A1" s="7" t="s">
         <v>127</v>
       </c>
-      <c r="B1" s="9" t="s">
+      <c r="B1" s="7" t="s">
         <v>128</v>
       </c>
-      <c r="C1" s="9" t="s">
+      <c r="C1" s="7" t="s">
         <v>129</v>
       </c>
-      <c r="D1" s="9" t="s">
+      <c r="D1" s="7" t="s">
         <v>130</v>
       </c>
-      <c r="E1" s="9" t="s">
+      <c r="E1" s="7" t="s">
         <v>131</v>
       </c>
-      <c r="F1" s="12" t="s">
+      <c r="F1" s="10" t="s">
         <v>132</v>
       </c>
-      <c r="G1" s="12" t="s">
+      <c r="G1" s="10" t="s">
         <v>133</v>
       </c>
-      <c r="H1" s="12" t="s">
+      <c r="H1" s="10" t="s">
         <v>134</v>
       </c>
-      <c r="I1" s="12" t="s">
+      <c r="I1" s="10" t="s">
         <v>135</v>
       </c>
-      <c r="J1" s="12" t="s">
+      <c r="J1" s="10" t="s">
         <v>136</v>
       </c>
-      <c r="K1" s="12" t="s">
+      <c r="K1" s="10" t="s">
         <v>137</v>
       </c>
     </row>
     <row r="2" spans="1:11">
-      <c r="A2" s="9" t="s">
+      <c r="A2" s="7" t="s">
         <v>138</v>
       </c>
-      <c r="B2" s="9" t="s">
+      <c r="B2" s="7" t="s">
         <v>139</v>
       </c>
-      <c r="C2" s="9" t="s">
+      <c r="C2" s="7" t="s">
         <v>140</v>
       </c>
-      <c r="D2" s="9" t="s">
+      <c r="D2" s="7" t="s">
         <v>141</v>
       </c>
-      <c r="E2" s="9" t="s">
+      <c r="E2" s="7" t="s">
         <v>142</v>
       </c>
       <c r="F2" s="2" t="s">
@@ -1791,13 +2403,13 @@
       </c>
     </row>
     <row r="3" spans="1:11">
-      <c r="A3" s="13" t="s">
+      <c r="A3" s="11" t="s">
         <v>148</v>
       </c>
       <c r="B3" s="2" t="s">
         <v>149</v>
       </c>
-      <c r="C3" s="9" t="s">
+      <c r="C3" s="7" t="s">
         <v>140</v>
       </c>
       <c r="D3" s="2" t="s">
@@ -1827,23 +2439,25 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
   <dimension ref="A1:E4"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="8.85185185185185" defaultRowHeight="14.4" outlineLevelRow="3" outlineLevelCol="4"/>
   <cols>
-    <col min="1" max="1" width="13.5703125" customWidth="1"/>
+    <col min="1" max="1" width="13.5740740740741" customWidth="1"/>
     <col min="2" max="2" width="6" customWidth="1"/>
-    <col min="3" max="3" width="14.42578125" customWidth="1"/>
-    <col min="4" max="4" width="18.140625" customWidth="1"/>
-    <col min="5" max="5" width="19.5703125" customWidth="1"/>
+    <col min="3" max="3" width="14.4259259259259" customWidth="1"/>
+    <col min="4" max="4" width="18.1388888888889" customWidth="1"/>
+    <col min="5" max="5" width="19.5740740740741" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5">
-      <c r="A1" s="9" t="s">
+      <c r="A1" s="7" t="s">
         <v>153</v>
       </c>
       <c r="B1" s="2" t="s">
@@ -1859,20 +2473,20 @@
         <v>157</v>
       </c>
     </row>
-    <row r="2" spans="1:5" ht="30">
-      <c r="A2" s="9" t="s">
+    <row r="2" spans="1:5">
+      <c r="A2" s="7" t="s">
         <v>158</v>
       </c>
-      <c r="B2" s="9" t="s">
+      <c r="B2" s="7" t="s">
         <v>159</v>
       </c>
-      <c r="C2" s="10" t="s">
+      <c r="C2" s="8" t="s">
         <v>138</v>
       </c>
-      <c r="D2" s="11" t="s">
+      <c r="D2" s="9" t="s">
         <v>139</v>
       </c>
-      <c r="E2" s="9" t="s">
+      <c r="E2" s="7" t="s">
         <v>160</v>
       </c>
     </row>
@@ -1912,21 +2526,23 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
   <dimension ref="A1:G11"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="8.85185185185185" defaultRowHeight="14.4" outlineLevelCol="6"/>
   <cols>
-    <col min="1" max="1" width="25.7109375" customWidth="1"/>
-    <col min="2" max="2" width="8.85546875" customWidth="1"/>
-    <col min="3" max="3" width="12.28515625" customWidth="1"/>
-    <col min="4" max="4" width="7.140625" customWidth="1"/>
-    <col min="5" max="5" width="5.28515625" customWidth="1"/>
-    <col min="6" max="6" width="17.42578125" customWidth="1"/>
-    <col min="7" max="7" width="12.42578125" customWidth="1"/>
+    <col min="1" max="1" width="25.712962962963" customWidth="1"/>
+    <col min="2" max="2" width="8.85185185185185" customWidth="1"/>
+    <col min="3" max="3" width="12.287037037037" customWidth="1"/>
+    <col min="4" max="4" width="7.13888888888889" customWidth="1"/>
+    <col min="5" max="5" width="5.28703703703704" customWidth="1"/>
+    <col min="6" max="6" width="17.4259259259259" customWidth="1"/>
+    <col min="7" max="7" width="12.4259259259259" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7">
@@ -2114,87 +2730,89 @@
       </c>
     </row>
     <row r="9" spans="1:7">
-      <c r="A9" s="7" t="s">
+      <c r="A9" s="5" t="s">
         <v>189</v>
       </c>
-      <c r="B9" s="7" t="s">
+      <c r="B9" s="5" t="s">
         <v>179</v>
       </c>
-      <c r="C9" s="8" t="s">
+      <c r="C9" s="6" t="s">
         <v>190</v>
       </c>
-      <c r="D9" s="8" t="s">
+      <c r="D9" s="6" t="s">
         <v>158</v>
       </c>
-      <c r="E9" s="8" t="s">
+      <c r="E9" s="6" t="s">
         <v>159</v>
       </c>
-      <c r="F9" s="7" t="s">
+      <c r="F9" s="5" t="s">
         <v>181</v>
       </c>
-      <c r="G9" s="7" t="s">
+      <c r="G9" s="5" t="s">
         <v>182</v>
       </c>
     </row>
     <row r="10" spans="1:7">
-      <c r="A10" s="7" t="s">
+      <c r="A10" s="5" t="s">
         <v>191</v>
       </c>
-      <c r="B10" s="7" t="s">
+      <c r="B10" s="5" t="s">
         <v>179</v>
       </c>
-      <c r="C10" s="8" t="s">
+      <c r="C10" s="6" t="s">
         <v>192</v>
       </c>
-      <c r="D10" s="8" t="s">
+      <c r="D10" s="6" t="s">
         <v>158</v>
       </c>
-      <c r="E10" s="8" t="s">
+      <c r="E10" s="6" t="s">
         <v>159</v>
       </c>
-      <c r="F10" s="7" t="s">
+      <c r="F10" s="5" t="s">
         <v>181</v>
       </c>
-      <c r="G10" s="7" t="s">
+      <c r="G10" s="5" t="s">
         <v>182</v>
       </c>
     </row>
     <row r="11" spans="1:7">
-      <c r="A11" s="7" t="s">
+      <c r="A11" s="5" t="s">
         <v>193</v>
       </c>
-      <c r="B11" s="7" t="s">
+      <c r="B11" s="5" t="s">
         <v>179</v>
       </c>
-      <c r="C11" s="8" t="s">
+      <c r="C11" s="6" t="s">
         <v>194</v>
       </c>
-      <c r="D11" s="8" t="s">
+      <c r="D11" s="6" t="s">
         <v>158</v>
       </c>
-      <c r="E11" s="8" t="s">
+      <c r="E11" s="6" t="s">
         <v>159</v>
       </c>
-      <c r="F11" s="7" t="s">
+      <c r="F11" s="5" t="s">
         <v>181</v>
       </c>
-      <c r="G11" s="7" t="s">
+      <c r="G11" s="5" t="s">
         <v>182</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
   <dimension ref="A1:C3"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="8.85185185185185" defaultRowHeight="14.4" outlineLevelRow="2" outlineLevelCol="2"/>
   <cols>
-    <col min="1" max="1" width="25.5703125" customWidth="1"/>
-    <col min="2" max="2" width="15.140625" customWidth="1"/>
-    <col min="3" max="3" width="16.42578125" customWidth="1"/>
+    <col min="1" max="1" width="25.5740740740741" customWidth="1"/>
+    <col min="2" max="2" width="15.1388888888889" customWidth="1"/>
+    <col min="3" max="3" width="16.4259259259259" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3">
@@ -2232,259 +2850,311 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <headerFooter/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
+  <dimension ref="A1:C3"/>
+  <sheetFormatPr defaultColWidth="8.88888888888889" defaultRowHeight="14.4" outlineLevelRow="2" outlineLevelCol="2"/>
+  <cols>
+    <col min="1" max="1" width="21.4444444444444" customWidth="1"/>
+    <col min="2" max="2" width="11.5555555555556" customWidth="1"/>
+    <col min="3" max="3" width="9" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3">
+      <c r="A1" s="1" t="s">
+        <v>195</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>196</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3">
+      <c r="A2" s="2" t="s">
+        <v>200</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>198</v>
+      </c>
+      <c r="C2" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3">
+      <c r="A3" s="2" t="s">
+        <v>201</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>198</v>
+      </c>
+      <c r="C3" s="2">
+        <v>2</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
   <dimension ref="A1:T10"/>
-  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="8.71296296296296" defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="30" customWidth="1"/>
-    <col min="2" max="2" width="36.42578125" customWidth="1"/>
+    <col min="2" max="2" width="36.4259259259259" customWidth="1"/>
     <col min="3" max="3" width="6" customWidth="1"/>
-    <col min="4" max="4" width="13.7109375" customWidth="1"/>
-    <col min="5" max="5" width="5.28515625" customWidth="1"/>
-    <col min="6" max="6" width="17.28515625" customWidth="1"/>
-    <col min="7" max="7" width="30.28515625" customWidth="1"/>
-    <col min="8" max="8" width="26.85546875" customWidth="1"/>
-    <col min="9" max="9" width="17.28515625" customWidth="1"/>
-    <col min="10" max="10" width="13.28515625" customWidth="1"/>
-    <col min="11" max="11" width="22.7109375" customWidth="1"/>
-    <col min="12" max="12" width="12.7109375" customWidth="1"/>
-    <col min="13" max="13" width="29.5703125" customWidth="1"/>
-    <col min="14" max="14" width="18.28515625" customWidth="1"/>
-    <col min="15" max="15" width="16.28515625" customWidth="1"/>
-    <col min="16" max="16" width="15.5703125" customWidth="1"/>
-    <col min="17" max="17" width="17.7109375" customWidth="1"/>
-    <col min="18" max="18" width="24.140625" customWidth="1"/>
-    <col min="19" max="19" width="13.42578125" customWidth="1"/>
-    <col min="20" max="20" width="13.5703125" customWidth="1"/>
+    <col min="4" max="4" width="13.712962962963" customWidth="1"/>
+    <col min="5" max="5" width="5.28703703703704" customWidth="1"/>
+    <col min="6" max="6" width="17.287037037037" customWidth="1"/>
+    <col min="7" max="7" width="30.287037037037" customWidth="1"/>
+    <col min="8" max="8" width="26.8518518518519" customWidth="1"/>
+    <col min="9" max="9" width="17.287037037037" customWidth="1"/>
+    <col min="10" max="10" width="13.287037037037" customWidth="1"/>
+    <col min="11" max="11" width="22.712962962963" customWidth="1"/>
+    <col min="12" max="12" width="12.712962962963" customWidth="1"/>
+    <col min="13" max="13" width="29.5740740740741" customWidth="1"/>
+    <col min="14" max="14" width="18.287037037037" customWidth="1"/>
+    <col min="15" max="15" width="16.287037037037" customWidth="1"/>
+    <col min="16" max="16" width="15.5740740740741" customWidth="1"/>
+    <col min="17" max="17" width="17.712962962963" customWidth="1"/>
+    <col min="18" max="18" width="24.1388888888889" customWidth="1"/>
+    <col min="19" max="19" width="13.4259259259259" customWidth="1"/>
+    <col min="20" max="20" width="13.5740740740741" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:20">
-      <c r="A1" s="15" t="s">
+      <c r="A1" s="12" t="s">
         <v>25</v>
       </c>
-      <c r="B1" s="15" t="s">
+      <c r="B1" s="12" t="s">
         <v>26</v>
       </c>
-      <c r="C1" s="15" t="s">
+      <c r="C1" s="12" t="s">
         <v>27</v>
       </c>
-      <c r="D1" s="15" t="s">
+      <c r="D1" s="12" t="s">
         <v>28</v>
       </c>
-      <c r="E1" s="15" t="s">
+      <c r="E1" s="12" t="s">
         <v>29</v>
       </c>
-      <c r="F1" s="15" t="s">
+      <c r="F1" s="12" t="s">
         <v>2</v>
       </c>
-      <c r="G1" s="15" t="s">
+      <c r="G1" s="12" t="s">
         <v>1</v>
       </c>
-      <c r="H1" s="15" t="s">
+      <c r="H1" s="12" t="s">
         <v>30</v>
       </c>
-      <c r="I1" s="15" t="s">
+      <c r="I1" s="12" t="s">
         <v>31</v>
       </c>
-      <c r="J1" s="15" t="s">
+      <c r="J1" s="12" t="s">
         <v>32</v>
       </c>
-      <c r="K1" s="15" t="s">
+      <c r="K1" s="12" t="s">
         <v>33</v>
       </c>
-      <c r="L1" s="15" t="s">
+      <c r="L1" s="12" t="s">
         <v>6</v>
       </c>
-      <c r="M1" s="15" t="s">
+      <c r="M1" s="12" t="s">
         <v>7</v>
       </c>
-      <c r="N1" s="15" t="s">
+      <c r="N1" s="12" t="s">
         <v>8</v>
       </c>
-      <c r="O1" s="15" t="s">
+      <c r="O1" s="12" t="s">
         <v>9</v>
       </c>
-      <c r="P1" s="15" t="s">
+      <c r="P1" s="12" t="s">
         <v>34</v>
       </c>
-      <c r="Q1" s="15" t="s">
+      <c r="Q1" s="12" t="s">
         <v>35</v>
       </c>
-      <c r="R1" s="15" t="s">
+      <c r="R1" s="12" t="s">
         <v>36</v>
       </c>
-      <c r="S1" s="15" t="s">
+      <c r="S1" s="12" t="s">
         <v>37</v>
       </c>
-      <c r="T1" s="15" t="s">
+      <c r="T1" s="12" t="s">
         <v>38</v>
       </c>
     </row>
     <row r="2" spans="1:20">
-      <c r="A2" s="15" t="s">
+      <c r="A2" s="12" t="s">
         <v>18</v>
       </c>
-      <c r="B2" s="15" t="s">
+      <c r="B2" s="12" t="s">
         <v>39</v>
       </c>
-      <c r="C2" s="15" t="s">
+      <c r="C2" s="12" t="s">
         <v>20</v>
       </c>
-      <c r="D2" s="15" t="s">
+      <c r="D2" s="12" t="s">
         <v>40</v>
       </c>
-      <c r="E2" s="15">
+      <c r="E2" s="12">
         <v>12</v>
       </c>
-      <c r="F2" s="21" t="s">
+      <c r="F2" s="18" t="s">
         <v>12</v>
       </c>
-      <c r="G2" s="15" t="s">
+      <c r="G2" s="12" t="s">
         <v>11</v>
       </c>
-      <c r="H2" s="15" t="s">
+      <c r="H2" s="12" t="s">
         <v>19</v>
       </c>
-      <c r="I2" s="15" t="s">
+      <c r="I2" s="12" t="s">
         <v>41</v>
       </c>
-      <c r="J2" s="15" t="s">
+      <c r="J2" s="12" t="s">
         <v>14</v>
       </c>
-      <c r="K2" s="15">
+      <c r="K2" s="12">
         <v>6</v>
       </c>
-      <c r="L2" s="15">
+      <c r="L2" s="12">
         <v>1010301033</v>
       </c>
-      <c r="M2" s="15" t="s">
+      <c r="M2" s="12" t="s">
         <v>15</v>
       </c>
-      <c r="N2" s="15" t="s">
+      <c r="N2" s="12" t="s">
         <v>16</v>
       </c>
-      <c r="O2" s="15" t="s">
+      <c r="O2" s="12" t="s">
         <v>17</v>
       </c>
-      <c r="P2" s="15"/>
-      <c r="Q2" s="15"/>
-      <c r="R2" s="15"/>
-      <c r="S2" s="15">
+      <c r="P2" s="12"/>
+      <c r="Q2" s="12"/>
+      <c r="R2" s="12"/>
+      <c r="S2" s="12">
         <v>0</v>
       </c>
-      <c r="T2" s="15"/>
+      <c r="T2" s="12"/>
     </row>
     <row r="3" spans="1:20">
-      <c r="A3" s="15" t="s">
+      <c r="A3" s="12" t="s">
         <v>10</v>
       </c>
-      <c r="B3" s="15" t="s">
+      <c r="B3" s="12" t="s">
         <v>42</v>
       </c>
-      <c r="C3" s="15" t="s">
+      <c r="C3" s="12" t="s">
         <v>14</v>
       </c>
-      <c r="D3" s="22" t="s">
+      <c r="D3" s="19" t="s">
         <v>43</v>
       </c>
-      <c r="E3" s="15">
+      <c r="E3" s="12">
         <v>5</v>
       </c>
-      <c r="F3" s="15" t="s">
+      <c r="F3" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="G3" s="15" t="s">
+      <c r="G3" s="12" t="s">
         <v>11</v>
       </c>
-      <c r="H3" s="15" t="s">
+      <c r="H3" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="I3" s="15" t="s">
+      <c r="I3" s="12" t="s">
         <v>44</v>
       </c>
-      <c r="J3" s="15" t="s">
+      <c r="J3" s="12" t="s">
         <v>14</v>
       </c>
-      <c r="K3" s="15">
+      <c r="K3" s="12">
         <v>1</v>
       </c>
-      <c r="L3" s="15">
+      <c r="L3" s="12">
         <v>1010301033</v>
       </c>
-      <c r="M3" s="15" t="s">
+      <c r="M3" s="12" t="s">
         <v>15</v>
       </c>
-      <c r="N3" s="15" t="s">
+      <c r="N3" s="12" t="s">
         <v>16</v>
       </c>
-      <c r="O3" s="15" t="s">
+      <c r="O3" s="12" t="s">
         <v>17</v>
       </c>
-      <c r="P3" s="15"/>
-      <c r="Q3" s="15"/>
-      <c r="R3" s="15"/>
-      <c r="S3" s="15">
+      <c r="P3" s="12"/>
+      <c r="Q3" s="12"/>
+      <c r="R3" s="12"/>
+      <c r="S3" s="12">
         <v>0</v>
       </c>
-      <c r="T3" s="15"/>
+      <c r="T3" s="12"/>
     </row>
     <row r="4" spans="1:20">
-      <c r="A4" s="15" t="s">
+      <c r="A4" s="12" t="s">
         <v>21</v>
       </c>
-      <c r="B4" s="15" t="s">
+      <c r="B4" s="12" t="s">
         <v>45</v>
       </c>
-      <c r="C4" s="15" t="s">
+      <c r="C4" s="12" t="s">
         <v>14</v>
       </c>
-      <c r="D4" s="15">
+      <c r="D4" s="12">
         <v>123562</v>
       </c>
-      <c r="E4" s="15">
+      <c r="E4" s="12">
         <v>18</v>
       </c>
-      <c r="F4" s="15" t="s">
+      <c r="F4" s="12" t="s">
         <v>22</v>
       </c>
-      <c r="G4" s="15" t="s">
+      <c r="G4" s="12" t="s">
         <v>22</v>
       </c>
-      <c r="H4" s="15" t="s">
+      <c r="H4" s="12" t="s">
         <v>23</v>
       </c>
-      <c r="I4" s="15" t="s">
+      <c r="I4" s="12" t="s">
         <v>44</v>
       </c>
-      <c r="J4" s="15" t="s">
+      <c r="J4" s="12" t="s">
         <v>14</v>
       </c>
-      <c r="K4" s="15">
+      <c r="K4" s="12">
         <v>1</v>
       </c>
-      <c r="L4" s="15">
+      <c r="L4" s="12">
         <v>1011134888</v>
       </c>
-      <c r="M4" s="15" t="s">
+      <c r="M4" s="12" t="s">
         <v>46</v>
       </c>
-      <c r="N4" s="15" t="s">
+      <c r="N4" s="12" t="s">
         <v>16</v>
       </c>
-      <c r="O4" s="15" t="s">
+      <c r="O4" s="12" t="s">
         <v>17</v>
       </c>
-      <c r="P4" s="15"/>
-      <c r="Q4" s="15"/>
-      <c r="R4" s="15"/>
-      <c r="S4" s="15">
+      <c r="P4" s="12"/>
+      <c r="Q4" s="12"/>
+      <c r="R4" s="12"/>
+      <c r="S4" s="12">
         <v>0</v>
       </c>
-      <c r="T4" s="15"/>
+      <c r="T4" s="12"/>
     </row>
     <row r="5" spans="1:20">
       <c r="A5" s="2" t="s">
@@ -2493,7 +3163,7 @@
       <c r="B5" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="C5" s="15" t="s">
+      <c r="C5" s="12" t="s">
         <v>14</v>
       </c>
       <c r="D5" s="2" t="s">
@@ -2535,7 +3205,7 @@
       <c r="P5" s="2"/>
       <c r="Q5" s="2"/>
       <c r="R5" s="2"/>
-      <c r="S5" s="15">
+      <c r="S5" s="12">
         <v>0</v>
       </c>
       <c r="T5" s="2"/>
@@ -2550,16 +3220,16 @@
       <c r="C6" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="D6" s="20" t="s">
+      <c r="D6" s="17" t="s">
         <v>43</v>
       </c>
       <c r="E6">
         <v>5</v>
       </c>
-      <c r="F6" s="23" t="s">
+      <c r="F6" s="20" t="s">
         <v>12</v>
       </c>
-      <c r="G6" s="23" t="s">
+      <c r="G6" s="20" t="s">
         <v>11</v>
       </c>
       <c r="H6" s="2" t="s">
@@ -2589,172 +3259,172 @@
       <c r="P6" s="2"/>
       <c r="Q6" s="2"/>
       <c r="R6" s="2"/>
-      <c r="S6" s="15">
+      <c r="S6" s="12">
         <v>0</v>
       </c>
       <c r="T6" s="2"/>
     </row>
     <row r="7" spans="1:20">
-      <c r="A7" s="24" t="s">
+      <c r="A7" s="21" t="s">
         <v>55</v>
       </c>
-      <c r="B7" s="24" t="s">
+      <c r="B7" s="21" t="s">
         <v>56</v>
       </c>
-      <c r="C7" s="24" t="s">
+      <c r="C7" s="21" t="s">
         <v>20</v>
       </c>
-      <c r="D7" s="24" t="s">
+      <c r="D7" s="21" t="s">
         <v>40</v>
       </c>
-      <c r="E7" s="24">
+      <c r="E7" s="21">
         <v>12</v>
       </c>
-      <c r="F7" s="25" t="s">
+      <c r="F7" s="22" t="s">
         <v>12</v>
       </c>
-      <c r="G7" s="24" t="s">
+      <c r="G7" s="21" t="s">
         <v>11</v>
       </c>
-      <c r="H7" s="24" t="s">
+      <c r="H7" s="21" t="s">
         <v>57</v>
       </c>
-      <c r="I7" s="24" t="s">
+      <c r="I7" s="21" t="s">
         <v>41</v>
       </c>
-      <c r="J7" s="24" t="s">
+      <c r="J7" s="21" t="s">
         <v>14</v>
       </c>
-      <c r="K7" s="24">
+      <c r="K7" s="21">
         <v>3</v>
       </c>
-      <c r="L7" s="24">
+      <c r="L7" s="21">
         <v>1010301003</v>
       </c>
-      <c r="M7" s="24" t="s">
+      <c r="M7" s="21" t="s">
         <v>58</v>
       </c>
-      <c r="N7" s="24" t="s">
+      <c r="N7" s="21" t="s">
         <v>16</v>
       </c>
-      <c r="O7" s="24" t="s">
+      <c r="O7" s="21" t="s">
         <v>17</v>
       </c>
-      <c r="P7" s="24"/>
-      <c r="Q7" s="24"/>
-      <c r="R7" s="24"/>
-      <c r="S7" s="24">
+      <c r="P7" s="21"/>
+      <c r="Q7" s="21"/>
+      <c r="R7" s="21"/>
+      <c r="S7" s="21">
         <v>0</v>
       </c>
-      <c r="T7" s="24"/>
+      <c r="T7" s="21"/>
     </row>
     <row r="8" spans="1:20">
-      <c r="A8" s="24" t="s">
+      <c r="A8" s="21" t="s">
         <v>59</v>
       </c>
-      <c r="B8" s="24" t="s">
+      <c r="B8" s="21" t="s">
         <v>60</v>
       </c>
-      <c r="C8" s="24" t="s">
+      <c r="C8" s="21" t="s">
         <v>14</v>
       </c>
-      <c r="D8" s="24" t="s">
+      <c r="D8" s="21" t="s">
         <v>43</v>
       </c>
-      <c r="E8" s="24">
+      <c r="E8" s="21">
         <v>5</v>
       </c>
-      <c r="F8" s="25" t="s">
+      <c r="F8" s="22" t="s">
         <v>12</v>
       </c>
-      <c r="G8" s="24" t="s">
+      <c r="G8" s="21" t="s">
         <v>11</v>
       </c>
-      <c r="H8" s="24" t="s">
+      <c r="H8" s="21" t="s">
         <v>57</v>
       </c>
-      <c r="I8" s="24" t="s">
+      <c r="I8" s="21" t="s">
         <v>41</v>
       </c>
-      <c r="J8" s="24" t="s">
+      <c r="J8" s="21" t="s">
         <v>14</v>
       </c>
-      <c r="K8" s="24">
+      <c r="K8" s="21">
         <v>0</v>
       </c>
-      <c r="L8" s="24">
+      <c r="L8" s="21">
         <v>1010301003</v>
       </c>
-      <c r="M8" s="24" t="s">
+      <c r="M8" s="21" t="s">
         <v>58</v>
       </c>
-      <c r="N8" s="24" t="s">
+      <c r="N8" s="21" t="s">
         <v>16</v>
       </c>
-      <c r="O8" s="24" t="s">
+      <c r="O8" s="21" t="s">
         <v>17</v>
       </c>
-      <c r="P8" s="24"/>
-      <c r="Q8" s="24"/>
-      <c r="R8" s="24"/>
-      <c r="S8" s="24">
+      <c r="P8" s="21"/>
+      <c r="Q8" s="21"/>
+      <c r="R8" s="21"/>
+      <c r="S8" s="21">
         <v>0</v>
       </c>
-      <c r="T8" s="24"/>
+      <c r="T8" s="21"/>
     </row>
     <row r="9" spans="1:20">
-      <c r="A9" s="24" t="s">
+      <c r="A9" s="21" t="s">
         <v>61</v>
       </c>
-      <c r="B9" s="24" t="s">
+      <c r="B9" s="21" t="s">
         <v>61</v>
       </c>
-      <c r="C9" s="24" t="s">
+      <c r="C9" s="21" t="s">
         <v>14</v>
       </c>
-      <c r="D9" s="24" t="s">
+      <c r="D9" s="21" t="s">
         <v>43</v>
       </c>
-      <c r="E9" s="24">
+      <c r="E9" s="21">
         <v>5</v>
       </c>
-      <c r="F9" s="25" t="s">
+      <c r="F9" s="22" t="s">
         <v>12</v>
       </c>
-      <c r="G9" s="24" t="s">
+      <c r="G9" s="21" t="s">
         <v>11</v>
       </c>
-      <c r="H9" s="24" t="s">
+      <c r="H9" s="21" t="s">
         <v>57</v>
       </c>
-      <c r="I9" s="24" t="s">
+      <c r="I9" s="21" t="s">
         <v>41</v>
       </c>
-      <c r="J9" s="24" t="s">
+      <c r="J9" s="21" t="s">
         <v>14</v>
       </c>
-      <c r="K9" s="24">
+      <c r="K9" s="21">
         <v>0</v>
       </c>
-      <c r="L9" s="24">
+      <c r="L9" s="21">
         <v>1010301003</v>
       </c>
-      <c r="M9" s="24" t="s">
+      <c r="M9" s="21" t="s">
         <v>58</v>
       </c>
-      <c r="N9" s="24" t="s">
+      <c r="N9" s="21" t="s">
         <v>16</v>
       </c>
-      <c r="O9" s="24" t="s">
+      <c r="O9" s="21" t="s">
         <v>17</v>
       </c>
-      <c r="P9" s="24"/>
-      <c r="Q9" s="24"/>
-      <c r="R9" s="24"/>
-      <c r="S9" s="24">
+      <c r="P9" s="21"/>
+      <c r="Q9" s="21"/>
+      <c r="R9" s="21"/>
+      <c r="S9" s="21">
         <v>0</v>
       </c>
-      <c r="T9" s="24"/>
+      <c r="T9" s="21"/>
     </row>
     <row r="10" spans="1:20">
       <c r="A10" s="2" t="s">
@@ -2766,31 +3436,31 @@
       <c r="C10" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="D10" s="24" t="s">
+      <c r="D10" s="21" t="s">
         <v>43</v>
       </c>
-      <c r="E10" s="24">
+      <c r="E10" s="21">
         <v>5</v>
       </c>
-      <c r="F10" s="15" t="s">
+      <c r="F10" s="12" t="s">
         <v>22</v>
       </c>
-      <c r="G10" s="15" t="s">
+      <c r="G10" s="12" t="s">
         <v>22</v>
       </c>
-      <c r="H10" s="15" t="s">
+      <c r="H10" s="12" t="s">
         <v>63</v>
       </c>
-      <c r="I10" s="15" t="s">
+      <c r="I10" s="12" t="s">
         <v>44</v>
       </c>
-      <c r="J10" s="15" t="s">
+      <c r="J10" s="12" t="s">
         <v>14</v>
       </c>
-      <c r="K10" s="15">
+      <c r="K10" s="12">
         <v>1</v>
       </c>
-      <c r="L10" s="18">
+      <c r="L10" s="15">
         <v>1000000001</v>
       </c>
       <c r="M10" s="2" t="s">
@@ -2802,35 +3472,37 @@
       <c r="O10" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="P10" s="24"/>
-      <c r="Q10" s="24"/>
-      <c r="R10" s="24"/>
-      <c r="S10" s="24">
+      <c r="P10" s="21"/>
+      <c r="Q10" s="21"/>
+      <c r="R10" s="21"/>
+      <c r="S10" s="21">
         <v>0</v>
       </c>
-      <c r="T10" s="24"/>
+      <c r="T10" s="21"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
   <dimension ref="A1:R3"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="8.85185185185185" defaultRowHeight="14.4" outlineLevelRow="2"/>
   <cols>
     <col min="1" max="2" width="21" customWidth="1"/>
     <col min="3" max="3" width="6" customWidth="1"/>
-    <col min="4" max="4" width="12.7109375" customWidth="1"/>
-    <col min="5" max="5" width="19.42578125" customWidth="1"/>
-    <col min="6" max="6" width="15.140625" customWidth="1"/>
-    <col min="7" max="7" width="15.42578125" customWidth="1"/>
-    <col min="8" max="8" width="19.5703125" customWidth="1"/>
-    <col min="9" max="9" width="10.85546875" customWidth="1"/>
-    <col min="10" max="10" width="17.5703125" customWidth="1"/>
-    <col min="11" max="11" width="11.28515625" customWidth="1"/>
-    <col min="12" max="12" width="21.7109375" customWidth="1"/>
+    <col min="4" max="4" width="12.712962962963" customWidth="1"/>
+    <col min="5" max="5" width="19.4259259259259" customWidth="1"/>
+    <col min="6" max="6" width="15.1388888888889" customWidth="1"/>
+    <col min="7" max="7" width="15.4259259259259" customWidth="1"/>
+    <col min="8" max="8" width="19.5740740740741" customWidth="1"/>
+    <col min="9" max="9" width="10.8518518518519" customWidth="1"/>
+    <col min="10" max="10" width="17.5740740740741" customWidth="1"/>
+    <col min="11" max="11" width="11.287037037037" customWidth="1"/>
+    <col min="12" max="12" width="21.712962962963" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:18">
@@ -2843,16 +3515,16 @@
       <c r="C1" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="D1" s="15" t="s">
+      <c r="D1" s="12" t="s">
         <v>6</v>
       </c>
-      <c r="E1" s="15" t="s">
+      <c r="E1" s="12" t="s">
         <v>7</v>
       </c>
-      <c r="F1" s="15" t="s">
+      <c r="F1" s="12" t="s">
         <v>8</v>
       </c>
-      <c r="G1" s="15" t="s">
+      <c r="G1" s="12" t="s">
         <v>9</v>
       </c>
       <c r="H1" s="2" t="s">
@@ -2870,12 +3542,12 @@
       <c r="L1" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="M1" s="19"/>
-      <c r="N1" s="19"/>
-      <c r="O1" s="19"/>
-      <c r="P1" s="19"/>
-      <c r="Q1" s="19"/>
-      <c r="R1" s="19"/>
+      <c r="M1" s="16"/>
+      <c r="N1" s="16"/>
+      <c r="O1" s="16"/>
+      <c r="P1" s="16"/>
+      <c r="Q1" s="16"/>
+      <c r="R1" s="16"/>
     </row>
     <row r="2" spans="1:18">
       <c r="A2" s="2" t="s">
@@ -2902,7 +3574,7 @@
       <c r="H2" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="I2" s="20" t="s">
+      <c r="I2" s="17" t="s">
         <v>43</v>
       </c>
       <c r="J2" s="2" t="s">
@@ -2914,14 +3586,14 @@
       <c r="L2" s="2">
         <v>1</v>
       </c>
-      <c r="M2" s="19"/>
-      <c r="N2" s="19"/>
-      <c r="O2" s="19"/>
-      <c r="P2" s="19"/>
-      <c r="Q2" s="19"/>
-      <c r="R2" s="19"/>
-    </row>
-    <row r="3" spans="1:18">
+      <c r="M2" s="16"/>
+      <c r="N2" s="16"/>
+      <c r="O2" s="16"/>
+      <c r="P2" s="16"/>
+      <c r="Q2" s="16"/>
+      <c r="R2" s="16"/>
+    </row>
+    <row r="3" spans="1:12">
       <c r="A3" s="2" t="s">
         <v>62</v>
       </c>
@@ -2931,7 +3603,7 @@
       <c r="C3" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="D3" s="18">
+      <c r="D3" s="15">
         <v>1000000001</v>
       </c>
       <c r="E3" s="2" t="s">
@@ -2946,7 +3618,7 @@
       <c r="H3" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="I3" s="20" t="s">
+      <c r="I3" s="17" t="s">
         <v>43</v>
       </c>
       <c r="J3" s="2" t="s">
@@ -2961,39 +3633,41 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
   <dimension ref="A1:F3"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="8.85185185185185" defaultRowHeight="14.4" outlineLevelRow="2" outlineLevelCol="5"/>
   <cols>
-    <col min="1" max="1" width="27.140625" customWidth="1"/>
-    <col min="2" max="2" width="10.42578125" customWidth="1"/>
-    <col min="3" max="3" width="11.42578125" customWidth="1"/>
-    <col min="4" max="4" width="11.7109375" customWidth="1"/>
-    <col min="5" max="5" width="14.5703125" customWidth="1"/>
-    <col min="6" max="6" width="17.7109375" customWidth="1"/>
+    <col min="1" max="1" width="27.1388888888889" customWidth="1"/>
+    <col min="2" max="2" width="10.4259259259259" customWidth="1"/>
+    <col min="3" max="3" width="11.4259259259259" customWidth="1"/>
+    <col min="4" max="4" width="11.712962962963" customWidth="1"/>
+    <col min="5" max="5" width="14.5740740740741" customWidth="1"/>
+    <col min="6" max="6" width="17.712962962963" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6">
-      <c r="A1" s="16" t="s">
+      <c r="A1" s="13" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="16" t="s">
+      <c r="B1" s="13" t="s">
         <v>66</v>
       </c>
-      <c r="C1" s="16" t="s">
+      <c r="C1" s="13" t="s">
         <v>67</v>
       </c>
-      <c r="D1" s="17" t="s">
+      <c r="D1" s="14" t="s">
         <v>68</v>
       </c>
-      <c r="E1" s="15" t="s">
+      <c r="E1" s="12" t="s">
         <v>69</v>
       </c>
-      <c r="F1" s="15" t="s">
+      <c r="F1" s="12" t="s">
         <v>70</v>
       </c>
     </row>
@@ -3011,7 +3685,7 @@
         <v>71</v>
       </c>
       <c r="E2" s="2"/>
-      <c r="F2" s="9" t="s">
+      <c r="F2" s="7" t="s">
         <v>72</v>
       </c>
     </row>
@@ -3028,53 +3702,55 @@
       <c r="D3" s="2" t="s">
         <v>73</v>
       </c>
-      <c r="E3" s="9" t="s">
+      <c r="E3" s="7" t="s">
         <v>74</v>
       </c>
-      <c r="F3" s="9">
+      <c r="F3" s="7">
         <v>2</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
   <dimension ref="A1:F4"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="8.85185185185185" defaultRowHeight="14.4" outlineLevelRow="3" outlineLevelCol="5"/>
   <cols>
-    <col min="1" max="1" width="27.140625" customWidth="1"/>
-    <col min="2" max="2" width="10.42578125" customWidth="1"/>
-    <col min="3" max="3" width="11.42578125" customWidth="1"/>
-    <col min="4" max="4" width="11.7109375" customWidth="1"/>
-    <col min="5" max="5" width="14.5703125" customWidth="1"/>
-    <col min="6" max="6" width="17.7109375" customWidth="1"/>
+    <col min="1" max="1" width="27.1388888888889" customWidth="1"/>
+    <col min="2" max="2" width="10.4259259259259" customWidth="1"/>
+    <col min="3" max="3" width="11.4259259259259" customWidth="1"/>
+    <col min="4" max="4" width="11.712962962963" customWidth="1"/>
+    <col min="5" max="5" width="14.5740740740741" customWidth="1"/>
+    <col min="6" max="6" width="17.712962962963" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6">
-      <c r="A1" s="16" t="s">
+      <c r="A1" s="13" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="16" t="s">
+      <c r="B1" s="13" t="s">
         <v>66</v>
       </c>
-      <c r="C1" s="16" t="s">
+      <c r="C1" s="13" t="s">
         <v>67</v>
       </c>
-      <c r="D1" s="17" t="s">
+      <c r="D1" s="14" t="s">
         <v>68</v>
       </c>
-      <c r="E1" s="15" t="s">
+      <c r="E1" s="12" t="s">
         <v>69</v>
       </c>
-      <c r="F1" s="15" t="s">
+      <c r="F1" s="12" t="s">
         <v>70</v>
       </c>
     </row>
     <row r="2" spans="1:6">
-      <c r="A2" s="15" t="s">
+      <c r="A2" s="12" t="s">
         <v>59</v>
       </c>
       <c r="B2" s="2">
@@ -3087,12 +3763,12 @@
         <v>71</v>
       </c>
       <c r="E2" s="2"/>
-      <c r="F2" s="9" t="s">
+      <c r="F2" s="7" t="s">
         <v>75</v>
       </c>
     </row>
     <row r="3" spans="1:6">
-      <c r="A3" s="15" t="s">
+      <c r="A3" s="12" t="s">
         <v>76</v>
       </c>
       <c r="B3" s="2">
@@ -3104,15 +3780,15 @@
       <c r="D3" s="2" t="s">
         <v>77</v>
       </c>
-      <c r="E3" s="9" t="s">
+      <c r="E3" s="7" t="s">
         <v>74</v>
       </c>
-      <c r="F3" s="9">
+      <c r="F3" s="7">
         <v>2</v>
       </c>
     </row>
     <row r="4" spans="1:6">
-      <c r="A4" s="15" t="s">
+      <c r="A4" s="12" t="s">
         <v>61</v>
       </c>
       <c r="B4" s="2">
@@ -3127,19 +3803,21 @@
       <c r="E4" s="2" t="s">
         <v>75</v>
       </c>
-      <c r="F4" s="9"/>
+      <c r="F4" s="7"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
   <dimension ref="A1:C3"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="8.85185185185185" defaultRowHeight="14.4" outlineLevelRow="2" outlineLevelCol="2"/>
   <cols>
-    <col min="1" max="1" width="28.7109375" customWidth="1"/>
+    <col min="1" max="1" width="28.712962962963" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3">
@@ -3177,86 +3855,88 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
   <dimension ref="A1:G4"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="8.85185185185185" defaultRowHeight="14.4" outlineLevelRow="3" outlineLevelCol="6"/>
   <cols>
-    <col min="1" max="1" width="19.7109375" customWidth="1"/>
-    <col min="2" max="2" width="8.140625" customWidth="1"/>
-    <col min="3" max="3" width="8.5703125" customWidth="1"/>
-    <col min="4" max="4" width="17.85546875" customWidth="1"/>
-    <col min="5" max="5" width="12.7109375" customWidth="1"/>
-    <col min="6" max="6" width="14.5703125" customWidth="1"/>
-    <col min="7" max="7" width="17.7109375" customWidth="1"/>
+    <col min="1" max="1" width="19.712962962963" customWidth="1"/>
+    <col min="2" max="2" width="8.13888888888889" customWidth="1"/>
+    <col min="3" max="3" width="8.57407407407407" customWidth="1"/>
+    <col min="4" max="4" width="17.8518518518519" customWidth="1"/>
+    <col min="5" max="5" width="12.712962962963" customWidth="1"/>
+    <col min="6" max="6" width="14.5740740740741" customWidth="1"/>
+    <col min="7" max="7" width="17.712962962963" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7">
-      <c r="A1" s="15" t="s">
+      <c r="A1" s="12" t="s">
         <v>83</v>
       </c>
-      <c r="B1" s="15" t="s">
+      <c r="B1" s="12" t="s">
         <v>84</v>
       </c>
-      <c r="C1" s="15" t="s">
+      <c r="C1" s="12" t="s">
         <v>80</v>
       </c>
-      <c r="D1" s="15" t="s">
+      <c r="D1" s="12" t="s">
         <v>85</v>
       </c>
-      <c r="E1" s="15" t="s">
+      <c r="E1" s="12" t="s">
         <v>68</v>
       </c>
-      <c r="F1" s="15" t="s">
+      <c r="F1" s="12" t="s">
         <v>69</v>
       </c>
-      <c r="G1" s="15" t="s">
+      <c r="G1" s="12" t="s">
         <v>70</v>
       </c>
     </row>
     <row r="2" spans="1:7">
-      <c r="A2" s="15" t="s">
+      <c r="A2" s="12" t="s">
         <v>86</v>
       </c>
-      <c r="B2" s="15">
+      <c r="B2" s="12">
         <v>524</v>
       </c>
-      <c r="C2" s="15">
+      <c r="C2" s="12">
         <v>524</v>
       </c>
-      <c r="D2" s="15">
+      <c r="D2" s="12">
         <v>2</v>
       </c>
-      <c r="E2" s="9" t="s">
+      <c r="E2" s="7" t="s">
         <v>71</v>
       </c>
-      <c r="F2" s="9" t="s">
+      <c r="F2" s="7" t="s">
         <v>74</v>
       </c>
-      <c r="G2" s="9" t="s">
+      <c r="G2" s="7" t="s">
         <v>87</v>
       </c>
     </row>
     <row r="3" spans="1:7">
-      <c r="A3" s="15" t="s">
+      <c r="A3" s="12" t="s">
         <v>88</v>
       </c>
-      <c r="B3" s="15">
+      <c r="B3" s="12">
         <v>232</v>
       </c>
-      <c r="C3" s="15">
+      <c r="C3" s="12">
         <v>232</v>
       </c>
-      <c r="D3" s="15">
+      <c r="D3" s="12">
         <v>7.9</v>
       </c>
-      <c r="E3" s="9" t="s">
+      <c r="E3" s="7" t="s">
         <v>73</v>
       </c>
-      <c r="F3" s="9" t="s">
+      <c r="F3" s="7" t="s">
         <v>89</v>
       </c>
       <c r="G3" s="2"/>
@@ -3272,9 +3952,9 @@
         <v>232</v>
       </c>
       <c r="D4" s="2">
-        <v>2.3199999999999998</v>
-      </c>
-      <c r="E4" s="9" t="s">
+        <v>2.32</v>
+      </c>
+      <c r="E4" s="7" t="s">
         <v>77</v>
       </c>
       <c r="F4" s="2"/>
@@ -3282,86 +3962,88 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
   <dimension ref="A1:G4"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="8.85185185185185" defaultRowHeight="14.4" outlineLevelRow="3" outlineLevelCol="6"/>
   <cols>
-    <col min="1" max="1" width="19.7109375" customWidth="1"/>
-    <col min="2" max="2" width="8.140625" customWidth="1"/>
-    <col min="3" max="3" width="8.5703125" customWidth="1"/>
-    <col min="4" max="4" width="17.85546875" customWidth="1"/>
-    <col min="5" max="5" width="12.7109375" customWidth="1"/>
-    <col min="6" max="6" width="14.5703125" customWidth="1"/>
-    <col min="7" max="7" width="17.7109375" customWidth="1"/>
+    <col min="1" max="1" width="19.712962962963" customWidth="1"/>
+    <col min="2" max="2" width="8.13888888888889" customWidth="1"/>
+    <col min="3" max="3" width="8.57407407407407" customWidth="1"/>
+    <col min="4" max="4" width="17.8518518518519" customWidth="1"/>
+    <col min="5" max="5" width="12.712962962963" customWidth="1"/>
+    <col min="6" max="6" width="14.5740740740741" customWidth="1"/>
+    <col min="7" max="7" width="17.712962962963" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7">
-      <c r="A1" s="15" t="s">
+      <c r="A1" s="12" t="s">
         <v>83</v>
       </c>
-      <c r="B1" s="15" t="s">
+      <c r="B1" s="12" t="s">
         <v>84</v>
       </c>
-      <c r="C1" s="15" t="s">
+      <c r="C1" s="12" t="s">
         <v>80</v>
       </c>
-      <c r="D1" s="15" t="s">
+      <c r="D1" s="12" t="s">
         <v>85</v>
       </c>
-      <c r="E1" s="15" t="s">
+      <c r="E1" s="12" t="s">
         <v>68</v>
       </c>
-      <c r="F1" s="15" t="s">
+      <c r="F1" s="12" t="s">
         <v>69</v>
       </c>
-      <c r="G1" s="15" t="s">
+      <c r="G1" s="12" t="s">
         <v>70</v>
       </c>
     </row>
     <row r="2" spans="1:7">
-      <c r="A2" s="15" t="s">
+      <c r="A2" s="12" t="s">
         <v>86</v>
       </c>
-      <c r="B2" s="15">
+      <c r="B2" s="12">
         <v>22</v>
       </c>
-      <c r="C2" s="15">
+      <c r="C2" s="12">
         <v>524</v>
       </c>
-      <c r="D2" s="15">
+      <c r="D2" s="12">
         <v>2</v>
       </c>
-      <c r="E2" s="9" t="s">
+      <c r="E2" s="7" t="s">
         <v>71</v>
       </c>
-      <c r="F2" s="9" t="s">
+      <c r="F2" s="7" t="s">
         <v>74</v>
       </c>
-      <c r="G2" s="9" t="s">
+      <c r="G2" s="7" t="s">
         <v>87</v>
       </c>
     </row>
     <row r="3" spans="1:7">
-      <c r="A3" s="15" t="s">
+      <c r="A3" s="12" t="s">
         <v>88</v>
       </c>
-      <c r="B3" s="15">
+      <c r="B3" s="12">
         <v>34</v>
       </c>
-      <c r="C3" s="15">
+      <c r="C3" s="12">
         <v>232</v>
       </c>
-      <c r="D3" s="15">
+      <c r="D3" s="12">
         <v>7.9</v>
       </c>
-      <c r="E3" s="9" t="s">
+      <c r="E3" s="7" t="s">
         <v>73</v>
       </c>
-      <c r="F3" s="9" t="s">
+      <c r="F3" s="7" t="s">
         <v>89</v>
       </c>
       <c r="G3" s="2"/>
@@ -3377,9 +4059,9 @@
         <v>232</v>
       </c>
       <c r="D4" s="2">
-        <v>2.3199999999999998</v>
-      </c>
-      <c r="E4" s="9" t="s">
+        <v>2.32</v>
+      </c>
+      <c r="E4" s="7" t="s">
         <v>77</v>
       </c>
       <c r="F4" s="2"/>
@@ -3387,31 +4069,33 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
   <dimension ref="A1:S11"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="8.85185185185185" defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="39.7109375" customWidth="1"/>
-    <col min="2" max="2" width="10.140625" customWidth="1"/>
-    <col min="3" max="3" width="39.7109375" customWidth="1"/>
+    <col min="1" max="1" width="39.712962962963" customWidth="1"/>
+    <col min="2" max="2" width="10.1388888888889" customWidth="1"/>
+    <col min="3" max="3" width="39.712962962963" customWidth="1"/>
     <col min="4" max="4" width="11" customWidth="1"/>
-    <col min="5" max="5" width="13.28515625" customWidth="1"/>
-    <col min="6" max="6" width="8.85546875" customWidth="1"/>
-    <col min="7" max="7" width="17.85546875" customWidth="1"/>
-    <col min="8" max="8" width="19.5703125" customWidth="1"/>
-    <col min="9" max="9" width="23.7109375" customWidth="1"/>
-    <col min="10" max="10" width="12.7109375" customWidth="1"/>
-    <col min="11" max="11" width="11.85546875" customWidth="1"/>
-    <col min="12" max="12" width="17.42578125" customWidth="1"/>
-    <col min="13" max="14" width="39.7109375" customWidth="1"/>
-    <col min="15" max="15" width="25.7109375" customWidth="1"/>
-    <col min="16" max="17" width="16.5703125" customWidth="1"/>
-    <col min="18" max="18" width="11.5703125" customWidth="1"/>
-    <col min="19" max="19" width="14.85546875" customWidth="1"/>
+    <col min="5" max="5" width="13.287037037037" customWidth="1"/>
+    <col min="6" max="6" width="8.85185185185185" customWidth="1"/>
+    <col min="7" max="7" width="17.8518518518519" customWidth="1"/>
+    <col min="8" max="8" width="19.5740740740741" customWidth="1"/>
+    <col min="9" max="9" width="23.712962962963" customWidth="1"/>
+    <col min="10" max="10" width="12.712962962963" customWidth="1"/>
+    <col min="11" max="11" width="11.8518518518519" customWidth="1"/>
+    <col min="12" max="12" width="17.4259259259259" customWidth="1"/>
+    <col min="13" max="14" width="39.712962962963" customWidth="1"/>
+    <col min="15" max="15" width="25.712962962963" customWidth="1"/>
+    <col min="16" max="17" width="16.5740740740741" customWidth="1"/>
+    <col min="18" max="18" width="11.5740740740741" customWidth="1"/>
+    <col min="19" max="19" width="14.8518518518519" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:19">
@@ -3469,18 +4153,18 @@
       <c r="R1" s="2" t="s">
         <v>104</v>
       </c>
-      <c r="S1" s="14" t="s">
+      <c r="S1" s="5" t="s">
         <v>105</v>
       </c>
     </row>
     <row r="2" spans="1:19">
-      <c r="A2" s="13" t="s">
+      <c r="A2" s="11" t="s">
         <v>106</v>
       </c>
       <c r="B2" s="2">
         <v>0</v>
       </c>
-      <c r="C2" s="13" t="s">
+      <c r="C2" s="11" t="s">
         <v>106</v>
       </c>
       <c r="D2" s="2" t="s">
@@ -3508,36 +4192,36 @@
       </c>
       <c r="M2" s="2"/>
       <c r="N2" s="2"/>
-      <c r="O2" s="9" t="s">
+      <c r="O2" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="P2" s="9" t="s">
+      <c r="P2" s="7" t="s">
         <v>15</v>
       </c>
-      <c r="Q2" s="9" t="s">
+      <c r="Q2" s="7" t="s">
         <v>15</v>
       </c>
       <c r="R2" s="2" t="s">
         <v>108</v>
       </c>
-      <c r="S2" s="12" t="s">
+      <c r="S2" s="10" t="s">
         <v>109</v>
       </c>
     </row>
     <row r="3" spans="1:19">
-      <c r="A3" s="13" t="s">
+      <c r="A3" s="11" t="s">
         <v>110</v>
       </c>
       <c r="B3" s="2">
         <v>0</v>
       </c>
-      <c r="C3" s="13" t="s">
+      <c r="C3" s="11" t="s">
         <v>110</v>
       </c>
       <c r="D3" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="E3" s="13">
+      <c r="E3" s="11">
         <v>772213</v>
       </c>
       <c r="F3" s="2">
@@ -3559,19 +4243,19 @@
       </c>
       <c r="M3" s="2"/>
       <c r="N3" s="2"/>
-      <c r="O3" s="9" t="s">
+      <c r="O3" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="P3" s="9" t="s">
+      <c r="P3" s="7" t="s">
         <v>15</v>
       </c>
-      <c r="Q3" s="9" t="s">
+      <c r="Q3" s="7" t="s">
         <v>15</v>
       </c>
       <c r="R3" s="2" t="s">
         <v>108</v>
       </c>
-      <c r="S3" s="12" t="s">
+      <c r="S3" s="10" t="s">
         <v>109</v>
       </c>
     </row>
@@ -3585,7 +4269,7 @@
       <c r="C4" s="2" t="s">
         <v>111</v>
       </c>
-      <c r="D4" s="14" t="s">
+      <c r="D4" s="5" t="s">
         <v>14</v>
       </c>
       <c r="E4" s="2" t="s">
@@ -3594,7 +4278,7 @@
       <c r="F4" s="2">
         <v>12</v>
       </c>
-      <c r="G4" s="14" t="s">
+      <c r="G4" s="5" t="s">
         <v>112</v>
       </c>
       <c r="H4" s="2"/>
@@ -3614,19 +4298,19 @@
       <c r="N4" s="2" t="s">
         <v>111</v>
       </c>
-      <c r="O4" s="9" t="s">
+      <c r="O4" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="P4" s="9" t="s">
+      <c r="P4" s="7" t="s">
         <v>15</v>
       </c>
-      <c r="Q4" s="9" t="s">
+      <c r="Q4" s="7" t="s">
         <v>15</v>
       </c>
       <c r="R4" s="2" t="s">
         <v>108</v>
       </c>
-      <c r="S4" s="12" t="s">
+      <c r="S4" s="10" t="s">
         <v>109</v>
       </c>
     </row>
@@ -3634,30 +4318,30 @@
       <c r="A5" s="2" t="s">
         <v>113</v>
       </c>
-      <c r="B5" s="14">
+      <c r="B5" s="5">
         <v>0</v>
       </c>
       <c r="C5" s="2" t="s">
         <v>113</v>
       </c>
-      <c r="D5" s="14" t="s">
+      <c r="D5" s="5" t="s">
         <v>14</v>
       </c>
       <c r="E5" s="2">
         <v>75052200</v>
       </c>
-      <c r="F5" s="14">
+      <c r="F5" s="5">
         <v>5</v>
       </c>
-      <c r="G5" s="14" t="s">
+      <c r="G5" s="5" t="s">
         <v>112</v>
       </c>
       <c r="H5" s="2"/>
       <c r="I5" s="2"/>
-      <c r="J5" s="14" t="s">
+      <c r="J5" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="K5" s="14">
+      <c r="K5" s="5">
         <v>2</v>
       </c>
       <c r="L5" s="2" t="s">
@@ -3669,133 +4353,133 @@
       <c r="N5" s="2" t="s">
         <v>113</v>
       </c>
-      <c r="O5" s="9" t="s">
+      <c r="O5" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="P5" s="9" t="s">
+      <c r="P5" s="7" t="s">
         <v>15</v>
       </c>
-      <c r="Q5" s="9" t="s">
+      <c r="Q5" s="7" t="s">
         <v>15</v>
       </c>
       <c r="R5" s="2" t="s">
         <v>114</v>
       </c>
-      <c r="S5" s="12" t="s">
+      <c r="S5" s="10" t="s">
         <v>109</v>
       </c>
     </row>
     <row r="6" spans="1:19">
-      <c r="A6" s="14" t="s">
+      <c r="A6" s="5" t="s">
         <v>115</v>
       </c>
-      <c r="B6" s="14">
+      <c r="B6" s="5">
         <v>0</v>
       </c>
       <c r="C6" s="2" t="s">
         <v>115</v>
       </c>
-      <c r="D6" s="14" t="s">
+      <c r="D6" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="E6" s="14" t="s">
+      <c r="E6" s="5" t="s">
         <v>40</v>
       </c>
-      <c r="F6" s="14">
+      <c r="F6" s="5">
         <v>12</v>
       </c>
-      <c r="G6" s="14" t="s">
+      <c r="G6" s="5" t="s">
         <v>116</v>
       </c>
-      <c r="H6" s="14" t="s">
+      <c r="H6" s="5" t="s">
         <v>117</v>
       </c>
       <c r="I6" s="2"/>
-      <c r="J6" s="14" t="s">
+      <c r="J6" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="K6" s="14">
+      <c r="K6" s="5">
         <v>1</v>
       </c>
       <c r="L6" s="2" t="s">
         <v>107</v>
       </c>
-      <c r="M6" s="14" t="s">
+      <c r="M6" s="5" t="s">
         <v>115</v>
       </c>
-      <c r="N6" s="14" t="s">
+      <c r="N6" s="5" t="s">
         <v>115</v>
       </c>
-      <c r="O6" s="9" t="s">
+      <c r="O6" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="P6" s="9" t="s">
+      <c r="P6" s="7" t="s">
         <v>15</v>
       </c>
-      <c r="Q6" s="9" t="s">
+      <c r="Q6" s="7" t="s">
         <v>15</v>
       </c>
       <c r="R6" s="2" t="s">
         <v>108</v>
       </c>
-      <c r="S6" s="12" t="s">
+      <c r="S6" s="10" t="s">
         <v>109</v>
       </c>
     </row>
     <row r="7" spans="1:19">
-      <c r="A7" s="14" t="s">
+      <c r="A7" s="5" t="s">
         <v>118</v>
       </c>
-      <c r="B7" s="14">
+      <c r="B7" s="5">
         <v>0</v>
       </c>
       <c r="C7" s="2" t="s">
         <v>118</v>
       </c>
-      <c r="D7" s="14" t="s">
+      <c r="D7" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="E7" s="14" t="s">
+      <c r="E7" s="5" t="s">
         <v>40</v>
       </c>
-      <c r="F7" s="14">
+      <c r="F7" s="5">
         <v>12</v>
       </c>
-      <c r="G7" s="14" t="s">
+      <c r="G7" s="5" t="s">
         <v>116</v>
       </c>
-      <c r="H7" s="14" t="s">
+      <c r="H7" s="5" t="s">
         <v>119</v>
       </c>
       <c r="I7" s="2"/>
-      <c r="J7" s="14" t="s">
+      <c r="J7" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="K7" s="14">
+      <c r="K7" s="5">
         <v>4</v>
       </c>
       <c r="L7" s="2" t="s">
         <v>107</v>
       </c>
-      <c r="M7" s="14" t="s">
+      <c r="M7" s="5" t="s">
         <v>118</v>
       </c>
-      <c r="N7" s="14" t="s">
+      <c r="N7" s="5" t="s">
         <v>118</v>
       </c>
-      <c r="O7" s="9" t="s">
+      <c r="O7" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="P7" s="9" t="s">
+      <c r="P7" s="7" t="s">
         <v>15</v>
       </c>
-      <c r="Q7" s="9" t="s">
+      <c r="Q7" s="7" t="s">
         <v>15</v>
       </c>
       <c r="R7" s="2" t="s">
         <v>108</v>
       </c>
-      <c r="S7" s="12" t="s">
+      <c r="S7" s="10" t="s">
         <v>109</v>
       </c>
     </row>
@@ -3803,32 +4487,32 @@
       <c r="A8" s="2" t="s">
         <v>120</v>
       </c>
-      <c r="B8" s="14">
+      <c r="B8" s="5">
         <v>0</v>
       </c>
       <c r="C8" s="2" t="s">
         <v>120</v>
       </c>
-      <c r="D8" s="14" t="s">
+      <c r="D8" s="5" t="s">
         <v>14</v>
       </c>
       <c r="E8" s="2" t="s">
         <v>121</v>
       </c>
-      <c r="F8" s="14">
+      <c r="F8" s="5">
         <v>5</v>
       </c>
-      <c r="G8" s="14" t="s">
+      <c r="G8" s="5" t="s">
         <v>122</v>
       </c>
       <c r="H8" s="2"/>
       <c r="I8" s="2">
         <v>95</v>
       </c>
-      <c r="J8" s="14" t="s">
+      <c r="J8" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="K8" s="14">
+      <c r="K8" s="5">
         <v>1</v>
       </c>
       <c r="L8" s="2" t="s">
@@ -3840,76 +4524,76 @@
       <c r="N8" s="2" t="s">
         <v>120</v>
       </c>
-      <c r="O8" s="9" t="s">
+      <c r="O8" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="P8" s="9" t="s">
+      <c r="P8" s="7" t="s">
         <v>15</v>
       </c>
-      <c r="Q8" s="9" t="s">
+      <c r="Q8" s="7" t="s">
         <v>15</v>
       </c>
       <c r="R8" s="2" t="s">
         <v>108</v>
       </c>
-      <c r="S8" s="12" t="s">
+      <c r="S8" s="10" t="s">
         <v>109</v>
       </c>
     </row>
     <row r="9" spans="1:19">
-      <c r="A9" s="14" t="s">
+      <c r="A9" s="5" t="s">
         <v>123</v>
       </c>
-      <c r="B9" s="14">
+      <c r="B9" s="5">
         <v>0</v>
       </c>
       <c r="C9" s="2" t="s">
         <v>123</v>
       </c>
-      <c r="D9" s="14" t="s">
+      <c r="D9" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="E9" s="14" t="s">
+      <c r="E9" s="5" t="s">
         <v>40</v>
       </c>
-      <c r="F9" s="14">
+      <c r="F9" s="5">
         <v>12</v>
       </c>
-      <c r="G9" s="14" t="s">
+      <c r="G9" s="5" t="s">
         <v>122</v>
       </c>
       <c r="H9" s="2"/>
       <c r="I9" s="2">
         <v>97</v>
       </c>
-      <c r="J9" s="14" t="s">
+      <c r="J9" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="K9" s="14">
+      <c r="K9" s="5">
         <v>4</v>
       </c>
       <c r="L9" s="2" t="s">
         <v>107</v>
       </c>
-      <c r="M9" s="14" t="s">
+      <c r="M9" s="5" t="s">
         <v>123</v>
       </c>
-      <c r="N9" s="14" t="s">
+      <c r="N9" s="5" t="s">
         <v>123</v>
       </c>
-      <c r="O9" s="9" t="s">
+      <c r="O9" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="P9" s="9" t="s">
+      <c r="P9" s="7" t="s">
         <v>15</v>
       </c>
-      <c r="Q9" s="9" t="s">
+      <c r="Q9" s="7" t="s">
         <v>15</v>
       </c>
       <c r="R9" s="2" t="s">
         <v>108</v>
       </c>
-      <c r="S9" s="12" t="s">
+      <c r="S9" s="10" t="s">
         <v>109</v>
       </c>
     </row>
@@ -4025,5 +4709,6 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <headerFooter/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Added BOM E2E Scenario and GRN Test Scenarios
Added BOM E2E Scenario and GRN, MRV and QC documents Test Scenarios
</commit_message>
<xml_diff>
--- a/testdata/ItemDetails.xlsx
+++ b/testdata/ItemDetails.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="23040" windowHeight="9120" firstSheet="7" activeTab="13"/>
+    <workbookView windowWidth="19200" windowHeight="6920" activeTab="7"/>
   </bookViews>
   <sheets>
     <sheet name="PR Details" sheetId="1" r:id="rId1"/>
@@ -870,7 +870,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="36">
+  <fills count="35">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1071,12 +1071,6 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor theme="9" tint="0.399975585192419"/>
         <bgColor indexed="64"/>
       </patternFill>
@@ -1346,10 +1340,10 @@
     <xf numFmtId="0" fontId="28" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="28" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="35" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="28" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0">
@@ -1974,16 +1968,16 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1:J20"/>
-  <sheetFormatPr defaultColWidth="8.71296296296296" defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultColWidth="8.70909090909091" defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="20.712962962963" customWidth="1"/>
-    <col min="2" max="3" width="12.712962962963" customWidth="1"/>
-    <col min="4" max="4" width="14.712962962963" customWidth="1"/>
-    <col min="5" max="5" width="9.85185185185185" customWidth="1"/>
-    <col min="6" max="6" width="14.1388888888889" customWidth="1"/>
-    <col min="7" max="7" width="14.8518518518519" customWidth="1"/>
-    <col min="8" max="8" width="22.287037037037" customWidth="1"/>
-    <col min="9" max="9" width="14.4259259259259" customWidth="1"/>
+    <col min="1" max="1" width="20.7090909090909" customWidth="1"/>
+    <col min="2" max="3" width="12.7090909090909" customWidth="1"/>
+    <col min="4" max="4" width="14.7090909090909" customWidth="1"/>
+    <col min="5" max="5" width="9.85454545454546" customWidth="1"/>
+    <col min="6" max="6" width="14.1363636363636" customWidth="1"/>
+    <col min="7" max="7" width="14.8545454545455" customWidth="1"/>
+    <col min="8" max="8" width="22.2909090909091" customWidth="1"/>
+    <col min="9" max="9" width="14.4272727272727" customWidth="1"/>
     <col min="10" max="10" width="13" customWidth="1"/>
   </cols>
   <sheetData>
@@ -2019,7 +2013,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="2" s="23" customFormat="1" ht="20.4" spans="1:10">
+    <row r="2" s="23" customFormat="1" ht="21" spans="1:10">
       <c r="A2" s="25" t="s">
         <v>10</v>
       </c>
@@ -2317,19 +2311,19 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1:K3"/>
-  <sheetFormatPr defaultColWidth="8.85185185185185" defaultRowHeight="14.4" outlineLevelRow="2"/>
+  <sheetFormatPr defaultColWidth="8.85454545454546" defaultRowHeight="14.5" outlineLevelRow="2"/>
   <cols>
     <col min="1" max="1" width="9" customWidth="1"/>
-    <col min="2" max="2" width="25.712962962963" customWidth="1"/>
-    <col min="3" max="3" width="12.4259259259259" customWidth="1"/>
-    <col min="4" max="4" width="16.287037037037" customWidth="1"/>
-    <col min="5" max="5" width="20.287037037037" customWidth="1"/>
-    <col min="6" max="6" width="25.712962962963" customWidth="1"/>
-    <col min="7" max="7" width="12.287037037037" customWidth="1"/>
-    <col min="8" max="8" width="14.5740740740741" customWidth="1"/>
-    <col min="9" max="9" width="28.5740740740741" customWidth="1"/>
+    <col min="2" max="2" width="25.7090909090909" customWidth="1"/>
+    <col min="3" max="3" width="12.4272727272727" customWidth="1"/>
+    <col min="4" max="4" width="16.2909090909091" customWidth="1"/>
+    <col min="5" max="5" width="20.2909090909091" customWidth="1"/>
+    <col min="6" max="6" width="25.7090909090909" customWidth="1"/>
+    <col min="7" max="7" width="12.2909090909091" customWidth="1"/>
+    <col min="8" max="8" width="14.5727272727273" customWidth="1"/>
+    <col min="9" max="9" width="28.5727272727273" customWidth="1"/>
     <col min="10" max="10" width="23" customWidth="1"/>
-    <col min="11" max="11" width="14.712962962963" customWidth="1"/>
+    <col min="11" max="11" width="14.7090909090909" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:11">
@@ -2447,13 +2441,13 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1:E4"/>
-  <sheetFormatPr defaultColWidth="8.85185185185185" defaultRowHeight="14.4" outlineLevelRow="3" outlineLevelCol="4"/>
+  <sheetFormatPr defaultColWidth="8.85454545454546" defaultRowHeight="14.5" outlineLevelRow="3" outlineLevelCol="4"/>
   <cols>
-    <col min="1" max="1" width="13.5740740740741" customWidth="1"/>
+    <col min="1" max="1" width="13.5727272727273" customWidth="1"/>
     <col min="2" max="2" width="6" customWidth="1"/>
-    <col min="3" max="3" width="14.4259259259259" customWidth="1"/>
-    <col min="4" max="4" width="18.1388888888889" customWidth="1"/>
-    <col min="5" max="5" width="19.5740740740741" customWidth="1"/>
+    <col min="3" max="3" width="14.4272727272727" customWidth="1"/>
+    <col min="4" max="4" width="18.1363636363636" customWidth="1"/>
+    <col min="5" max="5" width="19.5727272727273" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5">
@@ -2534,15 +2528,15 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1:G11"/>
-  <sheetFormatPr defaultColWidth="8.85185185185185" defaultRowHeight="14.4" outlineLevelCol="6"/>
+  <sheetFormatPr defaultColWidth="8.85454545454546" defaultRowHeight="14.5" outlineLevelCol="6"/>
   <cols>
-    <col min="1" max="1" width="25.712962962963" customWidth="1"/>
-    <col min="2" max="2" width="8.85185185185185" customWidth="1"/>
-    <col min="3" max="3" width="12.287037037037" customWidth="1"/>
-    <col min="4" max="4" width="7.13888888888889" customWidth="1"/>
-    <col min="5" max="5" width="5.28703703703704" customWidth="1"/>
-    <col min="6" max="6" width="17.4259259259259" customWidth="1"/>
-    <col min="7" max="7" width="12.4259259259259" customWidth="1"/>
+    <col min="1" max="1" width="25.7090909090909" customWidth="1"/>
+    <col min="2" max="2" width="8.85454545454546" customWidth="1"/>
+    <col min="3" max="3" width="12.2909090909091" customWidth="1"/>
+    <col min="4" max="4" width="7.13636363636364" customWidth="1"/>
+    <col min="5" max="5" width="5.29090909090909" customWidth="1"/>
+    <col min="6" max="6" width="17.4272727272727" customWidth="1"/>
+    <col min="7" max="7" width="12.4272727272727" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7">
@@ -2808,11 +2802,11 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1:C3"/>
-  <sheetFormatPr defaultColWidth="8.85185185185185" defaultRowHeight="14.4" outlineLevelRow="2" outlineLevelCol="2"/>
+  <sheetFormatPr defaultColWidth="8.85454545454546" defaultRowHeight="14.5" outlineLevelRow="2" outlineLevelCol="2"/>
   <cols>
-    <col min="1" max="1" width="25.5740740740741" customWidth="1"/>
-    <col min="2" max="2" width="15.1388888888889" customWidth="1"/>
-    <col min="3" max="3" width="16.4259259259259" customWidth="1"/>
+    <col min="1" max="1" width="25.5727272727273" customWidth="1"/>
+    <col min="2" max="2" width="15.1363636363636" customWidth="1"/>
+    <col min="3" max="3" width="16.4272727272727" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3">
@@ -2858,10 +2852,10 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1:C3"/>
-  <sheetFormatPr defaultColWidth="8.88888888888889" defaultRowHeight="14.4" outlineLevelRow="2" outlineLevelCol="2"/>
+  <sheetFormatPr defaultColWidth="8.89090909090909" defaultRowHeight="14.5" outlineLevelRow="2" outlineLevelCol="2"/>
   <cols>
-    <col min="1" max="1" width="21.4444444444444" customWidth="1"/>
-    <col min="2" max="2" width="11.5555555555556" customWidth="1"/>
+    <col min="1" max="1" width="21.4454545454545" customWidth="1"/>
+    <col min="2" max="2" width="11.5545454545455" customWidth="1"/>
     <col min="3" max="3" width="9" customWidth="1"/>
   </cols>
   <sheetData>
@@ -2908,28 +2902,28 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1:T10"/>
-  <sheetFormatPr defaultColWidth="8.71296296296296" defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultColWidth="8.70909090909091" defaultRowHeight="14.5"/>
   <cols>
     <col min="1" max="1" width="30" customWidth="1"/>
-    <col min="2" max="2" width="36.4259259259259" customWidth="1"/>
+    <col min="2" max="2" width="36.4272727272727" customWidth="1"/>
     <col min="3" max="3" width="6" customWidth="1"/>
-    <col min="4" max="4" width="13.712962962963" customWidth="1"/>
-    <col min="5" max="5" width="5.28703703703704" customWidth="1"/>
-    <col min="6" max="6" width="17.287037037037" customWidth="1"/>
-    <col min="7" max="7" width="30.287037037037" customWidth="1"/>
-    <col min="8" max="8" width="26.8518518518519" customWidth="1"/>
-    <col min="9" max="9" width="17.287037037037" customWidth="1"/>
-    <col min="10" max="10" width="13.287037037037" customWidth="1"/>
-    <col min="11" max="11" width="22.712962962963" customWidth="1"/>
-    <col min="12" max="12" width="12.712962962963" customWidth="1"/>
-    <col min="13" max="13" width="29.5740740740741" customWidth="1"/>
-    <col min="14" max="14" width="18.287037037037" customWidth="1"/>
-    <col min="15" max="15" width="16.287037037037" customWidth="1"/>
-    <col min="16" max="16" width="15.5740740740741" customWidth="1"/>
-    <col min="17" max="17" width="17.712962962963" customWidth="1"/>
-    <col min="18" max="18" width="24.1388888888889" customWidth="1"/>
-    <col min="19" max="19" width="13.4259259259259" customWidth="1"/>
-    <col min="20" max="20" width="13.5740740740741" customWidth="1"/>
+    <col min="4" max="4" width="13.7090909090909" customWidth="1"/>
+    <col min="5" max="5" width="5.29090909090909" customWidth="1"/>
+    <col min="6" max="6" width="17.2909090909091" customWidth="1"/>
+    <col min="7" max="7" width="30.2909090909091" customWidth="1"/>
+    <col min="8" max="8" width="26.8545454545455" customWidth="1"/>
+    <col min="9" max="9" width="17.2909090909091" customWidth="1"/>
+    <col min="10" max="10" width="13.2909090909091" customWidth="1"/>
+    <col min="11" max="11" width="22.7090909090909" customWidth="1"/>
+    <col min="12" max="12" width="12.7090909090909" customWidth="1"/>
+    <col min="13" max="13" width="29.5727272727273" customWidth="1"/>
+    <col min="14" max="14" width="18.2909090909091" customWidth="1"/>
+    <col min="15" max="15" width="16.2909090909091" customWidth="1"/>
+    <col min="16" max="16" width="15.5727272727273" customWidth="1"/>
+    <col min="17" max="17" width="17.7090909090909" customWidth="1"/>
+    <col min="18" max="18" width="24.1363636363636" customWidth="1"/>
+    <col min="19" max="19" width="13.4272727272727" customWidth="1"/>
+    <col min="20" max="20" width="13.5727272727273" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:20">
@@ -3490,19 +3484,19 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1:R3"/>
-  <sheetFormatPr defaultColWidth="8.85185185185185" defaultRowHeight="14.4" outlineLevelRow="2"/>
+  <sheetFormatPr defaultColWidth="8.85454545454546" defaultRowHeight="14.5" outlineLevelRow="2"/>
   <cols>
     <col min="1" max="2" width="21" customWidth="1"/>
     <col min="3" max="3" width="6" customWidth="1"/>
-    <col min="4" max="4" width="12.712962962963" customWidth="1"/>
-    <col min="5" max="5" width="19.4259259259259" customWidth="1"/>
-    <col min="6" max="6" width="15.1388888888889" customWidth="1"/>
-    <col min="7" max="7" width="15.4259259259259" customWidth="1"/>
-    <col min="8" max="8" width="19.5740740740741" customWidth="1"/>
-    <col min="9" max="9" width="10.8518518518519" customWidth="1"/>
-    <col min="10" max="10" width="17.5740740740741" customWidth="1"/>
-    <col min="11" max="11" width="11.287037037037" customWidth="1"/>
-    <col min="12" max="12" width="21.712962962963" customWidth="1"/>
+    <col min="4" max="4" width="12.7090909090909" customWidth="1"/>
+    <col min="5" max="5" width="19.4272727272727" customWidth="1"/>
+    <col min="6" max="6" width="15.1363636363636" customWidth="1"/>
+    <col min="7" max="7" width="15.4272727272727" customWidth="1"/>
+    <col min="8" max="8" width="19.5727272727273" customWidth="1"/>
+    <col min="9" max="9" width="10.8545454545455" customWidth="1"/>
+    <col min="10" max="10" width="17.5727272727273" customWidth="1"/>
+    <col min="11" max="11" width="11.2909090909091" customWidth="1"/>
+    <col min="12" max="12" width="21.7090909090909" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:18">
@@ -3641,14 +3635,14 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1:F3"/>
-  <sheetFormatPr defaultColWidth="8.85185185185185" defaultRowHeight="14.4" outlineLevelRow="2" outlineLevelCol="5"/>
+  <sheetFormatPr defaultColWidth="8.85454545454546" defaultRowHeight="14.5" outlineLevelRow="2" outlineLevelCol="5"/>
   <cols>
-    <col min="1" max="1" width="27.1388888888889" customWidth="1"/>
-    <col min="2" max="2" width="10.4259259259259" customWidth="1"/>
-    <col min="3" max="3" width="11.4259259259259" customWidth="1"/>
-    <col min="4" max="4" width="11.712962962963" customWidth="1"/>
-    <col min="5" max="5" width="14.5740740740741" customWidth="1"/>
-    <col min="6" max="6" width="17.712962962963" customWidth="1"/>
+    <col min="1" max="1" width="27.1363636363636" customWidth="1"/>
+    <col min="2" max="2" width="10.4272727272727" customWidth="1"/>
+    <col min="3" max="3" width="11.4272727272727" customWidth="1"/>
+    <col min="4" max="4" width="11.7090909090909" customWidth="1"/>
+    <col min="5" max="5" width="14.5727272727273" customWidth="1"/>
+    <col min="6" max="6" width="17.7090909090909" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6">
@@ -3676,7 +3670,7 @@
         <v>59</v>
       </c>
       <c r="B2" s="2">
-        <v>50</v>
+        <v>2</v>
       </c>
       <c r="C2" s="2">
         <v>70</v>
@@ -3719,14 +3713,14 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1:F4"/>
-  <sheetFormatPr defaultColWidth="8.85185185185185" defaultRowHeight="14.4" outlineLevelRow="3" outlineLevelCol="5"/>
+  <sheetFormatPr defaultColWidth="8.85454545454546" defaultRowHeight="14.5" outlineLevelRow="3" outlineLevelCol="5"/>
   <cols>
-    <col min="1" max="1" width="27.1388888888889" customWidth="1"/>
-    <col min="2" max="2" width="10.4259259259259" customWidth="1"/>
-    <col min="3" max="3" width="11.4259259259259" customWidth="1"/>
-    <col min="4" max="4" width="11.712962962963" customWidth="1"/>
-    <col min="5" max="5" width="14.5740740740741" customWidth="1"/>
-    <col min="6" max="6" width="17.712962962963" customWidth="1"/>
+    <col min="1" max="1" width="27.1363636363636" customWidth="1"/>
+    <col min="2" max="2" width="10.4272727272727" customWidth="1"/>
+    <col min="3" max="3" width="11.4272727272727" customWidth="1"/>
+    <col min="4" max="4" width="11.7090909090909" customWidth="1"/>
+    <col min="5" max="5" width="14.5727272727273" customWidth="1"/>
+    <col min="6" max="6" width="17.7090909090909" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6">
@@ -3754,7 +3748,7 @@
         <v>59</v>
       </c>
       <c r="B2" s="2">
-        <v>150</v>
+        <v>2</v>
       </c>
       <c r="C2" s="2">
         <v>45</v>
@@ -3815,9 +3809,9 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1:C3"/>
-  <sheetFormatPr defaultColWidth="8.85185185185185" defaultRowHeight="14.4" outlineLevelRow="2" outlineLevelCol="2"/>
+  <sheetFormatPr defaultColWidth="8.85454545454546" defaultRowHeight="14.5" outlineLevelRow="2" outlineLevelCol="2"/>
   <cols>
-    <col min="1" max="1" width="28.712962962963" customWidth="1"/>
+    <col min="1" max="1" width="28.7090909090909" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3">
@@ -3863,15 +3857,15 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1:G4"/>
-  <sheetFormatPr defaultColWidth="8.85185185185185" defaultRowHeight="14.4" outlineLevelRow="3" outlineLevelCol="6"/>
+  <sheetFormatPr defaultColWidth="8.85454545454546" defaultRowHeight="14.5" outlineLevelRow="3" outlineLevelCol="6"/>
   <cols>
-    <col min="1" max="1" width="19.712962962963" customWidth="1"/>
-    <col min="2" max="2" width="8.13888888888889" customWidth="1"/>
-    <col min="3" max="3" width="8.57407407407407" customWidth="1"/>
-    <col min="4" max="4" width="17.8518518518519" customWidth="1"/>
-    <col min="5" max="5" width="12.712962962963" customWidth="1"/>
-    <col min="6" max="6" width="14.5740740740741" customWidth="1"/>
-    <col min="7" max="7" width="17.712962962963" customWidth="1"/>
+    <col min="1" max="1" width="19.7090909090909" customWidth="1"/>
+    <col min="2" max="2" width="8.13636363636364" customWidth="1"/>
+    <col min="3" max="3" width="8.57272727272727" customWidth="1"/>
+    <col min="4" max="4" width="17.8545454545455" customWidth="1"/>
+    <col min="5" max="5" width="12.7090909090909" customWidth="1"/>
+    <col min="6" max="6" width="14.5727272727273" customWidth="1"/>
+    <col min="7" max="7" width="17.7090909090909" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7">
@@ -3902,7 +3896,7 @@
         <v>86</v>
       </c>
       <c r="B2" s="12">
-        <v>524</v>
+        <v>2</v>
       </c>
       <c r="C2" s="12">
         <v>524</v>
@@ -3970,15 +3964,15 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1:G4"/>
-  <sheetFormatPr defaultColWidth="8.85185185185185" defaultRowHeight="14.4" outlineLevelRow="3" outlineLevelCol="6"/>
+  <sheetFormatPr defaultColWidth="8.85454545454546" defaultRowHeight="14.5" outlineLevelRow="3" outlineLevelCol="6"/>
   <cols>
-    <col min="1" max="1" width="19.712962962963" customWidth="1"/>
-    <col min="2" max="2" width="8.13888888888889" customWidth="1"/>
-    <col min="3" max="3" width="8.57407407407407" customWidth="1"/>
-    <col min="4" max="4" width="17.8518518518519" customWidth="1"/>
-    <col min="5" max="5" width="12.712962962963" customWidth="1"/>
-    <col min="6" max="6" width="14.5740740740741" customWidth="1"/>
-    <col min="7" max="7" width="17.712962962963" customWidth="1"/>
+    <col min="1" max="1" width="19.7090909090909" customWidth="1"/>
+    <col min="2" max="2" width="8.13636363636364" customWidth="1"/>
+    <col min="3" max="3" width="8.57272727272727" customWidth="1"/>
+    <col min="4" max="4" width="17.8545454545455" customWidth="1"/>
+    <col min="5" max="5" width="12.7090909090909" customWidth="1"/>
+    <col min="6" max="6" width="14.5727272727273" customWidth="1"/>
+    <col min="7" max="7" width="17.7090909090909" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7">
@@ -4009,7 +4003,7 @@
         <v>86</v>
       </c>
       <c r="B2" s="12">
-        <v>22</v>
+        <v>2</v>
       </c>
       <c r="C2" s="12">
         <v>524</v>
@@ -4077,25 +4071,25 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1:S11"/>
-  <sheetFormatPr defaultColWidth="8.85185185185185" defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultColWidth="8.85454545454546" defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="39.712962962963" customWidth="1"/>
-    <col min="2" max="2" width="10.1388888888889" customWidth="1"/>
-    <col min="3" max="3" width="39.712962962963" customWidth="1"/>
+    <col min="1" max="1" width="39.7090909090909" customWidth="1"/>
+    <col min="2" max="2" width="10.1363636363636" customWidth="1"/>
+    <col min="3" max="3" width="39.7090909090909" customWidth="1"/>
     <col min="4" max="4" width="11" customWidth="1"/>
-    <col min="5" max="5" width="13.287037037037" customWidth="1"/>
-    <col min="6" max="6" width="8.85185185185185" customWidth="1"/>
-    <col min="7" max="7" width="17.8518518518519" customWidth="1"/>
-    <col min="8" max="8" width="19.5740740740741" customWidth="1"/>
-    <col min="9" max="9" width="23.712962962963" customWidth="1"/>
-    <col min="10" max="10" width="12.712962962963" customWidth="1"/>
-    <col min="11" max="11" width="11.8518518518519" customWidth="1"/>
-    <col min="12" max="12" width="17.4259259259259" customWidth="1"/>
-    <col min="13" max="14" width="39.712962962963" customWidth="1"/>
-    <col min="15" max="15" width="25.712962962963" customWidth="1"/>
-    <col min="16" max="17" width="16.5740740740741" customWidth="1"/>
-    <col min="18" max="18" width="11.5740740740741" customWidth="1"/>
-    <col min="19" max="19" width="14.8518518518519" customWidth="1"/>
+    <col min="5" max="5" width="13.2909090909091" customWidth="1"/>
+    <col min="6" max="6" width="8.85454545454546" customWidth="1"/>
+    <col min="7" max="7" width="17.8545454545455" customWidth="1"/>
+    <col min="8" max="8" width="19.5727272727273" customWidth="1"/>
+    <col min="9" max="9" width="23.7090909090909" customWidth="1"/>
+    <col min="10" max="10" width="12.7090909090909" customWidth="1"/>
+    <col min="11" max="11" width="11.8545454545455" customWidth="1"/>
+    <col min="12" max="12" width="17.4272727272727" customWidth="1"/>
+    <col min="13" max="14" width="39.7090909090909" customWidth="1"/>
+    <col min="15" max="15" width="25.7090909090909" customWidth="1"/>
+    <col min="16" max="17" width="16.5727272727273" customWidth="1"/>
+    <col min="18" max="18" width="11.5727272727273" customWidth="1"/>
+    <col min="19" max="19" width="14.8545454545455" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:19">

</xml_diff>

<commit_message>
Updated Item Details for GRN Scenario
Updated Item Details for GRN Scenario
</commit_message>
<xml_diff>
--- a/testdata/ItemDetails.xlsx
+++ b/testdata/ItemDetails.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="19200" windowHeight="6920" activeTab="7"/>
+    <workbookView windowWidth="19200" windowHeight="6920" firstSheet="16" activeTab="19"/>
   </bookViews>
   <sheets>
     <sheet name="PR Details" sheetId="1" r:id="rId1"/>
@@ -21,6 +21,12 @@
     <sheet name="SI Details" sheetId="12" r:id="rId12"/>
     <sheet name="MRTOMRV Data" sheetId="13" r:id="rId13"/>
     <sheet name="MRTOMRVWip Data" sheetId="14" r:id="rId14"/>
+    <sheet name="RateContract_SER" sheetId="15" r:id="rId15"/>
+    <sheet name="PricelistItem" sheetId="16" r:id="rId16"/>
+    <sheet name="ST_ITEM_RATECONTRACT" sheetId="17" r:id="rId17"/>
+    <sheet name="ServiceItemPriceList" sheetId="18" r:id="rId18"/>
+    <sheet name="ST_Item_PriceList" sheetId="19" r:id="rId19"/>
+    <sheet name="DIS_UOM_GEN_UD" sheetId="20" r:id="rId20"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -40,7 +46,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="556" uniqueCount="202">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="599" uniqueCount="216">
   <si>
     <t>ITEM_NAME</t>
   </si>
@@ -647,6 +653,48 @@
   </si>
   <si>
     <t>GWL_ITEM_STOCK_07</t>
+  </si>
+  <si>
+    <t>RateContrac_Ser_tItem</t>
+  </si>
+  <si>
+    <t>PK-SERV-MAC-NA-01</t>
+  </si>
+  <si>
+    <t>PricelistItem</t>
+  </si>
+  <si>
+    <t>TVS-RM-KDK-26</t>
+  </si>
+  <si>
+    <t>TVS-RM-KDK-25</t>
+  </si>
+  <si>
+    <t>TVS-SIM-257793</t>
+  </si>
+  <si>
+    <t>TVS-SIM-395809</t>
+  </si>
+  <si>
+    <t>PriceList_Ser_tItem</t>
+  </si>
+  <si>
+    <t>TVS-SER-10005</t>
+  </si>
+  <si>
+    <t>TVS-SIM-599803</t>
+  </si>
+  <si>
+    <t>TVS-SIM-050035</t>
+  </si>
+  <si>
+    <t>TVS-RM-KPK-01</t>
+  </si>
+  <si>
+    <t>RMLG</t>
+  </si>
+  <si>
+    <t>TVS-KPK-NA-DIS-10001</t>
   </si>
 </sst>
 </file>
@@ -659,13 +707,32 @@
     <numFmt numFmtId="178" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
     <numFmt numFmtId="179" formatCode="_ &quot;₹&quot;* #,##0_ ;_ &quot;₹&quot;* \-#,##0_ ;_ &quot;₹&quot;* &quot;-&quot;_ ;_ @_ "/>
   </numFmts>
-  <fonts count="29">
+  <fonts count="32">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <charset val="134"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Times New Roman"/>
+      <charset val="134"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
+      <charset val="134"/>
     </font>
     <font>
       <b/>
@@ -1198,7 +1265,7 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="50">
+  <cellStyleXfs count="51">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
@@ -1217,149 +1284,182 @@
     <xf numFmtId="179" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="2" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="17" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="6" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="7" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="7" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="8" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="6" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="7" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="7" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="8" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
   </cellStyleXfs>
-  <cellXfs count="28">
+  <cellXfs count="35">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="50" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="49" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="50" applyFont="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="50" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
@@ -1369,13 +1469,10 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1385,56 +1482,50 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="6" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="49" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="49" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="49" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="49" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="justify" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1">
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
-  <cellStyles count="50">
+  <cellStyles count="51">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Comma" xfId="1" builtinId="3"/>
     <cellStyle name="Currency" xfId="2" builtinId="4"/>
@@ -1485,6 +1576,7 @@
     <cellStyle name="40% - Accent6" xfId="47" builtinId="51"/>
     <cellStyle name="60% - Accent6" xfId="48" builtinId="52"/>
     <cellStyle name="Normal 2" xfId="49"/>
+    <cellStyle name="Normal 3" xfId="50"/>
   </cellStyles>
   <dxfs count="17">
     <dxf>
@@ -1982,324 +2074,324 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10">
-      <c r="A1" s="24" t="s">
+      <c r="A1" s="31" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="24" t="s">
+      <c r="B1" s="31" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="24" t="s">
+      <c r="C1" s="31" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="24" t="s">
+      <c r="D1" s="31" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="24" t="s">
+      <c r="E1" s="31" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="24" t="s">
+      <c r="F1" s="31" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="24" t="s">
+      <c r="G1" s="31" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="24" t="s">
+      <c r="H1" s="31" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="24" t="s">
+      <c r="I1" s="31" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="24" t="s">
+      <c r="J1" s="31" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="2" s="23" customFormat="1" ht="21" spans="1:10">
-      <c r="A2" s="25" t="s">
+    <row r="2" s="30" customFormat="1" ht="21" spans="1:10">
+      <c r="A2" s="32" t="s">
         <v>10</v>
       </c>
-      <c r="B2" s="26" t="s">
+      <c r="B2" s="33" t="s">
         <v>11</v>
       </c>
-      <c r="C2" s="26" t="s">
+      <c r="C2" s="33" t="s">
         <v>12</v>
       </c>
-      <c r="D2" s="25" t="s">
+      <c r="D2" s="32" t="s">
         <v>13</v>
       </c>
-      <c r="E2" s="25">
+      <c r="E2" s="32">
         <v>1</v>
       </c>
-      <c r="F2" s="25" t="s">
+      <c r="F2" s="32" t="s">
         <v>14</v>
       </c>
-      <c r="G2" s="25">
+      <c r="G2" s="32">
         <v>1010301033</v>
       </c>
-      <c r="H2" s="25" t="s">
+      <c r="H2" s="32" t="s">
         <v>15</v>
       </c>
-      <c r="I2" s="25" t="s">
+      <c r="I2" s="32" t="s">
         <v>16</v>
       </c>
-      <c r="J2" s="25" t="s">
+      <c r="J2" s="32" t="s">
         <v>17</v>
       </c>
     </row>
     <row r="3" ht="15" customHeight="1" spans="1:10">
-      <c r="A3" s="25" t="s">
+      <c r="A3" s="32" t="s">
         <v>18</v>
       </c>
-      <c r="B3" s="26" t="s">
+      <c r="B3" s="33" t="s">
         <v>11</v>
       </c>
-      <c r="C3" s="26" t="s">
+      <c r="C3" s="33" t="s">
         <v>12</v>
       </c>
-      <c r="D3" s="25" t="s">
+      <c r="D3" s="32" t="s">
         <v>19</v>
       </c>
-      <c r="E3" s="25">
+      <c r="E3" s="32">
         <v>6</v>
       </c>
-      <c r="F3" s="26" t="s">
+      <c r="F3" s="33" t="s">
         <v>20</v>
       </c>
-      <c r="G3" s="25">
+      <c r="G3" s="32">
         <v>1010301033</v>
       </c>
-      <c r="H3" s="25" t="s">
+      <c r="H3" s="32" t="s">
         <v>15</v>
       </c>
-      <c r="I3" s="25" t="s">
+      <c r="I3" s="32" t="s">
         <v>16</v>
       </c>
-      <c r="J3" s="25" t="s">
+      <c r="J3" s="32" t="s">
         <v>17</v>
       </c>
     </row>
     <row r="4" spans="1:10">
-      <c r="A4" s="25" t="s">
+      <c r="A4" s="32" t="s">
         <v>21</v>
       </c>
-      <c r="B4" s="26" t="s">
+      <c r="B4" s="33" t="s">
         <v>22</v>
       </c>
-      <c r="C4" s="26" t="s">
+      <c r="C4" s="33" t="s">
         <v>22</v>
       </c>
-      <c r="D4" s="25" t="s">
+      <c r="D4" s="32" t="s">
         <v>23</v>
       </c>
-      <c r="E4" s="25">
+      <c r="E4" s="32">
         <v>1</v>
       </c>
-      <c r="F4" s="26" t="s">
+      <c r="F4" s="33" t="s">
         <v>14</v>
       </c>
-      <c r="G4" s="25">
+      <c r="G4" s="32">
         <v>5010100004</v>
       </c>
-      <c r="H4" s="25" t="s">
+      <c r="H4" s="32" t="s">
         <v>24</v>
       </c>
-      <c r="I4" s="25" t="s">
+      <c r="I4" s="32" t="s">
         <v>16</v>
       </c>
-      <c r="J4" s="25" t="s">
+      <c r="J4" s="32" t="s">
         <v>17</v>
       </c>
     </row>
     <row r="5" spans="1:10">
-      <c r="A5" s="27"/>
-      <c r="B5" s="27"/>
-      <c r="C5" s="27"/>
-      <c r="D5" s="27"/>
-      <c r="E5" s="27"/>
-      <c r="F5" s="27"/>
-      <c r="G5" s="27"/>
-      <c r="H5" s="27"/>
-      <c r="I5" s="27"/>
-      <c r="J5" s="27"/>
+      <c r="A5" s="34"/>
+      <c r="B5" s="34"/>
+      <c r="C5" s="34"/>
+      <c r="D5" s="34"/>
+      <c r="E5" s="34"/>
+      <c r="F5" s="34"/>
+      <c r="G5" s="34"/>
+      <c r="H5" s="34"/>
+      <c r="I5" s="34"/>
+      <c r="J5" s="34"/>
     </row>
     <row r="6" spans="1:10">
-      <c r="A6" s="27"/>
-      <c r="B6" s="27"/>
-      <c r="C6" s="27"/>
-      <c r="D6" s="27"/>
-      <c r="E6" s="27"/>
-      <c r="F6" s="27"/>
-      <c r="G6" s="27"/>
-      <c r="H6" s="27"/>
-      <c r="I6" s="27"/>
-      <c r="J6" s="27"/>
+      <c r="A6" s="34"/>
+      <c r="B6" s="34"/>
+      <c r="C6" s="34"/>
+      <c r="D6" s="34"/>
+      <c r="E6" s="34"/>
+      <c r="F6" s="34"/>
+      <c r="G6" s="34"/>
+      <c r="H6" s="34"/>
+      <c r="I6" s="34"/>
+      <c r="J6" s="34"/>
     </row>
     <row r="7" spans="1:10">
-      <c r="A7" s="27"/>
-      <c r="B7" s="27"/>
-      <c r="C7" s="27"/>
-      <c r="D7" s="27"/>
-      <c r="E7" s="27"/>
-      <c r="F7" s="27"/>
-      <c r="G7" s="27"/>
-      <c r="H7" s="27"/>
-      <c r="I7" s="27"/>
-      <c r="J7" s="27"/>
+      <c r="A7" s="34"/>
+      <c r="B7" s="34"/>
+      <c r="C7" s="34"/>
+      <c r="D7" s="34"/>
+      <c r="E7" s="34"/>
+      <c r="F7" s="34"/>
+      <c r="G7" s="34"/>
+      <c r="H7" s="34"/>
+      <c r="I7" s="34"/>
+      <c r="J7" s="34"/>
     </row>
     <row r="8" spans="1:10">
-      <c r="A8" s="27"/>
-      <c r="B8" s="27"/>
-      <c r="C8" s="27"/>
-      <c r="D8" s="27"/>
-      <c r="E8" s="27"/>
-      <c r="F8" s="27"/>
-      <c r="G8" s="27"/>
-      <c r="H8" s="27"/>
-      <c r="I8" s="27"/>
-      <c r="J8" s="27"/>
+      <c r="A8" s="34"/>
+      <c r="B8" s="34"/>
+      <c r="C8" s="34"/>
+      <c r="D8" s="34"/>
+      <c r="E8" s="34"/>
+      <c r="F8" s="34"/>
+      <c r="G8" s="34"/>
+      <c r="H8" s="34"/>
+      <c r="I8" s="34"/>
+      <c r="J8" s="34"/>
     </row>
     <row r="9" spans="1:10">
-      <c r="A9" s="27"/>
-      <c r="B9" s="27"/>
-      <c r="C9" s="27"/>
-      <c r="D9" s="27"/>
-      <c r="E9" s="27"/>
-      <c r="F9" s="27"/>
-      <c r="G9" s="27"/>
-      <c r="H9" s="27"/>
-      <c r="I9" s="27"/>
-      <c r="J9" s="27"/>
+      <c r="A9" s="34"/>
+      <c r="B9" s="34"/>
+      <c r="C9" s="34"/>
+      <c r="D9" s="34"/>
+      <c r="E9" s="34"/>
+      <c r="F9" s="34"/>
+      <c r="G9" s="34"/>
+      <c r="H9" s="34"/>
+      <c r="I9" s="34"/>
+      <c r="J9" s="34"/>
     </row>
     <row r="10" spans="1:10">
-      <c r="A10" s="27"/>
-      <c r="B10" s="27"/>
-      <c r="C10" s="27"/>
-      <c r="D10" s="27"/>
-      <c r="E10" s="27"/>
-      <c r="F10" s="27"/>
-      <c r="G10" s="27"/>
-      <c r="H10" s="27"/>
-      <c r="I10" s="27"/>
-      <c r="J10" s="27"/>
+      <c r="A10" s="34"/>
+      <c r="B10" s="34"/>
+      <c r="C10" s="34"/>
+      <c r="D10" s="34"/>
+      <c r="E10" s="34"/>
+      <c r="F10" s="34"/>
+      <c r="G10" s="34"/>
+      <c r="H10" s="34"/>
+      <c r="I10" s="34"/>
+      <c r="J10" s="34"/>
     </row>
     <row r="11" spans="1:10">
-      <c r="A11" s="27"/>
-      <c r="B11" s="27"/>
-      <c r="C11" s="27"/>
-      <c r="D11" s="27"/>
-      <c r="E11" s="27"/>
-      <c r="F11" s="27"/>
-      <c r="G11" s="27"/>
-      <c r="H11" s="27"/>
-      <c r="I11" s="27"/>
-      <c r="J11" s="27"/>
+      <c r="A11" s="34"/>
+      <c r="B11" s="34"/>
+      <c r="C11" s="34"/>
+      <c r="D11" s="34"/>
+      <c r="E11" s="34"/>
+      <c r="F11" s="34"/>
+      <c r="G11" s="34"/>
+      <c r="H11" s="34"/>
+      <c r="I11" s="34"/>
+      <c r="J11" s="34"/>
     </row>
     <row r="12" spans="1:10">
-      <c r="A12" s="27"/>
-      <c r="B12" s="27"/>
-      <c r="C12" s="27"/>
-      <c r="D12" s="27"/>
-      <c r="E12" s="27"/>
-      <c r="F12" s="27"/>
-      <c r="G12" s="27"/>
-      <c r="H12" s="27"/>
-      <c r="I12" s="27"/>
-      <c r="J12" s="27"/>
+      <c r="A12" s="34"/>
+      <c r="B12" s="34"/>
+      <c r="C12" s="34"/>
+      <c r="D12" s="34"/>
+      <c r="E12" s="34"/>
+      <c r="F12" s="34"/>
+      <c r="G12" s="34"/>
+      <c r="H12" s="34"/>
+      <c r="I12" s="34"/>
+      <c r="J12" s="34"/>
     </row>
     <row r="13" spans="1:10">
-      <c r="A13" s="27"/>
-      <c r="B13" s="27"/>
-      <c r="C13" s="27"/>
-      <c r="D13" s="27"/>
-      <c r="E13" s="27"/>
-      <c r="F13" s="27"/>
-      <c r="G13" s="27"/>
-      <c r="H13" s="27"/>
-      <c r="I13" s="27"/>
-      <c r="J13" s="27"/>
+      <c r="A13" s="34"/>
+      <c r="B13" s="34"/>
+      <c r="C13" s="34"/>
+      <c r="D13" s="34"/>
+      <c r="E13" s="34"/>
+      <c r="F13" s="34"/>
+      <c r="G13" s="34"/>
+      <c r="H13" s="34"/>
+      <c r="I13" s="34"/>
+      <c r="J13" s="34"/>
     </row>
     <row r="14" spans="1:10">
-      <c r="A14" s="27"/>
-      <c r="B14" s="27"/>
-      <c r="C14" s="27"/>
-      <c r="D14" s="27"/>
-      <c r="E14" s="27"/>
-      <c r="F14" s="27"/>
-      <c r="G14" s="27"/>
-      <c r="H14" s="27"/>
-      <c r="I14" s="27"/>
-      <c r="J14" s="27"/>
+      <c r="A14" s="34"/>
+      <c r="B14" s="34"/>
+      <c r="C14" s="34"/>
+      <c r="D14" s="34"/>
+      <c r="E14" s="34"/>
+      <c r="F14" s="34"/>
+      <c r="G14" s="34"/>
+      <c r="H14" s="34"/>
+      <c r="I14" s="34"/>
+      <c r="J14" s="34"/>
     </row>
     <row r="15" spans="1:10">
-      <c r="A15" s="27"/>
-      <c r="B15" s="27"/>
-      <c r="C15" s="27"/>
-      <c r="D15" s="27"/>
-      <c r="E15" s="27"/>
-      <c r="F15" s="27"/>
-      <c r="G15" s="27"/>
-      <c r="H15" s="27"/>
-      <c r="I15" s="27"/>
-      <c r="J15" s="27"/>
+      <c r="A15" s="34"/>
+      <c r="B15" s="34"/>
+      <c r="C15" s="34"/>
+      <c r="D15" s="34"/>
+      <c r="E15" s="34"/>
+      <c r="F15" s="34"/>
+      <c r="G15" s="34"/>
+      <c r="H15" s="34"/>
+      <c r="I15" s="34"/>
+      <c r="J15" s="34"/>
     </row>
     <row r="16" spans="1:10">
-      <c r="A16" s="27"/>
-      <c r="B16" s="27"/>
-      <c r="C16" s="27"/>
-      <c r="D16" s="27"/>
-      <c r="E16" s="27"/>
-      <c r="F16" s="27"/>
-      <c r="G16" s="27"/>
-      <c r="H16" s="27"/>
-      <c r="I16" s="27"/>
-      <c r="J16" s="27"/>
+      <c r="A16" s="34"/>
+      <c r="B16" s="34"/>
+      <c r="C16" s="34"/>
+      <c r="D16" s="34"/>
+      <c r="E16" s="34"/>
+      <c r="F16" s="34"/>
+      <c r="G16" s="34"/>
+      <c r="H16" s="34"/>
+      <c r="I16" s="34"/>
+      <c r="J16" s="34"/>
     </row>
     <row r="17" spans="1:10">
-      <c r="A17" s="27"/>
-      <c r="B17" s="27"/>
-      <c r="C17" s="27"/>
-      <c r="D17" s="27"/>
-      <c r="E17" s="27"/>
-      <c r="F17" s="27"/>
-      <c r="G17" s="27"/>
-      <c r="H17" s="27"/>
-      <c r="I17" s="27"/>
-      <c r="J17" s="27"/>
+      <c r="A17" s="34"/>
+      <c r="B17" s="34"/>
+      <c r="C17" s="34"/>
+      <c r="D17" s="34"/>
+      <c r="E17" s="34"/>
+      <c r="F17" s="34"/>
+      <c r="G17" s="34"/>
+      <c r="H17" s="34"/>
+      <c r="I17" s="34"/>
+      <c r="J17" s="34"/>
     </row>
     <row r="18" spans="1:10">
-      <c r="A18" s="27"/>
-      <c r="B18" s="27"/>
-      <c r="C18" s="27"/>
-      <c r="D18" s="27"/>
-      <c r="E18" s="27"/>
-      <c r="F18" s="27"/>
-      <c r="G18" s="27"/>
-      <c r="H18" s="27"/>
-      <c r="I18" s="27"/>
-      <c r="J18" s="27"/>
+      <c r="A18" s="34"/>
+      <c r="B18" s="34"/>
+      <c r="C18" s="34"/>
+      <c r="D18" s="34"/>
+      <c r="E18" s="34"/>
+      <c r="F18" s="34"/>
+      <c r="G18" s="34"/>
+      <c r="H18" s="34"/>
+      <c r="I18" s="34"/>
+      <c r="J18" s="34"/>
     </row>
     <row r="19" spans="1:10">
-      <c r="A19" s="27"/>
-      <c r="B19" s="27"/>
-      <c r="C19" s="27"/>
-      <c r="D19" s="27"/>
-      <c r="E19" s="27"/>
-      <c r="F19" s="27"/>
-      <c r="G19" s="27"/>
-      <c r="H19" s="27"/>
-      <c r="I19" s="27"/>
-      <c r="J19" s="27"/>
+      <c r="A19" s="34"/>
+      <c r="B19" s="34"/>
+      <c r="C19" s="34"/>
+      <c r="D19" s="34"/>
+      <c r="E19" s="34"/>
+      <c r="F19" s="34"/>
+      <c r="G19" s="34"/>
+      <c r="H19" s="34"/>
+      <c r="I19" s="34"/>
+      <c r="J19" s="34"/>
     </row>
     <row r="20" spans="1:10">
-      <c r="A20" s="27"/>
-      <c r="B20" s="27"/>
-      <c r="C20" s="27"/>
-      <c r="D20" s="27"/>
-      <c r="E20" s="27"/>
-      <c r="F20" s="27"/>
-      <c r="G20" s="27"/>
-      <c r="H20" s="27"/>
-      <c r="I20" s="27"/>
-      <c r="J20" s="27"/>
+      <c r="A20" s="34"/>
+      <c r="B20" s="34"/>
+      <c r="C20" s="34"/>
+      <c r="D20" s="34"/>
+      <c r="E20" s="34"/>
+      <c r="F20" s="34"/>
+      <c r="G20" s="34"/>
+      <c r="H20" s="34"/>
+      <c r="I20" s="34"/>
+      <c r="J20" s="34"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2327,107 +2419,107 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11">
-      <c r="A1" s="7" t="s">
+      <c r="A1" s="6" t="s">
         <v>127</v>
       </c>
-      <c r="B1" s="7" t="s">
+      <c r="B1" s="6" t="s">
         <v>128</v>
       </c>
-      <c r="C1" s="7" t="s">
+      <c r="C1" s="6" t="s">
         <v>129</v>
       </c>
-      <c r="D1" s="7" t="s">
+      <c r="D1" s="6" t="s">
         <v>130</v>
       </c>
-      <c r="E1" s="7" t="s">
+      <c r="E1" s="6" t="s">
         <v>131</v>
       </c>
-      <c r="F1" s="10" t="s">
+      <c r="F1" s="19" t="s">
         <v>132</v>
       </c>
-      <c r="G1" s="10" t="s">
+      <c r="G1" s="19" t="s">
         <v>133</v>
       </c>
-      <c r="H1" s="10" t="s">
+      <c r="H1" s="19" t="s">
         <v>134</v>
       </c>
-      <c r="I1" s="10" t="s">
+      <c r="I1" s="19" t="s">
         <v>135</v>
       </c>
-      <c r="J1" s="10" t="s">
+      <c r="J1" s="19" t="s">
         <v>136</v>
       </c>
-      <c r="K1" s="10" t="s">
+      <c r="K1" s="19" t="s">
         <v>137</v>
       </c>
     </row>
     <row r="2" spans="1:11">
-      <c r="A2" s="7" t="s">
+      <c r="A2" s="6" t="s">
         <v>138</v>
       </c>
-      <c r="B2" s="7" t="s">
+      <c r="B2" s="6" t="s">
         <v>139</v>
       </c>
-      <c r="C2" s="7" t="s">
+      <c r="C2" s="6" t="s">
         <v>140</v>
       </c>
-      <c r="D2" s="7" t="s">
+      <c r="D2" s="6" t="s">
         <v>141</v>
       </c>
-      <c r="E2" s="7" t="s">
+      <c r="E2" s="6" t="s">
         <v>142</v>
       </c>
-      <c r="F2" s="2" t="s">
+      <c r="F2" s="4" t="s">
         <v>139</v>
       </c>
-      <c r="G2" s="2" t="s">
+      <c r="G2" s="4" t="s">
         <v>143</v>
       </c>
-      <c r="H2" s="2" t="s">
+      <c r="H2" s="4" t="s">
         <v>144</v>
       </c>
-      <c r="I2" s="2" t="s">
+      <c r="I2" s="4" t="s">
         <v>145</v>
       </c>
-      <c r="J2" s="2" t="s">
+      <c r="J2" s="4" t="s">
         <v>146</v>
       </c>
-      <c r="K2" s="2" t="s">
+      <c r="K2" s="4" t="s">
         <v>147</v>
       </c>
     </row>
     <row r="3" spans="1:11">
-      <c r="A3" s="11" t="s">
+      <c r="A3" s="20" t="s">
         <v>148</v>
       </c>
-      <c r="B3" s="2" t="s">
+      <c r="B3" s="4" t="s">
         <v>149</v>
       </c>
-      <c r="C3" s="7" t="s">
+      <c r="C3" s="6" t="s">
         <v>140</v>
       </c>
-      <c r="D3" s="2" t="s">
+      <c r="D3" s="4" t="s">
         <v>150</v>
       </c>
-      <c r="E3" s="2" t="s">
+      <c r="E3" s="4" t="s">
         <v>150</v>
       </c>
-      <c r="F3" s="2" t="s">
+      <c r="F3" s="4" t="s">
         <v>149</v>
       </c>
-      <c r="G3" s="2" t="s">
+      <c r="G3" s="4" t="s">
         <v>151</v>
       </c>
-      <c r="H3" s="2" t="s">
+      <c r="H3" s="4" t="s">
         <v>151</v>
       </c>
-      <c r="I3" s="2" t="s">
+      <c r="I3" s="4" t="s">
         <v>152</v>
       </c>
-      <c r="J3" s="2" t="s">
+      <c r="J3" s="4" t="s">
         <v>146</v>
       </c>
-      <c r="K3" s="2" t="s">
+      <c r="K3" s="4" t="s">
         <v>147</v>
       </c>
     </row>
@@ -2451,70 +2543,70 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5">
-      <c r="A1" s="7" t="s">
+      <c r="A1" s="6" t="s">
         <v>153</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="B1" s="4" t="s">
         <v>154</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="C1" s="4" t="s">
         <v>155</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="D1" s="4" t="s">
         <v>156</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="E1" s="4" t="s">
         <v>157</v>
       </c>
     </row>
     <row r="2" spans="1:5">
-      <c r="A2" s="7" t="s">
+      <c r="A2" s="6" t="s">
         <v>158</v>
       </c>
-      <c r="B2" s="7" t="s">
+      <c r="B2" s="6" t="s">
         <v>159</v>
       </c>
-      <c r="C2" s="8" t="s">
+      <c r="C2" s="17" t="s">
         <v>138</v>
       </c>
-      <c r="D2" s="9" t="s">
+      <c r="D2" s="18" t="s">
         <v>139</v>
       </c>
-      <c r="E2" s="7" t="s">
+      <c r="E2" s="6" t="s">
         <v>160</v>
       </c>
     </row>
     <row r="3" spans="1:5">
-      <c r="A3" s="2" t="s">
+      <c r="A3" s="4" t="s">
         <v>161</v>
       </c>
-      <c r="B3" s="2" t="s">
+      <c r="B3" s="4" t="s">
         <v>162</v>
       </c>
-      <c r="C3" s="2" t="s">
+      <c r="C3" s="4" t="s">
         <v>163</v>
       </c>
-      <c r="D3" s="2" t="s">
+      <c r="D3" s="4" t="s">
         <v>164</v>
       </c>
-      <c r="E3" s="2" t="s">
+      <c r="E3" s="4" t="s">
         <v>165</v>
       </c>
     </row>
     <row r="4" spans="1:5">
-      <c r="A4" s="2" t="s">
+      <c r="A4" s="4" t="s">
         <v>166</v>
       </c>
-      <c r="B4" s="2" t="s">
+      <c r="B4" s="4" t="s">
         <v>167</v>
       </c>
-      <c r="C4" s="2" t="s">
+      <c r="C4" s="4" t="s">
         <v>168</v>
       </c>
-      <c r="D4" s="2" t="s">
+      <c r="D4" s="4" t="s">
         <v>169</v>
       </c>
-      <c r="E4" s="2" t="s">
+      <c r="E4" s="4" t="s">
         <v>170</v>
       </c>
     </row>
@@ -2540,255 +2632,255 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7">
-      <c r="A1" s="3" t="s">
+      <c r="A1" s="13" t="s">
         <v>171</v>
       </c>
-      <c r="B1" s="3" t="s">
+      <c r="B1" s="13" t="s">
         <v>172</v>
       </c>
-      <c r="C1" s="4" t="s">
+      <c r="C1" s="14" t="s">
         <v>173</v>
       </c>
-      <c r="D1" s="4" t="s">
+      <c r="D1" s="14" t="s">
         <v>174</v>
       </c>
-      <c r="E1" s="4" t="s">
+      <c r="E1" s="14" t="s">
         <v>175</v>
       </c>
-      <c r="F1" s="3" t="s">
+      <c r="F1" s="13" t="s">
         <v>176</v>
       </c>
-      <c r="G1" s="3" t="s">
+      <c r="G1" s="13" t="s">
         <v>177</v>
       </c>
     </row>
     <row r="2" spans="1:7">
-      <c r="A2" s="5" t="s">
+      <c r="A2" s="15" t="s">
         <v>178</v>
       </c>
-      <c r="B2" s="5" t="s">
+      <c r="B2" s="15" t="s">
         <v>179</v>
       </c>
-      <c r="C2" s="6" t="s">
+      <c r="C2" s="16" t="s">
         <v>180</v>
       </c>
-      <c r="D2" s="6" t="s">
+      <c r="D2" s="16" t="s">
         <v>158</v>
       </c>
-      <c r="E2" s="6" t="s">
+      <c r="E2" s="16" t="s">
         <v>159</v>
       </c>
-      <c r="F2" s="5" t="s">
+      <c r="F2" s="15" t="s">
         <v>181</v>
       </c>
-      <c r="G2" s="5" t="s">
+      <c r="G2" s="15" t="s">
         <v>182</v>
       </c>
     </row>
     <row r="3" spans="1:7">
-      <c r="A3" s="5" t="s">
+      <c r="A3" s="15" t="s">
         <v>149</v>
       </c>
-      <c r="B3" s="5" t="s">
+      <c r="B3" s="15" t="s">
         <v>183</v>
       </c>
-      <c r="C3" s="6" t="s">
+      <c r="C3" s="16" t="s">
         <v>180</v>
       </c>
-      <c r="D3" s="6" t="s">
+      <c r="D3" s="16" t="s">
         <v>158</v>
       </c>
-      <c r="E3" s="6" t="s">
+      <c r="E3" s="16" t="s">
         <v>159</v>
       </c>
-      <c r="F3" s="5" t="s">
+      <c r="F3" s="15" t="s">
         <v>150</v>
       </c>
-      <c r="G3" s="5" t="s">
+      <c r="G3" s="15" t="s">
         <v>140</v>
       </c>
     </row>
     <row r="4" spans="1:7">
-      <c r="A4" s="5" t="s">
+      <c r="A4" s="15" t="s">
         <v>184</v>
       </c>
-      <c r="B4" s="5" t="s">
+      <c r="B4" s="15" t="s">
         <v>179</v>
       </c>
-      <c r="C4" s="6" t="s">
+      <c r="C4" s="16" t="s">
         <v>180</v>
       </c>
-      <c r="D4" s="6" t="s">
+      <c r="D4" s="16" t="s">
         <v>158</v>
       </c>
-      <c r="E4" s="6" t="s">
+      <c r="E4" s="16" t="s">
         <v>159</v>
       </c>
-      <c r="F4" s="5" t="s">
+      <c r="F4" s="15" t="s">
         <v>181</v>
       </c>
-      <c r="G4" s="5" t="s">
+      <c r="G4" s="15" t="s">
         <v>182</v>
       </c>
     </row>
     <row r="5" spans="1:7">
-      <c r="A5" s="5" t="s">
+      <c r="A5" s="15" t="s">
         <v>139</v>
       </c>
-      <c r="B5" s="5" t="s">
+      <c r="B5" s="15" t="s">
         <v>179</v>
       </c>
-      <c r="C5" s="6" t="s">
+      <c r="C5" s="16" t="s">
         <v>180</v>
       </c>
-      <c r="D5" s="6" t="s">
+      <c r="D5" s="16" t="s">
         <v>158</v>
       </c>
-      <c r="E5" s="6" t="s">
+      <c r="E5" s="16" t="s">
         <v>159</v>
       </c>
-      <c r="F5" s="5" t="s">
+      <c r="F5" s="15" t="s">
         <v>141</v>
       </c>
-      <c r="G5" s="5" t="s">
+      <c r="G5" s="15" t="s">
         <v>140</v>
       </c>
     </row>
     <row r="6" spans="1:7">
-      <c r="A6" s="5" t="s">
+      <c r="A6" s="15" t="s">
         <v>185</v>
       </c>
-      <c r="B6" s="5" t="s">
+      <c r="B6" s="15" t="s">
         <v>179</v>
       </c>
-      <c r="C6" s="6" t="s">
+      <c r="C6" s="16" t="s">
         <v>180</v>
       </c>
-      <c r="D6" s="6" t="s">
+      <c r="D6" s="16" t="s">
         <v>158</v>
       </c>
-      <c r="E6" s="6" t="s">
+      <c r="E6" s="16" t="s">
         <v>159</v>
       </c>
-      <c r="F6" s="5" t="s">
+      <c r="F6" s="15" t="s">
         <v>141</v>
       </c>
-      <c r="G6" s="5" t="s">
+      <c r="G6" s="15" t="s">
         <v>182</v>
       </c>
     </row>
     <row r="7" spans="1:7">
-      <c r="A7" s="5" t="s">
+      <c r="A7" s="15" t="s">
         <v>186</v>
       </c>
-      <c r="B7" s="5" t="s">
+      <c r="B7" s="15" t="s">
         <v>179</v>
       </c>
-      <c r="C7" s="6" t="s">
+      <c r="C7" s="16" t="s">
         <v>180</v>
       </c>
-      <c r="D7" s="6" t="s">
+      <c r="D7" s="16" t="s">
         <v>158</v>
       </c>
-      <c r="E7" s="6" t="s">
+      <c r="E7" s="16" t="s">
         <v>159</v>
       </c>
-      <c r="F7" s="5" t="s">
+      <c r="F7" s="15" t="s">
         <v>141</v>
       </c>
-      <c r="G7" s="5" t="s">
+      <c r="G7" s="15" t="s">
         <v>182</v>
       </c>
     </row>
     <row r="8" spans="1:7">
-      <c r="A8" s="5" t="s">
+      <c r="A8" s="15" t="s">
         <v>187</v>
       </c>
-      <c r="B8" s="5" t="s">
+      <c r="B8" s="15" t="s">
         <v>179</v>
       </c>
-      <c r="C8" s="6" t="s">
+      <c r="C8" s="16" t="s">
         <v>180</v>
       </c>
-      <c r="D8" s="6" t="s">
+      <c r="D8" s="16" t="s">
         <v>158</v>
       </c>
-      <c r="E8" s="6" t="s">
+      <c r="E8" s="16" t="s">
         <v>159</v>
       </c>
-      <c r="F8" s="5" t="s">
+      <c r="F8" s="15" t="s">
         <v>188</v>
       </c>
-      <c r="G8" s="5" t="s">
+      <c r="G8" s="15" t="s">
         <v>182</v>
       </c>
     </row>
     <row r="9" spans="1:7">
-      <c r="A9" s="5" t="s">
+      <c r="A9" s="15" t="s">
         <v>189</v>
       </c>
-      <c r="B9" s="5" t="s">
+      <c r="B9" s="15" t="s">
         <v>179</v>
       </c>
-      <c r="C9" s="6" t="s">
+      <c r="C9" s="16" t="s">
         <v>190</v>
       </c>
-      <c r="D9" s="6" t="s">
+      <c r="D9" s="16" t="s">
         <v>158</v>
       </c>
-      <c r="E9" s="6" t="s">
+      <c r="E9" s="16" t="s">
         <v>159</v>
       </c>
-      <c r="F9" s="5" t="s">
+      <c r="F9" s="15" t="s">
         <v>181</v>
       </c>
-      <c r="G9" s="5" t="s">
+      <c r="G9" s="15" t="s">
         <v>182</v>
       </c>
     </row>
     <row r="10" spans="1:7">
-      <c r="A10" s="5" t="s">
+      <c r="A10" s="15" t="s">
         <v>191</v>
       </c>
-      <c r="B10" s="5" t="s">
+      <c r="B10" s="15" t="s">
         <v>179</v>
       </c>
-      <c r="C10" s="6" t="s">
+      <c r="C10" s="16" t="s">
         <v>192</v>
       </c>
-      <c r="D10" s="6" t="s">
+      <c r="D10" s="16" t="s">
         <v>158</v>
       </c>
-      <c r="E10" s="6" t="s">
+      <c r="E10" s="16" t="s">
         <v>159</v>
       </c>
-      <c r="F10" s="5" t="s">
+      <c r="F10" s="15" t="s">
         <v>181</v>
       </c>
-      <c r="G10" s="5" t="s">
+      <c r="G10" s="15" t="s">
         <v>182</v>
       </c>
     </row>
     <row r="11" spans="1:7">
-      <c r="A11" s="5" t="s">
+      <c r="A11" s="15" t="s">
         <v>193</v>
       </c>
-      <c r="B11" s="5" t="s">
+      <c r="B11" s="15" t="s">
         <v>179</v>
       </c>
-      <c r="C11" s="6" t="s">
+      <c r="C11" s="16" t="s">
         <v>194</v>
       </c>
-      <c r="D11" s="6" t="s">
+      <c r="D11" s="16" t="s">
         <v>158</v>
       </c>
-      <c r="E11" s="6" t="s">
+      <c r="E11" s="16" t="s">
         <v>159</v>
       </c>
-      <c r="F11" s="5" t="s">
+      <c r="F11" s="15" t="s">
         <v>181</v>
       </c>
-      <c r="G11" s="5" t="s">
+      <c r="G11" s="15" t="s">
         <v>182</v>
       </c>
     </row>
@@ -2810,35 +2902,35 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:3">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="12" t="s">
         <v>195</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="12" t="s">
         <v>196</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="12" t="s">
         <v>84</v>
       </c>
     </row>
     <row r="2" spans="1:3">
-      <c r="A2" s="2" t="s">
+      <c r="A2" s="4" t="s">
         <v>197</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="B2" s="4" t="s">
         <v>198</v>
       </c>
-      <c r="C2" s="2">
+      <c r="C2" s="4">
         <v>2</v>
       </c>
     </row>
     <row r="3" spans="1:3">
-      <c r="A3" s="2" t="s">
+      <c r="A3" s="4" t="s">
         <v>199</v>
       </c>
-      <c r="B3" s="2" t="s">
+      <c r="B3" s="4" t="s">
         <v>198</v>
       </c>
-      <c r="C3" s="2">
+      <c r="C3" s="4">
         <v>2</v>
       </c>
     </row>
@@ -2860,36 +2952,258 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:3">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="12" t="s">
         <v>195</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="12" t="s">
         <v>196</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="12" t="s">
         <v>84</v>
       </c>
     </row>
     <row r="2" spans="1:3">
-      <c r="A2" s="2" t="s">
+      <c r="A2" s="4" t="s">
         <v>200</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="B2" s="4" t="s">
         <v>198</v>
       </c>
-      <c r="C2" s="2">
+      <c r="C2" s="4">
         <v>2</v>
       </c>
     </row>
     <row r="3" spans="1:3">
-      <c r="A3" s="2" t="s">
+      <c r="A3" s="4" t="s">
         <v>201</v>
       </c>
-      <c r="B3" s="2" t="s">
+      <c r="B3" s="4" t="s">
         <v>198</v>
       </c>
-      <c r="C3" s="2">
+      <c r="C3" s="4">
         <v>2</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <headerFooter/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
+  <dimension ref="A1:B2"/>
+  <sheetFormatPr defaultColWidth="8.72727272727273" defaultRowHeight="14.5" outlineLevelRow="1" outlineLevelCol="1"/>
+  <cols>
+    <col min="1" max="1" width="20.3636363636364" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2">
+      <c r="A1" s="8" t="s">
+        <v>202</v>
+      </c>
+      <c r="B1" s="8" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2">
+      <c r="A2" s="8" t="s">
+        <v>203</v>
+      </c>
+      <c r="B2" s="8">
+        <v>10</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <headerFooter/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
+  <dimension ref="A1:G3"/>
+  <sheetFormatPr defaultColWidth="8.72727272727273" defaultRowHeight="14.5" outlineLevelRow="2" outlineLevelCol="6"/>
+  <sheetData>
+    <row r="1" spans="1:7">
+      <c r="A1" s="7" t="s">
+        <v>204</v>
+      </c>
+      <c r="B1" s="7" t="s">
+        <v>84</v>
+      </c>
+      <c r="C1" s="7" t="s">
+        <v>80</v>
+      </c>
+      <c r="D1" s="7" t="s">
+        <v>85</v>
+      </c>
+      <c r="E1" s="7" t="s">
+        <v>68</v>
+      </c>
+      <c r="F1" s="7" t="s">
+        <v>69</v>
+      </c>
+      <c r="G1" s="7" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7">
+      <c r="A2" s="10" t="s">
+        <v>205</v>
+      </c>
+      <c r="B2" s="7">
+        <v>22</v>
+      </c>
+      <c r="C2" s="7">
+        <v>524</v>
+      </c>
+      <c r="D2" s="7">
+        <v>2</v>
+      </c>
+      <c r="E2" s="10" t="s">
+        <v>73</v>
+      </c>
+      <c r="F2" s="10" t="s">
+        <v>74</v>
+      </c>
+      <c r="G2" s="10" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7">
+      <c r="A3" s="10" t="s">
+        <v>206</v>
+      </c>
+      <c r="B3" s="7">
+        <v>34</v>
+      </c>
+      <c r="C3" s="7">
+        <v>232</v>
+      </c>
+      <c r="D3" s="7">
+        <v>7.9</v>
+      </c>
+      <c r="E3" s="10" t="s">
+        <v>73</v>
+      </c>
+      <c r="F3" s="10" t="s">
+        <v>89</v>
+      </c>
+      <c r="G3" s="11"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <headerFooter/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
+  <dimension ref="A1:C3"/>
+  <sheetFormatPr defaultColWidth="8.72727272727273" defaultRowHeight="14.5" outlineLevelRow="2" outlineLevelCol="2"/>
+  <sheetData>
+    <row r="1" spans="1:3">
+      <c r="A1" s="7" t="s">
+        <v>204</v>
+      </c>
+      <c r="B1" s="7" t="s">
+        <v>84</v>
+      </c>
+      <c r="C1" s="7" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3">
+      <c r="A2" s="9" t="s">
+        <v>207</v>
+      </c>
+      <c r="B2" s="7">
+        <v>22</v>
+      </c>
+      <c r="C2" s="7">
+        <v>524</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3">
+      <c r="A3" s="9" t="s">
+        <v>208</v>
+      </c>
+      <c r="B3" s="7">
+        <v>40</v>
+      </c>
+      <c r="C3" s="7">
+        <v>450</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <headerFooter/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
+  <dimension ref="A1:B2"/>
+  <sheetFormatPr defaultColWidth="8.72727272727273" defaultRowHeight="14.5" outlineLevelRow="1" outlineLevelCol="1"/>
+  <sheetData>
+    <row r="1" spans="1:2">
+      <c r="A1" s="8" t="s">
+        <v>209</v>
+      </c>
+      <c r="B1" s="8" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2">
+      <c r="A2" s="8" t="s">
+        <v>210</v>
+      </c>
+      <c r="B2" s="8">
+        <v>10</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <headerFooter/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
+  <dimension ref="A1:C3"/>
+  <sheetFormatPr defaultColWidth="8.72727272727273" defaultRowHeight="14.5" outlineLevelRow="2" outlineLevelCol="2"/>
+  <sheetData>
+    <row r="1" spans="1:3">
+      <c r="A1" t="s">
+        <v>204</v>
+      </c>
+      <c r="B1" s="7" t="s">
+        <v>84</v>
+      </c>
+      <c r="C1" s="7" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2">
+      <c r="A2" t="s">
+        <v>211</v>
+      </c>
+      <c r="B2">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2">
+      <c r="A3" t="s">
+        <v>212</v>
+      </c>
+      <c r="B3">
+        <v>45</v>
       </c>
     </row>
   </sheetData>
@@ -2927,552 +3241,622 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:20">
-      <c r="A1" s="12" t="s">
+      <c r="A1" s="21" t="s">
         <v>25</v>
       </c>
-      <c r="B1" s="12" t="s">
+      <c r="B1" s="21" t="s">
         <v>26</v>
       </c>
-      <c r="C1" s="12" t="s">
+      <c r="C1" s="21" t="s">
         <v>27</v>
       </c>
-      <c r="D1" s="12" t="s">
+      <c r="D1" s="21" t="s">
         <v>28</v>
       </c>
-      <c r="E1" s="12" t="s">
+      <c r="E1" s="21" t="s">
         <v>29</v>
       </c>
-      <c r="F1" s="12" t="s">
+      <c r="F1" s="21" t="s">
         <v>2</v>
       </c>
-      <c r="G1" s="12" t="s">
+      <c r="G1" s="21" t="s">
         <v>1</v>
       </c>
-      <c r="H1" s="12" t="s">
+      <c r="H1" s="21" t="s">
         <v>30</v>
       </c>
-      <c r="I1" s="12" t="s">
+      <c r="I1" s="21" t="s">
         <v>31</v>
       </c>
-      <c r="J1" s="12" t="s">
+      <c r="J1" s="21" t="s">
         <v>32</v>
       </c>
-      <c r="K1" s="12" t="s">
+      <c r="K1" s="21" t="s">
         <v>33</v>
       </c>
-      <c r="L1" s="12" t="s">
+      <c r="L1" s="21" t="s">
         <v>6</v>
       </c>
-      <c r="M1" s="12" t="s">
+      <c r="M1" s="21" t="s">
         <v>7</v>
       </c>
-      <c r="N1" s="12" t="s">
+      <c r="N1" s="21" t="s">
         <v>8</v>
       </c>
-      <c r="O1" s="12" t="s">
+      <c r="O1" s="21" t="s">
         <v>9</v>
       </c>
-      <c r="P1" s="12" t="s">
+      <c r="P1" s="21" t="s">
         <v>34</v>
       </c>
-      <c r="Q1" s="12" t="s">
+      <c r="Q1" s="21" t="s">
         <v>35</v>
       </c>
-      <c r="R1" s="12" t="s">
+      <c r="R1" s="21" t="s">
         <v>36</v>
       </c>
-      <c r="S1" s="12" t="s">
+      <c r="S1" s="21" t="s">
         <v>37</v>
       </c>
-      <c r="T1" s="12" t="s">
+      <c r="T1" s="21" t="s">
         <v>38</v>
       </c>
     </row>
     <row r="2" spans="1:20">
-      <c r="A2" s="12" t="s">
+      <c r="A2" s="21" t="s">
         <v>18</v>
       </c>
-      <c r="B2" s="12" t="s">
+      <c r="B2" s="21" t="s">
         <v>39</v>
       </c>
-      <c r="C2" s="12" t="s">
+      <c r="C2" s="21" t="s">
         <v>20</v>
       </c>
-      <c r="D2" s="12" t="s">
+      <c r="D2" s="21" t="s">
         <v>40</v>
       </c>
-      <c r="E2" s="12">
+      <c r="E2" s="21">
         <v>12</v>
       </c>
-      <c r="F2" s="18" t="s">
+      <c r="F2" s="25" t="s">
         <v>12</v>
       </c>
-      <c r="G2" s="12" t="s">
+      <c r="G2" s="21" t="s">
         <v>11</v>
       </c>
-      <c r="H2" s="12" t="s">
+      <c r="H2" s="21" t="s">
         <v>19</v>
       </c>
-      <c r="I2" s="12" t="s">
+      <c r="I2" s="21" t="s">
         <v>41</v>
       </c>
-      <c r="J2" s="12" t="s">
+      <c r="J2" s="21" t="s">
         <v>14</v>
       </c>
-      <c r="K2" s="12">
+      <c r="K2" s="21">
         <v>6</v>
       </c>
-      <c r="L2" s="12">
+      <c r="L2" s="21">
         <v>1010301033</v>
       </c>
-      <c r="M2" s="12" t="s">
+      <c r="M2" s="21" t="s">
         <v>15</v>
       </c>
-      <c r="N2" s="12" t="s">
+      <c r="N2" s="21" t="s">
         <v>16</v>
       </c>
-      <c r="O2" s="12" t="s">
+      <c r="O2" s="21" t="s">
         <v>17</v>
       </c>
-      <c r="P2" s="12"/>
-      <c r="Q2" s="12"/>
-      <c r="R2" s="12"/>
-      <c r="S2" s="12">
+      <c r="P2" s="21"/>
+      <c r="Q2" s="21"/>
+      <c r="R2" s="21"/>
+      <c r="S2" s="21">
         <v>0</v>
       </c>
-      <c r="T2" s="12"/>
+      <c r="T2" s="21"/>
     </row>
     <row r="3" spans="1:20">
-      <c r="A3" s="12" t="s">
+      <c r="A3" s="21" t="s">
         <v>10</v>
       </c>
-      <c r="B3" s="12" t="s">
+      <c r="B3" s="21" t="s">
         <v>42</v>
       </c>
-      <c r="C3" s="12" t="s">
+      <c r="C3" s="21" t="s">
         <v>14</v>
       </c>
-      <c r="D3" s="19" t="s">
+      <c r="D3" s="26" t="s">
         <v>43</v>
       </c>
-      <c r="E3" s="12">
+      <c r="E3" s="21">
         <v>5</v>
       </c>
-      <c r="F3" s="12" t="s">
+      <c r="F3" s="21" t="s">
         <v>12</v>
       </c>
-      <c r="G3" s="12" t="s">
+      <c r="G3" s="21" t="s">
         <v>11</v>
       </c>
-      <c r="H3" s="12" t="s">
+      <c r="H3" s="21" t="s">
         <v>13</v>
       </c>
-      <c r="I3" s="12" t="s">
+      <c r="I3" s="21" t="s">
         <v>44</v>
       </c>
-      <c r="J3" s="12" t="s">
+      <c r="J3" s="21" t="s">
         <v>14</v>
       </c>
-      <c r="K3" s="12">
+      <c r="K3" s="21">
         <v>1</v>
       </c>
-      <c r="L3" s="12">
+      <c r="L3" s="21">
         <v>1010301033</v>
       </c>
-      <c r="M3" s="12" t="s">
+      <c r="M3" s="21" t="s">
         <v>15</v>
       </c>
-      <c r="N3" s="12" t="s">
+      <c r="N3" s="21" t="s">
         <v>16</v>
       </c>
-      <c r="O3" s="12" t="s">
+      <c r="O3" s="21" t="s">
         <v>17</v>
       </c>
-      <c r="P3" s="12"/>
-      <c r="Q3" s="12"/>
-      <c r="R3" s="12"/>
-      <c r="S3" s="12">
+      <c r="P3" s="21"/>
+      <c r="Q3" s="21"/>
+      <c r="R3" s="21"/>
+      <c r="S3" s="21">
         <v>0</v>
       </c>
-      <c r="T3" s="12"/>
+      <c r="T3" s="21"/>
     </row>
     <row r="4" spans="1:20">
-      <c r="A4" s="12" t="s">
+      <c r="A4" s="21" t="s">
         <v>21</v>
       </c>
-      <c r="B4" s="12" t="s">
+      <c r="B4" s="21" t="s">
         <v>45</v>
       </c>
-      <c r="C4" s="12" t="s">
+      <c r="C4" s="21" t="s">
         <v>14</v>
       </c>
-      <c r="D4" s="12">
+      <c r="D4" s="21">
         <v>123562</v>
       </c>
-      <c r="E4" s="12">
+      <c r="E4" s="21">
         <v>18</v>
       </c>
-      <c r="F4" s="12" t="s">
+      <c r="F4" s="21" t="s">
         <v>22</v>
       </c>
-      <c r="G4" s="12" t="s">
+      <c r="G4" s="21" t="s">
         <v>22</v>
       </c>
-      <c r="H4" s="12" t="s">
+      <c r="H4" s="21" t="s">
         <v>23</v>
       </c>
-      <c r="I4" s="12" t="s">
+      <c r="I4" s="21" t="s">
         <v>44</v>
       </c>
-      <c r="J4" s="12" t="s">
+      <c r="J4" s="21" t="s">
         <v>14</v>
       </c>
-      <c r="K4" s="12">
+      <c r="K4" s="21">
         <v>1</v>
       </c>
-      <c r="L4" s="12">
+      <c r="L4" s="21">
         <v>1011134888</v>
       </c>
-      <c r="M4" s="12" t="s">
+      <c r="M4" s="21" t="s">
         <v>46</v>
       </c>
-      <c r="N4" s="12" t="s">
+      <c r="N4" s="21" t="s">
         <v>16</v>
       </c>
-      <c r="O4" s="12" t="s">
+      <c r="O4" s="21" t="s">
         <v>17</v>
       </c>
-      <c r="P4" s="12"/>
-      <c r="Q4" s="12"/>
-      <c r="R4" s="12"/>
-      <c r="S4" s="12">
+      <c r="P4" s="21"/>
+      <c r="Q4" s="21"/>
+      <c r="R4" s="21"/>
+      <c r="S4" s="21">
         <v>0</v>
       </c>
-      <c r="T4" s="12"/>
+      <c r="T4" s="21"/>
     </row>
     <row r="5" spans="1:20">
-      <c r="A5" s="2" t="s">
+      <c r="A5" s="4" t="s">
         <v>47</v>
       </c>
-      <c r="B5" s="2" t="s">
+      <c r="B5" s="4" t="s">
         <v>47</v>
       </c>
-      <c r="C5" s="12" t="s">
+      <c r="C5" s="21" t="s">
         <v>14</v>
       </c>
-      <c r="D5" s="2" t="s">
+      <c r="D5" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="E5" s="2">
+      <c r="E5" s="4">
         <v>12</v>
       </c>
-      <c r="F5" s="2" t="s">
+      <c r="F5" s="4" t="s">
         <v>48</v>
       </c>
-      <c r="G5" s="2" t="s">
+      <c r="G5" s="4" t="s">
         <v>49</v>
       </c>
-      <c r="H5" s="2" t="s">
+      <c r="H5" s="4" t="s">
         <v>50</v>
       </c>
-      <c r="I5" s="2" t="s">
+      <c r="I5" s="4" t="s">
         <v>44</v>
       </c>
-      <c r="J5" s="2" t="s">
+      <c r="J5" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="K5" s="2">
+      <c r="K5" s="4">
         <v>1</v>
       </c>
-      <c r="L5" s="2">
+      <c r="L5" s="4">
         <v>1010301001</v>
       </c>
-      <c r="M5" s="2" t="s">
+      <c r="M5" s="4" t="s">
         <v>51</v>
       </c>
-      <c r="N5" s="2" t="s">
+      <c r="N5" s="4" t="s">
         <v>52</v>
       </c>
-      <c r="O5" s="2" t="s">
+      <c r="O5" s="4" t="s">
         <v>53</v>
       </c>
-      <c r="P5" s="2"/>
-      <c r="Q5" s="2"/>
-      <c r="R5" s="2"/>
-      <c r="S5" s="12">
+      <c r="P5" s="4"/>
+      <c r="Q5" s="4"/>
+      <c r="R5" s="4"/>
+      <c r="S5" s="21">
         <v>0</v>
       </c>
-      <c r="T5" s="2"/>
+      <c r="T5" s="4"/>
     </row>
     <row r="6" spans="1:20">
-      <c r="A6" s="2" t="s">
+      <c r="A6" s="4" t="s">
         <v>54</v>
       </c>
-      <c r="B6" s="2" t="s">
+      <c r="B6" s="4" t="s">
         <v>54</v>
       </c>
-      <c r="C6" s="2" t="s">
+      <c r="C6" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="D6" s="17" t="s">
+      <c r="D6" s="24" t="s">
         <v>43</v>
       </c>
       <c r="E6">
         <v>5</v>
       </c>
-      <c r="F6" s="20" t="s">
+      <c r="F6" s="27" t="s">
         <v>12</v>
       </c>
-      <c r="G6" s="20" t="s">
+      <c r="G6" s="27" t="s">
         <v>11</v>
       </c>
-      <c r="H6" s="2" t="s">
+      <c r="H6" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="I6" s="2" t="s">
+      <c r="I6" s="4" t="s">
         <v>44</v>
       </c>
-      <c r="J6" s="2" t="s">
+      <c r="J6" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="K6" s="2">
+      <c r="K6" s="4">
         <v>1</v>
       </c>
-      <c r="L6" s="2">
+      <c r="L6" s="4">
         <v>1010301033</v>
       </c>
-      <c r="M6" s="2" t="s">
+      <c r="M6" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="N6" s="2" t="s">
+      <c r="N6" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="O6" s="2" t="s">
+      <c r="O6" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="P6" s="2"/>
-      <c r="Q6" s="2"/>
-      <c r="R6" s="2"/>
-      <c r="S6" s="12">
+      <c r="P6" s="4"/>
+      <c r="Q6" s="4"/>
+      <c r="R6" s="4"/>
+      <c r="S6" s="21">
         <v>0</v>
       </c>
-      <c r="T6" s="2"/>
+      <c r="T6" s="4"/>
     </row>
     <row r="7" spans="1:20">
-      <c r="A7" s="21" t="s">
+      <c r="A7" s="28" t="s">
         <v>55</v>
       </c>
-      <c r="B7" s="21" t="s">
+      <c r="B7" s="28" t="s">
         <v>56</v>
       </c>
-      <c r="C7" s="21" t="s">
+      <c r="C7" s="28" t="s">
         <v>20</v>
       </c>
-      <c r="D7" s="21" t="s">
+      <c r="D7" s="28" t="s">
         <v>40</v>
       </c>
-      <c r="E7" s="21">
+      <c r="E7" s="28">
         <v>12</v>
       </c>
-      <c r="F7" s="22" t="s">
+      <c r="F7" s="29" t="s">
         <v>12</v>
       </c>
-      <c r="G7" s="21" t="s">
+      <c r="G7" s="28" t="s">
         <v>11</v>
       </c>
-      <c r="H7" s="21" t="s">
+      <c r="H7" s="28" t="s">
         <v>57</v>
       </c>
-      <c r="I7" s="21" t="s">
+      <c r="I7" s="28" t="s">
         <v>41</v>
       </c>
-      <c r="J7" s="21" t="s">
+      <c r="J7" s="28" t="s">
         <v>14</v>
       </c>
-      <c r="K7" s="21">
+      <c r="K7" s="28">
         <v>3</v>
       </c>
-      <c r="L7" s="21">
+      <c r="L7" s="28">
         <v>1010301003</v>
       </c>
-      <c r="M7" s="21" t="s">
+      <c r="M7" s="28" t="s">
         <v>58</v>
       </c>
-      <c r="N7" s="21" t="s">
+      <c r="N7" s="28" t="s">
         <v>16</v>
       </c>
-      <c r="O7" s="21" t="s">
+      <c r="O7" s="28" t="s">
         <v>17</v>
       </c>
-      <c r="P7" s="21"/>
-      <c r="Q7" s="21"/>
-      <c r="R7" s="21"/>
-      <c r="S7" s="21">
+      <c r="P7" s="28"/>
+      <c r="Q7" s="28"/>
+      <c r="R7" s="28"/>
+      <c r="S7" s="28">
         <v>0</v>
       </c>
-      <c r="T7" s="21"/>
+      <c r="T7" s="28"/>
     </row>
     <row r="8" spans="1:20">
-      <c r="A8" s="21" t="s">
+      <c r="A8" s="28" t="s">
         <v>59</v>
       </c>
-      <c r="B8" s="21" t="s">
+      <c r="B8" s="28" t="s">
         <v>60</v>
       </c>
-      <c r="C8" s="21" t="s">
+      <c r="C8" s="28" t="s">
         <v>14</v>
       </c>
-      <c r="D8" s="21" t="s">
+      <c r="D8" s="28" t="s">
         <v>43</v>
       </c>
-      <c r="E8" s="21">
+      <c r="E8" s="28">
         <v>5</v>
       </c>
-      <c r="F8" s="22" t="s">
+      <c r="F8" s="29" t="s">
         <v>12</v>
       </c>
-      <c r="G8" s="21" t="s">
+      <c r="G8" s="28" t="s">
         <v>11</v>
       </c>
-      <c r="H8" s="21" t="s">
+      <c r="H8" s="28" t="s">
         <v>57</v>
       </c>
-      <c r="I8" s="21" t="s">
+      <c r="I8" s="28" t="s">
         <v>41</v>
       </c>
-      <c r="J8" s="21" t="s">
+      <c r="J8" s="28" t="s">
         <v>14</v>
       </c>
-      <c r="K8" s="21">
+      <c r="K8" s="28">
         <v>0</v>
       </c>
-      <c r="L8" s="21">
+      <c r="L8" s="28">
         <v>1010301003</v>
       </c>
-      <c r="M8" s="21" t="s">
+      <c r="M8" s="28" t="s">
         <v>58</v>
       </c>
-      <c r="N8" s="21" t="s">
+      <c r="N8" s="28" t="s">
         <v>16</v>
       </c>
-      <c r="O8" s="21" t="s">
+      <c r="O8" s="28" t="s">
         <v>17</v>
       </c>
-      <c r="P8" s="21"/>
-      <c r="Q8" s="21"/>
-      <c r="R8" s="21"/>
-      <c r="S8" s="21">
+      <c r="P8" s="28"/>
+      <c r="Q8" s="28"/>
+      <c r="R8" s="28"/>
+      <c r="S8" s="28">
         <v>0</v>
       </c>
-      <c r="T8" s="21"/>
+      <c r="T8" s="28"/>
     </row>
     <row r="9" spans="1:20">
-      <c r="A9" s="21" t="s">
+      <c r="A9" s="28" t="s">
         <v>61</v>
       </c>
-      <c r="B9" s="21" t="s">
+      <c r="B9" s="28" t="s">
         <v>61</v>
       </c>
-      <c r="C9" s="21" t="s">
+      <c r="C9" s="28" t="s">
         <v>14</v>
       </c>
-      <c r="D9" s="21" t="s">
+      <c r="D9" s="28" t="s">
         <v>43</v>
       </c>
-      <c r="E9" s="21">
+      <c r="E9" s="28">
         <v>5</v>
       </c>
-      <c r="F9" s="22" t="s">
+      <c r="F9" s="29" t="s">
         <v>12</v>
       </c>
-      <c r="G9" s="21" t="s">
+      <c r="G9" s="28" t="s">
         <v>11</v>
       </c>
-      <c r="H9" s="21" t="s">
+      <c r="H9" s="28" t="s">
         <v>57</v>
       </c>
-      <c r="I9" s="21" t="s">
+      <c r="I9" s="28" t="s">
         <v>41</v>
       </c>
-      <c r="J9" s="21" t="s">
+      <c r="J9" s="28" t="s">
         <v>14</v>
       </c>
-      <c r="K9" s="21">
+      <c r="K9" s="28">
         <v>0</v>
       </c>
-      <c r="L9" s="21">
+      <c r="L9" s="28">
         <v>1010301003</v>
       </c>
-      <c r="M9" s="21" t="s">
+      <c r="M9" s="28" t="s">
         <v>58</v>
       </c>
-      <c r="N9" s="21" t="s">
+      <c r="N9" s="28" t="s">
         <v>16</v>
       </c>
-      <c r="O9" s="21" t="s">
+      <c r="O9" s="28" t="s">
         <v>17</v>
       </c>
-      <c r="P9" s="21"/>
-      <c r="Q9" s="21"/>
-      <c r="R9" s="21"/>
-      <c r="S9" s="21">
+      <c r="P9" s="28"/>
+      <c r="Q9" s="28"/>
+      <c r="R9" s="28"/>
+      <c r="S9" s="28">
         <v>0</v>
       </c>
-      <c r="T9" s="21"/>
+      <c r="T9" s="28"/>
     </row>
     <row r="10" spans="1:20">
-      <c r="A10" s="2" t="s">
+      <c r="A10" s="4" t="s">
         <v>62</v>
       </c>
-      <c r="B10" s="2" t="s">
+      <c r="B10" s="4" t="s">
         <v>62</v>
       </c>
-      <c r="C10" s="2" t="s">
+      <c r="C10" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="D10" s="21" t="s">
+      <c r="D10" s="28" t="s">
         <v>43</v>
       </c>
-      <c r="E10" s="21">
+      <c r="E10" s="28">
         <v>5</v>
       </c>
-      <c r="F10" s="12" t="s">
+      <c r="F10" s="21" t="s">
         <v>22</v>
       </c>
-      <c r="G10" s="12" t="s">
+      <c r="G10" s="21" t="s">
         <v>22</v>
       </c>
-      <c r="H10" s="12" t="s">
+      <c r="H10" s="21" t="s">
         <v>63</v>
       </c>
-      <c r="I10" s="12" t="s">
+      <c r="I10" s="21" t="s">
         <v>44</v>
       </c>
-      <c r="J10" s="12" t="s">
+      <c r="J10" s="21" t="s">
         <v>14</v>
       </c>
-      <c r="K10" s="12">
+      <c r="K10" s="21">
         <v>1</v>
       </c>
-      <c r="L10" s="15">
+      <c r="L10" s="22">
         <v>1000000001</v>
       </c>
-      <c r="M10" s="2" t="s">
+      <c r="M10" s="4" t="s">
         <v>64</v>
       </c>
-      <c r="N10" s="2" t="s">
+      <c r="N10" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="O10" s="2" t="s">
+      <c r="O10" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="P10" s="21"/>
-      <c r="Q10" s="21"/>
-      <c r="R10" s="21"/>
-      <c r="S10" s="21">
+      <c r="P10" s="28"/>
+      <c r="Q10" s="28"/>
+      <c r="R10" s="28"/>
+      <c r="S10" s="28">
         <v>0</v>
       </c>
-      <c r="T10" s="21"/>
+      <c r="T10" s="28"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <headerFooter/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
+  <dimension ref="A1:F3"/>
+  <sheetFormatPr defaultColWidth="8.72727272727273" defaultRowHeight="14.5" outlineLevelRow="2" outlineLevelCol="5"/>
+  <sheetData>
+    <row r="1" spans="1:6">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="E1" s="3" t="s">
+        <v>69</v>
+      </c>
+      <c r="F1" s="3" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6">
+      <c r="A2" s="3" t="s">
+        <v>213</v>
+      </c>
+      <c r="B2" s="4">
+        <v>10</v>
+      </c>
+      <c r="C2" s="4">
+        <v>45</v>
+      </c>
+      <c r="D2" s="4" t="s">
+        <v>73</v>
+      </c>
+      <c r="E2" s="5" t="s">
+        <v>214</v>
+      </c>
+      <c r="F2" s="6" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6">
+      <c r="A3" s="3" t="s">
+        <v>215</v>
+      </c>
+      <c r="B3" s="4">
+        <v>50</v>
+      </c>
+      <c r="C3" s="4">
+        <v>70</v>
+      </c>
+      <c r="D3" s="4" t="s">
+        <v>77</v>
+      </c>
+      <c r="E3" s="4" t="s">
+        <v>75</v>
+      </c>
+      <c r="F3" s="6"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -3500,128 +3884,128 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:18">
-      <c r="A1" s="2" t="s">
+      <c r="A1" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="B1" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="C1" s="4" t="s">
         <v>27</v>
       </c>
-      <c r="D1" s="12" t="s">
+      <c r="D1" s="21" t="s">
         <v>6</v>
       </c>
-      <c r="E1" s="12" t="s">
+      <c r="E1" s="21" t="s">
         <v>7</v>
       </c>
-      <c r="F1" s="12" t="s">
+      <c r="F1" s="21" t="s">
         <v>8</v>
       </c>
-      <c r="G1" s="12" t="s">
+      <c r="G1" s="21" t="s">
         <v>9</v>
       </c>
-      <c r="H1" s="2" t="s">
+      <c r="H1" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="I1" s="2" t="s">
+      <c r="I1" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="J1" s="2" t="s">
+      <c r="J1" s="4" t="s">
         <v>31</v>
       </c>
-      <c r="K1" s="2" t="s">
+      <c r="K1" s="4" t="s">
         <v>65</v>
       </c>
-      <c r="L1" s="2" t="s">
+      <c r="L1" s="4" t="s">
         <v>33</v>
       </c>
-      <c r="M1" s="16"/>
-      <c r="N1" s="16"/>
-      <c r="O1" s="16"/>
-      <c r="P1" s="16"/>
-      <c r="Q1" s="16"/>
-      <c r="R1" s="16"/>
+      <c r="M1" s="23"/>
+      <c r="N1" s="23"/>
+      <c r="O1" s="23"/>
+      <c r="P1" s="23"/>
+      <c r="Q1" s="23"/>
+      <c r="R1" s="23"/>
     </row>
     <row r="2" spans="1:18">
-      <c r="A2" s="2" t="s">
+      <c r="A2" s="4" t="s">
         <v>54</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="B2" s="4" t="s">
         <v>54</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="C2" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="D2" s="2">
+      <c r="D2" s="4">
         <v>1010301033</v>
       </c>
-      <c r="E2" s="2" t="s">
+      <c r="E2" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="F2" s="2" t="s">
+      <c r="F2" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="G2" s="2" t="s">
+      <c r="G2" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="H2" s="2" t="s">
+      <c r="H2" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="I2" s="17" t="s">
+      <c r="I2" s="24" t="s">
         <v>43</v>
       </c>
-      <c r="J2" s="2" t="s">
+      <c r="J2" s="4" t="s">
         <v>44</v>
       </c>
-      <c r="K2" s="2" t="s">
+      <c r="K2" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="L2" s="2">
+      <c r="L2" s="4">
         <v>1</v>
       </c>
-      <c r="M2" s="16"/>
-      <c r="N2" s="16"/>
-      <c r="O2" s="16"/>
-      <c r="P2" s="16"/>
-      <c r="Q2" s="16"/>
-      <c r="R2" s="16"/>
+      <c r="M2" s="23"/>
+      <c r="N2" s="23"/>
+      <c r="O2" s="23"/>
+      <c r="P2" s="23"/>
+      <c r="Q2" s="23"/>
+      <c r="R2" s="23"/>
     </row>
     <row r="3" spans="1:12">
-      <c r="A3" s="2" t="s">
+      <c r="A3" s="4" t="s">
         <v>62</v>
       </c>
-      <c r="B3" s="2" t="s">
+      <c r="B3" s="4" t="s">
         <v>62</v>
       </c>
-      <c r="C3" s="2" t="s">
+      <c r="C3" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="D3" s="15">
+      <c r="D3" s="22">
         <v>1000000001</v>
       </c>
-      <c r="E3" s="2" t="s">
+      <c r="E3" s="4" t="s">
         <v>64</v>
       </c>
-      <c r="F3" s="2" t="s">
+      <c r="F3" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="G3" s="2" t="s">
+      <c r="G3" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="H3" s="2" t="s">
+      <c r="H3" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="I3" s="17" t="s">
+      <c r="I3" s="24" t="s">
         <v>43</v>
       </c>
-      <c r="J3" s="2" t="s">
+      <c r="J3" s="4" t="s">
         <v>44</v>
       </c>
-      <c r="K3" s="2" t="s">
+      <c r="K3" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="L3" s="2">
+      <c r="L3" s="4">
         <v>1</v>
       </c>
     </row>
@@ -3646,60 +4030,60 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6">
-      <c r="A1" s="13" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="13" t="s">
+      <c r="B1" s="1" t="s">
         <v>66</v>
       </c>
-      <c r="C1" s="13" t="s">
+      <c r="C1" s="1" t="s">
         <v>67</v>
       </c>
-      <c r="D1" s="14" t="s">
+      <c r="D1" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="E1" s="12" t="s">
+      <c r="E1" s="21" t="s">
         <v>69</v>
       </c>
-      <c r="F1" s="12" t="s">
+      <c r="F1" s="21" t="s">
         <v>70</v>
       </c>
     </row>
     <row r="2" spans="1:6">
-      <c r="A2" s="2" t="s">
+      <c r="A2" s="4" t="s">
         <v>59</v>
       </c>
-      <c r="B2" s="2">
+      <c r="B2" s="4">
         <v>2</v>
       </c>
-      <c r="C2" s="2">
+      <c r="C2" s="4">
         <v>70</v>
       </c>
-      <c r="D2" s="2" t="s">
+      <c r="D2" s="4" t="s">
         <v>71</v>
       </c>
-      <c r="E2" s="2"/>
-      <c r="F2" s="7" t="s">
+      <c r="E2" s="4"/>
+      <c r="F2" s="6" t="s">
         <v>72</v>
       </c>
     </row>
     <row r="3" spans="1:6">
-      <c r="A3" s="2" t="s">
+      <c r="A3" s="4" t="s">
         <v>61</v>
       </c>
-      <c r="B3" s="2">
+      <c r="B3" s="4">
         <v>40</v>
       </c>
-      <c r="C3" s="2">
+      <c r="C3" s="4">
         <v>26</v>
       </c>
-      <c r="D3" s="2" t="s">
+      <c r="D3" s="4" t="s">
         <v>73</v>
       </c>
-      <c r="E3" s="7" t="s">
+      <c r="E3" s="6" t="s">
         <v>74</v>
       </c>
-      <c r="F3" s="7">
+      <c r="F3" s="6">
         <v>2</v>
       </c>
     </row>
@@ -3724,80 +4108,80 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6">
-      <c r="A1" s="13" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="13" t="s">
+      <c r="B1" s="1" t="s">
         <v>66</v>
       </c>
-      <c r="C1" s="13" t="s">
+      <c r="C1" s="1" t="s">
         <v>67</v>
       </c>
-      <c r="D1" s="14" t="s">
+      <c r="D1" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="E1" s="12" t="s">
+      <c r="E1" s="21" t="s">
         <v>69</v>
       </c>
-      <c r="F1" s="12" t="s">
+      <c r="F1" s="21" t="s">
         <v>70</v>
       </c>
     </row>
     <row r="2" spans="1:6">
-      <c r="A2" s="12" t="s">
+      <c r="A2" s="21" t="s">
         <v>59</v>
       </c>
-      <c r="B2" s="2">
+      <c r="B2" s="4">
         <v>2</v>
       </c>
-      <c r="C2" s="2">
+      <c r="C2" s="4">
         <v>45</v>
       </c>
-      <c r="D2" s="2" t="s">
+      <c r="D2" s="4" t="s">
         <v>71</v>
       </c>
-      <c r="E2" s="2"/>
-      <c r="F2" s="7" t="s">
+      <c r="E2" s="4"/>
+      <c r="F2" s="6" t="s">
         <v>75</v>
       </c>
     </row>
     <row r="3" spans="1:6">
-      <c r="A3" s="12" t="s">
+      <c r="A3" s="21" t="s">
         <v>76</v>
       </c>
-      <c r="B3" s="2">
+      <c r="B3" s="4">
         <v>40</v>
       </c>
-      <c r="C3" s="2">
+      <c r="C3" s="4">
         <v>26</v>
       </c>
-      <c r="D3" s="2" t="s">
+      <c r="D3" s="4" t="s">
         <v>77</v>
       </c>
-      <c r="E3" s="7" t="s">
+      <c r="E3" s="6" t="s">
         <v>74</v>
       </c>
-      <c r="F3" s="7">
+      <c r="F3" s="6">
         <v>2</v>
       </c>
     </row>
     <row r="4" spans="1:6">
-      <c r="A4" s="12" t="s">
+      <c r="A4" s="21" t="s">
         <v>61</v>
       </c>
-      <c r="B4" s="2">
+      <c r="B4" s="4">
         <v>50</v>
       </c>
-      <c r="C4" s="2">
+      <c r="C4" s="4">
         <v>70</v>
       </c>
-      <c r="D4" s="2" t="s">
+      <c r="D4" s="4" t="s">
         <v>73</v>
       </c>
-      <c r="E4" s="2" t="s">
+      <c r="E4" s="4" t="s">
         <v>75</v>
       </c>
-      <c r="F4" s="7"/>
+      <c r="F4" s="6"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -3869,90 +4253,90 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7">
-      <c r="A1" s="12" t="s">
+      <c r="A1" s="21" t="s">
         <v>83</v>
       </c>
-      <c r="B1" s="12" t="s">
+      <c r="B1" s="21" t="s">
         <v>84</v>
       </c>
-      <c r="C1" s="12" t="s">
+      <c r="C1" s="21" t="s">
         <v>80</v>
       </c>
-      <c r="D1" s="12" t="s">
+      <c r="D1" s="21" t="s">
         <v>85</v>
       </c>
-      <c r="E1" s="12" t="s">
+      <c r="E1" s="21" t="s">
         <v>68</v>
       </c>
-      <c r="F1" s="12" t="s">
+      <c r="F1" s="21" t="s">
         <v>69</v>
       </c>
-      <c r="G1" s="12" t="s">
+      <c r="G1" s="21" t="s">
         <v>70</v>
       </c>
     </row>
     <row r="2" spans="1:7">
-      <c r="A2" s="12" t="s">
+      <c r="A2" s="21" t="s">
         <v>86</v>
       </c>
-      <c r="B2" s="12">
+      <c r="B2" s="21">
         <v>2</v>
       </c>
-      <c r="C2" s="12">
+      <c r="C2" s="21">
         <v>524</v>
       </c>
-      <c r="D2" s="12">
+      <c r="D2" s="21">
         <v>2</v>
       </c>
-      <c r="E2" s="7" t="s">
+      <c r="E2" s="6" t="s">
         <v>71</v>
       </c>
-      <c r="F2" s="7" t="s">
+      <c r="F2" s="6" t="s">
         <v>74</v>
       </c>
-      <c r="G2" s="7" t="s">
+      <c r="G2" s="6" t="s">
         <v>87</v>
       </c>
     </row>
     <row r="3" spans="1:7">
-      <c r="A3" s="12" t="s">
+      <c r="A3" s="21" t="s">
         <v>88</v>
       </c>
-      <c r="B3" s="12">
+      <c r="B3" s="21">
         <v>232</v>
       </c>
-      <c r="C3" s="12">
+      <c r="C3" s="21">
         <v>232</v>
       </c>
-      <c r="D3" s="12">
+      <c r="D3" s="21">
         <v>7.9</v>
       </c>
-      <c r="E3" s="7" t="s">
+      <c r="E3" s="6" t="s">
         <v>73</v>
       </c>
-      <c r="F3" s="7" t="s">
+      <c r="F3" s="6" t="s">
         <v>89</v>
       </c>
-      <c r="G3" s="2"/>
+      <c r="G3" s="4"/>
     </row>
     <row r="4" spans="1:7">
-      <c r="A4" s="2" t="s">
+      <c r="A4" s="4" t="s">
         <v>90</v>
       </c>
-      <c r="B4" s="2">
+      <c r="B4" s="4">
         <v>232</v>
       </c>
-      <c r="C4" s="2">
+      <c r="C4" s="4">
         <v>232</v>
       </c>
-      <c r="D4" s="2">
+      <c r="D4" s="4">
         <v>2.32</v>
       </c>
-      <c r="E4" s="7" t="s">
+      <c r="E4" s="6" t="s">
         <v>77</v>
       </c>
-      <c r="F4" s="2"/>
-      <c r="G4" s="2"/>
+      <c r="F4" s="4"/>
+      <c r="G4" s="4"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -3976,90 +4360,90 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7">
-      <c r="A1" s="12" t="s">
+      <c r="A1" s="21" t="s">
         <v>83</v>
       </c>
-      <c r="B1" s="12" t="s">
+      <c r="B1" s="21" t="s">
         <v>84</v>
       </c>
-      <c r="C1" s="12" t="s">
+      <c r="C1" s="21" t="s">
         <v>80</v>
       </c>
-      <c r="D1" s="12" t="s">
+      <c r="D1" s="21" t="s">
         <v>85</v>
       </c>
-      <c r="E1" s="12" t="s">
+      <c r="E1" s="21" t="s">
         <v>68</v>
       </c>
-      <c r="F1" s="12" t="s">
+      <c r="F1" s="21" t="s">
         <v>69</v>
       </c>
-      <c r="G1" s="12" t="s">
+      <c r="G1" s="21" t="s">
         <v>70</v>
       </c>
     </row>
     <row r="2" spans="1:7">
-      <c r="A2" s="12" t="s">
+      <c r="A2" s="21" t="s">
         <v>86</v>
       </c>
-      <c r="B2" s="12">
+      <c r="B2" s="21">
         <v>2</v>
       </c>
-      <c r="C2" s="12">
+      <c r="C2" s="21">
         <v>524</v>
       </c>
-      <c r="D2" s="12">
+      <c r="D2" s="21">
         <v>2</v>
       </c>
-      <c r="E2" s="7" t="s">
+      <c r="E2" s="6" t="s">
         <v>71</v>
       </c>
-      <c r="F2" s="7" t="s">
+      <c r="F2" s="6" t="s">
         <v>74</v>
       </c>
-      <c r="G2" s="7" t="s">
+      <c r="G2" s="6" t="s">
         <v>87</v>
       </c>
     </row>
     <row r="3" spans="1:7">
-      <c r="A3" s="12" t="s">
+      <c r="A3" s="21" t="s">
         <v>88</v>
       </c>
-      <c r="B3" s="12">
+      <c r="B3" s="21">
         <v>34</v>
       </c>
-      <c r="C3" s="12">
+      <c r="C3" s="21">
         <v>232</v>
       </c>
-      <c r="D3" s="12">
+      <c r="D3" s="21">
         <v>7.9</v>
       </c>
-      <c r="E3" s="7" t="s">
+      <c r="E3" s="6" t="s">
         <v>73</v>
       </c>
-      <c r="F3" s="7" t="s">
+      <c r="F3" s="6" t="s">
         <v>89</v>
       </c>
-      <c r="G3" s="2"/>
+      <c r="G3" s="4"/>
     </row>
     <row r="4" spans="1:7">
-      <c r="A4" s="2" t="s">
+      <c r="A4" s="4" t="s">
         <v>90</v>
       </c>
-      <c r="B4" s="2">
+      <c r="B4" s="4">
         <v>67</v>
       </c>
-      <c r="C4" s="2">
+      <c r="C4" s="4">
         <v>232</v>
       </c>
-      <c r="D4" s="2">
+      <c r="D4" s="4">
         <v>2.32</v>
       </c>
-      <c r="E4" s="7" t="s">
+      <c r="E4" s="6" t="s">
         <v>77</v>
       </c>
-      <c r="F4" s="2"/>
-      <c r="G4" s="2"/>
+      <c r="F4" s="4"/>
+      <c r="G4" s="4"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -4093,611 +4477,611 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:19">
-      <c r="A1" s="2" t="s">
+      <c r="A1" s="4" t="s">
         <v>91</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="B1" s="4" t="s">
         <v>92</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="C1" s="4" t="s">
         <v>93</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="D1" s="4" t="s">
         <v>94</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="E1" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="F1" s="2" t="s">
+      <c r="F1" s="4" t="s">
         <v>95</v>
       </c>
-      <c r="G1" s="2" t="s">
+      <c r="G1" s="4" t="s">
         <v>96</v>
       </c>
-      <c r="H1" s="2" t="s">
+      <c r="H1" s="4" t="s">
         <v>34</v>
       </c>
-      <c r="I1" s="2" t="s">
+      <c r="I1" s="4" t="s">
         <v>97</v>
       </c>
-      <c r="J1" s="2" t="s">
+      <c r="J1" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="K1" s="2" t="s">
+      <c r="K1" s="4" t="s">
         <v>98</v>
       </c>
-      <c r="L1" s="2" t="s">
+      <c r="L1" s="4" t="s">
         <v>99</v>
       </c>
-      <c r="M1" s="2" t="s">
+      <c r="M1" s="4" t="s">
         <v>100</v>
       </c>
-      <c r="N1" s="2" t="s">
+      <c r="N1" s="4" t="s">
         <v>101</v>
       </c>
-      <c r="O1" s="2" t="s">
+      <c r="O1" s="4" t="s">
         <v>102</v>
       </c>
-      <c r="P1" s="2" t="s">
+      <c r="P1" s="4" t="s">
         <v>103</v>
       </c>
-      <c r="Q1" s="2" t="s">
+      <c r="Q1" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="R1" s="2" t="s">
+      <c r="R1" s="4" t="s">
         <v>104</v>
       </c>
-      <c r="S1" s="5" t="s">
+      <c r="S1" s="15" t="s">
         <v>105</v>
       </c>
     </row>
     <row r="2" spans="1:19">
-      <c r="A2" s="11" t="s">
+      <c r="A2" s="20" t="s">
         <v>106</v>
       </c>
-      <c r="B2" s="2">
+      <c r="B2" s="4">
         <v>0</v>
       </c>
-      <c r="C2" s="11" t="s">
+      <c r="C2" s="20" t="s">
         <v>106</v>
       </c>
-      <c r="D2" s="2" t="s">
+      <c r="D2" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="E2" s="2" t="s">
+      <c r="E2" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="F2" s="2">
+      <c r="F2" s="4">
         <v>12</v>
       </c>
-      <c r="G2" s="2" t="s">
+      <c r="G2" s="4" t="s">
         <v>41</v>
       </c>
-      <c r="H2" s="2"/>
-      <c r="I2" s="2"/>
-      <c r="J2" s="2" t="s">
+      <c r="H2" s="4"/>
+      <c r="I2" s="4"/>
+      <c r="J2" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="K2" s="2">
+      <c r="K2" s="4">
         <v>1</v>
       </c>
-      <c r="L2" s="2" t="s">
+      <c r="L2" s="4" t="s">
         <v>107</v>
       </c>
-      <c r="M2" s="2"/>
-      <c r="N2" s="2"/>
-      <c r="O2" s="7" t="s">
+      <c r="M2" s="4"/>
+      <c r="N2" s="4"/>
+      <c r="O2" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="P2" s="7" t="s">
+      <c r="P2" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="Q2" s="7" t="s">
+      <c r="Q2" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="R2" s="2" t="s">
+      <c r="R2" s="4" t="s">
         <v>108</v>
       </c>
-      <c r="S2" s="10" t="s">
+      <c r="S2" s="19" t="s">
         <v>109</v>
       </c>
     </row>
     <row r="3" spans="1:19">
-      <c r="A3" s="11" t="s">
+      <c r="A3" s="20" t="s">
         <v>110</v>
       </c>
-      <c r="B3" s="2">
+      <c r="B3" s="4">
         <v>0</v>
       </c>
-      <c r="C3" s="11" t="s">
+      <c r="C3" s="20" t="s">
         <v>110</v>
       </c>
-      <c r="D3" s="2" t="s">
+      <c r="D3" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="E3" s="11">
+      <c r="E3" s="20">
         <v>772213</v>
       </c>
-      <c r="F3" s="2">
+      <c r="F3" s="4">
         <v>5</v>
       </c>
-      <c r="G3" s="2" t="s">
+      <c r="G3" s="4" t="s">
         <v>41</v>
       </c>
-      <c r="H3" s="2"/>
-      <c r="I3" s="2"/>
-      <c r="J3" s="2" t="s">
+      <c r="H3" s="4"/>
+      <c r="I3" s="4"/>
+      <c r="J3" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="K3" s="2">
+      <c r="K3" s="4">
         <v>3</v>
       </c>
-      <c r="L3" s="2" t="s">
+      <c r="L3" s="4" t="s">
         <v>107</v>
       </c>
-      <c r="M3" s="2"/>
-      <c r="N3" s="2"/>
-      <c r="O3" s="7" t="s">
+      <c r="M3" s="4"/>
+      <c r="N3" s="4"/>
+      <c r="O3" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="P3" s="7" t="s">
+      <c r="P3" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="Q3" s="7" t="s">
+      <c r="Q3" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="R3" s="2" t="s">
+      <c r="R3" s="4" t="s">
         <v>108</v>
       </c>
-      <c r="S3" s="10" t="s">
+      <c r="S3" s="19" t="s">
         <v>109</v>
       </c>
     </row>
     <row r="4" spans="1:19">
-      <c r="A4" s="2" t="s">
+      <c r="A4" s="4" t="s">
         <v>111</v>
       </c>
-      <c r="B4" s="2">
+      <c r="B4" s="4">
         <v>0</v>
       </c>
-      <c r="C4" s="2" t="s">
+      <c r="C4" s="4" t="s">
         <v>111</v>
       </c>
-      <c r="D4" s="5" t="s">
+      <c r="D4" s="15" t="s">
         <v>14</v>
       </c>
-      <c r="E4" s="2" t="s">
+      <c r="E4" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="F4" s="2">
+      <c r="F4" s="4">
         <v>12</v>
       </c>
-      <c r="G4" s="5" t="s">
+      <c r="G4" s="15" t="s">
         <v>112</v>
       </c>
-      <c r="H4" s="2"/>
-      <c r="I4" s="2"/>
-      <c r="J4" s="2" t="s">
+      <c r="H4" s="4"/>
+      <c r="I4" s="4"/>
+      <c r="J4" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="K4" s="2">
+      <c r="K4" s="4">
         <v>1</v>
       </c>
-      <c r="L4" s="2" t="s">
+      <c r="L4" s="4" t="s">
         <v>107</v>
       </c>
-      <c r="M4" s="2" t="s">
+      <c r="M4" s="4" t="s">
         <v>111</v>
       </c>
-      <c r="N4" s="2" t="s">
+      <c r="N4" s="4" t="s">
         <v>111</v>
       </c>
-      <c r="O4" s="7" t="s">
+      <c r="O4" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="P4" s="7" t="s">
+      <c r="P4" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="Q4" s="7" t="s">
+      <c r="Q4" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="R4" s="2" t="s">
+      <c r="R4" s="4" t="s">
         <v>108</v>
       </c>
-      <c r="S4" s="10" t="s">
+      <c r="S4" s="19" t="s">
         <v>109</v>
       </c>
     </row>
     <row r="5" spans="1:19">
-      <c r="A5" s="2" t="s">
+      <c r="A5" s="4" t="s">
         <v>113</v>
       </c>
-      <c r="B5" s="5">
+      <c r="B5" s="15">
         <v>0</v>
       </c>
-      <c r="C5" s="2" t="s">
+      <c r="C5" s="4" t="s">
         <v>113</v>
       </c>
-      <c r="D5" s="5" t="s">
+      <c r="D5" s="15" t="s">
         <v>14</v>
       </c>
-      <c r="E5" s="2">
+      <c r="E5" s="4">
         <v>75052200</v>
       </c>
-      <c r="F5" s="5">
+      <c r="F5" s="15">
         <v>5</v>
       </c>
-      <c r="G5" s="5" t="s">
+      <c r="G5" s="15" t="s">
         <v>112</v>
       </c>
-      <c r="H5" s="2"/>
-      <c r="I5" s="2"/>
-      <c r="J5" s="5" t="s">
+      <c r="H5" s="4"/>
+      <c r="I5" s="4"/>
+      <c r="J5" s="15" t="s">
         <v>20</v>
       </c>
-      <c r="K5" s="5">
+      <c r="K5" s="15">
         <v>2</v>
       </c>
-      <c r="L5" s="2" t="s">
+      <c r="L5" s="4" t="s">
         <v>107</v>
       </c>
-      <c r="M5" s="2" t="s">
+      <c r="M5" s="4" t="s">
         <v>113</v>
       </c>
-      <c r="N5" s="2" t="s">
+      <c r="N5" s="4" t="s">
         <v>113</v>
       </c>
-      <c r="O5" s="7" t="s">
+      <c r="O5" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="P5" s="7" t="s">
+      <c r="P5" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="Q5" s="7" t="s">
+      <c r="Q5" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="R5" s="2" t="s">
+      <c r="R5" s="4" t="s">
         <v>114</v>
       </c>
-      <c r="S5" s="10" t="s">
+      <c r="S5" s="19" t="s">
         <v>109</v>
       </c>
     </row>
     <row r="6" spans="1:19">
-      <c r="A6" s="5" t="s">
+      <c r="A6" s="15" t="s">
         <v>115</v>
       </c>
-      <c r="B6" s="5">
+      <c r="B6" s="15">
         <v>0</v>
       </c>
-      <c r="C6" s="2" t="s">
+      <c r="C6" s="4" t="s">
         <v>115</v>
       </c>
-      <c r="D6" s="5" t="s">
+      <c r="D6" s="15" t="s">
         <v>14</v>
       </c>
-      <c r="E6" s="5" t="s">
+      <c r="E6" s="15" t="s">
         <v>40</v>
       </c>
-      <c r="F6" s="5">
+      <c r="F6" s="15">
         <v>12</v>
       </c>
-      <c r="G6" s="5" t="s">
+      <c r="G6" s="15" t="s">
         <v>116</v>
       </c>
-      <c r="H6" s="5" t="s">
+      <c r="H6" s="15" t="s">
         <v>117</v>
       </c>
-      <c r="I6" s="2"/>
-      <c r="J6" s="5" t="s">
+      <c r="I6" s="4"/>
+      <c r="J6" s="15" t="s">
         <v>14</v>
       </c>
-      <c r="K6" s="5">
+      <c r="K6" s="15">
         <v>1</v>
       </c>
-      <c r="L6" s="2" t="s">
+      <c r="L6" s="4" t="s">
         <v>107</v>
       </c>
-      <c r="M6" s="5" t="s">
+      <c r="M6" s="15" t="s">
         <v>115</v>
       </c>
-      <c r="N6" s="5" t="s">
+      <c r="N6" s="15" t="s">
         <v>115</v>
       </c>
-      <c r="O6" s="7" t="s">
+      <c r="O6" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="P6" s="7" t="s">
+      <c r="P6" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="Q6" s="7" t="s">
+      <c r="Q6" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="R6" s="2" t="s">
+      <c r="R6" s="4" t="s">
         <v>108</v>
       </c>
-      <c r="S6" s="10" t="s">
+      <c r="S6" s="19" t="s">
         <v>109</v>
       </c>
     </row>
     <row r="7" spans="1:19">
-      <c r="A7" s="5" t="s">
+      <c r="A7" s="15" t="s">
         <v>118</v>
       </c>
-      <c r="B7" s="5">
+      <c r="B7" s="15">
         <v>0</v>
       </c>
-      <c r="C7" s="2" t="s">
+      <c r="C7" s="4" t="s">
         <v>118</v>
       </c>
-      <c r="D7" s="5" t="s">
+      <c r="D7" s="15" t="s">
         <v>14</v>
       </c>
-      <c r="E7" s="5" t="s">
+      <c r="E7" s="15" t="s">
         <v>40</v>
       </c>
-      <c r="F7" s="5">
+      <c r="F7" s="15">
         <v>12</v>
       </c>
-      <c r="G7" s="5" t="s">
+      <c r="G7" s="15" t="s">
         <v>116</v>
       </c>
-      <c r="H7" s="5" t="s">
+      <c r="H7" s="15" t="s">
         <v>119</v>
       </c>
-      <c r="I7" s="2"/>
-      <c r="J7" s="5" t="s">
+      <c r="I7" s="4"/>
+      <c r="J7" s="15" t="s">
         <v>20</v>
       </c>
-      <c r="K7" s="5">
+      <c r="K7" s="15">
         <v>4</v>
       </c>
-      <c r="L7" s="2" t="s">
+      <c r="L7" s="4" t="s">
         <v>107</v>
       </c>
-      <c r="M7" s="5" t="s">
+      <c r="M7" s="15" t="s">
         <v>118</v>
       </c>
-      <c r="N7" s="5" t="s">
+      <c r="N7" s="15" t="s">
         <v>118</v>
       </c>
-      <c r="O7" s="7" t="s">
+      <c r="O7" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="P7" s="7" t="s">
+      <c r="P7" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="Q7" s="7" t="s">
+      <c r="Q7" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="R7" s="2" t="s">
+      <c r="R7" s="4" t="s">
         <v>108</v>
       </c>
-      <c r="S7" s="10" t="s">
+      <c r="S7" s="19" t="s">
         <v>109</v>
       </c>
     </row>
     <row r="8" spans="1:19">
-      <c r="A8" s="2" t="s">
+      <c r="A8" s="4" t="s">
         <v>120</v>
       </c>
-      <c r="B8" s="5">
+      <c r="B8" s="15">
         <v>0</v>
       </c>
-      <c r="C8" s="2" t="s">
+      <c r="C8" s="4" t="s">
         <v>120</v>
       </c>
-      <c r="D8" s="5" t="s">
+      <c r="D8" s="15" t="s">
         <v>14</v>
       </c>
-      <c r="E8" s="2" t="s">
+      <c r="E8" s="4" t="s">
         <v>121</v>
       </c>
-      <c r="F8" s="5">
+      <c r="F8" s="15">
         <v>5</v>
       </c>
-      <c r="G8" s="5" t="s">
+      <c r="G8" s="15" t="s">
         <v>122</v>
       </c>
-      <c r="H8" s="2"/>
-      <c r="I8" s="2">
+      <c r="H8" s="4"/>
+      <c r="I8" s="4">
         <v>95</v>
       </c>
-      <c r="J8" s="5" t="s">
+      <c r="J8" s="15" t="s">
         <v>14</v>
       </c>
-      <c r="K8" s="5">
+      <c r="K8" s="15">
         <v>1</v>
       </c>
-      <c r="L8" s="2" t="s">
+      <c r="L8" s="4" t="s">
         <v>107</v>
       </c>
-      <c r="M8" s="2" t="s">
+      <c r="M8" s="4" t="s">
         <v>120</v>
       </c>
-      <c r="N8" s="2" t="s">
+      <c r="N8" s="4" t="s">
         <v>120</v>
       </c>
-      <c r="O8" s="7" t="s">
+      <c r="O8" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="P8" s="7" t="s">
+      <c r="P8" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="Q8" s="7" t="s">
+      <c r="Q8" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="R8" s="2" t="s">
+      <c r="R8" s="4" t="s">
         <v>108</v>
       </c>
-      <c r="S8" s="10" t="s">
+      <c r="S8" s="19" t="s">
         <v>109</v>
       </c>
     </row>
     <row r="9" spans="1:19">
-      <c r="A9" s="5" t="s">
+      <c r="A9" s="15" t="s">
         <v>123</v>
       </c>
-      <c r="B9" s="5">
+      <c r="B9" s="15">
         <v>0</v>
       </c>
-      <c r="C9" s="2" t="s">
+      <c r="C9" s="4" t="s">
         <v>123</v>
       </c>
-      <c r="D9" s="5" t="s">
+      <c r="D9" s="15" t="s">
         <v>14</v>
       </c>
-      <c r="E9" s="5" t="s">
+      <c r="E9" s="15" t="s">
         <v>40</v>
       </c>
-      <c r="F9" s="5">
+      <c r="F9" s="15">
         <v>12</v>
       </c>
-      <c r="G9" s="5" t="s">
+      <c r="G9" s="15" t="s">
         <v>122</v>
       </c>
-      <c r="H9" s="2"/>
-      <c r="I9" s="2">
+      <c r="H9" s="4"/>
+      <c r="I9" s="4">
         <v>97</v>
       </c>
-      <c r="J9" s="5" t="s">
+      <c r="J9" s="15" t="s">
         <v>20</v>
       </c>
-      <c r="K9" s="5">
+      <c r="K9" s="15">
         <v>4</v>
       </c>
-      <c r="L9" s="2" t="s">
+      <c r="L9" s="4" t="s">
         <v>107</v>
       </c>
-      <c r="M9" s="5" t="s">
+      <c r="M9" s="15" t="s">
         <v>123</v>
       </c>
-      <c r="N9" s="5" t="s">
+      <c r="N9" s="15" t="s">
         <v>123</v>
       </c>
-      <c r="O9" s="7" t="s">
+      <c r="O9" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="P9" s="7" t="s">
+      <c r="P9" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="Q9" s="7" t="s">
+      <c r="Q9" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="R9" s="2" t="s">
+      <c r="R9" s="4" t="s">
         <v>108</v>
       </c>
-      <c r="S9" s="10" t="s">
+      <c r="S9" s="19" t="s">
         <v>109</v>
       </c>
     </row>
     <row r="10" spans="1:19">
-      <c r="A10" s="2" t="s">
+      <c r="A10" s="4" t="s">
         <v>124</v>
       </c>
-      <c r="B10" s="2">
+      <c r="B10" s="4">
         <v>0</v>
       </c>
-      <c r="C10" s="2" t="s">
+      <c r="C10" s="4" t="s">
         <v>124</v>
       </c>
-      <c r="D10" s="2" t="s">
+      <c r="D10" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="E10" s="2" t="s">
+      <c r="E10" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="F10" s="2">
+      <c r="F10" s="4">
         <v>12</v>
       </c>
-      <c r="G10" s="2" t="s">
+      <c r="G10" s="4" t="s">
         <v>125</v>
       </c>
-      <c r="H10" s="2"/>
-      <c r="I10" s="2"/>
-      <c r="J10" s="2" t="s">
+      <c r="H10" s="4"/>
+      <c r="I10" s="4"/>
+      <c r="J10" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="K10" s="2">
+      <c r="K10" s="4">
         <v>1</v>
       </c>
-      <c r="L10" s="2" t="s">
+      <c r="L10" s="4" t="s">
         <v>107</v>
       </c>
-      <c r="M10" s="2" t="s">
+      <c r="M10" s="4" t="s">
         <v>124</v>
       </c>
-      <c r="N10" s="2" t="s">
+      <c r="N10" s="4" t="s">
         <v>124</v>
       </c>
-      <c r="O10" s="2" t="s">
+      <c r="O10" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="P10" s="2" t="s">
+      <c r="P10" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="Q10" s="2" t="s">
+      <c r="Q10" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="R10" s="2" t="s">
+      <c r="R10" s="4" t="s">
         <v>108</v>
       </c>
-      <c r="S10" s="2" t="s">
+      <c r="S10" s="4" t="s">
         <v>109</v>
       </c>
     </row>
     <row r="11" spans="1:19">
-      <c r="A11" s="2" t="s">
+      <c r="A11" s="4" t="s">
         <v>126</v>
       </c>
-      <c r="B11" s="2">
+      <c r="B11" s="4">
         <v>0</v>
       </c>
-      <c r="C11" s="2" t="s">
+      <c r="C11" s="4" t="s">
         <v>126</v>
       </c>
-      <c r="D11" s="2" t="s">
+      <c r="D11" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="E11" s="2" t="s">
+      <c r="E11" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="F11" s="2">
+      <c r="F11" s="4">
         <v>12</v>
       </c>
-      <c r="G11" s="2" t="s">
+      <c r="G11" s="4" t="s">
         <v>125</v>
       </c>
-      <c r="H11" s="2"/>
-      <c r="I11" s="2"/>
-      <c r="J11" s="2" t="s">
+      <c r="H11" s="4"/>
+      <c r="I11" s="4"/>
+      <c r="J11" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="K11" s="2">
+      <c r="K11" s="4">
         <v>4</v>
       </c>
-      <c r="L11" s="2" t="s">
+      <c r="L11" s="4" t="s">
         <v>107</v>
       </c>
-      <c r="M11" s="2" t="s">
+      <c r="M11" s="4" t="s">
         <v>126</v>
       </c>
-      <c r="N11" s="2" t="s">
+      <c r="N11" s="4" t="s">
         <v>126</v>
       </c>
-      <c r="O11" s="2" t="s">
+      <c r="O11" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="P11" s="2" t="s">
+      <c r="P11" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="Q11" s="2" t="s">
+      <c r="Q11" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="R11" s="2" t="s">
+      <c r="R11" s="4" t="s">
         <v>108</v>
       </c>
-      <c r="S11" s="2" t="s">
+      <c r="S11" s="4" t="s">
         <v>109</v>
       </c>
     </row>

</xml_diff>

<commit_message>
FIXES FOR RFQ AND PAYROLL SCREEN FAILED TEST SCENARIOS
FIXES FOR RFQ AND PAYROLL SCREEN FAILED TEST SCENARIOS
</commit_message>
<xml_diff>
--- a/testdata/ItemDetails.xlsx
+++ b/testdata/ItemDetails.xlsx
@@ -1,10 +1,10 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
+  <fileVersion appName="xl" lastEdited="4" lowestEdited="5" rupBuild="4505"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="23040" windowHeight="9120" firstSheet="17" activeTab="19"/>
+    <workbookView xWindow="0" yWindow="2520" windowWidth="15150" windowHeight="6540" firstSheet="21" activeTab="25"/>
   </bookViews>
   <sheets>
     <sheet name="PR Details" sheetId="1" r:id="rId1"/>
@@ -30,8 +30,12 @@
     <sheet name="SimilarItem" sheetId="21" r:id="rId21"/>
     <sheet name="POAServiceSheet" sheetId="22" r:id="rId22"/>
     <sheet name="DIS_UOM_MAT_UD" sheetId="23" r:id="rId23"/>
+    <sheet name="PRMULTI" sheetId="24" r:id="rId24"/>
+    <sheet name="RFQ" sheetId="25" r:id="rId25"/>
+    <sheet name="RFQDOM" sheetId="26" r:id="rId26"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="124519"/>
+  <oleSize ref="A1:O20"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -49,7 +53,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="699" uniqueCount="239">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="716" uniqueCount="248">
   <si>
     <t>ITEM_NAME</t>
   </si>
@@ -767,19 +771,40 @@
   </si>
   <si>
     <t>RML2</t>
+  </si>
+  <si>
+    <t>ITEM</t>
+  </si>
+  <si>
+    <t>COST</t>
+  </si>
+  <si>
+    <t>TVS-RM-KDK-01</t>
+  </si>
+  <si>
+    <t>TVS-RM-KDK-02</t>
+  </si>
+  <si>
+    <t>Supplier</t>
+  </si>
+  <si>
+    <t>Curr</t>
+  </si>
+  <si>
+    <t>AFT PRIVATE LIMITED</t>
+  </si>
+  <si>
+    <t>ARAVIND AGENCY</t>
+  </si>
+  <si>
+    <t>JJ AUTOMOBILES</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="xr9">
-  <numFmts count="4">
-    <numFmt numFmtId="176" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
-    <numFmt numFmtId="177" formatCode="_ &quot;₹&quot;* #,##0.00_ ;_ &quot;₹&quot;* \-#,##0.00_ ;_ &quot;₹&quot;* &quot;-&quot;??_ ;_ @_ "/>
-    <numFmt numFmtId="178" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
-    <numFmt numFmtId="179" formatCode="_ &quot;₹&quot;* #,##0_ ;_ &quot;₹&quot;* \-#,##0_ ;_ &quot;₹&quot;* &quot;-&quot;_ ;_ @_ "/>
-  </numFmts>
-  <fonts count="29">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <fonts count="11">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -846,151 +871,14 @@
       <charset val="134"/>
     </font>
     <font>
-      <u/>
       <sz val="11"/>
-      <color rgb="FF0000FF"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <u/>
-      <sz val="11"/>
-      <color rgb="FF800080"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FFFF0000"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="18"/>
-      <color theme="3"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <charset val="134"/>
       <scheme val="minor"/>
     </font>
-    <font>
-      <i/>
-      <sz val="11"/>
-      <color rgb="FF7F7F7F"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="15"/>
-      <color theme="3"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="13"/>
-      <color theme="3"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="3"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF3F3F76"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FF3F3F3F"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FFFA7D00"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FFFFFFFF"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FFFA7D00"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF006100"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF9C0006"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF9C6500"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="0"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
   </fonts>
-  <fills count="35">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -999,7 +887,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.599993896298105"/>
+        <fgColor theme="9" tint="0.59999389629810485"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1015,188 +903,8 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFFCC"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFCC99"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFF2F2F2"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFA5A5A5"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFC6EFCE"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFC7CE"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFEB9C"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
   </fills>
-  <borders count="10">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -1219,257 +927,15 @@
       </bottom>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color rgb="FFB2B2B2"/>
-      </left>
-      <right style="thin">
-        <color rgb="FFB2B2B2"/>
-      </right>
-      <top style="thin">
-        <color rgb="FFB2B2B2"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FFB2B2B2"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="medium">
-        <color theme="4"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="medium">
-        <color theme="4" tint="0.499984740745262"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF7F7F7F"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF7F7F7F"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF7F7F7F"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF7F7F7F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF3F3F3F"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF3F3F3F"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF3F3F3F"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF3F3F3F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="double">
-        <color rgb="FF3F3F3F"/>
-      </left>
-      <right style="double">
-        <color rgb="FF3F3F3F"/>
-      </right>
-      <top style="double">
-        <color rgb="FF3F3F3F"/>
-      </top>
-      <bottom style="double">
-        <color rgb="FF3F3F3F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="double">
-        <color rgb="FFFF8001"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color theme="4"/>
-      </top>
-      <bottom style="double">
-        <color theme="4"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
-  <cellStyleXfs count="51">
+  <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="176" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="177" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="178" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="179" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="2" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="6" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="7" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="7" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="8" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
@@ -1498,19 +964,19 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="50" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="49" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="50" applyFont="1" applyBorder="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="2" applyFont="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="50" applyBorder="1">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="2" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1">
@@ -1554,10 +1020,10 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="49" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="49" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -1576,91 +1042,160 @@
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
-  <cellStyles count="51">
+  <cellStyles count="3">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Comma" xfId="1" builtinId="3"/>
-    <cellStyle name="Currency" xfId="2" builtinId="4"/>
-    <cellStyle name="Percent" xfId="3" builtinId="5"/>
-    <cellStyle name="Comma [0]" xfId="4" builtinId="6"/>
-    <cellStyle name="Currency [0]" xfId="5" builtinId="7"/>
-    <cellStyle name="Hyperlink" xfId="6" builtinId="8"/>
-    <cellStyle name="Followed Hyperlink" xfId="7" builtinId="9"/>
-    <cellStyle name="Note" xfId="8" builtinId="10"/>
-    <cellStyle name="Warning Text" xfId="9" builtinId="11"/>
-    <cellStyle name="Title" xfId="10" builtinId="15"/>
-    <cellStyle name="CExplanatory Text" xfId="11" builtinId="53"/>
-    <cellStyle name="Heading 1" xfId="12" builtinId="16"/>
-    <cellStyle name="Heading 2" xfId="13" builtinId="17"/>
-    <cellStyle name="Heading 3" xfId="14" builtinId="18"/>
-    <cellStyle name="Heading 4" xfId="15" builtinId="19"/>
-    <cellStyle name="Input" xfId="16" builtinId="20"/>
-    <cellStyle name="Output" xfId="17" builtinId="21"/>
-    <cellStyle name="Calculation" xfId="18" builtinId="22"/>
-    <cellStyle name="Check Cell" xfId="19" builtinId="23"/>
-    <cellStyle name="Linked Cell" xfId="20" builtinId="24"/>
-    <cellStyle name="Total" xfId="21" builtinId="25"/>
-    <cellStyle name="Good" xfId="22" builtinId="26"/>
-    <cellStyle name="Bad" xfId="23" builtinId="27"/>
-    <cellStyle name="Neutral" xfId="24" builtinId="28"/>
-    <cellStyle name="Accent1" xfId="25" builtinId="29"/>
-    <cellStyle name="20% - Accent1" xfId="26" builtinId="30"/>
-    <cellStyle name="40% - Accent1" xfId="27" builtinId="31"/>
-    <cellStyle name="60% - Accent1" xfId="28" builtinId="32"/>
-    <cellStyle name="Accent2" xfId="29" builtinId="33"/>
-    <cellStyle name="20% - Accent2" xfId="30" builtinId="34"/>
-    <cellStyle name="40% - Accent2" xfId="31" builtinId="35"/>
-    <cellStyle name="60% - Accent2" xfId="32" builtinId="36"/>
-    <cellStyle name="Accent3" xfId="33" builtinId="37"/>
-    <cellStyle name="20% - Accent3" xfId="34" builtinId="38"/>
-    <cellStyle name="40% - Accent3" xfId="35" builtinId="39"/>
-    <cellStyle name="60% - Accent3" xfId="36" builtinId="40"/>
-    <cellStyle name="Accent4" xfId="37" builtinId="41"/>
-    <cellStyle name="20% - Accent4" xfId="38" builtinId="42"/>
-    <cellStyle name="40% - Accent4" xfId="39" builtinId="43"/>
-    <cellStyle name="60% - Accent4" xfId="40" builtinId="44"/>
-    <cellStyle name="Accent5" xfId="41" builtinId="45"/>
-    <cellStyle name="20% - Accent5" xfId="42" builtinId="46"/>
-    <cellStyle name="40% - Accent5" xfId="43" builtinId="47"/>
-    <cellStyle name="60% - Accent5" xfId="44" builtinId="48"/>
-    <cellStyle name="Accent6" xfId="45" builtinId="49"/>
-    <cellStyle name="20% - Accent6" xfId="46" builtinId="50"/>
-    <cellStyle name="40% - Accent6" xfId="47" builtinId="51"/>
-    <cellStyle name="60% - Accent6" xfId="48" builtinId="52"/>
-    <cellStyle name="Normal 2" xfId="49"/>
-    <cellStyle name="Normal 3" xfId="50"/>
+    <cellStyle name="Normal 2" xfId="1"/>
+    <cellStyle name="Normal 3" xfId="2"/>
   </cellStyles>
   <dxfs count="17">
     <dxf>
       <fill>
         <patternFill patternType="solid">
-          <fgColor theme="4" tint="0.799981688894314"/>
-          <bgColor theme="4" tint="0.799981688894314"/>
+          <fgColor theme="4" tint="0.79995117038483843"/>
+          <bgColor theme="4" tint="0.79995117038483843"/>
+        </patternFill>
+      </fill>
+      <border>
+        <bottom style="thin">
+          <color theme="4" tint="0.39994506668294322"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor theme="4" tint="0.79995117038483843"/>
+          <bgColor theme="4" tint="0.79995117038483843"/>
+        </patternFill>
+      </fill>
+      <border>
+        <bottom style="thin">
+          <color theme="4" tint="0.39994506668294322"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="1"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="1"/>
+      </font>
+      <border>
+        <bottom style="thin">
+          <color theme="4" tint="0.39994506668294322"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <color theme="1"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <color theme="1"/>
+      </font>
+      <border>
+        <top style="thin">
+          <color theme="4"/>
+        </top>
+        <bottom style="thin">
+          <color theme="4"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor theme="4" tint="0.79995117038483843"/>
+          <bgColor theme="4" tint="0.79995117038483843"/>
         </patternFill>
       </fill>
     </dxf>
     <dxf>
       <fill>
         <patternFill patternType="solid">
-          <fgColor theme="4" tint="0.799981688894314"/>
-          <bgColor theme="4" tint="0.799981688894314"/>
+          <fgColor theme="4" tint="0.79995117038483843"/>
+          <bgColor theme="4" tint="0.79995117038483843"/>
         </patternFill>
       </fill>
     </dxf>
     <dxf>
       <font>
-        <b val="1"/>
+        <b/>
+        <color theme="1"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor theme="4" tint="0.79995117038483843"/>
+          <bgColor theme="4" tint="0.79995117038483843"/>
+        </patternFill>
+      </fill>
+      <border>
+        <top style="thin">
+          <color theme="4" tint="0.39994506668294322"/>
+        </top>
+        <bottom style="thin">
+          <color theme="4" tint="0.39994506668294322"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <color theme="1"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor theme="4" tint="0.79995117038483843"/>
+          <bgColor theme="4" tint="0.79995117038483843"/>
+        </patternFill>
+      </fill>
+      <border>
+        <bottom style="thin">
+          <color theme="4" tint="0.39994506668294322"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor theme="4" tint="0.79995117038483843"/>
+          <bgColor theme="4" tint="0.79995117038483843"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor theme="4" tint="0.79995117038483843"/>
+          <bgColor theme="4" tint="0.79995117038483843"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
         <color theme="1"/>
       </font>
     </dxf>
     <dxf>
       <font>
-        <b val="1"/>
+        <b/>
         <color theme="1"/>
       </font>
     </dxf>
     <dxf>
       <font>
-        <b val="1"/>
+        <b/>
         <color theme="1"/>
       </font>
       <border>
@@ -1671,7 +1206,7 @@
     </dxf>
     <dxf>
       <font>
-        <b val="1"/>
+        <b/>
         <color theme="0"/>
       </font>
       <fill>
@@ -1699,149 +1234,32 @@
           <color theme="4"/>
         </bottom>
         <horizontal style="thin">
-          <color theme="4" tint="0.399975585192419"/>
+          <color theme="4" tint="0.39994506668294322"/>
         </horizontal>
-      </border>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor theme="4" tint="0.799981688894314"/>
-          <bgColor theme="4" tint="0.799981688894314"/>
-        </patternFill>
-      </fill>
-      <border>
-        <bottom style="thin">
-          <color theme="4" tint="0.399975585192419"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="1"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor theme="4" tint="0.799981688894314"/>
-          <bgColor theme="4" tint="0.799981688894314"/>
-        </patternFill>
-      </fill>
-      <border>
-        <bottom style="thin">
-          <color theme="4" tint="0.399975585192419"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="1"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="1"/>
-      </font>
-      <border>
-        <bottom style="thin">
-          <color theme="4" tint="0.399975585192419"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="1"/>
-        <color theme="1"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="1"/>
-        <color theme="1"/>
-      </font>
-      <border>
-        <top style="thin">
-          <color theme="4"/>
-        </top>
-        <bottom style="thin">
-          <color theme="4"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor theme="4" tint="0.799981688894314"/>
-          <bgColor theme="4" tint="0.799981688894314"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor theme="4" tint="0.799981688894314"/>
-          <bgColor theme="4" tint="0.799981688894314"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="1"/>
-        <color theme="1"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor theme="4" tint="0.799981688894314"/>
-          <bgColor theme="4" tint="0.799981688894314"/>
-        </patternFill>
-      </fill>
-      <border>
-        <top style="thin">
-          <color theme="4" tint="0.399975585192419"/>
-        </top>
-        <bottom style="thin">
-          <color theme="4" tint="0.399975585192419"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="1"/>
-        <color theme="1"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor theme="4" tint="0.799981688894314"/>
-          <bgColor theme="4" tint="0.799981688894314"/>
-        </patternFill>
-      </fill>
-      <border>
-        <bottom style="thin">
-          <color theme="4" tint="0.399975585192419"/>
-        </bottom>
       </border>
     </dxf>
   </dxfs>
   <tableStyles count="2" defaultTableStyle="TableStylePreset3_Accent1" defaultPivotStyle="PivotStylePreset2_Accent1">
-    <tableStyle name="TableStylePreset3_Accent1" pivot="0" count="7" xr9:uid="{59DB682C-5494-4EDE-A608-00C9E5F0F923}">
-      <tableStyleElement type="wholeTable" dxfId="6"/>
-      <tableStyleElement type="headerRow" dxfId="5"/>
-      <tableStyleElement type="totalRow" dxfId="4"/>
-      <tableStyleElement type="firstColumn" dxfId="3"/>
-      <tableStyleElement type="lastColumn" dxfId="2"/>
-      <tableStyleElement type="firstRowStripe" dxfId="1"/>
-      <tableStyleElement type="firstColumnStripe" dxfId="0"/>
+    <tableStyle name="TableStylePreset3_Accent1" pivot="0" count="7">
+      <tableStyleElement type="wholeTable" dxfId="16"/>
+      <tableStyleElement type="headerRow" dxfId="15"/>
+      <tableStyleElement type="totalRow" dxfId="14"/>
+      <tableStyleElement type="firstColumn" dxfId="13"/>
+      <tableStyleElement type="lastColumn" dxfId="12"/>
+      <tableStyleElement type="firstRowStripe" dxfId="11"/>
+      <tableStyleElement type="firstColumnStripe" dxfId="10"/>
     </tableStyle>
-    <tableStyle name="PivotStylePreset2_Accent1" table="0" count="10" xr9:uid="{267968C8-6FFD-4C36-ACC1-9EA1FD1885CA}">
-      <tableStyleElement type="headerRow" dxfId="16"/>
-      <tableStyleElement type="totalRow" dxfId="15"/>
-      <tableStyleElement type="firstRowStripe" dxfId="14"/>
-      <tableStyleElement type="firstColumnStripe" dxfId="13"/>
-      <tableStyleElement type="firstSubtotalRow" dxfId="12"/>
-      <tableStyleElement type="secondSubtotalRow" dxfId="11"/>
-      <tableStyleElement type="firstRowSubheading" dxfId="10"/>
-      <tableStyleElement type="secondRowSubheading" dxfId="9"/>
-      <tableStyleElement type="pageFieldLabels" dxfId="8"/>
-      <tableStyleElement type="pageFieldValues" dxfId="7"/>
+    <tableStyle name="PivotStylePreset2_Accent1" table="0" count="10">
+      <tableStyleElement type="headerRow" dxfId="9"/>
+      <tableStyleElement type="totalRow" dxfId="8"/>
+      <tableStyleElement type="firstRowStripe" dxfId="7"/>
+      <tableStyleElement type="firstColumnStripe" dxfId="6"/>
+      <tableStyleElement type="firstSubtotalRow" dxfId="5"/>
+      <tableStyleElement type="secondSubtotalRow" dxfId="4"/>
+      <tableStyleElement type="firstRowSubheading" dxfId="3"/>
+      <tableStyleElement type="secondRowSubheading" dxfId="2"/>
+      <tableStyleElement type="pageFieldLabels" dxfId="1"/>
+      <tableStyleElement type="pageFieldValues" dxfId="0"/>
     </tableStyle>
   </tableStyles>
   <extLst>
@@ -2104,23 +1522,23 @@
     </a:fmtScheme>
   </a:themeElements>
   <a:objectDefaults/>
+  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
-  <sheetPr/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:J20"/>
-  <sheetFormatPr defaultColWidth="8.71296296296296" defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="20.712962962963" customWidth="1"/>
-    <col min="2" max="3" width="12.712962962963" customWidth="1"/>
-    <col min="4" max="4" width="14.712962962963" customWidth="1"/>
-    <col min="5" max="5" width="9.85185185185185" customWidth="1"/>
-    <col min="6" max="6" width="14.1388888888889" customWidth="1"/>
-    <col min="7" max="7" width="14.8518518518519" customWidth="1"/>
-    <col min="8" max="8" width="22.287037037037" customWidth="1"/>
-    <col min="9" max="9" width="14.4259259259259" customWidth="1"/>
+    <col min="1" max="1" width="20.7109375" customWidth="1"/>
+    <col min="2" max="3" width="12.7109375" customWidth="1"/>
+    <col min="4" max="4" width="14.7109375" customWidth="1"/>
+    <col min="5" max="5" width="9.85546875" customWidth="1"/>
+    <col min="6" max="6" width="14.140625" customWidth="1"/>
+    <col min="7" max="7" width="14.85546875" customWidth="1"/>
+    <col min="8" max="8" width="22.28515625" customWidth="1"/>
+    <col min="9" max="9" width="14.42578125" customWidth="1"/>
     <col min="10" max="10" width="13" customWidth="1"/>
   </cols>
   <sheetData>
@@ -2156,7 +1574,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="2" s="30" customFormat="1" ht="20.4" spans="1:10">
+    <row r="2" spans="1:10" s="30" customFormat="1" ht="22.5">
       <c r="A2" s="32" t="s">
         <v>10</v>
       </c>
@@ -2188,7 +1606,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="3" ht="15" customHeight="1" spans="1:10">
+    <row r="3" spans="1:10" ht="15" customHeight="1">
       <c r="A3" s="32" t="s">
         <v>18</v>
       </c>
@@ -2220,7 +1638,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="4" spans="1:10">
+    <row r="4" spans="1:10" ht="22.5">
       <c r="A4" s="32" t="s">
         <v>21</v>
       </c>
@@ -2446,27 +1864,25 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
-  <sheetPr/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:K5"/>
-  <sheetFormatPr defaultColWidth="8.85185185185185" defaultRowHeight="14.4" outlineLevelRow="4"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="9" customWidth="1"/>
-    <col min="2" max="2" width="25.712962962963" customWidth="1"/>
-    <col min="3" max="3" width="12.4259259259259" customWidth="1"/>
-    <col min="4" max="4" width="16.287037037037" customWidth="1"/>
-    <col min="5" max="5" width="20.287037037037" customWidth="1"/>
-    <col min="6" max="6" width="25.712962962963" customWidth="1"/>
-    <col min="7" max="7" width="12.287037037037" customWidth="1"/>
-    <col min="8" max="8" width="14.5740740740741" customWidth="1"/>
-    <col min="9" max="9" width="28.5740740740741" customWidth="1"/>
+    <col min="2" max="2" width="25.7109375" customWidth="1"/>
+    <col min="3" max="3" width="12.42578125" customWidth="1"/>
+    <col min="4" max="4" width="16.28515625" customWidth="1"/>
+    <col min="5" max="5" width="20.28515625" customWidth="1"/>
+    <col min="6" max="6" width="25.7109375" customWidth="1"/>
+    <col min="7" max="7" width="12.28515625" customWidth="1"/>
+    <col min="8" max="8" width="14.5703125" customWidth="1"/>
+    <col min="9" max="9" width="28.5703125" customWidth="1"/>
     <col min="10" max="10" width="23" customWidth="1"/>
-    <col min="11" max="11" width="14.712962962963" customWidth="1"/>
+    <col min="11" max="11" width="14.7109375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:11">
@@ -2646,21 +2062,19 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
-  <sheetPr/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:E4"/>
-  <sheetFormatPr defaultColWidth="8.85185185185185" defaultRowHeight="14.4" outlineLevelRow="3" outlineLevelCol="4"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="13.5740740740741" customWidth="1"/>
+    <col min="1" max="1" width="13.5703125" customWidth="1"/>
     <col min="2" max="2" width="6" customWidth="1"/>
-    <col min="3" max="3" width="14.4259259259259" customWidth="1"/>
-    <col min="4" max="4" width="18.1388888888889" customWidth="1"/>
-    <col min="5" max="5" width="19.5740740740741" customWidth="1"/>
+    <col min="3" max="3" width="14.42578125" customWidth="1"/>
+    <col min="4" max="4" width="18.140625" customWidth="1"/>
+    <col min="5" max="5" width="19.5703125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5">
@@ -2680,7 +2094,7 @@
         <v>180</v>
       </c>
     </row>
-    <row r="2" spans="1:5">
+    <row r="2" spans="1:5" ht="30">
       <c r="A2" s="7" t="s">
         <v>181</v>
       </c>
@@ -2733,23 +2147,21 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
-  <sheetPr/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:G11"/>
-  <sheetFormatPr defaultColWidth="8.85185185185185" defaultRowHeight="14.4" outlineLevelCol="6"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="25.712962962963" customWidth="1"/>
-    <col min="2" max="2" width="8.85185185185185" customWidth="1"/>
-    <col min="3" max="3" width="12.287037037037" customWidth="1"/>
-    <col min="4" max="4" width="7.13888888888889" customWidth="1"/>
-    <col min="5" max="5" width="5.28703703703704" customWidth="1"/>
-    <col min="6" max="6" width="17.4259259259259" customWidth="1"/>
-    <col min="7" max="7" width="12.4259259259259" customWidth="1"/>
+    <col min="1" max="1" width="25.7109375" customWidth="1"/>
+    <col min="2" max="2" width="8.85546875" customWidth="1"/>
+    <col min="3" max="3" width="12.28515625" customWidth="1"/>
+    <col min="4" max="4" width="7.140625" customWidth="1"/>
+    <col min="5" max="5" width="5.28515625" customWidth="1"/>
+    <col min="6" max="6" width="17.42578125" customWidth="1"/>
+    <col min="7" max="7" width="12.42578125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7">
@@ -3007,19 +2419,17 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
-  <sheetPr/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:C3"/>
-  <sheetFormatPr defaultColWidth="8.85185185185185" defaultRowHeight="14.4" outlineLevelRow="2" outlineLevelCol="2"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="25.5740740740741" customWidth="1"/>
-    <col min="2" max="2" width="15.1388888888889" customWidth="1"/>
-    <col min="3" max="3" width="16.4259259259259" customWidth="1"/>
+    <col min="1" max="1" width="25.5703125" customWidth="1"/>
+    <col min="2" max="2" width="15.140625" customWidth="1"/>
+    <col min="3" max="3" width="16.42578125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3">
@@ -3057,18 +2467,16 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
-  <sheetPr/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:C3"/>
-  <sheetFormatPr defaultColWidth="8.85185185185185" defaultRowHeight="14.4" outlineLevelRow="2" outlineLevelCol="2"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="21.4259259259259" customWidth="1"/>
-    <col min="2" max="2" width="11.5740740740741" customWidth="1"/>
+    <col min="1" max="1" width="21.42578125" customWidth="1"/>
+    <col min="2" max="2" width="11.5703125" customWidth="1"/>
     <col min="3" max="3" width="9" customWidth="1"/>
   </cols>
   <sheetData>
@@ -3107,17 +2515,15 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
-  <sheetPr/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:B2"/>
-  <sheetFormatPr defaultColWidth="8.71296296296296" defaultRowHeight="14.4" outlineLevelRow="1" outlineLevelCol="1"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="20.4259259259259" customWidth="1"/>
+    <col min="1" max="1" width="20.42578125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2">
@@ -3138,15 +2544,13 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
-  <sheetPr/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:G3"/>
-  <sheetFormatPr defaultColWidth="8.71296296296296" defaultRowHeight="14.4" outlineLevelRow="2" outlineLevelCol="6"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:7">
       <c r="A1" s="8" t="s">
@@ -3217,15 +2621,13 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
-  <sheetPr/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:C3"/>
-  <sheetFormatPr defaultColWidth="8.71296296296296" defaultRowHeight="14.4" outlineLevelRow="2" outlineLevelCol="2"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:3">
       <c r="A1" s="8" t="s">
@@ -3262,15 +2664,13 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
-  <sheetPr/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:B2"/>
-  <sheetFormatPr defaultColWidth="8.71296296296296" defaultRowHeight="14.4" outlineLevelRow="1" outlineLevelCol="1"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:2">
       <c r="A1" s="9" t="s">
@@ -3290,15 +2690,13 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
-  <sheetPr/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:C3"/>
-  <sheetFormatPr defaultColWidth="8.71296296296296" defaultRowHeight="14.4" outlineLevelRow="2" outlineLevelCol="2"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:3">
       <c r="A1" t="s">
@@ -3311,7 +2709,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="2" spans="1:2">
+    <row r="2" spans="1:3">
       <c r="A2" t="s">
         <v>229</v>
       </c>
@@ -3319,7 +2717,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="3" spans="1:2">
+    <row r="3" spans="1:3">
       <c r="A3" t="s">
         <v>230</v>
       </c>
@@ -3329,36 +2727,34 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
-  <sheetPr/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:T10"/>
-  <sheetFormatPr defaultColWidth="8.71296296296296" defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="30" customWidth="1"/>
-    <col min="2" max="2" width="36.4259259259259" customWidth="1"/>
+    <col min="2" max="2" width="36.42578125" customWidth="1"/>
     <col min="3" max="3" width="6" customWidth="1"/>
-    <col min="4" max="4" width="13.712962962963" customWidth="1"/>
-    <col min="5" max="5" width="5.28703703703704" customWidth="1"/>
-    <col min="6" max="6" width="17.287037037037" customWidth="1"/>
-    <col min="7" max="7" width="30.287037037037" customWidth="1"/>
-    <col min="8" max="8" width="26.8518518518519" customWidth="1"/>
-    <col min="9" max="9" width="17.287037037037" customWidth="1"/>
-    <col min="10" max="10" width="13.287037037037" customWidth="1"/>
-    <col min="11" max="11" width="22.712962962963" customWidth="1"/>
-    <col min="12" max="12" width="12.712962962963" customWidth="1"/>
-    <col min="13" max="13" width="29.5740740740741" customWidth="1"/>
-    <col min="14" max="14" width="18.287037037037" customWidth="1"/>
-    <col min="15" max="15" width="16.287037037037" customWidth="1"/>
-    <col min="16" max="16" width="15.5740740740741" customWidth="1"/>
-    <col min="17" max="17" width="17.712962962963" customWidth="1"/>
-    <col min="18" max="18" width="24.1388888888889" customWidth="1"/>
-    <col min="19" max="19" width="13.4259259259259" customWidth="1"/>
-    <col min="20" max="20" width="13.5740740740741" customWidth="1"/>
+    <col min="4" max="4" width="13.7109375" customWidth="1"/>
+    <col min="5" max="5" width="5.28515625" customWidth="1"/>
+    <col min="6" max="6" width="17.28515625" customWidth="1"/>
+    <col min="7" max="7" width="30.28515625" customWidth="1"/>
+    <col min="8" max="8" width="26.85546875" customWidth="1"/>
+    <col min="9" max="9" width="17.28515625" customWidth="1"/>
+    <col min="10" max="10" width="13.28515625" customWidth="1"/>
+    <col min="11" max="11" width="22.7109375" customWidth="1"/>
+    <col min="12" max="12" width="12.7109375" customWidth="1"/>
+    <col min="13" max="13" width="29.5703125" customWidth="1"/>
+    <col min="14" max="14" width="18.28515625" customWidth="1"/>
+    <col min="15" max="15" width="16.28515625" customWidth="1"/>
+    <col min="16" max="16" width="15.5703125" customWidth="1"/>
+    <col min="17" max="17" width="17.7109375" customWidth="1"/>
+    <col min="18" max="18" width="24.140625" customWidth="1"/>
+    <col min="19" max="19" width="13.42578125" customWidth="1"/>
+    <col min="20" max="20" width="13.5703125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:20">
@@ -3911,22 +3307,20 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
-  <sheetPr/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:F3"/>
-  <sheetFormatPr defaultColWidth="8.71296296296296" defaultRowHeight="14.4" outlineLevelRow="2" outlineLevelCol="5"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="23.2222222222222" customWidth="1"/>
-    <col min="2" max="2" width="10.4444444444444" customWidth="1"/>
-    <col min="3" max="3" width="11.4444444444444" customWidth="1"/>
-    <col min="4" max="4" width="11.6666666666667" customWidth="1"/>
-    <col min="5" max="5" width="14.5555555555556" customWidth="1"/>
-    <col min="6" max="6" width="17.6666666666667" customWidth="1"/>
+    <col min="1" max="1" width="23.28515625" customWidth="1"/>
+    <col min="2" max="2" width="10.42578125" customWidth="1"/>
+    <col min="3" max="3" width="11.42578125" customWidth="1"/>
+    <col min="4" max="4" width="11.7109375" customWidth="1"/>
+    <col min="5" max="5" width="14.5703125" customWidth="1"/>
+    <col min="6" max="6" width="17.7109375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6">
@@ -3989,22 +3383,20 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
-  <sheetPr/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:F3"/>
-  <sheetFormatPr defaultColWidth="8.88888888888889" defaultRowHeight="14.4" outlineLevelRow="2" outlineLevelCol="5"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="20.8888888888889" customWidth="1"/>
+    <col min="1" max="1" width="20.85546875" customWidth="1"/>
     <col min="2" max="2" width="9" customWidth="1"/>
-    <col min="3" max="3" width="8.88888888888889" customWidth="1"/>
-    <col min="4" max="4" width="6.11111111111111" customWidth="1"/>
-    <col min="5" max="5" width="16.7777777777778" customWidth="1"/>
-    <col min="6" max="6" width="16.2222222222222" customWidth="1"/>
+    <col min="3" max="3" width="8.85546875" customWidth="1"/>
+    <col min="4" max="4" width="6.140625" customWidth="1"/>
+    <col min="5" max="5" width="16.7109375" customWidth="1"/>
+    <col min="6" max="6" width="16.28515625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6">
@@ -4069,22 +3461,20 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
-  <sheetPr/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:F3"/>
-  <sheetFormatPr defaultColWidth="8.88888888888889" defaultRowHeight="14.4" outlineLevelRow="2" outlineLevelCol="5"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="21.6666666666667" customWidth="1"/>
+    <col min="1" max="1" width="21.7109375" customWidth="1"/>
     <col min="2" max="2" width="9" customWidth="1"/>
-    <col min="3" max="3" width="8.88888888888889" customWidth="1"/>
-    <col min="4" max="4" width="6.11111111111111" customWidth="1"/>
-    <col min="5" max="5" width="16.7777777777778" customWidth="1"/>
-    <col min="6" max="6" width="16.2222222222222" customWidth="1"/>
+    <col min="3" max="3" width="8.85546875" customWidth="1"/>
+    <col min="4" max="4" width="6.140625" customWidth="1"/>
+    <col min="5" max="5" width="16.7109375" customWidth="1"/>
+    <col min="6" max="6" width="16.28515625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6">
@@ -4149,22 +3539,20 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
-  <sheetPr/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:F3"/>
-  <sheetFormatPr defaultColWidth="8.88888888888889" defaultRowHeight="14.4" outlineLevelRow="2" outlineLevelCol="5"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="15.4444444444444" customWidth="1"/>
-    <col min="2" max="2" width="10.5555555555556" customWidth="1"/>
-    <col min="3" max="3" width="11.5555555555556" customWidth="1"/>
-    <col min="4" max="4" width="11.8888888888889" customWidth="1"/>
+    <col min="1" max="1" width="15.42578125" customWidth="1"/>
+    <col min="2" max="2" width="10.5703125" customWidth="1"/>
+    <col min="3" max="3" width="11.5703125" customWidth="1"/>
+    <col min="4" max="4" width="11.85546875" customWidth="1"/>
     <col min="5" max="5" width="14" customWidth="1"/>
-    <col min="6" max="6" width="16.8888888888889" customWidth="1"/>
+    <col min="6" max="6" width="16.85546875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6">
@@ -4229,27 +3617,136 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <headerFooter/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:C3"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1" spans="1:3">
+      <c r="A1" t="s">
+        <v>239</v>
+      </c>
+      <c r="B1" t="s">
+        <v>79</v>
+      </c>
+      <c r="C1" t="s">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3">
+      <c r="A2" t="s">
+        <v>241</v>
+      </c>
+      <c r="B2">
+        <v>5</v>
+      </c>
+      <c r="C2">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3">
+      <c r="A3" t="s">
+        <v>242</v>
+      </c>
+      <c r="B3">
+        <v>6</v>
+      </c>
+      <c r="C3">
+        <v>200</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet25.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:B3"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1" spans="1:2">
+      <c r="A1" t="s">
+        <v>243</v>
+      </c>
+      <c r="B1" t="s">
+        <v>244</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2">
+      <c r="A2" t="s">
+        <v>245</v>
+      </c>
+      <c r="B2" t="s">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2">
+      <c r="A3" t="s">
+        <v>246</v>
+      </c>
+      <c r="B3" t="s">
+        <v>201</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet26.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:B3"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1" spans="1:2">
+      <c r="A1" t="s">
+        <v>243</v>
+      </c>
+      <c r="B1" t="s">
+        <v>244</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2">
+      <c r="A2" t="s">
+        <v>246</v>
+      </c>
+      <c r="B2" t="s">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2">
+      <c r="A3" t="s">
+        <v>247</v>
+      </c>
+      <c r="B3" t="s">
+        <v>201</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
-  <sheetPr/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:R3"/>
-  <sheetFormatPr defaultColWidth="8.85185185185185" defaultRowHeight="14.4" outlineLevelRow="2"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="2" width="21" customWidth="1"/>
     <col min="3" max="3" width="6" customWidth="1"/>
-    <col min="4" max="4" width="12.712962962963" customWidth="1"/>
-    <col min="5" max="5" width="19.4259259259259" customWidth="1"/>
-    <col min="6" max="6" width="15.1388888888889" customWidth="1"/>
-    <col min="7" max="7" width="15.4259259259259" customWidth="1"/>
-    <col min="8" max="8" width="19.5740740740741" customWidth="1"/>
-    <col min="9" max="9" width="10.8518518518519" customWidth="1"/>
-    <col min="10" max="10" width="17.5740740740741" customWidth="1"/>
-    <col min="11" max="11" width="11.287037037037" customWidth="1"/>
-    <col min="12" max="12" width="21.712962962963" customWidth="1"/>
+    <col min="4" max="4" width="12.7109375" customWidth="1"/>
+    <col min="5" max="5" width="19.42578125" customWidth="1"/>
+    <col min="6" max="6" width="15.140625" customWidth="1"/>
+    <col min="7" max="7" width="15.42578125" customWidth="1"/>
+    <col min="8" max="8" width="19.5703125" customWidth="1"/>
+    <col min="9" max="9" width="10.85546875" customWidth="1"/>
+    <col min="10" max="10" width="17.5703125" customWidth="1"/>
+    <col min="11" max="11" width="11.28515625" customWidth="1"/>
+    <col min="12" max="12" width="21.7109375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:18">
@@ -4340,7 +3837,7 @@
       <c r="Q2" s="23"/>
       <c r="R2" s="23"/>
     </row>
-    <row r="3" spans="1:12">
+    <row r="3" spans="1:18">
       <c r="A3" s="2" t="s">
         <v>62</v>
       </c>
@@ -4380,22 +3877,20 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
-  <sheetPr/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:F3"/>
-  <sheetFormatPr defaultColWidth="8.85185185185185" defaultRowHeight="14.4" outlineLevelRow="2" outlineLevelCol="5"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="27.1388888888889" customWidth="1"/>
-    <col min="2" max="2" width="10.4259259259259" customWidth="1"/>
-    <col min="3" max="3" width="11.4259259259259" customWidth="1"/>
-    <col min="4" max="4" width="11.712962962963" customWidth="1"/>
-    <col min="5" max="5" width="14.5740740740741" customWidth="1"/>
-    <col min="6" max="6" width="17.712962962963" customWidth="1"/>
+    <col min="1" max="1" width="27.140625" customWidth="1"/>
+    <col min="2" max="2" width="10.42578125" customWidth="1"/>
+    <col min="3" max="3" width="11.42578125" customWidth="1"/>
+    <col min="4" max="4" width="11.7109375" customWidth="1"/>
+    <col min="5" max="5" width="14.5703125" customWidth="1"/>
+    <col min="6" max="6" width="17.7109375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6">
@@ -4458,22 +3953,20 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
-  <sheetPr/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:F4"/>
-  <sheetFormatPr defaultColWidth="8.85185185185185" defaultRowHeight="14.4" outlineLevelRow="3" outlineLevelCol="5"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="27.1388888888889" customWidth="1"/>
-    <col min="2" max="2" width="10.4259259259259" customWidth="1"/>
-    <col min="3" max="3" width="11.4259259259259" customWidth="1"/>
-    <col min="4" max="4" width="11.712962962963" customWidth="1"/>
-    <col min="5" max="5" width="14.5740740740741" customWidth="1"/>
-    <col min="6" max="6" width="17.712962962963" customWidth="1"/>
+    <col min="1" max="1" width="27.140625" customWidth="1"/>
+    <col min="2" max="2" width="10.42578125" customWidth="1"/>
+    <col min="3" max="3" width="11.42578125" customWidth="1"/>
+    <col min="4" max="4" width="11.7109375" customWidth="1"/>
+    <col min="5" max="5" width="14.5703125" customWidth="1"/>
+    <col min="6" max="6" width="17.7109375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6">
@@ -4554,17 +4047,15 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
-  <sheetPr/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:C3"/>
-  <sheetFormatPr defaultColWidth="8.85185185185185" defaultRowHeight="14.4" outlineLevelRow="2" outlineLevelCol="2"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="28.712962962963" customWidth="1"/>
+    <col min="1" max="1" width="28.7109375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3">
@@ -4602,23 +4093,21 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
-  <sheetPr/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:G4"/>
-  <sheetFormatPr defaultColWidth="8.85185185185185" defaultRowHeight="14.4" outlineLevelRow="3" outlineLevelCol="6"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="19.712962962963" customWidth="1"/>
-    <col min="2" max="2" width="8.13888888888889" customWidth="1"/>
-    <col min="3" max="3" width="8.57407407407407" customWidth="1"/>
-    <col min="4" max="4" width="17.8518518518519" customWidth="1"/>
-    <col min="5" max="5" width="12.712962962963" customWidth="1"/>
-    <col min="6" max="6" width="14.5740740740741" customWidth="1"/>
-    <col min="7" max="7" width="17.712962962963" customWidth="1"/>
+    <col min="1" max="1" width="19.7109375" customWidth="1"/>
+    <col min="2" max="2" width="8.140625" customWidth="1"/>
+    <col min="3" max="3" width="8.5703125" customWidth="1"/>
+    <col min="4" max="4" width="17.85546875" customWidth="1"/>
+    <col min="5" max="5" width="12.7109375" customWidth="1"/>
+    <col min="6" max="6" width="14.5703125" customWidth="1"/>
+    <col min="7" max="7" width="17.7109375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7">
@@ -4699,7 +4188,7 @@
         <v>232</v>
       </c>
       <c r="D4" s="2">
-        <v>2.32</v>
+        <v>2.3199999999999998</v>
       </c>
       <c r="E4" s="7" t="s">
         <v>77</v>
@@ -4709,23 +4198,21 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
-  <sheetPr/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:G4"/>
-  <sheetFormatPr defaultColWidth="8.85185185185185" defaultRowHeight="14.4" outlineLevelRow="3" outlineLevelCol="6"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="19.712962962963" customWidth="1"/>
-    <col min="2" max="2" width="8.13888888888889" customWidth="1"/>
-    <col min="3" max="3" width="8.57407407407407" customWidth="1"/>
-    <col min="4" max="4" width="17.8518518518519" customWidth="1"/>
-    <col min="5" max="5" width="12.712962962963" customWidth="1"/>
-    <col min="6" max="6" width="14.5740740740741" customWidth="1"/>
-    <col min="7" max="7" width="17.712962962963" customWidth="1"/>
+    <col min="1" max="1" width="19.7109375" customWidth="1"/>
+    <col min="2" max="2" width="8.140625" customWidth="1"/>
+    <col min="3" max="3" width="8.5703125" customWidth="1"/>
+    <col min="4" max="4" width="17.85546875" customWidth="1"/>
+    <col min="5" max="5" width="12.7109375" customWidth="1"/>
+    <col min="6" max="6" width="14.5703125" customWidth="1"/>
+    <col min="7" max="7" width="17.7109375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7">
@@ -4806,7 +4293,7 @@
         <v>232</v>
       </c>
       <c r="D4" s="2">
-        <v>2.32</v>
+        <v>2.3199999999999998</v>
       </c>
       <c r="E4" s="7" t="s">
         <v>77</v>
@@ -4816,33 +4303,31 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
-  <sheetPr/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:S15"/>
-  <sheetFormatPr defaultColWidth="8.85185185185185" defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="39.712962962963" customWidth="1"/>
-    <col min="2" max="2" width="10.1388888888889" customWidth="1"/>
-    <col min="3" max="3" width="39.712962962963" customWidth="1"/>
+    <col min="1" max="1" width="39.7109375" customWidth="1"/>
+    <col min="2" max="2" width="10.140625" customWidth="1"/>
+    <col min="3" max="3" width="39.7109375" customWidth="1"/>
     <col min="4" max="4" width="11" customWidth="1"/>
-    <col min="5" max="5" width="13.287037037037" customWidth="1"/>
-    <col min="6" max="6" width="8.85185185185185" customWidth="1"/>
-    <col min="7" max="7" width="17.8518518518519" customWidth="1"/>
-    <col min="8" max="8" width="19.5740740740741" customWidth="1"/>
-    <col min="9" max="9" width="23.712962962963" customWidth="1"/>
-    <col min="10" max="10" width="12.712962962963" customWidth="1"/>
-    <col min="11" max="11" width="11.8518518518519" customWidth="1"/>
-    <col min="12" max="12" width="17.4259259259259" customWidth="1"/>
-    <col min="13" max="14" width="39.712962962963" customWidth="1"/>
-    <col min="15" max="15" width="25.712962962963" customWidth="1"/>
-    <col min="16" max="17" width="16.5740740740741" customWidth="1"/>
-    <col min="18" max="18" width="11.5740740740741" customWidth="1"/>
-    <col min="19" max="19" width="14.8518518518519" customWidth="1"/>
+    <col min="5" max="5" width="13.28515625" customWidth="1"/>
+    <col min="6" max="6" width="8.85546875" customWidth="1"/>
+    <col min="7" max="7" width="17.85546875" customWidth="1"/>
+    <col min="8" max="8" width="19.5703125" customWidth="1"/>
+    <col min="9" max="9" width="23.7109375" customWidth="1"/>
+    <col min="10" max="10" width="12.7109375" customWidth="1"/>
+    <col min="11" max="11" width="11.85546875" customWidth="1"/>
+    <col min="12" max="12" width="17.42578125" customWidth="1"/>
+    <col min="13" max="14" width="39.7109375" customWidth="1"/>
+    <col min="15" max="15" width="25.7109375" customWidth="1"/>
+    <col min="16" max="17" width="16.5703125" customWidth="1"/>
+    <col min="18" max="18" width="11.5703125" customWidth="1"/>
+    <col min="19" max="19" width="14.85546875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:19">
@@ -5658,6 +5143,5 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <headerFooter/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
ADDED NEW TEST SCENARIOS FOR THE PAYROLL MODULE AND ADDED CHANGES FOR THE FAILED TEST SCENARIOS
ADDED NEW TEST SCENARIOS FOR THE PAYROLL MODULE AND ADDED CHANGES FOR THE FAILED TEST SCENARIOS
</commit_message>
<xml_diff>
--- a/testdata/ItemDetails.xlsx
+++ b/testdata/ItemDetails.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="4" lowestEdited="5" rupBuild="4505"/>
   <workbookPr/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="2520" windowWidth="15150" windowHeight="6540" firstSheet="21" activeTab="25"/>
+    <workbookView xWindow="0" yWindow="2520" windowWidth="15150" windowHeight="6540" firstSheet="21" activeTab="23"/>
   </bookViews>
   <sheets>
     <sheet name="PR Details" sheetId="1" r:id="rId1"/>
@@ -3624,6 +3624,9 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:C3"/>
   <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="15" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:3">
       <c r="A1" t="s">

</xml_diff>

<commit_message>
ADDING NEW TEST SCENARIOS FOR THE SALES ORDER AMENDMENT AND CREDIT NOTE SCREENS
ADDING NEW TEST SCENARIOS FOR THE SALES ORDER AMENDMENT AND CREDIT NOTE SCREENS
</commit_message>
<xml_diff>
--- a/testdata/ItemDetails.xlsx
+++ b/testdata/ItemDetails.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="4" lowestEdited="5" rupBuild="4505"/>
   <workbookPr/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="2520" windowWidth="15150" windowHeight="6540" firstSheet="21" activeTab="23"/>
+    <workbookView xWindow="0" yWindow="2520" windowWidth="15150" windowHeight="6540" firstSheet="9" activeTab="11"/>
   </bookViews>
   <sheets>
     <sheet name="PR Details" sheetId="1" r:id="rId1"/>
@@ -35,7 +35,6 @@
     <sheet name="RFQDOM" sheetId="26" r:id="rId26"/>
   </sheets>
   <calcPr calcId="124519"/>
-  <oleSize ref="A1:O20"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -53,7 +52,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="716" uniqueCount="248">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="737" uniqueCount="254">
   <si>
     <t>ITEM_NAME</t>
   </si>
@@ -798,6 +797,24 @@
   </si>
   <si>
     <t>JJ AUTOMOBILES</t>
+  </si>
+  <si>
+    <t>GANESH ENTERPRISE</t>
+  </si>
+  <si>
+    <t>SI - SERVICE</t>
+  </si>
+  <si>
+    <t>SAI ENTERPRISE06</t>
+  </si>
+  <si>
+    <t>LOC49</t>
+  </si>
+  <si>
+    <t>L3</t>
+  </si>
+  <si>
+    <t>WEGA ASSOCIATES</t>
   </si>
 </sst>
 </file>
@@ -2152,7 +2169,7 @@
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G11"/>
+  <dimension ref="A1:G14"/>
   <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="25.7109375" customWidth="1"/>
@@ -2415,6 +2432,75 @@
       </c>
       <c r="G11" s="15" t="s">
         <v>165</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7">
+      <c r="A12" s="2" t="s">
+        <v>248</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>201</v>
+      </c>
+      <c r="C12" s="2" t="s">
+        <v>249</v>
+      </c>
+      <c r="D12" s="2" t="s">
+        <v>181</v>
+      </c>
+      <c r="E12" s="2" t="s">
+        <v>182</v>
+      </c>
+      <c r="F12" s="2" t="s">
+        <v>166</v>
+      </c>
+      <c r="G12" s="2" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7">
+      <c r="A13" s="2" t="s">
+        <v>250</v>
+      </c>
+      <c r="B13" s="2" t="s">
+        <v>201</v>
+      </c>
+      <c r="C13" s="2" t="s">
+        <v>202</v>
+      </c>
+      <c r="D13" s="2" t="s">
+        <v>251</v>
+      </c>
+      <c r="E13" s="2" t="s">
+        <v>252</v>
+      </c>
+      <c r="F13" s="2" t="s">
+        <v>166</v>
+      </c>
+      <c r="G13" s="2" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7">
+      <c r="A14" s="2" t="s">
+        <v>253</v>
+      </c>
+      <c r="B14" s="2" t="s">
+        <v>203</v>
+      </c>
+      <c r="C14" s="2" t="s">
+        <v>202</v>
+      </c>
+      <c r="D14" s="2" t="s">
+        <v>251</v>
+      </c>
+      <c r="E14" s="2" t="s">
+        <v>252</v>
+      </c>
+      <c r="F14" s="2" t="s">
+        <v>160</v>
+      </c>
+      <c r="G14" s="2" t="s">
+        <v>150</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
FIXES FOR FAILED TEST CASES OF SALES ORDER AND SALES INVOICE
FIXES FOR FAILED TEST CASES OF SALES ORDER AND SALES INVOICE
</commit_message>
<xml_diff>
--- a/testdata/ItemDetails.xlsx
+++ b/testdata/ItemDetails.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="4" lowestEdited="5" rupBuild="4505"/>
   <workbookPr/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="2520" windowWidth="15150" windowHeight="6540" firstSheet="9" activeTab="11"/>
+    <workbookView xWindow="0" yWindow="2520" windowWidth="15150" windowHeight="6540" firstSheet="8" activeTab="9"/>
   </bookViews>
   <sheets>
     <sheet name="PR Details" sheetId="1" r:id="rId1"/>
@@ -52,7 +52,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="737" uniqueCount="254">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="772" uniqueCount="261">
   <si>
     <t>ITEM_NAME</t>
   </si>
@@ -815,18 +815,46 @@
   </si>
   <si>
     <t>WEGA ASSOCIATES</t>
+  </si>
+  <si>
+    <t>HK-TVS-FG-10001</t>
+  </si>
+  <si>
+    <t>MTON</t>
+  </si>
+  <si>
+    <t>.0001</t>
+  </si>
+  <si>
+    <t>HK-TVS-FG-10002</t>
+  </si>
+  <si>
+    <t>HK-CUS-001</t>
+  </si>
+  <si>
+    <t>HARI TRADERS</t>
+  </si>
+  <si>
+    <t>TAMILNADU</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="11">
+  <fonts count="12">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -949,24 +977,24 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="35">
+  <cellXfs count="36">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
@@ -975,25 +1003,25 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="2" applyFont="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="2" applyBorder="1">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" xfId="2" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1">
@@ -1005,10 +1033,10 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1019,7 +1047,7 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1">
@@ -1028,34 +1056,37 @@
     <xf numFmtId="49" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="justify" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -1886,7 +1917,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:K5"/>
+  <dimension ref="A1:K6"/>
   <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="9" customWidth="1"/>
@@ -2075,6 +2106,41 @@
       </c>
       <c r="K5" s="2" t="s">
         <v>170</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11">
+      <c r="A6" s="15" t="s">
+        <v>258</v>
+      </c>
+      <c r="B6" s="15" t="s">
+        <v>259</v>
+      </c>
+      <c r="C6" s="35" t="s">
+        <v>165</v>
+      </c>
+      <c r="D6" s="35" t="s">
+        <v>166</v>
+      </c>
+      <c r="E6" s="35" t="s">
+        <v>166</v>
+      </c>
+      <c r="F6" s="15" t="s">
+        <v>259</v>
+      </c>
+      <c r="G6" s="2" t="s">
+        <v>260</v>
+      </c>
+      <c r="H6" s="2" t="s">
+        <v>168</v>
+      </c>
+      <c r="I6" s="2" t="s">
+        <v>162</v>
+      </c>
+      <c r="J6" s="2" t="s">
+        <v>156</v>
+      </c>
+      <c r="K6" s="2" t="s">
+        <v>157</v>
       </c>
     </row>
   </sheetData>
@@ -4397,7 +4463,7 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:S15"/>
+  <dimension ref="A1:S17"/>
   <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="39.7109375" customWidth="1"/>
@@ -5230,6 +5296,108 @@
         <v>109</v>
       </c>
     </row>
+    <row r="16" spans="1:19">
+      <c r="A16" s="2" t="s">
+        <v>254</v>
+      </c>
+      <c r="B16" s="15">
+        <v>0</v>
+      </c>
+      <c r="C16" s="2" t="s">
+        <v>254</v>
+      </c>
+      <c r="D16" s="35" t="s">
+        <v>255</v>
+      </c>
+      <c r="E16" s="2">
+        <v>88363222</v>
+      </c>
+      <c r="F16" s="2">
+        <v>18</v>
+      </c>
+      <c r="G16" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="H16" s="2"/>
+      <c r="I16" s="2"/>
+      <c r="J16" s="35" t="s">
+        <v>14</v>
+      </c>
+      <c r="K16" s="24" t="s">
+        <v>256</v>
+      </c>
+      <c r="L16" s="35" t="s">
+        <v>107</v>
+      </c>
+      <c r="M16" s="2"/>
+      <c r="N16" s="2"/>
+      <c r="O16" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="P16" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="Q16" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="R16" s="2" t="s">
+        <v>108</v>
+      </c>
+      <c r="S16" s="2" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="17" spans="1:19">
+      <c r="A17" s="35" t="s">
+        <v>257</v>
+      </c>
+      <c r="B17" s="2">
+        <v>0</v>
+      </c>
+      <c r="C17" s="35" t="s">
+        <v>257</v>
+      </c>
+      <c r="D17" s="35" t="s">
+        <v>255</v>
+      </c>
+      <c r="E17" s="2">
+        <v>88363222</v>
+      </c>
+      <c r="F17" s="2">
+        <v>18</v>
+      </c>
+      <c r="G17" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="H17" s="2"/>
+      <c r="I17" s="2"/>
+      <c r="J17" s="35" t="s">
+        <v>14</v>
+      </c>
+      <c r="K17" s="24" t="s">
+        <v>256</v>
+      </c>
+      <c r="L17" s="35" t="s">
+        <v>107</v>
+      </c>
+      <c r="M17" s="2"/>
+      <c r="N17" s="2"/>
+      <c r="O17" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="P17" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="Q17" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="R17" s="2" t="s">
+        <v>108</v>
+      </c>
+      <c r="S17" s="2" t="s">
+        <v>109</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Modified The Existing Scenarios And Added New Test Scenarios For The Customer Schedule And Customer Schedule Amendment
Modified The Existing Scenarios And Added New Test Scenarios For The Customer Schedule And Customer Schedule Amendment
</commit_message>
<xml_diff>
--- a/testdata/ItemDetails.xlsx
+++ b/testdata/ItemDetails.xlsx
@@ -1,10 +1,10 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
+  <fileVersion appName="xl" lastEdited="4" lowestEdited="5" rupBuild="4505"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="23040" windowHeight="9120" firstSheet="19" activeTab="26"/>
+    <workbookView xWindow="0" yWindow="2520" windowWidth="15150" windowHeight="6540" firstSheet="7" activeTab="8"/>
   </bookViews>
   <sheets>
     <sheet name="PR Details" sheetId="1" r:id="rId1"/>
@@ -35,7 +35,8 @@
     <sheet name="RFQDOM" sheetId="26" r:id="rId26"/>
     <sheet name="GATEITEM" sheetId="27" r:id="rId27"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="124519"/>
+  <oleSize ref="A4:G23"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -53,7 +54,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="777" uniqueCount="264">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="778" uniqueCount="263">
   <si>
     <t>ITEM_NAME</t>
   </si>
@@ -396,9 +397,6 @@
   </si>
   <si>
     <t>HK-FG-STD-PRICE-DISSIMILAR ITEM-10001</t>
-  </si>
-  <si>
-    <t>GENERAL</t>
   </si>
   <si>
     <t>HK-LOT-MAC-10001(FG)</t>
@@ -851,19 +849,20 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="xr9">
-  <numFmts count="4">
-    <numFmt numFmtId="176" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
-    <numFmt numFmtId="177" formatCode="_ &quot;₹&quot;* #,##0.00_ ;_ &quot;₹&quot;* \-#,##0.00_ ;_ &quot;₹&quot;* &quot;-&quot;??_ ;_ @_ "/>
-    <numFmt numFmtId="178" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
-    <numFmt numFmtId="179" formatCode="_ &quot;₹&quot;* #,##0_ ;_ &quot;₹&quot;* \-#,##0_ ;_ &quot;₹&quot;* &quot;-&quot;_ ;_ @_ "/>
-  </numFmts>
-  <fonts count="30">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <fonts count="12">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -931,152 +930,8 @@
       <name val="Times New Roman"/>
       <charset val="134"/>
     </font>
-    <font>
-      <u/>
-      <sz val="11"/>
-      <color rgb="FF0000FF"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <u/>
-      <sz val="11"/>
-      <color rgb="FF800080"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FFFF0000"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="18"/>
-      <color theme="3"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <i/>
-      <sz val="11"/>
-      <color rgb="FF7F7F7F"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="15"/>
-      <color theme="3"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="13"/>
-      <color theme="3"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="3"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF3F3F76"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FF3F3F3F"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FFFA7D00"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FFFFFFFF"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FFFA7D00"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF006100"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF9C0006"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF9C6500"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="0"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
   </fonts>
-  <fills count="36">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1085,7 +940,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.599993896298105"/>
+        <fgColor theme="9" tint="0.59999389629810485"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1101,194 +956,8 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFFCC"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFCC99"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFF2F2F2"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFA5A5A5"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFC6EFCE"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFC7CE"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFEB9C"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
   </fills>
-  <borders count="10">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -1311,274 +980,32 @@
       </bottom>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color rgb="FFB2B2B2"/>
-      </left>
-      <right style="thin">
-        <color rgb="FFB2B2B2"/>
-      </right>
-      <top style="thin">
-        <color rgb="FFB2B2B2"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FFB2B2B2"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="medium">
-        <color theme="4"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="medium">
-        <color theme="4" tint="0.499984740745262"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF7F7F7F"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF7F7F7F"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF7F7F7F"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF7F7F7F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF3F3F3F"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF3F3F3F"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF3F3F3F"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF3F3F3F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="double">
-        <color rgb="FF3F3F3F"/>
-      </left>
-      <right style="double">
-        <color rgb="FF3F3F3F"/>
-      </right>
-      <top style="double">
-        <color rgb="FF3F3F3F"/>
-      </top>
-      <bottom style="double">
-        <color rgb="FF3F3F3F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="double">
-        <color rgb="FFFF8001"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color theme="4"/>
-      </top>
-      <bottom style="double">
-        <color theme="4"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
-  <cellStyleXfs count="51">
+  <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="176" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="177" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="178" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="179" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="2" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="6" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="7" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="7" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="8" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="35" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="37">
+  <cellXfs count="38">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
@@ -1587,25 +1014,25 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="50" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="49" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="50" applyFont="1" applyBorder="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="2" applyFont="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="50" applyBorder="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="2" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1">
@@ -1617,10 +1044,10 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1630,135 +1057,207 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="49" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="49" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="justify" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
-  <cellStyles count="51">
+  <cellStyles count="3">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Comma" xfId="1" builtinId="3"/>
-    <cellStyle name="Currency" xfId="2" builtinId="4"/>
-    <cellStyle name="Percent" xfId="3" builtinId="5"/>
-    <cellStyle name="Comma [0]" xfId="4" builtinId="6"/>
-    <cellStyle name="Currency [0]" xfId="5" builtinId="7"/>
-    <cellStyle name="Hyperlink" xfId="6" builtinId="8"/>
-    <cellStyle name="Followed Hyperlink" xfId="7" builtinId="9"/>
-    <cellStyle name="Note" xfId="8" builtinId="10"/>
-    <cellStyle name="Warning Text" xfId="9" builtinId="11"/>
-    <cellStyle name="Title" xfId="10" builtinId="15"/>
-    <cellStyle name="CExplanatory Text" xfId="11" builtinId="53"/>
-    <cellStyle name="Heading 1" xfId="12" builtinId="16"/>
-    <cellStyle name="Heading 2" xfId="13" builtinId="17"/>
-    <cellStyle name="Heading 3" xfId="14" builtinId="18"/>
-    <cellStyle name="Heading 4" xfId="15" builtinId="19"/>
-    <cellStyle name="Input" xfId="16" builtinId="20"/>
-    <cellStyle name="Output" xfId="17" builtinId="21"/>
-    <cellStyle name="Calculation" xfId="18" builtinId="22"/>
-    <cellStyle name="Check Cell" xfId="19" builtinId="23"/>
-    <cellStyle name="Linked Cell" xfId="20" builtinId="24"/>
-    <cellStyle name="Total" xfId="21" builtinId="25"/>
-    <cellStyle name="Good" xfId="22" builtinId="26"/>
-    <cellStyle name="Bad" xfId="23" builtinId="27"/>
-    <cellStyle name="Neutral" xfId="24" builtinId="28"/>
-    <cellStyle name="Accent1" xfId="25" builtinId="29"/>
-    <cellStyle name="20% - Accent1" xfId="26" builtinId="30"/>
-    <cellStyle name="40% - Accent1" xfId="27" builtinId="31"/>
-    <cellStyle name="60% - Accent1" xfId="28" builtinId="32"/>
-    <cellStyle name="Accent2" xfId="29" builtinId="33"/>
-    <cellStyle name="20% - Accent2" xfId="30" builtinId="34"/>
-    <cellStyle name="40% - Accent2" xfId="31" builtinId="35"/>
-    <cellStyle name="60% - Accent2" xfId="32" builtinId="36"/>
-    <cellStyle name="Accent3" xfId="33" builtinId="37"/>
-    <cellStyle name="20% - Accent3" xfId="34" builtinId="38"/>
-    <cellStyle name="40% - Accent3" xfId="35" builtinId="39"/>
-    <cellStyle name="60% - Accent3" xfId="36" builtinId="40"/>
-    <cellStyle name="Accent4" xfId="37" builtinId="41"/>
-    <cellStyle name="20% - Accent4" xfId="38" builtinId="42"/>
-    <cellStyle name="40% - Accent4" xfId="39" builtinId="43"/>
-    <cellStyle name="60% - Accent4" xfId="40" builtinId="44"/>
-    <cellStyle name="Accent5" xfId="41" builtinId="45"/>
-    <cellStyle name="20% - Accent5" xfId="42" builtinId="46"/>
-    <cellStyle name="40% - Accent5" xfId="43" builtinId="47"/>
-    <cellStyle name="60% - Accent5" xfId="44" builtinId="48"/>
-    <cellStyle name="Accent6" xfId="45" builtinId="49"/>
-    <cellStyle name="20% - Accent6" xfId="46" builtinId="50"/>
-    <cellStyle name="40% - Accent6" xfId="47" builtinId="51"/>
-    <cellStyle name="60% - Accent6" xfId="48" builtinId="52"/>
-    <cellStyle name="Normal 2" xfId="49"/>
-    <cellStyle name="Normal 3" xfId="50"/>
+    <cellStyle name="Normal 2" xfId="1"/>
+    <cellStyle name="Normal 3" xfId="2"/>
   </cellStyles>
   <dxfs count="17">
     <dxf>
       <fill>
         <patternFill patternType="solid">
-          <fgColor theme="4" tint="0.799981688894314"/>
-          <bgColor theme="4" tint="0.799981688894314"/>
+          <fgColor theme="4" tint="0.79995117038483843"/>
+          <bgColor theme="4" tint="0.79995117038483843"/>
+        </patternFill>
+      </fill>
+      <border>
+        <bottom style="thin">
+          <color theme="4" tint="0.39994506668294322"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor theme="4" tint="0.79995117038483843"/>
+          <bgColor theme="4" tint="0.79995117038483843"/>
+        </patternFill>
+      </fill>
+      <border>
+        <bottom style="thin">
+          <color theme="4" tint="0.39994506668294322"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="1"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="1"/>
+      </font>
+      <border>
+        <bottom style="thin">
+          <color theme="4" tint="0.39994506668294322"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <color theme="1"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <color theme="1"/>
+      </font>
+      <border>
+        <top style="thin">
+          <color theme="4"/>
+        </top>
+        <bottom style="thin">
+          <color theme="4"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor theme="4" tint="0.79995117038483843"/>
+          <bgColor theme="4" tint="0.79995117038483843"/>
         </patternFill>
       </fill>
     </dxf>
     <dxf>
       <fill>
         <patternFill patternType="solid">
-          <fgColor theme="4" tint="0.799981688894314"/>
-          <bgColor theme="4" tint="0.799981688894314"/>
+          <fgColor theme="4" tint="0.79995117038483843"/>
+          <bgColor theme="4" tint="0.79995117038483843"/>
         </patternFill>
       </fill>
     </dxf>
     <dxf>
       <font>
-        <b val="1"/>
+        <b/>
+        <color theme="1"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor theme="4" tint="0.79995117038483843"/>
+          <bgColor theme="4" tint="0.79995117038483843"/>
+        </patternFill>
+      </fill>
+      <border>
+        <top style="thin">
+          <color theme="4" tint="0.39994506668294322"/>
+        </top>
+        <bottom style="thin">
+          <color theme="4" tint="0.39994506668294322"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <color theme="1"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor theme="4" tint="0.79995117038483843"/>
+          <bgColor theme="4" tint="0.79995117038483843"/>
+        </patternFill>
+      </fill>
+      <border>
+        <bottom style="thin">
+          <color theme="4" tint="0.39994506668294322"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor theme="4" tint="0.79995117038483843"/>
+          <bgColor theme="4" tint="0.79995117038483843"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor theme="4" tint="0.79995117038483843"/>
+          <bgColor theme="4" tint="0.79995117038483843"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
         <color theme="1"/>
       </font>
     </dxf>
     <dxf>
       <font>
-        <b val="1"/>
+        <b/>
         <color theme="1"/>
       </font>
     </dxf>
     <dxf>
       <font>
-        <b val="1"/>
+        <b/>
         <color theme="1"/>
       </font>
       <border>
@@ -1769,7 +1268,7 @@
     </dxf>
     <dxf>
       <font>
-        <b val="1"/>
+        <b/>
         <color theme="0"/>
       </font>
       <fill>
@@ -1797,149 +1296,32 @@
           <color theme="4"/>
         </bottom>
         <horizontal style="thin">
-          <color theme="4" tint="0.399975585192419"/>
+          <color theme="4" tint="0.39994506668294322"/>
         </horizontal>
-      </border>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor theme="4" tint="0.799981688894314"/>
-          <bgColor theme="4" tint="0.799981688894314"/>
-        </patternFill>
-      </fill>
-      <border>
-        <bottom style="thin">
-          <color theme="4" tint="0.399975585192419"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="1"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor theme="4" tint="0.799981688894314"/>
-          <bgColor theme="4" tint="0.799981688894314"/>
-        </patternFill>
-      </fill>
-      <border>
-        <bottom style="thin">
-          <color theme="4" tint="0.399975585192419"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="1"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="1"/>
-      </font>
-      <border>
-        <bottom style="thin">
-          <color theme="4" tint="0.399975585192419"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="1"/>
-        <color theme="1"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="1"/>
-        <color theme="1"/>
-      </font>
-      <border>
-        <top style="thin">
-          <color theme="4"/>
-        </top>
-        <bottom style="thin">
-          <color theme="4"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor theme="4" tint="0.799981688894314"/>
-          <bgColor theme="4" tint="0.799981688894314"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor theme="4" tint="0.799981688894314"/>
-          <bgColor theme="4" tint="0.799981688894314"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="1"/>
-        <color theme="1"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor theme="4" tint="0.799981688894314"/>
-          <bgColor theme="4" tint="0.799981688894314"/>
-        </patternFill>
-      </fill>
-      <border>
-        <top style="thin">
-          <color theme="4" tint="0.399975585192419"/>
-        </top>
-        <bottom style="thin">
-          <color theme="4" tint="0.399975585192419"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="1"/>
-        <color theme="1"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor theme="4" tint="0.799981688894314"/>
-          <bgColor theme="4" tint="0.799981688894314"/>
-        </patternFill>
-      </fill>
-      <border>
-        <bottom style="thin">
-          <color theme="4" tint="0.399975585192419"/>
-        </bottom>
       </border>
     </dxf>
   </dxfs>
   <tableStyles count="2" defaultTableStyle="TableStylePreset3_Accent1" defaultPivotStyle="PivotStylePreset2_Accent1">
-    <tableStyle name="TableStylePreset3_Accent1" pivot="0" count="7" xr9:uid="{59DB682C-5494-4EDE-A608-00C9E5F0F923}">
-      <tableStyleElement type="wholeTable" dxfId="6"/>
-      <tableStyleElement type="headerRow" dxfId="5"/>
-      <tableStyleElement type="totalRow" dxfId="4"/>
-      <tableStyleElement type="firstColumn" dxfId="3"/>
-      <tableStyleElement type="lastColumn" dxfId="2"/>
-      <tableStyleElement type="firstRowStripe" dxfId="1"/>
-      <tableStyleElement type="firstColumnStripe" dxfId="0"/>
+    <tableStyle name="TableStylePreset3_Accent1" pivot="0" count="7">
+      <tableStyleElement type="wholeTable" dxfId="16"/>
+      <tableStyleElement type="headerRow" dxfId="15"/>
+      <tableStyleElement type="totalRow" dxfId="14"/>
+      <tableStyleElement type="firstColumn" dxfId="13"/>
+      <tableStyleElement type="lastColumn" dxfId="12"/>
+      <tableStyleElement type="firstRowStripe" dxfId="11"/>
+      <tableStyleElement type="firstColumnStripe" dxfId="10"/>
     </tableStyle>
-    <tableStyle name="PivotStylePreset2_Accent1" table="0" count="10" xr9:uid="{267968C8-6FFD-4C36-ACC1-9EA1FD1885CA}">
-      <tableStyleElement type="headerRow" dxfId="16"/>
-      <tableStyleElement type="totalRow" dxfId="15"/>
-      <tableStyleElement type="firstRowStripe" dxfId="14"/>
-      <tableStyleElement type="firstColumnStripe" dxfId="13"/>
-      <tableStyleElement type="firstSubtotalRow" dxfId="12"/>
-      <tableStyleElement type="secondSubtotalRow" dxfId="11"/>
-      <tableStyleElement type="firstRowSubheading" dxfId="10"/>
-      <tableStyleElement type="secondRowSubheading" dxfId="9"/>
-      <tableStyleElement type="pageFieldLabels" dxfId="8"/>
-      <tableStyleElement type="pageFieldValues" dxfId="7"/>
+    <tableStyle name="PivotStylePreset2_Accent1" table="0" count="10">
+      <tableStyleElement type="headerRow" dxfId="9"/>
+      <tableStyleElement type="totalRow" dxfId="8"/>
+      <tableStyleElement type="firstRowStripe" dxfId="7"/>
+      <tableStyleElement type="firstColumnStripe" dxfId="6"/>
+      <tableStyleElement type="firstSubtotalRow" dxfId="5"/>
+      <tableStyleElement type="secondSubtotalRow" dxfId="4"/>
+      <tableStyleElement type="firstRowSubheading" dxfId="3"/>
+      <tableStyleElement type="secondRowSubheading" dxfId="2"/>
+      <tableStyleElement type="pageFieldLabels" dxfId="1"/>
+      <tableStyleElement type="pageFieldValues" dxfId="0"/>
     </tableStyle>
   </tableStyles>
   <extLst>
@@ -2202,23 +1584,23 @@
     </a:fmtScheme>
   </a:themeElements>
   <a:objectDefaults/>
+  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
-  <sheetPr/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:J20"/>
-  <sheetFormatPr defaultColWidth="8.71296296296296" defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="20.712962962963" customWidth="1"/>
-    <col min="2" max="3" width="12.712962962963" customWidth="1"/>
-    <col min="4" max="4" width="14.712962962963" customWidth="1"/>
-    <col min="5" max="5" width="9.85185185185185" customWidth="1"/>
-    <col min="6" max="6" width="14.1388888888889" customWidth="1"/>
-    <col min="7" max="7" width="14.8518518518519" customWidth="1"/>
-    <col min="8" max="8" width="22.287037037037" customWidth="1"/>
-    <col min="9" max="9" width="14.4259259259259" customWidth="1"/>
+    <col min="1" max="1" width="20.7109375" customWidth="1"/>
+    <col min="2" max="3" width="12.7109375" customWidth="1"/>
+    <col min="4" max="4" width="14.7109375" customWidth="1"/>
+    <col min="5" max="5" width="9.85546875" customWidth="1"/>
+    <col min="6" max="6" width="14.140625" customWidth="1"/>
+    <col min="7" max="7" width="14.85546875" customWidth="1"/>
+    <col min="8" max="8" width="22.28515625" customWidth="1"/>
+    <col min="9" max="9" width="14.42578125" customWidth="1"/>
     <col min="10" max="10" width="13" customWidth="1"/>
   </cols>
   <sheetData>
@@ -2254,7 +1636,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="2" s="32" customFormat="1" ht="20.4" spans="1:10">
+    <row r="2" spans="1:10" s="32" customFormat="1" ht="22.5">
       <c r="A2" s="34" t="s">
         <v>10</v>
       </c>
@@ -2286,7 +1668,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="3" ht="15" customHeight="1" spans="1:10">
+    <row r="3" spans="1:10" ht="15" customHeight="1">
       <c r="A3" s="34" t="s">
         <v>18</v>
       </c>
@@ -2318,7 +1700,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="4" spans="1:10">
+    <row r="4" spans="1:10" ht="22.5">
       <c r="A4" s="34" t="s">
         <v>21</v>
       </c>
@@ -2544,692 +1926,684 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
-  <sheetPr/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:K6"/>
-  <sheetFormatPr defaultColWidth="8.85185185185185" defaultRowHeight="14.4" outlineLevelRow="5"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="9" customWidth="1"/>
-    <col min="2" max="2" width="25.712962962963" customWidth="1"/>
-    <col min="3" max="3" width="12.4259259259259" customWidth="1"/>
-    <col min="4" max="4" width="16.287037037037" customWidth="1"/>
-    <col min="5" max="5" width="20.287037037037" customWidth="1"/>
-    <col min="6" max="6" width="25.712962962963" customWidth="1"/>
-    <col min="7" max="7" width="12.287037037037" customWidth="1"/>
-    <col min="8" max="8" width="14.5740740740741" customWidth="1"/>
-    <col min="9" max="9" width="28.5740740740741" customWidth="1"/>
+    <col min="2" max="2" width="25.7109375" customWidth="1"/>
+    <col min="3" max="3" width="12.42578125" customWidth="1"/>
+    <col min="4" max="4" width="16.28515625" customWidth="1"/>
+    <col min="5" max="5" width="20.28515625" customWidth="1"/>
+    <col min="6" max="6" width="25.7109375" customWidth="1"/>
+    <col min="7" max="7" width="12.28515625" customWidth="1"/>
+    <col min="8" max="8" width="14.5703125" customWidth="1"/>
+    <col min="9" max="9" width="28.5703125" customWidth="1"/>
     <col min="10" max="10" width="23" customWidth="1"/>
-    <col min="11" max="11" width="14.712962962963" customWidth="1"/>
+    <col min="11" max="11" width="14.7109375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:11">
       <c r="A1" s="8" t="s">
+        <v>140</v>
+      </c>
+      <c r="B1" s="8" t="s">
         <v>141</v>
       </c>
-      <c r="B1" s="8" t="s">
+      <c r="C1" s="8" t="s">
         <v>142</v>
       </c>
-      <c r="C1" s="8" t="s">
+      <c r="D1" s="8" t="s">
         <v>143</v>
       </c>
-      <c r="D1" s="8" t="s">
+      <c r="E1" s="8" t="s">
         <v>144</v>
       </c>
-      <c r="E1" s="8" t="s">
+      <c r="F1" s="20" t="s">
         <v>145</v>
       </c>
-      <c r="F1" s="20" t="s">
+      <c r="G1" s="20" t="s">
         <v>146</v>
       </c>
-      <c r="G1" s="20" t="s">
+      <c r="H1" s="20" t="s">
         <v>147</v>
       </c>
-      <c r="H1" s="20" t="s">
+      <c r="I1" s="20" t="s">
         <v>148</v>
       </c>
-      <c r="I1" s="20" t="s">
+      <c r="J1" s="20" t="s">
         <v>149</v>
       </c>
-      <c r="J1" s="20" t="s">
+      <c r="K1" s="20" t="s">
         <v>150</v>
-      </c>
-      <c r="K1" s="20" t="s">
-        <v>151</v>
       </c>
     </row>
     <row r="2" spans="1:11">
       <c r="A2" s="8" t="s">
+        <v>151</v>
+      </c>
+      <c r="B2" s="8" t="s">
         <v>152</v>
       </c>
-      <c r="B2" s="8" t="s">
+      <c r="C2" s="8" t="s">
         <v>153</v>
       </c>
-      <c r="C2" s="8" t="s">
+      <c r="D2" s="8" t="s">
         <v>154</v>
       </c>
-      <c r="D2" s="8" t="s">
+      <c r="E2" s="8" t="s">
         <v>155</v>
       </c>
-      <c r="E2" s="8" t="s">
+      <c r="F2" s="3" t="s">
+        <v>152</v>
+      </c>
+      <c r="G2" s="3" t="s">
         <v>156</v>
       </c>
-      <c r="F2" s="3" t="s">
-        <v>153</v>
-      </c>
-      <c r="G2" s="3" t="s">
+      <c r="H2" s="3" t="s">
         <v>157</v>
       </c>
-      <c r="H2" s="3" t="s">
+      <c r="I2" s="3" t="s">
         <v>158</v>
       </c>
-      <c r="I2" s="3" t="s">
+      <c r="J2" s="3" t="s">
         <v>159</v>
       </c>
-      <c r="J2" s="3" t="s">
+      <c r="K2" s="3" t="s">
         <v>160</v>
-      </c>
-      <c r="K2" s="3" t="s">
-        <v>161</v>
       </c>
     </row>
     <row r="3" spans="1:11">
       <c r="A3" s="21" t="s">
+        <v>161</v>
+      </c>
+      <c r="B3" s="3" t="s">
         <v>162</v>
       </c>
-      <c r="B3" s="3" t="s">
+      <c r="C3" s="8" t="s">
+        <v>153</v>
+      </c>
+      <c r="D3" s="3" t="s">
         <v>163</v>
       </c>
-      <c r="C3" s="8" t="s">
-        <v>154</v>
-      </c>
-      <c r="D3" s="3" t="s">
+      <c r="E3" s="3" t="s">
+        <v>163</v>
+      </c>
+      <c r="F3" s="3" t="s">
+        <v>162</v>
+      </c>
+      <c r="G3" s="3" t="s">
         <v>164</v>
       </c>
-      <c r="E3" s="3" t="s">
+      <c r="H3" s="3" t="s">
         <v>164</v>
       </c>
-      <c r="F3" s="3" t="s">
-        <v>163</v>
-      </c>
-      <c r="G3" s="3" t="s">
+      <c r="I3" s="3" t="s">
         <v>165</v>
       </c>
-      <c r="H3" s="3" t="s">
-        <v>165</v>
-      </c>
-      <c r="I3" s="3" t="s">
-        <v>166</v>
-      </c>
       <c r="J3" s="3" t="s">
+        <v>159</v>
+      </c>
+      <c r="K3" s="3" t="s">
         <v>160</v>
-      </c>
-      <c r="K3" s="3" t="s">
-        <v>161</v>
       </c>
     </row>
     <row r="4" spans="1:11">
       <c r="A4" s="3" t="s">
+        <v>166</v>
+      </c>
+      <c r="B4" s="3" t="s">
         <v>167</v>
       </c>
-      <c r="B4" s="3" t="s">
+      <c r="C4" s="8" t="s">
         <v>168</v>
       </c>
-      <c r="C4" s="8" t="s">
+      <c r="D4" s="8" t="s">
         <v>169</v>
       </c>
-      <c r="D4" s="8" t="s">
+      <c r="E4" s="8" t="s">
+        <v>169</v>
+      </c>
+      <c r="F4" s="3" t="s">
+        <v>167</v>
+      </c>
+      <c r="G4" s="3" t="s">
         <v>170</v>
       </c>
-      <c r="E4" s="8" t="s">
-        <v>170</v>
-      </c>
-      <c r="F4" s="3" t="s">
-        <v>168</v>
-      </c>
-      <c r="G4" s="3" t="s">
+      <c r="H4" s="3" t="s">
         <v>171</v>
       </c>
-      <c r="H4" s="3" t="s">
+      <c r="I4" s="3" t="s">
         <v>172</v>
       </c>
-      <c r="I4" s="3" t="s">
+      <c r="J4" s="3" t="s">
+        <v>159</v>
+      </c>
+      <c r="K4" s="3" t="s">
         <v>173</v>
-      </c>
-      <c r="J4" s="3" t="s">
-        <v>160</v>
-      </c>
-      <c r="K4" s="3" t="s">
-        <v>174</v>
       </c>
     </row>
     <row r="5" spans="1:11">
       <c r="A5" s="3" t="s">
+        <v>174</v>
+      </c>
+      <c r="B5" s="3" t="s">
         <v>175</v>
       </c>
-      <c r="B5" s="3" t="s">
+      <c r="C5" s="8" t="s">
+        <v>168</v>
+      </c>
+      <c r="D5" s="3" t="s">
         <v>176</v>
       </c>
-      <c r="C5" s="8" t="s">
-        <v>169</v>
-      </c>
-      <c r="D5" s="3" t="s">
+      <c r="E5" s="3" t="s">
+        <v>176</v>
+      </c>
+      <c r="F5" s="3" t="s">
+        <v>175</v>
+      </c>
+      <c r="G5" s="3" t="s">
         <v>177</v>
       </c>
-      <c r="E5" s="3" t="s">
-        <v>177</v>
-      </c>
-      <c r="F5" s="3" t="s">
-        <v>176</v>
-      </c>
-      <c r="G5" s="3" t="s">
+      <c r="H5" s="3" t="s">
         <v>178</v>
       </c>
-      <c r="H5" s="3" t="s">
-        <v>179</v>
-      </c>
       <c r="I5" s="3" t="s">
+        <v>172</v>
+      </c>
+      <c r="J5" s="3" t="s">
+        <v>159</v>
+      </c>
+      <c r="K5" s="3" t="s">
         <v>173</v>
-      </c>
-      <c r="J5" s="3" t="s">
-        <v>160</v>
-      </c>
-      <c r="K5" s="3" t="s">
-        <v>174</v>
       </c>
     </row>
     <row r="6" spans="1:11">
       <c r="A6" s="16" t="s">
+        <v>179</v>
+      </c>
+      <c r="B6" s="16" t="s">
         <v>180</v>
       </c>
-      <c r="B6" s="16" t="s">
+      <c r="C6" s="22" t="s">
+        <v>168</v>
+      </c>
+      <c r="D6" s="22" t="s">
+        <v>169</v>
+      </c>
+      <c r="E6" s="22" t="s">
+        <v>169</v>
+      </c>
+      <c r="F6" s="16" t="s">
+        <v>180</v>
+      </c>
+      <c r="G6" s="3" t="s">
         <v>181</v>
       </c>
-      <c r="C6" s="22" t="s">
-        <v>169</v>
-      </c>
-      <c r="D6" s="22" t="s">
-        <v>170</v>
-      </c>
-      <c r="E6" s="22" t="s">
-        <v>170</v>
-      </c>
-      <c r="F6" s="16" t="s">
-        <v>181</v>
-      </c>
-      <c r="G6" s="3" t="s">
-        <v>182</v>
-      </c>
       <c r="H6" s="3" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="I6" s="3" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="J6" s="3" t="s">
+        <v>159</v>
+      </c>
+      <c r="K6" s="3" t="s">
         <v>160</v>
-      </c>
-      <c r="K6" s="3" t="s">
-        <v>161</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
-  <sheetPr/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:E4"/>
-  <sheetFormatPr defaultColWidth="8.85185185185185" defaultRowHeight="14.4" outlineLevelRow="3" outlineLevelCol="4"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="13.5740740740741" customWidth="1"/>
+    <col min="1" max="1" width="13.5703125" customWidth="1"/>
     <col min="2" max="2" width="6" customWidth="1"/>
-    <col min="3" max="3" width="14.4259259259259" customWidth="1"/>
-    <col min="4" max="4" width="18.1388888888889" customWidth="1"/>
-    <col min="5" max="5" width="19.5740740740741" customWidth="1"/>
+    <col min="3" max="3" width="14.42578125" customWidth="1"/>
+    <col min="4" max="4" width="18.140625" customWidth="1"/>
+    <col min="5" max="5" width="19.5703125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5">
       <c r="A1" s="8" t="s">
+        <v>182</v>
+      </c>
+      <c r="B1" s="3" t="s">
         <v>183</v>
       </c>
-      <c r="B1" s="3" t="s">
+      <c r="C1" s="3" t="s">
         <v>184</v>
       </c>
-      <c r="C1" s="3" t="s">
+      <c r="D1" s="3" t="s">
         <v>185</v>
       </c>
-      <c r="D1" s="3" t="s">
+      <c r="E1" s="3" t="s">
         <v>186</v>
       </c>
-      <c r="E1" s="3" t="s">
+    </row>
+    <row r="2" spans="1:5" ht="30">
+      <c r="A2" s="8" t="s">
         <v>187</v>
       </c>
-    </row>
-    <row r="2" spans="1:5">
-      <c r="A2" s="8" t="s">
+      <c r="B2" s="8" t="s">
         <v>188</v>
       </c>
-      <c r="B2" s="8" t="s">
+      <c r="C2" s="18" t="s">
+        <v>151</v>
+      </c>
+      <c r="D2" s="19" t="s">
+        <v>152</v>
+      </c>
+      <c r="E2" s="8" t="s">
         <v>189</v>
-      </c>
-      <c r="C2" s="18" t="s">
-        <v>152</v>
-      </c>
-      <c r="D2" s="19" t="s">
-        <v>153</v>
-      </c>
-      <c r="E2" s="8" t="s">
-        <v>190</v>
       </c>
     </row>
     <row r="3" spans="1:5">
       <c r="A3" s="3" t="s">
+        <v>190</v>
+      </c>
+      <c r="B3" s="3" t="s">
         <v>191</v>
       </c>
-      <c r="B3" s="3" t="s">
+      <c r="C3" s="3" t="s">
         <v>192</v>
       </c>
-      <c r="C3" s="3" t="s">
+      <c r="D3" s="3" t="s">
         <v>193</v>
       </c>
-      <c r="D3" s="3" t="s">
+      <c r="E3" s="3" t="s">
         <v>194</v>
-      </c>
-      <c r="E3" s="3" t="s">
-        <v>195</v>
       </c>
     </row>
     <row r="4" spans="1:5">
       <c r="A4" s="3" t="s">
+        <v>195</v>
+      </c>
+      <c r="B4" s="3" t="s">
         <v>196</v>
       </c>
-      <c r="B4" s="3" t="s">
+      <c r="C4" s="3" t="s">
         <v>197</v>
       </c>
-      <c r="C4" s="3" t="s">
+      <c r="D4" s="3" t="s">
         <v>198</v>
       </c>
-      <c r="D4" s="3" t="s">
+      <c r="E4" s="3" t="s">
         <v>199</v>
-      </c>
-      <c r="E4" s="3" t="s">
-        <v>200</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
-  <sheetPr/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:G14"/>
-  <sheetFormatPr defaultColWidth="8.85185185185185" defaultRowHeight="14.4" outlineLevelCol="6"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="25.712962962963" customWidth="1"/>
-    <col min="2" max="2" width="8.85185185185185" customWidth="1"/>
-    <col min="3" max="3" width="12.287037037037" customWidth="1"/>
-    <col min="4" max="4" width="7.13888888888889" customWidth="1"/>
-    <col min="5" max="5" width="5.28703703703704" customWidth="1"/>
-    <col min="6" max="6" width="17.4259259259259" customWidth="1"/>
-    <col min="7" max="7" width="12.4259259259259" customWidth="1"/>
+    <col min="1" max="1" width="25.7109375" customWidth="1"/>
+    <col min="2" max="2" width="8.85546875" customWidth="1"/>
+    <col min="3" max="3" width="12.28515625" customWidth="1"/>
+    <col min="4" max="4" width="7.140625" customWidth="1"/>
+    <col min="5" max="5" width="5.28515625" customWidth="1"/>
+    <col min="6" max="6" width="17.42578125" customWidth="1"/>
+    <col min="7" max="7" width="12.42578125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7">
       <c r="A1" s="14" t="s">
+        <v>200</v>
+      </c>
+      <c r="B1" s="14" t="s">
         <v>201</v>
       </c>
-      <c r="B1" s="14" t="s">
+      <c r="C1" s="15" t="s">
         <v>202</v>
       </c>
-      <c r="C1" s="15" t="s">
+      <c r="D1" s="15" t="s">
         <v>203</v>
       </c>
-      <c r="D1" s="15" t="s">
+      <c r="E1" s="15" t="s">
         <v>204</v>
       </c>
-      <c r="E1" s="15" t="s">
+      <c r="F1" s="14" t="s">
         <v>205</v>
       </c>
-      <c r="F1" s="14" t="s">
+      <c r="G1" s="14" t="s">
         <v>206</v>
-      </c>
-      <c r="G1" s="14" t="s">
-        <v>207</v>
       </c>
     </row>
     <row r="2" spans="1:7">
       <c r="A2" s="16" t="s">
+        <v>167</v>
+      </c>
+      <c r="B2" s="16" t="s">
+        <v>207</v>
+      </c>
+      <c r="C2" s="17" t="s">
+        <v>208</v>
+      </c>
+      <c r="D2" s="17" t="s">
+        <v>187</v>
+      </c>
+      <c r="E2" s="17" t="s">
+        <v>188</v>
+      </c>
+      <c r="F2" s="16" t="s">
+        <v>169</v>
+      </c>
+      <c r="G2" s="16" t="s">
         <v>168</v>
-      </c>
-      <c r="B2" s="16" t="s">
-        <v>208</v>
-      </c>
-      <c r="C2" s="17" t="s">
-        <v>209</v>
-      </c>
-      <c r="D2" s="17" t="s">
-        <v>188</v>
-      </c>
-      <c r="E2" s="17" t="s">
-        <v>189</v>
-      </c>
-      <c r="F2" s="16" t="s">
-        <v>170</v>
-      </c>
-      <c r="G2" s="16" t="s">
-        <v>169</v>
       </c>
     </row>
     <row r="3" spans="1:7">
       <c r="A3" s="16" t="s">
+        <v>162</v>
+      </c>
+      <c r="B3" s="16" t="s">
+        <v>209</v>
+      </c>
+      <c r="C3" s="17" t="s">
+        <v>208</v>
+      </c>
+      <c r="D3" s="17" t="s">
+        <v>187</v>
+      </c>
+      <c r="E3" s="17" t="s">
+        <v>188</v>
+      </c>
+      <c r="F3" s="16" t="s">
         <v>163</v>
       </c>
-      <c r="B3" s="16" t="s">
-        <v>210</v>
-      </c>
-      <c r="C3" s="17" t="s">
-        <v>209</v>
-      </c>
-      <c r="D3" s="17" t="s">
-        <v>188</v>
-      </c>
-      <c r="E3" s="17" t="s">
-        <v>189</v>
-      </c>
-      <c r="F3" s="16" t="s">
-        <v>164</v>
-      </c>
       <c r="G3" s="16" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
     </row>
     <row r="4" spans="1:7">
       <c r="A4" s="16" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="B4" s="16" t="s">
+        <v>207</v>
+      </c>
+      <c r="C4" s="17" t="s">
         <v>208</v>
       </c>
-      <c r="C4" s="17" t="s">
-        <v>209</v>
-      </c>
       <c r="D4" s="17" t="s">
+        <v>187</v>
+      </c>
+      <c r="E4" s="17" t="s">
         <v>188</v>
       </c>
-      <c r="E4" s="17" t="s">
-        <v>189</v>
-      </c>
       <c r="F4" s="16" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="G4" s="16" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
     </row>
     <row r="5" spans="1:7">
       <c r="A5" s="16" t="s">
+        <v>152</v>
+      </c>
+      <c r="B5" s="16" t="s">
+        <v>207</v>
+      </c>
+      <c r="C5" s="17" t="s">
+        <v>208</v>
+      </c>
+      <c r="D5" s="17" t="s">
+        <v>187</v>
+      </c>
+      <c r="E5" s="17" t="s">
+        <v>188</v>
+      </c>
+      <c r="F5" s="16" t="s">
+        <v>154</v>
+      </c>
+      <c r="G5" s="16" t="s">
         <v>153</v>
-      </c>
-      <c r="B5" s="16" t="s">
-        <v>208</v>
-      </c>
-      <c r="C5" s="17" t="s">
-        <v>209</v>
-      </c>
-      <c r="D5" s="17" t="s">
-        <v>188</v>
-      </c>
-      <c r="E5" s="17" t="s">
-        <v>189</v>
-      </c>
-      <c r="F5" s="16" t="s">
-        <v>155</v>
-      </c>
-      <c r="G5" s="16" t="s">
-        <v>154</v>
       </c>
     </row>
     <row r="6" spans="1:7">
       <c r="A6" s="16" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="B6" s="16" t="s">
+        <v>207</v>
+      </c>
+      <c r="C6" s="17" t="s">
         <v>208</v>
       </c>
-      <c r="C6" s="17" t="s">
-        <v>209</v>
-      </c>
       <c r="D6" s="17" t="s">
+        <v>187</v>
+      </c>
+      <c r="E6" s="17" t="s">
         <v>188</v>
       </c>
-      <c r="E6" s="17" t="s">
-        <v>189</v>
-      </c>
       <c r="F6" s="16" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="G6" s="16" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
     </row>
     <row r="7" spans="1:7">
       <c r="A7" s="16" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="B7" s="16" t="s">
+        <v>207</v>
+      </c>
+      <c r="C7" s="17" t="s">
         <v>208</v>
       </c>
-      <c r="C7" s="17" t="s">
-        <v>209</v>
-      </c>
       <c r="D7" s="17" t="s">
+        <v>187</v>
+      </c>
+      <c r="E7" s="17" t="s">
         <v>188</v>
       </c>
-      <c r="E7" s="17" t="s">
-        <v>189</v>
-      </c>
       <c r="F7" s="16" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="G7" s="16" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
     </row>
     <row r="8" spans="1:7">
       <c r="A8" s="16" t="s">
+        <v>175</v>
+      </c>
+      <c r="B8" s="16" t="s">
+        <v>207</v>
+      </c>
+      <c r="C8" s="17" t="s">
+        <v>208</v>
+      </c>
+      <c r="D8" s="17" t="s">
+        <v>187</v>
+      </c>
+      <c r="E8" s="17" t="s">
+        <v>188</v>
+      </c>
+      <c r="F8" s="16" t="s">
         <v>176</v>
       </c>
-      <c r="B8" s="16" t="s">
-        <v>208</v>
-      </c>
-      <c r="C8" s="17" t="s">
-        <v>209</v>
-      </c>
-      <c r="D8" s="17" t="s">
-        <v>188</v>
-      </c>
-      <c r="E8" s="17" t="s">
-        <v>189</v>
-      </c>
-      <c r="F8" s="16" t="s">
-        <v>177</v>
-      </c>
       <c r="G8" s="16" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
     </row>
     <row r="9" spans="1:7">
       <c r="A9" s="16" t="s">
+        <v>213</v>
+      </c>
+      <c r="B9" s="16" t="s">
+        <v>207</v>
+      </c>
+      <c r="C9" s="17" t="s">
         <v>214</v>
       </c>
-      <c r="B9" s="16" t="s">
-        <v>208</v>
-      </c>
-      <c r="C9" s="17" t="s">
-        <v>215</v>
-      </c>
       <c r="D9" s="17" t="s">
+        <v>187</v>
+      </c>
+      <c r="E9" s="17" t="s">
         <v>188</v>
       </c>
-      <c r="E9" s="17" t="s">
-        <v>189</v>
-      </c>
       <c r="F9" s="16" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="G9" s="16" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
     </row>
     <row r="10" spans="1:7">
       <c r="A10" s="16" t="s">
+        <v>215</v>
+      </c>
+      <c r="B10" s="16" t="s">
+        <v>207</v>
+      </c>
+      <c r="C10" s="17" t="s">
         <v>216</v>
       </c>
-      <c r="B10" s="16" t="s">
-        <v>208</v>
-      </c>
-      <c r="C10" s="17" t="s">
-        <v>217</v>
-      </c>
       <c r="D10" s="17" t="s">
+        <v>187</v>
+      </c>
+      <c r="E10" s="17" t="s">
         <v>188</v>
       </c>
-      <c r="E10" s="17" t="s">
-        <v>189</v>
-      </c>
       <c r="F10" s="16" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="G10" s="16" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
     </row>
     <row r="11" spans="1:7">
       <c r="A11" s="16" t="s">
+        <v>217</v>
+      </c>
+      <c r="B11" s="16" t="s">
+        <v>207</v>
+      </c>
+      <c r="C11" s="17" t="s">
         <v>218</v>
       </c>
-      <c r="B11" s="16" t="s">
-        <v>208</v>
-      </c>
-      <c r="C11" s="17" t="s">
-        <v>219</v>
-      </c>
       <c r="D11" s="17" t="s">
+        <v>187</v>
+      </c>
+      <c r="E11" s="17" t="s">
         <v>188</v>
       </c>
-      <c r="E11" s="17" t="s">
-        <v>189</v>
-      </c>
       <c r="F11" s="16" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="G11" s="16" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
     </row>
     <row r="12" spans="1:7">
       <c r="A12" s="3" t="s">
+        <v>219</v>
+      </c>
+      <c r="B12" s="3" t="s">
+        <v>207</v>
+      </c>
+      <c r="C12" s="3" t="s">
         <v>220</v>
       </c>
-      <c r="B12" s="3" t="s">
-        <v>208</v>
-      </c>
-      <c r="C12" s="3" t="s">
-        <v>221</v>
-      </c>
       <c r="D12" s="3" t="s">
+        <v>187</v>
+      </c>
+      <c r="E12" s="3" t="s">
         <v>188</v>
       </c>
-      <c r="E12" s="3" t="s">
-        <v>189</v>
-      </c>
       <c r="F12" s="3" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="G12" s="3" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
     </row>
     <row r="13" spans="1:7">
       <c r="A13" s="3" t="s">
+        <v>221</v>
+      </c>
+      <c r="B13" s="3" t="s">
+        <v>207</v>
+      </c>
+      <c r="C13" s="3" t="s">
+        <v>208</v>
+      </c>
+      <c r="D13" s="3" t="s">
         <v>222</v>
       </c>
-      <c r="B13" s="3" t="s">
-        <v>208</v>
-      </c>
-      <c r="C13" s="3" t="s">
-        <v>209</v>
-      </c>
-      <c r="D13" s="3" t="s">
+      <c r="E13" s="3" t="s">
         <v>223</v>
       </c>
-      <c r="E13" s="3" t="s">
-        <v>224</v>
-      </c>
       <c r="F13" s="3" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="G13" s="3" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
     </row>
     <row r="14" spans="1:7">
       <c r="A14" s="3" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="C14" s="3" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="D14" s="3" t="s">
+        <v>222</v>
+      </c>
+      <c r="E14" s="3" t="s">
         <v>223</v>
       </c>
-      <c r="E14" s="3" t="s">
-        <v>224</v>
-      </c>
       <c r="F14" s="3" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="G14" s="3" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
-  <sheetPr/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:C3"/>
-  <sheetFormatPr defaultColWidth="8.85185185185185" defaultRowHeight="14.4" outlineLevelRow="2" outlineLevelCol="2"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="25.5740740740741" customWidth="1"/>
-    <col min="2" max="2" width="15.1388888888889" customWidth="1"/>
-    <col min="3" max="3" width="16.4259259259259" customWidth="1"/>
+    <col min="1" max="1" width="25.5703125" customWidth="1"/>
+    <col min="2" max="2" width="15.140625" customWidth="1"/>
+    <col min="3" max="3" width="16.42578125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3">
       <c r="A1" s="4" t="s">
+        <v>225</v>
+      </c>
+      <c r="B1" s="4" t="s">
         <v>226</v>
-      </c>
-      <c r="B1" s="4" t="s">
-        <v>227</v>
       </c>
       <c r="C1" s="4" t="s">
         <v>84</v>
@@ -3237,10 +2611,10 @@
     </row>
     <row r="2" spans="1:3">
       <c r="A2" s="3" t="s">
+        <v>227</v>
+      </c>
+      <c r="B2" s="3" t="s">
         <v>228</v>
-      </c>
-      <c r="B2" s="3" t="s">
-        <v>229</v>
       </c>
       <c r="C2" s="3">
         <v>2</v>
@@ -3248,10 +2622,10 @@
     </row>
     <row r="3" spans="1:3">
       <c r="A3" s="3" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="C3" s="3">
         <v>2</v>
@@ -3259,27 +2633,25 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
-  <sheetPr/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:C3"/>
-  <sheetFormatPr defaultColWidth="8.85185185185185" defaultRowHeight="14.4" outlineLevelRow="2" outlineLevelCol="2"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="21.4259259259259" customWidth="1"/>
-    <col min="2" max="2" width="11.5740740740741" customWidth="1"/>
+    <col min="1" max="1" width="21.42578125" customWidth="1"/>
+    <col min="2" max="2" width="11.5703125" customWidth="1"/>
     <col min="3" max="3" width="9" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3">
       <c r="A1" s="4" t="s">
+        <v>225</v>
+      </c>
+      <c r="B1" s="4" t="s">
         <v>226</v>
-      </c>
-      <c r="B1" s="4" t="s">
-        <v>227</v>
       </c>
       <c r="C1" s="4" t="s">
         <v>84</v>
@@ -3287,10 +2659,10 @@
     </row>
     <row r="2" spans="1:3">
       <c r="A2" s="3" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="C2" s="3">
         <v>2</v>
@@ -3298,10 +2670,10 @@
     </row>
     <row r="3" spans="1:3">
       <c r="A3" s="3" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="C3" s="3">
         <v>2</v>
@@ -3309,22 +2681,20 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
-  <sheetPr/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:B2"/>
-  <sheetFormatPr defaultColWidth="8.71296296296296" defaultRowHeight="14.4" outlineLevelRow="1" outlineLevelCol="1"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="20.4259259259259" customWidth="1"/>
+    <col min="1" max="1" width="20.42578125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2">
       <c r="A1" s="10" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="B1" s="10" t="s">
         <v>84</v>
@@ -3332,7 +2702,7 @@
     </row>
     <row r="2" spans="1:2">
       <c r="A2" s="10" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="B2" s="10">
         <v>10</v>
@@ -3340,19 +2710,17 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
-  <sheetPr/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:G3"/>
-  <sheetFormatPr defaultColWidth="8.71296296296296" defaultRowHeight="14.4" outlineLevelRow="2" outlineLevelCol="6"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:7">
       <c r="A1" s="9" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="B1" s="9" t="s">
         <v>84</v>
@@ -3375,7 +2743,7 @@
     </row>
     <row r="2" spans="1:7">
       <c r="A2" s="12" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="B2" s="9">
         <v>22</v>
@@ -3398,7 +2766,7 @@
     </row>
     <row r="3" spans="1:7">
       <c r="A3" s="12" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="B3" s="9">
         <v>34</v>
@@ -3419,19 +2787,17 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
-  <sheetPr/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:C3"/>
-  <sheetFormatPr defaultColWidth="8.71296296296296" defaultRowHeight="14.4" outlineLevelRow="2" outlineLevelCol="2"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:3">
       <c r="A1" s="9" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="B1" s="9" t="s">
         <v>84</v>
@@ -3442,7 +2808,7 @@
     </row>
     <row r="2" spans="1:3">
       <c r="A2" s="11" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="B2" s="9">
         <v>22</v>
@@ -3453,7 +2819,7 @@
     </row>
     <row r="3" spans="1:3">
       <c r="A3" s="11" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="B3" s="9">
         <v>40</v>
@@ -3464,19 +2830,17 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
-  <sheetPr/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:B2"/>
-  <sheetFormatPr defaultColWidth="8.71296296296296" defaultRowHeight="14.4" outlineLevelRow="1" outlineLevelCol="1"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:2">
       <c r="A1" s="10" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="B1" s="10" t="s">
         <v>84</v>
@@ -3484,7 +2848,7 @@
     </row>
     <row r="2" spans="1:2">
       <c r="A2" s="10" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="B2" s="10">
         <v>10</v>
@@ -3492,19 +2856,17 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
-  <sheetPr/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:C3"/>
-  <sheetFormatPr defaultColWidth="8.71296296296296" defaultRowHeight="14.4" outlineLevelRow="2" outlineLevelCol="2"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:3">
       <c r="A1" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="B1" s="9" t="s">
         <v>84</v>
@@ -3513,17 +2875,17 @@
         <v>80</v>
       </c>
     </row>
-    <row r="2" spans="1:2">
+    <row r="2" spans="1:3">
       <c r="A2" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="B2">
         <v>23</v>
       </c>
     </row>
-    <row r="3" spans="1:2">
+    <row r="3" spans="1:3">
       <c r="A3" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="B3">
         <v>45</v>
@@ -3531,36 +2893,34 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
-  <sheetPr/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:T10"/>
-  <sheetFormatPr defaultColWidth="8.71296296296296" defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="30" customWidth="1"/>
-    <col min="2" max="2" width="36.4259259259259" customWidth="1"/>
+    <col min="2" max="2" width="36.42578125" customWidth="1"/>
     <col min="3" max="3" width="6" customWidth="1"/>
-    <col min="4" max="4" width="13.712962962963" customWidth="1"/>
-    <col min="5" max="5" width="5.28703703703704" customWidth="1"/>
-    <col min="6" max="6" width="17.287037037037" customWidth="1"/>
-    <col min="7" max="7" width="30.287037037037" customWidth="1"/>
-    <col min="8" max="8" width="26.8518518518519" customWidth="1"/>
-    <col min="9" max="9" width="17.287037037037" customWidth="1"/>
-    <col min="10" max="10" width="13.287037037037" customWidth="1"/>
-    <col min="11" max="11" width="22.712962962963" customWidth="1"/>
-    <col min="12" max="12" width="12.712962962963" customWidth="1"/>
-    <col min="13" max="13" width="29.5740740740741" customWidth="1"/>
-    <col min="14" max="14" width="18.287037037037" customWidth="1"/>
-    <col min="15" max="15" width="16.287037037037" customWidth="1"/>
-    <col min="16" max="16" width="15.5740740740741" customWidth="1"/>
-    <col min="17" max="17" width="17.712962962963" customWidth="1"/>
-    <col min="18" max="18" width="24.1388888888889" customWidth="1"/>
-    <col min="19" max="19" width="13.4259259259259" customWidth="1"/>
-    <col min="20" max="20" width="13.5740740740741" customWidth="1"/>
+    <col min="4" max="4" width="13.7109375" customWidth="1"/>
+    <col min="5" max="5" width="5.28515625" customWidth="1"/>
+    <col min="6" max="6" width="17.28515625" customWidth="1"/>
+    <col min="7" max="7" width="30.28515625" customWidth="1"/>
+    <col min="8" max="8" width="26.85546875" customWidth="1"/>
+    <col min="9" max="9" width="17.28515625" customWidth="1"/>
+    <col min="10" max="10" width="13.28515625" customWidth="1"/>
+    <col min="11" max="11" width="22.7109375" customWidth="1"/>
+    <col min="12" max="12" width="12.7109375" customWidth="1"/>
+    <col min="13" max="13" width="29.5703125" customWidth="1"/>
+    <col min="14" max="14" width="18.28515625" customWidth="1"/>
+    <col min="15" max="15" width="16.28515625" customWidth="1"/>
+    <col min="16" max="16" width="15.5703125" customWidth="1"/>
+    <col min="17" max="17" width="17.7109375" customWidth="1"/>
+    <col min="18" max="18" width="24.140625" customWidth="1"/>
+    <col min="19" max="19" width="13.42578125" customWidth="1"/>
+    <col min="20" max="20" width="13.5703125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:20">
@@ -4113,22 +3473,20 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
-  <sheetPr/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:F3"/>
-  <sheetFormatPr defaultColWidth="8.71296296296296" defaultRowHeight="14.4" outlineLevelRow="2" outlineLevelCol="5"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="23.287037037037" customWidth="1"/>
-    <col min="2" max="2" width="10.4259259259259" customWidth="1"/>
-    <col min="3" max="3" width="11.4259259259259" customWidth="1"/>
-    <col min="4" max="4" width="11.712962962963" customWidth="1"/>
-    <col min="5" max="5" width="14.5740740740741" customWidth="1"/>
-    <col min="6" max="6" width="17.712962962963" customWidth="1"/>
+    <col min="1" max="1" width="23.28515625" customWidth="1"/>
+    <col min="2" max="2" width="10.42578125" customWidth="1"/>
+    <col min="3" max="3" width="11.42578125" customWidth="1"/>
+    <col min="4" max="4" width="11.7109375" customWidth="1"/>
+    <col min="5" max="5" width="14.5703125" customWidth="1"/>
+    <col min="6" max="6" width="17.7109375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6">
@@ -4153,7 +3511,7 @@
     </row>
     <row r="2" spans="1:6">
       <c r="A2" s="7" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="B2" s="3">
         <v>10</v>
@@ -4165,7 +3523,7 @@
         <v>73</v>
       </c>
       <c r="E2" s="8" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="F2" s="8" t="s">
         <v>75</v>
@@ -4173,7 +3531,7 @@
     </row>
     <row r="3" spans="1:6">
       <c r="A3" s="7" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="B3" s="3">
         <v>50</v>
@@ -4191,27 +3549,25 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
-  <sheetPr/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:F3"/>
-  <sheetFormatPr defaultColWidth="8.85185185185185" defaultRowHeight="14.4" outlineLevelRow="2" outlineLevelCol="5"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="20.8518518518519" customWidth="1"/>
+    <col min="1" max="1" width="20.85546875" customWidth="1"/>
     <col min="2" max="2" width="9" customWidth="1"/>
-    <col min="3" max="3" width="8.85185185185185" customWidth="1"/>
-    <col min="4" max="4" width="6.13888888888889" customWidth="1"/>
-    <col min="5" max="5" width="16.712962962963" customWidth="1"/>
-    <col min="6" max="6" width="16.287037037037" customWidth="1"/>
+    <col min="3" max="3" width="8.85546875" customWidth="1"/>
+    <col min="4" max="4" width="6.140625" customWidth="1"/>
+    <col min="5" max="5" width="16.7109375" customWidth="1"/>
+    <col min="6" max="6" width="16.28515625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6">
       <c r="A1" s="4" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="B1" s="4" t="s">
         <v>84</v>
@@ -4223,10 +3579,10 @@
         <v>27</v>
       </c>
       <c r="E1" s="2" t="s">
+        <v>246</v>
+      </c>
+      <c r="F1" s="2" t="s">
         <v>247</v>
-      </c>
-      <c r="F1" s="2" t="s">
-        <v>248</v>
       </c>
     </row>
     <row r="2" spans="1:6">
@@ -4251,7 +3607,7 @@
     </row>
     <row r="3" spans="1:6">
       <c r="A3" s="3" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="B3" s="3">
         <v>15</v>
@@ -4271,27 +3627,25 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
-  <sheetPr/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:F3"/>
-  <sheetFormatPr defaultColWidth="8.85185185185185" defaultRowHeight="14.4" outlineLevelRow="2" outlineLevelCol="5"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="21.712962962963" customWidth="1"/>
+    <col min="1" max="1" width="21.7109375" customWidth="1"/>
     <col min="2" max="2" width="9" customWidth="1"/>
-    <col min="3" max="3" width="8.85185185185185" customWidth="1"/>
-    <col min="4" max="4" width="6.13888888888889" customWidth="1"/>
-    <col min="5" max="5" width="16.712962962963" customWidth="1"/>
-    <col min="6" max="6" width="16.287037037037" customWidth="1"/>
+    <col min="3" max="3" width="8.85546875" customWidth="1"/>
+    <col min="4" max="4" width="6.140625" customWidth="1"/>
+    <col min="5" max="5" width="16.7109375" customWidth="1"/>
+    <col min="6" max="6" width="16.28515625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6">
       <c r="A1" s="4" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="B1" s="4" t="s">
         <v>84</v>
@@ -4303,10 +3657,10 @@
         <v>27</v>
       </c>
       <c r="E1" s="2" t="s">
+        <v>246</v>
+      </c>
+      <c r="F1" s="2" t="s">
         <v>247</v>
-      </c>
-      <c r="F1" s="2" t="s">
-        <v>248</v>
       </c>
     </row>
     <row r="2" spans="1:6">
@@ -4351,22 +3705,20 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
-  <sheetPr/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:F3"/>
-  <sheetFormatPr defaultColWidth="8.85185185185185" defaultRowHeight="14.4" outlineLevelRow="2" outlineLevelCol="5"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="15.4259259259259" customWidth="1"/>
-    <col min="2" max="2" width="10.5740740740741" customWidth="1"/>
-    <col min="3" max="3" width="11.5740740740741" customWidth="1"/>
-    <col min="4" max="4" width="11.8518518518519" customWidth="1"/>
+    <col min="1" max="1" width="15.42578125" customWidth="1"/>
+    <col min="2" max="2" width="10.5703125" customWidth="1"/>
+    <col min="3" max="3" width="11.5703125" customWidth="1"/>
+    <col min="4" max="4" width="11.85546875" customWidth="1"/>
     <col min="5" max="5" width="14" customWidth="1"/>
-    <col min="6" max="6" width="16.8518518518519" customWidth="1"/>
+    <col min="6" max="6" width="16.85546875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6">
@@ -4391,7 +3743,7 @@
     </row>
     <row r="2" spans="1:6">
       <c r="A2" s="3" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="B2" s="3">
         <v>10</v>
@@ -4403,7 +3755,7 @@
         <v>73</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="F2" s="3" t="s">
         <v>75</v>
@@ -4411,7 +3763,7 @@
     </row>
     <row r="3" spans="1:6">
       <c r="A3" s="3" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="B3" s="3">
         <v>20</v>
@@ -4423,7 +3775,7 @@
         <v>73</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="F3" s="3" t="s">
         <v>75</v>
@@ -4431,33 +3783,31 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
-  <sheetPr/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:C3"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.4" outlineLevelRow="2" outlineLevelCol="2"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="15" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3">
       <c r="A1" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="B1" t="s">
         <v>79</v>
       </c>
       <c r="C1" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
     </row>
     <row r="2" spans="1:3">
       <c r="A2" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="B2">
         <v>5</v>
@@ -4468,7 +3818,7 @@
     </row>
     <row r="3" spans="1:3">
       <c r="A3" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="B3">
         <v>6</v>
@@ -4479,107 +3829,101 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet25.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
-  <sheetPr/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:B3"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.4" outlineLevelRow="2" outlineLevelCol="1"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:2">
       <c r="A1" t="s">
+        <v>255</v>
+      </c>
+      <c r="B1" t="s">
         <v>256</v>
-      </c>
-      <c r="B1" t="s">
-        <v>257</v>
       </c>
     </row>
     <row r="2" spans="1:2">
       <c r="A2" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="B2" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
     </row>
     <row r="3" spans="1:2">
       <c r="A3" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="B3" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet26.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
-  <sheetPr/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:B3"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.4" outlineLevelRow="2" outlineLevelCol="1"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:2">
       <c r="A1" t="s">
+        <v>255</v>
+      </c>
+      <c r="B1" t="s">
         <v>256</v>
-      </c>
-      <c r="B1" t="s">
-        <v>257</v>
       </c>
     </row>
     <row r="2" spans="1:2">
       <c r="A2" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="B2" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
     </row>
     <row r="3" spans="1:2">
       <c r="A3" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="B3" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet27.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
-  <sheetPr/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:C3"/>
-  <sheetFormatPr defaultColWidth="8.88888888888889" defaultRowHeight="14.4" outlineLevelRow="2" outlineLevelCol="2"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="15.7777777777778" customWidth="1"/>
+    <col min="1" max="1" width="15.7109375" customWidth="1"/>
     <col min="2" max="2" width="5" customWidth="1"/>
     <col min="3" max="3" width="6" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3">
       <c r="A1" s="1" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>79</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
     </row>
     <row r="2" spans="1:3">
       <c r="A2" s="1" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="B2" s="1">
         <v>10</v>
@@ -4590,7 +3934,7 @@
     </row>
     <row r="3" spans="1:3">
       <c r="A3" s="1" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="B3" s="1">
         <v>20</v>
@@ -4601,27 +3945,25 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
-  <sheetPr/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:R3"/>
-  <sheetFormatPr defaultColWidth="8.85185185185185" defaultRowHeight="14.4" outlineLevelRow="2"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="2" width="21" customWidth="1"/>
     <col min="3" max="3" width="6" customWidth="1"/>
-    <col min="4" max="4" width="12.712962962963" customWidth="1"/>
-    <col min="5" max="5" width="19.4259259259259" customWidth="1"/>
-    <col min="6" max="6" width="15.1388888888889" customWidth="1"/>
-    <col min="7" max="7" width="15.4259259259259" customWidth="1"/>
-    <col min="8" max="8" width="19.5740740740741" customWidth="1"/>
-    <col min="9" max="9" width="10.8518518518519" customWidth="1"/>
-    <col min="10" max="10" width="17.5740740740741" customWidth="1"/>
-    <col min="11" max="11" width="11.287037037037" customWidth="1"/>
-    <col min="12" max="12" width="21.712962962963" customWidth="1"/>
+    <col min="4" max="4" width="12.7109375" customWidth="1"/>
+    <col min="5" max="5" width="19.42578125" customWidth="1"/>
+    <col min="6" max="6" width="15.140625" customWidth="1"/>
+    <col min="7" max="7" width="15.42578125" customWidth="1"/>
+    <col min="8" max="8" width="19.5703125" customWidth="1"/>
+    <col min="9" max="9" width="10.85546875" customWidth="1"/>
+    <col min="10" max="10" width="17.5703125" customWidth="1"/>
+    <col min="11" max="11" width="11.28515625" customWidth="1"/>
+    <col min="12" max="12" width="21.7109375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:18">
@@ -4712,7 +4054,7 @@
       <c r="Q2" s="26"/>
       <c r="R2" s="26"/>
     </row>
-    <row r="3" spans="1:12">
+    <row r="3" spans="1:18">
       <c r="A3" s="3" t="s">
         <v>62</v>
       </c>
@@ -4752,22 +4094,20 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
-  <sheetPr/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:F3"/>
-  <sheetFormatPr defaultColWidth="8.85185185185185" defaultRowHeight="14.4" outlineLevelRow="2" outlineLevelCol="5"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="27.1388888888889" customWidth="1"/>
-    <col min="2" max="2" width="10.4259259259259" customWidth="1"/>
-    <col min="3" max="3" width="11.4259259259259" customWidth="1"/>
-    <col min="4" max="4" width="11.712962962963" customWidth="1"/>
-    <col min="5" max="5" width="14.5740740740741" customWidth="1"/>
-    <col min="6" max="6" width="17.712962962963" customWidth="1"/>
+    <col min="1" max="1" width="27.140625" customWidth="1"/>
+    <col min="2" max="2" width="10.42578125" customWidth="1"/>
+    <col min="3" max="3" width="11.42578125" customWidth="1"/>
+    <col min="4" max="4" width="11.7109375" customWidth="1"/>
+    <col min="5" max="5" width="14.5703125" customWidth="1"/>
+    <col min="6" max="6" width="17.7109375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6">
@@ -4830,22 +4170,20 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
-  <sheetPr/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:F4"/>
-  <sheetFormatPr defaultColWidth="8.85185185185185" defaultRowHeight="14.4" outlineLevelRow="3" outlineLevelCol="5"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="27.1388888888889" customWidth="1"/>
-    <col min="2" max="2" width="10.4259259259259" customWidth="1"/>
-    <col min="3" max="3" width="11.4259259259259" customWidth="1"/>
-    <col min="4" max="4" width="11.712962962963" customWidth="1"/>
-    <col min="5" max="5" width="14.5740740740741" customWidth="1"/>
-    <col min="6" max="6" width="17.712962962963" customWidth="1"/>
+    <col min="1" max="1" width="27.140625" customWidth="1"/>
+    <col min="2" max="2" width="10.42578125" customWidth="1"/>
+    <col min="3" max="3" width="11.42578125" customWidth="1"/>
+    <col min="4" max="4" width="11.7109375" customWidth="1"/>
+    <col min="5" max="5" width="14.5703125" customWidth="1"/>
+    <col min="6" max="6" width="17.7109375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6">
@@ -4926,17 +4264,15 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
-  <sheetPr/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:C3"/>
-  <sheetFormatPr defaultColWidth="8.85185185185185" defaultRowHeight="14.4" outlineLevelRow="2" outlineLevelCol="2"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="28.712962962963" customWidth="1"/>
+    <col min="1" max="1" width="28.7109375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3">
@@ -4974,23 +4310,21 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
-  <sheetPr/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:G4"/>
-  <sheetFormatPr defaultColWidth="8.85185185185185" defaultRowHeight="14.4" outlineLevelRow="3" outlineLevelCol="6"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="19.712962962963" customWidth="1"/>
-    <col min="2" max="2" width="8.13888888888889" customWidth="1"/>
-    <col min="3" max="3" width="8.57407407407407" customWidth="1"/>
-    <col min="4" max="4" width="17.8518518518519" customWidth="1"/>
-    <col min="5" max="5" width="12.712962962963" customWidth="1"/>
-    <col min="6" max="6" width="14.5740740740741" customWidth="1"/>
-    <col min="7" max="7" width="17.712962962963" customWidth="1"/>
+    <col min="1" max="1" width="19.7109375" customWidth="1"/>
+    <col min="2" max="2" width="8.140625" customWidth="1"/>
+    <col min="3" max="3" width="8.5703125" customWidth="1"/>
+    <col min="4" max="4" width="17.85546875" customWidth="1"/>
+    <col min="5" max="5" width="12.7109375" customWidth="1"/>
+    <col min="6" max="6" width="14.5703125" customWidth="1"/>
+    <col min="7" max="7" width="17.7109375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7">
@@ -5071,7 +4405,7 @@
         <v>232</v>
       </c>
       <c r="D4" s="3">
-        <v>2.32</v>
+        <v>2.3199999999999998</v>
       </c>
       <c r="E4" s="8" t="s">
         <v>77</v>
@@ -5081,23 +4415,21 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
-  <sheetPr/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:G4"/>
-  <sheetFormatPr defaultColWidth="8.85185185185185" defaultRowHeight="14.4" outlineLevelRow="3" outlineLevelCol="6"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="19.712962962963" customWidth="1"/>
-    <col min="2" max="2" width="8.13888888888889" customWidth="1"/>
-    <col min="3" max="3" width="8.57407407407407" customWidth="1"/>
-    <col min="4" max="4" width="17.8518518518519" customWidth="1"/>
-    <col min="5" max="5" width="12.712962962963" customWidth="1"/>
-    <col min="6" max="6" width="14.5740740740741" customWidth="1"/>
-    <col min="7" max="7" width="17.712962962963" customWidth="1"/>
+    <col min="1" max="1" width="19.7109375" customWidth="1"/>
+    <col min="2" max="2" width="8.140625" customWidth="1"/>
+    <col min="3" max="3" width="8.5703125" customWidth="1"/>
+    <col min="4" max="4" width="17.85546875" customWidth="1"/>
+    <col min="5" max="5" width="12.7109375" customWidth="1"/>
+    <col min="6" max="6" width="14.5703125" customWidth="1"/>
+    <col min="7" max="7" width="17.7109375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7">
@@ -5178,7 +4510,7 @@
         <v>232</v>
       </c>
       <c r="D4" s="3">
-        <v>2.32</v>
+        <v>2.3199999999999998</v>
       </c>
       <c r="E4" s="8" t="s">
         <v>77</v>
@@ -5188,33 +4520,31 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
-  <sheetPr/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:S17"/>
-  <sheetFormatPr defaultColWidth="8.85185185185185" defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="39.712962962963" customWidth="1"/>
-    <col min="2" max="2" width="10.1388888888889" customWidth="1"/>
-    <col min="3" max="3" width="39.712962962963" customWidth="1"/>
+    <col min="1" max="1" width="39.7109375" customWidth="1"/>
+    <col min="2" max="2" width="10.140625" customWidth="1"/>
+    <col min="3" max="3" width="39.7109375" customWidth="1"/>
     <col min="4" max="4" width="11" customWidth="1"/>
-    <col min="5" max="5" width="13.287037037037" customWidth="1"/>
-    <col min="6" max="6" width="8.85185185185185" customWidth="1"/>
-    <col min="7" max="7" width="17.8518518518519" customWidth="1"/>
-    <col min="8" max="8" width="19.5740740740741" customWidth="1"/>
-    <col min="9" max="9" width="23.712962962963" customWidth="1"/>
-    <col min="10" max="10" width="12.712962962963" customWidth="1"/>
-    <col min="11" max="11" width="11.8518518518519" customWidth="1"/>
-    <col min="12" max="12" width="17.4259259259259" customWidth="1"/>
-    <col min="13" max="14" width="39.712962962963" customWidth="1"/>
-    <col min="15" max="15" width="25.712962962963" customWidth="1"/>
-    <col min="16" max="17" width="16.5740740740741" customWidth="1"/>
-    <col min="18" max="18" width="11.5740740740741" customWidth="1"/>
-    <col min="19" max="19" width="14.8518518518519" customWidth="1"/>
+    <col min="5" max="5" width="13.28515625" customWidth="1"/>
+    <col min="6" max="6" width="8.85546875" customWidth="1"/>
+    <col min="7" max="7" width="17.85546875" customWidth="1"/>
+    <col min="8" max="8" width="19.5703125" customWidth="1"/>
+    <col min="9" max="9" width="23.7109375" customWidth="1"/>
+    <col min="10" max="10" width="12.7109375" customWidth="1"/>
+    <col min="11" max="11" width="11.85546875" customWidth="1"/>
+    <col min="12" max="12" width="17.42578125" customWidth="1"/>
+    <col min="13" max="14" width="39.7109375" customWidth="1"/>
+    <col min="15" max="15" width="25.7109375" customWidth="1"/>
+    <col min="16" max="17" width="16.5703125" customWidth="1"/>
+    <col min="18" max="18" width="11.5703125" customWidth="1"/>
+    <col min="19" max="19" width="14.85546875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:19">
@@ -5446,11 +4776,11 @@
       <c r="D5" s="16" t="s">
         <v>14</v>
       </c>
-      <c r="E5" s="3">
-        <v>75052200</v>
-      </c>
-      <c r="F5" s="16">
-        <v>5</v>
+      <c r="E5" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="F5" s="3">
+        <v>12</v>
       </c>
       <c r="G5" s="16" t="s">
         <v>112</v>
@@ -5482,7 +4812,7 @@
         <v>15</v>
       </c>
       <c r="R5" s="3" t="s">
-        <v>114</v>
+        <v>108</v>
       </c>
       <c r="S5" s="20" t="s">
         <v>109</v>
@@ -5490,13 +4820,13 @@
     </row>
     <row r="6" spans="1:19">
       <c r="A6" s="16" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="B6" s="16">
         <v>0</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="D6" s="16" t="s">
         <v>14</v>
@@ -5508,10 +4838,10 @@
         <v>12</v>
       </c>
       <c r="G6" s="16" t="s">
+        <v>115</v>
+      </c>
+      <c r="H6" s="16" t="s">
         <v>116</v>
-      </c>
-      <c r="H6" s="16" t="s">
-        <v>117</v>
       </c>
       <c r="I6" s="3"/>
       <c r="J6" s="16" t="s">
@@ -5524,10 +4854,10 @@
         <v>107</v>
       </c>
       <c r="M6" s="16" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="N6" s="16" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="O6" s="8" t="s">
         <v>13</v>
@@ -5547,13 +4877,13 @@
     </row>
     <row r="7" spans="1:19">
       <c r="A7" s="16" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="B7" s="16">
         <v>0</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="D7" s="16" t="s">
         <v>14</v>
@@ -5565,10 +4895,10 @@
         <v>12</v>
       </c>
       <c r="G7" s="16" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="H7" s="16" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="I7" s="3"/>
       <c r="J7" s="16" t="s">
@@ -5581,10 +4911,10 @@
         <v>107</v>
       </c>
       <c r="M7" s="16" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="N7" s="16" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="O7" s="8" t="s">
         <v>13</v>
@@ -5604,25 +4934,25 @@
     </row>
     <row r="8" spans="1:19">
       <c r="A8" s="3" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="B8" s="16">
         <v>0</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="D8" s="16" t="s">
         <v>14</v>
       </c>
       <c r="E8" s="3" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="F8" s="16">
         <v>5</v>
       </c>
       <c r="G8" s="16" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="H8" s="3"/>
       <c r="I8" s="3">
@@ -5638,10 +4968,10 @@
         <v>107</v>
       </c>
       <c r="M8" s="3" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="N8" s="3" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="O8" s="8" t="s">
         <v>13</v>
@@ -5661,13 +4991,13 @@
     </row>
     <row r="9" spans="1:19">
       <c r="A9" s="16" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="B9" s="16">
         <v>0</v>
       </c>
       <c r="C9" s="3" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="D9" s="16" t="s">
         <v>14</v>
@@ -5679,7 +5009,7 @@
         <v>12</v>
       </c>
       <c r="G9" s="16" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="H9" s="3"/>
       <c r="I9" s="3">
@@ -5695,10 +5025,10 @@
         <v>107</v>
       </c>
       <c r="M9" s="16" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="N9" s="16" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="O9" s="8" t="s">
         <v>13</v>
@@ -5718,13 +5048,13 @@
     </row>
     <row r="10" spans="1:19">
       <c r="A10" s="3" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="B10" s="3">
         <v>0</v>
       </c>
       <c r="C10" s="3" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="D10" s="3" t="s">
         <v>14</v>
@@ -5736,7 +5066,7 @@
         <v>12</v>
       </c>
       <c r="G10" s="3" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="H10" s="3"/>
       <c r="I10" s="3"/>
@@ -5750,10 +5080,10 @@
         <v>107</v>
       </c>
       <c r="M10" s="3" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="N10" s="3" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="O10" s="3" t="s">
         <v>13</v>
@@ -5773,13 +5103,13 @@
     </row>
     <row r="11" spans="1:19">
       <c r="A11" s="3" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="B11" s="3">
         <v>0</v>
       </c>
       <c r="C11" s="3" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="D11" s="3" t="s">
         <v>14</v>
@@ -5791,7 +5121,7 @@
         <v>12</v>
       </c>
       <c r="G11" s="3" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="H11" s="3"/>
       <c r="I11" s="3"/>
@@ -5805,10 +5135,10 @@
         <v>107</v>
       </c>
       <c r="M11" s="3" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="N11" s="3" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="O11" s="3" t="s">
         <v>13</v>
@@ -5828,16 +5158,16 @@
     </row>
     <row r="12" spans="1:19">
       <c r="A12" s="3" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="B12" s="16">
         <v>0</v>
       </c>
       <c r="C12" s="3" t="s">
-        <v>127</v>
-      </c>
-      <c r="D12" s="8" t="s">
-        <v>20</v>
+        <v>126</v>
+      </c>
+      <c r="D12" s="3" t="s">
+        <v>14</v>
       </c>
       <c r="E12" s="21">
         <v>772213</v>
@@ -5850,8 +5180,8 @@
       </c>
       <c r="H12" s="3"/>
       <c r="I12" s="3"/>
-      <c r="J12" s="8" t="s">
-        <v>20</v>
+      <c r="J12" s="3" t="s">
+        <v>14</v>
       </c>
       <c r="K12" s="16">
         <v>1</v>
@@ -5865,10 +5195,10 @@
         <v>57</v>
       </c>
       <c r="P12" s="3" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="Q12" s="3" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="R12" s="3" t="s">
         <v>108</v>
@@ -5879,13 +5209,13 @@
     </row>
     <row r="13" spans="1:19">
       <c r="A13" s="3" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="B13" s="16">
         <v>0</v>
       </c>
       <c r="C13" s="3" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="D13" s="16" t="s">
         <v>14</v>
@@ -5928,13 +5258,13 @@
     </row>
     <row r="14" spans="1:19">
       <c r="A14" s="3" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="B14" s="16">
         <v>0</v>
       </c>
       <c r="C14" s="16" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="D14" s="16" t="s">
         <v>14</v>
@@ -5974,24 +5304,24 @@
         <v>108</v>
       </c>
       <c r="S14" s="3" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
     </row>
     <row r="15" spans="1:19">
       <c r="A15" s="3" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="B15" s="16">
         <v>0</v>
       </c>
       <c r="C15" s="3" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="D15" s="8" t="s">
         <v>14</v>
       </c>
       <c r="E15" s="23" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="F15" s="16">
         <v>12</v>
@@ -6030,16 +5360,16 @@
     </row>
     <row r="16" spans="1:19">
       <c r="A16" s="3" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="B16" s="16">
         <v>0</v>
       </c>
       <c r="C16" s="3" t="s">
+        <v>136</v>
+      </c>
+      <c r="D16" s="37" t="s">
         <v>137</v>
-      </c>
-      <c r="D16" s="22" t="s">
-        <v>138</v>
       </c>
       <c r="E16" s="3">
         <v>88363222</v>
@@ -6052,13 +5382,13 @@
       </c>
       <c r="H16" s="3"/>
       <c r="I16" s="3"/>
-      <c r="J16" s="22" t="s">
+      <c r="J16" s="37" t="s">
         <v>14</v>
       </c>
       <c r="K16" s="24" t="s">
-        <v>139</v>
-      </c>
-      <c r="L16" s="22" t="s">
+        <v>138</v>
+      </c>
+      <c r="L16" s="37" t="s">
         <v>107</v>
       </c>
       <c r="M16" s="3"/>
@@ -6080,17 +5410,17 @@
       </c>
     </row>
     <row r="17" spans="1:19">
-      <c r="A17" s="22" t="s">
-        <v>140</v>
+      <c r="A17" s="37" t="s">
+        <v>139</v>
       </c>
       <c r="B17" s="3">
         <v>0</v>
       </c>
-      <c r="C17" s="22" t="s">
-        <v>140</v>
-      </c>
-      <c r="D17" s="22" t="s">
-        <v>138</v>
+      <c r="C17" s="37" t="s">
+        <v>139</v>
+      </c>
+      <c r="D17" s="37" t="s">
+        <v>137</v>
       </c>
       <c r="E17" s="3">
         <v>88363222</v>
@@ -6103,13 +5433,13 @@
       </c>
       <c r="H17" s="3"/>
       <c r="I17" s="3"/>
-      <c r="J17" s="22" t="s">
+      <c r="J17" s="37" t="s">
         <v>14</v>
       </c>
       <c r="K17" s="24" t="s">
-        <v>139</v>
-      </c>
-      <c r="L17" s="22" t="s">
+        <v>138</v>
+      </c>
+      <c r="L17" s="37" t="s">
         <v>107</v>
       </c>
       <c r="M17" s="3"/>
@@ -6132,6 +5462,5 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <headerFooter/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Updated Functions And Locators For Sales Order Management And Inventory Modules
Updated The Functions And Locators Of Sales Order, Sales Order Amendment, Customer Schedule, Customer Schedule Amendment, Material Request And Stock Adjustment Screens
</commit_message>
<xml_diff>
--- a/testdata/ItemDetails.xlsx
+++ b/testdata/ItemDetails.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="4" lowestEdited="5" rupBuild="4505"/>
   <workbookPr/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="2520" windowWidth="15150" windowHeight="6540" firstSheet="7" activeTab="8"/>
+    <workbookView xWindow="0" yWindow="2520" windowWidth="15150" windowHeight="6540" firstSheet="21" activeTab="28"/>
   </bookViews>
   <sheets>
     <sheet name="PR Details" sheetId="1" r:id="rId1"/>
@@ -20,23 +20,24 @@
     <sheet name="Open Sales" sheetId="11" r:id="rId11"/>
     <sheet name="SI Details" sheetId="12" r:id="rId12"/>
     <sheet name="MRTOMRV Data" sheetId="13" r:id="rId13"/>
-    <sheet name="MRTOMRVWip Data" sheetId="14" r:id="rId14"/>
-    <sheet name="RateContract_SER" sheetId="15" r:id="rId15"/>
-    <sheet name="PricelistItem" sheetId="16" r:id="rId16"/>
-    <sheet name="ST_ITEM_RATECONTRACT" sheetId="17" r:id="rId17"/>
-    <sheet name="ServiceItemPriceList" sheetId="18" r:id="rId18"/>
-    <sheet name="ST_Item_PriceList" sheetId="19" r:id="rId19"/>
-    <sheet name="DIS_UOM_GEN_UD" sheetId="20" r:id="rId20"/>
-    <sheet name="SimilarItem" sheetId="21" r:id="rId21"/>
-    <sheet name="POAServiceSheet" sheetId="22" r:id="rId22"/>
-    <sheet name="DIS_UOM_MAT_UD" sheetId="23" r:id="rId23"/>
-    <sheet name="PRMULTI" sheetId="24" r:id="rId24"/>
-    <sheet name="RFQ" sheetId="25" r:id="rId25"/>
-    <sheet name="RFQDOM" sheetId="26" r:id="rId26"/>
-    <sheet name="GATEITEM" sheetId="27" r:id="rId27"/>
+    <sheet name="MRCustomer" sheetId="28" r:id="rId14"/>
+    <sheet name="MRTOMRVWip Data" sheetId="14" r:id="rId15"/>
+    <sheet name="RateContract_SER" sheetId="15" r:id="rId16"/>
+    <sheet name="PricelistItem" sheetId="16" r:id="rId17"/>
+    <sheet name="ST_ITEM_RATECONTRACT" sheetId="17" r:id="rId18"/>
+    <sheet name="ServiceItemPriceList" sheetId="18" r:id="rId19"/>
+    <sheet name="ST_Item_PriceList" sheetId="19" r:id="rId20"/>
+    <sheet name="DIS_UOM_GEN_UD" sheetId="20" r:id="rId21"/>
+    <sheet name="SimilarItem" sheetId="21" r:id="rId22"/>
+    <sheet name="POAServiceSheet" sheetId="22" r:id="rId23"/>
+    <sheet name="DIS_UOM_MAT_UD" sheetId="23" r:id="rId24"/>
+    <sheet name="PRMULTI" sheetId="24" r:id="rId25"/>
+    <sheet name="RFQ" sheetId="25" r:id="rId26"/>
+    <sheet name="RFQDOM" sheetId="26" r:id="rId27"/>
+    <sheet name="GATEITEM" sheetId="27" r:id="rId28"/>
+    <sheet name="StockAdjustment" sheetId="29" r:id="rId29"/>
   </sheets>
   <calcPr calcId="124519"/>
-  <oleSize ref="A4:G23"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -54,7 +55,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="778" uniqueCount="263">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="838" uniqueCount="313">
   <si>
     <t>ITEM_NAME</t>
   </si>
@@ -844,18 +845,183 @@
   </si>
   <si>
     <t>TVS-SIM-290004</t>
+  </si>
+  <si>
+    <t>HK-LOT-MAC-10001</t>
+  </si>
+  <si>
+    <t>F100</t>
+  </si>
+  <si>
+    <t>Stock Cost</t>
+  </si>
+  <si>
+    <t>Line Amount</t>
+  </si>
+  <si>
+    <t>13.27173</t>
+  </si>
+  <si>
+    <t>84.75</t>
+  </si>
+  <si>
+    <t>Unit Cost</t>
+  </si>
+  <si>
+    <t>84.74822</t>
+  </si>
+  <si>
+    <t>13.27</t>
+  </si>
+  <si>
+    <t>SNO</t>
+  </si>
+  <si>
+    <t>ITEM ID</t>
+  </si>
+  <si>
+    <t>ITEM REV</t>
+  </si>
+  <si>
+    <t>ITEM DESC</t>
+  </si>
+  <si>
+    <t>UNIT COST</t>
+  </si>
+  <si>
+    <t>LOTNUMBER</t>
+  </si>
+  <si>
+    <t>LOT QTY</t>
+  </si>
+  <si>
+    <t>LOT EXPIRY DATE</t>
+  </si>
+  <si>
+    <t>HK-FIFO-LOT-BATCH-10001</t>
+  </si>
+  <si>
+    <t>21-10-2025</t>
+  </si>
+  <si>
+    <t>FROM SERIAL NUMBER</t>
+  </si>
+  <si>
+    <t>PREFIX</t>
+  </si>
+  <si>
+    <t>OB</t>
+  </si>
+  <si>
+    <t>HK-SER-MAC-10001</t>
+  </si>
+  <si>
+    <t>BEFORE STOCK QTY</t>
+  </si>
+  <si>
+    <t>AFTER STOCK QTY</t>
+  </si>
+  <si>
+    <t>119139.4</t>
+  </si>
+  <si>
+    <t>100115</t>
+  </si>
+  <si>
+    <t>500003</t>
+  </si>
+  <si>
+    <t>300033</t>
+  </si>
+  <si>
+    <t>HEAT NO</t>
+  </si>
+  <si>
+    <t>TEST NO</t>
+  </si>
+  <si>
+    <t>119237.4</t>
+  </si>
+  <si>
+    <t>100125</t>
+  </si>
+  <si>
+    <t>500004</t>
+  </si>
+  <si>
+    <t>300044</t>
+  </si>
+  <si>
+    <t>119337.4</t>
+  </si>
+  <si>
+    <t>100135</t>
+  </si>
+  <si>
+    <t>300055</t>
+  </si>
+  <si>
+    <t>500005</t>
+  </si>
+  <si>
+    <t>119437.4</t>
+  </si>
+  <si>
+    <t>100145</t>
+  </si>
+  <si>
+    <t>300066</t>
+  </si>
+  <si>
+    <t>500006</t>
+  </si>
+  <si>
+    <t>119537.4</t>
+  </si>
+  <si>
+    <t>100155</t>
+  </si>
+  <si>
+    <t>300077</t>
+  </si>
+  <si>
+    <t>500007</t>
+  </si>
+  <si>
+    <t>119637.4</t>
+  </si>
+  <si>
+    <t>100165</t>
+  </si>
+  <si>
+    <t>300088</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="12">
+  <numFmts count="0"/>
+  <fonts count="15">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -930,8 +1096,16 @@
       <name val="Times New Roman"/>
       <charset val="134"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -956,8 +1130,14 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -980,32 +1160,43 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="38">
+  <cellXfs count="43">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
@@ -1014,25 +1205,25 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="2" applyFont="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="2" applyBorder="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="2" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1">
@@ -1044,10 +1235,10 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1057,50 +1248,65 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="5" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="justify" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1">
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -1593,15 +1799,15 @@
   <dimension ref="A1:J20"/>
   <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="20.7109375" customWidth="1"/>
-    <col min="2" max="3" width="12.7109375" customWidth="1"/>
-    <col min="4" max="4" width="14.7109375" customWidth="1"/>
-    <col min="5" max="5" width="9.85546875" customWidth="1"/>
-    <col min="6" max="6" width="14.140625" customWidth="1"/>
-    <col min="7" max="7" width="14.85546875" customWidth="1"/>
-    <col min="8" max="8" width="22.28515625" customWidth="1"/>
-    <col min="9" max="9" width="14.42578125" customWidth="1"/>
-    <col min="10" max="10" width="13" customWidth="1"/>
+    <col min="1" max="1" customWidth="true" width="20.7109375"/>
+    <col min="2" max="3" customWidth="true" width="12.7109375"/>
+    <col min="4" max="4" customWidth="true" width="14.7109375"/>
+    <col min="5" max="5" customWidth="true" width="9.85546875"/>
+    <col min="6" max="6" customWidth="true" width="14.140625"/>
+    <col min="7" max="7" customWidth="true" width="14.85546875"/>
+    <col min="8" max="8" customWidth="true" width="22.28515625"/>
+    <col min="9" max="9" customWidth="true" width="14.42578125"/>
+    <col min="10" max="10" customWidth="true" width="13.0"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:10">
@@ -1934,17 +2140,17 @@
   <dimension ref="A1:K6"/>
   <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="9" customWidth="1"/>
-    <col min="2" max="2" width="25.7109375" customWidth="1"/>
-    <col min="3" max="3" width="12.42578125" customWidth="1"/>
-    <col min="4" max="4" width="16.28515625" customWidth="1"/>
-    <col min="5" max="5" width="20.28515625" customWidth="1"/>
-    <col min="6" max="6" width="25.7109375" customWidth="1"/>
-    <col min="7" max="7" width="12.28515625" customWidth="1"/>
-    <col min="8" max="8" width="14.5703125" customWidth="1"/>
-    <col min="9" max="9" width="28.5703125" customWidth="1"/>
-    <col min="10" max="10" width="23" customWidth="1"/>
-    <col min="11" max="11" width="14.7109375" customWidth="1"/>
+    <col min="1" max="1" customWidth="true" width="9.0"/>
+    <col min="2" max="2" customWidth="true" width="25.7109375"/>
+    <col min="3" max="3" customWidth="true" width="12.42578125"/>
+    <col min="4" max="4" customWidth="true" width="16.28515625"/>
+    <col min="5" max="5" customWidth="true" width="20.28515625"/>
+    <col min="6" max="6" customWidth="true" width="25.7109375"/>
+    <col min="7" max="7" customWidth="true" width="12.28515625"/>
+    <col min="8" max="8" customWidth="true" width="14.5703125"/>
+    <col min="9" max="9" customWidth="true" width="28.5703125"/>
+    <col min="10" max="10" customWidth="true" width="23.0"/>
+    <col min="11" max="11" customWidth="true" width="14.7109375"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:11">
@@ -2167,11 +2373,11 @@
   <dimension ref="A1:E4"/>
   <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="13.5703125" customWidth="1"/>
-    <col min="2" max="2" width="6" customWidth="1"/>
-    <col min="3" max="3" width="14.42578125" customWidth="1"/>
-    <col min="4" max="4" width="18.140625" customWidth="1"/>
-    <col min="5" max="5" width="19.5703125" customWidth="1"/>
+    <col min="1" max="1" customWidth="true" width="13.5703125"/>
+    <col min="2" max="2" customWidth="true" width="6.0"/>
+    <col min="3" max="3" customWidth="true" width="14.42578125"/>
+    <col min="4" max="4" customWidth="true" width="18.140625"/>
+    <col min="5" max="5" customWidth="true" width="19.5703125"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5">
@@ -2252,13 +2458,13 @@
   <dimension ref="A1:G14"/>
   <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="25.7109375" customWidth="1"/>
-    <col min="2" max="2" width="8.85546875" customWidth="1"/>
-    <col min="3" max="3" width="12.28515625" customWidth="1"/>
-    <col min="4" max="4" width="7.140625" customWidth="1"/>
-    <col min="5" max="5" width="5.28515625" customWidth="1"/>
-    <col min="6" max="6" width="17.42578125" customWidth="1"/>
-    <col min="7" max="7" width="12.42578125" customWidth="1"/>
+    <col min="1" max="1" customWidth="true" width="25.7109375"/>
+    <col min="2" max="2" customWidth="true" width="8.85546875"/>
+    <col min="3" max="3" customWidth="true" width="12.28515625"/>
+    <col min="4" max="4" customWidth="true" width="7.140625"/>
+    <col min="5" max="5" customWidth="true" width="5.28515625"/>
+    <col min="6" max="6" customWidth="true" width="17.42578125"/>
+    <col min="7" max="7" customWidth="true" width="12.42578125"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7">
@@ -2593,9 +2799,9 @@
   <dimension ref="A1:C3"/>
   <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="25.5703125" customWidth="1"/>
-    <col min="2" max="2" width="15.140625" customWidth="1"/>
-    <col min="3" max="3" width="16.42578125" customWidth="1"/>
+    <col min="1" max="1" customWidth="true" width="25.5703125"/>
+    <col min="2" max="2" customWidth="true" width="15.140625"/>
+    <col min="3" max="3" customWidth="true" width="16.42578125"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3">
@@ -2638,15 +2844,18 @@
 
 <file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C3"/>
+  <dimension ref="A1:F3"/>
   <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="21.42578125" customWidth="1"/>
-    <col min="2" max="2" width="11.5703125" customWidth="1"/>
-    <col min="3" max="3" width="9" customWidth="1"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" width="24.85546875"/>
+    <col min="2" max="2" customWidth="true" width="11.5703125"/>
+    <col min="3" max="3" customWidth="true" width="9.0"/>
+    <col min="4" max="4" bestFit="true" customWidth="true" width="19.28515625"/>
+    <col min="5" max="5" customWidth="true" width="19.28515625"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" width="12.28515625"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3">
+    <row r="1" spans="1:6">
       <c r="A1" s="4" t="s">
         <v>225</v>
       </c>
@@ -2656,27 +2865,56 @@
       <c r="C1" s="4" t="s">
         <v>84</v>
       </c>
-    </row>
-    <row r="2" spans="1:3">
+      <c r="D1" s="38" t="s">
+        <v>269</v>
+      </c>
+      <c r="E1" s="38" t="s">
+        <v>265</v>
+      </c>
+      <c r="F1" s="38" t="s">
+        <v>266</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6">
       <c r="A2" s="3" t="s">
-        <v>230</v>
+        <v>263</v>
       </c>
       <c r="B2" s="3" t="s">
         <v>228</v>
       </c>
       <c r="C2" s="3">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3">
+        <v>10</v>
+      </c>
+      <c r="D2" t="s" s="0">
+        <v>268</v>
+      </c>
+      <c r="E2" t="s" s="0">
+        <v>270</v>
+      </c>
+      <c r="F2" s="0">
+        <f>ROUND(C2*E2,2)</f>
+        <v>847.48</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6">
       <c r="A3" s="3" t="s">
-        <v>231</v>
+        <v>114</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>228</v>
+        <v>264</v>
       </c>
       <c r="C3" s="3">
-        <v>2</v>
+        <v>12</v>
+      </c>
+      <c r="D3" t="s" s="0">
+        <v>271</v>
+      </c>
+      <c r="E3" t="s" s="0">
+        <v>267</v>
+      </c>
+      <c r="F3" s="0">
+        <f>ROUND(C3*E3,2)</f>
+        <v>159.26</v>
       </c>
     </row>
   </sheetData>
@@ -2686,26 +2924,45 @@
 
 <file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B2"/>
-  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15"/>
+  <dimension ref="A1:C3"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="20.42578125" customWidth="1"/>
+    <col min="1" max="1" customWidth="true" width="21.42578125"/>
+    <col min="2" max="2" customWidth="true" width="11.5703125"/>
+    <col min="3" max="3" customWidth="true" width="9.0"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2">
-      <c r="A1" s="10" t="s">
-        <v>232</v>
-      </c>
-      <c r="B1" s="10" t="s">
+    <row r="1" spans="1:3">
+      <c r="A1" s="4" t="s">
+        <v>225</v>
+      </c>
+      <c r="B1" s="4" t="s">
+        <v>226</v>
+      </c>
+      <c r="C1" s="4" t="s">
         <v>84</v>
       </c>
     </row>
-    <row r="2" spans="1:2">
-      <c r="A2" s="10" t="s">
-        <v>233</v>
-      </c>
-      <c r="B2" s="10">
-        <v>10</v>
+    <row r="2" spans="1:3">
+      <c r="A2" s="3" t="s">
+        <v>230</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>228</v>
+      </c>
+      <c r="C2" s="3">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3">
+      <c r="A3" s="3" t="s">
+        <v>231</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>228</v>
+      </c>
+      <c r="C3" s="3">
+        <v>2</v>
       </c>
     </row>
   </sheetData>
@@ -2715,75 +2972,27 @@
 
 <file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G3"/>
+  <dimension ref="A1:B2"/>
   <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" customWidth="true" width="20.42578125"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:7">
-      <c r="A1" s="9" t="s">
-        <v>234</v>
-      </c>
-      <c r="B1" s="9" t="s">
+    <row r="1" spans="1:2">
+      <c r="A1" s="10" t="s">
+        <v>232</v>
+      </c>
+      <c r="B1" s="10" t="s">
         <v>84</v>
       </c>
-      <c r="C1" s="9" t="s">
-        <v>80</v>
-      </c>
-      <c r="D1" s="9" t="s">
-        <v>85</v>
-      </c>
-      <c r="E1" s="9" t="s">
-        <v>68</v>
-      </c>
-      <c r="F1" s="9" t="s">
-        <v>69</v>
-      </c>
-      <c r="G1" s="9" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="2" spans="1:7">
-      <c r="A2" s="12" t="s">
-        <v>235</v>
-      </c>
-      <c r="B2" s="9">
-        <v>22</v>
-      </c>
-      <c r="C2" s="9">
-        <v>524</v>
-      </c>
-      <c r="D2" s="9">
-        <v>2</v>
-      </c>
-      <c r="E2" s="12" t="s">
-        <v>73</v>
-      </c>
-      <c r="F2" s="12" t="s">
-        <v>74</v>
-      </c>
-      <c r="G2" s="12" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="3" spans="1:7">
-      <c r="A3" s="12" t="s">
-        <v>236</v>
-      </c>
-      <c r="B3" s="9">
-        <v>34</v>
-      </c>
-      <c r="C3" s="9">
-        <v>232</v>
-      </c>
-      <c r="D3" s="9">
-        <v>7.9</v>
-      </c>
-      <c r="E3" s="12" t="s">
-        <v>73</v>
-      </c>
-      <c r="F3" s="12" t="s">
-        <v>89</v>
-      </c>
-      <c r="G3" s="13"/>
+    </row>
+    <row r="2" spans="1:2">
+      <c r="A2" s="10" t="s">
+        <v>233</v>
+      </c>
+      <c r="B2" s="10">
+        <v>10</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2792,10 +3001,10 @@
 
 <file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C3"/>
+  <dimension ref="A1:G3"/>
   <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:3">
+    <row r="1" spans="1:7">
       <c r="A1" s="9" t="s">
         <v>234</v>
       </c>
@@ -2805,10 +3014,22 @@
       <c r="C1" s="9" t="s">
         <v>80</v>
       </c>
-    </row>
-    <row r="2" spans="1:3">
-      <c r="A2" s="11" t="s">
-        <v>237</v>
+      <c r="D1" s="9" t="s">
+        <v>85</v>
+      </c>
+      <c r="E1" s="9" t="s">
+        <v>68</v>
+      </c>
+      <c r="F1" s="9" t="s">
+        <v>69</v>
+      </c>
+      <c r="G1" s="9" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7">
+      <c r="A2" s="12" t="s">
+        <v>235</v>
       </c>
       <c r="B2" s="9">
         <v>22</v>
@@ -2816,17 +3037,39 @@
       <c r="C2" s="9">
         <v>524</v>
       </c>
-    </row>
-    <row r="3" spans="1:3">
-      <c r="A3" s="11" t="s">
-        <v>238</v>
+      <c r="D2" s="9">
+        <v>2</v>
+      </c>
+      <c r="E2" s="12" t="s">
+        <v>73</v>
+      </c>
+      <c r="F2" s="12" t="s">
+        <v>74</v>
+      </c>
+      <c r="G2" s="12" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7">
+      <c r="A3" s="12" t="s">
+        <v>236</v>
       </c>
       <c r="B3" s="9">
-        <v>40</v>
+        <v>34</v>
       </c>
       <c r="C3" s="9">
-        <v>450</v>
-      </c>
+        <v>232</v>
+      </c>
+      <c r="D3" s="9">
+        <v>7.9</v>
+      </c>
+      <c r="E3" s="12" t="s">
+        <v>73</v>
+      </c>
+      <c r="F3" s="12" t="s">
+        <v>89</v>
+      </c>
+      <c r="G3" s="13"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2835,23 +3078,40 @@
 
 <file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B2"/>
+  <dimension ref="A1:C3"/>
   <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:2">
-      <c r="A1" s="10" t="s">
-        <v>239</v>
-      </c>
-      <c r="B1" s="10" t="s">
+    <row r="1" spans="1:3">
+      <c r="A1" s="9" t="s">
+        <v>234</v>
+      </c>
+      <c r="B1" s="9" t="s">
         <v>84</v>
       </c>
-    </row>
-    <row r="2" spans="1:2">
-      <c r="A2" s="10" t="s">
-        <v>240</v>
-      </c>
-      <c r="B2" s="10">
-        <v>10</v>
+      <c r="C1" s="9" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3">
+      <c r="A2" s="11" t="s">
+        <v>237</v>
+      </c>
+      <c r="B2" s="9">
+        <v>22</v>
+      </c>
+      <c r="C2" s="9">
+        <v>524</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3">
+      <c r="A3" s="11" t="s">
+        <v>238</v>
+      </c>
+      <c r="B3" s="9">
+        <v>40</v>
+      </c>
+      <c r="C3" s="9">
+        <v>450</v>
       </c>
     </row>
   </sheetData>
@@ -2861,34 +3121,23 @@
 
 <file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C3"/>
+  <dimension ref="A1:B2"/>
   <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:3">
-      <c r="A1" t="s">
-        <v>234</v>
-      </c>
-      <c r="B1" s="9" t="s">
+    <row r="1" spans="1:2">
+      <c r="A1" s="10" t="s">
+        <v>239</v>
+      </c>
+      <c r="B1" s="10" t="s">
         <v>84</v>
       </c>
-      <c r="C1" s="9" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3">
-      <c r="A2" t="s">
-        <v>241</v>
-      </c>
-      <c r="B2">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3">
-      <c r="A3" t="s">
-        <v>242</v>
-      </c>
-      <c r="B3">
-        <v>45</v>
+    </row>
+    <row r="2" spans="1:2">
+      <c r="A2" s="10" t="s">
+        <v>240</v>
+      </c>
+      <c r="B2" s="10">
+        <v>10</v>
       </c>
     </row>
   </sheetData>
@@ -2901,26 +3150,26 @@
   <dimension ref="A1:T10"/>
   <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="30" customWidth="1"/>
-    <col min="2" max="2" width="36.42578125" customWidth="1"/>
-    <col min="3" max="3" width="6" customWidth="1"/>
-    <col min="4" max="4" width="13.7109375" customWidth="1"/>
-    <col min="5" max="5" width="5.28515625" customWidth="1"/>
-    <col min="6" max="6" width="17.28515625" customWidth="1"/>
-    <col min="7" max="7" width="30.28515625" customWidth="1"/>
-    <col min="8" max="8" width="26.85546875" customWidth="1"/>
-    <col min="9" max="9" width="17.28515625" customWidth="1"/>
-    <col min="10" max="10" width="13.28515625" customWidth="1"/>
-    <col min="11" max="11" width="22.7109375" customWidth="1"/>
-    <col min="12" max="12" width="12.7109375" customWidth="1"/>
-    <col min="13" max="13" width="29.5703125" customWidth="1"/>
-    <col min="14" max="14" width="18.28515625" customWidth="1"/>
-    <col min="15" max="15" width="16.28515625" customWidth="1"/>
-    <col min="16" max="16" width="15.5703125" customWidth="1"/>
-    <col min="17" max="17" width="17.7109375" customWidth="1"/>
-    <col min="18" max="18" width="24.140625" customWidth="1"/>
-    <col min="19" max="19" width="13.42578125" customWidth="1"/>
-    <col min="20" max="20" width="13.5703125" customWidth="1"/>
+    <col min="1" max="1" customWidth="true" width="30.0"/>
+    <col min="2" max="2" customWidth="true" width="36.42578125"/>
+    <col min="3" max="3" customWidth="true" width="6.0"/>
+    <col min="4" max="4" customWidth="true" width="13.7109375"/>
+    <col min="5" max="5" customWidth="true" width="5.28515625"/>
+    <col min="6" max="6" customWidth="true" width="17.28515625"/>
+    <col min="7" max="7" customWidth="true" width="30.28515625"/>
+    <col min="8" max="8" customWidth="true" width="26.85546875"/>
+    <col min="9" max="9" customWidth="true" width="17.28515625"/>
+    <col min="10" max="10" customWidth="true" width="13.28515625"/>
+    <col min="11" max="11" customWidth="true" width="22.7109375"/>
+    <col min="12" max="12" customWidth="true" width="12.7109375"/>
+    <col min="13" max="13" customWidth="true" width="29.5703125"/>
+    <col min="14" max="14" customWidth="true" width="18.28515625"/>
+    <col min="15" max="15" customWidth="true" width="16.28515625"/>
+    <col min="16" max="16" customWidth="true" width="15.5703125"/>
+    <col min="17" max="17" customWidth="true" width="17.7109375"/>
+    <col min="18" max="18" customWidth="true" width="24.140625"/>
+    <col min="19" max="19" customWidth="true" width="13.42578125"/>
+    <col min="20" max="20" customWidth="true" width="13.5703125"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:20">
@@ -3214,7 +3463,7 @@
       <c r="D6" s="24" t="s">
         <v>43</v>
       </c>
-      <c r="E6">
+      <c r="E6" s="0">
         <v>5</v>
       </c>
       <c r="F6" s="29" t="s">
@@ -3478,74 +3727,35 @@
 
 <file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F3"/>
+  <dimension ref="A1:C3"/>
   <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15"/>
-  <cols>
-    <col min="1" max="1" width="23.28515625" customWidth="1"/>
-    <col min="2" max="2" width="10.42578125" customWidth="1"/>
-    <col min="3" max="3" width="11.42578125" customWidth="1"/>
-    <col min="4" max="4" width="11.7109375" customWidth="1"/>
-    <col min="5" max="5" width="14.5703125" customWidth="1"/>
-    <col min="6" max="6" width="17.7109375" customWidth="1"/>
-  </cols>
   <sheetData>
-    <row r="1" spans="1:6">
-      <c r="A1" s="5" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="5" t="s">
-        <v>66</v>
-      </c>
-      <c r="C1" s="5" t="s">
-        <v>67</v>
-      </c>
-      <c r="D1" s="6" t="s">
-        <v>68</v>
-      </c>
-      <c r="E1" s="7" t="s">
-        <v>69</v>
-      </c>
-      <c r="F1" s="7" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="2" spans="1:6">
-      <c r="A2" s="7" t="s">
-        <v>243</v>
-      </c>
-      <c r="B2" s="3">
-        <v>10</v>
-      </c>
-      <c r="C2" s="3">
+    <row r="1" spans="1:3">
+      <c r="A1" t="s" s="0">
+        <v>234</v>
+      </c>
+      <c r="B1" s="9" t="s">
+        <v>84</v>
+      </c>
+      <c r="C1" s="9" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3">
+      <c r="A2" t="s" s="0">
+        <v>241</v>
+      </c>
+      <c r="B2" s="0">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3">
+      <c r="A3" t="s" s="0">
+        <v>242</v>
+      </c>
+      <c r="B3" s="0">
         <v>45</v>
       </c>
-      <c r="D2" s="3" t="s">
-        <v>73</v>
-      </c>
-      <c r="E2" s="8" t="s">
-        <v>244</v>
-      </c>
-      <c r="F2" s="8" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6">
-      <c r="A3" s="7" t="s">
-        <v>245</v>
-      </c>
-      <c r="B3" s="3">
-        <v>50</v>
-      </c>
-      <c r="C3" s="3">
-        <v>70</v>
-      </c>
-      <c r="D3" s="3" t="s">
-        <v>77</v>
-      </c>
-      <c r="E3" s="3" t="s">
-        <v>75</v>
-      </c>
-      <c r="F3" s="8"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -3555,75 +3765,73 @@
 <file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:F3"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="20.85546875" customWidth="1"/>
-    <col min="2" max="2" width="9" customWidth="1"/>
-    <col min="3" max="3" width="8.85546875" customWidth="1"/>
-    <col min="4" max="4" width="6.140625" customWidth="1"/>
-    <col min="5" max="5" width="16.7109375" customWidth="1"/>
-    <col min="6" max="6" width="16.28515625" customWidth="1"/>
+    <col min="1" max="1" customWidth="true" width="23.28515625"/>
+    <col min="2" max="2" customWidth="true" width="10.42578125"/>
+    <col min="3" max="3" customWidth="true" width="11.42578125"/>
+    <col min="4" max="4" customWidth="true" width="11.7109375"/>
+    <col min="5" max="5" customWidth="true" width="14.5703125"/>
+    <col min="6" max="6" customWidth="true" width="17.7109375"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6">
-      <c r="A1" s="4" t="s">
-        <v>225</v>
-      </c>
-      <c r="B1" s="4" t="s">
-        <v>84</v>
-      </c>
-      <c r="C1" s="4" t="s">
-        <v>80</v>
-      </c>
-      <c r="D1" s="4" t="s">
-        <v>27</v>
-      </c>
-      <c r="E1" s="2" t="s">
-        <v>246</v>
-      </c>
-      <c r="F1" s="2" t="s">
-        <v>247</v>
+      <c r="A1" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="5" t="s">
+        <v>66</v>
+      </c>
+      <c r="C1" s="5" t="s">
+        <v>67</v>
+      </c>
+      <c r="D1" s="6" t="s">
+        <v>68</v>
+      </c>
+      <c r="E1" s="7" t="s">
+        <v>69</v>
+      </c>
+      <c r="F1" s="7" t="s">
+        <v>70</v>
       </c>
     </row>
     <row r="2" spans="1:6">
-      <c r="A2" s="3" t="s">
-        <v>10</v>
+      <c r="A2" s="7" t="s">
+        <v>243</v>
       </c>
       <c r="B2" s="3">
         <v>10</v>
       </c>
       <c r="C2" s="3">
-        <v>200</v>
+        <v>45</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="E2" s="3">
-        <v>5</v>
-      </c>
-      <c r="F2" s="3">
-        <v>6</v>
+        <v>73</v>
+      </c>
+      <c r="E2" s="8" t="s">
+        <v>244</v>
+      </c>
+      <c r="F2" s="8" t="s">
+        <v>75</v>
       </c>
     </row>
     <row r="3" spans="1:6">
-      <c r="A3" s="3" t="s">
-        <v>248</v>
+      <c r="A3" s="7" t="s">
+        <v>245</v>
       </c>
       <c r="B3" s="3">
-        <v>15</v>
+        <v>50</v>
       </c>
       <c r="C3" s="3">
-        <v>250</v>
+        <v>70</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="E3" s="3">
-        <v>15</v>
-      </c>
-      <c r="F3" s="3">
-        <v>5</v>
-      </c>
+        <v>77</v>
+      </c>
+      <c r="E3" s="3" t="s">
+        <v>75</v>
+      </c>
+      <c r="F3" s="8"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -3635,12 +3843,12 @@
   <dimension ref="A1:F3"/>
   <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="21.7109375" customWidth="1"/>
-    <col min="2" max="2" width="9" customWidth="1"/>
-    <col min="3" max="3" width="8.85546875" customWidth="1"/>
-    <col min="4" max="4" width="6.140625" customWidth="1"/>
-    <col min="5" max="5" width="16.7109375" customWidth="1"/>
-    <col min="6" max="6" width="16.28515625" customWidth="1"/>
+    <col min="1" max="1" customWidth="true" width="20.85546875"/>
+    <col min="2" max="2" customWidth="true" width="9.0"/>
+    <col min="3" max="3" customWidth="true" width="8.85546875"/>
+    <col min="4" max="4" customWidth="true" width="6.140625"/>
+    <col min="5" max="5" customWidth="true" width="16.7109375"/>
+    <col min="6" max="6" customWidth="true" width="16.28515625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6">
@@ -3665,7 +3873,7 @@
     </row>
     <row r="2" spans="1:6">
       <c r="A2" s="3" t="s">
-        <v>21</v>
+        <v>10</v>
       </c>
       <c r="B2" s="3">
         <v>10</v>
@@ -3685,7 +3893,7 @@
     </row>
     <row r="3" spans="1:6">
       <c r="A3" s="3" t="s">
-        <v>62</v>
+        <v>248</v>
       </c>
       <c r="B3" s="3">
         <v>15</v>
@@ -3713,72 +3921,72 @@
   <dimension ref="A1:F3"/>
   <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="15.42578125" customWidth="1"/>
-    <col min="2" max="2" width="10.5703125" customWidth="1"/>
-    <col min="3" max="3" width="11.5703125" customWidth="1"/>
-    <col min="4" max="4" width="11.85546875" customWidth="1"/>
-    <col min="5" max="5" width="14" customWidth="1"/>
-    <col min="6" max="6" width="16.85546875" customWidth="1"/>
+    <col min="1" max="1" customWidth="true" width="21.7109375"/>
+    <col min="2" max="2" customWidth="true" width="9.0"/>
+    <col min="3" max="3" customWidth="true" width="8.85546875"/>
+    <col min="4" max="4" customWidth="true" width="6.140625"/>
+    <col min="5" max="5" customWidth="true" width="16.7109375"/>
+    <col min="6" max="6" customWidth="true" width="16.28515625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6">
-      <c r="A1" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="2" t="s">
-        <v>66</v>
-      </c>
-      <c r="C1" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="D1" s="2" t="s">
-        <v>68</v>
+      <c r="A1" s="4" t="s">
+        <v>225</v>
+      </c>
+      <c r="B1" s="4" t="s">
+        <v>84</v>
+      </c>
+      <c r="C1" s="4" t="s">
+        <v>80</v>
+      </c>
+      <c r="D1" s="4" t="s">
+        <v>27</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>69</v>
+        <v>246</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>70</v>
+        <v>247</v>
       </c>
     </row>
     <row r="2" spans="1:6">
       <c r="A2" s="3" t="s">
-        <v>243</v>
+        <v>21</v>
       </c>
       <c r="B2" s="3">
         <v>10</v>
       </c>
       <c r="C2" s="3">
-        <v>45</v>
+        <v>200</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>73</v>
-      </c>
-      <c r="E2" s="3" t="s">
-        <v>244</v>
-      </c>
-      <c r="F2" s="3" t="s">
-        <v>75</v>
+        <v>14</v>
+      </c>
+      <c r="E2" s="3">
+        <v>5</v>
+      </c>
+      <c r="F2" s="3">
+        <v>6</v>
       </c>
     </row>
     <row r="3" spans="1:6">
       <c r="A3" s="3" t="s">
-        <v>249</v>
+        <v>62</v>
       </c>
       <c r="B3" s="3">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="C3" s="3">
-        <v>40</v>
+        <v>250</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>73</v>
-      </c>
-      <c r="E3" s="3" t="s">
-        <v>250</v>
-      </c>
-      <c r="F3" s="3" t="s">
-        <v>75</v>
+        <v>14</v>
+      </c>
+      <c r="E3" s="3">
+        <v>15</v>
+      </c>
+      <c r="F3" s="3">
+        <v>5</v>
       </c>
     </row>
   </sheetData>
@@ -3788,77 +3996,121 @@
 
 <file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C3"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
+  <dimension ref="A1:F3"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="15" customWidth="1"/>
+    <col min="1" max="1" customWidth="true" width="15.42578125"/>
+    <col min="2" max="2" customWidth="true" width="10.5703125"/>
+    <col min="3" max="3" customWidth="true" width="11.5703125"/>
+    <col min="4" max="4" customWidth="true" width="11.85546875"/>
+    <col min="5" max="5" customWidth="true" width="14.0"/>
+    <col min="6" max="6" customWidth="true" width="16.85546875"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3">
-      <c r="A1" t="s">
-        <v>251</v>
-      </c>
-      <c r="B1" t="s">
-        <v>79</v>
-      </c>
-      <c r="C1" t="s">
-        <v>252</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3">
-      <c r="A2" t="s">
-        <v>253</v>
-      </c>
-      <c r="B2">
-        <v>5</v>
-      </c>
-      <c r="C2">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3">
-      <c r="A3" t="s">
-        <v>254</v>
-      </c>
-      <c r="B3">
-        <v>6</v>
-      </c>
-      <c r="C3">
-        <v>200</v>
+    <row r="1" spans="1:6">
+      <c r="A1" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6">
+      <c r="A2" s="3" t="s">
+        <v>243</v>
+      </c>
+      <c r="B2" s="3">
+        <v>10</v>
+      </c>
+      <c r="C2" s="3">
+        <v>45</v>
+      </c>
+      <c r="D2" s="3" t="s">
+        <v>73</v>
+      </c>
+      <c r="E2" s="3" t="s">
+        <v>244</v>
+      </c>
+      <c r="F2" s="3" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6">
+      <c r="A3" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="B3" s="3">
+        <v>20</v>
+      </c>
+      <c r="C3" s="3">
+        <v>40</v>
+      </c>
+      <c r="D3" s="3" t="s">
+        <v>73</v>
+      </c>
+      <c r="E3" s="3" t="s">
+        <v>250</v>
+      </c>
+      <c r="F3" s="3" t="s">
+        <v>75</v>
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet25.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B3"/>
+  <dimension ref="A1:C3"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" customWidth="true" width="15.0"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:2">
-      <c r="A1" t="s">
-        <v>255</v>
-      </c>
-      <c r="B1" t="s">
-        <v>256</v>
-      </c>
-    </row>
-    <row r="2" spans="1:2">
-      <c r="A2" t="s">
-        <v>257</v>
-      </c>
-      <c r="B2" t="s">
-        <v>209</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2">
-      <c r="A3" t="s">
-        <v>258</v>
-      </c>
-      <c r="B3" t="s">
-        <v>207</v>
+    <row r="1" spans="1:3">
+      <c r="A1" t="s" s="0">
+        <v>251</v>
+      </c>
+      <c r="B1" t="s" s="0">
+        <v>79</v>
+      </c>
+      <c r="C1" t="s" s="0">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3">
+      <c r="A2" t="s" s="0">
+        <v>253</v>
+      </c>
+      <c r="B2" s="0">
+        <v>5</v>
+      </c>
+      <c r="C2" s="0">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3">
+      <c r="A3" t="s" s="0">
+        <v>254</v>
+      </c>
+      <c r="B3" s="0">
+        <v>6</v>
+      </c>
+      <c r="C3" s="0">
+        <v>200</v>
       </c>
     </row>
   </sheetData>
@@ -3872,26 +4124,26 @@
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:2">
-      <c r="A1" t="s">
+      <c r="A1" t="s" s="0">
         <v>255</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" t="s" s="0">
         <v>256</v>
       </c>
     </row>
     <row r="2" spans="1:2">
-      <c r="A2" t="s">
+      <c r="A2" t="s" s="0">
+        <v>257</v>
+      </c>
+      <c r="B2" t="s" s="0">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2">
+      <c r="A3" t="s" s="0">
         <v>258</v>
       </c>
-      <c r="B2" t="s">
-        <v>209</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2">
-      <c r="A3" t="s">
-        <v>259</v>
-      </c>
-      <c r="B3" t="s">
+      <c r="B3" t="s" s="0">
         <v>207</v>
       </c>
     </row>
@@ -3902,12 +4154,46 @@
 
 <file path=xl/worksheets/sheet27.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:B3"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1" spans="1:2">
+      <c r="A1" t="s" s="0">
+        <v>255</v>
+      </c>
+      <c r="B1" t="s" s="0">
+        <v>256</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2">
+      <c r="A2" t="s" s="0">
+        <v>258</v>
+      </c>
+      <c r="B2" t="s" s="0">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2">
+      <c r="A3" t="s" s="0">
+        <v>259</v>
+      </c>
+      <c r="B3" t="s" s="0">
+        <v>207</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet28.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:C3"/>
   <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="15.7109375" customWidth="1"/>
-    <col min="2" max="2" width="5" customWidth="1"/>
-    <col min="3" max="3" width="6" customWidth="1"/>
+    <col min="1" max="1" customWidth="true" width="15.7109375"/>
+    <col min="2" max="2" customWidth="true" width="5.0"/>
+    <col min="3" max="3" customWidth="true" width="6.0"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3">
@@ -3945,6 +4231,167 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet29.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:O3"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" bestFit="true" customWidth="true" width="4.85546875"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" width="7.0"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" width="28.7109375"/>
+    <col min="4" max="4" bestFit="true" customWidth="true" width="9.28515625"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" width="28.7109375"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" width="4.5703125"/>
+    <col min="7" max="7" bestFit="true" customWidth="true" width="10.42578125"/>
+    <col min="8" max="8" bestFit="true" customWidth="true" width="13.140625"/>
+    <col min="9" max="9" bestFit="true" customWidth="true" width="8.28515625"/>
+    <col min="10" max="10" bestFit="true" customWidth="true" width="21.5703125"/>
+    <col min="11" max="11" bestFit="true" customWidth="true" width="16.0"/>
+    <col min="12" max="12" bestFit="true" customWidth="true" width="18.140625"/>
+    <col min="13" max="13" bestFit="true" customWidth="true" width="16.7109375"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:15">
+      <c r="A1" s="39" t="s">
+        <v>272</v>
+      </c>
+      <c r="B1" s="39" t="s">
+        <v>283</v>
+      </c>
+      <c r="C1" s="39" t="s">
+        <v>273</v>
+      </c>
+      <c r="D1" s="39" t="s">
+        <v>274</v>
+      </c>
+      <c r="E1" s="39" t="s">
+        <v>275</v>
+      </c>
+      <c r="F1" s="39" t="s">
+        <v>79</v>
+      </c>
+      <c r="G1" s="39" t="s">
+        <v>276</v>
+      </c>
+      <c r="H1" s="39" t="s">
+        <v>277</v>
+      </c>
+      <c r="I1" s="39" t="s">
+        <v>278</v>
+      </c>
+      <c r="J1" s="39" t="s">
+        <v>282</v>
+      </c>
+      <c r="K1" s="39" t="s">
+        <v>279</v>
+      </c>
+      <c r="L1" s="42" t="s">
+        <v>286</v>
+      </c>
+      <c r="M1" s="42" t="s">
+        <v>287</v>
+      </c>
+      <c r="N1" s="42" t="s">
+        <v>292</v>
+      </c>
+      <c r="O1" s="42" t="s">
+        <v>293</v>
+      </c>
+    </row>
+    <row r="2" spans="1:15">
+      <c r="A2" s="3">
+        <v>1</v>
+      </c>
+      <c r="B2" s="40" t="s">
+        <v>284</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>280</v>
+      </c>
+      <c r="D2" s="3">
+        <v>0</v>
+      </c>
+      <c r="E2" s="40" t="s">
+        <v>280</v>
+      </c>
+      <c r="F2" s="3">
+        <v>100</v>
+      </c>
+      <c r="G2" s="3">
+        <v>1200</v>
+      </c>
+      <c r="H2" t="s" s="0">
+        <v>309</v>
+      </c>
+      <c r="I2" s="3">
+        <v>100</v>
+      </c>
+      <c r="J2" s="40"/>
+      <c r="K2" s="40" t="s">
+        <v>281</v>
+      </c>
+      <c r="L2" t="s" s="0">
+        <v>310</v>
+      </c>
+      <c r="M2" s="0">
+        <f>SUM(L2+F2)</f>
+        <v>100</v>
+      </c>
+      <c r="N2" t="str" s="0">
+        <f>H2</f>
+        <v>500003</v>
+      </c>
+      <c r="O2" t="str" s="0">
+        <f>H2</f>
+        <v>500003</v>
+      </c>
+    </row>
+    <row r="3" spans="1:15">
+      <c r="A3" s="3">
+        <v>2</v>
+      </c>
+      <c r="B3" s="40" t="s">
+        <v>284</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>285</v>
+      </c>
+      <c r="D3" s="3">
+        <v>0</v>
+      </c>
+      <c r="E3" s="3" t="s">
+        <v>285</v>
+      </c>
+      <c r="F3" s="3">
+        <v>10</v>
+      </c>
+      <c r="G3" s="3">
+        <v>3244</v>
+      </c>
+      <c r="H3" s="41"/>
+      <c r="I3" s="3">
+        <v>10</v>
+      </c>
+      <c r="J3" t="s" s="0">
+        <v>312</v>
+      </c>
+      <c r="K3" s="40" t="s">
+        <v>281</v>
+      </c>
+      <c r="L3" t="s" s="0">
+        <v>311</v>
+      </c>
+      <c r="M3" s="0">
+        <f>SUM(L3+F3)</f>
+        <v>10</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -3953,17 +4400,17 @@
   <dimension ref="A1:R3"/>
   <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="2" width="21" customWidth="1"/>
-    <col min="3" max="3" width="6" customWidth="1"/>
-    <col min="4" max="4" width="12.7109375" customWidth="1"/>
-    <col min="5" max="5" width="19.42578125" customWidth="1"/>
-    <col min="6" max="6" width="15.140625" customWidth="1"/>
-    <col min="7" max="7" width="15.42578125" customWidth="1"/>
-    <col min="8" max="8" width="19.5703125" customWidth="1"/>
-    <col min="9" max="9" width="10.85546875" customWidth="1"/>
-    <col min="10" max="10" width="17.5703125" customWidth="1"/>
-    <col min="11" max="11" width="11.28515625" customWidth="1"/>
-    <col min="12" max="12" width="21.7109375" customWidth="1"/>
+    <col min="1" max="2" customWidth="true" width="21.0"/>
+    <col min="3" max="3" customWidth="true" width="6.0"/>
+    <col min="4" max="4" customWidth="true" width="12.7109375"/>
+    <col min="5" max="5" customWidth="true" width="19.42578125"/>
+    <col min="6" max="6" customWidth="true" width="15.140625"/>
+    <col min="7" max="7" customWidth="true" width="15.42578125"/>
+    <col min="8" max="8" customWidth="true" width="19.5703125"/>
+    <col min="9" max="9" customWidth="true" width="10.85546875"/>
+    <col min="10" max="10" customWidth="true" width="17.5703125"/>
+    <col min="11" max="11" customWidth="true" width="11.28515625"/>
+    <col min="12" max="12" customWidth="true" width="21.7109375"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:18">
@@ -4102,12 +4549,12 @@
   <dimension ref="A1:F3"/>
   <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="27.140625" customWidth="1"/>
-    <col min="2" max="2" width="10.42578125" customWidth="1"/>
-    <col min="3" max="3" width="11.42578125" customWidth="1"/>
-    <col min="4" max="4" width="11.7109375" customWidth="1"/>
-    <col min="5" max="5" width="14.5703125" customWidth="1"/>
-    <col min="6" max="6" width="17.7109375" customWidth="1"/>
+    <col min="1" max="1" customWidth="true" width="27.140625"/>
+    <col min="2" max="2" customWidth="true" width="10.42578125"/>
+    <col min="3" max="3" customWidth="true" width="11.42578125"/>
+    <col min="4" max="4" customWidth="true" width="11.7109375"/>
+    <col min="5" max="5" customWidth="true" width="14.5703125"/>
+    <col min="6" max="6" customWidth="true" width="17.7109375"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6">
@@ -4178,12 +4625,12 @@
   <dimension ref="A1:F4"/>
   <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="27.140625" customWidth="1"/>
-    <col min="2" max="2" width="10.42578125" customWidth="1"/>
-    <col min="3" max="3" width="11.42578125" customWidth="1"/>
-    <col min="4" max="4" width="11.7109375" customWidth="1"/>
-    <col min="5" max="5" width="14.5703125" customWidth="1"/>
-    <col min="6" max="6" width="17.7109375" customWidth="1"/>
+    <col min="1" max="1" customWidth="true" width="27.140625"/>
+    <col min="2" max="2" customWidth="true" width="10.42578125"/>
+    <col min="3" max="3" customWidth="true" width="11.42578125"/>
+    <col min="4" max="4" customWidth="true" width="11.7109375"/>
+    <col min="5" max="5" customWidth="true" width="14.5703125"/>
+    <col min="6" max="6" customWidth="true" width="17.7109375"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6">
@@ -4272,39 +4719,39 @@
   <dimension ref="A1:C3"/>
   <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="28.7109375" customWidth="1"/>
+    <col min="1" max="1" customWidth="true" width="28.7109375"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3">
-      <c r="A1" t="s">
+      <c r="A1" t="s" s="0">
         <v>78</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" t="s" s="0">
         <v>79</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" t="s" s="0">
         <v>80</v>
       </c>
     </row>
     <row r="2" spans="1:3">
-      <c r="A2" t="s">
+      <c r="A2" t="s" s="0">
         <v>81</v>
       </c>
-      <c r="B2">
+      <c r="B2" s="0">
         <v>100</v>
       </c>
-      <c r="C2">
+      <c r="C2" s="0">
         <v>34</v>
       </c>
     </row>
     <row r="3" spans="1:3">
-      <c r="A3" t="s">
+      <c r="A3" t="s" s="0">
         <v>82</v>
       </c>
-      <c r="B3">
+      <c r="B3" s="0">
         <v>50</v>
       </c>
-      <c r="C3">
+      <c r="C3" s="0">
         <v>30</v>
       </c>
     </row>
@@ -4318,13 +4765,13 @@
   <dimension ref="A1:G4"/>
   <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="19.7109375" customWidth="1"/>
-    <col min="2" max="2" width="8.140625" customWidth="1"/>
-    <col min="3" max="3" width="8.5703125" customWidth="1"/>
-    <col min="4" max="4" width="17.85546875" customWidth="1"/>
-    <col min="5" max="5" width="12.7109375" customWidth="1"/>
-    <col min="6" max="6" width="14.5703125" customWidth="1"/>
-    <col min="7" max="7" width="17.7109375" customWidth="1"/>
+    <col min="1" max="1" customWidth="true" width="19.7109375"/>
+    <col min="2" max="2" customWidth="true" width="8.140625"/>
+    <col min="3" max="3" customWidth="true" width="8.5703125"/>
+    <col min="4" max="4" customWidth="true" width="17.85546875"/>
+    <col min="5" max="5" customWidth="true" width="12.7109375"/>
+    <col min="6" max="6" customWidth="true" width="14.5703125"/>
+    <col min="7" max="7" customWidth="true" width="17.7109375"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7">
@@ -4423,13 +4870,13 @@
   <dimension ref="A1:G4"/>
   <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="19.7109375" customWidth="1"/>
-    <col min="2" max="2" width="8.140625" customWidth="1"/>
-    <col min="3" max="3" width="8.5703125" customWidth="1"/>
-    <col min="4" max="4" width="17.85546875" customWidth="1"/>
-    <col min="5" max="5" width="12.7109375" customWidth="1"/>
-    <col min="6" max="6" width="14.5703125" customWidth="1"/>
-    <col min="7" max="7" width="17.7109375" customWidth="1"/>
+    <col min="1" max="1" customWidth="true" width="19.7109375"/>
+    <col min="2" max="2" customWidth="true" width="8.140625"/>
+    <col min="3" max="3" customWidth="true" width="8.5703125"/>
+    <col min="4" max="4" customWidth="true" width="17.85546875"/>
+    <col min="5" max="5" customWidth="true" width="12.7109375"/>
+    <col min="6" max="6" customWidth="true" width="14.5703125"/>
+    <col min="7" max="7" customWidth="true" width="17.7109375"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7">
@@ -4528,23 +4975,23 @@
   <dimension ref="A1:S17"/>
   <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="39.7109375" customWidth="1"/>
-    <col min="2" max="2" width="10.140625" customWidth="1"/>
-    <col min="3" max="3" width="39.7109375" customWidth="1"/>
-    <col min="4" max="4" width="11" customWidth="1"/>
-    <col min="5" max="5" width="13.28515625" customWidth="1"/>
-    <col min="6" max="6" width="8.85546875" customWidth="1"/>
-    <col min="7" max="7" width="17.85546875" customWidth="1"/>
-    <col min="8" max="8" width="19.5703125" customWidth="1"/>
-    <col min="9" max="9" width="23.7109375" customWidth="1"/>
-    <col min="10" max="10" width="12.7109375" customWidth="1"/>
-    <col min="11" max="11" width="11.85546875" customWidth="1"/>
-    <col min="12" max="12" width="17.42578125" customWidth="1"/>
-    <col min="13" max="14" width="39.7109375" customWidth="1"/>
-    <col min="15" max="15" width="25.7109375" customWidth="1"/>
-    <col min="16" max="17" width="16.5703125" customWidth="1"/>
-    <col min="18" max="18" width="11.5703125" customWidth="1"/>
-    <col min="19" max="19" width="14.85546875" customWidth="1"/>
+    <col min="1" max="1" customWidth="true" width="39.7109375"/>
+    <col min="2" max="2" customWidth="true" width="10.140625"/>
+    <col min="3" max="3" customWidth="true" width="39.7109375"/>
+    <col min="4" max="4" customWidth="true" width="11.0"/>
+    <col min="5" max="5" customWidth="true" width="13.28515625"/>
+    <col min="6" max="6" customWidth="true" width="8.85546875"/>
+    <col min="7" max="7" customWidth="true" width="17.85546875"/>
+    <col min="8" max="8" customWidth="true" width="19.5703125"/>
+    <col min="9" max="9" customWidth="true" width="23.7109375"/>
+    <col min="10" max="10" customWidth="true" width="12.7109375"/>
+    <col min="11" max="11" customWidth="true" width="11.85546875"/>
+    <col min="12" max="12" customWidth="true" width="17.42578125"/>
+    <col min="13" max="14" customWidth="true" width="39.7109375"/>
+    <col min="15" max="15" customWidth="true" width="25.7109375"/>
+    <col min="16" max="17" customWidth="true" width="16.5703125"/>
+    <col min="18" max="18" customWidth="true" width="11.5703125"/>
+    <col min="19" max="19" customWidth="true" width="14.85546875"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:19">

</xml_diff>

<commit_message>
Updated Locator And Fixed Failed Scenarios
 Updated Locator And Fixed Failed Scenarios
</commit_message>
<xml_diff>
--- a/testdata/ItemDetails.xlsx
+++ b/testdata/ItemDetails.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="4" lowestEdited="5" rupBuild="4505"/>
   <workbookPr/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="2520" windowWidth="15150" windowHeight="6540" firstSheet="21" activeTab="28"/>
+    <workbookView xWindow="0" yWindow="2520" windowWidth="15150" windowHeight="6540" firstSheet="24" activeTab="30"/>
   </bookViews>
   <sheets>
     <sheet name="PR Details" sheetId="1" r:id="rId1"/>
@@ -36,6 +36,8 @@
     <sheet name="RFQDOM" sheetId="26" r:id="rId27"/>
     <sheet name="GATEITEM" sheetId="27" r:id="rId28"/>
     <sheet name="StockAdjustment" sheetId="29" r:id="rId29"/>
+    <sheet name="LandedCostField" sheetId="30" r:id="rId30"/>
+    <sheet name="ChargeItem" sheetId="31" r:id="rId31"/>
   </sheets>
   <calcPr calcId="124519"/>
   <extLst>
@@ -55,7 +57,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="838" uniqueCount="313">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="846" uniqueCount="318">
   <si>
     <t>ITEM_NAME</t>
   </si>
@@ -922,69 +924,12 @@
     <t>AFTER STOCK QTY</t>
   </si>
   <si>
-    <t>119139.4</t>
-  </si>
-  <si>
-    <t>100115</t>
-  </si>
-  <si>
-    <t>500003</t>
-  </si>
-  <si>
-    <t>300033</t>
-  </si>
-  <si>
     <t>HEAT NO</t>
   </si>
   <si>
     <t>TEST NO</t>
   </si>
   <si>
-    <t>119237.4</t>
-  </si>
-  <si>
-    <t>100125</t>
-  </si>
-  <si>
-    <t>500004</t>
-  </si>
-  <si>
-    <t>300044</t>
-  </si>
-  <si>
-    <t>119337.4</t>
-  </si>
-  <si>
-    <t>100135</t>
-  </si>
-  <si>
-    <t>300055</t>
-  </si>
-  <si>
-    <t>500005</t>
-  </si>
-  <si>
-    <t>119437.4</t>
-  </si>
-  <si>
-    <t>100145</t>
-  </si>
-  <si>
-    <t>300066</t>
-  </si>
-  <si>
-    <t>500006</t>
-  </si>
-  <si>
-    <t>119537.4</t>
-  </si>
-  <si>
-    <t>100155</t>
-  </si>
-  <si>
-    <t>300077</t>
-  </si>
-  <si>
     <t>500007</t>
   </si>
   <si>
@@ -995,13 +940,84 @@
   </si>
   <si>
     <t>300088</t>
+  </si>
+  <si>
+    <t>LandedCostItem</t>
+  </si>
+  <si>
+    <t>landedCostSupplier</t>
+  </si>
+  <si>
+    <t>LandedCostAmount</t>
+  </si>
+  <si>
+    <t>LandedCostDocumentNumber</t>
+  </si>
+  <si>
+    <t>AICselection</t>
+  </si>
+  <si>
+    <t>TVS-CH-00011</t>
+  </si>
+  <si>
+    <t>C00009</t>
+  </si>
+  <si>
+    <t>APM1001</t>
+  </si>
+  <si>
+    <t>Y</t>
+  </si>
+  <si>
+    <t>TVS-CH-00002</t>
+  </si>
+  <si>
+    <t>SUP00124</t>
+  </si>
+  <si>
+    <t>APM1002</t>
+  </si>
+  <si>
+    <t>N</t>
+  </si>
+  <si>
+    <t>TVS-CH-00003</t>
+  </si>
+  <si>
+    <t>APM1003</t>
+  </si>
+  <si>
+    <t>D</t>
+  </si>
+  <si>
+    <t>ChargesBasis</t>
+  </si>
+  <si>
+    <t>ItemName</t>
+  </si>
+  <si>
+    <t>Amount</t>
+  </si>
+  <si>
+    <t>GLAccount</t>
+  </si>
+  <si>
+    <t>P</t>
+  </si>
+  <si>
+    <t>FRIEGHT CHARGES</t>
+  </si>
+  <si>
+    <t>V</t>
+  </si>
+  <si>
+    <t>PACKING CHARGES</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
   <fonts count="15">
     <font>
       <sz val="11"/>
@@ -1183,7 +1199,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="43">
+  <cellXfs count="45">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -1307,6 +1323,12 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="14" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -1799,15 +1821,15 @@
   <dimension ref="A1:J20"/>
   <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" customWidth="true" width="20.7109375"/>
-    <col min="2" max="3" customWidth="true" width="12.7109375"/>
-    <col min="4" max="4" customWidth="true" width="14.7109375"/>
-    <col min="5" max="5" customWidth="true" width="9.85546875"/>
-    <col min="6" max="6" customWidth="true" width="14.140625"/>
-    <col min="7" max="7" customWidth="true" width="14.85546875"/>
-    <col min="8" max="8" customWidth="true" width="22.28515625"/>
-    <col min="9" max="9" customWidth="true" width="14.42578125"/>
-    <col min="10" max="10" customWidth="true" width="13.0"/>
+    <col min="1" max="1" width="20.7109375" customWidth="1"/>
+    <col min="2" max="3" width="12.7109375" customWidth="1"/>
+    <col min="4" max="4" width="14.7109375" customWidth="1"/>
+    <col min="5" max="5" width="9.85546875" customWidth="1"/>
+    <col min="6" max="6" width="14.140625" customWidth="1"/>
+    <col min="7" max="7" width="14.85546875" customWidth="1"/>
+    <col min="8" max="8" width="22.28515625" customWidth="1"/>
+    <col min="9" max="9" width="14.42578125" customWidth="1"/>
+    <col min="10" max="10" width="13" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:10">
@@ -2140,17 +2162,17 @@
   <dimension ref="A1:K6"/>
   <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" customWidth="true" width="9.0"/>
-    <col min="2" max="2" customWidth="true" width="25.7109375"/>
-    <col min="3" max="3" customWidth="true" width="12.42578125"/>
-    <col min="4" max="4" customWidth="true" width="16.28515625"/>
-    <col min="5" max="5" customWidth="true" width="20.28515625"/>
-    <col min="6" max="6" customWidth="true" width="25.7109375"/>
-    <col min="7" max="7" customWidth="true" width="12.28515625"/>
-    <col min="8" max="8" customWidth="true" width="14.5703125"/>
-    <col min="9" max="9" customWidth="true" width="28.5703125"/>
-    <col min="10" max="10" customWidth="true" width="23.0"/>
-    <col min="11" max="11" customWidth="true" width="14.7109375"/>
+    <col min="1" max="1" width="9" customWidth="1"/>
+    <col min="2" max="2" width="25.7109375" customWidth="1"/>
+    <col min="3" max="3" width="12.42578125" customWidth="1"/>
+    <col min="4" max="4" width="16.28515625" customWidth="1"/>
+    <col min="5" max="5" width="20.28515625" customWidth="1"/>
+    <col min="6" max="6" width="25.7109375" customWidth="1"/>
+    <col min="7" max="7" width="12.28515625" customWidth="1"/>
+    <col min="8" max="8" width="14.5703125" customWidth="1"/>
+    <col min="9" max="9" width="28.5703125" customWidth="1"/>
+    <col min="10" max="10" width="23" customWidth="1"/>
+    <col min="11" max="11" width="14.7109375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:11">
@@ -2373,11 +2395,11 @@
   <dimension ref="A1:E4"/>
   <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" customWidth="true" width="13.5703125"/>
-    <col min="2" max="2" customWidth="true" width="6.0"/>
-    <col min="3" max="3" customWidth="true" width="14.42578125"/>
-    <col min="4" max="4" customWidth="true" width="18.140625"/>
-    <col min="5" max="5" customWidth="true" width="19.5703125"/>
+    <col min="1" max="1" width="13.5703125" customWidth="1"/>
+    <col min="2" max="2" width="6" customWidth="1"/>
+    <col min="3" max="3" width="14.42578125" customWidth="1"/>
+    <col min="4" max="4" width="18.140625" customWidth="1"/>
+    <col min="5" max="5" width="19.5703125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5">
@@ -2458,13 +2480,13 @@
   <dimension ref="A1:G14"/>
   <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" customWidth="true" width="25.7109375"/>
-    <col min="2" max="2" customWidth="true" width="8.85546875"/>
-    <col min="3" max="3" customWidth="true" width="12.28515625"/>
-    <col min="4" max="4" customWidth="true" width="7.140625"/>
-    <col min="5" max="5" customWidth="true" width="5.28515625"/>
-    <col min="6" max="6" customWidth="true" width="17.42578125"/>
-    <col min="7" max="7" customWidth="true" width="12.42578125"/>
+    <col min="1" max="1" width="25.7109375" customWidth="1"/>
+    <col min="2" max="2" width="8.85546875" customWidth="1"/>
+    <col min="3" max="3" width="12.28515625" customWidth="1"/>
+    <col min="4" max="4" width="7.140625" customWidth="1"/>
+    <col min="5" max="5" width="5.28515625" customWidth="1"/>
+    <col min="6" max="6" width="17.42578125" customWidth="1"/>
+    <col min="7" max="7" width="12.42578125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7">
@@ -2799,9 +2821,9 @@
   <dimension ref="A1:C3"/>
   <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" customWidth="true" width="25.5703125"/>
-    <col min="2" max="2" customWidth="true" width="15.140625"/>
-    <col min="3" max="3" customWidth="true" width="16.42578125"/>
+    <col min="1" max="1" width="25.5703125" customWidth="1"/>
+    <col min="2" max="2" width="15.140625" customWidth="1"/>
+    <col min="3" max="3" width="16.42578125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3">
@@ -2847,12 +2869,12 @@
   <dimension ref="A1:F3"/>
   <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" bestFit="true" customWidth="true" width="24.85546875"/>
-    <col min="2" max="2" customWidth="true" width="11.5703125"/>
-    <col min="3" max="3" customWidth="true" width="9.0"/>
-    <col min="4" max="4" bestFit="true" customWidth="true" width="19.28515625"/>
-    <col min="5" max="5" customWidth="true" width="19.28515625"/>
-    <col min="6" max="6" bestFit="true" customWidth="true" width="12.28515625"/>
+    <col min="1" max="1" width="24.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="11.5703125" customWidth="1"/>
+    <col min="3" max="3" width="9" customWidth="1"/>
+    <col min="4" max="4" width="19.28515625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="19.28515625" customWidth="1"/>
+    <col min="6" max="6" width="12.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6">
@@ -2885,13 +2907,13 @@
       <c r="C2" s="3">
         <v>10</v>
       </c>
-      <c r="D2" t="s" s="0">
+      <c r="D2" t="s">
         <v>268</v>
       </c>
-      <c r="E2" t="s" s="0">
+      <c r="E2" t="s">
         <v>270</v>
       </c>
-      <c r="F2" s="0">
+      <c r="F2">
         <f>ROUND(C2*E2,2)</f>
         <v>847.48</v>
       </c>
@@ -2906,13 +2928,13 @@
       <c r="C3" s="3">
         <v>12</v>
       </c>
-      <c r="D3" t="s" s="0">
+      <c r="D3" t="s">
         <v>271</v>
       </c>
-      <c r="E3" t="s" s="0">
+      <c r="E3" t="s">
         <v>267</v>
       </c>
-      <c r="F3" s="0">
+      <c r="F3">
         <f>ROUND(C3*E3,2)</f>
         <v>159.26</v>
       </c>
@@ -2927,9 +2949,9 @@
   <dimension ref="A1:C3"/>
   <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" customWidth="true" width="21.42578125"/>
-    <col min="2" max="2" customWidth="true" width="11.5703125"/>
-    <col min="3" max="3" customWidth="true" width="9.0"/>
+    <col min="1" max="1" width="21.42578125" customWidth="1"/>
+    <col min="2" max="2" width="11.5703125" customWidth="1"/>
+    <col min="3" max="3" width="9" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3">
@@ -2975,7 +2997,7 @@
   <dimension ref="A1:B2"/>
   <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" customWidth="true" width="20.42578125"/>
+    <col min="1" max="1" width="20.42578125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2">
@@ -3150,26 +3172,26 @@
   <dimension ref="A1:T10"/>
   <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" customWidth="true" width="30.0"/>
-    <col min="2" max="2" customWidth="true" width="36.42578125"/>
-    <col min="3" max="3" customWidth="true" width="6.0"/>
-    <col min="4" max="4" customWidth="true" width="13.7109375"/>
-    <col min="5" max="5" customWidth="true" width="5.28515625"/>
-    <col min="6" max="6" customWidth="true" width="17.28515625"/>
-    <col min="7" max="7" customWidth="true" width="30.28515625"/>
-    <col min="8" max="8" customWidth="true" width="26.85546875"/>
-    <col min="9" max="9" customWidth="true" width="17.28515625"/>
-    <col min="10" max="10" customWidth="true" width="13.28515625"/>
-    <col min="11" max="11" customWidth="true" width="22.7109375"/>
-    <col min="12" max="12" customWidth="true" width="12.7109375"/>
-    <col min="13" max="13" customWidth="true" width="29.5703125"/>
-    <col min="14" max="14" customWidth="true" width="18.28515625"/>
-    <col min="15" max="15" customWidth="true" width="16.28515625"/>
-    <col min="16" max="16" customWidth="true" width="15.5703125"/>
-    <col min="17" max="17" customWidth="true" width="17.7109375"/>
-    <col min="18" max="18" customWidth="true" width="24.140625"/>
-    <col min="19" max="19" customWidth="true" width="13.42578125"/>
-    <col min="20" max="20" customWidth="true" width="13.5703125"/>
+    <col min="1" max="1" width="30" customWidth="1"/>
+    <col min="2" max="2" width="36.42578125" customWidth="1"/>
+    <col min="3" max="3" width="6" customWidth="1"/>
+    <col min="4" max="4" width="13.7109375" customWidth="1"/>
+    <col min="5" max="5" width="5.28515625" customWidth="1"/>
+    <col min="6" max="6" width="17.28515625" customWidth="1"/>
+    <col min="7" max="7" width="30.28515625" customWidth="1"/>
+    <col min="8" max="8" width="26.85546875" customWidth="1"/>
+    <col min="9" max="9" width="17.28515625" customWidth="1"/>
+    <col min="10" max="10" width="13.28515625" customWidth="1"/>
+    <col min="11" max="11" width="22.7109375" customWidth="1"/>
+    <col min="12" max="12" width="12.7109375" customWidth="1"/>
+    <col min="13" max="13" width="29.5703125" customWidth="1"/>
+    <col min="14" max="14" width="18.28515625" customWidth="1"/>
+    <col min="15" max="15" width="16.28515625" customWidth="1"/>
+    <col min="16" max="16" width="15.5703125" customWidth="1"/>
+    <col min="17" max="17" width="17.7109375" customWidth="1"/>
+    <col min="18" max="18" width="24.140625" customWidth="1"/>
+    <col min="19" max="19" width="13.42578125" customWidth="1"/>
+    <col min="20" max="20" width="13.5703125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:20">
@@ -3463,7 +3485,7 @@
       <c r="D6" s="24" t="s">
         <v>43</v>
       </c>
-      <c r="E6" s="0">
+      <c r="E6">
         <v>5</v>
       </c>
       <c r="F6" s="29" t="s">
@@ -3731,7 +3753,7 @@
   <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:3">
-      <c r="A1" t="s" s="0">
+      <c r="A1" t="s">
         <v>234</v>
       </c>
       <c r="B1" s="9" t="s">
@@ -3742,18 +3764,18 @@
       </c>
     </row>
     <row r="2" spans="1:3">
-      <c r="A2" t="s" s="0">
+      <c r="A2" t="s">
         <v>241</v>
       </c>
-      <c r="B2" s="0">
+      <c r="B2">
         <v>23</v>
       </c>
     </row>
     <row r="3" spans="1:3">
-      <c r="A3" t="s" s="0">
+      <c r="A3" t="s">
         <v>242</v>
       </c>
-      <c r="B3" s="0">
+      <c r="B3">
         <v>45</v>
       </c>
     </row>
@@ -3767,12 +3789,12 @@
   <dimension ref="A1:F3"/>
   <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" customWidth="true" width="23.28515625"/>
-    <col min="2" max="2" customWidth="true" width="10.42578125"/>
-    <col min="3" max="3" customWidth="true" width="11.42578125"/>
-    <col min="4" max="4" customWidth="true" width="11.7109375"/>
-    <col min="5" max="5" customWidth="true" width="14.5703125"/>
-    <col min="6" max="6" customWidth="true" width="17.7109375"/>
+    <col min="1" max="1" width="23.28515625" customWidth="1"/>
+    <col min="2" max="2" width="10.42578125" customWidth="1"/>
+    <col min="3" max="3" width="11.42578125" customWidth="1"/>
+    <col min="4" max="4" width="11.7109375" customWidth="1"/>
+    <col min="5" max="5" width="14.5703125" customWidth="1"/>
+    <col min="6" max="6" width="17.7109375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6">
@@ -3843,12 +3865,12 @@
   <dimension ref="A1:F3"/>
   <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" customWidth="true" width="20.85546875"/>
-    <col min="2" max="2" customWidth="true" width="9.0"/>
-    <col min="3" max="3" customWidth="true" width="8.85546875"/>
-    <col min="4" max="4" customWidth="true" width="6.140625"/>
-    <col min="5" max="5" customWidth="true" width="16.7109375"/>
-    <col min="6" max="6" customWidth="true" width="16.28515625"/>
+    <col min="1" max="1" width="20.85546875" customWidth="1"/>
+    <col min="2" max="2" width="9" customWidth="1"/>
+    <col min="3" max="3" width="8.85546875" customWidth="1"/>
+    <col min="4" max="4" width="6.140625" customWidth="1"/>
+    <col min="5" max="5" width="16.7109375" customWidth="1"/>
+    <col min="6" max="6" width="16.28515625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6">
@@ -3921,12 +3943,12 @@
   <dimension ref="A1:F3"/>
   <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" customWidth="true" width="21.7109375"/>
-    <col min="2" max="2" customWidth="true" width="9.0"/>
-    <col min="3" max="3" customWidth="true" width="8.85546875"/>
-    <col min="4" max="4" customWidth="true" width="6.140625"/>
-    <col min="5" max="5" customWidth="true" width="16.7109375"/>
-    <col min="6" max="6" customWidth="true" width="16.28515625"/>
+    <col min="1" max="1" width="21.7109375" customWidth="1"/>
+    <col min="2" max="2" width="9" customWidth="1"/>
+    <col min="3" max="3" width="8.85546875" customWidth="1"/>
+    <col min="4" max="4" width="6.140625" customWidth="1"/>
+    <col min="5" max="5" width="16.7109375" customWidth="1"/>
+    <col min="6" max="6" width="16.28515625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6">
@@ -3999,12 +4021,12 @@
   <dimension ref="A1:F3"/>
   <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" customWidth="true" width="15.42578125"/>
-    <col min="2" max="2" customWidth="true" width="10.5703125"/>
-    <col min="3" max="3" customWidth="true" width="11.5703125"/>
-    <col min="4" max="4" customWidth="true" width="11.85546875"/>
-    <col min="5" max="5" customWidth="true" width="14.0"/>
-    <col min="6" max="6" customWidth="true" width="16.85546875"/>
+    <col min="1" max="1" width="15.42578125" customWidth="1"/>
+    <col min="2" max="2" width="10.5703125" customWidth="1"/>
+    <col min="3" max="3" width="11.5703125" customWidth="1"/>
+    <col min="4" max="4" width="11.85546875" customWidth="1"/>
+    <col min="5" max="5" width="14" customWidth="1"/>
+    <col min="6" max="6" width="16.85546875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6">
@@ -4077,39 +4099,39 @@
   <dimension ref="A1:C3"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" customWidth="true" width="15.0"/>
+    <col min="1" max="1" width="15" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3">
-      <c r="A1" t="s" s="0">
+      <c r="A1" t="s">
         <v>251</v>
       </c>
-      <c r="B1" t="s" s="0">
+      <c r="B1" t="s">
         <v>79</v>
       </c>
-      <c r="C1" t="s" s="0">
+      <c r="C1" t="s">
         <v>252</v>
       </c>
     </row>
     <row r="2" spans="1:3">
-      <c r="A2" t="s" s="0">
+      <c r="A2" t="s">
         <v>253</v>
       </c>
-      <c r="B2" s="0">
+      <c r="B2">
         <v>5</v>
       </c>
-      <c r="C2" s="0">
+      <c r="C2">
         <v>150</v>
       </c>
     </row>
     <row r="3" spans="1:3">
-      <c r="A3" t="s" s="0">
+      <c r="A3" t="s">
         <v>254</v>
       </c>
-      <c r="B3" s="0">
+      <c r="B3">
         <v>6</v>
       </c>
-      <c r="C3" s="0">
+      <c r="C3">
         <v>200</v>
       </c>
     </row>
@@ -4124,26 +4146,26 @@
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:2">
-      <c r="A1" t="s" s="0">
+      <c r="A1" t="s">
         <v>255</v>
       </c>
-      <c r="B1" t="s" s="0">
+      <c r="B1" t="s">
         <v>256</v>
       </c>
     </row>
     <row r="2" spans="1:2">
-      <c r="A2" t="s" s="0">
+      <c r="A2" t="s">
         <v>257</v>
       </c>
-      <c r="B2" t="s" s="0">
+      <c r="B2" t="s">
         <v>209</v>
       </c>
     </row>
     <row r="3" spans="1:2">
-      <c r="A3" t="s" s="0">
+      <c r="A3" t="s">
         <v>258</v>
       </c>
-      <c r="B3" t="s" s="0">
+      <c r="B3" t="s">
         <v>207</v>
       </c>
     </row>
@@ -4158,26 +4180,26 @@
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:2">
-      <c r="A1" t="s" s="0">
+      <c r="A1" t="s">
         <v>255</v>
       </c>
-      <c r="B1" t="s" s="0">
+      <c r="B1" t="s">
         <v>256</v>
       </c>
     </row>
     <row r="2" spans="1:2">
-      <c r="A2" t="s" s="0">
+      <c r="A2" t="s">
         <v>258</v>
       </c>
-      <c r="B2" t="s" s="0">
+      <c r="B2" t="s">
         <v>209</v>
       </c>
     </row>
     <row r="3" spans="1:2">
-      <c r="A3" t="s" s="0">
+      <c r="A3" t="s">
         <v>259</v>
       </c>
-      <c r="B3" t="s" s="0">
+      <c r="B3" t="s">
         <v>207</v>
       </c>
     </row>
@@ -4191,9 +4213,9 @@
   <dimension ref="A1:C3"/>
   <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" customWidth="true" width="15.7109375"/>
-    <col min="2" max="2" customWidth="true" width="5.0"/>
-    <col min="3" max="3" customWidth="true" width="6.0"/>
+    <col min="1" max="1" width="15.7109375" customWidth="1"/>
+    <col min="2" max="2" width="5" customWidth="1"/>
+    <col min="3" max="3" width="6" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3">
@@ -4239,19 +4261,19 @@
   <dimension ref="A1:O3"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" bestFit="true" customWidth="true" width="4.85546875"/>
-    <col min="2" max="2" bestFit="true" customWidth="true" width="7.0"/>
-    <col min="3" max="3" bestFit="true" customWidth="true" width="28.7109375"/>
-    <col min="4" max="4" bestFit="true" customWidth="true" width="9.28515625"/>
-    <col min="5" max="5" bestFit="true" customWidth="true" width="28.7109375"/>
-    <col min="6" max="6" bestFit="true" customWidth="true" width="4.5703125"/>
-    <col min="7" max="7" bestFit="true" customWidth="true" width="10.42578125"/>
-    <col min="8" max="8" bestFit="true" customWidth="true" width="13.140625"/>
-    <col min="9" max="9" bestFit="true" customWidth="true" width="8.28515625"/>
-    <col min="10" max="10" bestFit="true" customWidth="true" width="21.5703125"/>
-    <col min="11" max="11" bestFit="true" customWidth="true" width="16.0"/>
-    <col min="12" max="12" bestFit="true" customWidth="true" width="18.140625"/>
-    <col min="13" max="13" bestFit="true" customWidth="true" width="16.7109375"/>
+    <col min="1" max="1" width="4.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="7" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="28.7109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="9.28515625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="28.7109375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="4.5703125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="13.140625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="8.28515625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="21.5703125" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="16" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="18.140625" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="16.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:15">
@@ -4295,10 +4317,10 @@
         <v>287</v>
       </c>
       <c r="N1" s="42" t="s">
-        <v>292</v>
+        <v>288</v>
       </c>
       <c r="O1" s="42" t="s">
-        <v>293</v>
+        <v>289</v>
       </c>
     </row>
     <row r="2" spans="1:15">
@@ -4323,8 +4345,8 @@
       <c r="G2" s="3">
         <v>1200</v>
       </c>
-      <c r="H2" t="s" s="0">
-        <v>309</v>
+      <c r="H2" t="s">
+        <v>290</v>
       </c>
       <c r="I2" s="3">
         <v>100</v>
@@ -4333,18 +4355,18 @@
       <c r="K2" s="40" t="s">
         <v>281</v>
       </c>
-      <c r="L2" t="s" s="0">
-        <v>310</v>
-      </c>
-      <c r="M2" s="0">
+      <c r="L2" t="s">
+        <v>291</v>
+      </c>
+      <c r="M2">
         <f>SUM(L2+F2)</f>
         <v>100</v>
       </c>
-      <c r="N2" t="str" s="0">
+      <c r="N2" t="str">
         <f>H2</f>
         <v>500003</v>
       </c>
-      <c r="O2" t="str" s="0">
+      <c r="O2" t="str">
         <f>H2</f>
         <v>500003</v>
       </c>
@@ -4375,16 +4397,16 @@
       <c r="I3" s="3">
         <v>10</v>
       </c>
-      <c r="J3" t="s" s="0">
-        <v>312</v>
+      <c r="J3" t="s">
+        <v>293</v>
       </c>
       <c r="K3" s="40" t="s">
         <v>281</v>
       </c>
-      <c r="L3" t="s" s="0">
-        <v>311</v>
-      </c>
-      <c r="M3" s="0">
+      <c r="L3" t="s">
+        <v>292</v>
+      </c>
+      <c r="M3">
         <f>SUM(L3+F3)</f>
         <v>10</v>
       </c>
@@ -4400,17 +4422,17 @@
   <dimension ref="A1:R3"/>
   <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="2" customWidth="true" width="21.0"/>
-    <col min="3" max="3" customWidth="true" width="6.0"/>
-    <col min="4" max="4" customWidth="true" width="12.7109375"/>
-    <col min="5" max="5" customWidth="true" width="19.42578125"/>
-    <col min="6" max="6" customWidth="true" width="15.140625"/>
-    <col min="7" max="7" customWidth="true" width="15.42578125"/>
-    <col min="8" max="8" customWidth="true" width="19.5703125"/>
-    <col min="9" max="9" customWidth="true" width="10.85546875"/>
-    <col min="10" max="10" customWidth="true" width="17.5703125"/>
-    <col min="11" max="11" customWidth="true" width="11.28515625"/>
-    <col min="12" max="12" customWidth="true" width="21.7109375"/>
+    <col min="1" max="2" width="21" customWidth="1"/>
+    <col min="3" max="3" width="6" customWidth="1"/>
+    <col min="4" max="4" width="12.7109375" customWidth="1"/>
+    <col min="5" max="5" width="19.42578125" customWidth="1"/>
+    <col min="6" max="6" width="15.140625" customWidth="1"/>
+    <col min="7" max="7" width="15.42578125" customWidth="1"/>
+    <col min="8" max="8" width="19.5703125" customWidth="1"/>
+    <col min="9" max="9" width="10.85546875" customWidth="1"/>
+    <col min="10" max="10" width="17.5703125" customWidth="1"/>
+    <col min="11" max="11" width="11.28515625" customWidth="1"/>
+    <col min="12" max="12" width="21.7109375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:18">
@@ -4541,6 +4563,147 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet30.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:E4"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="15.5703125" bestFit="1" customWidth="1"/>
+    <col min="2" max="3" width="18.7109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="28.28515625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.140625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5">
+      <c r="A1" t="s">
+        <v>294</v>
+      </c>
+      <c r="B1" t="s">
+        <v>295</v>
+      </c>
+      <c r="C1" t="s">
+        <v>296</v>
+      </c>
+      <c r="D1" t="s">
+        <v>297</v>
+      </c>
+      <c r="E1" t="s">
+        <v>298</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5">
+      <c r="A2" t="s">
+        <v>299</v>
+      </c>
+      <c r="B2" t="s">
+        <v>300</v>
+      </c>
+      <c r="C2">
+        <v>10020</v>
+      </c>
+      <c r="D2" t="s">
+        <v>301</v>
+      </c>
+      <c r="E2" s="43" t="s">
+        <v>302</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5">
+      <c r="A3" t="s">
+        <v>303</v>
+      </c>
+      <c r="B3" t="s">
+        <v>304</v>
+      </c>
+      <c r="C3">
+        <v>10100</v>
+      </c>
+      <c r="D3" t="s">
+        <v>305</v>
+      </c>
+      <c r="E3" s="43" t="s">
+        <v>306</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5">
+      <c r="A4" t="s">
+        <v>307</v>
+      </c>
+      <c r="B4" t="s">
+        <v>300</v>
+      </c>
+      <c r="C4">
+        <v>10020</v>
+      </c>
+      <c r="D4" t="s">
+        <v>308</v>
+      </c>
+      <c r="E4" s="43" t="s">
+        <v>309</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet31.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:D3"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="12.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="17" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="21.140625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4">
+      <c r="A1" s="44" t="s">
+        <v>310</v>
+      </c>
+      <c r="B1" s="44" t="s">
+        <v>311</v>
+      </c>
+      <c r="C1" s="44" t="s">
+        <v>312</v>
+      </c>
+      <c r="D1" s="44" t="s">
+        <v>313</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4">
+      <c r="A2" s="3" t="s">
+        <v>314</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>315</v>
+      </c>
+      <c r="C2" s="3">
+        <v>5</v>
+      </c>
+      <c r="D2" s="3" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4">
+      <c r="A3" s="3" t="s">
+        <v>316</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>317</v>
+      </c>
+      <c r="C3" s="3">
+        <v>100</v>
+      </c>
+      <c r="D3" s="3" t="s">
+        <v>46</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
@@ -4549,12 +4712,12 @@
   <dimension ref="A1:F3"/>
   <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" customWidth="true" width="27.140625"/>
-    <col min="2" max="2" customWidth="true" width="10.42578125"/>
-    <col min="3" max="3" customWidth="true" width="11.42578125"/>
-    <col min="4" max="4" customWidth="true" width="11.7109375"/>
-    <col min="5" max="5" customWidth="true" width="14.5703125"/>
-    <col min="6" max="6" customWidth="true" width="17.7109375"/>
+    <col min="1" max="1" width="27.140625" customWidth="1"/>
+    <col min="2" max="2" width="10.42578125" customWidth="1"/>
+    <col min="3" max="3" width="11.42578125" customWidth="1"/>
+    <col min="4" max="4" width="11.7109375" customWidth="1"/>
+    <col min="5" max="5" width="14.5703125" customWidth="1"/>
+    <col min="6" max="6" width="17.7109375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6">
@@ -4625,12 +4788,12 @@
   <dimension ref="A1:F4"/>
   <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" customWidth="true" width="27.140625"/>
-    <col min="2" max="2" customWidth="true" width="10.42578125"/>
-    <col min="3" max="3" customWidth="true" width="11.42578125"/>
-    <col min="4" max="4" customWidth="true" width="11.7109375"/>
-    <col min="5" max="5" customWidth="true" width="14.5703125"/>
-    <col min="6" max="6" customWidth="true" width="17.7109375"/>
+    <col min="1" max="1" width="27.140625" customWidth="1"/>
+    <col min="2" max="2" width="10.42578125" customWidth="1"/>
+    <col min="3" max="3" width="11.42578125" customWidth="1"/>
+    <col min="4" max="4" width="11.7109375" customWidth="1"/>
+    <col min="5" max="5" width="14.5703125" customWidth="1"/>
+    <col min="6" max="6" width="17.7109375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6">
@@ -4719,39 +4882,39 @@
   <dimension ref="A1:C3"/>
   <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" customWidth="true" width="28.7109375"/>
+    <col min="1" max="1" width="28.7109375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3">
-      <c r="A1" t="s" s="0">
+      <c r="A1" t="s">
         <v>78</v>
       </c>
-      <c r="B1" t="s" s="0">
+      <c r="B1" t="s">
         <v>79</v>
       </c>
-      <c r="C1" t="s" s="0">
+      <c r="C1" t="s">
         <v>80</v>
       </c>
     </row>
     <row r="2" spans="1:3">
-      <c r="A2" t="s" s="0">
+      <c r="A2" t="s">
         <v>81</v>
       </c>
-      <c r="B2" s="0">
+      <c r="B2">
         <v>100</v>
       </c>
-      <c r="C2" s="0">
+      <c r="C2">
         <v>34</v>
       </c>
     </row>
     <row r="3" spans="1:3">
-      <c r="A3" t="s" s="0">
+      <c r="A3" t="s">
         <v>82</v>
       </c>
-      <c r="B3" s="0">
+      <c r="B3">
         <v>50</v>
       </c>
-      <c r="C3" s="0">
+      <c r="C3">
         <v>30</v>
       </c>
     </row>
@@ -4765,13 +4928,13 @@
   <dimension ref="A1:G4"/>
   <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" customWidth="true" width="19.7109375"/>
-    <col min="2" max="2" customWidth="true" width="8.140625"/>
-    <col min="3" max="3" customWidth="true" width="8.5703125"/>
-    <col min="4" max="4" customWidth="true" width="17.85546875"/>
-    <col min="5" max="5" customWidth="true" width="12.7109375"/>
-    <col min="6" max="6" customWidth="true" width="14.5703125"/>
-    <col min="7" max="7" customWidth="true" width="17.7109375"/>
+    <col min="1" max="1" width="19.7109375" customWidth="1"/>
+    <col min="2" max="2" width="8.140625" customWidth="1"/>
+    <col min="3" max="3" width="8.5703125" customWidth="1"/>
+    <col min="4" max="4" width="17.85546875" customWidth="1"/>
+    <col min="5" max="5" width="12.7109375" customWidth="1"/>
+    <col min="6" max="6" width="14.5703125" customWidth="1"/>
+    <col min="7" max="7" width="17.7109375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7">
@@ -4870,13 +5033,13 @@
   <dimension ref="A1:G4"/>
   <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" customWidth="true" width="19.7109375"/>
-    <col min="2" max="2" customWidth="true" width="8.140625"/>
-    <col min="3" max="3" customWidth="true" width="8.5703125"/>
-    <col min="4" max="4" customWidth="true" width="17.85546875"/>
-    <col min="5" max="5" customWidth="true" width="12.7109375"/>
-    <col min="6" max="6" customWidth="true" width="14.5703125"/>
-    <col min="7" max="7" customWidth="true" width="17.7109375"/>
+    <col min="1" max="1" width="19.7109375" customWidth="1"/>
+    <col min="2" max="2" width="8.140625" customWidth="1"/>
+    <col min="3" max="3" width="8.5703125" customWidth="1"/>
+    <col min="4" max="4" width="17.85546875" customWidth="1"/>
+    <col min="5" max="5" width="12.7109375" customWidth="1"/>
+    <col min="6" max="6" width="14.5703125" customWidth="1"/>
+    <col min="7" max="7" width="17.7109375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7">
@@ -4975,23 +5138,23 @@
   <dimension ref="A1:S17"/>
   <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" customWidth="true" width="39.7109375"/>
-    <col min="2" max="2" customWidth="true" width="10.140625"/>
-    <col min="3" max="3" customWidth="true" width="39.7109375"/>
-    <col min="4" max="4" customWidth="true" width="11.0"/>
-    <col min="5" max="5" customWidth="true" width="13.28515625"/>
-    <col min="6" max="6" customWidth="true" width="8.85546875"/>
-    <col min="7" max="7" customWidth="true" width="17.85546875"/>
-    <col min="8" max="8" customWidth="true" width="19.5703125"/>
-    <col min="9" max="9" customWidth="true" width="23.7109375"/>
-    <col min="10" max="10" customWidth="true" width="12.7109375"/>
-    <col min="11" max="11" customWidth="true" width="11.85546875"/>
-    <col min="12" max="12" customWidth="true" width="17.42578125"/>
-    <col min="13" max="14" customWidth="true" width="39.7109375"/>
-    <col min="15" max="15" customWidth="true" width="25.7109375"/>
-    <col min="16" max="17" customWidth="true" width="16.5703125"/>
-    <col min="18" max="18" customWidth="true" width="11.5703125"/>
-    <col min="19" max="19" customWidth="true" width="14.85546875"/>
+    <col min="1" max="1" width="39.7109375" customWidth="1"/>
+    <col min="2" max="2" width="10.140625" customWidth="1"/>
+    <col min="3" max="3" width="39.7109375" customWidth="1"/>
+    <col min="4" max="4" width="11" customWidth="1"/>
+    <col min="5" max="5" width="13.28515625" customWidth="1"/>
+    <col min="6" max="6" width="8.85546875" customWidth="1"/>
+    <col min="7" max="7" width="17.85546875" customWidth="1"/>
+    <col min="8" max="8" width="19.5703125" customWidth="1"/>
+    <col min="9" max="9" width="23.7109375" customWidth="1"/>
+    <col min="10" max="10" width="12.7109375" customWidth="1"/>
+    <col min="11" max="11" width="11.85546875" customWidth="1"/>
+    <col min="12" max="12" width="17.42578125" customWidth="1"/>
+    <col min="13" max="14" width="39.7109375" customWidth="1"/>
+    <col min="15" max="15" width="25.7109375" customWidth="1"/>
+    <col min="16" max="17" width="16.5703125" customWidth="1"/>
+    <col min="18" max="18" width="11.5703125" customWidth="1"/>
+    <col min="19" max="19" width="14.85546875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:19">

</xml_diff>

<commit_message>
Updated Fixes For GRN Test And Purchase Order Functions
Updated Fixes For GRN Test And Purchase Order Functions
</commit_message>
<xml_diff>
--- a/testdata/ItemDetails.xlsx
+++ b/testdata/ItemDetails.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="4" lowestEdited="5" rupBuild="4505"/>
   <workbookPr/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="2520" windowWidth="15150" windowHeight="6540" firstSheet="7" activeTab="8"/>
+    <workbookView xWindow="0" yWindow="2520" windowWidth="15150" windowHeight="6540" firstSheet="24" activeTab="30"/>
   </bookViews>
   <sheets>
     <sheet name="PR Details" sheetId="1" r:id="rId1"/>
@@ -57,7 +57,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="850" uniqueCount="318">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="840" uniqueCount="311">
   <si>
     <t>ITEM_NAME</t>
   </si>
@@ -960,34 +960,13 @@
     <t>TVS-CH-00011</t>
   </si>
   <si>
-    <t>C00009</t>
-  </si>
-  <si>
     <t>APM1001</t>
   </si>
   <si>
     <t>Y</t>
   </si>
   <si>
-    <t>TVS-CH-00002</t>
-  </si>
-  <si>
     <t>SUP00124</t>
-  </si>
-  <si>
-    <t>APM1002</t>
-  </si>
-  <si>
-    <t>N</t>
-  </si>
-  <si>
-    <t>TVS-CH-00003</t>
-  </si>
-  <si>
-    <t>APM1003</t>
-  </si>
-  <si>
-    <t>D</t>
   </si>
   <si>
     <t>ChargesBasis</t>
@@ -1199,7 +1178,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="45">
+  <cellXfs count="47">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -1329,6 +1308,12 @@
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -4595,55 +4580,35 @@
       </c>
     </row>
     <row r="2" spans="1:5">
-      <c r="A2" t="s">
+      <c r="A2" s="45" t="s">
         <v>299</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B2" s="45" t="s">
+        <v>302</v>
+      </c>
+      <c r="C2" s="45">
+        <v>10020</v>
+      </c>
+      <c r="D2" s="45" t="s">
         <v>300</v>
       </c>
-      <c r="C2">
-        <v>10020</v>
-      </c>
-      <c r="D2" t="s">
+      <c r="E2" s="43" t="s">
         <v>301</v>
       </c>
-      <c r="E2" s="43" t="s">
-        <v>302</v>
-      </c>
     </row>
     <row r="3" spans="1:5">
-      <c r="A3" t="s">
-        <v>303</v>
-      </c>
-      <c r="B3" t="s">
-        <v>304</v>
-      </c>
-      <c r="C3">
-        <v>10100</v>
-      </c>
-      <c r="D3" t="s">
-        <v>305</v>
-      </c>
-      <c r="E3" s="43" t="s">
-        <v>306</v>
-      </c>
+      <c r="A3" s="45"/>
+      <c r="B3" s="45"/>
+      <c r="C3" s="45"/>
+      <c r="D3" s="45"/>
+      <c r="E3" s="43"/>
     </row>
     <row r="4" spans="1:5">
-      <c r="A4" t="s">
-        <v>307</v>
-      </c>
-      <c r="B4" t="s">
-        <v>300</v>
-      </c>
-      <c r="C4">
-        <v>10020</v>
-      </c>
-      <c r="D4" t="s">
-        <v>308</v>
-      </c>
-      <c r="E4" s="43" t="s">
-        <v>309</v>
-      </c>
+      <c r="A4" s="45"/>
+      <c r="B4" s="45"/>
+      <c r="C4" s="45"/>
+      <c r="D4" s="45"/>
+      <c r="E4" s="43"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -4662,44 +4627,44 @@
   <sheetData>
     <row r="1" spans="1:4">
       <c r="A1" s="44" t="s">
+        <v>303</v>
+      </c>
+      <c r="B1" s="44" t="s">
+        <v>304</v>
+      </c>
+      <c r="C1" s="44" t="s">
+        <v>305</v>
+      </c>
+      <c r="D1" s="44" t="s">
+        <v>306</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4">
+      <c r="A2" s="46" t="s">
+        <v>307</v>
+      </c>
+      <c r="B2" s="46" t="s">
+        <v>308</v>
+      </c>
+      <c r="C2" s="46">
+        <v>5</v>
+      </c>
+      <c r="D2" s="46">
+        <v>5040101000</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4">
+      <c r="A3" s="46" t="s">
+        <v>309</v>
+      </c>
+      <c r="B3" s="46" t="s">
         <v>310</v>
       </c>
-      <c r="B1" s="44" t="s">
-        <v>311</v>
-      </c>
-      <c r="C1" s="44" t="s">
-        <v>312</v>
-      </c>
-      <c r="D1" s="44" t="s">
-        <v>313</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4">
-      <c r="A2" s="3" t="s">
-        <v>314</v>
-      </c>
-      <c r="B2" s="3" t="s">
-        <v>315</v>
-      </c>
-      <c r="C2" s="3">
-        <v>5</v>
-      </c>
-      <c r="D2" s="3" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4">
-      <c r="A3" s="3" t="s">
-        <v>316</v>
-      </c>
-      <c r="B3" s="3" t="s">
-        <v>317</v>
-      </c>
-      <c r="C3" s="3">
+      <c r="C3" s="46">
         <v>100</v>
       </c>
-      <c r="D3" s="3" t="s">
-        <v>46</v>
+      <c r="D3" s="46">
+        <v>5040101000</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Locators changes , Test Data Changes are Fixed
Locators changes , Test Data Changes are Fixed  in Open so , Open So Amd , SalesPriceList Locators, Purchase Req , RFQ Locators are updated
</commit_message>
<xml_diff>
--- a/testdata/ItemDetails.xlsx
+++ b/testdata/ItemDetails.xlsx
@@ -1,10 +1,10 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="4" lowestEdited="5" rupBuild="4505"/>
+  <fileVersion appName="xl" lastEdited="4" lowestEdited="5" rupBuild="4507"/>
   <workbookPr/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="2520" windowWidth="11430" windowHeight="6540" firstSheet="8" activeTab="11"/>
+    <workbookView xWindow="0" yWindow="2520" windowWidth="11430" windowHeight="6540" firstSheet="23" activeTab="24"/>
   </bookViews>
   <sheets>
     <sheet name="PR Details" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
     <sheet name="LandedCostField" sheetId="30" r:id="rId30"/>
     <sheet name="ChargeItem" sheetId="31" r:id="rId31"/>
   </sheets>
-  <calcPr calcId="124519"/>
+  <calcPr calcId="125725"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -801,12 +801,6 @@
     <t>COST</t>
   </si>
   <si>
-    <t>TVS-RM-KDK-01</t>
-  </si>
-  <si>
-    <t>TVS-RM-KDK-02</t>
-  </si>
-  <si>
     <t>Supplier</t>
   </si>
   <si>
@@ -979,6 +973,12 @@
   </si>
   <si>
     <t>1</t>
+  </si>
+  <si>
+    <t>ROAU-RFQ-KDK-01</t>
+  </si>
+  <si>
+    <t>ROAU-RFQ-KDK-02</t>
   </si>
 </sst>
 </file>
@@ -2861,18 +2861,18 @@
         <v>84</v>
       </c>
       <c r="D1" s="37" t="s">
-        <v>263</v>
+        <v>261</v>
       </c>
       <c r="E1" s="37" t="s">
-        <v>259</v>
+        <v>257</v>
       </c>
       <c r="F1" s="37" t="s">
-        <v>260</v>
+        <v>258</v>
       </c>
     </row>
     <row r="2" spans="1:6">
       <c r="A2" s="3" t="s">
-        <v>257</v>
+        <v>255</v>
       </c>
       <c r="B2" s="3" t="s">
         <v>222</v>
@@ -2881,10 +2881,10 @@
         <v>10</v>
       </c>
       <c r="D2" t="s">
+        <v>260</v>
+      </c>
+      <c r="E2" t="s">
         <v>262</v>
-      </c>
-      <c r="E2" t="s">
-        <v>264</v>
       </c>
       <c r="F2">
         <f>ROUND(C2*E2,2)</f>
@@ -2896,16 +2896,16 @@
         <v>114</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="C3" s="3">
         <v>12</v>
       </c>
       <c r="D3" t="s">
-        <v>265</v>
+        <v>263</v>
       </c>
       <c r="E3" t="s">
-        <v>261</v>
+        <v>259</v>
       </c>
       <c r="F3">
         <f>ROUND(C3*E3,2)</f>
@@ -4072,7 +4072,7 @@
   <dimension ref="A1:C3"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="15" customWidth="1"/>
+    <col min="1" max="1" width="17.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3">
@@ -4088,7 +4088,7 @@
     </row>
     <row r="2" spans="1:3">
       <c r="A2" t="s">
-        <v>247</v>
+        <v>305</v>
       </c>
       <c r="B2">
         <v>5</v>
@@ -4099,7 +4099,7 @@
     </row>
     <row r="3" spans="1:3">
       <c r="A3" t="s">
-        <v>248</v>
+        <v>306</v>
       </c>
       <c r="B3">
         <v>6</v>
@@ -4120,15 +4120,15 @@
   <sheetData>
     <row r="1" spans="1:2">
       <c r="A1" t="s">
-        <v>249</v>
+        <v>247</v>
       </c>
       <c r="B1" t="s">
-        <v>250</v>
+        <v>248</v>
       </c>
     </row>
     <row r="2" spans="1:2">
       <c r="A2" t="s">
-        <v>251</v>
+        <v>249</v>
       </c>
       <c r="B2" t="s">
         <v>205</v>
@@ -4136,7 +4136,7 @@
     </row>
     <row r="3" spans="1:2">
       <c r="A3" t="s">
-        <v>252</v>
+        <v>250</v>
       </c>
       <c r="B3" t="s">
         <v>203</v>
@@ -4154,15 +4154,15 @@
   <sheetData>
     <row r="1" spans="1:2">
       <c r="A1" t="s">
-        <v>249</v>
+        <v>247</v>
       </c>
       <c r="B1" t="s">
-        <v>250</v>
+        <v>248</v>
       </c>
     </row>
     <row r="2" spans="1:2">
       <c r="A2" t="s">
-        <v>252</v>
+        <v>250</v>
       </c>
       <c r="B2" t="s">
         <v>205</v>
@@ -4170,7 +4170,7 @@
     </row>
     <row r="3" spans="1:2">
       <c r="A3" t="s">
-        <v>253</v>
+        <v>251</v>
       </c>
       <c r="B3" t="s">
         <v>203</v>
@@ -4193,7 +4193,7 @@
   <sheetData>
     <row r="1" spans="1:3">
       <c r="A1" s="1" t="s">
-        <v>254</v>
+        <v>252</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>79</v>
@@ -4204,7 +4204,7 @@
     </row>
     <row r="2" spans="1:3">
       <c r="A2" s="1" t="s">
-        <v>255</v>
+        <v>253</v>
       </c>
       <c r="B2" s="1">
         <v>10</v>
@@ -4215,7 +4215,7 @@
     </row>
     <row r="3" spans="1:3">
       <c r="A3" s="1" t="s">
-        <v>256</v>
+        <v>254</v>
       </c>
       <c r="B3" s="1">
         <v>20</v>
@@ -4251,49 +4251,49 @@
   <sheetData>
     <row r="1" spans="1:15">
       <c r="A1" s="38" t="s">
+        <v>264</v>
+      </c>
+      <c r="B1" s="38" t="s">
+        <v>275</v>
+      </c>
+      <c r="C1" s="38" t="s">
+        <v>265</v>
+      </c>
+      <c r="D1" s="38" t="s">
         <v>266</v>
       </c>
-      <c r="B1" s="38" t="s">
-        <v>277</v>
-      </c>
-      <c r="C1" s="38" t="s">
+      <c r="E1" s="38" t="s">
         <v>267</v>
-      </c>
-      <c r="D1" s="38" t="s">
-        <v>268</v>
-      </c>
-      <c r="E1" s="38" t="s">
-        <v>269</v>
       </c>
       <c r="F1" s="38" t="s">
         <v>79</v>
       </c>
       <c r="G1" s="38" t="s">
+        <v>268</v>
+      </c>
+      <c r="H1" s="38" t="s">
+        <v>269</v>
+      </c>
+      <c r="I1" s="38" t="s">
         <v>270</v>
       </c>
-      <c r="H1" s="38" t="s">
+      <c r="J1" s="38" t="s">
+        <v>274</v>
+      </c>
+      <c r="K1" s="38" t="s">
         <v>271</v>
       </c>
-      <c r="I1" s="38" t="s">
-        <v>272</v>
-      </c>
-      <c r="J1" s="38" t="s">
-        <v>276</v>
-      </c>
-      <c r="K1" s="38" t="s">
-        <v>273</v>
-      </c>
       <c r="L1" s="41" t="s">
+        <v>278</v>
+      </c>
+      <c r="M1" s="41" t="s">
+        <v>279</v>
+      </c>
+      <c r="N1" s="41" t="s">
         <v>280</v>
       </c>
-      <c r="M1" s="41" t="s">
+      <c r="O1" s="41" t="s">
         <v>281</v>
-      </c>
-      <c r="N1" s="41" t="s">
-        <v>282</v>
-      </c>
-      <c r="O1" s="41" t="s">
-        <v>283</v>
       </c>
     </row>
     <row r="2" spans="1:15">
@@ -4301,16 +4301,16 @@
         <v>1</v>
       </c>
       <c r="B2" s="39" t="s">
-        <v>278</v>
+        <v>276</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>274</v>
+        <v>272</v>
       </c>
       <c r="D2" s="3">
         <v>0</v>
       </c>
       <c r="E2" s="39" t="s">
-        <v>274</v>
+        <v>272</v>
       </c>
       <c r="F2" s="3">
         <v>100</v>
@@ -4319,17 +4319,17 @@
         <v>1200</v>
       </c>
       <c r="H2" t="s">
-        <v>284</v>
+        <v>282</v>
       </c>
       <c r="I2" s="3">
         <v>100</v>
       </c>
       <c r="J2" s="39"/>
       <c r="K2" s="39" t="s">
-        <v>275</v>
+        <v>273</v>
       </c>
       <c r="L2" t="s">
-        <v>285</v>
+        <v>283</v>
       </c>
       <c r="M2">
         <f>SUM(L2+F2)</f>
@@ -4349,16 +4349,16 @@
         <v>2</v>
       </c>
       <c r="B3" s="39" t="s">
-        <v>278</v>
+        <v>276</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
       <c r="D3" s="3">
         <v>0</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
       <c r="F3" s="3">
         <v>10</v>
@@ -4371,13 +4371,13 @@
         <v>10</v>
       </c>
       <c r="J3" t="s">
-        <v>287</v>
+        <v>285</v>
       </c>
       <c r="K3" s="39" t="s">
-        <v>275</v>
+        <v>273</v>
       </c>
       <c r="L3" t="s">
-        <v>286</v>
+        <v>284</v>
       </c>
       <c r="M3">
         <f>SUM(L3+F3)</f>
@@ -4552,36 +4552,36 @@
   <sheetData>
     <row r="1" spans="1:5">
       <c r="A1" t="s">
+        <v>286</v>
+      </c>
+      <c r="B1" t="s">
+        <v>287</v>
+      </c>
+      <c r="C1" t="s">
         <v>288</v>
       </c>
-      <c r="B1" t="s">
+      <c r="D1" t="s">
         <v>289</v>
       </c>
-      <c r="C1" t="s">
+      <c r="E1" t="s">
         <v>290</v>
-      </c>
-      <c r="D1" t="s">
-        <v>291</v>
-      </c>
-      <c r="E1" t="s">
-        <v>292</v>
       </c>
     </row>
     <row r="2" spans="1:5">
       <c r="A2" s="44" t="s">
-        <v>293</v>
+        <v>291</v>
       </c>
       <c r="B2" s="44" t="s">
-        <v>296</v>
+        <v>294</v>
       </c>
       <c r="C2" s="44">
         <v>10020</v>
       </c>
       <c r="D2" s="44" t="s">
-        <v>294</v>
+        <v>292</v>
       </c>
       <c r="E2" s="42" t="s">
-        <v>295</v>
+        <v>293</v>
       </c>
     </row>
     <row r="3" spans="1:5">
@@ -4615,24 +4615,24 @@
   <sheetData>
     <row r="1" spans="1:4">
       <c r="A1" s="43" t="s">
+        <v>295</v>
+      </c>
+      <c r="B1" s="43" t="s">
+        <v>296</v>
+      </c>
+      <c r="C1" s="43" t="s">
         <v>297</v>
       </c>
-      <c r="B1" s="43" t="s">
+      <c r="D1" s="43" t="s">
         <v>298</v>
-      </c>
-      <c r="C1" s="43" t="s">
-        <v>299</v>
-      </c>
-      <c r="D1" s="43" t="s">
-        <v>300</v>
       </c>
     </row>
     <row r="2" spans="1:4">
       <c r="A2" s="45" t="s">
-        <v>301</v>
+        <v>299</v>
       </c>
       <c r="B2" s="45" t="s">
-        <v>302</v>
+        <v>300</v>
       </c>
       <c r="C2" s="45">
         <v>5</v>
@@ -4643,10 +4643,10 @@
     </row>
     <row r="3" spans="1:4">
       <c r="A3" s="45" t="s">
-        <v>303</v>
+        <v>301</v>
       </c>
       <c r="B3" s="45" t="s">
-        <v>304</v>
+        <v>302</v>
       </c>
       <c r="C3" s="45">
         <v>100</v>
@@ -5949,7 +5949,7 @@
         <v>14</v>
       </c>
       <c r="K16" s="24" t="s">
-        <v>305</v>
+        <v>303</v>
       </c>
       <c r="L16" s="46" t="s">
         <v>107</v>
@@ -6000,7 +6000,7 @@
         <v>14</v>
       </c>
       <c r="K17" s="24" t="s">
-        <v>306</v>
+        <v>304</v>
       </c>
       <c r="L17" s="46" t="s">
         <v>107</v>

</xml_diff>

<commit_message>
Updated The Sales Order Locators And Methods
Updated The Sales Order Locators And Methods
</commit_message>
<xml_diff>
--- a/testdata/ItemDetails.xlsx
+++ b/testdata/ItemDetails.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="4" lowestEdited="5" rupBuild="4505"/>
   <workbookPr/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="2520" windowWidth="11430" windowHeight="6540" firstSheet="9" activeTab="11"/>
+    <workbookView xWindow="0" yWindow="2520" windowWidth="11430" windowHeight="6540" firstSheet="8" activeTab="8"/>
   </bookViews>
   <sheets>
     <sheet name="PR Details" sheetId="1" r:id="rId1"/>
@@ -57,7 +57,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="827" uniqueCount="309">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="843" uniqueCount="309">
   <si>
     <t>ITEM_NAME</t>
   </si>
@@ -5208,8 +5208,12 @@
       <c r="L2" s="3" t="s">
         <v>107</v>
       </c>
-      <c r="M2" s="3"/>
-      <c r="N2" s="3"/>
+      <c r="M2" s="21" t="s">
+        <v>106</v>
+      </c>
+      <c r="N2" s="21" t="s">
+        <v>106</v>
+      </c>
       <c r="O2" s="8" t="s">
         <v>13</v>
       </c>
@@ -5259,8 +5263,12 @@
       <c r="L3" s="3" t="s">
         <v>107</v>
       </c>
-      <c r="M3" s="3"/>
-      <c r="N3" s="3"/>
+      <c r="M3" s="21" t="s">
+        <v>110</v>
+      </c>
+      <c r="N3" s="21" t="s">
+        <v>110</v>
+      </c>
       <c r="O3" s="8" t="s">
         <v>13</v>
       </c>
@@ -5758,8 +5766,12 @@
       <c r="L12" s="3" t="s">
         <v>107</v>
       </c>
-      <c r="M12" s="3"/>
-      <c r="N12" s="3"/>
+      <c r="M12" s="3" t="s">
+        <v>125</v>
+      </c>
+      <c r="N12" s="3" t="s">
+        <v>125</v>
+      </c>
       <c r="O12" s="3" t="s">
         <v>57</v>
       </c>
@@ -5809,8 +5821,12 @@
       <c r="L13" s="3" t="s">
         <v>107</v>
       </c>
-      <c r="M13" s="3"/>
-      <c r="N13" s="3"/>
+      <c r="M13" s="3" t="s">
+        <v>127</v>
+      </c>
+      <c r="N13" s="3" t="s">
+        <v>127</v>
+      </c>
       <c r="O13" s="3"/>
       <c r="P13" s="3" t="s">
         <v>22</v>
@@ -5858,8 +5874,12 @@
       <c r="L14" s="16" t="s">
         <v>107</v>
       </c>
-      <c r="M14" s="3"/>
-      <c r="N14" s="3"/>
+      <c r="M14" s="3" t="s">
+        <v>128</v>
+      </c>
+      <c r="N14" s="3" t="s">
+        <v>128</v>
+      </c>
       <c r="O14" s="3" t="s">
         <v>57</v>
       </c>
@@ -5909,8 +5929,12 @@
       <c r="L15" s="16" t="s">
         <v>107</v>
       </c>
-      <c r="M15" s="3"/>
-      <c r="N15" s="3"/>
+      <c r="M15" s="3" t="s">
+        <v>131</v>
+      </c>
+      <c r="N15" s="3" t="s">
+        <v>131</v>
+      </c>
       <c r="O15" s="8" t="s">
         <v>13</v>
       </c>
@@ -5960,8 +5984,12 @@
       <c r="L16" s="46" t="s">
         <v>107</v>
       </c>
-      <c r="M16" s="3"/>
-      <c r="N16" s="3"/>
+      <c r="M16" s="3" t="s">
+        <v>133</v>
+      </c>
+      <c r="N16" s="3" t="s">
+        <v>133</v>
+      </c>
       <c r="O16" s="3" t="s">
         <v>13</v>
       </c>
@@ -6011,8 +6039,12 @@
       <c r="L17" s="46" t="s">
         <v>107</v>
       </c>
-      <c r="M17" s="3"/>
-      <c r="N17" s="3"/>
+      <c r="M17" s="46" t="s">
+        <v>135</v>
+      </c>
+      <c r="N17" s="46" t="s">
+        <v>135</v>
+      </c>
       <c r="O17" s="3" t="s">
         <v>13</v>
       </c>

</xml_diff>